<commit_message>
feat: enemy weight, range and critical rate read
enemy weight, range and critical rate read; register gains regression
conditions

The enemy's term in the order of turns is the float at 0x44 of its
record (getter at 0x4f2150). Range factors are those of the game's
lesson. The register lists the model parts each row needs, drops the
'kept' status and adds a sheet of regression conditions.
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -9,6 +9,8 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Criticisms" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ModelParts" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regression" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -418,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K134"/>
+  <dimension ref="A1:L134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -429,7 +431,7 @@
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="100" customWidth="1" min="8" max="8"/>
-    <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
     <col width="30" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
   </cols>
@@ -477,15 +479,20 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
+          <t>Needs</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>Vanilla_Result</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Balance_Result</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
@@ -532,9 +539,12 @@
           <t>Damage per unit of time and survival of the same character across weapon ranks stay inside the band</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>P01, P02, P03, P04, P07, P09, P10, P15</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -581,9 +591,12 @@
           <t>Caster damage per unit of time against every boss inside the band of its role</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr">
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>P04, P07, P10, P13</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -630,9 +643,12 @@
           <t>For every skill, effect per TP at the top level is not below a stated share of level 1, or the level buys something else that is stated</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>P11, P13</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -679,9 +695,12 @@
           <t>Every boss has a winning party without a Valkyrie inside the win-rate window</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr">
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>P03, P09, P10, P13, P14, P15</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -728,9 +747,12 @@
           <t>Encounters per expedition without a Maid meets the target; every boss has a winning party without one</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr">
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>P03, P10, P11, P12, P13, P14, P15</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -777,9 +799,12 @@
           <t>A gun build is inside the weapon band</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr">
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>P01, P02, P03, P08, P10, P14, P15</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -826,9 +851,12 @@
           <t>Two-handed builds are inside the weapon band at every gear tier</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr">
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>P01, P02, P03, P08, P10, P14, P15, P19</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -865,15 +893,17 @@
           <t>Tedium</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
           <t>Encounters per expedition in the first three dungeons meets the target</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr">
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>P11, P12, P13</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -910,15 +940,17 @@
           <t>Unfair</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
           <t>Hit chance of front-line classes against the enemies of the first three dungeons above a stated floor</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr">
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>P03</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -955,15 +987,17 @@
           <t>Trap</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
           <t>Cost of a skill at the levels reachable in a dungeon against the TP pool of that level</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr">
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>P11, P13</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -1000,15 +1034,17 @@
           <t>Curve</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
           <t>Caster share of party damage is steady across the game, no spike and no cliff</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr">
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>P04, P07, P10, P13</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -1045,15 +1081,17 @@
           <t>Unfair</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
           <t>Survival of a Berserker at promotion level against the enemies of that point</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr">
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>P01, P02, P03, P08, P10, P15</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -1090,15 +1128,17 @@
           <t>Information</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
           <t>The text states what each mercenary does</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr">
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>P03</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -1145,9 +1185,12 @@
           <t>Share of chants completed against each boss above a stated floor</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr">
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>P04, P06, P07, P10, P13</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -1184,15 +1227,17 @@
           <t>Tedium</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
           <t>Expected turns a buff lasts against each boss against its cost</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr">
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>P01, P02, P03, P09, P10, P12, P13, P15</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -1239,9 +1284,12 @@
           <t>No boss blocks every element and every ailment at once</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr">
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>P04, P07, P08, P10, P13</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -1278,15 +1326,17 @@
           <t>Unfair</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr">
         <is>
           <t>Largest single hit of each boss against the HP of an on-level back row, with and without guard</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr">
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>P03, P04, P07, P09, P10, P13</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -1333,9 +1383,12 @@
           <t>Expected actions of a doll before it dies against each boss</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr">
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>P01, P02, P03, P10, P12, P13, P14, P15, P16</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -1372,15 +1425,17 @@
           <t>Unviable</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
           <t>Berserker inside the damage-dealer band at every checkpoint</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr">
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>P01, P02, P03, P04, P07, P10, P13, P14, P15</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -1417,15 +1472,17 @@
           <t>Unviable</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
           <t>A Paladin party clears every boss a Valkyrie party clears, inside the window</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr">
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>P03, P09, P10, P13, P14, P15</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -1472,9 +1529,12 @@
           <t>Dark Lord inside the band, neither above nor below</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr">
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>P01, P02, P03, P09, P10, P14, P15</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -1511,15 +1571,17 @@
           <t>Unviable</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr">
         <is>
           <t>Samurai inside the damage-dealer band</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr">
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>P03, P04, P07, P10, P14, P15</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -1566,9 +1628,12 @@
           <t>Witch and Sage inside the band of their role against postgame bosses</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr">
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>P03, P04, P07, P10, P13, P14, P15</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -1605,15 +1670,17 @@
           <t>Unviable</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr">
         <is>
           <t>Healing per unit of time against boss damage per unit of time</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr">
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>P03, P04, P07, P10, P11, P13, P14, P15</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -1660,9 +1727,12 @@
           <t>Magical Princess inside the band without a crown</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr">
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>P03, P04, P07, P10, P12, P13, P14, P15</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -1699,15 +1769,17 @@
           <t>Unviable</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr">
         <is>
           <t>Treasure Hunter has a stated battle role that is inside its band</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr">
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>P03, P04, P07, P10, P13, P14, P15, P17</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -1754,9 +1826,12 @@
           <t>Kunoichi inside the band of a stated role</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr">
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>P03, P04, P07, P10, P14, P15</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -1793,15 +1868,17 @@
           <t>Mandatory</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr">
         <is>
           <t>Heavy-weapon builds inside the band without the song</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr">
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>P01, P02, P03, P14, P15</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -1848,9 +1925,12 @@
           <t>Mistress inside the band of a stated role</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr">
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>P01, P02, P03, P14, P15</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -1887,15 +1967,17 @@
           <t>Unfair</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr">
         <is>
           <t>Expected value of each chance skill against a plain attack</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr">
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>P03, P12, P13, P14, P15</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -1942,9 +2024,12 @@
           <t>No boss can be denied every action; the skill keeps a use against every boss</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr">
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>P03, P08, P10, P13, P14, P15</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -1991,9 +2076,12 @@
           <t>Joker inside the band; survivable without a Valkyrie with a stated plan</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr">
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>P03, P09, P10, P14, P15</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -2030,15 +2118,17 @@
           <t>Trap</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr">
         <is>
           <t>Checked against the data first: the community file itself says power rises strongly</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr">
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>P03, P04, P07, P10, P14, P15</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -2075,15 +2165,17 @@
           <t>Information</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr">
         <is>
           <t>False in the data; the text already states the real figure (QoL)</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr"/>
-      <c r="K35" t="inlineStr">
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>P03, P14, P15, P17</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -2120,15 +2212,17 @@
           <t>Tedium</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr">
         <is>
           <t>Damage gained per gold spent on forging against other uses of the gold</t>
         </is>
       </c>
-      <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr"/>
-      <c r="K36" t="inlineStr">
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>P04, P07, P10, P15, P19</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -2165,15 +2259,17 @@
           <t>Tedium</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr">
         <is>
           <t>Steps a meal lasts against steps to the boss of each dungeon</t>
         </is>
       </c>
-      <c r="I37" t="inlineStr"/>
-      <c r="J37" t="inlineStr"/>
-      <c r="K37" t="inlineStr">
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>P10, P13</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -2220,9 +2316,12 @@
           <t>Hours to one crown and to all crowns meet the target</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr"/>
-      <c r="J38" t="inlineStr"/>
-      <c r="K38" t="inlineStr">
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>P12, P13</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -2269,9 +2368,12 @@
           <t>Every boss has winning parties that lack each of the three</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr"/>
-      <c r="J39" t="inlineStr"/>
-      <c r="K39" t="inlineStr">
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>P03, P04, P07, P09, P10, P11, P13</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -2308,15 +2410,17 @@
           <t>Mandatory</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr">
         <is>
           <t>Number of class paths with a working answer to boss buffs</t>
         </is>
       </c>
-      <c r="I40" t="inlineStr"/>
-      <c r="J40" t="inlineStr"/>
-      <c r="K40" t="inlineStr">
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>P03, P04, P07, P09, P10, P13</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -2363,9 +2467,12 @@
           <t>Mistress inside the band of a stated role</t>
         </is>
       </c>
-      <c r="I41" t="inlineStr"/>
-      <c r="J41" t="inlineStr"/>
-      <c r="K41" t="inlineStr">
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>P01, P02, P03, P14, P15</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -2412,9 +2519,12 @@
           <t>Kunoichi inside the band of a stated role</t>
         </is>
       </c>
-      <c r="I42" t="inlineStr"/>
-      <c r="J42" t="inlineStr"/>
-      <c r="K42" t="inlineStr">
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>P03, P14, P15</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -2461,9 +2571,12 @@
           <t>Magical Princess inside the band</t>
         </is>
       </c>
-      <c r="I43" t="inlineStr"/>
-      <c r="J43" t="inlineStr"/>
-      <c r="K43" t="inlineStr">
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>P01, P02, P03, P04, P07, P10, P11, P13, P14, P15</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -2510,9 +2623,12 @@
           <t>A mage-heavy party clears every progression boss without that sealbook, or the zones leave it an answer</t>
         </is>
       </c>
-      <c r="I44" t="inlineStr"/>
-      <c r="J44" t="inlineStr"/>
-      <c r="K44" t="inlineStr">
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>P04, P07, P10, P13, P15, P18, P19</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -2559,9 +2675,12 @@
           <t>Every boss has a winning party without a Valkyrie</t>
         </is>
       </c>
-      <c r="I45" t="inlineStr"/>
-      <c r="J45" t="inlineStr"/>
-      <c r="K45" t="inlineStr">
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>P03, P09, P10, P13, P14, P15</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -2608,9 +2727,12 @@
           <t>Two-handed builds inside the weapon band at the last gear tier</t>
         </is>
       </c>
-      <c r="I46" t="inlineStr"/>
-      <c r="J46" t="inlineStr"/>
-      <c r="K46" t="inlineStr">
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>P01, P02, P03, P14, P15, P19</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -2657,9 +2779,12 @@
           <t>Whip builds inside the weapon band</t>
         </is>
       </c>
-      <c r="I47" t="inlineStr"/>
-      <c r="J47" t="inlineStr"/>
-      <c r="K47" t="inlineStr">
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>P01, P02, P03, P14, P15</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -2706,9 +2831,12 @@
           <t>Gun builds have a skill set and are inside the weapon band</t>
         </is>
       </c>
-      <c r="I48" t="inlineStr"/>
-      <c r="J48" t="inlineStr"/>
-      <c r="K48" t="inlineStr">
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>P01, P02, P03, P14, P15</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -2745,15 +2873,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr">
         <is>
           <t>A basic-attack build is inside the band, or those passives feed something that is</t>
         </is>
       </c>
-      <c r="I49" t="inlineStr"/>
-      <c r="J49" t="inlineStr"/>
-      <c r="K49" t="inlineStr">
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>P06</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -2790,15 +2920,17 @@
           <t>Unfair</t>
         </is>
       </c>
-      <c r="G50" t="inlineStr"/>
       <c r="H50" t="inlineStr">
         <is>
           <t>Short-range builds inside the band against enemies that carry it</t>
         </is>
       </c>
-      <c r="I50" t="inlineStr"/>
-      <c r="J50" t="inlineStr"/>
-      <c r="K50" t="inlineStr">
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>P10, P13</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -2835,15 +2967,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G51" t="inlineStr"/>
       <c r="H51" t="inlineStr">
         <is>
           <t>A magic defence change of the size these skills give moves damage by a stated share</t>
         </is>
       </c>
-      <c r="I51" t="inlineStr"/>
-      <c r="J51" t="inlineStr"/>
-      <c r="K51" t="inlineStr">
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>P04, P07, P10</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -2880,15 +3014,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G52" t="inlineStr"/>
       <c r="H52" t="inlineStr">
         <is>
           <t>Value of resistance skills for a party with endgame gear</t>
         </is>
       </c>
-      <c r="I52" t="inlineStr"/>
-      <c r="J52" t="inlineStr"/>
-      <c r="K52" t="inlineStr">
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>P04, P07, P08, P10, P15, P19</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -2925,15 +3061,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G53" t="inlineStr"/>
       <c r="H53" t="inlineStr">
         <is>
           <t>Share of bosses on which each ailment can land</t>
         </is>
       </c>
-      <c r="I53" t="inlineStr"/>
-      <c r="J53" t="inlineStr"/>
-      <c r="K53" t="inlineStr">
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>P08, P10, P13</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -2970,15 +3108,17 @@
           <t>Dominant</t>
         </is>
       </c>
-      <c r="G54" t="inlineStr"/>
       <c r="H54" t="inlineStr">
         <is>
           <t>Healing per unit of time of the song against enemy damage per unit of time at each checkpoint</t>
         </is>
       </c>
-      <c r="I54" t="inlineStr"/>
-      <c r="J54" t="inlineStr"/>
-      <c r="K54" t="inlineStr">
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>P01, P02, P03, P04, P07, P10, P11, P14, P15</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -3025,9 +3165,12 @@
           <t>Joker inside the band in random encounters and with on-curve gear</t>
         </is>
       </c>
-      <c r="I55" t="inlineStr"/>
-      <c r="J55" t="inlineStr"/>
-      <c r="K55" t="inlineStr">
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>P03, P10, P13, P14, P15, P19</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -3074,9 +3217,12 @@
           <t>Dark Lord burst inside the band</t>
         </is>
       </c>
-      <c r="I56" t="inlineStr"/>
-      <c r="J56" t="inlineStr"/>
-      <c r="K56" t="inlineStr">
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>P03, P14, P15</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -3113,15 +3259,17 @@
           <t>Trap</t>
         </is>
       </c>
-      <c r="G57" t="inlineStr"/>
       <c r="H57" t="inlineStr">
         <is>
           <t>Value per skill point is not concentrated in the last level</t>
         </is>
       </c>
-      <c r="I57" t="inlineStr"/>
-      <c r="J57" t="inlineStr"/>
-      <c r="K57" t="inlineStr">
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>P10, P13</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -3158,15 +3306,17 @@
           <t>Trap</t>
         </is>
       </c>
-      <c r="G58" t="inlineStr"/>
       <c r="H58" t="inlineStr">
         <is>
           <t>Every level of a skill buys a stated gain</t>
         </is>
       </c>
-      <c r="I58" t="inlineStr"/>
-      <c r="J58" t="inlineStr"/>
-      <c r="K58" t="inlineStr">
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>P03</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -3203,15 +3353,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G59" t="inlineStr"/>
       <c r="H59" t="inlineStr">
         <is>
           <t>Each of these skills is better than its item in a stated situation</t>
         </is>
       </c>
-      <c r="I59" t="inlineStr"/>
-      <c r="J59" t="inlineStr"/>
-      <c r="K59" t="inlineStr">
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>P01, P02, P03, P11, P15</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -3248,15 +3400,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G60" t="inlineStr"/>
       <c r="H60" t="inlineStr">
         <is>
           <t>Expected value of each against the best plain action</t>
         </is>
       </c>
-      <c r="I60" t="inlineStr"/>
-      <c r="J60" t="inlineStr"/>
-      <c r="K60" t="inlineStr">
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>P04, P07, P10, P12, P13</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -3303,9 +3457,12 @@
           <t>Expected share of boss turns skipped by a stacked party below a stated ceiling</t>
         </is>
       </c>
-      <c r="I61" t="inlineStr"/>
-      <c r="J61" t="inlineStr"/>
-      <c r="K61" t="inlineStr">
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>P01, P02, P03, P08, P10, P12, P13, P15</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -3342,15 +3499,17 @@
           <t>Curve</t>
         </is>
       </c>
-      <c r="G62" t="inlineStr"/>
       <c r="H62" t="inlineStr">
         <is>
           <t>Turn share of physical skill users against casters and item users</t>
         </is>
       </c>
-      <c r="I62" t="inlineStr"/>
-      <c r="J62" t="inlineStr"/>
-      <c r="K62" t="inlineStr">
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>P01, P02, P03, P04, P07, P10, P15</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -3397,9 +3556,12 @@
           <t>Hours to one crown</t>
         </is>
       </c>
-      <c r="I63" t="inlineStr"/>
-      <c r="J63" t="inlineStr"/>
-      <c r="K63" t="inlineStr">
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>P12, P13</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -3446,9 +3608,12 @@
           <t>Encounters per expedition and boss fights without a second Maid</t>
         </is>
       </c>
-      <c r="I64" t="inlineStr"/>
-      <c r="J64" t="inlineStr"/>
-      <c r="K64" t="inlineStr">
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>P10, P11, P12, P13</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -3485,15 +3650,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G65" t="inlineStr"/>
       <c r="H65" t="inlineStr">
         <is>
           <t>There is a situation in which this is the best action, or a build it is part of that is inside the band</t>
         </is>
       </c>
-      <c r="I65" t="inlineStr"/>
-      <c r="J65" t="inlineStr"/>
-      <c r="K65" t="inlineStr">
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>P03, P09, P10, P14, P15</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -3530,15 +3697,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G66" t="inlineStr"/>
       <c r="H66" t="inlineStr">
         <is>
           <t>There is a situation in which this is the best action, or a build it is part of that is inside the band</t>
         </is>
       </c>
-      <c r="I66" t="inlineStr"/>
-      <c r="J66" t="inlineStr"/>
-      <c r="K66" t="inlineStr">
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>P03, P09, P10, P14, P15</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -3575,15 +3744,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G67" t="inlineStr"/>
       <c r="H67" t="inlineStr">
         <is>
           <t>There is a situation in which this is the best action, or a build it is part of that is inside the band</t>
         </is>
       </c>
-      <c r="I67" t="inlineStr"/>
-      <c r="J67" t="inlineStr"/>
-      <c r="K67" t="inlineStr">
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>P01, P02, P03, P14, P15</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -3620,15 +3791,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G68" t="inlineStr"/>
       <c r="H68" t="inlineStr">
         <is>
           <t>There is a situation in which this is the best action, or a build it is part of that is inside the band</t>
         </is>
       </c>
-      <c r="I68" t="inlineStr"/>
-      <c r="J68" t="inlineStr"/>
-      <c r="K68" t="inlineStr">
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>P03, P12, P13, P14, P15</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -3665,15 +3838,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G69" t="inlineStr"/>
       <c r="H69" t="inlineStr">
         <is>
           <t>There is a situation in which this is the best action, or a build it is part of that is inside the band</t>
         </is>
       </c>
-      <c r="I69" t="inlineStr"/>
-      <c r="J69" t="inlineStr"/>
-      <c r="K69" t="inlineStr">
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>P03, P14, P15</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -3710,15 +3885,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G70" t="inlineStr"/>
       <c r="H70" t="inlineStr">
         <is>
           <t>There is a situation in which this is the best action, or a build it is part of that is inside the band</t>
         </is>
       </c>
-      <c r="I70" t="inlineStr"/>
-      <c r="J70" t="inlineStr"/>
-      <c r="K70" t="inlineStr">
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>P03, P14, P15</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -3755,15 +3932,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G71" t="inlineStr"/>
       <c r="H71" t="inlineStr">
         <is>
           <t>There is a situation in which this is the best action, or a build it is part of that is inside the band</t>
         </is>
       </c>
-      <c r="I71" t="inlineStr"/>
-      <c r="J71" t="inlineStr"/>
-      <c r="K71" t="inlineStr">
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>P03, P04, P07, P10, P14, P15</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -3800,15 +3979,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G72" t="inlineStr"/>
       <c r="H72" t="inlineStr">
         <is>
           <t>There is a situation in which this is the best action, or a build it is part of that is inside the band</t>
         </is>
       </c>
-      <c r="I72" t="inlineStr"/>
-      <c r="J72" t="inlineStr"/>
-      <c r="K72" t="inlineStr">
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>P03, P14, P15</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -3845,15 +4026,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G73" t="inlineStr"/>
       <c r="H73" t="inlineStr">
         <is>
           <t>There is a situation in which this is the best action, or a build it is part of that is inside the band</t>
         </is>
       </c>
-      <c r="I73" t="inlineStr"/>
-      <c r="J73" t="inlineStr"/>
-      <c r="K73" t="inlineStr">
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>P03, P14, P15</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -3890,15 +4073,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G74" t="inlineStr"/>
       <c r="H74" t="inlineStr">
         <is>
           <t>There is a situation in which this is the best action, or a build it is part of that is inside the band</t>
         </is>
       </c>
-      <c r="I74" t="inlineStr"/>
-      <c r="J74" t="inlineStr"/>
-      <c r="K74" t="inlineStr">
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>P03, P14, P15</t>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -3935,15 +4120,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G75" t="inlineStr"/>
       <c r="H75" t="inlineStr">
         <is>
           <t>There is a situation in which this is the best action, or a build it is part of that is inside the band</t>
         </is>
       </c>
-      <c r="I75" t="inlineStr"/>
-      <c r="J75" t="inlineStr"/>
-      <c r="K75" t="inlineStr">
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>P03, P14, P15</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -3980,15 +4167,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G76" t="inlineStr"/>
       <c r="H76" t="inlineStr">
         <is>
           <t>There is a situation in which this is the best action, or a build it is part of that is inside the band</t>
         </is>
       </c>
-      <c r="I76" t="inlineStr"/>
-      <c r="J76" t="inlineStr"/>
-      <c r="K76" t="inlineStr">
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>P03, P10, P13, P14, P15</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -4025,15 +4214,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G77" t="inlineStr"/>
       <c r="H77" t="inlineStr">
         <is>
           <t>There is a situation in which this is the best action, or a build it is part of that is inside the band</t>
         </is>
       </c>
-      <c r="I77" t="inlineStr"/>
-      <c r="J77" t="inlineStr"/>
-      <c r="K77" t="inlineStr">
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>P03, P08, P10, P14, P15</t>
+        </is>
+      </c>
+      <c r="L77" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -4070,15 +4261,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G78" t="inlineStr"/>
       <c r="H78" t="inlineStr">
         <is>
           <t>There is a situation in which this is the best action, or a build it is part of that is inside the band</t>
         </is>
       </c>
-      <c r="I78" t="inlineStr"/>
-      <c r="J78" t="inlineStr"/>
-      <c r="K78" t="inlineStr">
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>P03, P11, P14, P15</t>
+        </is>
+      </c>
+      <c r="L78" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -4115,15 +4308,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G79" t="inlineStr"/>
       <c r="H79" t="inlineStr">
         <is>
           <t>There is a situation in which this is the best action, or a build it is part of that is inside the band</t>
         </is>
       </c>
-      <c r="I79" t="inlineStr"/>
-      <c r="J79" t="inlineStr"/>
-      <c r="K79" t="inlineStr">
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>P03, P11, P14, P15</t>
+        </is>
+      </c>
+      <c r="L79" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -4160,15 +4355,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G80" t="inlineStr"/>
       <c r="H80" t="inlineStr">
         <is>
           <t>There is a situation in which this is the best action, or a build it is part of that is inside the band</t>
         </is>
       </c>
-      <c r="I80" t="inlineStr"/>
-      <c r="J80" t="inlineStr"/>
-      <c r="K80" t="inlineStr">
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>P03, P14, P15</t>
+        </is>
+      </c>
+      <c r="L80" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -4205,15 +4402,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G81" t="inlineStr"/>
       <c r="H81" t="inlineStr">
         <is>
           <t>There is a situation in which this is the best action, or a build it is part of that is inside the band</t>
         </is>
       </c>
-      <c r="I81" t="inlineStr"/>
-      <c r="J81" t="inlineStr"/>
-      <c r="K81" t="inlineStr">
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>P03, P14, P15</t>
+        </is>
+      </c>
+      <c r="L81" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -4250,15 +4449,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G82" t="inlineStr"/>
       <c r="H82" t="inlineStr">
         <is>
           <t>There is a situation in which this is the best action, or a build it is part of that is inside the band</t>
         </is>
       </c>
-      <c r="I82" t="inlineStr"/>
-      <c r="J82" t="inlineStr"/>
-      <c r="K82" t="inlineStr">
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>P03, P14, P15</t>
+        </is>
+      </c>
+      <c r="L82" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -4295,15 +4496,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G83" t="inlineStr"/>
       <c r="H83" t="inlineStr">
         <is>
           <t>There is a situation in which this is the best action, or a build it is part of that is inside the band</t>
         </is>
       </c>
-      <c r="I83" t="inlineStr"/>
-      <c r="J83" t="inlineStr"/>
-      <c r="K83" t="inlineStr">
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>P03, P04, P07, P10, P14, P15</t>
+        </is>
+      </c>
+      <c r="L83" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -4340,15 +4543,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G84" t="inlineStr"/>
       <c r="H84" t="inlineStr">
         <is>
           <t>There is a situation in which this is the best action, or a build it is part of that is inside the band</t>
         </is>
       </c>
-      <c r="I84" t="inlineStr"/>
-      <c r="J84" t="inlineStr"/>
-      <c r="K84" t="inlineStr">
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>P03, P04, P07, P10, P14, P15</t>
+        </is>
+      </c>
+      <c r="L84" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -4385,15 +4590,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G85" t="inlineStr"/>
       <c r="H85" t="inlineStr">
         <is>
           <t>There is a situation in which this is the best action, or a build it is part of that is inside the band</t>
         </is>
       </c>
-      <c r="I85" t="inlineStr"/>
-      <c r="J85" t="inlineStr"/>
-      <c r="K85" t="inlineStr">
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>P03, P14, P15</t>
+        </is>
+      </c>
+      <c r="L85" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -4430,15 +4637,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G86" t="inlineStr"/>
       <c r="H86" t="inlineStr">
         <is>
           <t>There is a situation in which this is the best action, or a build it is part of that is inside the band</t>
         </is>
       </c>
-      <c r="I86" t="inlineStr"/>
-      <c r="J86" t="inlineStr"/>
-      <c r="K86" t="inlineStr">
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>P03, P14, P15</t>
+        </is>
+      </c>
+      <c r="L86" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -4475,15 +4684,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G87" t="inlineStr"/>
       <c r="H87" t="inlineStr">
         <is>
           <t>There is a situation in which this is the best action, or a build it is part of that is inside the band</t>
         </is>
       </c>
-      <c r="I87" t="inlineStr"/>
-      <c r="J87" t="inlineStr"/>
-      <c r="K87" t="inlineStr">
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>P03, P14, P15, P17</t>
+        </is>
+      </c>
+      <c r="L87" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -4520,15 +4731,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G88" t="inlineStr"/>
       <c r="H88" t="inlineStr">
         <is>
           <t>There is a situation in which this is the best action, or a build it is part of that is inside the band</t>
         </is>
       </c>
-      <c r="I88" t="inlineStr"/>
-      <c r="J88" t="inlineStr"/>
-      <c r="K88" t="inlineStr">
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>P03, P08, P10, P14, P15</t>
+        </is>
+      </c>
+      <c r="L88" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -4565,15 +4778,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G89" t="inlineStr"/>
       <c r="H89" t="inlineStr">
         <is>
           <t>There is a situation in which this is the best action, or a build it is part of that is inside the band</t>
         </is>
       </c>
-      <c r="I89" t="inlineStr"/>
-      <c r="J89" t="inlineStr"/>
-      <c r="K89" t="inlineStr">
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>P03, P04, P07, P10, P14, P15</t>
+        </is>
+      </c>
+      <c r="L89" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -4610,15 +4825,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G90" t="inlineStr"/>
       <c r="H90" t="inlineStr">
         <is>
           <t>There is a situation in which this is the best action, or a build it is part of that is inside the band</t>
         </is>
       </c>
-      <c r="I90" t="inlineStr"/>
-      <c r="J90" t="inlineStr"/>
-      <c r="K90" t="inlineStr">
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>P03, P14, P15</t>
+        </is>
+      </c>
+      <c r="L90" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -4655,15 +4872,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G91" t="inlineStr"/>
       <c r="H91" t="inlineStr">
         <is>
           <t>There is a situation in which this is the best action, or a build it is part of that is inside the band</t>
         </is>
       </c>
-      <c r="I91" t="inlineStr"/>
-      <c r="J91" t="inlineStr"/>
-      <c r="K91" t="inlineStr">
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>P01, P02, P03, P14, P15</t>
+        </is>
+      </c>
+      <c r="L91" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -4700,15 +4919,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G92" t="inlineStr"/>
       <c r="H92" t="inlineStr">
         <is>
           <t>There is a situation in which this is the best action, or a build it is part of that is inside the band</t>
         </is>
       </c>
-      <c r="I92" t="inlineStr"/>
-      <c r="J92" t="inlineStr"/>
-      <c r="K92" t="inlineStr">
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>P03, P14, P15</t>
+        </is>
+      </c>
+      <c r="L92" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -4745,15 +4966,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G93" t="inlineStr"/>
       <c r="H93" t="inlineStr">
         <is>
           <t>There is a situation in which this is the best action, or a build it is part of that is inside the band</t>
         </is>
       </c>
-      <c r="I93" t="inlineStr"/>
-      <c r="J93" t="inlineStr"/>
-      <c r="K93" t="inlineStr">
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>P03, P14, P15</t>
+        </is>
+      </c>
+      <c r="L93" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -4790,15 +5013,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G94" t="inlineStr"/>
       <c r="H94" t="inlineStr">
         <is>
           <t>There is a situation in which this is the best action, or a build it is part of that is inside the band</t>
         </is>
       </c>
-      <c r="I94" t="inlineStr"/>
-      <c r="J94" t="inlineStr"/>
-      <c r="K94" t="inlineStr">
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>P03, P14, P15</t>
+        </is>
+      </c>
+      <c r="L94" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -4835,15 +5060,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G95" t="inlineStr"/>
       <c r="H95" t="inlineStr">
         <is>
           <t>There is a situation in which this is the best action, or a build it is part of that is inside the band</t>
         </is>
       </c>
-      <c r="I95" t="inlineStr"/>
-      <c r="J95" t="inlineStr"/>
-      <c r="K95" t="inlineStr">
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>P01, P02, P03, P14, P15</t>
+        </is>
+      </c>
+      <c r="L95" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -4880,15 +5107,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G96" t="inlineStr"/>
       <c r="H96" t="inlineStr">
         <is>
           <t>There is a situation in which this is the best action, or a build it is part of that is inside the band</t>
         </is>
       </c>
-      <c r="I96" t="inlineStr"/>
-      <c r="J96" t="inlineStr"/>
-      <c r="K96" t="inlineStr">
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>P03, P08, P10, P14, P15</t>
+        </is>
+      </c>
+      <c r="L96" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -4925,15 +5154,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G97" t="inlineStr"/>
       <c r="H97" t="inlineStr">
         <is>
           <t>There is a situation in which this is the best action, or a build it is part of that is inside the band</t>
         </is>
       </c>
-      <c r="I97" t="inlineStr"/>
-      <c r="J97" t="inlineStr"/>
-      <c r="K97" t="inlineStr">
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>P03, P14, P15</t>
+        </is>
+      </c>
+      <c r="L97" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -4970,15 +5201,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G98" t="inlineStr"/>
       <c r="H98" t="inlineStr">
         <is>
           <t>There is a situation in which this is the best action, or a build it is part of that is inside the band</t>
         </is>
       </c>
-      <c r="I98" t="inlineStr"/>
-      <c r="J98" t="inlineStr"/>
-      <c r="K98" t="inlineStr">
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>P01, P02, P03, P14, P15</t>
+        </is>
+      </c>
+      <c r="L98" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -5015,15 +5248,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G99" t="inlineStr"/>
       <c r="H99" t="inlineStr">
         <is>
           <t>There is a situation in which this is the best action, or a build it is part of that is inside the band</t>
         </is>
       </c>
-      <c r="I99" t="inlineStr"/>
-      <c r="J99" t="inlineStr"/>
-      <c r="K99" t="inlineStr">
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>P01, P02, P03, P08, P10, P14, P15</t>
+        </is>
+      </c>
+      <c r="L99" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -5060,15 +5295,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G100" t="inlineStr"/>
       <c r="H100" t="inlineStr">
         <is>
           <t>There is a situation in which this is the best action, or a build it is part of that is inside the band</t>
         </is>
       </c>
-      <c r="I100" t="inlineStr"/>
-      <c r="J100" t="inlineStr"/>
-      <c r="K100" t="inlineStr">
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>P03, P14, P15</t>
+        </is>
+      </c>
+      <c r="L100" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -5105,15 +5342,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G101" t="inlineStr"/>
       <c r="H101" t="inlineStr">
         <is>
           <t>There is a situation in which this is the best action, or a build it is part of that is inside the band</t>
         </is>
       </c>
-      <c r="I101" t="inlineStr"/>
-      <c r="J101" t="inlineStr"/>
-      <c r="K101" t="inlineStr">
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>P03, P06, P14, P15</t>
+        </is>
+      </c>
+      <c r="L101" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -5150,15 +5389,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G102" t="inlineStr"/>
       <c r="H102" t="inlineStr">
         <is>
           <t>There is a situation in which this is the best action, or a build it is part of that is inside the band</t>
         </is>
       </c>
-      <c r="I102" t="inlineStr"/>
-      <c r="J102" t="inlineStr"/>
-      <c r="K102" t="inlineStr">
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>P03, P14, P15</t>
+        </is>
+      </c>
+      <c r="L102" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -5195,15 +5436,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G103" t="inlineStr"/>
       <c r="H103" t="inlineStr">
         <is>
           <t>There is a situation in which this is the best action, or a build it is part of that is inside the band</t>
         </is>
       </c>
-      <c r="I103" t="inlineStr"/>
-      <c r="J103" t="inlineStr"/>
-      <c r="K103" t="inlineStr">
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>P03, P14, P15</t>
+        </is>
+      </c>
+      <c r="L103" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -5240,15 +5483,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G104" t="inlineStr"/>
       <c r="H104" t="inlineStr">
         <is>
           <t>There is a situation in which this is the best action, or a build it is part of that is inside the band</t>
         </is>
       </c>
-      <c r="I104" t="inlineStr"/>
-      <c r="J104" t="inlineStr"/>
-      <c r="K104" t="inlineStr">
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>P03, P06, P14, P15</t>
+        </is>
+      </c>
+      <c r="L104" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -5285,15 +5530,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G105" t="inlineStr"/>
       <c r="H105" t="inlineStr">
         <is>
           <t>There is a situation in which this is the best action, or a build it is part of that is inside the band</t>
         </is>
       </c>
-      <c r="I105" t="inlineStr"/>
-      <c r="J105" t="inlineStr"/>
-      <c r="K105" t="inlineStr">
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>P03, P14, P15</t>
+        </is>
+      </c>
+      <c r="L105" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -5330,15 +5577,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G106" t="inlineStr"/>
       <c r="H106" t="inlineStr">
         <is>
           <t>There is a situation in which this is the best action, or a build it is part of that is inside the band</t>
         </is>
       </c>
-      <c r="I106" t="inlineStr"/>
-      <c r="J106" t="inlineStr"/>
-      <c r="K106" t="inlineStr">
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>P01, P02, P03, P14, P15</t>
+        </is>
+      </c>
+      <c r="L106" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -5375,15 +5624,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G107" t="inlineStr"/>
       <c r="H107" t="inlineStr">
         <is>
           <t>There is a situation in which this is the best action, or a build it is part of that is inside the band</t>
         </is>
       </c>
-      <c r="I107" t="inlineStr"/>
-      <c r="J107" t="inlineStr"/>
-      <c r="K107" t="inlineStr">
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>P03, P14, P15</t>
+        </is>
+      </c>
+      <c r="L107" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -5420,15 +5671,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G108" t="inlineStr"/>
       <c r="H108" t="inlineStr">
         <is>
           <t>There is a situation in which this is the best action, or a build it is part of that is inside the band</t>
         </is>
       </c>
-      <c r="I108" t="inlineStr"/>
-      <c r="J108" t="inlineStr"/>
-      <c r="K108" t="inlineStr">
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>P03, P14, P15</t>
+        </is>
+      </c>
+      <c r="L108" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -5465,15 +5718,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G109" t="inlineStr"/>
       <c r="H109" t="inlineStr">
         <is>
           <t>There is a situation in which this is the best action, or a build it is part of that is inside the band</t>
         </is>
       </c>
-      <c r="I109" t="inlineStr"/>
-      <c r="J109" t="inlineStr"/>
-      <c r="K109" t="inlineStr">
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>P03, P14, P15, P16</t>
+        </is>
+      </c>
+      <c r="L109" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -5510,15 +5765,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G110" t="inlineStr"/>
       <c r="H110" t="inlineStr">
         <is>
           <t>There is a situation in which this is the best action, or a build it is part of that is inside the band</t>
         </is>
       </c>
-      <c r="I110" t="inlineStr"/>
-      <c r="J110" t="inlineStr"/>
-      <c r="K110" t="inlineStr">
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>P03, P14, P15</t>
+        </is>
+      </c>
+      <c r="L110" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -5555,15 +5812,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G111" t="inlineStr"/>
       <c r="H111" t="inlineStr">
         <is>
           <t>There is a situation in which this is the best action, or a build it is part of that is inside the band</t>
         </is>
       </c>
-      <c r="I111" t="inlineStr"/>
-      <c r="J111" t="inlineStr"/>
-      <c r="K111" t="inlineStr">
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>P01, P02, P03, P14, P15</t>
+        </is>
+      </c>
+      <c r="L111" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -5600,15 +5859,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G112" t="inlineStr"/>
       <c r="H112" t="inlineStr">
         <is>
           <t>There is a situation in which this is the best action, or a build it is part of that is inside the band</t>
         </is>
       </c>
-      <c r="I112" t="inlineStr"/>
-      <c r="J112" t="inlineStr"/>
-      <c r="K112" t="inlineStr">
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>P03, P14, P15</t>
+        </is>
+      </c>
+      <c r="L112" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -5645,15 +5906,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G113" t="inlineStr"/>
       <c r="H113" t="inlineStr">
         <is>
           <t>There is a situation in which this is the best action, or a build it is part of that is inside the band</t>
         </is>
       </c>
-      <c r="I113" t="inlineStr"/>
-      <c r="J113" t="inlineStr"/>
-      <c r="K113" t="inlineStr">
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>P03, P14, P15</t>
+        </is>
+      </c>
+      <c r="L113" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -5690,15 +5953,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G114" t="inlineStr"/>
       <c r="H114" t="inlineStr">
         <is>
           <t>There is a situation in which this is the best action, or a build it is part of that is inside the band</t>
         </is>
       </c>
-      <c r="I114" t="inlineStr"/>
-      <c r="J114" t="inlineStr"/>
-      <c r="K114" t="inlineStr">
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>P03, P14, P15</t>
+        </is>
+      </c>
+      <c r="L114" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -5735,15 +6000,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G115" t="inlineStr"/>
       <c r="H115" t="inlineStr">
         <is>
           <t>There is a situation in which this is the best action, or a build it is part of that is inside the band</t>
         </is>
       </c>
-      <c r="I115" t="inlineStr"/>
-      <c r="J115" t="inlineStr"/>
-      <c r="K115" t="inlineStr">
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>P03, P14, P15, P16</t>
+        </is>
+      </c>
+      <c r="L115" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -5780,15 +6047,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G116" t="inlineStr"/>
       <c r="H116" t="inlineStr">
         <is>
           <t>There is a situation in which this is the best action, or a build it is part of that is inside the band</t>
         </is>
       </c>
-      <c r="I116" t="inlineStr"/>
-      <c r="J116" t="inlineStr"/>
-      <c r="K116" t="inlineStr">
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>P03, P06, P14, P15</t>
+        </is>
+      </c>
+      <c r="L116" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -5825,15 +6094,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G117" t="inlineStr"/>
       <c r="H117" t="inlineStr">
         <is>
           <t>There is a situation in which this is the best action, or a build it is part of that is inside the band</t>
         </is>
       </c>
-      <c r="I117" t="inlineStr"/>
-      <c r="J117" t="inlineStr"/>
-      <c r="K117" t="inlineStr">
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>P03, P06, P14, P15</t>
+        </is>
+      </c>
+      <c r="L117" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -5870,15 +6141,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G118" t="inlineStr"/>
       <c r="H118" t="inlineStr">
         <is>
           <t>There is a situation in which this is the best action, or a build it is part of that is inside the band</t>
         </is>
       </c>
-      <c r="I118" t="inlineStr"/>
-      <c r="J118" t="inlineStr"/>
-      <c r="K118" t="inlineStr">
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>P03, P14, P15</t>
+        </is>
+      </c>
+      <c r="L118" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -5915,15 +6188,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G119" t="inlineStr"/>
       <c r="H119" t="inlineStr">
         <is>
           <t>There is a situation in which this is the best action, or a build it is part of that is inside the band</t>
         </is>
       </c>
-      <c r="I119" t="inlineStr"/>
-      <c r="J119" t="inlineStr"/>
-      <c r="K119" t="inlineStr">
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>P03, P14, P15</t>
+        </is>
+      </c>
+      <c r="L119" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -5960,15 +6235,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G120" t="inlineStr"/>
       <c r="H120" t="inlineStr">
         <is>
           <t>There is a situation in which this is the best action, or a build it is part of that is inside the band</t>
         </is>
       </c>
-      <c r="I120" t="inlineStr"/>
-      <c r="J120" t="inlineStr"/>
-      <c r="K120" t="inlineStr">
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>P03, P14, P15</t>
+        </is>
+      </c>
+      <c r="L120" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -6005,15 +6282,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G121" t="inlineStr"/>
       <c r="H121" t="inlineStr">
         <is>
           <t>There is a situation in which this is the best action, or a build it is part of that is inside the band</t>
         </is>
       </c>
-      <c r="I121" t="inlineStr"/>
-      <c r="J121" t="inlineStr"/>
-      <c r="K121" t="inlineStr">
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>P01, P02, P03, P14, P15</t>
+        </is>
+      </c>
+      <c r="L121" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -6050,15 +6329,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G122" t="inlineStr"/>
       <c r="H122" t="inlineStr">
         <is>
           <t>There is a situation in which this is the best action, or a build it is part of that is inside the band</t>
         </is>
       </c>
-      <c r="I122" t="inlineStr"/>
-      <c r="J122" t="inlineStr"/>
-      <c r="K122" t="inlineStr">
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>P03, P14, P15</t>
+        </is>
+      </c>
+      <c r="L122" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -6095,15 +6376,17 @@
           <t>Dominant</t>
         </is>
       </c>
-      <c r="G123" t="inlineStr"/>
       <c r="H123" t="inlineStr">
         <is>
           <t>Share of a boss HP removed by the best joint opening below a stated ceiling</t>
         </is>
       </c>
-      <c r="I123" t="inlineStr"/>
-      <c r="J123" t="inlineStr"/>
-      <c r="K123" t="inlineStr">
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>P10, P13</t>
+        </is>
+      </c>
+      <c r="L123" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -6150,9 +6433,12 @@
           <t>No boss action kills a full on-level party from full HP without a counter the party could have had</t>
         </is>
       </c>
-      <c r="I124" t="inlineStr"/>
-      <c r="J124" t="inlineStr"/>
-      <c r="K124" t="inlineStr">
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>P03, P04, P07, P08, P09, P10, P13</t>
+        </is>
+      </c>
+      <c r="L124" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -6199,9 +6485,12 @@
           <t>Sniper inside the band, with bow and with gun</t>
         </is>
       </c>
-      <c r="I125" t="inlineStr"/>
-      <c r="J125" t="inlineStr"/>
-      <c r="K125" t="inlineStr">
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>P01, P02, P03, P14, P15</t>
+        </is>
+      </c>
+      <c r="L125" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -6238,15 +6527,17 @@
           <t>Unviable</t>
         </is>
       </c>
-      <c r="G126" t="inlineStr"/>
       <c r="H126" t="inlineStr">
         <is>
           <t>Their best gear set puts them inside the band</t>
         </is>
       </c>
-      <c r="I126" t="inlineStr"/>
-      <c r="J126" t="inlineStr"/>
-      <c r="K126" t="inlineStr">
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>P15, P19</t>
+        </is>
+      </c>
+      <c r="L126" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -6283,15 +6574,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G127" t="inlineStr"/>
       <c r="H127" t="inlineStr">
         <is>
           <t>Each grand sealbook is the best choice for some party or task</t>
         </is>
       </c>
-      <c r="I127" t="inlineStr"/>
-      <c r="J127" t="inlineStr"/>
-      <c r="K127" t="inlineStr">
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>P11, P13, P15, P19</t>
+        </is>
+      </c>
+      <c r="L127" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -6328,15 +6621,17 @@
           <t>Tedium</t>
         </is>
       </c>
-      <c r="G128" t="inlineStr"/>
       <c r="H128" t="inlineStr">
         <is>
           <t>Expected kills per wanted drop below a stated ceiling</t>
         </is>
       </c>
-      <c r="I128" t="inlineStr"/>
-      <c r="J128" t="inlineStr"/>
-      <c r="K128" t="inlineStr">
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>P12, P13, P17</t>
+        </is>
+      </c>
+      <c r="L128" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -6373,15 +6668,17 @@
           <t>Curve</t>
         </is>
       </c>
-      <c r="G129" t="inlineStr"/>
       <c r="H129" t="inlineStr">
         <is>
           <t>Largest swing a zone gives to a fight inside a stated range</t>
         </is>
       </c>
-      <c r="I129" t="inlineStr"/>
-      <c r="J129" t="inlineStr"/>
-      <c r="K129" t="inlineStr">
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>P04, P07, P10, P12, P13, P18</t>
+        </is>
+      </c>
+      <c r="L129" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -6428,9 +6725,12 @@
           <t>Hours to one crown without DLC equipment meet the target</t>
         </is>
       </c>
-      <c r="I130" t="inlineStr"/>
-      <c r="J130" t="inlineStr"/>
-      <c r="K130" t="inlineStr">
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>P12, P13</t>
+        </is>
+      </c>
+      <c r="L130" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -6467,15 +6767,17 @@
           <t>Tedium</t>
         </is>
       </c>
-      <c r="G131" t="inlineStr"/>
       <c r="H131" t="inlineStr">
         <is>
           <t>Hours to bring an unused character to 75</t>
         </is>
       </c>
-      <c r="I131" t="inlineStr"/>
-      <c r="J131" t="inlineStr"/>
-      <c r="K131" t="inlineStr">
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>P12, P13</t>
+        </is>
+      </c>
+      <c r="L131" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -6512,15 +6814,17 @@
           <t>Dead</t>
         </is>
       </c>
-      <c r="G132" t="inlineStr"/>
       <c r="H132" t="inlineStr">
         <is>
           <t>Share of a mercenary turn spent on actions without effect</t>
         </is>
       </c>
-      <c r="I132" t="inlineStr"/>
-      <c r="J132" t="inlineStr"/>
-      <c r="K132" t="inlineStr">
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>P01, P02, P03, P15, P17</t>
+        </is>
+      </c>
+      <c r="L132" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -6557,15 +6861,17 @@
           <t>Mandatory</t>
         </is>
       </c>
-      <c r="G133" t="inlineStr"/>
       <c r="H133" t="inlineStr">
         <is>
           <t>Those bosses have winning parties without a Treasure Hunter</t>
         </is>
       </c>
-      <c r="I133" t="inlineStr"/>
-      <c r="J133" t="inlineStr"/>
-      <c r="K133" t="inlineStr">
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>P04, P07, P10, P11, P13</t>
+        </is>
+      </c>
+      <c r="L133" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -6602,15 +6908,17 @@
           <t>Curve</t>
         </is>
       </c>
-      <c r="G134" t="inlineStr"/>
       <c r="H134" t="inlineStr">
         <is>
           <t>Kill time of each against a matched party above a stated floor</t>
         </is>
       </c>
-      <c r="I134" t="inlineStr"/>
-      <c r="J134" t="inlineStr"/>
-      <c r="K134" t="inlineStr">
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>P18</t>
+        </is>
+      </c>
+      <c r="L134" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -6627,7 +6935,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -6654,7 +6962,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Every complaint of the Japanese community and every criticism of the GameFAQs guides for this game (Hentaicheg, faqs/80834). Claims are paraphrased, not quoted.</t>
+          <t>Every complaint of the Japanese community and every criticism of the GameFAQs guide for this game (Hentaicheg, faqs/80834). Claims are paraphrased, not quoted.</t>
         </is>
       </c>
     </row>
@@ -6666,67 +6974,757 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Definition of the user (2026-10-05): the Balance variant is finished when every Japanese complaint is addressed and no criticism of the guide holds any more. Status of every row must be "closed" or "kept", with its result.</t>
+          <t>Definition of the user (2026-10-05): every row of Criticisms is "closed" or "not a problem", AND every row of Regression holds on the built variant. Closing the known criticisms is not enough: a fix that makes something else dominant must be caught, and nobody complained about it in vanilla.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Kind</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Dead: never worth using. Unviable: a class or build that cannot keep up. Dominant: so strong that it removes choices. Mandatory: the game cannot be played without it. Trap: a choice that punishes the player. Tedium: time without decisions. Unfair: a loss the player could not prevent. Curve: the shape of difficulty over the game. Mixed: both too strong and too weak. Information: a fact to state or to check.</t>
+          <t>open; closed (the test fails in vanilla and passes on the built variant); not a problem (the simulator shows the claim is false in vanilla, with the measure). There is no "kept": a criticism that is true in vanilla is fixed. Hard to fix is not a reason.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Test</t>
+          <t>Needs</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>How the model decides the claim. The bands, windows and floors are the targets of docs/BALANCE_PLAN.md, phase 3.</t>
+          <t>The parts of the model a row depends on (sheet ModelParts). A row cannot be judged, in vanilla or in the variant, while one of them is not "read": speed, locks and tanks wait for the weight of enemies, ailments against resistance, targeting and the enemy AI.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Vanilla_Result / Balance_Result</t>
+          <t>Kind</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Filled by the simulator, never by hand: confirmed, partly, false, with the measure.</t>
+          <t>Dead: never worth using. Unviable: a class or build that cannot keep up. Dominant: so strong that it removes choices. Mandatory: the game cannot be played without it. Trap: a choice that punishes the player. Tedium: time without decisions. Unfair: a loss the player could not prevent. Curve: the shape of difficulty over the game. Mixed: both too strong and too weak. Information: a fact to state or to check.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Status</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>open, closed (no longer true), kept (true on purpose, with the reason), not a problem (false in vanilla).</t>
+          <t>How the model decides the claim. The bands, windows and floors are the targets of docs/BALANCE_PLAN.md, phase 3.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>Vanilla_Result / Balance_Result</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Filled by the simulator, never by hand.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>No figures</t>
         </is>
       </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>No value of the game is typed in this workbook. Vanilla figures are generated into docs/generated/BALANCE_BASELINE.md.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="90" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Part</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>What</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Where</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Order of turns</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>docs/FORMULAS.md 5; checked against a player test</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>P02</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Weight of an enemy in the order of turns</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>EnemyStatusData 0x44, getter 0x4f2150 (slot 0xf4 of the enemy class)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>P03</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Physical damage</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>docs/FORMULAS.md 2; range factor read; critical multiplier and minimum damage open</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>P04</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Magic damage</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>read in part</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>docs/FORMULAS.md 3; defence side and caps to finish</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>P05</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Hit chance</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>docs/FORMULAS.md 2.1, 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>P06</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Critical hits</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>read in part</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Rate read (0x44f190); multiplier open</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>P07</t>
+        </is>
+      </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>No value of the game is typed in this workbook. Vanilla figures are generated into docs/generated/BALANCE_BASELINE.md.</t>
+          <t>Chant interruption</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>read in part</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Damage against max HP read; the 1 in 3 on a critical hit not located</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>P08</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Ailment chance against resistance</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>ccommandprobabilitybase.cpp</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>P09</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Targeting and enmity</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>cbattleai2.cpp; effect 170</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Enemy AI (which attack, when)</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>EnemyAIData.bin, Battle::CBattleAI2</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>P11</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Healing and TP recovery</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Message at 0x66ce90</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>P12</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>EXP: division and factor by level gap</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>cbattleresult.cpp</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>P13</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Encounters per floor</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Floor parameter files; records of 22 ints</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>P14</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Class growth: which row is which class path</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>ClassLevelData read; mapping open</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>P15</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Equipment stats</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>EquipmentData 0x24-0x58</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>P16</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Summons and dolls</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Summon.pck; effects 228-233</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>P17</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Drops</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>EnemyStatusData 0x68-0xA8</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>P18</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Zones</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>read in part</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Multiply attack A (0x44fbb0)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>P19</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Enchantment sizes</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>read in part</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Constants after each count of pieces; table to generate</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="120" customWidth="1" min="3" max="3"/>
+    <col width="70" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Condition</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Meaning</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Measured on</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>R01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>No new dominant strategy</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>No class, weapon type, skill or party is above the top of its band at any checkpoint, including those nobody complained about in vanilla</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Every build the simulator enumerates, not only the criticised ones</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>R02</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Nothing viable in vanilla becomes unviable</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Every class, weapon type and skill that is inside its band in vanilla stays inside it</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Vanilla result against Balance result for every build</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>R03</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>The curve has no jump</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>From one floor or boss to the next, the lethality an on-level party meets does not rise by more than the stated step, and never falls below the previous one by more than it</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Expected party level from encounter EXP; every floor and boss in order</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>R04</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>No new mandatory piece</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>For every boss, removing any single class from the pool leaves winning parties</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Win rate over compositions with each class excluded</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>R05</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>No new lock</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>No boss can be denied every action by any combination of skills, items, mercenaries and summons</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Largest expected share of boss turns removed</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>R06</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>No change without a row</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Every value that differs from vanilla serves a row of Criticisms or a row of this sheet</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Build check: every change names the row it serves</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>R07</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Smallest change</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Among the sets of values that pass every test, the one closest to vanilla is the one shipped</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Distance from vanilla reported with the result</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>R08</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Difficulty is kept</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Win rate and fight length of a sensible on-level party against each boss stay inside the window of vanilla for that boss, except where a row of Criticisms says vanilla was unfair there</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Per boss, vanilla against Balance</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: ailment chance against resistance read from the command code
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -7259,12 +7259,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>read in part</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>ccommandprobabilitybase.cpp</t>
+          <t>docs/FORMULAS.md 5b: ailments read (0x481ea0); turn delay (effect 54) and turn skipping open</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: enemy AI decoder and the weighted roll that picks an enemy's
enemy AI decoder and the weighted roll that picks an enemy's target
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -7281,12 +7281,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>read</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>cbattleai2.cpp; effect 170</t>
+          <t>docs/FORMULAS.md 9.1: weighted roll (0x43f450, 0x44a630); formation row number and scope names to confirm</t>
         </is>
       </c>
     </row>
@@ -7303,12 +7303,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>read</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>EnemyAIData.bin, Battle::CBattleAI2</t>
+          <t>docs/FORMULAS.md 9; tools/enemy_ai.py decodes the 516 scripts</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: critical hit read in full
critical hit read in full (limits 5 to 50, factor 1.25) and the minimum
damage
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -7154,7 +7154,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>docs/FORMULAS.md 2; range factor read; critical multiplier and minimum damage open</t>
+          <t>docs/FORMULAS.md 2 and 4: range, critical factor and minimum damage read; zone factor case by case open</t>
         </is>
       </c>
     </row>
@@ -7215,12 +7215,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>read in part</t>
+          <t>read</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Rate read (0x44f190); multiplier open</t>
+          <t>docs/FORMULAS.md 4: rate, limits 5-50, factor 1.25 (0x44f190)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: healing formula and its cap read from the heal command
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -7325,12 +7325,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>read in part</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Message at 0x66ce90</t>
+          <t>docs/FORMULAS.md 6b: HP heal and its cap read (0x48d730); TP recovery, revival and after-battle recovery open</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: class growth row by class and route, read from GetClassLevelID
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -7352,7 +7352,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>cbattleresult.cpp</t>
+          <t>cbattleresult.cpp; an enemy keeps its EXP at offset 8 of its object (0x4f0794); the division is not located</t>
         </is>
       </c>
     </row>
@@ -7391,12 +7391,12 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>read</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>ClassLevelData read; mapping open</t>
+          <t>docs/FORMULAS.md 10; tools/class_data.py (row by class and previous class, 0x5545b0)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: equipment stats and upgrade rule read
equipment stats and upgrade rule read; equipment and enemy attack
columns named
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -7413,12 +7413,12 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>read</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>EquipmentData 0x24-0x58</t>
+          <t>docs/FORMULAS.md 10.1: bases at 0x24-0x38, upgrade rate 0x3C, swing 0x48; named columns in the Equipment sheet</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: random formations of every floor decoded
random formations of every floor decoded, with their chance and rows
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -7369,12 +7369,12 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>located</t>
+          <t>read</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Floor parameter files; records of 22 ints</t>
+          <t>tools/floor_data.py: 1,330 formations on 103 floors with their chance and rows; event battles (bosses) not listed yet</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: table of enchantment sizes generated from the executable
table of enchantment sizes generated from the executable; EXP share
recorded from the player guide
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -7347,12 +7347,12 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>player guide</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>cbattleresult.cpp; an enemy keeps its EXP at offset 8 of its object (0x4f0794); the division is not located</t>
+          <t>docs/FORMULAS.md 6: even share among living members per atwiki page 232; not located in the code (an enemy keeps its EXP at offset 8 of its object, 0x4f0794)</t>
         </is>
       </c>
     </row>
@@ -7501,12 +7501,12 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>read in part</t>
+          <t>read</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Constants after each count of pieces; table to generate</t>
+          <t>docs/generated/ENCHANT_SIZES.md (tools/exe_enchants.py); the rows marked "?" are to be read by hand</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: levers classed by crash risk
levers classed by crash risk, benign changes first as a principle of the
plan
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -11,6 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ModelParts" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regression" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levers" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -7731,4 +7732,1008 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="70" customWidth="1" min="6" max="6"/>
+    <col width="90" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Lever</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>File</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Field</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Condition the build must check</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Evidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Enemy stats: HP, ATK, DEF, INT, RES, DEX, AGI, EXP, gold</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Enemy.pck / EnemyStatusData</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>0x18-0x38</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Benign</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Positive ints; max HP above 0</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Read as plain numbers by the constructor of the enemy (0x4f25f0, 0x4f0794); the record keeps its size</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>L02</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Enemy resistances (eight)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Enemy.pck / EnemyStatusData</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>0x48-0x64</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Benign</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>None for damage; for ailments 100 or more blocks and a negative value adds</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>docs/FORMULAS.md 2.4 and 5b: used as a factor, never as an index</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>L03</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Enemy weight in the order of turns and swing</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Enemy.pck / EnemyStatusData</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>0x44, 0x40</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Benign</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Weight not negative</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>docs/FORMULAS.md 5 and 2.2: a float in a product; the result is capped by the code</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>L04</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Enemy level</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Enemy.pck / EnemyStatusData</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>0x14</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Benign with a condition</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>1 to 99</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Enters the turn order, the critical rate and the EXP shown; values outside the range of the level table are untested</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>L05</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Weights of an enemy AI set</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Enemy.pck / EnemyAIData</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>the 16 bytes after a set</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Benign with a condition</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Each set keeps a weight above 0 on a slot the enemy has an attack in; a byte is 0 to 255</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Runner 0x430f10: a set whose weights add up to 0 picks no attack and the choice loops; a weight on an empty slot does the same</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>L06</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Thresholds of an AI condition (turn number, percent, use count)</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Enemy.pck / EnemyAIData</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>argument bytes</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Benign</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>A byte, 0 to 255; the length of the script does not change</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>docs/FORMULAS.md 9: compared, never used as an index</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>L07</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Adding, removing or reordering AI commands</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Enemy.pck / EnemyAIData</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>whole script</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Structural</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Script must decode with tools/enemy_ai.py and end in 0xFF; every set number used must exist</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>The parser stops the game on an unknown command (0x431949); a set that does not exist is only reported in a message</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>L08</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Speed factors and effect values of an enemy attack</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>EnemyAttackData</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>0x34, 0x44, effect values</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Benign</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Factors above 0</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>docs/FORMULAS.md 5: multiplied into the speed of the enemy</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>L09</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Effect ids, target scope or attribute of an enemy attack</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>EnemyAttackData</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>ids</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Structural</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Only values another vanilla attack already uses in the same position</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>An id with no command class has no handler (CreateCommand 0x47b220)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>L10</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Growth of a class</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>ClassLevelData</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>99 levels of eight ints per row</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Benign</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Positive; HP above 0</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>docs/FORMULAS.md 10: added to the bonuses of the character</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>L11</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>EXP needed per level and skill points per level</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>LvExpSkptData</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>per level</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Benign with a condition</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>EXP strictly increasing with level; skill points not negative</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>The level-up code walks the table level by level (0x448560); skill points are capped at 999 by the code</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Values of a skill per level, TP cost, speed factor</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Technique/Magic/Passive/UniqueSkillData</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>level values</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Benign</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Same sign and scale as vanilla (a fraction stays a fraction); speed factor above 0</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Read as numbers by the command of the effect; the QoL build already rewrites these files byte for byte</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>L13</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>What a skill does: its effect ids, its weapon requirement, its target</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>skill files</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>ids</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Structural</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Only ids and combinations that a vanilla skill of the same kind already uses</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>The user allows it; the risk is an effect the code does not expect in that kind of skill</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>L14</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Stats, upgrade rate and swing of a piece of equipment</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>EquipmentData</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>0x24-0x3C, 0x48</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Benign</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Not negative</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>docs/FORMULAS.md 10.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>L15</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Weapon rank of a weapon and its innate enchantments</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>EquipmentData</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>0x4C, 0x5C-0x6C</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Benign with a condition</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Rank 0 to 11 on weapons and -1 elsewhere; enchantment ids that exist; count equal to the ids listed, at most 4</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>The rank is an index into WeaponRankData; the count is checked by extract_vanilla</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>L16</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Delay of a weapon rank</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>WeaponRankData</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>0x10</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Benign</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Above 0</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>docs/FORMULAS.md 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>L17</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Chance of each random formation of a floor</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Dungeon/stNN/Data.pck floor file</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>formation 0x40</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Benign with a condition</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>The chances of a floor add up to 100, each at least 1</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Vanilla keeps 100 on all 103 floors; how the code walks them is not read</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>L18</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Which enemies a formation holds and their rows</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Dungeon/stNN/Data.pck floor file</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>formation 0x04, 0x34</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Structural</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Enemy ids that exist; no more enemies than the formation had; a lone enemy in front</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Each formation has a layout file (.epd) and the game loads a model per enemy; more enemies than vanilla is untested</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>L19</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Prices, item effects, food, quest rewards</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>ItemData, FoodMenuData, Shop*, QuestRankData</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>values</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Benign</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Not negative</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Already rewritten byte for byte by the QoL build (texts); the values are plain numbers</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>L20</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Texts</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>every pack with strings</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>strings</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Benign</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>The limits of the QoL variant (line widths, voice of the game)</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>The QoL writers rebuild each pack and verify it</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>L21</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Share of each party position when an enemy picks a target</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>executable, table 0x6517a0</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>11 rows of five ints</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Executable</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Every row adds up to more than 0; data of one use, not code</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>docs/FORMULAS.md 9.1; the table is read at one place (0x43dac7)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>L22</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>A constant written inside one instruction (critical factor 1.25, minimum damage 3, Enmity UP 10)</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>executable</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>four bytes of one instruction</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Executable</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Same length; the instruction is the only user</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>docs/FORMULAS.md 4 and 9.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>L23</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>A shared float constant (0.885, 1.35, 2, 4 per piece, 0.02...)</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>executable, .rdata</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Executable</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Not to be changed in place: the same constant serves unrelated formulas. Needs a new constant and a patched instruction</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>For example the float 4 at 0x6d9430 is used by the accuracy, attack, defence and critical enchantments alike</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>L24</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Any change of program logic</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>executable code</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Executable</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Only when no data lever exists, with the case written and the patch verified instruction by instruction</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Decision of the user: only when it can be confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Meaning</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Benign</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>A number inside an existing record of fixed size. The code uses it in arithmetic only. Cannot stop the game.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Benign with a condition</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>The same, but one stated condition must hold or the game can hang or misbehave. The build checks the condition and refuses to install when it fails.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Structural</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Changes what a record contains or how long it is (ids, counts, script commands). Allowed, but each use is justified in balance_changes.xlsx and limited to shapes vanilla already has.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Executable</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>A patch of the program file. Last resort, one change at a time, each verified.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: EXP after a battle read from the code
EXP after a battle read from the code; catching up measured per
checkpoint and added as a requirement
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L134"/>
+  <dimension ref="A1:L135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -6920,6 +6920,63 @@
         </is>
       </c>
       <c r="L134" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>U01</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>Catching up</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>A member who is behind (a new one, a class change, an experiment) takes too long to reach the party; swapping members and trying things must be fluid in every part of the game from about level 20 on</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>Tedium</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>JP community (J37)</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>Random battles a member 10 and 20 levels behind needs to reach the party, on the floor the party is on, at every checkpoint from level 20; against the target</t>
+        </is>
+      </c>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>P12, P13</t>
+        </is>
+      </c>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t>Generated: section "Catching up" of docs/generated/BALANCE_BASELINE.md</t>
+        </is>
+      </c>
+      <c r="L135" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -7348,12 +7405,12 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>player guide</t>
+          <t>read</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>docs/FORMULAS.md 6: even share among living members per atwiki page 232; not located in the code (an enemy keeps its EXP at offset 8 of its object, 0x4f0794)</t>
+          <t>docs/FORMULAS.md 6c, sim/progression.py: factor by level gap (0x450710), even share among the living, doublings (0x445830)</t>
         </is>
       </c>
     </row>
@@ -7740,7 +7797,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -8656,7 +8713,6 @@
           <t>executable code</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
           <t>Executable</t>
@@ -8673,61 +8729,99 @@
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Class</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Meaning</t>
-        </is>
-      </c>
-    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>L25</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>EXP factor by level gap between member and enemy (eight factors)</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>executable, 0x45073e - 0x45080d</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>the address of a float in eight instructions</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Executable</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Each instruction is pointed at another float that already exists in the program; same length, no new data, no change of flow</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>docs/FORMULAS.md 6c. The floats themselves are shared and must not be edited in place</t>
+        </is>
+      </c>
+    </row>
+    <row r="27"/>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Benign</t>
+          <t>Class</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>A number inside an existing record of fixed size. The code uses it in arithmetic only. Cannot stop the game.</t>
+          <t>Meaning</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Benign with a condition</t>
+          <t>Benign</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>The same, but one stated condition must hold or the game can hang or misbehave. The build checks the condition and refuses to install when it fails.</t>
+          <t>A number inside an existing record of fixed size. The code uses it in arithmetic only. Cannot stop the game.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Structural</t>
+          <t>Benign with a condition</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Changes what a record contains or how long it is (ids, counts, script commands). Allowed, but each use is justified in balance_changes.xlsx and limited to shapes vanilla already has.</t>
+          <t>The same, but one stated condition must hold or the game can hang or misbehave. The build checks the condition and refuses to install when it fails.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
+          <t>Structural</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Changes what a record contains or how long it is (ids, counts, script commands). Allowed, but each use is justified in balance_changes.xlsx and limited to shapes vanilla already has.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
           <t>Executable</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B32" t="inlineStr">
         <is>
           <t>A patch of the program file. Last resort, one change at a time, each verified.</t>
         </is>

</xml_diff>

<commit_message>
feat: turn delay roll and its immunity bit read
turn delay roll and its immunity bit read; immunity flags documented as
a benign lever
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -7317,12 +7317,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>read in part</t>
+          <t>read</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>docs/FORMULAS.md 5b: ailments read (0x481ea0); turn delay (effect 54) and turn skipping open</t>
+          <t>docs/FORMULAS.md 5b and 5c: ailments against resistance, immunity flags, turn delay roll; the size of the push back and of a lost turn still open</t>
         </is>
       </c>
     </row>
@@ -7797,7 +7797,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -8766,62 +8766,99 @@
         </is>
       </c>
     </row>
-    <row r="27"/>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Class</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Meaning</t>
-        </is>
-      </c>
-    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>L26</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Immunity of an enemy to each ailment and to turn delay</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Enemy.pck / EnemyStatusData</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>0x3C, bits 2 to 12</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Benign</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Only the decoded bits are changed; the others keep their vanilla value</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>docs/FORMULAS.md 5c: each bit is tested by one ailment before its roll</t>
+        </is>
+      </c>
+    </row>
+    <row r="28"/>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Benign</t>
+          <t>Class</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>A number inside an existing record of fixed size. The code uses it in arithmetic only. Cannot stop the game.</t>
+          <t>Meaning</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Benign with a condition</t>
+          <t>Benign</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>The same, but one stated condition must hold or the game can hang or misbehave. The build checks the condition and refuses to install when it fails.</t>
+          <t>A number inside an existing record of fixed size. The code uses it in arithmetic only. Cannot stop the game.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Structural</t>
+          <t>Benign with a condition</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Changes what a record contains or how long it is (ids, counts, script commands). Allowed, but each use is justified in balance_changes.xlsx and limited to shapes vanilla already has.</t>
+          <t>The same, but one stated condition must hold or the game can hang or misbehave. The build checks the condition and refuses to install when it fails.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
+          <t>Structural</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Changes what a record contains or how long it is (ids, counts, script commands). Allowed, but each use is justified in balance_changes.xlsx and limited to shapes vanilla already has.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
           <t>Executable</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B33" t="inlineStr">
         <is>
           <t>A patch of the program file. Last resort, one change at a time, each verified.</t>
         </is>

</xml_diff>

<commit_message>
feat: level reset bonus read
level reset bonus read; it matches the three crown recipes of the player
guide
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -7797,7 +7797,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:G34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -8803,62 +8803,99 @@
         </is>
       </c>
     </row>
-    <row r="28"/>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Class</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Meaning</t>
-        </is>
-      </c>
-    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>L27</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Bonus of a level reset: points per reset, levels it asks for, the cap of 50</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>executable, 0x4f94f7 - 0x4f9540</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>one byte in each of eleven instructions</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Executable</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Same length; a byte each (points 1 to 127, levels 1 to 98); the cap is a four-byte constant inside its instruction</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>docs/FORMULAS.md 10. No data field holds these; the only data levers on the crown grind are the EXP table and the EXP of enemies</t>
+        </is>
+      </c>
+    </row>
+    <row r="29"/>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Benign</t>
+          <t>Class</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>A number inside an existing record of fixed size. The code uses it in arithmetic only. Cannot stop the game.</t>
+          <t>Meaning</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Benign with a condition</t>
+          <t>Benign</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>The same, but one stated condition must hold or the game can hang or misbehave. The build checks the condition and refuses to install when it fails.</t>
+          <t>A number inside an existing record of fixed size. The code uses it in arithmetic only. Cannot stop the game.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Structural</t>
+          <t>Benign with a condition</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Changes what a record contains or how long it is (ids, counts, script commands). Allowed, but each use is justified in balance_changes.xlsx and limited to shapes vanilla already has.</t>
+          <t>The same, but one stated condition must hold or the game can hang or misbehave. The build checks the condition and refuses to install when it fails.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
+          <t>Structural</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Changes what a record contains or how long it is (ids, counts, script commands). Allowed, but each use is justified in balance_changes.xlsx and limited to shapes vanilla already has.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
           <t>Executable</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B34" t="inlineStr">
         <is>
           <t>A patch of the program file. Last resort, one change at a time, each verified.</t>
         </is>

</xml_diff>

<commit_message>
fix: a floor holds several zones, each with its own formation table
a floor holds several zones, each with its own formation table; the
reader takes them all
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -7432,7 +7432,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>tools/floor_data.py: 1,330 formations on 103 floors with their chance and rows; event battles (bosses) not listed yet</t>
+          <t>tools/floor_data.py: every random formation of every zone of every floor, with its chance and rows; which part of the map a zone covers and the battles placed by events are not decoded</t>
         </is>
       </c>
     </row>
@@ -8446,7 +8446,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Chance of each random formation of a floor</t>
+          <t>Chance of each random formation of a zone</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -8466,12 +8466,12 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>The chances of a floor add up to 100, each at least 1</t>
+          <t>The chances of a zone add up to 100, each at least 1</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Vanilla keeps 100 on all 103 floors; how the code walks them is not read</t>
+          <t>Vanilla keeps 100 in every zone; how the code walks them is not read</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: damage zones read; their factors are data per zone of a floor
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -7537,12 +7537,12 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>read in part</t>
+          <t>read</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Multiply attack A (0x44fbb0)</t>
+          <t>docs/FORMULAS.md 2.5: five factors per zone of a floor, data (tools/floor_data.py); the side of slots 3/5 against 4/6 to confirm</t>
         </is>
       </c>
     </row>
@@ -7797,7 +7797,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G34"/>
+  <dimension ref="A1:G35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -8840,62 +8840,99 @@
         </is>
       </c>
     </row>
-    <row r="29"/>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Class</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Meaning</t>
-        </is>
-      </c>
-    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>L28</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Factors of the damage zones of a floor</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Dungeon/stNN/Data.pck floor file</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>zone 0xB8, five floats</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Benign</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Above 0</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>docs/FORMULAS.md 2.5: copied into the battle and used as factors of attack A</t>
+        </is>
+      </c>
+    </row>
+    <row r="30"/>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Benign</t>
+          <t>Class</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>A number inside an existing record of fixed size. The code uses it in arithmetic only. Cannot stop the game.</t>
+          <t>Meaning</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Benign with a condition</t>
+          <t>Benign</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>The same, but one stated condition must hold or the game can hang or misbehave. The build checks the condition and refuses to install when it fails.</t>
+          <t>A number inside an existing record of fixed size. The code uses it in arithmetic only. Cannot stop the game.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Structural</t>
+          <t>Benign with a condition</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Changes what a record contains or how long it is (ids, counts, script commands). Allowed, but each use is justified in balance_changes.xlsx and limited to shapes vanilla already has.</t>
+          <t>The same, but one stated condition must hold or the game can hang or misbehave. The build checks the condition and refuses to install when it fails.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
+          <t>Structural</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Changes what a record contains or how long it is (ids, counts, script commands). Allowed, but each use is justified in balance_changes.xlsx and limited to shapes vanilla already has.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
           <t>Executable</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B35" t="inlineStr">
         <is>
           <t>A patch of the program file. Last resort, one change at a time, each verified.</t>
         </is>

</xml_diff>

<commit_message>
feat: chant interruption by a critical hit located
chant interruption by a critical hit located (a second roll of 33 in
100)
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -7295,12 +7295,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>read in part</t>
+          <t>read</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Damage against max HP read; the 1 in 3 on a critical hit not located</t>
+          <t>docs/FORMULAS.md 2.6: damage against max HP, and a second roll of 33 in 100 on a critical hit (0x44d238)</t>
         </is>
       </c>
     </row>
@@ -8877,7 +8877,6 @@
         </is>
       </c>
     </row>
-    <row r="30"/>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat: catch-up and crown options compared in the model
catch-up and crown options compared in the model (data only, Double EXP
piece, gap factors)
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -12,6 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ModelParts" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regression" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levers" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CatchUpOptions" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -8940,4 +8941,257 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
+    <col width="120" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Option</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Kind</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Values</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Curve</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Vanilla</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>vanilla</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Nothing changed</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Kept curve</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>curve</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>9,1, 15,0.954, 30,0.80, 50,0.75, 70,0.70, 99,0.60</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Data only. EXP per level of the earlier proposal the user asked to keep, through the five steps he gave (level, share of vanilla)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Steep 2.5%</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>steep</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1.025, 20</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Data only. EXP per level and EXP of enemies both grow 2.5% more per level from level 20: about the steepest that stays exact in the float arithmetic of the game</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Steep 6%</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>steep</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1.06, 20</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Data only, shown to see how far data alone would have to go. It does not fit in the arithmetic of the game</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Double EXP piece</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Data only. The member who is behind wears a piece with enchantment 275</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Gap B</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>gap</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>0.85, 0.9, 1, 1, 2, 4, 8</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Program. Factors by level gap: unchanged down to 4 levels below the enemy, then 2, 4 from 10 below, 8 from 20 below</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Gap D</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>gap</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>0.85, 0.9, 1, 1.5, 3, 5, 10</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Program. 1.5 from 1 level below the enemy, 3 from 5 below, 5 from 10 below, 10 from 20 below</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Kept curve + Gap B</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>gap</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>0.85, 0.9, 1, 1, 2, 4, 8</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>9,1, 15,0.954, 30,0.80, 50,0.75, 70,0.70, 99,0.60</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Program and data: the kept curve with the factors of B</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Kept curve + Gap D</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>gap</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>0.85, 0.9, 1, 1.5, 3, 5, 10</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>9,1, 15,0.954, 30,0.80, 50,0.75, 70,0.70, 99,0.60</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Program and data: the kept curve with the factors of D</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Values of a gap option: the factor for a member 10 or more levels above the enemy, 5 to 9 above, 0 to 4 above, 1 to 4 below, 5 to 9 below, 10 to 19 below, 20 or more below. Each must be a float the program already holds.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: faster catch-up sets and crown rules compared
faster catch-up sets and crown rules compared; decisions recorded
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -13,6 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regression" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levers" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CatchUpOptions" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CrownOptions" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -9050,46 +9051,51 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Steep 6%</t>
+          <t>Double EXP piece</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>steep</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>1.06, 20</t>
+          <t>piece</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Data only, shown to see how far data alone would have to go. It does not fit in the arithmetic of the game</t>
+          <t>Data only. The member who is behind wears a piece with enchantment 275</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Double EXP piece</t>
+          <t>Kept + B</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>piece</t>
+          <t>gap</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>0.85, 0.9, 1, 1, 2, 4, 8</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>9,1, 15,0.954, 30,0.80, 50,0.75, 70,0.70, 99,0.60</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Data only. The member who is behind wears a piece with enchantment 275</t>
+          <t>Kept curve; factors by gap unchanged down to 4 levels below the enemy, then 2, 4 from 10 below, 8 from 20 below</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Gap B</t>
+          <t>Kept + B2</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -9099,19 +9105,24 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>0.85, 0.9, 1, 1, 2, 4, 8</t>
+          <t>0.85, 0.9, 1, 1, 3, 5, 10</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>9,1, 15,0.954, 30,0.80, 50,0.75, 70,0.70, 99,0.60</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Program. Factors by level gap: unchanged down to 4 levels below the enemy, then 2, 4 from 10 below, 8 from 20 below</t>
+          <t>Kept curve; unchanged down to 4 below, then 3, 5 and 10</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Gap D</t>
+          <t>Kept + B3</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -9121,19 +9132,24 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>0.85, 0.9, 1, 1.5, 3, 5, 10</t>
+          <t>0.85, 0.9, 1, 1.25, 2, 4, 8</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>9,1, 15,0.954, 30,0.80, 50,0.75, 70,0.70, 99,0.60</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Program. 1.5 from 1 level below the enemy, 3 from 5 below, 5 from 10 below, 10 from 20 below</t>
+          <t>Kept curve; as B, and 1.25 already from 1 level below the enemy</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Kept curve + Gap B</t>
+          <t>Kept + B4</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -9143,7 +9159,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>0.85, 0.9, 1, 1, 2, 4, 8</t>
+          <t>0.85, 0.9, 1, 1.25, 3, 5, 10</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -9153,14 +9169,14 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Program and data: the kept curve with the factors of B</t>
+          <t>Kept curve; as B2, and 1.25 already from 1 level below the enemy</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Kept curve + Gap D</t>
+          <t>Kept + D</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -9180,7 +9196,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Program and data: the kept curve with the factors of D</t>
+          <t>Kept curve; 1.5 from 1 level below the enemy, then 3, 5 and 10</t>
         </is>
       </c>
     </row>
@@ -9188,6 +9204,155 @@
       <c r="A12" t="inlineStr">
         <is>
           <t>Values of a gap option: the factor for a member 10 or more levels above the enemy, 5 to 9 above, 0 to 4 above, 1 to 4 below, 5 to 9 below, 10 to 19 below, 20 or more below. Each must be a float the program already holds.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="6" customWidth="1" min="3" max="3"/>
+    <col width="90" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Rule</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Steps</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Cap</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Vanilla</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>98:5, 89:4, 79:3, 69:2, 59:1</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>50</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>The rule of the program</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>One more point</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>98:6, 89:5, 79:4, 69:3, 59:2</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>50</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Every step gives one point more (five bytes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Ten levels sooner</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>88:5, 79:4, 69:3, 59:2, 49:1</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>50</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Every step asks for ten levels fewer (five bytes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>88:6, 79:5, 69:4, 59:3, 49:2</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>50</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>One point more and ten levels sooner (ten bytes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Double points</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>98:10, 89:8, 79:6, 69:4, 59:2</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>50</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Every step gives twice the points (five bytes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Steps: levels given up by the reset : points added to every stat. The program compares "levels given up" with a byte and adds a byte.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: critical Magic, magic cap and the recovery commands read
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -7231,12 +7231,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>read in part</t>
+          <t>read</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>docs/FORMULAS.md 3; defence side and caps to finish</t>
+          <t>docs/FORMULAS.md 3: damage, received-damage enchantments, cap, Critical Magic (20 in 100, factor 1.25); one roll before it not identified</t>
         </is>
       </c>
     </row>
@@ -7385,12 +7385,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>read in part</t>
+          <t>read</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>docs/FORMULAS.md 6b: HP heal and its cap read (0x48d730); TP recovery, revival and after-battle recovery open</t>
+          <t>docs/FORMULAS.md 6b and 6d: heal by RES with its cap; revival, HP, TP and percent recovery as a fraction of the maximum</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: fixed battles of every floor and the summons decoded
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -7434,7 +7434,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>tools/floor_data.py: every random formation of every zone of every floor, with its chance and rows; which part of the map a zone covers and the battles placed by events are not decoded</t>
+          <t>tools/floor_data.py: every random formation of every zone and every fixed battle (bosses, quest targets) of every floor; the map cells that carry each zone are not read</t>
         </is>
       </c>
     </row>
@@ -7495,12 +7495,12 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>read in part</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Summon.pck; effects 228-233</t>
+          <t>docs/FORMULAS.md 11, tools/summon_data.py: forms, level, stats, weight, attacks and scripts of the summons; their HP and the dolls (object creation at 0x484150) still open</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: item drops, steal and snack fields of the enemy record
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -7517,12 +7517,12 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>read in part</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>EnemyStatusData 0x68-0xA8</t>
+          <t>tools/enemy_data.py: item drops with their chance, what can be stolen, the snack item; two groups and two ints not identified. Economy only: no battle result depends on them</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: phase 0 closed; what is left for later listed with the work that
phase 0 closed; what is left for later listed with the work that needs
it
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -7324,7 +7324,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>docs/FORMULAS.md 5b and 5c: ailments against resistance, immunity flags, turn delay roll; the size of the push back and of a lost turn still open</t>
+          <t>docs/FORMULAS.md 5b and 5c: ailments against resistance, immunity flags, turn delay (roll, and a swap with the next unit); turns lost to stun and paralysis left for the rows about locks</t>
         </is>
       </c>
     </row>
@@ -7500,7 +7500,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>docs/FORMULAS.md 11, tools/summon_data.py: forms, level, stats, weight, attacks and scripts of the summons; their HP and the dolls (object creation at 0x484150) still open</t>
+          <t>docs/FORMULAS.md 11, tools/summon_data.py: forms, level, stats, weight, attacks and scripts of the summons. A doll is an object built from the tables of its skill (data). Left for the rows about them: the HP of a summon, what each doll does</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: second search of player complaints filed into the register
second search of player complaints filed into the register; choices on
catch-up and crown
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L135"/>
+  <dimension ref="A1:N162"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -437,6 +437,8 @@
     <col width="22" customWidth="1" min="9" max="9"/>
     <col width="30" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
+    <col width="110" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -500,6 +502,16 @@
           <t>Status</t>
         </is>
       </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Worth_It</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Why</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -534,7 +546,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>GameFAQs DT2-2</t>
+          <t>GameFAQs DT2-2; JP search 2 (AGI and action speed forging let a party "massacre" even bosses)</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -638,7 +650,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>GameFAQs DT2-2</t>
+          <t>GameFAQs DT2-2; JP search 2 (what a level changes is unclear and some levels lengthen the chant)</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -690,7 +702,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>GameFAQs DT2-2</t>
+          <t>GameFAQs DT2-2; JP search 2 (some Valkyrie builds are far too strong)</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -742,7 +754,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>GameFAQs DT2-2</t>
+          <t>GameFAQs DT2-2; JP search 2 (classes that restore TP are simply better)</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -1037,6 +1049,11 @@
           <t>Curve</t>
         </is>
       </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>JP search 2 (magic classes dominate and push physical ones aside; classes strong early and useless later)</t>
+        </is>
+      </c>
       <c r="H12" t="inlineStr">
         <is>
           <t>Caster share of party damage is steady across the game, no spike and no cliff</t>
@@ -1378,7 +1395,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>GameFAQs DT2-2</t>
+          <t>GameFAQs DT2-2; JP search 2 (summons act too late to matter in late content)</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1428,6 +1445,11 @@
           <t>Unviable</t>
         </is>
       </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>JP search 2 (skills barely beat a plain attack and she takes massive damage)</t>
+        </is>
+      </c>
       <c r="H20" t="inlineStr">
         <is>
           <t>Berserker inside the damage-dealer band at every checkpoint</t>
@@ -1722,7 +1744,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>GameFAQs DT2-2</t>
+          <t>GameFAQs DT2-2; JP search 2 (nerfed in skills and gear: not worth using in the whole game)</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -1920,7 +1942,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>GameFAQs DT2-2</t>
+          <t>GameFAQs DT2-2; JP search 2</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -2215,6 +2237,11 @@
           <t>Tedium</t>
         </is>
       </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>JP search 2 (says the opposite: forged pieces beat unique ones (row S16))</t>
+        </is>
+      </c>
       <c r="H36" t="inlineStr">
         <is>
           <t>Damage gained per gold spent on forging against other uses of the gold</t>
@@ -2311,7 +2338,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>GameFAQs DT2-2</t>
+          <t>GameFAQs DT2-2; JP search 2 (the grind is unbearable; resets are monotonous)</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -2566,7 +2593,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>JP community</t>
+          <t>JP community; JP search 2</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -2774,7 +2801,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>JP community</t>
+          <t>JP community; JP search 2 (whips lose all advantage as the game goes on)</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -3160,7 +3187,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>JP community</t>
+          <t>JP community; JP search 2 (Joker is far too strong)</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -3551,7 +3578,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>JP community</t>
+          <t>JP community; JP search 2 (the reset bonus was cut from the first game (+2 to 5 became +1 to 5))</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
@@ -3603,7 +3630,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>JP community</t>
+          <t>JP community; JP search 2</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
@@ -6671,6 +6698,11 @@
           <t>Curve</t>
         </is>
       </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>JP search 2</t>
+        </is>
+      </c>
       <c r="H129" t="inlineStr">
         <is>
           <t>Largest swing a zone gives to a fight inside a stated range</t>
@@ -6960,7 +6992,7 @@
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>JP community (J37)</t>
+          <t>JP community (J37); JP search 2 (late members join at a low level; trying another party means levelling it)</t>
         </is>
       </c>
       <c r="H135" t="inlineStr">
@@ -6981,6 +7013,1545 @@
       <c r="L135" t="inlineStr">
         <is>
           <t>open</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>S01</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>JP search 2</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>Pace of common fights</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>A fight against common enemies takes too long for the EXP it gives; the whole game is too long</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>Tedium</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>Turns and EXP of a random battle for an on-level party at every checkpoint, against the pace target</t>
+        </is>
+      </c>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>P03, P12, P13</t>
+        </is>
+      </c>
+      <c r="L136" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="M136" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N136" t="inlineStr">
+        <is>
+          <t>Data: EXP of enemies, EXP per level, HP and defence of common enemies. The factors by level gap chosen for U01 already shorten it</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>S02</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>JP search 2</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>Common enemies too resistant</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>Even normal enemies resist attacks too much</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>Unfair</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>Resistances and defence of the enemies of random formations per band, and the hits an on-level member needs</t>
+        </is>
+      </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>P03, P13</t>
+        </is>
+      </c>
+      <c r="L137" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="M137" t="inlineStr">
+        <is>
+          <t>to decide in the diagnosis</t>
+        </is>
+      </c>
+      <c r="N137" t="inlineStr">
+        <is>
+          <t>Data if true (resistances and DEF are plain numbers). The baseline lists them; the simulator says whether it is so</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>S03</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>JP search 2</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>Enemy passives</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>Enemies trigger their passive skills at a rate players call abnormal</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>Unfair</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>Chance of each enemy passive against the same passive in the hands of the party</t>
+        </is>
+      </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>Where enemy passives are stored (not read)</t>
+        </is>
+      </c>
+      <c r="L138" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="M138" t="inlineStr">
+        <is>
+          <t>to decide in the diagnosis</t>
+        </is>
+      </c>
+      <c r="N138" t="inlineStr">
+        <is>
+          <t>Needs one reading first: whether the chances are data. Worth it only if the rate is above what the party gets</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>S04</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>JP search 2</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Boss</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>Bosses beaten by levels and items</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>The only way through a boss is to out-level it and burn healing items; after the first act every fight is a check of damage per turn</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>Mandatory</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>Win rate of an on-level sensible party per boss, and whether a party built on defence or control wins at all</t>
+        </is>
+      </c>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>P09, P10, P13</t>
+        </is>
+      </c>
+      <c r="L139" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="M139" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N139" t="inlineStr">
+        <is>
+          <t>This is conditions R04, R05 and R08 seen from the player. Levers are data: boss stats, their scripts, immunity bits</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>S05</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>JP search 2</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>Ailments in common fights</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>Freezing, paralysing or putting enemies to sleep wastes a turn: killing them is faster</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>Dead</t>
+        </is>
+      </c>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>Damage and turns saved by an ailment against spending the same turn on damage, per band</t>
+        </is>
+      </c>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>P08, P13</t>
+        </is>
+      </c>
+      <c r="L140" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="M140" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N140" t="inlineStr">
+        <is>
+          <t>Data: chances per level of the skills, immunity bits, resistances. Row F15 holds the same for bosses</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>S06</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>JP search 2</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>Debuffs</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>Lowering accuracy or defence helps only marginally</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>Dead</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>Damage a debuff adds or prevents over its length against the turn it costs</t>
+        </is>
+      </c>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>P03, P05</t>
+        </is>
+      </c>
+      <c r="L141" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="M141" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N141" t="inlineStr">
+        <is>
+          <t>Data: values per level. The formulas already show why: modifiers add up inside a product, so a small one is lost</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>S07</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>JP search 2</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>Witch</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>So dominant through the story that she trivialises it ("a drug")</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>Dominant</t>
+        </is>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>Share of party damage and clear speed with and without her at every story checkpoint</t>
+        </is>
+      </c>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>P04, P13</t>
+        </is>
+      </c>
+      <c r="L142" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="M142" t="inlineStr">
+        <is>
+          <t>to decide in the diagnosis</t>
+        </is>
+      </c>
+      <c r="N142" t="inlineStr">
+        <is>
+          <t>Row J23 says she is useless in postgame and this says she rules the story: both can be true. Data levers either way</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>S08</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>JP search 2</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>Summons of the Soul Summoner</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>A summon acts too late to be useful in late content</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>Unviable</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>Turns before a summon first acts against the enemies of its band; its damage against a party member</t>
+        </is>
+      </c>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>P01, P16</t>
+        </is>
+      </c>
+      <c r="L143" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="M143" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N143" t="inlineStr">
+        <is>
+          <t>Data: the weapon rank each form names sets its weight, and its six factors its stats (tools/summon_data.py)</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>S09</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>JP search 2</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>All stats enchantments</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>Equipment bonuses of "+3 to all stats" do not add up: only one applies</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>Information</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>Read how enchantments 24 to 28 are applied</t>
+        </is>
+      </c>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>P19</t>
+        </is>
+      </c>
+      <c r="L144" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="M144" t="inlineStr">
+        <is>
+          <t>yes, small</t>
+        </is>
+      </c>
+      <c r="N144" t="inlineStr">
+        <is>
+          <t>If the code confirms it, the QoL variant says so on the enchantment; making them add up would be a change of program</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>S10</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>JP search 2</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>Moonlight Purgatory</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>The top damage skill of the Samurai does nothing against some races, so it fails when it matters</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>Trap</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>Share of bosses and late enemies it cannot hurt</t>
+        </is>
+      </c>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>P13</t>
+        </is>
+      </c>
+      <c r="L145" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="M145" t="inlineStr">
+        <is>
+          <t>to decide in the diagnosis</t>
+        </is>
+      </c>
+      <c r="N145" t="inlineStr">
+        <is>
+          <t>Effect 87 limits it to living targets. Removing the limit changes what the skill is (lever L13); its numbers are data</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>S11</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>JP search 2</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>Curve</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>Growth after level 70</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>Characters stop growing around level 70, so later levels do not pay</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>Curve</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>Stats gained per level before and after 70 in the growth tables; EXP per level against it</t>
+        </is>
+      </c>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>P14</t>
+        </is>
+      </c>
+      <c r="L146" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="M146" t="inlineStr">
+        <is>
+          <t>to decide in the diagnosis</t>
+        </is>
+      </c>
+      <c r="N146" t="inlineStr">
+        <is>
+          <t>The growth tables give the same per level before and after 70, so as stated it is not in the data. What rises is the EXP each level costs; the kept curve and the gap factors answer that</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>S12</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>JP search 2</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>Skill points</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>Skill points are too scarce and the reset loop to get more is frustrating</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>Tedium</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>Skill points by level against what a build needs at every checkpoint</t>
+        </is>
+      </c>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>P12</t>
+        </is>
+      </c>
+      <c r="L147" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="M147" t="inlineStr">
+        <is>
+          <t>to decide in the diagnosis</t>
+        </is>
+      </c>
+      <c r="N147" t="inlineStr">
+        <is>
+          <t>Data: skill points per level (lever L11). More points also remove choices, so only if the diagnosis shows builds that cannot work</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>S13</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>JP search 2</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>Encounter rate</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>A battle every few steps, worse at one-way doors, with no way to lower it; puzzles cannot be solved in peace</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>Tedium</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>Steps between battles per zone</t>
+        </is>
+      </c>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>The encounter fields of a zone (not read)</t>
+        </is>
+      </c>
+      <c r="L148" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="M148" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N148" t="inlineStr">
+        <is>
+          <t>Most repeated complaint of the search. Likely data: a zone of a floor holds unread numbers before its formations. To read before phase 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>S14</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>JP search 2</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>Harmful map zones</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>Zones that hurt or weaken are a nuisance, not fun</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>Tedium</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>How much the lowering zones cut damage and how much of a floor they cover</t>
+        </is>
+      </c>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>P18</t>
+        </is>
+      </c>
+      <c r="L149" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="M149" t="inlineStr">
+        <is>
+          <t>yes, small</t>
+        </is>
+      </c>
+      <c r="N149" t="inlineStr">
+        <is>
+          <t>Data: the factors of the zones of each floor (lever L28). Softening the lowering ones is benign; removing zones is not</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>S15</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>JP search 2</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>Traps</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>Gas and damage traps that cannot be avoided are frustrating</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>Tedium</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>Chance and effect of each trap against the skills that answer it</t>
+        </is>
+      </c>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>TrapData (partly read)</t>
+        </is>
+      </c>
+      <c r="L150" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="M150" t="inlineStr">
+        <is>
+          <t>yes, small</t>
+        </is>
+      </c>
+      <c r="N150" t="inlineStr">
+        <is>
+          <t>Data: TrapData holds a rate per trap. Worth a look with the TP economy, not before</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>S16</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>JP search 2</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>Forged pieces against unique ones</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>From the middle of the game a forged piece with chosen enchantments beats the unique ones, so nobody hunts for them</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>Dominant</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>Best forged piece against the unique pieces of the same slot at every band</t>
+        </is>
+      </c>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>P15, P19</t>
+        </is>
+      </c>
+      <c r="L151" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="M151" t="inlineStr">
+        <is>
+          <t>to decide in the diagnosis</t>
+        </is>
+      </c>
+      <c r="N151" t="inlineStr">
+        <is>
+          <t>Row J35 says forging pays little: they speak of different things (stats against enchantments). Data: stats and innate enchantments of unique pieces</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>S17</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>JP search 2</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>Cap of damage reduction</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>The cap of reduced damage went from 50% to 25%, which hurt defensive builds</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>Unviable</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>Survival of a defensive build against bosses with the cap as it is</t>
+        </is>
+      </c>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>P03</t>
+        </is>
+      </c>
+      <c r="L152" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="M152" t="inlineStr">
+        <is>
+          <t>to decide in the diagnosis</t>
+        </is>
+      </c>
+      <c r="N152" t="inlineStr">
+        <is>
+          <t>True in the code (the floor of 0.75), but it is a constant of the program shared with other formulas. Defensive builds have data levers (guard and cover skills, boss damage) that come first; the cap is touched only if they are not enough</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>S18</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>JP search 2</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>Bag of 30 slots</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>The bag is too small and what does not fit is thrown away, rare drops included</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>Tedium</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>Slots against what an expedition yields per band</t>
+        </is>
+      </c>
+      <c r="I153" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="L153" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="M153" t="inlineStr">
+        <is>
+          <t>yes, small</t>
+        </is>
+      </c>
+      <c r="N153" t="inlineStr">
+        <is>
+          <t>Data in part: quest ranks grant slots, and how many is a plain number. The starting 30 is not in the data read so far</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>S19</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>JP search 2</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Curve</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>Early economy</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>At the start everything is expensive and enemies and sales give almost nothing</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>Tedium</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>Gold per battle and per expedition against shop prices over the first bands</t>
+        </is>
+      </c>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>P13</t>
+        </is>
+      </c>
+      <c r="L154" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="M154" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N154" t="inlineStr">
+        <is>
+          <t>Data: gold of enemies and prices are plain numbers; the baseline already lists gold per battle by zone</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>S20</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>JP search 2</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>EXP of quests</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>Quest rewards give negligible EXP</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>Tedium</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>EXP of a quest against the battles it replaces</t>
+        </is>
+      </c>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>Quest reward fields (not read)</t>
+        </is>
+      </c>
+      <c r="L155" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="M155" t="inlineStr">
+        <is>
+          <t>yes, small</t>
+        </is>
+      </c>
+      <c r="N155" t="inlineStr">
+        <is>
+          <t>Likely data. Minor once fights pay better; keep for the pace targets</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>S21</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>JP search 2</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Boss</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>Optional and side-quest bosses</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>Bosses of side quests stand 20 levels or more above the party, and optional ones appear with no warning</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>Curve</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>Level of each fixed battle against the enemies of its floor</t>
+        </is>
+      </c>
+      <c r="I156" t="inlineStr">
+        <is>
+          <t>P13</t>
+        </is>
+      </c>
+      <c r="L156" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="M156" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N156" t="inlineStr">
+        <is>
+          <t>Now measurable: the fixed battles are read. Levers are data (their stats and level); a warning is text</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>S22</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>JP search 2</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Boss</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>Final boss of the main story</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>The last boss of the main story is a wall</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>Curve</t>
+        </is>
+      </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>Win rate of an on-level sensible party against it</t>
+        </is>
+      </c>
+      <c r="I157" t="inlineStr">
+        <is>
+          <t>P13; which fixed battle it is</t>
+        </is>
+      </c>
+      <c r="L157" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="M157" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N157" t="inlineStr">
+        <is>
+          <t>One fight, data levers. To identify among the fixed battles</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>S23</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>JP search 2</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Info</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>Order of actions</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>The order is not shown before choosing an action, so the end of a chant or the next turn is a guess</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>Information</t>
+        </is>
+      </c>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="I158" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="L158" t="inlineStr">
+        <is>
+          <t>out of scope</t>
+        </is>
+      </c>
+      <c r="M158" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="N158" t="inlineStr">
+        <is>
+          <t>Needs new behaviour of the program. The QoL variant already shows the speed and chant of every skill</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>S24</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>JP search 2</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>Functions the game lacks</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>No auto-move, repeat or fast battle; no skip of the sealbook animation; no multi-select; no separate volume for system voices; no difficulty setting; camera too close; pep hard to read; skill levels not shown in the management screen</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>Tedium</t>
+        </is>
+      </c>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="I159" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="L159" t="inlineStr">
+        <is>
+          <t>out of scope</t>
+        </is>
+      </c>
+      <c r="M159" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="N159" t="inlineStr">
+        <is>
+          <t>All are new behaviour of the program: large changes to the executable, which the user ranks last</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>S25</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>JP search 2</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>Design of the content</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>Too many warps and random dungeons, few and small dungeons, little side story, side events with conditions nobody can guess, dark and unvisited cells look alike</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>Tedium</t>
+        </is>
+      </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="I160" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="L160" t="inlineStr">
+        <is>
+          <t>out of scope</t>
+        </is>
+      </c>
+      <c r="M160" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="N160" t="inlineStr">
+        <is>
+          <t>Content and maps, not balance. The conditions of side events could become text of the QoL variant if they are ever read</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>S26</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>JP search 2</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>Reported crashes and bugs</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>A system error on a pit trap of one dungeon, crashes at the blacksmith and in one palace, an item duplication, monsters drawn off screen</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>Unfair</t>
+        </is>
+      </c>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="I161" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="L161" t="inlineStr">
+        <is>
+          <t>out of scope</t>
+        </is>
+      </c>
+      <c r="M161" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="N161" t="inlineStr">
+        <is>
+          <t>Reports from the console versions and early patches; none reproduced here and none is a balance matter</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>S27</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>JP search 2</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>Damage given and taken</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>The ratio of damage dealt to damage received feels wrong</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>Unfair</t>
+        </is>
+      </c>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>none of its own</t>
+        </is>
+      </c>
+      <c r="I162" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="L162" t="inlineStr">
+        <is>
+          <t>merged into R03 and R08</t>
+        </is>
+      </c>
+      <c r="M162" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="N162" t="inlineStr">
+        <is>
+          <t>Too vague to test as stated. It is what conditions R03 and R08 measure fight by fight</t>
         </is>
       </c>
     </row>
@@ -6995,7 +8566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -7107,6 +8678,42 @@
       <c r="B9" t="inlineStr">
         <is>
           <t>No value of the game is typed in this workbook. Vanilla figures are generated into docs/generated/BALANCE_BASELINE.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Status, added 2026-10-05</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>"out of scope": the row is not a claim about balance, or it can only be answered by new behaviour of the program (interface functions, content, crashes). It is kept so that the complaint is on record, with the reason in Why; it does not count against "finished". It is never used for a balance claim that is merely hard to fix. "merged into ...": the row has no test of its own and is measured by the rows named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Worth_It / Why</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>My proposal on whether the row deserves work, for the rows of JP search 2: yes; yes, small; to decide in the diagnosis; no. The user decides.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Source "JP search 2"</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>A search of Japanese player complaints made by another agent for the user on 2026-10-05 (reviews, boards, wikis, blogs). The user asked to take it with a grain of salt: players exaggerate and do not ask for exactly what they need. A complaint is treated at its root and only if it hurts the game; the mod eases the worst of the game without taking its charm; large changes to the program rank last. Entries that already had a row were added to its Also_Raised_By; the rest are rows S01 to S27 with Worth_It and Why. The text file was deleted after filing.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: dolls decoded (9,999 HP, life in turns, hidden action skills)
dolls decoded (9,999 HP, life in turns, hidden action skills); Doll
Master row added to the register
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N162"/>
+  <dimension ref="A1:N163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1413,6 +1413,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>As written it does not match the code: a doll is born with 9,999 HP and ends by its count of turns (docs/FORMULAS.md 11.1). The complaint about summons acting late is row S08; the Doll Master line is row U02</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -8552,6 +8557,68 @@
       <c r="N162" t="inlineStr">
         <is>
           <t>Too vague to test as stated. It is what conditions R03 and R08 measure fight by fight</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>U02</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>Doll Master line</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>The class is far behind the others (user, 2026-10-05: "esa clase esta muy rezagada")</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>Unviable</t>
+        </is>
+      </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>JP community (J18); GameFAQs DT2-2 (F71, F77)</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr">
+        <is>
+          <t>Damage, healing and control of a Doll Master with her dolls per turn and per TP against the band of her checkpoint, dolls counted over their whole life</t>
+        </is>
+      </c>
+      <c r="I163" t="inlineStr">
+        <is>
+          <t>P03, P04, P16</t>
+        </is>
+      </c>
+      <c r="L163" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="M163" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N163" t="inlineStr">
+        <is>
+          <t>All data and benign: the hidden action skills (power, chances, heal and spell power), the turns a doll lasts, TP cost and speed of the cast, Doll Mastery, the growth row of the class</t>
         </is>
       </c>
     </row>
@@ -9102,12 +9169,12 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>read in part</t>
+          <t>read</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>docs/FORMULAS.md 11, tools/summon_data.py: forms, level, stats, weight, attacks and scripts of the summons. A doll is an object built from the tables of its skill (data). Left for the rows about them: the HP of a summon, what each doll does</t>
+          <t>docs/FORMULAS.md 11 and 11.1; tools/summon_data.py, tools/doll_data.py: summons (forms, level, stats, weight, attacks, scripts) and dolls (9,999 HP, life in turns, hidden action skills, modifiers). Open: the HP of a summon, the class and level behind the stats of a doll</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: effect rules sheet started (hit counts, hit application)
effect rules sheet started (hit counts, hit application); digest and
context tools
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -14,8 +14,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levers" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CatchUpOptions" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CrownOptions" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EffectNotes" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Extraction" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Extraction" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EffectRules" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EffectCoverage" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
@@ -9054,15 +9054,15 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr"/>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>0x42196e, 0x421a83, 0x422d3b</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>applying a hit</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -9680,15 +9680,15 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr"/>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>0x4226c4</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>applying a hit</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -9707,15 +9707,15 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr"/>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>0x42155a, 0x4215af, 0x422eda</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>applying a hit</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -9734,15 +9734,15 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr"/>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>0x421604, 0x421659, 0x422fc7</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>applying a hit</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -9953,15 +9953,15 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr"/>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>0x417db0</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>hits of an action</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -9980,15 +9980,15 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr"/>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>0x417df3</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>hits of an action</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -10007,15 +10007,15 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr"/>
-      <c r="H50" t="inlineStr">
-        <is>
-          <t>0x417e0c</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>hits of an action</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -10034,15 +10034,15 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr"/>
-      <c r="H51" t="inlineStr">
-        <is>
-          <t>0x417e25</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>hits of an action</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -10088,15 +10088,15 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr"/>
-      <c r="H53" t="inlineStr">
-        <is>
-          <t>0x417e93</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>hits of an action</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -10115,15 +10115,15 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr"/>
-      <c r="H54" t="inlineStr">
-        <is>
-          <t>0x417ed0</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>hits of an action</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -10142,15 +10142,15 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr"/>
-      <c r="H55" t="inlineStr">
-        <is>
-          <t>0x417f0e</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>hits of an action</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -10169,15 +10169,15 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr"/>
-      <c r="H56" t="inlineStr">
-        <is>
-          <t>0x417f4e</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>hits of an action</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -10196,15 +10196,15 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F57" t="inlineStr"/>
-      <c r="H57" t="inlineStr">
-        <is>
-          <t>0x417f67</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>hits of an action</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -10223,15 +10223,15 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F58" t="inlineStr"/>
-      <c r="H58" t="inlineStr">
-        <is>
-          <t>0x417f80</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>hits of an action</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -10250,15 +10250,15 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F59" t="inlineStr"/>
-      <c r="H59" t="inlineStr">
-        <is>
-          <t>0x417fbe</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>hits of an action</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -10596,20 +10596,20 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F71" t="inlineStr"/>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>5b ailments</t>
+        </is>
+      </c>
       <c r="G71" t="inlineStr">
         <is>
           <t>0x481ea0</t>
         </is>
       </c>
-      <c r="H71" t="inlineStr">
-        <is>
-          <t>0x42126b, 0x4fb572</t>
-        </is>
-      </c>
+      <c r="H71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -10628,20 +10628,20 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F72" t="inlineStr"/>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>5b ailments</t>
+        </is>
+      </c>
       <c r="G72" t="inlineStr">
         <is>
           <t>0x4822c0</t>
         </is>
       </c>
-      <c r="H72" t="inlineStr">
-        <is>
-          <t>0x42135e, 0x4fb582, 0x512384</t>
-        </is>
-      </c>
+      <c r="H72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -10660,20 +10660,20 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F73" t="inlineStr"/>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>5b ailments</t>
+        </is>
+      </c>
       <c r="G73" t="inlineStr">
         <is>
           <t>0x482530</t>
         </is>
       </c>
-      <c r="H73" t="inlineStr">
-        <is>
-          <t>0x4213af, 0x4fb592, 0x51210b</t>
-        </is>
-      </c>
+      <c r="H73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -10692,20 +10692,20 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F74" t="inlineStr"/>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>5b ailments</t>
+        </is>
+      </c>
       <c r="G74" t="inlineStr">
         <is>
           <t>0x4827a0</t>
         </is>
       </c>
-      <c r="H74" t="inlineStr">
-        <is>
-          <t>0x4212bc, 0x4fb5a2</t>
-        </is>
-      </c>
+      <c r="H74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -10724,20 +10724,20 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F75" t="inlineStr"/>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>5b ailments</t>
+        </is>
+      </c>
       <c r="G75" t="inlineStr">
         <is>
           <t>0x482a10</t>
         </is>
       </c>
-      <c r="H75" t="inlineStr">
-        <is>
-          <t>0x42130d, 0x4fb5b2, 0x51294d</t>
-        </is>
-      </c>
+      <c r="H75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -10756,20 +10756,20 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F76" t="inlineStr"/>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>5b ailments</t>
+        </is>
+      </c>
       <c r="G76" t="inlineStr">
         <is>
           <t>0x482c80</t>
         </is>
       </c>
-      <c r="H76" t="inlineStr">
-        <is>
-          <t>0x421400</t>
-        </is>
-      </c>
+      <c r="H76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -10788,12 +10788,12 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>located</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>2 physical attack</t>
+          <t>2 physical attack, 5b ailments</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -10801,11 +10801,7 @@
           <t>0x482e40</t>
         </is>
       </c>
-      <c r="H77" t="inlineStr">
-        <is>
-          <t>0x4214a2, 0x4214f3, 0x423617</t>
-        </is>
-      </c>
+      <c r="H77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -10824,20 +10820,20 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F78" t="inlineStr"/>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>5b ailments</t>
+        </is>
+      </c>
       <c r="G78" t="inlineStr">
         <is>
           <t>0x4831f0</t>
         </is>
       </c>
-      <c r="H78" t="inlineStr">
-        <is>
-          <t>0x421451, 0x451dbd, 0x4f9ace, 0x4f9b27, 0x4fb5c3, 0x4fb603, 0x51071b</t>
-        </is>
-      </c>
+      <c r="H78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -10888,20 +10884,20 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F80" t="inlineStr"/>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>5b ailments</t>
+        </is>
+      </c>
       <c r="G80" t="inlineStr">
         <is>
           <t>0x4835d0</t>
         </is>
       </c>
-      <c r="H80" t="inlineStr">
-        <is>
-          <t>0x4216ae, 0x422933, 0x4244dc, 0x4fb642</t>
-        </is>
-      </c>
+      <c r="H80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -11899,20 +11895,20 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F117" t="inlineStr"/>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>hits of an action</t>
+        </is>
+      </c>
       <c r="G117" t="inlineStr">
         <is>
           <t>0x4869c0</t>
         </is>
       </c>
-      <c r="H117" t="inlineStr">
-        <is>
-          <t>0x417ffe</t>
-        </is>
-      </c>
+      <c r="H117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="n">
@@ -11958,15 +11954,15 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F119" t="inlineStr"/>
-      <c r="H119" t="inlineStr">
-        <is>
-          <t>0x4223d4</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>applying a hit</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="n">
@@ -12680,15 +12676,15 @@
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F145" t="inlineStr"/>
-      <c r="H145" t="inlineStr">
-        <is>
-          <t>0x417dc4, 0x417e36, 0x417ea4, 0x417ee1, 0x417f1f, 0x417f91, 0x417fcf</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>hits of an action</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="n">
@@ -13404,15 +13400,15 @@
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F173" t="inlineStr"/>
-      <c r="H173" t="inlineStr">
-        <is>
-          <t>0x422596</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>applying a hit</t>
+        </is>
+      </c>
+      <c r="H173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="n">
@@ -13431,15 +13427,15 @@
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F174" t="inlineStr"/>
-      <c r="H174" t="inlineStr">
-        <is>
-          <t>0x41808c</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>hits of an action</t>
+        </is>
+      </c>
+      <c r="H174" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" t="n">
@@ -13458,15 +13454,15 @@
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F175" t="inlineStr"/>
-      <c r="H175" t="inlineStr">
-        <is>
-          <t>0x418045</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>hits of an action</t>
+        </is>
+      </c>
+      <c r="H175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" t="n">
@@ -14686,15 +14682,15 @@
       </c>
       <c r="E223" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F223" t="inlineStr"/>
-      <c r="H223" t="inlineStr">
-        <is>
-          <t>0x422207</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F223" t="inlineStr">
+        <is>
+          <t>applying a hit</t>
+        </is>
+      </c>
+      <c r="H223" t="inlineStr"/>
     </row>
     <row r="224">
       <c r="A224" t="n">
@@ -14813,15 +14809,15 @@
       </c>
       <c r="E228" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F228" t="inlineStr"/>
-      <c r="H228" t="inlineStr">
-        <is>
-          <t>0x421dc4</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F228" t="inlineStr">
+        <is>
+          <t>applying a hit</t>
+        </is>
+      </c>
+      <c r="H228" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" t="n">
@@ -17996,253 +17992,442 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="70" customWidth="1" min="3" max="3"/>
+    <col width="52" customWidth="1" min="1" max="1"/>
+    <col width="70" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="110" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Effect_ID</t>
+          <t>Item</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Section</t>
+          <t>What the simulator needs from it</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>How it was read</t>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Where / what is missing</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>0</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Effects of skills and enemy attacks</t>
+        </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2 physical attack</t>
+          <t>What each effect does, with its rolls</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>The hit itself: the attack functions run for it</t>
+          <t>in progress</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Measured by tools/exe_effects.py: docs/generated/EFFECT_COVERAGE.md and the sheet EffectCoverage. Closed when no effect a skill uses is "located" or "not found"</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
-        <v>125</v>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Applying an action (0x4200e0)</t>
+        </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>4 critical hits</t>
+          <t>Order of a hit: accuracy, damage, absorption, ailments, what a kill triggers</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>0x44f477: +5 per earlier hit</t>
+          <t>not read</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Handles 29 effects; the largest single block</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
-        <v>264</v>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Number of hits and targets (0x417cd0)</t>
+        </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2 physical attack</t>
+          <t>Multi-hit and multi-target skills</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>0x44cfad: divides the interruption rate</t>
+          <t>not read</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Handles effects 89 to 100, 178, 210, 251, 252</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
-        <v>301</v>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>States of a unit over turns (0x4fbc40, 0x4fb100, 0x423560)</t>
+        </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>3 magic attack</t>
+          <t>What poison, sleep, paralysis and the rest do each turn and how long they last; regeneration</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>0x44edbe: the id is compared in a register (Critical Magic)</t>
+          <t>not read</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Only the roll that applies each ailment is read</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
-        <v>296</v>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Passive and unique skills</t>
+        </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>3 magic attack</t>
+          <t>Chance and effect of Auto-Guard, Counter, Parry, Cover, Double Attack and the rest</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>0x44f0ce: damage cap</t>
+          <t>not read</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>The debug messages name each roll; the code of none is read</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
-        <v>295</v>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Buff rules</t>
+        </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>6b healing</t>
+          <t>How long a buff lasts, whether two stack, how dispel removes them</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>0x48c5c7: heal cap</t>
+          <t>not read</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Formulas add the buffs present; where they come from and go is not read</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="n">
-        <v>146</v>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Skills of each class</t>
+        </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>11.1 dolls</t>
+          <t>Which class learns which skill, at what cost</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>0x484330: number of units created</t>
+          <t>not read</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>ClassData is ten unnamed ints; the skill files hold a group field not decoded</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="n">
-        <v>147</v>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Characters</t>
+        </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>11.1 dolls</t>
+          <t>Base class and unique skill of each girl</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>0x4843c9: turns a doll lasts</t>
+          <t>not read</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>CharacterData holds two ints per character</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="n">
-        <v>228</v>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Mercenaries</t>
+        </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>11.1 dolls</t>
+          <t>Stats, attacks and behaviour of the hired allies</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Doll: the id is stored in the doll and compared (0x44bb1c)</t>
+          <t>not read</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Their table (program global 0x738a04) is not located in the data files yet</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="n">
-        <v>229</v>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Pep</t>
+        </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>11.1 dolls</t>
+          <t>What pep changes in battle</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>As 228</t>
+          <t>not read</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>The messages list what raises and lowers it; its effect on stats is not read</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="n">
-        <v>230</v>
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Party and joint skills</t>
+        </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>11.1 dolls</t>
+          <t>What each does in numbers</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>As 228</t>
+          <t>partly</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>The QoL variant decoded their texts and fields; their effects in battle are not tied to code</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="n">
-        <v>231</v>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Items and meals in battle</t>
+        </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>11.1 dolls</t>
+          <t>Healing items, attack items, meals</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>As 228</t>
+          <t>partly</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Effects named by the QoL work; 21 items still undecoded</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="n">
-        <v>232</v>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Encounter rate</t>
+        </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>11.1 dolls</t>
+          <t>Steps between battles per zone</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>As 228</t>
+          <t>not read</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Row S13: the most repeated complaint. Unread numbers at the start of each zone record</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="n">
-        <v>233</v>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Enemy passives</t>
+        </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>11.1 dolls</t>
+          <t>Passive skills enemies carry</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>As 228</t>
+          <t>not read</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Row S03. Where they are stored is not known</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="n">
-        <v>286</v>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Enemy attack record</t>
+        </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>11.1 dolls</t>
+          <t>Every field</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>0x44b4fd, 0x44dda8, 0x48d7a1: Doll Mastery</t>
+          <t>partly</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Three fields unnamed (0x38, 0x3C, 0x40) and the tail of each effect</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Summons</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>HP</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>partly</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Everything else read (docs/FORMULAS.md 11)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Dolls</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Class and level behind their stats; what removes one early</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>partly</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>docs/FORMULAS.md 11.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Formulas of a hit, turn order, targets, EXP, resets, zones, healing</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>docs/FORMULAS.md; open details in its section 8</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Enemies, formations, fixed battles, class growth, equipment stats, enchantment sizes</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>tools/ and docs/generated/</t>
         </is>
       </c>
     </row>
@@ -18257,442 +18442,899 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="52" customWidth="1" min="1" max="1"/>
-    <col width="70" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="110" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="120" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Item</t>
+          <t>Effect_ID</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>What the simulator needs from it</t>
+          <t>Section</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>State</t>
+          <t>Rule</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Where / what is missing</t>
+          <t>Read_At</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Effects of skills and enemy attacks</t>
-        </is>
+      <c r="A2" t="n">
+        <v>0</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>What each effect does, with its rolls</t>
+          <t>2 physical attack</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>in progress</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Measured by tools/exe_effects.py: docs/generated/EFFECT_COVERAGE.md and the sheet EffectCoverage. Closed when no effect a skill uses is "located" or "not found"</t>
+          <t>The hit itself: the attack functions run for it</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Applying an action (0x4200e0)</t>
-        </is>
+      <c r="A3" t="n">
+        <v>125</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Order of a hit: accuracy, damage, absorption, ailments, what a kill triggers</t>
+          <t>4 critical hits</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>not read</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Handles 29 effects; the largest single block</t>
+          <t>0x44f477: +5 per earlier hit</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Number of hits and targets (0x417cd0)</t>
-        </is>
+      <c r="A4" t="n">
+        <v>264</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Multi-hit and multi-target skills</t>
+          <t>2 physical attack</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>not read</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Handles effects 89 to 100, 178, 210, 251, 252</t>
+          <t>0x44cfad: divides the interruption rate</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>States of a unit over turns (0x4fbc40, 0x4fb100, 0x423560)</t>
-        </is>
+      <c r="A5" t="n">
+        <v>301</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>What poison, sleep, paralysis and the rest do each turn and how long they last; regeneration</t>
+          <t>3 magic attack</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>not read</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Only the roll that applies each ailment is read</t>
+          <t>0x44edbe: the id is compared in a register (Critical Magic)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Passive and unique skills</t>
-        </is>
+      <c r="A6" t="n">
+        <v>296</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Chance and effect of Auto-Guard, Counter, Parry, Cover, Double Attack and the rest</t>
+          <t>3 magic attack</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>not read</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>The debug messages name each roll; the code of none is read</t>
+          <t>0x44f0ce: damage cap</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Buff rules</t>
-        </is>
+      <c r="A7" t="n">
+        <v>295</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>How long a buff lasts, whether two stack, how dispel removes them</t>
+          <t>6b healing</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>not read</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Formulas add the buffs present; where they come from and go is not read</t>
+          <t>0x48c5c7: heal cap</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Skills of each class</t>
-        </is>
+      <c r="A8" t="n">
+        <v>146</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Which class learns which skill, at what cost</t>
+          <t>11.1 dolls</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>not read</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>ClassData is ten unnamed ints; the skill files hold a group field not decoded</t>
+          <t>0x484330: number of units created</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Characters</t>
-        </is>
+      <c r="A9" t="n">
+        <v>147</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Base class and unique skill of each girl</t>
+          <t>11.1 dolls</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>not read</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>CharacterData holds two ints per character</t>
+          <t>0x4843c9: turns a doll lasts</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Mercenaries</t>
-        </is>
+      <c r="A10" t="n">
+        <v>228</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Stats, attacks and behaviour of the hired allies</t>
+          <t>11.1 dolls</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>not read</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Their table (program global 0x738a04) is not located in the data files yet</t>
+          <t>Doll: the id is stored in the doll and compared (0x44bb1c)</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Pep</t>
-        </is>
+      <c r="A11" t="n">
+        <v>229</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>What pep changes in battle</t>
+          <t>11.1 dolls</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>not read</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>The messages list what raises and lowers it; its effect on stats is not read</t>
+          <t>As 228</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Party and joint skills</t>
-        </is>
+      <c r="A12" t="n">
+        <v>230</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>What each does in numbers</t>
+          <t>11.1 dolls</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>partly</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>The QoL variant decoded their texts and fields; their effects in battle are not tied to code</t>
+          <t>As 228</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Items and meals in battle</t>
-        </is>
+      <c r="A13" t="n">
+        <v>231</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Healing items, attack items, meals</t>
+          <t>11.1 dolls</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>partly</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Effects named by the QoL work; 21 items still undecoded</t>
+          <t>As 228</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Encounter rate</t>
-        </is>
+      <c r="A14" t="n">
+        <v>232</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Steps between battles per zone</t>
+          <t>11.1 dolls</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>not read</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Row S13: the most repeated complaint. Unread numbers at the start of each zone record</t>
+          <t>As 228</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Enemy passives</t>
-        </is>
+      <c r="A15" t="n">
+        <v>233</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Passive skills enemies carry</t>
+          <t>11.1 dolls</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>not read</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Row S03. Where they are stored is not known</t>
+          <t>As 228</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Enemy attack record</t>
-        </is>
+      <c r="A16" t="n">
+        <v>286</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Every field</t>
+          <t>11.1 dolls</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>partly</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Three fields unnamed (0x38, 0x3C, 0x40) and the tail of each effect</t>
+          <t>0x44b4fd, 0x44dda8, 0x48d7a1: Doll Mastery</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Summons</t>
-        </is>
+      <c r="A17" t="n">
+        <v>89</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>hits of an action</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>partly</t>
+          <t>Number of hits: 2 plus a weighted pick among [0, 1, 2, 3] with weights [25, 25, 25, 25] ([15, 20, 35, 30] while effect 210 is in the action)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Everything else read (docs/FORMULAS.md 11)</t>
+          <t>0x417db0</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Dolls</t>
-        </is>
+      <c r="A18" t="n">
+        <v>90</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Class and level behind their stats; what removes one early</t>
+          <t>hits of an action</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>partly</t>
+          <t>Number of hits: 3</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>docs/FORMULAS.md 11.1</t>
+          <t>0x417e04</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Formulas of a hit, turn order, targets, EXP, resets, zones, healing</t>
+      <c r="A19" t="n">
+        <v>91</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>hits of an action</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>read</t>
+          <t>Number of hits: 8</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>docs/FORMULAS.md; open details in its section 8</t>
+          <t>0x417e1d</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Enemies, formations, fixed battles, class growth, equipment stats, enchantment sizes</t>
+      <c r="A20" t="n">
+        <v>92</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>hits of an action</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>read</t>
+          <t>Number of hits: 2 plus a weighted pick among [0, 1, 2] with weights [15, 50, 35] ([0, 50, 50] while effect 210 is in the action)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>tools/ and docs/generated/</t>
+          <t>0x417e25</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>94</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>hits of an action</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Number of hits: 0 plus a weighted pick among [0, 1, 2, 3, 4] with weights [10, 15, 30, 25, 20] ([0, 15, 25, 30, 30] while effect 210 is in the action)</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>0x417e93</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>95</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>hits of an action</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Number of hits: 1 plus a weighted pick among [0, 1, 2, 3, 4] with weights [10, 15, 30, 25, 20] ([0, 15, 30, 25, 30] while effect 210 is in the action)</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>0x417ed0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>96</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>hits of an action</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Number of hits: 3 plus a weighted pick among [0, 1, 2] with weights [20, 50, 30] ([0, 50, 50] while effect 210 is in the action)</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>0x417f0e</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>97</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>hits of an action</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Number of hits: 2</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>0x417f4e</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>98</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>hits of an action</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Number of hits: 7</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>0x417f67</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>99</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>hits of an action</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Number of hits: 1 plus a weighted pick among [0, 1, 2] with weights [20, 50, 30] ([0, 50, 50] while effect 210 is in the action)</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>0x417f80</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>100</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>hits of an action</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Number of hits: 4 plus a weighted pick among [0, 1, 2, 3] with weights [20, 20, 30, 30] ([0, 20, 30, 50] while effect 210 is in the action)</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>0x417fbe</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>178</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>hits of an action</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Adds int(value) + 1 hits to the action</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>0x417ffe</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>210</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>hits of an action</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>While it is in the action, the weighted picks of the multi-hit effects use their second table (never the lowest count)</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>0x417dc4</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>252</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>hits of an action</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Plain attack with no multi-hit effect: a roll below 100 under value * 100 adds 3 hits; tried before Double Attack</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>0x418045</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>251</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>hits of an action</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Plain attack with no multi-hit effect, when Triple Attack did not fire: a roll below 100 under value * 100 adds 2 hits</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>0x41808c</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>74</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>applying a hit</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>After the hit lands: a roll below 100 under value * 100 removes the buffs of the target (debug message "strengthening removed")</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>0x4226c4</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>180</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>applying a hit</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>While the target has it, a physical hit deals nothing; each hit so blocked rolls below 100 under value * 100 and on success the barrier ends (debug message "physical barrier B"). The Effects sheet calls it Parry</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>0x4223d4</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>250</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>applying a hit</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>When the target has it: a roll below 100 under value * 100 answers the hit with a counter (debug message "Counter")</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>0x42259f</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>310</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>applying a hit</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>When the target has it: a roll below 100 under value * 100 (debug message of the passive "Pretend")</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>0x421dcd</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>305</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>applying a hit</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>When the target has it: a roll below 100 under value * 100 (debug message of the passive "Knock Down")</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>0x422210</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>25</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>applying a hit</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>The action deals no damage: the damage step is skipped and only its other effects apply</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>0x42196e</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>75</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>applying a hit</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Absorbs HP from the damage dealt. A plain attack gets it from a piece with enchantment 161 (value 0.5) or 162 (value 0.15)</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>0x42155a, 0x422eda</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>76</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>applying a hit</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Absorbs TP. A plain attack gets it from a piece with enchantment 163 (value 0.2) or 164 (value 0.05)</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>0x421604, 0x422fc7</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>113</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>5b ailments</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Its own roll: docs/FORMULAS.md 5b. A plain attack with a piece of enchantment 153 tries it at 0.18</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>0x421261 - 0x4216d2</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>116</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>5b ailments</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Its own roll: docs/FORMULAS.md 5b. A plain attack with a piece of enchantment 154 tries it at 0.15</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>0x421261 - 0x4216d2</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>117</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>5b ailments</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Its own roll: docs/FORMULAS.md 5b. A plain attack with a piece of enchantment 155 tries it at 0.18</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>0x421261 - 0x4216d2</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>114</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>5b ailments</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Its own roll: docs/FORMULAS.md 5b. A plain attack with a piece of enchantment 156 tries it at 0.18</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>0x421261 - 0x4216d2</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>115</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>5b ailments</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Its own roll: docs/FORMULAS.md 5b. A plain attack with a piece of enchantment 157 tries it at 0.15</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>0x421261 - 0x4216d2</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>118</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>5b ailments</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Its own roll: docs/FORMULAS.md 5b. A plain attack with a piece of enchantment 158 tries it at 0.12</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>0x421261 - 0x4216d2</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>120</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>5b ailments</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Its own roll: docs/FORMULAS.md 5b. A plain attack with a piece of enchantment 159 tries it at 0.1</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>0x421261 - 0x4216d2</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>122</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>5b ailments</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Its own roll: docs/FORMULAS.md 5b. A plain attack with a piece of enchantment 165 tries it at 0.12</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>0x421261 - 0x4216d2</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>119</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>5b ailments</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Its own roll: docs/FORMULAS.md 5b (earth resistance). A plain attack tries it at 0.07 with a piece of enchantment 160 and at 0.75 with one of 197</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>0x421498, 0x4214e9</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: phase 4 reworded: solve every problem in full
phase 4 reworded: solve every problem in full, keep the essence,
closeness to vanilla only as a tie-break
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -8706,7 +8706,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -8764,7 +8763,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -8786,8 +8784,6 @@
           <t>not found</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -8809,8 +8805,6 @@
           <t>not found</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -8868,13 +8862,11 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
           <t>0x47fc30</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -8896,13 +8888,11 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
           <t>0x47fd00</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -8955,13 +8945,11 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
           <t>0x47fde0</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -8983,8 +8971,6 @@
           <t>read</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -9006,13 +8992,11 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
           <t>0x47ffc0</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -9034,8 +9018,6 @@
           <t>not found</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -9062,7 +9044,6 @@
           <t>applying a hit</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -9089,7 +9070,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -9111,8 +9091,6 @@
           <t>read</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -9139,7 +9117,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -9166,7 +9143,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -9193,7 +9169,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -9220,7 +9195,6 @@
           <t>4 critical hits</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -9247,7 +9221,6 @@
           <t>4 critical hits</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -9274,7 +9247,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -9296,13 +9268,11 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
           <t>0x48bd60</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -9329,7 +9299,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -9356,7 +9325,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -9414,7 +9382,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -9436,7 +9403,6 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr"/>
       <c r="H29" t="inlineStr">
         <is>
           <t>0x42310f, 0x44fe2c, 0x44ff20</t>
@@ -9463,7 +9429,6 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr"/>
       <c r="H30" t="inlineStr">
         <is>
           <t>0x423120, 0x44fe55, 0x45036a</t>
@@ -9490,7 +9455,6 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr"/>
       <c r="H31" t="inlineStr">
         <is>
           <t>0x44ff50</t>
@@ -9517,8 +9481,6 @@
           <t>read</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr"/>
-      <c r="H32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -9576,7 +9538,6 @@
           <t>4 critical hits</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -9603,7 +9564,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -9661,7 +9621,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -9688,7 +9647,6 @@
           <t>applying a hit</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -9715,7 +9673,6 @@
           <t>applying a hit</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -9742,7 +9699,6 @@
           <t>applying a hit</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -9764,13 +9720,11 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr">
         <is>
           <t>0x481060</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -9792,8 +9746,6 @@
           <t>not found</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr"/>
-      <c r="H42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -9815,13 +9767,11 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr">
         <is>
           <t>0x481160</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -9843,7 +9793,6 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr">
         <is>
           <t>0x4813a0</t>
@@ -9880,7 +9829,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -9907,7 +9855,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -9934,7 +9881,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -9961,7 +9907,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -9988,7 +9933,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -10015,7 +9959,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -10042,7 +9985,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -10064,7 +10006,6 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F52" t="inlineStr"/>
       <c r="H52" t="inlineStr">
         <is>
           <t>0x417e65</t>
@@ -10096,7 +10037,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -10123,7 +10063,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -10150,7 +10089,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -10177,7 +10115,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -10204,7 +10141,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -10231,7 +10167,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -10258,7 +10193,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -10280,8 +10214,6 @@
           <t>read</t>
         </is>
       </c>
-      <c r="F60" t="inlineStr"/>
-      <c r="H60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -10303,7 +10235,6 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F61" t="inlineStr"/>
       <c r="H61" t="inlineStr">
         <is>
           <t>0x41faaf</t>
@@ -10330,7 +10261,6 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F62" t="inlineStr"/>
       <c r="G62" t="inlineStr">
         <is>
           <t>0x4817c0</t>
@@ -10362,7 +10292,6 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr">
         <is>
           <t>0x481890</t>
@@ -10394,7 +10323,6 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F64" t="inlineStr"/>
       <c r="G64" t="inlineStr">
         <is>
           <t>0x481950</t>
@@ -10426,7 +10354,6 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr">
         <is>
           <t>0x481a20</t>
@@ -10458,7 +10385,6 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr">
         <is>
           <t>0x47fde0</t>
@@ -10490,13 +10416,11 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F67" t="inlineStr"/>
       <c r="G67" t="inlineStr">
         <is>
           <t>0x481d80</t>
         </is>
       </c>
-      <c r="H67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -10523,7 +10447,6 @@
           <t>4 critical hits</t>
         </is>
       </c>
-      <c r="H68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -10550,7 +10473,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -10572,7 +10494,6 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F70" t="inlineStr"/>
       <c r="H70" t="inlineStr">
         <is>
           <t>0x42e1ba, 0x43b08e, 0x43b183</t>
@@ -10609,7 +10530,6 @@
           <t>0x481ea0</t>
         </is>
       </c>
-      <c r="H71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -10641,7 +10561,6 @@
           <t>0x4822c0</t>
         </is>
       </c>
-      <c r="H72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -10673,7 +10592,6 @@
           <t>0x482530</t>
         </is>
       </c>
-      <c r="H73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -10705,7 +10623,6 @@
           <t>0x4827a0</t>
         </is>
       </c>
-      <c r="H74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -10737,7 +10654,6 @@
           <t>0x482a10</t>
         </is>
       </c>
-      <c r="H75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -10769,7 +10685,6 @@
           <t>0x482c80</t>
         </is>
       </c>
-      <c r="H76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -10801,7 +10716,6 @@
           <t>0x482e40</t>
         </is>
       </c>
-      <c r="H77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -10833,7 +10747,6 @@
           <t>0x4831f0</t>
         </is>
       </c>
-      <c r="H78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -10855,7 +10768,6 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F79" t="inlineStr"/>
       <c r="G79" t="inlineStr">
         <is>
           <t>0x4834b0</t>
@@ -10897,7 +10809,6 @@
           <t>0x4835d0</t>
         </is>
       </c>
-      <c r="H80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -10919,7 +10830,6 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F81" t="inlineStr"/>
       <c r="G81" t="inlineStr">
         <is>
           <t>0x483840</t>
@@ -10956,7 +10866,6 @@
           <t>4 critical hits</t>
         </is>
       </c>
-      <c r="H82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -10978,7 +10887,6 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F83" t="inlineStr"/>
       <c r="G83" t="inlineStr">
         <is>
           <t>0x483a60</t>
@@ -11010,13 +10918,11 @@
           <t>read</t>
         </is>
       </c>
-      <c r="F84" t="inlineStr"/>
       <c r="G84" t="inlineStr">
         <is>
           <t>0x483b30</t>
         </is>
       </c>
-      <c r="H84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -11038,13 +10944,11 @@
           <t>read</t>
         </is>
       </c>
-      <c r="F85" t="inlineStr"/>
       <c r="G85" t="inlineStr">
         <is>
           <t>0x483c20</t>
         </is>
       </c>
-      <c r="H85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -11066,7 +10970,6 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F86" t="inlineStr"/>
       <c r="G86" t="inlineStr">
         <is>
           <t>0x483d20</t>
@@ -11098,13 +11001,11 @@
           <t>read</t>
         </is>
       </c>
-      <c r="F87" t="inlineStr"/>
       <c r="G87" t="inlineStr">
         <is>
           <t>0x483e00</t>
         </is>
       </c>
-      <c r="H87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -11126,13 +11027,11 @@
           <t>read</t>
         </is>
       </c>
-      <c r="F88" t="inlineStr"/>
       <c r="G88" t="inlineStr">
         <is>
           <t>0x483ee0</t>
         </is>
       </c>
-      <c r="H88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -11154,8 +11053,6 @@
           <t>not found</t>
         </is>
       </c>
-      <c r="F89" t="inlineStr"/>
-      <c r="H89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -11177,7 +11074,6 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F90" t="inlineStr"/>
       <c r="H90" t="inlineStr">
         <is>
           <t>0x42017a</t>
@@ -11204,7 +11100,6 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F91" t="inlineStr"/>
       <c r="H91" t="inlineStr">
         <is>
           <t>0x43b16d</t>
@@ -11231,13 +11126,11 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr">
         <is>
           <t>0x484020</t>
         </is>
       </c>
-      <c r="H92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -11259,7 +11152,6 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F93" t="inlineStr"/>
       <c r="H93" t="inlineStr">
         <is>
           <t>0x422671</t>
@@ -11286,7 +11178,6 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F94" t="inlineStr"/>
       <c r="H94" t="inlineStr">
         <is>
           <t>0x422693, 0x44fa43, 0x44fb27</t>
@@ -11313,13 +11204,11 @@
           <t>read</t>
         </is>
       </c>
-      <c r="F95" t="inlineStr"/>
       <c r="G95" t="inlineStr">
         <is>
           <t>0x484150</t>
         </is>
       </c>
-      <c r="H95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -11351,7 +11240,6 @@
           <t>0x484330</t>
         </is>
       </c>
-      <c r="H96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -11378,7 +11266,6 @@
           <t>11.1 dolls</t>
         </is>
       </c>
-      <c r="H97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -11405,7 +11292,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -11432,7 +11318,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -11454,8 +11339,6 @@
           <t>not found</t>
         </is>
       </c>
-      <c r="F100" t="inlineStr"/>
-      <c r="H100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -11477,8 +11360,6 @@
           <t>not found</t>
         </is>
       </c>
-      <c r="F101" t="inlineStr"/>
-      <c r="H101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -11500,8 +11381,6 @@
           <t>not found</t>
         </is>
       </c>
-      <c r="F102" t="inlineStr"/>
-      <c r="H102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -11523,8 +11402,6 @@
           <t>not found</t>
         </is>
       </c>
-      <c r="F103" t="inlineStr"/>
-      <c r="H103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -11551,7 +11428,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -11578,7 +11454,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -11605,7 +11480,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -11632,7 +11506,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -11659,7 +11532,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="n">
@@ -11686,7 +11558,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="n">
@@ -11713,7 +11584,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -11771,7 +11641,6 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F112" t="inlineStr"/>
       <c r="H112" t="inlineStr">
         <is>
           <t>0x4fc054</t>
@@ -11798,8 +11667,6 @@
           <t>read</t>
         </is>
       </c>
-      <c r="F113" t="inlineStr"/>
-      <c r="H113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -11821,8 +11688,6 @@
           <t>read</t>
         </is>
       </c>
-      <c r="F114" t="inlineStr"/>
-      <c r="H114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="n">
@@ -11844,7 +11709,6 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F115" t="inlineStr"/>
       <c r="H115" t="inlineStr">
         <is>
           <t>0x4fc08d</t>
@@ -11876,7 +11740,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="n">
@@ -11908,7 +11771,6 @@
           <t>0x4869c0</t>
         </is>
       </c>
-      <c r="H117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="n">
@@ -11935,7 +11797,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="n">
@@ -11962,7 +11823,6 @@
           <t>applying a hit</t>
         </is>
       </c>
-      <c r="H119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="n">
@@ -11984,7 +11844,6 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F120" t="inlineStr"/>
       <c r="G120" t="inlineStr">
         <is>
           <t>0x486c70</t>
@@ -12016,13 +11875,11 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F121" t="inlineStr"/>
       <c r="G121" t="inlineStr">
         <is>
           <t>0x486e70</t>
         </is>
       </c>
-      <c r="H121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="n">
@@ -12044,8 +11901,6 @@
           <t>read</t>
         </is>
       </c>
-      <c r="F122" t="inlineStr"/>
-      <c r="H122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="n">
@@ -12067,7 +11922,6 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F123" t="inlineStr"/>
       <c r="H123" t="inlineStr">
         <is>
           <t>0x4fc0c9</t>
@@ -12094,7 +11948,6 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F124" t="inlineStr"/>
       <c r="H124" t="inlineStr">
         <is>
           <t>0x4fc0f2</t>
@@ -12121,7 +11974,6 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F125" t="inlineStr"/>
       <c r="H125" t="inlineStr">
         <is>
           <t>0x4fc11b</t>
@@ -12153,7 +12005,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="n">
@@ -12175,7 +12026,6 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F127" t="inlineStr"/>
       <c r="H127" t="inlineStr">
         <is>
           <t>0x47f936</t>
@@ -12202,7 +12052,6 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F128" t="inlineStr"/>
       <c r="H128" t="inlineStr">
         <is>
           <t>0x4fc144</t>
@@ -12260,8 +12109,6 @@
           <t>read</t>
         </is>
       </c>
-      <c r="F130" t="inlineStr"/>
-      <c r="H130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="n">
@@ -12283,13 +12130,11 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F131" t="inlineStr"/>
       <c r="G131" t="inlineStr">
         <is>
           <t>0x487540</t>
         </is>
       </c>
-      <c r="H131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="n">
@@ -12311,13 +12156,11 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F132" t="inlineStr"/>
       <c r="G132" t="inlineStr">
         <is>
           <t>0x487780</t>
         </is>
       </c>
-      <c r="H132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="n">
@@ -12339,13 +12182,11 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F133" t="inlineStr"/>
       <c r="G133" t="inlineStr">
         <is>
           <t>0x4879d0</t>
         </is>
       </c>
-      <c r="H133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -12377,7 +12218,6 @@
           <t>0x487bd0</t>
         </is>
       </c>
-      <c r="H134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="n">
@@ -12409,7 +12249,6 @@
           <t>0x487e00</t>
         </is>
       </c>
-      <c r="H135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="n">
@@ -12441,7 +12280,6 @@
           <t>0x488000</t>
         </is>
       </c>
-      <c r="H136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="n">
@@ -12473,7 +12311,6 @@
           <t>0x488200</t>
         </is>
       </c>
-      <c r="H137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="n">
@@ -12495,8 +12332,6 @@
           <t>read</t>
         </is>
       </c>
-      <c r="F138" t="inlineStr"/>
-      <c r="H138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="n">
@@ -12518,8 +12353,6 @@
           <t>read</t>
         </is>
       </c>
-      <c r="F139" t="inlineStr"/>
-      <c r="H139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="n">
@@ -12541,13 +12374,11 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F140" t="inlineStr"/>
       <c r="G140" t="inlineStr">
         <is>
           <t>0x4884f0</t>
         </is>
       </c>
-      <c r="H140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="n">
@@ -12569,7 +12400,6 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F141" t="inlineStr"/>
       <c r="G141" t="inlineStr">
         <is>
           <t>0x4886f0</t>
@@ -12601,8 +12431,6 @@
           <t>read</t>
         </is>
       </c>
-      <c r="F142" t="inlineStr"/>
-      <c r="H142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="n">
@@ -12624,8 +12452,6 @@
           <t>read</t>
         </is>
       </c>
-      <c r="F143" t="inlineStr"/>
-      <c r="H143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="n">
@@ -12657,7 +12483,6 @@
           <t>0x487e00</t>
         </is>
       </c>
-      <c r="H144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="n">
@@ -12684,7 +12509,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="n">
@@ -12711,7 +12535,6 @@
           <t>4 critical hits</t>
         </is>
       </c>
-      <c r="H146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="n">
@@ -12733,8 +12556,6 @@
           <t>not found</t>
         </is>
       </c>
-      <c r="F147" t="inlineStr"/>
-      <c r="H147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="n">
@@ -12761,7 +12582,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="n">
@@ -12788,7 +12608,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="n">
@@ -12810,8 +12629,6 @@
           <t>not found</t>
         </is>
       </c>
-      <c r="F150" t="inlineStr"/>
-      <c r="H150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="n">
@@ -12833,8 +12650,6 @@
           <t>not found</t>
         </is>
       </c>
-      <c r="F151" t="inlineStr"/>
-      <c r="H151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="n">
@@ -12861,7 +12676,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="n">
@@ -12883,8 +12697,6 @@
           <t>not found</t>
         </is>
       </c>
-      <c r="F153" t="inlineStr"/>
-      <c r="H153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="n">
@@ -12911,7 +12723,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="n">
@@ -12938,7 +12749,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="n">
@@ -12965,7 +12775,6 @@
           <t>2 physical attack, 5 order of turns</t>
         </is>
       </c>
-      <c r="H156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="n">
@@ -12992,7 +12801,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" t="n">
@@ -13019,7 +12827,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="n">
@@ -13046,7 +12853,6 @@
           <t>11.1 dolls</t>
         </is>
       </c>
-      <c r="H159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="n">
@@ -13073,7 +12879,6 @@
           <t>11.1 dolls</t>
         </is>
       </c>
-      <c r="H160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" t="n">
@@ -13100,7 +12905,6 @@
           <t>11.1 dolls</t>
         </is>
       </c>
-      <c r="H161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" t="n">
@@ -13127,7 +12931,6 @@
           <t>11.1 dolls</t>
         </is>
       </c>
-      <c r="H162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" t="n">
@@ -13154,7 +12957,6 @@
           <t>11.1 dolls</t>
         </is>
       </c>
-      <c r="H163" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" t="n">
@@ -13181,7 +12983,6 @@
           <t>11.1 dolls</t>
         </is>
       </c>
-      <c r="H164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="n">
@@ -13203,8 +13004,6 @@
           <t>not found</t>
         </is>
       </c>
-      <c r="F165" t="inlineStr"/>
-      <c r="H165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="n">
@@ -13226,7 +13025,6 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F166" t="inlineStr"/>
       <c r="H166" t="inlineStr">
         <is>
           <t>0x4f65ab</t>
@@ -13258,7 +13056,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H167" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" t="n">
@@ -13280,8 +13077,6 @@
           <t>not found</t>
         </is>
       </c>
-      <c r="F168" t="inlineStr"/>
-      <c r="H168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="n">
@@ -13303,8 +13098,6 @@
           <t>not found</t>
         </is>
       </c>
-      <c r="F169" t="inlineStr"/>
-      <c r="H169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" t="n">
@@ -13326,8 +13119,6 @@
           <t>not found</t>
         </is>
       </c>
-      <c r="F170" t="inlineStr"/>
-      <c r="H170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="n">
@@ -13349,7 +13140,6 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F171" t="inlineStr"/>
       <c r="H171" t="inlineStr">
         <is>
           <t>0x4fc236</t>
@@ -13376,7 +13166,6 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F172" t="inlineStr"/>
       <c r="H172" t="inlineStr">
         <is>
           <t>0x4246d2</t>
@@ -13408,7 +13197,6 @@
           <t>applying a hit</t>
         </is>
       </c>
-      <c r="H173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="n">
@@ -13435,7 +13223,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H174" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" t="n">
@@ -13462,7 +13249,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" t="n">
@@ -13489,7 +13275,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H176" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" t="n">
@@ -13511,7 +13296,6 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F177" t="inlineStr"/>
       <c r="H177" t="inlineStr">
         <is>
           <t>0x4238ad</t>
@@ -13538,7 +13322,6 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F178" t="inlineStr"/>
       <c r="H178" t="inlineStr">
         <is>
           <t>0x417309</t>
@@ -13565,7 +13348,6 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F179" t="inlineStr"/>
       <c r="H179" t="inlineStr">
         <is>
           <t>0x4fc26f</t>
@@ -13592,8 +13374,6 @@
           <t>not found</t>
         </is>
       </c>
-      <c r="F180" t="inlineStr"/>
-      <c r="H180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" t="n">
@@ -13620,7 +13400,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H181" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" t="n">
@@ -13642,8 +13421,6 @@
           <t>not found</t>
         </is>
       </c>
-      <c r="F182" t="inlineStr"/>
-      <c r="H182" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" t="n">
@@ -13665,8 +13442,6 @@
           <t>not found</t>
         </is>
       </c>
-      <c r="F183" t="inlineStr"/>
-      <c r="H183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="n">
@@ -13688,7 +13463,6 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F184" t="inlineStr"/>
       <c r="H184" t="inlineStr">
         <is>
           <t>0x47f8aa</t>
@@ -13715,7 +13489,6 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F185" t="inlineStr"/>
       <c r="H185" t="inlineStr">
         <is>
           <t>0x423d9b</t>
@@ -13747,7 +13520,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H186" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" t="n">
@@ -13774,7 +13546,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="n">
@@ -13801,7 +13572,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H188" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" t="n">
@@ -13823,8 +13593,6 @@
           <t>not found</t>
         </is>
       </c>
-      <c r="F189" t="inlineStr"/>
-      <c r="H189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" t="n">
@@ -13846,8 +13614,6 @@
           <t>not found</t>
         </is>
       </c>
-      <c r="F190" t="inlineStr"/>
-      <c r="H190" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" t="n">
@@ -13874,7 +13640,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" t="n">
@@ -13896,8 +13661,6 @@
           <t>not found</t>
         </is>
       </c>
-      <c r="F192" t="inlineStr"/>
-      <c r="H192" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" t="n">
@@ -13919,8 +13682,6 @@
           <t>not found</t>
         </is>
       </c>
-      <c r="F193" t="inlineStr"/>
-      <c r="H193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" t="n">
@@ -13942,8 +13703,6 @@
           <t>not found</t>
         </is>
       </c>
-      <c r="F194" t="inlineStr"/>
-      <c r="H194" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" t="n">
@@ -13965,7 +13724,6 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F195" t="inlineStr"/>
       <c r="H195" t="inlineStr">
         <is>
           <t>0x43d6cc</t>
@@ -13992,7 +13750,6 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F196" t="inlineStr"/>
       <c r="H196" t="inlineStr">
         <is>
           <t>0x43d705</t>
@@ -14019,7 +13776,6 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F197" t="inlineStr"/>
       <c r="H197" t="inlineStr">
         <is>
           <t>0x42d032</t>
@@ -14046,7 +13802,6 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F198" t="inlineStr"/>
       <c r="H198" t="inlineStr">
         <is>
           <t>0x50e789, 0x50ead5, 0x50edfc, 0x50f234, 0x50f51f, 0x50f7ea, 0x51266c, 0x512c75, 0x512f5a, 0x5131d0, 0x513470, 0x5134d1</t>
@@ -14078,7 +13833,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H199" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" t="n">
@@ -14105,7 +13859,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H200" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" t="n">
@@ -14132,7 +13885,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H201" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" t="n">
@@ -14154,8 +13906,6 @@
           <t>not found</t>
         </is>
       </c>
-      <c r="F202" t="inlineStr"/>
-      <c r="H202" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" t="n">
@@ -14177,8 +13927,6 @@
           <t>not found</t>
         </is>
       </c>
-      <c r="F203" t="inlineStr"/>
-      <c r="H203" t="inlineStr"/>
     </row>
     <row r="204">
       <c r="A204" t="n">
@@ -14205,7 +13953,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H204" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" t="n">
@@ -14227,8 +13974,6 @@
           <t>not found</t>
         </is>
       </c>
-      <c r="F205" t="inlineStr"/>
-      <c r="H205" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" t="n">
@@ -14250,8 +13995,6 @@
           <t>not found</t>
         </is>
       </c>
-      <c r="F206" t="inlineStr"/>
-      <c r="H206" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" t="n">
@@ -14273,8 +14016,6 @@
           <t>not found</t>
         </is>
       </c>
-      <c r="F207" t="inlineStr"/>
-      <c r="H207" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" t="n">
@@ -14296,7 +14037,6 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F208" t="inlineStr"/>
       <c r="H208" t="inlineStr">
         <is>
           <t>0x42208e</t>
@@ -14328,7 +14068,6 @@
           <t>11.1 dolls, 2 physical attack, 3 magic attack, 6b healing</t>
         </is>
       </c>
-      <c r="H209" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" t="n">
@@ -14350,8 +14089,6 @@
           <t>not found</t>
         </is>
       </c>
-      <c r="F210" t="inlineStr"/>
-      <c r="H210" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" t="n">
@@ -14373,8 +14110,6 @@
           <t>not found</t>
         </is>
       </c>
-      <c r="F211" t="inlineStr"/>
-      <c r="H211" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" t="n">
@@ -14396,8 +14131,6 @@
           <t>not found</t>
         </is>
       </c>
-      <c r="F212" t="inlineStr"/>
-      <c r="H212" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" t="n">
@@ -14419,7 +14152,6 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F213" t="inlineStr"/>
       <c r="H213" t="inlineStr">
         <is>
           <t>0x47f739</t>
@@ -14446,7 +14178,6 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F214" t="inlineStr"/>
       <c r="H214" t="inlineStr">
         <is>
           <t>0x424319</t>
@@ -14478,7 +14209,6 @@
           <t>6b heal cap, 6b healing</t>
         </is>
       </c>
-      <c r="H215" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" t="n">
@@ -14505,7 +14235,6 @@
           <t>3 magic attack, 6b heal cap</t>
         </is>
       </c>
-      <c r="H216" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" t="n">
@@ -14532,7 +14261,6 @@
           <t>11.1 dolls</t>
         </is>
       </c>
-      <c r="H217" t="inlineStr"/>
     </row>
     <row r="218">
       <c r="A218" t="n">
@@ -14554,7 +14282,6 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F218" t="inlineStr"/>
       <c r="H218" t="inlineStr">
         <is>
           <t>0x4f65d6</t>
@@ -14581,7 +14308,6 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F219" t="inlineStr"/>
       <c r="H219" t="inlineStr">
         <is>
           <t>0x4493d6</t>
@@ -14613,7 +14339,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H220" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" t="n">
@@ -14635,7 +14360,6 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F221" t="inlineStr"/>
       <c r="H221" t="inlineStr">
         <is>
           <t>0x4203fd</t>
@@ -14662,8 +14386,6 @@
           <t>not found</t>
         </is>
       </c>
-      <c r="F222" t="inlineStr"/>
-      <c r="H222" t="inlineStr"/>
     </row>
     <row r="223">
       <c r="A223" t="n">
@@ -14690,7 +14412,6 @@
           <t>applying a hit</t>
         </is>
       </c>
-      <c r="H223" t="inlineStr"/>
     </row>
     <row r="224">
       <c r="A224" t="n">
@@ -14712,7 +14433,6 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F224" t="inlineStr"/>
       <c r="H224" t="inlineStr">
         <is>
           <t>0x55609a</t>
@@ -14739,8 +14459,6 @@
           <t>not found</t>
         </is>
       </c>
-      <c r="F225" t="inlineStr"/>
-      <c r="H225" t="inlineStr"/>
     </row>
     <row r="226">
       <c r="A226" t="n">
@@ -14762,8 +14480,6 @@
           <t>not found</t>
         </is>
       </c>
-      <c r="F226" t="inlineStr"/>
-      <c r="H226" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" t="n">
@@ -14790,7 +14506,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H227" t="inlineStr"/>
     </row>
     <row r="228">
       <c r="A228" t="n">
@@ -14817,7 +14532,6 @@
           <t>applying a hit</t>
         </is>
       </c>
-      <c r="H228" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" t="n">
@@ -14839,8 +14553,6 @@
           <t>not found</t>
         </is>
       </c>
-      <c r="F229" t="inlineStr"/>
-      <c r="H229" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" t="n">
@@ -14862,7 +14574,6 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F230" t="inlineStr"/>
       <c r="H230" t="inlineStr">
         <is>
           <t>0x47f5e2</t>
@@ -14889,8 +14600,6 @@
           <t>not found</t>
         </is>
       </c>
-      <c r="F231" t="inlineStr"/>
-      <c r="H231" t="inlineStr"/>
     </row>
     <row r="232">
       <c r="A232" t="n">
@@ -14917,7 +14626,6 @@
           <t>11.1 dolls</t>
         </is>
       </c>
-      <c r="H232" t="inlineStr"/>
     </row>
     <row r="233">
       <c r="A233" t="n">
@@ -14939,8 +14647,6 @@
           <t>not found</t>
         </is>
       </c>
-      <c r="F233" t="inlineStr"/>
-      <c r="H233" t="inlineStr"/>
     </row>
     <row r="234">
       <c r="A234" t="n">
@@ -14967,7 +14673,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H234" t="inlineStr"/>
     </row>
     <row r="235">
       <c r="A235" t="n">
@@ -14989,8 +14694,6 @@
           <t>not found</t>
         </is>
       </c>
-      <c r="F235" t="inlineStr"/>
-      <c r="H235" t="inlineStr"/>
     </row>
     <row r="236">
       <c r="A236" t="n">
@@ -15012,8 +14715,6 @@
           <t>not found</t>
         </is>
       </c>
-      <c r="F236" t="inlineStr"/>
-      <c r="H236" t="inlineStr"/>
     </row>
     <row r="237">
       <c r="A237" t="n">
@@ -15035,7 +14736,6 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F237" t="inlineStr"/>
       <c r="H237" t="inlineStr">
         <is>
           <t>0x4235d5</t>
@@ -15062,8 +14762,6 @@
           <t>not found</t>
         </is>
       </c>
-      <c r="F238" t="inlineStr"/>
-      <c r="H238" t="inlineStr"/>
     </row>
     <row r="239">
       <c r="A239" t="n">
@@ -15090,7 +14788,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H239" t="inlineStr"/>
     </row>
     <row r="240">
       <c r="A240" t="n">
@@ -15117,7 +14814,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H240" t="inlineStr"/>
     </row>
     <row r="241">
       <c r="A241" t="n">
@@ -15144,7 +14840,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H241" t="inlineStr"/>
     </row>
     <row r="242">
       <c r="A242" t="n">
@@ -15171,7 +14866,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H242" t="inlineStr"/>
     </row>
     <row r="243">
       <c r="A243" t="n">
@@ -15198,7 +14892,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H243" t="inlineStr"/>
     </row>
     <row r="244">
       <c r="A244" t="n">
@@ -15225,7 +14918,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H244" t="inlineStr"/>
     </row>
     <row r="245">
       <c r="A245" t="n">
@@ -15252,7 +14944,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H245" t="inlineStr"/>
     </row>
     <row r="246">
       <c r="A246" t="n">
@@ -15279,7 +14970,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H246" t="inlineStr"/>
     </row>
     <row r="247">
       <c r="A247" t="n">
@@ -15306,7 +14996,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H247" t="inlineStr"/>
     </row>
     <row r="248">
       <c r="A248" t="n">
@@ -15328,8 +15017,6 @@
           <t>not found</t>
         </is>
       </c>
-      <c r="F248" t="inlineStr"/>
-      <c r="H248" t="inlineStr"/>
     </row>
     <row r="249">
       <c r="A249" t="n">
@@ -15356,7 +15043,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H249" t="inlineStr"/>
     </row>
     <row r="250">
       <c r="A250" t="n">
@@ -15378,8 +15064,6 @@
           <t>not found</t>
         </is>
       </c>
-      <c r="F250" t="inlineStr"/>
-      <c r="H250" t="inlineStr"/>
     </row>
     <row r="251">
       <c r="A251" t="n">
@@ -15401,8 +15085,6 @@
           <t>not found</t>
         </is>
       </c>
-      <c r="F251" t="inlineStr"/>
-      <c r="H251" t="inlineStr"/>
     </row>
     <row r="252">
       <c r="A252" t="n">
@@ -15424,8 +15106,6 @@
           <t>not found</t>
         </is>
       </c>
-      <c r="F252" t="inlineStr"/>
-      <c r="H252" t="inlineStr"/>
     </row>
     <row r="253">
       <c r="A253" t="n">
@@ -15447,8 +15127,6 @@
           <t>not found</t>
         </is>
       </c>
-      <c r="F253" t="inlineStr"/>
-      <c r="H253" t="inlineStr"/>
     </row>
     <row r="254">
       <c r="A254" t="n">
@@ -15470,7 +15148,6 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F254" t="inlineStr"/>
       <c r="H254" t="inlineStr">
         <is>
           <t>0x43aa0e</t>
@@ -15497,8 +15174,6 @@
           <t>not found</t>
         </is>
       </c>
-      <c r="F255" t="inlineStr"/>
-      <c r="H255" t="inlineStr"/>
     </row>
     <row r="256">
       <c r="A256" t="n">
@@ -15520,8 +15195,6 @@
           <t>not found</t>
         </is>
       </c>
-      <c r="F256" t="inlineStr"/>
-      <c r="H256" t="inlineStr"/>
     </row>
     <row r="257">
       <c r="A257" t="n">
@@ -15543,7 +15216,6 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F257" t="inlineStr"/>
       <c r="H257" t="inlineStr">
         <is>
           <t>0x44fa63</t>
@@ -15570,8 +15242,6 @@
           <t>not found</t>
         </is>
       </c>
-      <c r="F258" t="inlineStr"/>
-      <c r="H258" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -16206,7 +15876,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -16377,12 +16047,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Smallest change</t>
+          <t>No more change than the essence allows, no less than the problem needs</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Among the sets of values that pass every test, the one closest to vanilla is the one shipped</t>
+          <t>Every target is met with room to spare, not at its edge. Among the sets of values that do so and keep what each class and enemy is, the one that moves least from vanilla is shipped. Closeness to vanilla is a tie-break, never a reason to leave a problem half solved</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -16410,6 +16080,23 @@
       <c r="D9" t="inlineStr">
         <is>
           <t>Per boss, vanilla against Balance</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>R09</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>The mod does not fall short</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>No row of Criticisms that is true in vanilla is closed by a change so small that the player would not notice it: each closed row states the figure before and after, and the after sits inside its band with margin</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: second batch of effect rules
second batch of effect rules; status lookups found through both status
slots
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -8706,6 +8706,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -8724,7 +8725,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>located</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -8732,11 +8733,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>0x420165, 0x4da54f</t>
-        </is>
-      </c>
+      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -8763,6 +8760,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -8781,7 +8779,13 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>not found</t>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>0x422a18, 0x47f5fc, 0x47f633</t>
         </is>
       </c>
     </row>
@@ -8805,6 +8809,8 @@
           <t>not found</t>
         </is>
       </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -8823,7 +8829,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>located</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -8836,11 +8842,7 @@
           <t>0x47fb70</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>0x4807f1, 0x4808d1</t>
-        </is>
-      </c>
+      <c r="H7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -8859,7 +8861,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>located</t>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>actions</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -8867,6 +8874,7 @@
           <t>0x47fc30</t>
         </is>
       </c>
+      <c r="H8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -8885,7 +8893,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>located</t>
+          <t>partly read</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>actions</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -8893,6 +8906,7 @@
           <t>0x47fd00</t>
         </is>
       </c>
+      <c r="H9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -8942,7 +8956,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>located</t>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>outside battle</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -8950,6 +8969,7 @@
           <t>0x47fde0</t>
         </is>
       </c>
+      <c r="H11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -8971,6 +8991,8 @@
           <t>read</t>
         </is>
       </c>
+      <c r="F12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -8989,7 +9011,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>located</t>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>outside battle</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -8997,6 +9024,7 @@
           <t>0x47ffc0</t>
         </is>
       </c>
+      <c r="H13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -9018,6 +9046,8 @@
           <t>not found</t>
         </is>
       </c>
+      <c r="F14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -9044,6 +9074,7 @@
           <t>applying a hit</t>
         </is>
       </c>
+      <c r="H15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -9070,6 +9101,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -9091,6 +9123,8 @@
           <t>read</t>
         </is>
       </c>
+      <c r="F17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -9117,6 +9151,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -9143,6 +9178,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -9169,6 +9205,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -9195,6 +9232,7 @@
           <t>4 critical hits</t>
         </is>
       </c>
+      <c r="H21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -9221,6 +9259,7 @@
           <t>4 critical hits</t>
         </is>
       </c>
+      <c r="H22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -9247,6 +9286,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -9268,9 +9308,15 @@
           <t>located</t>
         </is>
       </c>
+      <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
           <t>0x48bd60</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>0x4fbfb4</t>
         </is>
       </c>
     </row>
@@ -9299,6 +9345,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -9325,6 +9372,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -9343,7 +9391,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>located</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -9351,11 +9399,7 @@
           <t>5c turn delay</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>0x4803a1, 0x480685</t>
-        </is>
-      </c>
+      <c r="H27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -9382,6 +9426,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -9400,14 +9445,15 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>0x42310f, 0x44fe2c, 0x44ff20</t>
-        </is>
-      </c>
+          <t>partly read</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>steal</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -9426,14 +9472,15 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>0x423120, 0x44fe55, 0x45036a</t>
-        </is>
-      </c>
+          <t>partly read</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>steal</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -9452,14 +9499,15 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>0x44ff50</t>
-        </is>
-      </c>
+          <t>partly read</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>steal</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -9481,6 +9529,8 @@
           <t>read</t>
         </is>
       </c>
+      <c r="F32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -9499,7 +9549,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>located</t>
+          <t>partly read</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -9507,11 +9557,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>0x42106c</t>
-        </is>
-      </c>
+      <c r="H33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -9538,6 +9584,7 @@
           <t>4 critical hits</t>
         </is>
       </c>
+      <c r="H34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -9564,6 +9611,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -9582,7 +9630,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>located</t>
+          <t>partly read</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -9590,11 +9638,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>0x421098</t>
-        </is>
-      </c>
+      <c r="H36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -9621,6 +9665,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -9647,6 +9692,7 @@
           <t>applying a hit</t>
         </is>
       </c>
+      <c r="H38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -9673,6 +9719,7 @@
           <t>applying a hit</t>
         </is>
       </c>
+      <c r="H39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -9699,6 +9746,7 @@
           <t>applying a hit</t>
         </is>
       </c>
+      <c r="H40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -9720,11 +9768,13 @@
           <t>located</t>
         </is>
       </c>
+      <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr">
         <is>
           <t>0x481060</t>
         </is>
       </c>
+      <c r="H41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -9746,6 +9796,8 @@
           <t>not found</t>
         </is>
       </c>
+      <c r="F42" t="inlineStr"/>
+      <c r="H42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -9767,11 +9819,13 @@
           <t>located</t>
         </is>
       </c>
+      <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr">
         <is>
           <t>0x481160</t>
         </is>
       </c>
+      <c r="H43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -9793,6 +9847,7 @@
           <t>located</t>
         </is>
       </c>
+      <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr">
         <is>
           <t>0x4813a0</t>
@@ -9829,6 +9884,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -9855,6 +9911,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -9881,6 +9938,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -9907,6 +9965,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -9933,6 +9992,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -9959,6 +10019,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -9985,6 +10046,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -10003,14 +10065,15 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="H52" t="inlineStr">
-        <is>
-          <t>0x417e65</t>
-        </is>
-      </c>
+          <t>partly read</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>hits of an action</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -10037,6 +10100,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -10063,6 +10127,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -10089,6 +10154,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -10115,6 +10181,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -10141,6 +10208,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -10167,6 +10235,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -10193,6 +10262,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -10211,7 +10281,13 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>read</t>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr"/>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>0x41f947</t>
         </is>
       </c>
     </row>
@@ -10235,6 +10311,7 @@
           <t>located</t>
         </is>
       </c>
+      <c r="F61" t="inlineStr"/>
       <c r="H61" t="inlineStr">
         <is>
           <t>0x41faaf</t>
@@ -10258,7 +10335,12 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>located</t>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>6b healing</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -10266,11 +10348,7 @@
           <t>0x4817c0</t>
         </is>
       </c>
-      <c r="H62" t="inlineStr">
-        <is>
-          <t>0x43b111</t>
-        </is>
-      </c>
+      <c r="H62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -10289,7 +10367,12 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>located</t>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>6d recovery</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -10297,11 +10380,7 @@
           <t>0x481890</t>
         </is>
       </c>
-      <c r="H63" t="inlineStr">
-        <is>
-          <t>0x43b128</t>
-        </is>
-      </c>
+      <c r="H63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -10320,7 +10399,12 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>located</t>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>6d recovery</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -10328,11 +10412,7 @@
           <t>0x481950</t>
         </is>
       </c>
-      <c r="H64" t="inlineStr">
-        <is>
-          <t>0x56d571</t>
-        </is>
-      </c>
+      <c r="H64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -10354,6 +10434,7 @@
           <t>located</t>
         </is>
       </c>
+      <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr">
         <is>
           <t>0x481a20</t>
@@ -10382,7 +10463,12 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>located</t>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>outside battle</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -10390,11 +10476,7 @@
           <t>0x47fde0</t>
         </is>
       </c>
-      <c r="H66" t="inlineStr">
-        <is>
-          <t>0x5103c4</t>
-        </is>
-      </c>
+      <c r="H66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -10413,7 +10495,12 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>located</t>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>outside battle</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -10421,6 +10508,7 @@
           <t>0x481d80</t>
         </is>
       </c>
+      <c r="H67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -10447,6 +10535,7 @@
           <t>4 critical hits</t>
         </is>
       </c>
+      <c r="H68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -10473,6 +10562,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -10494,6 +10584,7 @@
           <t>located</t>
         </is>
       </c>
+      <c r="F70" t="inlineStr"/>
       <c r="H70" t="inlineStr">
         <is>
           <t>0x42e1ba, 0x43b08e, 0x43b183</t>
@@ -10530,6 +10621,7 @@
           <t>0x481ea0</t>
         </is>
       </c>
+      <c r="H71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -10561,6 +10653,7 @@
           <t>0x4822c0</t>
         </is>
       </c>
+      <c r="H72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -10592,6 +10685,7 @@
           <t>0x482530</t>
         </is>
       </c>
+      <c r="H73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -10623,6 +10717,7 @@
           <t>0x4827a0</t>
         </is>
       </c>
+      <c r="H74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -10654,6 +10749,7 @@
           <t>0x482a10</t>
         </is>
       </c>
+      <c r="H75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -10685,6 +10781,7 @@
           <t>0x482c80</t>
         </is>
       </c>
+      <c r="H76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -10716,6 +10813,7 @@
           <t>0x482e40</t>
         </is>
       </c>
+      <c r="H77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -10747,6 +10845,7 @@
           <t>0x4831f0</t>
         </is>
       </c>
+      <c r="H78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -10768,6 +10867,7 @@
           <t>located</t>
         </is>
       </c>
+      <c r="F79" t="inlineStr"/>
       <c r="G79" t="inlineStr">
         <is>
           <t>0x4834b0</t>
@@ -10809,6 +10909,7 @@
           <t>0x4835d0</t>
         </is>
       </c>
+      <c r="H80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -10830,6 +10931,7 @@
           <t>located</t>
         </is>
       </c>
+      <c r="F81" t="inlineStr"/>
       <c r="G81" t="inlineStr">
         <is>
           <t>0x483840</t>
@@ -10866,6 +10968,7 @@
           <t>4 critical hits</t>
         </is>
       </c>
+      <c r="H82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -10884,7 +10987,12 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>located</t>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>6d recovery</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
@@ -10892,11 +11000,7 @@
           <t>0x483a60</t>
         </is>
       </c>
-      <c r="H83" t="inlineStr">
-        <is>
-          <t>0x43b13f</t>
-        </is>
-      </c>
+      <c r="H83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -10918,11 +11022,13 @@
           <t>read</t>
         </is>
       </c>
+      <c r="F84" t="inlineStr"/>
       <c r="G84" t="inlineStr">
         <is>
           <t>0x483b30</t>
         </is>
       </c>
+      <c r="H84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -10944,11 +11050,13 @@
           <t>read</t>
         </is>
       </c>
+      <c r="F85" t="inlineStr"/>
       <c r="G85" t="inlineStr">
         <is>
           <t>0x483c20</t>
         </is>
       </c>
+      <c r="H85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -10967,7 +11075,12 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>located</t>
+          <t>partly read</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>6d recovery</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
@@ -10975,11 +11088,7 @@
           <t>0x483d20</t>
         </is>
       </c>
-      <c r="H86" t="inlineStr">
-        <is>
-          <t>0x43b156</t>
-        </is>
-      </c>
+      <c r="H86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -10998,12 +11107,18 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>read</t>
-        </is>
-      </c>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr"/>
       <c r="G87" t="inlineStr">
         <is>
           <t>0x483e00</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>0x537db7</t>
         </is>
       </c>
     </row>
@@ -11027,11 +11142,13 @@
           <t>read</t>
         </is>
       </c>
+      <c r="F88" t="inlineStr"/>
       <c r="G88" t="inlineStr">
         <is>
           <t>0x483ee0</t>
         </is>
       </c>
+      <c r="H88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -11053,6 +11170,8 @@
           <t>not found</t>
         </is>
       </c>
+      <c r="F89" t="inlineStr"/>
+      <c r="H89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -11071,14 +11190,15 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="H90" t="inlineStr">
-        <is>
-          <t>0x42017a</t>
-        </is>
-      </c>
+          <t>partly read</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>applying a hit</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -11100,6 +11220,7 @@
           <t>located</t>
         </is>
       </c>
+      <c r="F91" t="inlineStr"/>
       <c r="H91" t="inlineStr">
         <is>
           <t>0x43b16d</t>
@@ -11126,11 +11247,13 @@
           <t>located</t>
         </is>
       </c>
+      <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr">
         <is>
           <t>0x484020</t>
         </is>
       </c>
+      <c r="H92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -11152,6 +11275,7 @@
           <t>located</t>
         </is>
       </c>
+      <c r="F93" t="inlineStr"/>
       <c r="H93" t="inlineStr">
         <is>
           <t>0x422671</t>
@@ -11178,6 +11302,7 @@
           <t>located</t>
         </is>
       </c>
+      <c r="F94" t="inlineStr"/>
       <c r="H94" t="inlineStr">
         <is>
           <t>0x422693, 0x44fa43, 0x44fb27</t>
@@ -11204,11 +11329,13 @@
           <t>read</t>
         </is>
       </c>
+      <c r="F95" t="inlineStr"/>
       <c r="G95" t="inlineStr">
         <is>
           <t>0x484150</t>
         </is>
       </c>
+      <c r="H95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -11240,6 +11367,7 @@
           <t>0x484330</t>
         </is>
       </c>
+      <c r="H96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -11266,6 +11394,7 @@
           <t>11.1 dolls</t>
         </is>
       </c>
+      <c r="H97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -11292,6 +11421,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -11318,6 +11448,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -11339,6 +11470,8 @@
           <t>not found</t>
         </is>
       </c>
+      <c r="F100" t="inlineStr"/>
+      <c r="H100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -11360,6 +11493,8 @@
           <t>not found</t>
         </is>
       </c>
+      <c r="F101" t="inlineStr"/>
+      <c r="H101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -11381,6 +11516,8 @@
           <t>not found</t>
         </is>
       </c>
+      <c r="F102" t="inlineStr"/>
+      <c r="H102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -11402,6 +11539,8 @@
           <t>not found</t>
         </is>
       </c>
+      <c r="F103" t="inlineStr"/>
+      <c r="H103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -11428,6 +11567,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -11454,6 +11594,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -11480,6 +11621,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -11506,6 +11648,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -11532,6 +11675,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="n">
@@ -11558,6 +11702,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="n">
@@ -11584,6 +11729,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -11602,7 +11748,7 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>located</t>
+          <t>partly read</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
@@ -11615,11 +11761,7 @@
           <t>0x4864c0</t>
         </is>
       </c>
-      <c r="H111" t="inlineStr">
-        <is>
-          <t>0x4229f4, 0x42456e</t>
-        </is>
-      </c>
+      <c r="H111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="n">
@@ -11638,14 +11780,15 @@
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="H112" t="inlineStr">
-        <is>
-          <t>0x4fc054</t>
-        </is>
-      </c>
+          <t>partly read</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>10 stats of a character</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="n">
@@ -11667,6 +11810,12 @@
           <t>read</t>
         </is>
       </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>9.1 targets</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -11685,7 +11834,13 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>read</t>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr"/>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>0x420cac</t>
         </is>
       </c>
     </row>
@@ -11706,14 +11861,15 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="H115" t="inlineStr">
-        <is>
-          <t>0x4fc08d</t>
-        </is>
-      </c>
+          <t>partly read</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>10 stats of a character</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="n">
@@ -11740,6 +11896,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="n">
@@ -11771,6 +11928,7 @@
           <t>0x4869c0</t>
         </is>
       </c>
+      <c r="H117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="n">
@@ -11797,6 +11955,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="n">
@@ -11823,6 +11982,7 @@
           <t>applying a hit</t>
         </is>
       </c>
+      <c r="H119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="n">
@@ -11844,6 +12004,7 @@
           <t>located</t>
         </is>
       </c>
+      <c r="F120" t="inlineStr"/>
       <c r="G120" t="inlineStr">
         <is>
           <t>0x486c70</t>
@@ -11875,11 +12036,13 @@
           <t>located</t>
         </is>
       </c>
+      <c r="F121" t="inlineStr"/>
       <c r="G121" t="inlineStr">
         <is>
           <t>0x486e70</t>
         </is>
       </c>
+      <c r="H121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="n">
@@ -11901,6 +12064,8 @@
           <t>read</t>
         </is>
       </c>
+      <c r="F122" t="inlineStr"/>
+      <c r="H122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="n">
@@ -11919,14 +12084,15 @@
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="H123" t="inlineStr">
-        <is>
-          <t>0x4fc0c9</t>
-        </is>
-      </c>
+          <t>partly read</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>10 stats of a character</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="n">
@@ -11945,14 +12111,15 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="H124" t="inlineStr">
-        <is>
-          <t>0x4fc0f2</t>
-        </is>
-      </c>
+          <t>partly read</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>10 stats of a character</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="n">
@@ -11971,14 +12138,15 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="H125" t="inlineStr">
-        <is>
-          <t>0x4fc11b</t>
-        </is>
-      </c>
+          <t>partly read</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>10 stats of a character</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="n">
@@ -12005,6 +12173,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="n">
@@ -12026,6 +12195,7 @@
           <t>located</t>
         </is>
       </c>
+      <c r="F127" t="inlineStr"/>
       <c r="H127" t="inlineStr">
         <is>
           <t>0x47f936</t>
@@ -12052,6 +12222,7 @@
           <t>located</t>
         </is>
       </c>
+      <c r="F128" t="inlineStr"/>
       <c r="H128" t="inlineStr">
         <is>
           <t>0x4fc144</t>
@@ -12109,6 +12280,8 @@
           <t>read</t>
         </is>
       </c>
+      <c r="F130" t="inlineStr"/>
+      <c r="H130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="n">
@@ -12130,11 +12303,13 @@
           <t>located</t>
         </is>
       </c>
+      <c r="F131" t="inlineStr"/>
       <c r="G131" t="inlineStr">
         <is>
           <t>0x487540</t>
         </is>
       </c>
+      <c r="H131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="n">
@@ -12156,9 +12331,15 @@
           <t>located</t>
         </is>
       </c>
+      <c r="F132" t="inlineStr"/>
       <c r="G132" t="inlineStr">
         <is>
           <t>0x487780</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>0x4fc156</t>
         </is>
       </c>
     </row>
@@ -12182,9 +12363,15 @@
           <t>located</t>
         </is>
       </c>
+      <c r="F133" t="inlineStr"/>
       <c r="G133" t="inlineStr">
         <is>
           <t>0x4879d0</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>0x4fc169</t>
         </is>
       </c>
     </row>
@@ -12218,6 +12405,7 @@
           <t>0x487bd0</t>
         </is>
       </c>
+      <c r="H134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="n">
@@ -12249,6 +12437,7 @@
           <t>0x487e00</t>
         </is>
       </c>
+      <c r="H135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="n">
@@ -12280,6 +12469,7 @@
           <t>0x488000</t>
         </is>
       </c>
+      <c r="H136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="n">
@@ -12311,6 +12501,7 @@
           <t>0x488200</t>
         </is>
       </c>
+      <c r="H137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="n">
@@ -12332,6 +12523,8 @@
           <t>read</t>
         </is>
       </c>
+      <c r="F138" t="inlineStr"/>
+      <c r="H138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="n">
@@ -12353,6 +12546,8 @@
           <t>read</t>
         </is>
       </c>
+      <c r="F139" t="inlineStr"/>
+      <c r="H139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="n">
@@ -12374,11 +12569,17 @@
           <t>located</t>
         </is>
       </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>5 order of turns</t>
+        </is>
+      </c>
       <c r="G140" t="inlineStr">
         <is>
           <t>0x4884f0</t>
         </is>
       </c>
+      <c r="H140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="n">
@@ -12400,6 +12601,7 @@
           <t>located</t>
         </is>
       </c>
+      <c r="F141" t="inlineStr"/>
       <c r="G141" t="inlineStr">
         <is>
           <t>0x4886f0</t>
@@ -12431,6 +12633,8 @@
           <t>read</t>
         </is>
       </c>
+      <c r="F142" t="inlineStr"/>
+      <c r="H142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="n">
@@ -12452,6 +12656,8 @@
           <t>read</t>
         </is>
       </c>
+      <c r="F143" t="inlineStr"/>
+      <c r="H143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="n">
@@ -12483,6 +12689,7 @@
           <t>0x487e00</t>
         </is>
       </c>
+      <c r="H144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="n">
@@ -12509,6 +12716,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="n">
@@ -12535,6 +12743,7 @@
           <t>4 critical hits</t>
         </is>
       </c>
+      <c r="H146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="n">
@@ -12556,6 +12765,8 @@
           <t>not found</t>
         </is>
       </c>
+      <c r="F147" t="inlineStr"/>
+      <c r="H147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="n">
@@ -12582,6 +12793,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="n">
@@ -12608,6 +12820,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="n">
@@ -12629,6 +12842,8 @@
           <t>not found</t>
         </is>
       </c>
+      <c r="F150" t="inlineStr"/>
+      <c r="H150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="n">
@@ -12650,6 +12865,8 @@
           <t>not found</t>
         </is>
       </c>
+      <c r="F151" t="inlineStr"/>
+      <c r="H151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="n">
@@ -12676,6 +12893,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="n">
@@ -12697,6 +12915,8 @@
           <t>not found</t>
         </is>
       </c>
+      <c r="F153" t="inlineStr"/>
+      <c r="H153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="n">
@@ -12723,6 +12943,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="n">
@@ -12749,6 +12970,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="n">
@@ -12775,6 +12997,7 @@
           <t>2 physical attack, 5 order of turns</t>
         </is>
       </c>
+      <c r="H156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="n">
@@ -12801,6 +13024,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" t="n">
@@ -12827,6 +13051,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="n">
@@ -12853,6 +13078,7 @@
           <t>11.1 dolls</t>
         </is>
       </c>
+      <c r="H159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="n">
@@ -12879,6 +13105,7 @@
           <t>11.1 dolls</t>
         </is>
       </c>
+      <c r="H160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" t="n">
@@ -12905,6 +13132,7 @@
           <t>11.1 dolls</t>
         </is>
       </c>
+      <c r="H161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" t="n">
@@ -12931,6 +13159,7 @@
           <t>11.1 dolls</t>
         </is>
       </c>
+      <c r="H162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" t="n">
@@ -12957,6 +13186,7 @@
           <t>11.1 dolls</t>
         </is>
       </c>
+      <c r="H163" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" t="n">
@@ -12983,6 +13213,7 @@
           <t>11.1 dolls</t>
         </is>
       </c>
+      <c r="H164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="n">
@@ -13004,6 +13235,8 @@
           <t>not found</t>
         </is>
       </c>
+      <c r="F165" t="inlineStr"/>
+      <c r="H165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="n">
@@ -13022,14 +13255,15 @@
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="H166" t="inlineStr">
-        <is>
-          <t>0x4f65ab</t>
-        </is>
-      </c>
+          <t>partly read</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>10 stats of a character</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" t="n">
@@ -13056,6 +13290,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H167" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" t="n">
@@ -13074,9 +13309,15 @@
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>not found</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>6b healing</t>
+        </is>
+      </c>
+      <c r="H168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="n">
@@ -13098,6 +13339,8 @@
           <t>not found</t>
         </is>
       </c>
+      <c r="F169" t="inlineStr"/>
+      <c r="H169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" t="n">
@@ -13119,6 +13362,8 @@
           <t>not found</t>
         </is>
       </c>
+      <c r="F170" t="inlineStr"/>
+      <c r="H170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="n">
@@ -13137,14 +13382,15 @@
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="H171" t="inlineStr">
-        <is>
-          <t>0x4fc236</t>
-        </is>
-      </c>
+          <t>partly read</t>
+        </is>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>10 stats of a character</t>
+        </is>
+      </c>
+      <c r="H171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="n">
@@ -13163,14 +13409,15 @@
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="H172" t="inlineStr">
-        <is>
-          <t>0x4246d2</t>
-        </is>
-      </c>
+          <t>partly read</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>passive rolls</t>
+        </is>
+      </c>
+      <c r="H172" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" t="n">
@@ -13197,6 +13444,7 @@
           <t>applying a hit</t>
         </is>
       </c>
+      <c r="H173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="n">
@@ -13223,6 +13471,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H174" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" t="n">
@@ -13249,6 +13498,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" t="n">
@@ -13275,6 +13525,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H176" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" t="n">
@@ -13293,14 +13544,15 @@
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="H177" t="inlineStr">
-        <is>
-          <t>0x4238ad</t>
-        </is>
-      </c>
+          <t>partly read</t>
+        </is>
+      </c>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>passive rolls</t>
+        </is>
+      </c>
+      <c r="H177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="n">
@@ -13319,14 +13571,15 @@
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="H178" t="inlineStr">
-        <is>
-          <t>0x417309</t>
-        </is>
-      </c>
+          <t>partly read</t>
+        </is>
+      </c>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>passive rolls</t>
+        </is>
+      </c>
+      <c r="H178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" t="n">
@@ -13348,6 +13601,7 @@
           <t>located</t>
         </is>
       </c>
+      <c r="F179" t="inlineStr"/>
       <c r="H179" t="inlineStr">
         <is>
           <t>0x4fc26f</t>
@@ -13371,7 +13625,13 @@
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>not found</t>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="F180" t="inlineStr"/>
+      <c r="H180" t="inlineStr">
+        <is>
+          <t>0x47e64d</t>
         </is>
       </c>
     </row>
@@ -13400,6 +13660,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H181" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" t="n">
@@ -13421,6 +13682,8 @@
           <t>not found</t>
         </is>
       </c>
+      <c r="F182" t="inlineStr"/>
+      <c r="H182" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" t="n">
@@ -13442,6 +13705,8 @@
           <t>not found</t>
         </is>
       </c>
+      <c r="F183" t="inlineStr"/>
+      <c r="H183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="n">
@@ -13463,6 +13728,11 @@
           <t>located</t>
         </is>
       </c>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>5 order of turns</t>
+        </is>
+      </c>
       <c r="H184" t="inlineStr">
         <is>
           <t>0x47f8aa</t>
@@ -13489,6 +13759,7 @@
           <t>located</t>
         </is>
       </c>
+      <c r="F185" t="inlineStr"/>
       <c r="H185" t="inlineStr">
         <is>
           <t>0x423d9b</t>
@@ -13520,6 +13791,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H186" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" t="n">
@@ -13546,6 +13818,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="n">
@@ -13572,6 +13845,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H188" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" t="n">
@@ -13590,7 +13864,13 @@
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>not found</t>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="F189" t="inlineStr"/>
+      <c r="H189" t="inlineStr">
+        <is>
+          <t>0x4fd331</t>
         </is>
       </c>
     </row>
@@ -13611,9 +13891,15 @@
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>not found</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>5 order of turns</t>
+        </is>
+      </c>
+      <c r="H190" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" t="n">
@@ -13640,6 +13926,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" t="n">
@@ -13658,7 +13945,13 @@
       </c>
       <c r="E192" t="inlineStr">
         <is>
-          <t>not found</t>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="F192" t="inlineStr"/>
+      <c r="H192" t="inlineStr">
+        <is>
+          <t>0x41adcd</t>
         </is>
       </c>
     </row>
@@ -13682,6 +13975,8 @@
           <t>not found</t>
         </is>
       </c>
+      <c r="F193" t="inlineStr"/>
+      <c r="H193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" t="n">
@@ -13703,6 +13998,8 @@
           <t>not found</t>
         </is>
       </c>
+      <c r="F194" t="inlineStr"/>
+      <c r="H194" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" t="n">
@@ -13721,14 +14018,15 @@
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="H195" t="inlineStr">
-        <is>
-          <t>0x43d6cc</t>
-        </is>
-      </c>
+          <t>partly read</t>
+        </is>
+      </c>
+      <c r="F195" t="inlineStr">
+        <is>
+          <t>after a battle</t>
+        </is>
+      </c>
+      <c r="H195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" t="n">
@@ -13747,14 +14045,15 @@
       </c>
       <c r="E196" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="H196" t="inlineStr">
-        <is>
-          <t>0x43d705</t>
-        </is>
-      </c>
+          <t>partly read</t>
+        </is>
+      </c>
+      <c r="F196" t="inlineStr">
+        <is>
+          <t>after a battle</t>
+        </is>
+      </c>
+      <c r="H196" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" t="n">
@@ -13773,14 +14072,15 @@
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="H197" t="inlineStr">
-        <is>
-          <t>0x42d032</t>
-        </is>
-      </c>
+          <t>partly read</t>
+        </is>
+      </c>
+      <c r="F197" t="inlineStr">
+        <is>
+          <t>passive rolls</t>
+        </is>
+      </c>
+      <c r="H197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" t="n">
@@ -13799,14 +14099,15 @@
       </c>
       <c r="E198" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="H198" t="inlineStr">
-        <is>
-          <t>0x50e789, 0x50ead5, 0x50edfc, 0x50f234, 0x50f51f, 0x50f7ea, 0x51266c, 0x512c75, 0x512f5a, 0x5131d0, 0x513470, 0x5134d1</t>
-        </is>
-      </c>
+          <t>partly read</t>
+        </is>
+      </c>
+      <c r="F198" t="inlineStr">
+        <is>
+          <t>items</t>
+        </is>
+      </c>
+      <c r="H198" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" t="n">
@@ -13833,6 +14134,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H199" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" t="n">
@@ -13859,6 +14161,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H200" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" t="n">
@@ -13885,6 +14188,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H201" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" t="n">
@@ -13906,6 +14210,8 @@
           <t>not found</t>
         </is>
       </c>
+      <c r="F202" t="inlineStr"/>
+      <c r="H202" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" t="n">
@@ -13927,6 +14233,8 @@
           <t>not found</t>
         </is>
       </c>
+      <c r="F203" t="inlineStr"/>
+      <c r="H203" t="inlineStr"/>
     </row>
     <row r="204">
       <c r="A204" t="n">
@@ -13953,6 +14261,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H204" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" t="n">
@@ -13974,6 +14283,8 @@
           <t>not found</t>
         </is>
       </c>
+      <c r="F205" t="inlineStr"/>
+      <c r="H205" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" t="n">
@@ -13995,6 +14306,8 @@
           <t>not found</t>
         </is>
       </c>
+      <c r="F206" t="inlineStr"/>
+      <c r="H206" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" t="n">
@@ -14016,6 +14329,8 @@
           <t>not found</t>
         </is>
       </c>
+      <c r="F207" t="inlineStr"/>
+      <c r="H207" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" t="n">
@@ -14034,14 +14349,15 @@
       </c>
       <c r="E208" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="H208" t="inlineStr">
-        <is>
-          <t>0x42208e</t>
-        </is>
-      </c>
+          <t>partly read</t>
+        </is>
+      </c>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t>applying a hit</t>
+        </is>
+      </c>
+      <c r="H208" t="inlineStr"/>
     </row>
     <row r="209">
       <c r="A209" t="n">
@@ -14068,6 +14384,7 @@
           <t>11.1 dolls, 2 physical attack, 3 magic attack, 6b healing</t>
         </is>
       </c>
+      <c r="H209" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" t="n">
@@ -14089,6 +14406,8 @@
           <t>not found</t>
         </is>
       </c>
+      <c r="F210" t="inlineStr"/>
+      <c r="H210" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" t="n">
@@ -14110,6 +14429,8 @@
           <t>not found</t>
         </is>
       </c>
+      <c r="F211" t="inlineStr"/>
+      <c r="H211" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" t="n">
@@ -14131,6 +14452,8 @@
           <t>not found</t>
         </is>
       </c>
+      <c r="F212" t="inlineStr"/>
+      <c r="H212" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" t="n">
@@ -14152,6 +14475,7 @@
           <t>located</t>
         </is>
       </c>
+      <c r="F213" t="inlineStr"/>
       <c r="H213" t="inlineStr">
         <is>
           <t>0x47f739</t>
@@ -14175,14 +14499,15 @@
       </c>
       <c r="E214" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="H214" t="inlineStr">
-        <is>
-          <t>0x424319</t>
-        </is>
-      </c>
+          <t>partly read</t>
+        </is>
+      </c>
+      <c r="F214" t="inlineStr">
+        <is>
+          <t>passive rolls</t>
+        </is>
+      </c>
+      <c r="H214" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" t="n">
@@ -14209,6 +14534,7 @@
           <t>6b heal cap, 6b healing</t>
         </is>
       </c>
+      <c r="H215" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" t="n">
@@ -14235,6 +14561,7 @@
           <t>3 magic attack, 6b heal cap</t>
         </is>
       </c>
+      <c r="H216" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" t="n">
@@ -14261,6 +14588,7 @@
           <t>11.1 dolls</t>
         </is>
       </c>
+      <c r="H217" t="inlineStr"/>
     </row>
     <row r="218">
       <c r="A218" t="n">
@@ -14279,14 +14607,15 @@
       </c>
       <c r="E218" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="H218" t="inlineStr">
-        <is>
-          <t>0x4f65d6</t>
-        </is>
-      </c>
+          <t>partly read</t>
+        </is>
+      </c>
+      <c r="F218" t="inlineStr">
+        <is>
+          <t>10 stats of a character</t>
+        </is>
+      </c>
+      <c r="H218" t="inlineStr"/>
     </row>
     <row r="219">
       <c r="A219" t="n">
@@ -14305,14 +14634,15 @@
       </c>
       <c r="E219" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="H219" t="inlineStr">
-        <is>
-          <t>0x4493d6</t>
-        </is>
-      </c>
+          <t>partly read</t>
+        </is>
+      </c>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t>passive rolls</t>
+        </is>
+      </c>
+      <c r="H219" t="inlineStr"/>
     </row>
     <row r="220">
       <c r="A220" t="n">
@@ -14339,6 +14669,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H220" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" t="n">
@@ -14357,14 +14688,15 @@
       </c>
       <c r="E221" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="H221" t="inlineStr">
-        <is>
-          <t>0x4203fd</t>
-        </is>
-      </c>
+          <t>partly read</t>
+        </is>
+      </c>
+      <c r="F221" t="inlineStr">
+        <is>
+          <t>applying a hit</t>
+        </is>
+      </c>
+      <c r="H221" t="inlineStr"/>
     </row>
     <row r="222">
       <c r="A222" t="n">
@@ -14386,6 +14718,8 @@
           <t>not found</t>
         </is>
       </c>
+      <c r="F222" t="inlineStr"/>
+      <c r="H222" t="inlineStr"/>
     </row>
     <row r="223">
       <c r="A223" t="n">
@@ -14412,6 +14746,7 @@
           <t>applying a hit</t>
         </is>
       </c>
+      <c r="H223" t="inlineStr"/>
     </row>
     <row r="224">
       <c r="A224" t="n">
@@ -14430,14 +14765,15 @@
       </c>
       <c r="E224" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="H224" t="inlineStr">
-        <is>
-          <t>0x55609a</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F224" t="inlineStr">
+        <is>
+          <t>outside battle</t>
+        </is>
+      </c>
+      <c r="H224" t="inlineStr"/>
     </row>
     <row r="225">
       <c r="A225" t="n">
@@ -14459,6 +14795,8 @@
           <t>not found</t>
         </is>
       </c>
+      <c r="F225" t="inlineStr"/>
+      <c r="H225" t="inlineStr"/>
     </row>
     <row r="226">
       <c r="A226" t="n">
@@ -14480,6 +14818,8 @@
           <t>not found</t>
         </is>
       </c>
+      <c r="F226" t="inlineStr"/>
+      <c r="H226" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" t="n">
@@ -14506,6 +14846,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H227" t="inlineStr"/>
     </row>
     <row r="228">
       <c r="A228" t="n">
@@ -14532,6 +14873,7 @@
           <t>applying a hit</t>
         </is>
       </c>
+      <c r="H228" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" t="n">
@@ -14553,6 +14895,8 @@
           <t>not found</t>
         </is>
       </c>
+      <c r="F229" t="inlineStr"/>
+      <c r="H229" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" t="n">
@@ -14574,6 +14918,7 @@
           <t>located</t>
         </is>
       </c>
+      <c r="F230" t="inlineStr"/>
       <c r="H230" t="inlineStr">
         <is>
           <t>0x47f5e2</t>
@@ -14600,6 +14945,8 @@
           <t>not found</t>
         </is>
       </c>
+      <c r="F231" t="inlineStr"/>
+      <c r="H231" t="inlineStr"/>
     </row>
     <row r="232">
       <c r="A232" t="n">
@@ -14626,6 +14973,7 @@
           <t>11.1 dolls</t>
         </is>
       </c>
+      <c r="H232" t="inlineStr"/>
     </row>
     <row r="233">
       <c r="A233" t="n">
@@ -14647,6 +14995,8 @@
           <t>not found</t>
         </is>
       </c>
+      <c r="F233" t="inlineStr"/>
+      <c r="H233" t="inlineStr"/>
     </row>
     <row r="234">
       <c r="A234" t="n">
@@ -14673,6 +15023,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H234" t="inlineStr"/>
     </row>
     <row r="235">
       <c r="A235" t="n">
@@ -14691,9 +15042,15 @@
       </c>
       <c r="E235" t="inlineStr">
         <is>
-          <t>not found</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F235" t="inlineStr">
+        <is>
+          <t>6b heal cap</t>
+        </is>
+      </c>
+      <c r="H235" t="inlineStr"/>
     </row>
     <row r="236">
       <c r="A236" t="n">
@@ -14715,6 +15072,8 @@
           <t>not found</t>
         </is>
       </c>
+      <c r="F236" t="inlineStr"/>
+      <c r="H236" t="inlineStr"/>
     </row>
     <row r="237">
       <c r="A237" t="n">
@@ -14733,14 +15092,15 @@
       </c>
       <c r="E237" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="H237" t="inlineStr">
-        <is>
-          <t>0x4235d5</t>
-        </is>
-      </c>
+          <t>partly read</t>
+        </is>
+      </c>
+      <c r="F237" t="inlineStr">
+        <is>
+          <t>applying a hit</t>
+        </is>
+      </c>
+      <c r="H237" t="inlineStr"/>
     </row>
     <row r="238">
       <c r="A238" t="n">
@@ -14759,9 +15119,15 @@
       </c>
       <c r="E238" t="inlineStr">
         <is>
-          <t>not found</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F238" t="inlineStr">
+        <is>
+          <t>5 order of turns</t>
+        </is>
+      </c>
+      <c r="H238" t="inlineStr"/>
     </row>
     <row r="239">
       <c r="A239" t="n">
@@ -14788,6 +15154,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H239" t="inlineStr"/>
     </row>
     <row r="240">
       <c r="A240" t="n">
@@ -14814,6 +15181,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H240" t="inlineStr"/>
     </row>
     <row r="241">
       <c r="A241" t="n">
@@ -14840,6 +15208,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H241" t="inlineStr"/>
     </row>
     <row r="242">
       <c r="A242" t="n">
@@ -14866,6 +15235,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H242" t="inlineStr"/>
     </row>
     <row r="243">
       <c r="A243" t="n">
@@ -14892,6 +15262,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H243" t="inlineStr"/>
     </row>
     <row r="244">
       <c r="A244" t="n">
@@ -14918,6 +15289,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H244" t="inlineStr"/>
     </row>
     <row r="245">
       <c r="A245" t="n">
@@ -14944,6 +15316,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H245" t="inlineStr"/>
     </row>
     <row r="246">
       <c r="A246" t="n">
@@ -14970,6 +15343,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H246" t="inlineStr"/>
     </row>
     <row r="247">
       <c r="A247" t="n">
@@ -14996,6 +15370,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H247" t="inlineStr"/>
     </row>
     <row r="248">
       <c r="A248" t="n">
@@ -15017,6 +15392,8 @@
           <t>not found</t>
         </is>
       </c>
+      <c r="F248" t="inlineStr"/>
+      <c r="H248" t="inlineStr"/>
     </row>
     <row r="249">
       <c r="A249" t="n">
@@ -15043,6 +15420,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H249" t="inlineStr"/>
     </row>
     <row r="250">
       <c r="A250" t="n">
@@ -15061,7 +15439,13 @@
       </c>
       <c r="E250" t="inlineStr">
         <is>
-          <t>not found</t>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="F250" t="inlineStr"/>
+      <c r="H250" t="inlineStr">
+        <is>
+          <t>0x4fc1fc</t>
         </is>
       </c>
     </row>
@@ -15085,6 +15469,8 @@
           <t>not found</t>
         </is>
       </c>
+      <c r="F251" t="inlineStr"/>
+      <c r="H251" t="inlineStr"/>
     </row>
     <row r="252">
       <c r="A252" t="n">
@@ -15106,6 +15492,8 @@
           <t>not found</t>
         </is>
       </c>
+      <c r="F252" t="inlineStr"/>
+      <c r="H252" t="inlineStr"/>
     </row>
     <row r="253">
       <c r="A253" t="n">
@@ -15127,6 +15515,8 @@
           <t>not found</t>
         </is>
       </c>
+      <c r="F253" t="inlineStr"/>
+      <c r="H253" t="inlineStr"/>
     </row>
     <row r="254">
       <c r="A254" t="n">
@@ -15145,14 +15535,15 @@
       </c>
       <c r="E254" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="H254" t="inlineStr">
-        <is>
-          <t>0x43aa0e</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>6c EXP</t>
+        </is>
+      </c>
+      <c r="H254" t="inlineStr"/>
     </row>
     <row r="255">
       <c r="A255" t="n">
@@ -15174,6 +15565,8 @@
           <t>not found</t>
         </is>
       </c>
+      <c r="F255" t="inlineStr"/>
+      <c r="H255" t="inlineStr"/>
     </row>
     <row r="256">
       <c r="A256" t="n">
@@ -15195,6 +15588,8 @@
           <t>not found</t>
         </is>
       </c>
+      <c r="F256" t="inlineStr"/>
+      <c r="H256" t="inlineStr"/>
     </row>
     <row r="257">
       <c r="A257" t="n">
@@ -15216,6 +15611,7 @@
           <t>located</t>
         </is>
       </c>
+      <c r="F257" t="inlineStr"/>
       <c r="H257" t="inlineStr">
         <is>
           <t>0x44fa63</t>
@@ -15242,6 +15638,8 @@
           <t>not found</t>
         </is>
       </c>
+      <c r="F258" t="inlineStr"/>
+      <c r="H258" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -18129,13 +18527,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D48"/>
+  <dimension ref="A1:E92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
     <col width="120" customWidth="1" min="3" max="3"/>
     <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -18159,6 +18558,11 @@
           <t>Read_At</t>
         </is>
       </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>How_Far</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -18174,6 +18578,11 @@
           <t>The hit itself: the attack functions run for it</t>
         </is>
       </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -18189,6 +18598,11 @@
           <t>0x44f477: +5 per earlier hit</t>
         </is>
       </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -18204,6 +18618,11 @@
           <t>0x44cfad: divides the interruption rate</t>
         </is>
       </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -18219,6 +18638,11 @@
           <t>0x44edbe: the id is compared in a register (Critical Magic)</t>
         </is>
       </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -18234,6 +18658,11 @@
           <t>0x44f0ce: damage cap</t>
         </is>
       </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -18249,6 +18678,11 @@
           <t>0x48c5c7: heal cap</t>
         </is>
       </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -18264,6 +18698,11 @@
           <t>0x484330: number of units created</t>
         </is>
       </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -18279,6 +18718,11 @@
           <t>0x4843c9: turns a doll lasts</t>
         </is>
       </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -18294,6 +18738,11 @@
           <t>Doll: the id is stored in the doll and compared (0x44bb1c)</t>
         </is>
       </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -18309,6 +18758,11 @@
           <t>As 228</t>
         </is>
       </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -18324,6 +18778,11 @@
           <t>As 228</t>
         </is>
       </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -18339,6 +18798,11 @@
           <t>As 228</t>
         </is>
       </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -18354,6 +18818,11 @@
           <t>As 228</t>
         </is>
       </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -18369,6 +18838,11 @@
           <t>As 228</t>
         </is>
       </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -18384,6 +18858,11 @@
           <t>0x44b4fd, 0x44dda8, 0x48d7a1: Doll Mastery</t>
         </is>
       </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -18404,6 +18883,11 @@
           <t>0x417db0</t>
         </is>
       </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -18424,6 +18908,11 @@
           <t>0x417e04</t>
         </is>
       </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -18444,6 +18933,11 @@
           <t>0x417e1d</t>
         </is>
       </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -18464,6 +18958,11 @@
           <t>0x417e25</t>
         </is>
       </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -18484,6 +18983,11 @@
           <t>0x417e93</t>
         </is>
       </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -18504,6 +19008,11 @@
           <t>0x417ed0</t>
         </is>
       </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -18524,6 +19033,11 @@
           <t>0x417f0e</t>
         </is>
       </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -18544,6 +19058,11 @@
           <t>0x417f4e</t>
         </is>
       </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -18564,6 +19083,11 @@
           <t>0x417f67</t>
         </is>
       </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -18584,6 +19108,11 @@
           <t>0x417f80</t>
         </is>
       </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -18604,6 +19133,11 @@
           <t>0x417fbe</t>
         </is>
       </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -18624,6 +19158,11 @@
           <t>0x417ffe</t>
         </is>
       </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -18644,6 +19183,11 @@
           <t>0x417dc4</t>
         </is>
       </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -18664,6 +19208,11 @@
           <t>0x418045</t>
         </is>
       </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -18684,6 +19233,11 @@
           <t>0x41808c</t>
         </is>
       </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -18704,6 +19258,11 @@
           <t>0x4226c4</t>
         </is>
       </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -18724,6 +19283,11 @@
           <t>0x4223d4</t>
         </is>
       </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -18744,6 +19308,11 @@
           <t>0x42259f</t>
         </is>
       </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -18764,6 +19333,11 @@
           <t>0x421dcd</t>
         </is>
       </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -18784,6 +19358,11 @@
           <t>0x422210</t>
         </is>
       </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -18804,6 +19383,11 @@
           <t>0x42196e</t>
         </is>
       </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -18824,6 +19408,11 @@
           <t>0x42155a, 0x422eda</t>
         </is>
       </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -18844,6 +19433,11 @@
           <t>0x421604, 0x422fc7</t>
         </is>
       </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -18864,6 +19458,11 @@
           <t>0x421261 - 0x4216d2</t>
         </is>
       </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -18884,6 +19483,11 @@
           <t>0x421261 - 0x4216d2</t>
         </is>
       </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -18904,6 +19508,11 @@
           <t>0x421261 - 0x4216d2</t>
         </is>
       </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -18924,6 +19533,11 @@
           <t>0x421261 - 0x4216d2</t>
         </is>
       </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -18944,6 +19558,11 @@
           <t>0x421261 - 0x4216d2</t>
         </is>
       </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -18964,6 +19583,11 @@
           <t>0x421261 - 0x4216d2</t>
         </is>
       </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -18984,6 +19608,11 @@
           <t>0x421261 - 0x4216d2</t>
         </is>
       </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -19004,6 +19633,11 @@
           <t>0x421261 - 0x4216d2</t>
         </is>
       </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -19022,6 +19656,1086 @@
       <c r="D48" t="inlineStr">
         <is>
           <t>0x421498, 0x4214e9</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>1</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>3 magic attack</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>The power of a spell: added to INT * (2 + swing) before the multipliers</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>0x44dc97</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>9</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>6b healing</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>A heal of a fixed amount: the value replaces the amount computed from RES</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>0x48d8ff</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>10</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>actions</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Defend: damage received is halved (2.4) and the gauge value is multiplied by 1.15 (5)</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>0x44c576, 0x44a326</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>11</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>actions</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Escape: chance 0.3 + (own AGI - average enemy AGI) / 50 + skill, as the debug message states; its code is not read</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>0x47fd00</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>partly</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>54</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>5c turn delay</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Turn delay: docs/FORMULAS.md 5c</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>0x423a41</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>60</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>steal</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Gold steal: chance 0.5 * (own DEX + 50) / (target AGI + 50) * factor, as the debug message states; the amount is not read</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>0x44fe2c</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>partly</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>61</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>steal</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Item steal: same chance formula as gold steal with its own factor (a constant 0.05 follows); the item comes from the steal fields of the enemy</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>0x44fe55</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>partly</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>62</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>steal</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Enemy gold steal: handled in the steal function after the roll; the amount is not read</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>0x44ff50</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>partly</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>69</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>2 physical attack</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Defence is not subtracted (2.4). The apply code also adds it by itself, with value 1, in one case not followed</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>0x42106c</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>partly</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>72</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>2 physical attack</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>The hit cannot miss. Added by the apply code with value 1 in cases not followed</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>0x421098</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>partly</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>93</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>hits of an action</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Number of hits: its value</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>0x417e65</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>partly</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>103</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>6b healing</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Heal by RES: docs/FORMULAS.md 6b. An enemy attack that carries it is aimed at the allies of its user</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>0x48d730, 0x43b111</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>104</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>6d recovery</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Full heal: HP becomes max HP</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>0x481890</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>105</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>6d recovery</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Revival: HP = int(max HP * value)</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>0x4819b2</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>128</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>6d recovery</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>HP recovery: int(max HP * value)</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>0x483ac5</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>131</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>6d recovery</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Heals the opposing side: a fraction of max HP, under the heal cap</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>0x483d20</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>partly</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>137</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>applying a hit</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Number of targets of the action: read with the spell power when the action starts; how the count is used is not followed</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>0x42017a</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>partly</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>168</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>5 order of turns</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Speed buff or debuff of a unit: enters the gauge value as a bonus (5). Its own command rolls below 100 under a chance; the apply code also creates it at -0.2 and -0.75 in two cases not followed</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>0x4864c0, 0x4229f4, 0x42456e</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>partly</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>169</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>10 stats of a character</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>While active it changes all five elemental resistances of the unit: read when its stats are recomputed; the arithmetic is not followed</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>0x4fbc40</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>partly</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>172</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>10 stats of a character</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>While active it changes max HP of the unit: read when its stats are recomputed; the arithmetic is not followed</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>0x4fbc40</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>partly</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>184</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>10 stats of a character</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>While active it changes stab resistance of the unit: read when its stats are recomputed; the arithmetic is not followed</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>0x4fbc40</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>partly</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>185</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>10 stats of a character</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>While active it changes slash resistance of the unit: read when its stats are recomputed; the arithmetic is not followed</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>0x4fbc40</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>partly</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>186</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>10 stats of a character</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>While active it changes bash resistance of the unit: read when its stats are recomputed; the arithmetic is not followed</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>0x4fbc40</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>partly</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>248</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>10 stats of a character</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>While active it changes a resistance of the unit: read when its stats are recomputed; the arithmetic is not followed</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>0x4fbc40</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>partly</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>243</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>10 stats of a character</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Weapon mastery: a modifier of attack for a kind of weapon, read when the stats of the unit are recomputed; the arithmetic is not followed</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>0x4f65ab</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>partly</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>298</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>10 stats of a character</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>A second weapon attack modifier, read next to 243</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>0x4f65d6</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>partly</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>249</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>passive rolls</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>When the target has it: a roll below 100 under value * 100 triggers Reprisal; what follows is not read</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>0x4246d2</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>partly</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>254</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>passive rolls</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Survival: a roll below 100 under value * 100 when a hit would bring HP to 0; what HP is left is not followed</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>0x4238ad</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>partly</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>255</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>passive rolls</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>When the target has it: a roll below 100 under value * 100 guards the hit (Auto-Guard)</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>0x417309</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>partly</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>274</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>passive rolls</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>When the unit has it: a roll below 100 under value * 100 triggers Loss Rate; its consequence is not read</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>0x42d032</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>partly</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>293</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>passive rolls</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>When the attacker has it: a roll below 100 under value * 100 slows its target</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>0x424319</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>partly</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>300</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>passive rolls</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>When a unit has it: a roll below 100 under value * 100 at the start of a battle gives it the first turn (First Grid)</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>0x4493d6</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>partly</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>285</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>applying a hit</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Elegant Dancing: checked on the target before a physical hit, with no roll; its consequence is not followed</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>0x42208e</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>partly</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>303</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>applying a hit</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Counter Whip: checked on the target when an action starts; its consequence is not followed</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>0x4203fd</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>partly</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>272</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>after a battle</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>HP restored after a battle: read with 273 when the battle ends, next to a constant 0.3; the arithmetic is not followed</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>0x43d6cc</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>partly</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>273</v>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>after a battle</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>TP restored after a battle: as 272</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>0x43d705</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>partly</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>275</v>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>items</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Modifier of healing items: read where an item heals</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>0x50e789</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>partly</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>320</v>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>applying a hit</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Devil's Whisper: when present the apply code creates an instant death command</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>0x4235d5</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>partly</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="n">
+        <v>428</v>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>6c EXP</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Gold of a fallen enemy multiplied by four (shl by 2), never below 100</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>0x43aa0e</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="n">
+        <v>17</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>outside battle</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Disable Traps: used on the map or in menus, not in a fight</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="n">
+        <v>20</v>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>outside battle</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Identify: used on the map or in menus, not in a fight</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="n">
+        <v>107</v>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>outside battle</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Light: used on the map or in menus, not in a fight</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="n">
+        <v>108</v>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>outside battle</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Return: used on the map or in menus, not in a fight</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="n">
+        <v>306</v>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>outside battle</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Present for Me: used on the map or in menus, not in a fight</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>read</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: rules of special damage and of the statuses that change stats
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -8806,10 +8806,14 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>not found</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr"/>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>2.7 special damage</t>
+        </is>
+      </c>
       <c r="H6" t="inlineStr"/>
     </row>
     <row r="7">
@@ -8925,19 +8929,15 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>located</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>3 magic attack</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>0x44fb84</t>
-        </is>
-      </c>
+          <t>2.7 special damage, 3 magic attack</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -9043,11 +9043,15 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>not found</t>
+          <t>located</t>
         </is>
       </c>
       <c r="F14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>0x42e9cb</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -9283,7 +9287,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2 physical attack</t>
+          <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
       <c r="H23" t="inlineStr"/>
@@ -9305,20 +9309,20 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr"/>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>10.2 statuses on stats</t>
+        </is>
+      </c>
       <c r="G24" t="inlineStr">
         <is>
           <t>0x48bd60</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>0x4fbfb4</t>
-        </is>
-      </c>
+      <c r="H24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -9423,7 +9427,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>2 physical attack</t>
+          <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
       <c r="H28" t="inlineStr"/>
@@ -10875,7 +10879,7 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>0x5107c9</t>
+          <t>0x4e585e, 0x5107c9</t>
         </is>
       </c>
     </row>
@@ -10939,7 +10943,7 @@
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>0x4fb652</t>
+          <t>0x4fa6d5, 0x4fb652</t>
         </is>
       </c>
     </row>
@@ -11217,15 +11221,15 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F91" t="inlineStr"/>
-      <c r="H91" t="inlineStr">
-        <is>
-          <t>0x43b16d</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>2.7 special damage</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -11253,7 +11257,11 @@
           <t>0x484020</t>
         </is>
       </c>
-      <c r="H92" t="inlineStr"/>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>0x4e5878</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -11272,15 +11280,15 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F93" t="inlineStr"/>
-      <c r="H93" t="inlineStr">
-        <is>
-          <t>0x422671</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>2.7 special damage</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -11299,15 +11307,15 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F94" t="inlineStr"/>
-      <c r="H94" t="inlineStr">
-        <is>
-          <t>0x422693, 0x44fa43, 0x44fb27</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>2.7 special damage</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -11780,12 +11788,12 @@
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>partly read</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>10 stats of a character</t>
+          <t>10.2 statuses on stats</t>
         </is>
       </c>
       <c r="H112" t="inlineStr"/>
@@ -11861,12 +11869,12 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>partly read</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>10 stats of a character</t>
+          <t>10.2 statuses on stats</t>
         </is>
       </c>
       <c r="H115" t="inlineStr"/>
@@ -12084,12 +12092,12 @@
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>partly read</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>10 stats of a character</t>
+          <t>10.2 statuses on stats</t>
         </is>
       </c>
       <c r="H123" t="inlineStr"/>
@@ -12111,12 +12119,12 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>partly read</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>10 stats of a character</t>
+          <t>10.2 statuses on stats</t>
         </is>
       </c>
       <c r="H124" t="inlineStr"/>
@@ -12138,12 +12146,12 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>partly read</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>10 stats of a character</t>
+          <t>10.2 statuses on stats</t>
         </is>
       </c>
       <c r="H125" t="inlineStr"/>
@@ -12219,15 +12227,15 @@
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F128" t="inlineStr"/>
-      <c r="H128" t="inlineStr">
-        <is>
-          <t>0x4fc144</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>10.2 statuses on stats</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="n">
@@ -12246,19 +12254,15 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>located</t>
+          <t>partly read</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>3 magic attack</t>
-        </is>
-      </c>
-      <c r="H129" t="inlineStr">
-        <is>
-          <t>0x44fb17</t>
-        </is>
-      </c>
+          <t>2.7 special damage, 3 magic attack</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="n">
@@ -12300,10 +12304,14 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F131" t="inlineStr"/>
+          <t>partly read</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>10.2 statuses on stats</t>
+        </is>
+      </c>
       <c r="G131" t="inlineStr">
         <is>
           <t>0x487540</t>
@@ -12328,20 +12336,20 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F132" t="inlineStr"/>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>10.2 statuses on stats</t>
+        </is>
+      </c>
       <c r="G132" t="inlineStr">
         <is>
           <t>0x487780</t>
         </is>
       </c>
-      <c r="H132" t="inlineStr">
-        <is>
-          <t>0x4fc156</t>
-        </is>
-      </c>
+      <c r="H132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="n">
@@ -12360,20 +12368,20 @@
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F133" t="inlineStr"/>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>10.2 statuses on stats</t>
+        </is>
+      </c>
       <c r="G133" t="inlineStr">
         <is>
           <t>0x4879d0</t>
         </is>
       </c>
-      <c r="H133" t="inlineStr">
-        <is>
-          <t>0x4fc169</t>
-        </is>
-      </c>
+      <c r="H133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -12520,11 +12528,15 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>read</t>
+          <t>located</t>
         </is>
       </c>
       <c r="F138" t="inlineStr"/>
-      <c r="H138" t="inlineStr"/>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>0x42f0fa</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="n">
@@ -12598,20 +12610,20 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F141" t="inlineStr"/>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>10.2 statuses on stats</t>
+        </is>
+      </c>
       <c r="G141" t="inlineStr">
         <is>
           <t>0x4886f0</t>
         </is>
       </c>
-      <c r="H141" t="inlineStr">
-        <is>
-          <t>0x4fc1ea</t>
-        </is>
-      </c>
+      <c r="H141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="n">
@@ -13382,12 +13394,12 @@
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>partly read</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F171" t="inlineStr">
         <is>
-          <t>10 stats of a character</t>
+          <t>10.2 statuses on stats</t>
         </is>
       </c>
       <c r="H171" t="inlineStr"/>
@@ -13598,15 +13610,15 @@
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F179" t="inlineStr"/>
-      <c r="H179" t="inlineStr">
-        <is>
-          <t>0x4fc26f</t>
-        </is>
-      </c>
+          <t>partly read</t>
+        </is>
+      </c>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>10.2 statuses on stats</t>
+        </is>
+      </c>
+      <c r="H179" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" t="n">
@@ -15389,11 +15401,15 @@
       </c>
       <c r="E248" t="inlineStr">
         <is>
-          <t>not found</t>
+          <t>located</t>
         </is>
       </c>
       <c r="F248" t="inlineStr"/>
-      <c r="H248" t="inlineStr"/>
+      <c r="H248" t="inlineStr">
+        <is>
+          <t>0x42f10a</t>
+        </is>
+      </c>
     </row>
     <row r="249">
       <c r="A249" t="n">
@@ -15439,15 +15455,15 @@
       </c>
       <c r="E250" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F250" t="inlineStr"/>
-      <c r="H250" t="inlineStr">
-        <is>
-          <t>0x4fc1fc</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F250" t="inlineStr">
+        <is>
+          <t>10.2 statuses on stats</t>
+        </is>
+      </c>
+      <c r="H250" t="inlineStr"/>
     </row>
     <row r="251">
       <c r="A251" t="n">
@@ -15608,15 +15624,15 @@
       </c>
       <c r="E257" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F257" t="inlineStr"/>
-      <c r="H257" t="inlineStr">
-        <is>
-          <t>0x44fa63</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F257" t="inlineStr">
+        <is>
+          <t>2.7 special damage</t>
+        </is>
+      </c>
+      <c r="H257" t="inlineStr"/>
     </row>
     <row r="258">
       <c r="A258" t="n">
@@ -15635,10 +15651,14 @@
       </c>
       <c r="E258" t="inlineStr">
         <is>
-          <t>not found</t>
-        </is>
-      </c>
-      <c r="F258" t="inlineStr"/>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F258" t="inlineStr">
+        <is>
+          <t>2.7 special damage</t>
+        </is>
+      </c>
       <c r="H258" t="inlineStr"/>
     </row>
   </sheetData>
@@ -18527,7 +18547,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E92"/>
+  <dimension ref="A1:E115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -20120,22 +20140,22 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>10 stats of a character</t>
+          <t>10.2 statuses on stats</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>While active it changes all five elemental resistances of the unit: read when its stats are recomputed; the arithmetic is not followed</t>
+          <t>While active adds int(value) to each of the five elemental resistances</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>0x4fbc40</t>
+          <t>0x4fc05b</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>partly</t>
+          <t>read</t>
         </is>
       </c>
     </row>
@@ -20145,22 +20165,22 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>10 stats of a character</t>
+          <t>10.2 statuses on stats</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>While active it changes max HP of the unit: read when its stats are recomputed; the arithmetic is not followed</t>
+          <t>While active max HP gains max HP * value</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>0x4fbc40</t>
+          <t>0x4fc094</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>partly</t>
+          <t>read</t>
         </is>
       </c>
     </row>
@@ -20170,22 +20190,22 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>10 stats of a character</t>
+          <t>10.2 statuses on stats</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>While active it changes stab resistance of the unit: read when its stats are recomputed; the arithmetic is not followed</t>
+          <t>While active adds int(value) to stab resistance</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>0x4fbc40</t>
+          <t>0x4fc0d0</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>partly</t>
+          <t>read</t>
         </is>
       </c>
     </row>
@@ -20195,22 +20215,22 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>10 stats of a character</t>
+          <t>10.2 statuses on stats</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>While active it changes slash resistance of the unit: read when its stats are recomputed; the arithmetic is not followed</t>
+          <t>While active adds int(value) to slash resistance</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>0x4fbc40</t>
+          <t>0x4fc0f9</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>partly</t>
+          <t>read</t>
         </is>
       </c>
     </row>
@@ -20220,22 +20240,22 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>10 stats of a character</t>
+          <t>10.2 statuses on stats</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>While active it changes bash resistance of the unit: read when its stats are recomputed; the arithmetic is not followed</t>
+          <t>While active adds int(value) to bash resistance</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>0x4fbc40</t>
+          <t>0x4fc122</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>partly</t>
+          <t>read</t>
         </is>
       </c>
     </row>
@@ -20245,22 +20265,22 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>10 stats of a character</t>
+          <t>10.2 statuses on stats</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>While active it changes a resistance of the unit: read when its stats are recomputed; the arithmetic is not followed</t>
+          <t>While active adds int(value) to each of the five elemental resistances</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>0x4fbc40</t>
+          <t>0x4fc23d</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>partly</t>
+          <t>read</t>
         </is>
       </c>
     </row>
@@ -20734,6 +20754,581 @@
         </is>
       </c>
       <c r="E92" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="n">
+        <v>8</v>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>2.7 special damage</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Fixed damage: the damage is int(value), whatever attack and defence say</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>0x44f758</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="n">
+        <v>12</v>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>2.7 special damage</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Self-destruct: the damage is int(user's current HP * value)</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>0x44f7a8</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="n">
+        <v>138</v>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>2.7 special damage</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Damage = target's max HP * value * the resistance factor of the element of the attack ((100 - resistance * 0.5) * 0.01)</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>0x44f858</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="n">
+        <v>140</v>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>2.7 special damage</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Halves HP: the damage is half the target's current HP. Against an enemy only when a byte of its object (0xa5) allows it</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>0x44f989</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="n">
+        <v>141</v>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>2.7 special damage</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>The damage is three quarters of the target's current HP, with the same condition as 140</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>0x44f9ec</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="n">
+        <v>142</v>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>2.7 special damage</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Reduces HP to 1: the damage is the target's current HP - 1</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>0x44fa4a</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="n">
+        <v>434</v>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>2.7 special damage</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>The damage is the user's current HP - 1</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>0x44fa6a</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="n">
+        <v>435</v>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>2.7 special damage</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>The damage is int(user's level * value)</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>0x44fa9f</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="n">
+        <v>190</v>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>2.7 special damage</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Limit Field: asked on the target after a special damage is chosen and again in the magic function; what it changes is not followed</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>0x44fb1c, 0x44ed53</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>partly</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="n">
+        <v>48</v>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>10.2 statuses on stats</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Trump Card: while active ATK gains int(DEF * value) and the DEF bonus is set to -10,000</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>0x4fbfca</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="n">
+        <v>189</v>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>10.2 statuses on stats</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>While active each of the six stats gains stat * value</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>0x4fc14b</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="n">
+        <v>193</v>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>10.2 statuses on stats</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>While active each of the six stats gains stat * value</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>0x4fc15e</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="n">
+        <v>194</v>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>10.2 statuses on stats</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>While active each of the six stats gains stat * value</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>0x4fc171</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="n">
+        <v>202</v>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>10.2 statuses on stats</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>While active adds int(value) to each of the five elemental resistances</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>0x4fc1f1</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="n">
+        <v>341</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>10.2 statuses on stats</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>While active adds int(value) to each of the five elemental resistances (an enemy debuff: the value is negative)</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>0x4fc204</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="n">
+        <v>256</v>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>10.2 statuses on stats</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Lefty Bonus: read at the end of the same recomputation; its arithmetic is not followed</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>0x4fc276</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>partly</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="n">
+        <v>192</v>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>10.2 statuses on stats</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>All Resistances 100: its own command only; where the resistances are set is not followed</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>0x487540</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>partly</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="n">
+        <v>41</v>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>10.2 statuses on stats</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>While active ATK gains int(ATK * value): a buff or debuff of the stat itself</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>0x4fbe0a - 0x4fbf85</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="n">
+        <v>42</v>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>10.2 statuses on stats</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>While active DEF gains int(DEF * value): a buff or debuff of the stat itself</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>0x4fbe0a - 0x4fbf85</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="n">
+        <v>43</v>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>10.2 statuses on stats</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>While active INT gains int(INT * value): a buff or debuff of the stat itself</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>0x4fbe0a - 0x4fbf85</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="n">
+        <v>44</v>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>10.2 statuses on stats</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>While active RES gains int(RES * value): a buff or debuff of the stat itself</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>0x4fbe0a - 0x4fbf85</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="n">
+        <v>45</v>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>10.2 statuses on stats</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>While active DEX gains int(DEX * value): a buff or debuff of the stat itself</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>0x4fbe0a - 0x4fbf85</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="n">
+        <v>46</v>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>10.2 statuses on stats</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>While active AGI gains int(AGI * value): a buff or debuff of the stat itself</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>0x4fbe0a - 0x4fbf85</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
         <is>
           <t>read</t>
         </is>

</xml_diff>

<commit_message>
feat: every command class decoded through the switch of CreateCommand
every command class decoded through the switch of CreateCommand; plain
classes told apart
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -8841,11 +8841,6 @@
           <t>6b healing</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>0x47fb70</t>
-        </is>
-      </c>
       <c r="H7" t="inlineStr"/>
     </row>
     <row r="8">
@@ -8873,11 +8868,6 @@
           <t>actions</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>0x47fc30</t>
-        </is>
-      </c>
       <c r="H8" t="inlineStr"/>
     </row>
     <row r="9">
@@ -8905,11 +8895,6 @@
           <t>actions</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>0x47fd00</t>
-        </is>
-      </c>
       <c r="H9" t="inlineStr"/>
     </row>
     <row r="10">
@@ -8964,11 +8949,6 @@
           <t>outside battle</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>0x47fde0</t>
-        </is>
-      </c>
       <c r="H11" t="inlineStr"/>
     </row>
     <row r="12">
@@ -8988,7 +8968,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>read</t>
+          <t>not found</t>
         </is>
       </c>
       <c r="F12" t="inlineStr"/>
@@ -9124,7 +9104,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>read</t>
+          <t>not found</t>
         </is>
       </c>
       <c r="F17" t="inlineStr"/>
@@ -9319,7 +9299,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>0x48bd60</t>
+          <t>0x480e20</t>
         </is>
       </c>
       <c r="H24" t="inlineStr"/>
@@ -9530,10 +9510,15 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>read</t>
+          <t>located</t>
         </is>
       </c>
       <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>0x480e20</t>
+        </is>
+      </c>
       <c r="H32" t="inlineStr"/>
     </row>
     <row r="33">
@@ -10289,6 +10274,11 @@
         </is>
       </c>
       <c r="F60" t="inlineStr"/>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>0x4817c0</t>
+        </is>
+      </c>
       <c r="H60" t="inlineStr">
         <is>
           <t>0x41f947</t>
@@ -10316,6 +10306,11 @@
         </is>
       </c>
       <c r="F61" t="inlineStr"/>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>0x4817c0</t>
+        </is>
+      </c>
       <c r="H61" t="inlineStr">
         <is>
           <t>0x41faaf</t>
@@ -10475,11 +10470,6 @@
           <t>outside battle</t>
         </is>
       </c>
-      <c r="G66" t="inlineStr">
-        <is>
-          <t>0x47fde0</t>
-        </is>
-      </c>
       <c r="H66" t="inlineStr"/>
     </row>
     <row r="67">
@@ -10507,11 +10497,6 @@
           <t>outside battle</t>
         </is>
       </c>
-      <c r="G67" t="inlineStr">
-        <is>
-          <t>0x481d80</t>
-        </is>
-      </c>
       <c r="H67" t="inlineStr"/>
     </row>
     <row r="68">
@@ -10622,7 +10607,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>0x481ea0</t>
+          <t>0x4822c0</t>
         </is>
       </c>
       <c r="H71" t="inlineStr"/>
@@ -10654,7 +10639,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>0x4822c0</t>
+          <t>0x482530</t>
         </is>
       </c>
       <c r="H72" t="inlineStr"/>
@@ -10686,7 +10671,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>0x482530</t>
+          <t>0x4827a0</t>
         </is>
       </c>
       <c r="H73" t="inlineStr"/>
@@ -10718,7 +10703,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>0x4827a0</t>
+          <t>0x482a10</t>
         </is>
       </c>
       <c r="H74" t="inlineStr"/>
@@ -10750,7 +10735,7 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>0x482a10</t>
+          <t>0x482e40</t>
         </is>
       </c>
       <c r="H75" t="inlineStr"/>
@@ -10782,7 +10767,7 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>0x482c80</t>
+          <t>0x482e40</t>
         </is>
       </c>
       <c r="H76" t="inlineStr"/>
@@ -10846,7 +10831,7 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>0x4831f0</t>
+          <t>0x4834b0</t>
         </is>
       </c>
       <c r="H78" t="inlineStr"/>
@@ -10874,7 +10859,7 @@
       <c r="F79" t="inlineStr"/>
       <c r="G79" t="inlineStr">
         <is>
-          <t>0x4834b0</t>
+          <t>0x4835d0</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
@@ -10910,7 +10895,7 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>0x4835d0</t>
+          <t>0x483a60</t>
         </is>
       </c>
       <c r="H80" t="inlineStr"/>
@@ -10938,7 +10923,7 @@
       <c r="F81" t="inlineStr"/>
       <c r="G81" t="inlineStr">
         <is>
-          <t>0x483840</t>
+          <t>0x483a60</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
@@ -11023,15 +11008,10 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>read</t>
+          <t>not found</t>
         </is>
       </c>
       <c r="F84" t="inlineStr"/>
-      <c r="G84" t="inlineStr">
-        <is>
-          <t>0x483b30</t>
-        </is>
-      </c>
       <c r="H84" t="inlineStr"/>
     </row>
     <row r="85">
@@ -11051,15 +11031,10 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>read</t>
+          <t>not found</t>
         </is>
       </c>
       <c r="F85" t="inlineStr"/>
-      <c r="G85" t="inlineStr">
-        <is>
-          <t>0x483c20</t>
-        </is>
-      </c>
       <c r="H85" t="inlineStr"/>
     </row>
     <row r="86">
@@ -11087,11 +11062,6 @@
           <t>6d recovery</t>
         </is>
       </c>
-      <c r="G86" t="inlineStr">
-        <is>
-          <t>0x483d20</t>
-        </is>
-      </c>
       <c r="H86" t="inlineStr"/>
     </row>
     <row r="87">
@@ -11143,15 +11113,10 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>read</t>
+          <t>not found</t>
         </is>
       </c>
       <c r="F88" t="inlineStr"/>
-      <c r="G88" t="inlineStr">
-        <is>
-          <t>0x483ee0</t>
-        </is>
-      </c>
       <c r="H88" t="inlineStr"/>
     </row>
     <row r="89">
@@ -11334,7 +11299,7 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>read</t>
+          <t>located</t>
         </is>
       </c>
       <c r="F95" t="inlineStr"/>
@@ -11729,12 +11694,17 @@
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>read</t>
+          <t>located</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
         <is>
           <t>3 magic attack</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>0x4864c0</t>
         </is>
       </c>
       <c r="H110" t="inlineStr"/>
@@ -11764,11 +11734,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="G111" t="inlineStr">
-        <is>
-          <t>0x4864c0</t>
-        </is>
-      </c>
       <c r="H111" t="inlineStr"/>
     </row>
     <row r="112">
@@ -11931,11 +11896,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="G117" t="inlineStr">
-        <is>
-          <t>0x4869c0</t>
-        </is>
-      </c>
       <c r="H117" t="inlineStr"/>
     </row>
     <row r="118">
@@ -12013,11 +11973,6 @@
         </is>
       </c>
       <c r="F120" t="inlineStr"/>
-      <c r="G120" t="inlineStr">
-        <is>
-          <t>0x486c70</t>
-        </is>
-      </c>
       <c r="H120" t="inlineStr">
         <is>
           <t>0x41fbd0</t>
@@ -12041,15 +11996,10 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>located</t>
+          <t>not found</t>
         </is>
       </c>
       <c r="F121" t="inlineStr"/>
-      <c r="G121" t="inlineStr">
-        <is>
-          <t>0x486e70</t>
-        </is>
-      </c>
       <c r="H121" t="inlineStr"/>
     </row>
     <row r="122">
@@ -12069,7 +12019,7 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>read</t>
+          <t>not found</t>
         </is>
       </c>
       <c r="F122" t="inlineStr"/>
@@ -12281,7 +12231,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>read</t>
+          <t>not found</t>
         </is>
       </c>
       <c r="F130" t="inlineStr"/>
@@ -12312,11 +12262,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="G131" t="inlineStr">
-        <is>
-          <t>0x487540</t>
-        </is>
-      </c>
       <c r="H131" t="inlineStr"/>
     </row>
     <row r="132">
@@ -12344,11 +12289,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="G132" t="inlineStr">
-        <is>
-          <t>0x487780</t>
-        </is>
-      </c>
       <c r="H132" t="inlineStr"/>
     </row>
     <row r="133">
@@ -12376,11 +12316,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="G133" t="inlineStr">
-        <is>
-          <t>0x4879d0</t>
-        </is>
-      </c>
       <c r="H133" t="inlineStr"/>
     </row>
     <row r="134">
@@ -12400,17 +12335,12 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>located</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
         <is>
           <t>2 physical attack, 3 magic attack</t>
-        </is>
-      </c>
-      <c r="G134" t="inlineStr">
-        <is>
-          <t>0x487bd0</t>
         </is>
       </c>
       <c r="H134" t="inlineStr"/>
@@ -12432,17 +12362,12 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>located</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
         <is>
           <t>2 physical attack, 3 magic attack</t>
-        </is>
-      </c>
-      <c r="G135" t="inlineStr">
-        <is>
-          <t>0x487e00</t>
         </is>
       </c>
       <c r="H135" t="inlineStr"/>
@@ -12464,17 +12389,12 @@
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>located</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
         <is>
           <t>2 physical attack, 3 magic attack</t>
-        </is>
-      </c>
-      <c r="G136" t="inlineStr">
-        <is>
-          <t>0x488000</t>
         </is>
       </c>
       <c r="H136" t="inlineStr"/>
@@ -12496,17 +12416,12 @@
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>located</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F137" t="inlineStr">
         <is>
           <t>2 physical attack, 3 magic attack</t>
-        </is>
-      </c>
-      <c r="G137" t="inlineStr">
-        <is>
-          <t>0x488200</t>
         </is>
       </c>
       <c r="H137" t="inlineStr"/>
@@ -12555,7 +12470,7 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>read</t>
+          <t>not found</t>
         </is>
       </c>
       <c r="F139" t="inlineStr"/>
@@ -12578,17 +12493,12 @@
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>located</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
         <is>
           <t>5 order of turns</t>
-        </is>
-      </c>
-      <c r="G140" t="inlineStr">
-        <is>
-          <t>0x4884f0</t>
         </is>
       </c>
       <c r="H140" t="inlineStr"/>
@@ -12618,11 +12528,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="G141" t="inlineStr">
-        <is>
-          <t>0x4886f0</t>
-        </is>
-      </c>
       <c r="H141" t="inlineStr"/>
     </row>
     <row r="142">
@@ -12642,7 +12547,7 @@
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>read</t>
+          <t>not found</t>
         </is>
       </c>
       <c r="F142" t="inlineStr"/>
@@ -12665,7 +12570,7 @@
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>read</t>
+          <t>not found</t>
         </is>
       </c>
       <c r="F143" t="inlineStr"/>
@@ -12688,17 +12593,12 @@
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>located</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F144" t="inlineStr">
         <is>
           <t>2 physical attack, 3 magic attack</t>
-        </is>
-      </c>
-      <c r="G144" t="inlineStr">
-        <is>
-          <t>0x487e00</t>
         </is>
       </c>
       <c r="H144" t="inlineStr"/>

</xml_diff>

<commit_message>
fix: a case of CreateCommand ends in a return
a case of CreateCommand ends in a return; an effect whose own command is
read counts as read
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -9297,11 +9297,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>0x480e20</t>
-        </is>
-      </c>
       <c r="H24" t="inlineStr"/>
     </row>
     <row r="25">
@@ -10274,11 +10269,6 @@
         </is>
       </c>
       <c r="F60" t="inlineStr"/>
-      <c r="G60" t="inlineStr">
-        <is>
-          <t>0x4817c0</t>
-        </is>
-      </c>
       <c r="H60" t="inlineStr">
         <is>
           <t>0x41f947</t>
@@ -10306,11 +10296,6 @@
         </is>
       </c>
       <c r="F61" t="inlineStr"/>
-      <c r="G61" t="inlineStr">
-        <is>
-          <t>0x4817c0</t>
-        </is>
-      </c>
       <c r="H61" t="inlineStr">
         <is>
           <t>0x41faaf</t>
@@ -10339,7 +10324,7 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>6b healing</t>
+          <t>6b healing, 6b, 6d recovery</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -10371,7 +10356,7 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>6d recovery</t>
+          <t>6b, 6d recovery, 6d recovery</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -10403,7 +10388,7 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>6d recovery</t>
+          <t>6b, 6d recovery, 6d recovery</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -10607,7 +10592,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>0x4822c0</t>
+          <t>0x481ea0</t>
         </is>
       </c>
       <c r="H71" t="inlineStr"/>
@@ -10639,7 +10624,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>0x482530</t>
+          <t>0x4822c0</t>
         </is>
       </c>
       <c r="H72" t="inlineStr"/>
@@ -10671,7 +10656,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>0x4827a0</t>
+          <t>0x482530</t>
         </is>
       </c>
       <c r="H73" t="inlineStr"/>
@@ -10703,7 +10688,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>0x482a10</t>
+          <t>0x4827a0</t>
         </is>
       </c>
       <c r="H74" t="inlineStr"/>
@@ -10735,7 +10720,7 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>0x482e40</t>
+          <t>0x482a10</t>
         </is>
       </c>
       <c r="H75" t="inlineStr"/>
@@ -10767,7 +10752,7 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>0x482e40</t>
+          <t>0x482c80</t>
         </is>
       </c>
       <c r="H76" t="inlineStr"/>
@@ -10831,7 +10816,7 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>0x4834b0</t>
+          <t>0x4831f0</t>
         </is>
       </c>
       <c r="H78" t="inlineStr"/>
@@ -10856,10 +10841,14 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F79" t="inlineStr"/>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>5b ailments</t>
+        </is>
+      </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>0x4835d0</t>
+          <t>0x4834b0</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
@@ -10895,7 +10884,7 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>0x483a60</t>
+          <t>0x4835d0</t>
         </is>
       </c>
       <c r="H80" t="inlineStr"/>
@@ -10920,10 +10909,14 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F81" t="inlineStr"/>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>5b ailments</t>
+        </is>
+      </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>0x483a60</t>
+          <t>0x483840</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
@@ -11008,10 +11001,19 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>not found</t>
-        </is>
-      </c>
-      <c r="F84" t="inlineStr"/>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>6d recovery</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>0x483b30</t>
+        </is>
+      </c>
       <c r="H84" t="inlineStr"/>
     </row>
     <row r="85">
@@ -11031,10 +11033,19 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>not found</t>
-        </is>
-      </c>
-      <c r="F85" t="inlineStr"/>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>6d recovery</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>0x483c20</t>
+        </is>
+      </c>
       <c r="H85" t="inlineStr"/>
     </row>
     <row r="86">
@@ -11062,6 +11073,11 @@
           <t>6d recovery</t>
         </is>
       </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>0x483d20</t>
+        </is>
+      </c>
       <c r="H86" t="inlineStr"/>
     </row>
     <row r="87">
@@ -11084,7 +11100,11 @@
           <t>located</t>
         </is>
       </c>
-      <c r="F87" t="inlineStr"/>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>6d recovery</t>
+        </is>
+      </c>
       <c r="G87" t="inlineStr">
         <is>
           <t>0x483e00</t>
@@ -11113,10 +11133,19 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>not found</t>
-        </is>
-      </c>
-      <c r="F88" t="inlineStr"/>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>6d recovery</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>0x483ee0</t>
+        </is>
+      </c>
       <c r="H88" t="inlineStr"/>
     </row>
     <row r="89">
@@ -11299,10 +11328,14 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F95" t="inlineStr"/>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>11.1 dolls</t>
+        </is>
+      </c>
       <c r="G95" t="inlineStr">
         <is>
           <t>0x484150</t>
@@ -11694,17 +11727,12 @@
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>located</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
         <is>
           <t>3 magic attack</t>
-        </is>
-      </c>
-      <c r="G110" t="inlineStr">
-        <is>
-          <t>0x4864c0</t>
         </is>
       </c>
       <c r="H110" t="inlineStr"/>
@@ -11732,6 +11760,11 @@
       <c r="F111" t="inlineStr">
         <is>
           <t>5 order of turns</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>0x4864c0</t>
         </is>
       </c>
       <c r="H111" t="inlineStr"/>

</xml_diff>

<commit_message>
feat: rules of damage received
rules of damage received, song and dance bonus and the start of a turn
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -8785,7 +8785,7 @@
       <c r="F5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
-          <t>0x422a18, 0x47f5fc, 0x47f633</t>
+          <t>0x422a18, 0x47f5fc, 0x47f633, 0x5b8b7a</t>
         </is>
       </c>
     </row>
@@ -10879,7 +10879,7 @@
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>5b ailments</t>
+          <t>5 order of turns, 5b ailments</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
@@ -11846,7 +11846,7 @@
       <c r="F114" t="inlineStr"/>
       <c r="H114" t="inlineStr">
         <is>
-          <t>0x420cac</t>
+          <t>0x420c48, 0x420cac, 0x42497a</t>
         </is>
       </c>
     </row>
@@ -12029,11 +12029,15 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>not found</t>
+          <t>located</t>
         </is>
       </c>
       <c r="F121" t="inlineStr"/>
-      <c r="H121" t="inlineStr"/>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>0x421c93</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="n">
@@ -12183,15 +12187,15 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F127" t="inlineStr"/>
-      <c r="H127" t="inlineStr">
-        <is>
-          <t>0x47f936</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>2.8 damage received</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="n">
@@ -12580,10 +12584,14 @@
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>not found</t>
-        </is>
-      </c>
-      <c r="F142" t="inlineStr"/>
+          <t>partly read</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>5d start of a turn</t>
+        </is>
+      </c>
       <c r="H142" t="inlineStr"/>
     </row>
     <row r="143">
@@ -12857,11 +12865,15 @@
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>not found</t>
+          <t>located</t>
         </is>
       </c>
       <c r="F153" t="inlineStr"/>
-      <c r="H153" t="inlineStr"/>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>0x439380</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="n">
@@ -13570,15 +13582,15 @@
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F180" t="inlineStr"/>
-      <c r="H180" t="inlineStr">
-        <is>
-          <t>0x47e64d</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>2.8 damage received</t>
+        </is>
+      </c>
+      <c r="H180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" t="n">
@@ -13624,10 +13636,14 @@
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>not found</t>
-        </is>
-      </c>
-      <c r="F182" t="inlineStr"/>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>5d start of a turn</t>
+        </is>
+      </c>
       <c r="H182" t="inlineStr"/>
     </row>
     <row r="183">
@@ -13647,11 +13663,15 @@
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>not found</t>
+          <t>located</t>
         </is>
       </c>
       <c r="F183" t="inlineStr"/>
-      <c r="H183" t="inlineStr"/>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>0x42540a</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="n">
@@ -13670,19 +13690,15 @@
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>located</t>
+          <t>partly read</t>
         </is>
       </c>
       <c r="F184" t="inlineStr">
         <is>
-          <t>5 order of turns</t>
-        </is>
-      </c>
-      <c r="H184" t="inlineStr">
-        <is>
-          <t>0x47f8aa</t>
-        </is>
-      </c>
+          <t>2.8 damage received, 5 order of turns</t>
+        </is>
+      </c>
+      <c r="H184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="n">
@@ -14152,10 +14168,14 @@
       </c>
       <c r="E202" t="inlineStr">
         <is>
-          <t>not found</t>
-        </is>
-      </c>
-      <c r="F202" t="inlineStr"/>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F202" t="inlineStr">
+        <is>
+          <t>11.2 songs and dances</t>
+        </is>
+      </c>
       <c r="H202" t="inlineStr"/>
     </row>
     <row r="203">
@@ -14175,10 +14195,14 @@
       </c>
       <c r="E203" t="inlineStr">
         <is>
-          <t>not found</t>
-        </is>
-      </c>
-      <c r="F203" t="inlineStr"/>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F203" t="inlineStr">
+        <is>
+          <t>11.2 songs and dances</t>
+        </is>
+      </c>
       <c r="H203" t="inlineStr"/>
     </row>
     <row r="204">
@@ -14248,10 +14272,14 @@
       </c>
       <c r="E206" t="inlineStr">
         <is>
-          <t>not found</t>
-        </is>
-      </c>
-      <c r="F206" t="inlineStr"/>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t>5d start of a turn</t>
+        </is>
+      </c>
       <c r="H206" t="inlineStr"/>
     </row>
     <row r="207">
@@ -14271,11 +14299,15 @@
       </c>
       <c r="E207" t="inlineStr">
         <is>
-          <t>not found</t>
+          <t>located</t>
         </is>
       </c>
       <c r="F207" t="inlineStr"/>
-      <c r="H207" t="inlineStr"/>
+      <c r="H207" t="inlineStr">
+        <is>
+          <t>0x43c47e, 0x43ccc8</t>
+        </is>
+      </c>
     </row>
     <row r="208">
       <c r="A208" t="n">
@@ -14348,11 +14380,15 @@
       </c>
       <c r="E210" t="inlineStr">
         <is>
-          <t>not found</t>
+          <t>located</t>
         </is>
       </c>
       <c r="F210" t="inlineStr"/>
-      <c r="H210" t="inlineStr"/>
+      <c r="H210" t="inlineStr">
+        <is>
+          <t>0x43bfbd</t>
+        </is>
+      </c>
     </row>
     <row r="211">
       <c r="A211" t="n">
@@ -14371,11 +14407,15 @@
       </c>
       <c r="E211" t="inlineStr">
         <is>
-          <t>not found</t>
+          <t>located</t>
         </is>
       </c>
       <c r="F211" t="inlineStr"/>
-      <c r="H211" t="inlineStr"/>
+      <c r="H211" t="inlineStr">
+        <is>
+          <t>0x439072</t>
+        </is>
+      </c>
     </row>
     <row r="212">
       <c r="A212" t="n">
@@ -14394,11 +14434,15 @@
       </c>
       <c r="E212" t="inlineStr">
         <is>
-          <t>not found</t>
+          <t>located</t>
         </is>
       </c>
       <c r="F212" t="inlineStr"/>
-      <c r="H212" t="inlineStr"/>
+      <c r="H212" t="inlineStr">
+        <is>
+          <t>0x4390b9</t>
+        </is>
+      </c>
     </row>
     <row r="213">
       <c r="A213" t="n">
@@ -14423,7 +14467,7 @@
       <c r="F213" t="inlineStr"/>
       <c r="H213" t="inlineStr">
         <is>
-          <t>0x47f739</t>
+          <t>0x438e53, 0x47f739</t>
         </is>
       </c>
     </row>
@@ -14660,11 +14704,15 @@
       </c>
       <c r="E222" t="inlineStr">
         <is>
-          <t>not found</t>
+          <t>located</t>
         </is>
       </c>
       <c r="F222" t="inlineStr"/>
-      <c r="H222" t="inlineStr"/>
+      <c r="H222" t="inlineStr">
+        <is>
+          <t>0x423d7a</t>
+        </is>
+      </c>
     </row>
     <row r="223">
       <c r="A223" t="n">
@@ -14737,11 +14785,15 @@
       </c>
       <c r="E225" t="inlineStr">
         <is>
-          <t>not found</t>
+          <t>located</t>
         </is>
       </c>
       <c r="F225" t="inlineStr"/>
-      <c r="H225" t="inlineStr"/>
+      <c r="H225" t="inlineStr">
+        <is>
+          <t>0x4203b4, 0x422582, 0x4246c2, 0x424739</t>
+        </is>
+      </c>
     </row>
     <row r="226">
       <c r="A226" t="n">
@@ -14837,11 +14889,15 @@
       </c>
       <c r="E229" t="inlineStr">
         <is>
-          <t>not found</t>
+          <t>located</t>
         </is>
       </c>
       <c r="F229" t="inlineStr"/>
-      <c r="H229" t="inlineStr"/>
+      <c r="H229" t="inlineStr">
+        <is>
+          <t>0x436727</t>
+        </is>
+      </c>
     </row>
     <row r="230">
       <c r="A230" t="n">
@@ -14887,11 +14943,15 @@
       </c>
       <c r="E231" t="inlineStr">
         <is>
-          <t>not found</t>
+          <t>located</t>
         </is>
       </c>
       <c r="F231" t="inlineStr"/>
-      <c r="H231" t="inlineStr"/>
+      <c r="H231" t="inlineStr">
+        <is>
+          <t>0x43c920</t>
+        </is>
+      </c>
     </row>
     <row r="232">
       <c r="A232" t="n">
@@ -14937,11 +14997,15 @@
       </c>
       <c r="E233" t="inlineStr">
         <is>
-          <t>not found</t>
+          <t>located</t>
         </is>
       </c>
       <c r="F233" t="inlineStr"/>
-      <c r="H233" t="inlineStr"/>
+      <c r="H233" t="inlineStr">
+        <is>
+          <t>0x42db82</t>
+        </is>
+      </c>
     </row>
     <row r="234">
       <c r="A234" t="n">
@@ -15014,11 +15078,15 @@
       </c>
       <c r="E236" t="inlineStr">
         <is>
-          <t>not found</t>
+          <t>located</t>
         </is>
       </c>
       <c r="F236" t="inlineStr"/>
-      <c r="H236" t="inlineStr"/>
+      <c r="H236" t="inlineStr">
+        <is>
+          <t>0x43736a</t>
+        </is>
+      </c>
     </row>
     <row r="237">
       <c r="A237" t="n">
@@ -15091,7 +15159,7 @@
       </c>
       <c r="E239" t="inlineStr">
         <is>
-          <t>read</t>
+          <t>located</t>
         </is>
       </c>
       <c r="F239" t="inlineStr">
@@ -15099,7 +15167,11 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H239" t="inlineStr"/>
+      <c r="H239" t="inlineStr">
+        <is>
+          <t>0x4161f5, 0x4164bf, 0x4167cf, 0x416adf, 0x416def</t>
+        </is>
+      </c>
     </row>
     <row r="240">
       <c r="A240" t="n">
@@ -15118,7 +15190,7 @@
       </c>
       <c r="E240" t="inlineStr">
         <is>
-          <t>read</t>
+          <t>located</t>
         </is>
       </c>
       <c r="F240" t="inlineStr">
@@ -15126,7 +15198,11 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H240" t="inlineStr"/>
+      <c r="H240" t="inlineStr">
+        <is>
+          <t>0x4161af, 0x416505, 0x4167df, 0x416aef, 0x416dff</t>
+        </is>
+      </c>
     </row>
     <row r="241">
       <c r="A241" t="n">
@@ -15145,7 +15221,7 @@
       </c>
       <c r="E241" t="inlineStr">
         <is>
-          <t>read</t>
+          <t>located</t>
         </is>
       </c>
       <c r="F241" t="inlineStr">
@@ -15153,7 +15229,11 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H241" t="inlineStr"/>
+      <c r="H241" t="inlineStr">
+        <is>
+          <t>0x4161bf, 0x4164cf, 0x4167f1, 0x416b01, 0x416e35</t>
+        </is>
+      </c>
     </row>
     <row r="242">
       <c r="A242" t="n">
@@ -15172,7 +15252,7 @@
       </c>
       <c r="E242" t="inlineStr">
         <is>
-          <t>read</t>
+          <t>located</t>
         </is>
       </c>
       <c r="F242" t="inlineStr">
@@ -15180,7 +15260,11 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H242" t="inlineStr"/>
+      <c r="H242" t="inlineStr">
+        <is>
+          <t>0x4161d1, 0x4164e1, 0x416815, 0x416b13, 0x416e11</t>
+        </is>
+      </c>
     </row>
     <row r="243">
       <c r="A243" t="n">
@@ -15199,7 +15283,7 @@
       </c>
       <c r="E243" t="inlineStr">
         <is>
-          <t>read</t>
+          <t>located</t>
         </is>
       </c>
       <c r="F243" t="inlineStr">
@@ -15207,7 +15291,11 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H243" t="inlineStr"/>
+      <c r="H243" t="inlineStr">
+        <is>
+          <t>0x4161e3, 0x4164f3, 0x416803, 0x416b25, 0x416e23</t>
+        </is>
+      </c>
     </row>
     <row r="244">
       <c r="A244" t="n">
@@ -18480,7 +18568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E115"/>
+  <dimension ref="A1:E123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -21267,6 +21355,206 @@
         </is>
       </c>
     </row>
+    <row r="116">
+      <c r="A116" t="n">
+        <v>257</v>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>2.8 damage received</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>TP Conversion: when its bearer takes damage it gains int(damage * value) TP, at least 1. Pieces of enchantment 72 and 73 add int(damage * min(0.5, 0.05 * pieces of 72 + 0.1 * pieces of 73)), at least 1 (5 with a piece of 73)</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>0x47e64d - 0x47e72e</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="n">
+        <v>188</v>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>2.8 damage received</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Resuscitate: when its bearer falls it rises again with int(max HP * value) HP</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>0x47f93d</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="n">
+        <v>261</v>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>2.8 damage received</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Stamina: after damage, when HP is at or below a share of max HP and the status is present, its command is run (0x48c1d0); the same status is a speed bonus while HP is at or below 40% (5)</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>0x47f8b3, 0x4499d0</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>partly</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="n">
+        <v>279</v>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>11.2 songs and dances</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Song Bonus: a song is applied with its value plus the value of this status of the singer plus min(0.05, 0.02 * pieces of enchantment 300 + 0.01 * pieces of 301)</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>0x48bf90</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="n">
+        <v>280</v>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>11.2 songs and dances</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Dance Bonus: as 279 for a dance, with enchantments 302 and 303</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>0x48bf90</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="n">
+        <v>259</v>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>5d start of a turn</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Warning Shot: when a unit is about to act, each opponent that has it rolls below 100 under value * 100; a success takes the turn away. The final damage of the bearer is also cut to 3/10 (4)</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>0x436d89, 0x44caed</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="n">
+        <v>283</v>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>5d start of a turn</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Mesmerized: when a unit is about to act, a roll below 100 under value * 100 for each opponent that has it; a success takes the turn away</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>0x436e2d</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="n">
+        <v>203</v>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>5d start of a turn</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Erotic Dance: the same roll at the start of a turn, on the dancer among the opponents (debug message of the dance)</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>0x436ee0</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>partly</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: effect coverage sees the small constructors and two more lookup
effect coverage sees the small constructors and two more lookup
functions
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -11165,10 +11165,14 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>not found</t>
-        </is>
-      </c>
-      <c r="F89" t="inlineStr"/>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>2 physical attack</t>
+        </is>
+      </c>
       <c r="H89" t="inlineStr"/>
     </row>
     <row r="90">
@@ -12246,7 +12250,7 @@
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>2.7 special damage, 3 magic attack</t>
+          <t>2 physical attack, 2.7 special damage, 3 magic attack</t>
         </is>
       </c>
       <c r="H129" t="inlineStr"/>
@@ -12268,10 +12272,14 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>not found</t>
-        </is>
-      </c>
-      <c r="F130" t="inlineStr"/>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>2 physical attack</t>
+        </is>
+      </c>
       <c r="H130" t="inlineStr"/>
     </row>
     <row r="131">
@@ -13189,10 +13197,15 @@
       </c>
       <c r="E165" t="inlineStr">
         <is>
-          <t>not found</t>
+          <t>located</t>
         </is>
       </c>
       <c r="F165" t="inlineStr"/>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>0x48a430</t>
+        </is>
+      </c>
       <c r="H165" t="inlineStr"/>
     </row>
     <row r="166">
@@ -13636,7 +13649,7 @@
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>read</t>
+          <t>partly read</t>
         </is>
       </c>
       <c r="F182" t="inlineStr">
@@ -13933,11 +13946,15 @@
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>not found</t>
+          <t>located</t>
         </is>
       </c>
       <c r="F193" t="inlineStr"/>
-      <c r="H193" t="inlineStr"/>
+      <c r="H193" t="inlineStr">
+        <is>
+          <t>0x5581ff</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" t="n">
@@ -13956,11 +13973,15 @@
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>not found</t>
+          <t>located</t>
         </is>
       </c>
       <c r="F194" t="inlineStr"/>
-      <c r="H194" t="inlineStr"/>
+      <c r="H194" t="inlineStr">
+        <is>
+          <t>0x43aa33</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="n">
@@ -14249,11 +14270,15 @@
       </c>
       <c r="E205" t="inlineStr">
         <is>
-          <t>not found</t>
+          <t>located</t>
         </is>
       </c>
       <c r="F205" t="inlineStr"/>
-      <c r="H205" t="inlineStr"/>
+      <c r="H205" t="inlineStr">
+        <is>
+          <t>0x4762d2</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" t="n">
@@ -14272,7 +14297,7 @@
       </c>
       <c r="E206" t="inlineStr">
         <is>
-          <t>read</t>
+          <t>partly read</t>
         </is>
       </c>
       <c r="F206" t="inlineStr">
@@ -14812,10 +14837,14 @@
       </c>
       <c r="E226" t="inlineStr">
         <is>
-          <t>not found</t>
-        </is>
-      </c>
-      <c r="F226" t="inlineStr"/>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F226" t="inlineStr">
+        <is>
+          <t>2 physical attack</t>
+        </is>
+      </c>
       <c r="H226" t="inlineStr"/>
     </row>
     <row r="227">
@@ -15622,10 +15651,15 @@
       </c>
       <c r="E256" t="inlineStr">
         <is>
-          <t>not found</t>
+          <t>located</t>
         </is>
       </c>
       <c r="F256" t="inlineStr"/>
+      <c r="G256" t="inlineStr">
+        <is>
+          <t>0x48b490</t>
+        </is>
+      </c>
       <c r="H256" t="inlineStr"/>
     </row>
     <row r="257">
@@ -21491,17 +21525,17 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Warning Shot: when a unit is about to act, each opponent that has it rolls below 100 under value * 100; a success takes the turn away. The final damage of the bearer is also cut to 3/10 (4)</t>
+          <t>Warning Shot: when a unit is about to act, each opponent that has it rolls below 100 under value * 100; on a success the bearer fires its shot (its final damage is cut to 3/10, section 4). Whether the unit then loses its turn is not followed</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>0x436d89, 0x44caed</t>
+          <t>0x436d89, 0x436f8b, 0x44caed</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>read</t>
+          <t>partly</t>
         </is>
       </c>
     </row>
@@ -21516,7 +21550,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Mesmerized: when a unit is about to act, a roll below 100 under value * 100 for each opponent that has it; a success takes the turn away</t>
+          <t>Mesmerized: when a unit is about to act, a roll below 100 under value * 100 for each opponent that has it; what a success does is not followed</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
@@ -21526,7 +21560,7 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>read</t>
+          <t>partly</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: effects that act every turn (regeneration, Carol, Chorale)
effects that act every turn (regeneration, Carol, Chorale); the coverage
looks at the per-turn method
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -12800,10 +12800,19 @@
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>not found</t>
-        </is>
-      </c>
-      <c r="F150" t="inlineStr"/>
+          <t>partly read</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>5e effects that act every turn</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>0x4894a0</t>
+        </is>
+      </c>
       <c r="H150" t="inlineStr"/>
     </row>
     <row r="151">
@@ -12823,10 +12832,19 @@
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>not found</t>
-        </is>
-      </c>
-      <c r="F151" t="inlineStr"/>
+          <t>partly read</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>5e effects that act every turn</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>0x4895e0</t>
+        </is>
+      </c>
       <c r="H151" t="inlineStr"/>
     </row>
     <row r="152">
@@ -13306,10 +13324,19 @@
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>not found</t>
-        </is>
-      </c>
-      <c r="F169" t="inlineStr"/>
+          <t>partly read</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>5e effects that act every turn</t>
+        </is>
+      </c>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>0x48a640</t>
+        </is>
+      </c>
       <c r="H169" t="inlineStr"/>
     </row>
     <row r="170">
@@ -13329,10 +13356,14 @@
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>not found</t>
-        </is>
-      </c>
-      <c r="F170" t="inlineStr"/>
+          <t>partly read</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>5e effects that act every turn</t>
+        </is>
+      </c>
       <c r="H170" t="inlineStr"/>
     </row>
     <row r="171">
@@ -18602,7 +18633,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E123"/>
+  <dimension ref="A1:E127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -21589,6 +21620,106 @@
         </is>
       </c>
     </row>
+    <row r="124">
+      <c r="A124" t="n">
+        <v>246</v>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>5e effects that act every turn</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>HP Regen: each time it ticks its bearer recovers int(max HP * value). When the tick fires is not followed</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>0x48a640</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>partly</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="n">
+        <v>247</v>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>5e effects that act every turn</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>TP Regen: each time it ticks its bearer (party side only) recovers int(value) TP. When the tick fires is not followed</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>0x48a710</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>partly</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="n">
+        <v>215</v>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>5e effects that act every turn</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Carol: each time it ticks it restores int(value * (1 + 10 * song bonus)), the song bonus being the one of effect 279. When the tick fires is not followed</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>0x4894a0</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>partly</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="n">
+        <v>216</v>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>5e effects that act every turn</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Chorale: each time it ticks it restores int(value + 100 * song bonus) TP to a member of the party. When the tick fires is not followed</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>0x4895e0</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>partly</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: how effects are built and handled (section 12)
how effects are built and handled (section 12); rules shown in the
generated coverage
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -18249,12 +18249,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>not read</t>
+          <t>partly</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Handles 29 effects; the largest single block</t>
+          <t>docs/FORMULAS.md 12: passive rolls on the target, barrier, dispel, absorption, the ailments of plain attacks and special damage are read; the order of the whole and several branches are not</t>
         </is>
       </c>
     </row>
@@ -18271,12 +18271,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>not read</t>
+          <t>partly</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Handles effects 89 to 100, 178, 210, 251, 252</t>
+          <t>docs/FORMULAS.md 12.2: every multi-hit table, Double and Triple Attack read; the number of targets (effect 137) not followed</t>
         </is>
       </c>
     </row>
@@ -18293,12 +18293,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>not read</t>
+          <t>partly</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Only the roll that applies each ailment is read</t>
+          <t>docs/FORMULAS.md 12.4 to 12.6: what stops a unit from acting, natural recovery, poison, statuses on stats; when the per-turn method runs is not followed</t>
         </is>
       </c>
     </row>
@@ -18315,12 +18315,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>not read</t>
+          <t>partly</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>The debug messages name each roll; the code of none is read</t>
+          <t>Rolls of Counter, Pretend, Knock Down, Auto-Guard, Reprisal, Survival, First Grid, Warning Shot, Mesmerized located and their chance read (sheet EffectRules); their consequences and the unique skills of the girls are not</t>
         </is>
       </c>
     </row>
@@ -18337,12 +18337,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>not read</t>
+          <t>partly</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Formulas add the buffs present; where they come from and go is not read</t>
+          <t>How an effect is built and applied is read (docs/FORMULAS.md 12.1); how long one lasts and whether two stack are not</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: rules of Power Charge, Imperial Guard, Dark Aura, Slow Target
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -12250,7 +12250,7 @@
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>2 physical attack, 2.7 special damage, 3 magic attack</t>
+          <t>2 physical attack, 2.4 other bonuses of final damage, 3 magic attack</t>
         </is>
       </c>
       <c r="H129" t="inlineStr"/>
@@ -12277,7 +12277,7 @@
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>2 physical attack</t>
+          <t>2 physical attack, 2.4 other bonuses of final damage</t>
         </is>
       </c>
       <c r="H130" t="inlineStr"/>
@@ -13761,15 +13761,15 @@
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F185" t="inlineStr"/>
-      <c r="H185" t="inlineStr">
-        <is>
-          <t>0x423d9b</t>
-        </is>
-      </c>
+          <t>partly read</t>
+        </is>
+      </c>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>12.9 after a hit</t>
+        </is>
+      </c>
+      <c r="H185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="n">
@@ -14544,12 +14544,12 @@
       </c>
       <c r="E214" t="inlineStr">
         <is>
-          <t>partly read</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F214" t="inlineStr">
         <is>
-          <t>passive rolls</t>
+          <t>12.9 after a hit</t>
         </is>
       </c>
       <c r="H214" t="inlineStr"/>
@@ -14760,15 +14760,15 @@
       </c>
       <c r="E222" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F222" t="inlineStr"/>
-      <c r="H222" t="inlineStr">
-        <is>
-          <t>0x423d7a</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F222" t="inlineStr">
+        <is>
+          <t>12.9 after a hit</t>
+        </is>
+      </c>
+      <c r="H222" t="inlineStr"/>
     </row>
     <row r="223">
       <c r="A223" t="n">
@@ -14873,7 +14873,7 @@
       </c>
       <c r="F226" t="inlineStr">
         <is>
-          <t>2 physical attack</t>
+          <t>2 physical attack, 2.4 other bonuses of final damage</t>
         </is>
       </c>
       <c r="H226" t="inlineStr"/>
@@ -15170,7 +15170,7 @@
       </c>
       <c r="F237" t="inlineStr">
         <is>
-          <t>applying a hit</t>
+          <t>12.9 after a hit</t>
         </is>
       </c>
       <c r="H237" t="inlineStr"/>
@@ -18633,7 +18633,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E127"/>
+  <dimension ref="A1:E131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -20526,22 +20526,22 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>passive rolls</t>
+          <t>12.9 after a hit</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>When the attacker has it: a roll below 100 under value * 100 slows its target</t>
+          <t>Slow Target: after a hit, a roll below 100 under value * 100 puts Slow on the target (value 1) and a speed modifier of -0.75</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>0x424319</t>
+          <t>0x424319 - 0x424579</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>partly</t>
+          <t>read</t>
         </is>
       </c>
     </row>
@@ -20701,12 +20701,12 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>applying a hit</t>
+          <t>12.9 after a hit</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Devil's Whisper: when present the apply code creates an instant death command</t>
+          <t>Devil's Whisper: when the action carries it the after-hit code creates an instant death command against the target; its chance is not followed</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -21051,17 +21051,17 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2.7 special damage</t>
+          <t>2.4 other bonuses of final damage</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Limit Field: asked on the target after a special damage is chosen and again in the magic function; what it changes is not followed</t>
+          <t>Limit Field: its value is added to the same "other" bonus of final physical damage. It is also asked in the magic function and after special damage, not followed there</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>0x44fb1c, 0x44ed53</t>
+          <t>0x44c723, 0x44ed53, 0x44fb1c</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
@@ -21717,6 +21717,106 @@
       <c r="E127" t="inlineStr">
         <is>
           <t>partly</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="n">
+        <v>191</v>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>2.4 other bonuses of final damage</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Power Charge: its value is added to the "other" bonus that multiplies final physical damage (final = damage C * (1 + other)); not for an action flagged as magic</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>0x44c748</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="n">
+        <v>308</v>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>2.4 other bonuses of final damage</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Imperial Guard: when the target is a party member in the back row, the lowest value among the allies who have this passive is added to the "other" bonus (a negative value: less damage)</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>0x44c7d7</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="n">
+        <v>262</v>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>12.9 after a hit</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Dark Aura: after a physical hit at short range on a unit that has it, unless the attacker has Anti-Dark Aura, the attacker receives stat debuffs of -0.1 each (effects 45, 44, 43, 42, 41, 46 in that order), how many depending on the value of the aura (the first from 1); a debuff already present is deepened by 0.1</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>0x423d9b - 0x424179</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>partly</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="n">
+        <v>304</v>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>12.9 after a hit</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Anti-Dark Aura: an attacker that has it is not touched by Dark Aura</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>0x423d7a</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>read</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: random move tables read from the executable
random move tables read from the executable; rules of escape, TP cost,
drops, gold, discount
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -8887,12 +8887,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>partly read</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>actions</t>
+          <t>12.11 passives outside the formulas</t>
         </is>
       </c>
       <c r="H9" t="inlineStr"/>
@@ -11477,10 +11477,14 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>not found</t>
-        </is>
-      </c>
-      <c r="F100" t="inlineStr"/>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>12.10 random moves</t>
+        </is>
+      </c>
       <c r="H100" t="inlineStr"/>
     </row>
     <row r="101">
@@ -11500,10 +11504,14 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>not found</t>
-        </is>
-      </c>
-      <c r="F101" t="inlineStr"/>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>12.10 random moves</t>
+        </is>
+      </c>
       <c r="H101" t="inlineStr"/>
     </row>
     <row r="102">
@@ -11523,10 +11531,14 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>not found</t>
-        </is>
-      </c>
-      <c r="F102" t="inlineStr"/>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>12.10 random moves</t>
+        </is>
+      </c>
       <c r="H102" t="inlineStr"/>
     </row>
     <row r="103">
@@ -11546,10 +11558,14 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>not found</t>
-        </is>
-      </c>
-      <c r="F103" t="inlineStr"/>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>12.10 random moves</t>
+        </is>
+      </c>
       <c r="H103" t="inlineStr"/>
     </row>
     <row r="104">
@@ -13869,15 +13885,15 @@
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F189" t="inlineStr"/>
-      <c r="H189" t="inlineStr">
-        <is>
-          <t>0x4fd331</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F189" t="inlineStr">
+        <is>
+          <t>12.11 passives outside the formulas</t>
+        </is>
+      </c>
+      <c r="H189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" t="n">
@@ -13950,15 +13966,15 @@
       </c>
       <c r="E192" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F192" t="inlineStr"/>
-      <c r="H192" t="inlineStr">
-        <is>
-          <t>0x41adcd</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F192" t="inlineStr">
+        <is>
+          <t>12.11 passives outside the formulas</t>
+        </is>
+      </c>
+      <c r="H192" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" t="n">
@@ -13977,15 +13993,15 @@
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F193" t="inlineStr"/>
-      <c r="H193" t="inlineStr">
-        <is>
-          <t>0x5581ff</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F193" t="inlineStr">
+        <is>
+          <t>12.11 passives outside the formulas</t>
+        </is>
+      </c>
+      <c r="H193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" t="n">
@@ -14004,15 +14020,15 @@
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F194" t="inlineStr"/>
-      <c r="H194" t="inlineStr">
-        <is>
-          <t>0x43aa33</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F194" t="inlineStr">
+        <is>
+          <t>12.11 passives outside the formulas</t>
+        </is>
+      </c>
+      <c r="H194" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" t="n">
@@ -14301,15 +14317,15 @@
       </c>
       <c r="E205" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F205" t="inlineStr"/>
-      <c r="H205" t="inlineStr">
-        <is>
-          <t>0x4762d2</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>12.11 passives outside the formulas</t>
+        </is>
+      </c>
+      <c r="H205" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" t="n">
@@ -15057,15 +15073,15 @@
       </c>
       <c r="E233" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F233" t="inlineStr"/>
-      <c r="H233" t="inlineStr">
-        <is>
-          <t>0x42db82</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F233" t="inlineStr">
+        <is>
+          <t>12.10 random moves</t>
+        </is>
+      </c>
+      <c r="H233" t="inlineStr"/>
     </row>
     <row r="234">
       <c r="A234" t="n">
@@ -15563,10 +15579,14 @@
       </c>
       <c r="E251" t="inlineStr">
         <is>
-          <t>not found</t>
-        </is>
-      </c>
-      <c r="F251" t="inlineStr"/>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F251" t="inlineStr">
+        <is>
+          <t>12.10 random moves</t>
+        </is>
+      </c>
       <c r="H251" t="inlineStr"/>
     </row>
     <row r="252">
@@ -15586,10 +15606,14 @@
       </c>
       <c r="E252" t="inlineStr">
         <is>
-          <t>not found</t>
-        </is>
-      </c>
-      <c r="F252" t="inlineStr"/>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F252" t="inlineStr">
+        <is>
+          <t>12.10 random moves</t>
+        </is>
+      </c>
       <c r="H252" t="inlineStr"/>
     </row>
     <row r="253">
@@ -15609,10 +15633,14 @@
       </c>
       <c r="E253" t="inlineStr">
         <is>
-          <t>not found</t>
-        </is>
-      </c>
-      <c r="F253" t="inlineStr"/>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F253" t="inlineStr">
+        <is>
+          <t>12.10 random moves</t>
+        </is>
+      </c>
       <c r="H253" t="inlineStr"/>
     </row>
     <row r="254">
@@ -15659,10 +15687,14 @@
       </c>
       <c r="E255" t="inlineStr">
         <is>
-          <t>not found</t>
-        </is>
-      </c>
-      <c r="F255" t="inlineStr"/>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F255" t="inlineStr">
+        <is>
+          <t>12.10 random moves</t>
+        </is>
+      </c>
       <c r="H255" t="inlineStr"/>
     </row>
     <row r="256">
@@ -15682,10 +15714,14 @@
       </c>
       <c r="E256" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F256" t="inlineStr"/>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>12.10 random moves</t>
+        </is>
+      </c>
       <c r="G256" t="inlineStr">
         <is>
           <t>0x48b490</t>
@@ -18633,7 +18669,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E131"/>
+  <dimension ref="A1:E146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -19851,22 +19887,22 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>actions</t>
+          <t>12.11 passives outside the formulas</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Escape: chance 0.3 + (own AGI - average enemy AGI) / 50 + skill, as the debug message states; its code is not read</t>
+          <t>Escape: chance 0.3 + (AGI of the runner - average AGI of the enemies) / 50 + Escape Chance (269), kept between 0.2 (0.5 with a piece of enchantment 262) and 0.95; when the action has a value it is added, up to 0.95; a flag of the battle makes it certain</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>0x47fd00</t>
+          <t>0x41ad59 - 0x41aeee</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>partly</t>
+          <t>read</t>
         </is>
       </c>
     </row>
@@ -21815,6 +21851,381 @@
         </is>
       </c>
       <c r="E131" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="n">
+        <v>152</v>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>12.10 random moves</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Roulette Circus: when the action is built a weighted roll on a table of the executable picks the hidden skill that is performed (tools/random_move_data.py; the tables are in docs/generated/BALANCE_BASELINE.md)</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>0x41e060, 0x42db00</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="n">
+        <v>153</v>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>12.10 random moves</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Magic Box: when the action is built a weighted roll on a table of the executable picks the hidden skill that is performed (tools/random_move_data.py; the tables are in docs/generated/BALANCE_BASELINE.md)</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>0x41e060, 0x42db00</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="n">
+        <v>154</v>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>12.10 random moves</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Showtime: when the action is built a weighted roll on a table of the executable picks the hidden skill that is performed (tools/random_move_data.py; the tables are in docs/generated/BALANCE_BASELINE.md)</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>0x41e060, 0x42db00</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="n">
+        <v>155</v>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>12.10 random moves</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Heaven or Hell: when the action is built a weighted roll on a table of the executable picks the hidden skill that is performed (tools/random_move_data.py; the tables are in docs/generated/BALANCE_BASELINE.md)</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>0x41e060, 0x42db00</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="n">
+        <v>315</v>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>12.10 random moves</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Triple Joker: a user that has it rolls on the second table of each random move</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>0x42db82</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="n">
+        <v>425</v>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>12.10 random moves</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>On each target, ends its chant, its song, its dance and its doll (four calls on the battle object of the unit)</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>0x48b060</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="n">
+        <v>426</v>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>12.10 random moves</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Each party member targeted recovers int(value) TP</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>0x48b120</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="n">
+        <v>427</v>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>12.10 random moves</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Genjimaru: unless one is already in the battle, creates a unit built like a doll (9,999 HP, same constructor 0x4fd840) that performs hidden skill 107. When one is already there the roll of Magic Box is swapped for its result with no effect</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>0x48b1f0, 0x41e3c2</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="n">
+        <v>432</v>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>12.10 random moves</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Enemies Flee: each enemy targeted is marked as gone when the battle allows running away (one byte of the battle set, the next clear)</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>0x48b3c0</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="n">
+        <v>433</v>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>12.10 random moves</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Money Loss: the party loses int(gold * value)</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>0x48b490</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="n">
+        <v>266</v>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>12.11 passives outside the formulas</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>TP Cost Reduction: the cost of a skill is first cut by enchantments (techniques: int(cost * 0.8) with a piece of 246, then int(cost * 0.6) with a piece of 247; spells: the same with 248 and 249), at least 1; then, in battle, this status takes away int(ceil(cost * value)), at least 1 left</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>0x4fd250</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="n">
+        <v>269</v>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>12.11 passives outside the formulas</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Escape Chance: added to the chance to run away, 0.3 + (AGI of the runner - average AGI of the enemies) / 50 + value, kept between 0.2 (0.5 with a piece of enchantment 262) and 0.95; the value of the Escape action itself is then added, up to 0.95. The roll is below 100 under chance * 100</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>0x41ad59 - 0x41aeee</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="n">
+        <v>270</v>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>12.11 passives outside the formulas</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Item Drop Rate Modifier: the highest value in the party, times 100, is added to the chance of every drop of a fallen enemy that has a chance above 0; the last (rare) drop also gains 20 per piece of enchantment 276 on the unit that felled it</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>0x5581ff - 0x55835c</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="n">
+        <v>271</v>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>12.11 passives outside the formulas</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Gold Drop Rate Modifier: the gold of a fallen enemy is int(gold * (1 + highest value in the party)), plus the gold it had stolen</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>0x43aa33</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="n">
+        <v>282</v>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>12.11 passives outside the formulas</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>Discount: a price becomes int(price - price * highest value in the party), at least 1</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>0x4762c0</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
         <is>
           <t>read</t>
         </is>

</xml_diff>

<commit_message>
feat: rules of Cover, clones, counters, Support Shot, Ecstasy, double
rules of Cover, clones, counters, Support Shot, Ecstasy, double actions;
wider effect detectors; equipment drop fields named
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -8785,7 +8785,7 @@
       <c r="F5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
-          <t>0x422a18, 0x47f5fc, 0x47f633, 0x5b8b7a</t>
+          <t>0x5b8b7a</t>
         </is>
       </c>
     </row>
@@ -9023,15 +9023,15 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr"/>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>0x42e9cb</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>outside battle</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -9104,10 +9104,14 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>not found</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr"/>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>3 magic attack</t>
+        </is>
+      </c>
       <c r="H17" t="inlineStr"/>
     </row>
     <row r="18">
@@ -10265,15 +10269,15 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F60" t="inlineStr"/>
-      <c r="H60" t="inlineStr">
-        <is>
-          <t>0x41f947</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>12.12 who takes the hit</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -10292,15 +10296,15 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F61" t="inlineStr"/>
-      <c r="H61" t="inlineStr">
-        <is>
-          <t>0x41faaf</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>12.12 who takes the hit</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -11860,15 +11864,15 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F114" t="inlineStr"/>
-      <c r="H114" t="inlineStr">
-        <is>
-          <t>0x420c48, 0x420cac, 0x42497a</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>12.12 who takes the hit</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="n">
@@ -12022,15 +12026,15 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F120" t="inlineStr"/>
-      <c r="H120" t="inlineStr">
-        <is>
-          <t>0x41fbd0</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>12.12 who takes the hit</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="n">
@@ -12049,15 +12053,15 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F121" t="inlineStr"/>
-      <c r="H121" t="inlineStr">
-        <is>
-          <t>0x421c93</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>12.12 who takes the hit</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="n">
@@ -12076,10 +12080,14 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>not found</t>
-        </is>
-      </c>
-      <c r="F122" t="inlineStr"/>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>3 magic attack</t>
+        </is>
+      </c>
       <c r="H122" t="inlineStr"/>
     </row>
     <row r="123">
@@ -12320,7 +12328,7 @@
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>10.2 statuses on stats</t>
+          <t>12.12 who takes the hit</t>
         </is>
       </c>
       <c r="H131" t="inlineStr"/>
@@ -12510,7 +12518,7 @@
       <c r="F138" t="inlineStr"/>
       <c r="H138" t="inlineStr">
         <is>
-          <t>0x42f0fa</t>
+          <t>0x42efd5, 0x42f0fa</t>
         </is>
       </c>
     </row>
@@ -12531,11 +12539,15 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>not found</t>
+          <t>located</t>
         </is>
       </c>
       <c r="F139" t="inlineStr"/>
-      <c r="H139" t="inlineStr"/>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>0x42b585</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="n">
@@ -12635,11 +12647,15 @@
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>not found</t>
+          <t>located</t>
         </is>
       </c>
       <c r="F143" t="inlineStr"/>
-      <c r="H143" t="inlineStr"/>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>0x42bbc7</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="n">
@@ -12739,10 +12755,14 @@
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>not found</t>
-        </is>
-      </c>
-      <c r="F147" t="inlineStr"/>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>3 magic attack</t>
+        </is>
+      </c>
       <c r="H147" t="inlineStr"/>
     </row>
     <row r="148">
@@ -12907,15 +12927,15 @@
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F153" t="inlineStr"/>
-      <c r="H153" t="inlineStr">
-        <is>
-          <t>0x439380</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>12.14 after an action and after a battle</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="n">
@@ -13426,12 +13446,12 @@
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>partly read</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F172" t="inlineStr">
         <is>
-          <t>passive rolls</t>
+          <t>12.13 counters and follow-ups</t>
         </is>
       </c>
       <c r="H172" t="inlineStr"/>
@@ -13458,7 +13478,7 @@
       </c>
       <c r="F173" t="inlineStr">
         <is>
-          <t>applying a hit</t>
+          <t>12.13 counters and follow-ups</t>
         </is>
       </c>
       <c r="H173" t="inlineStr"/>
@@ -13723,15 +13743,15 @@
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F183" t="inlineStr"/>
-      <c r="H183" t="inlineStr">
-        <is>
-          <t>0x42540a</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>12.13 counters and follow-ups</t>
+        </is>
+      </c>
+      <c r="H183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="n">
@@ -14371,15 +14391,15 @@
       </c>
       <c r="E207" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F207" t="inlineStr"/>
-      <c r="H207" t="inlineStr">
-        <is>
-          <t>0x43c47e, 0x43ccc8</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F207" t="inlineStr">
+        <is>
+          <t>12.14 after an action and after a battle</t>
+        </is>
+      </c>
+      <c r="H207" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" t="n">
@@ -14398,12 +14418,12 @@
       </c>
       <c r="E208" t="inlineStr">
         <is>
-          <t>partly read</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F208" t="inlineStr">
         <is>
-          <t>applying a hit</t>
+          <t>12.12 who takes the hit</t>
         </is>
       </c>
       <c r="H208" t="inlineStr"/>
@@ -14452,15 +14472,15 @@
       </c>
       <c r="E210" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F210" t="inlineStr"/>
-      <c r="H210" t="inlineStr">
-        <is>
-          <t>0x43bfbd</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F210" t="inlineStr">
+        <is>
+          <t>12.14 after an action and after a battle</t>
+        </is>
+      </c>
+      <c r="H210" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" t="n">
@@ -14479,15 +14499,15 @@
       </c>
       <c r="E211" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F211" t="inlineStr"/>
-      <c r="H211" t="inlineStr">
-        <is>
-          <t>0x439072</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F211" t="inlineStr">
+        <is>
+          <t>12.14 after an action and after a battle</t>
+        </is>
+      </c>
+      <c r="H211" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" t="n">
@@ -14506,15 +14526,15 @@
       </c>
       <c r="E212" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F212" t="inlineStr"/>
-      <c r="H212" t="inlineStr">
-        <is>
-          <t>0x4390b9</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F212" t="inlineStr">
+        <is>
+          <t>12.14 after an action and after a battle</t>
+        </is>
+      </c>
+      <c r="H212" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" t="n">
@@ -14533,15 +14553,15 @@
       </c>
       <c r="E213" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F213" t="inlineStr"/>
-      <c r="H213" t="inlineStr">
-        <is>
-          <t>0x438e53, 0x47f739</t>
-        </is>
-      </c>
+          <t>partly read</t>
+        </is>
+      </c>
+      <c r="F213" t="inlineStr">
+        <is>
+          <t>2.8 damage received</t>
+        </is>
+      </c>
+      <c r="H213" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" t="n">
@@ -14749,12 +14769,12 @@
       </c>
       <c r="E221" t="inlineStr">
         <is>
-          <t>partly read</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F221" t="inlineStr">
         <is>
-          <t>applying a hit</t>
+          <t>12.13 counters and follow-ups</t>
         </is>
       </c>
       <c r="H221" t="inlineStr"/>
@@ -14857,15 +14877,15 @@
       </c>
       <c r="E225" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F225" t="inlineStr"/>
-      <c r="H225" t="inlineStr">
-        <is>
-          <t>0x4203b4, 0x422582, 0x4246c2, 0x424739</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F225" t="inlineStr">
+        <is>
+          <t>12.13 counters and follow-ups</t>
+        </is>
+      </c>
+      <c r="H225" t="inlineStr"/>
     </row>
     <row r="226">
       <c r="A226" t="n">
@@ -14992,15 +15012,15 @@
       </c>
       <c r="E230" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F230" t="inlineStr"/>
-      <c r="H230" t="inlineStr">
-        <is>
-          <t>0x47f5e2</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F230" t="inlineStr">
+        <is>
+          <t>2.8 damage received</t>
+        </is>
+      </c>
+      <c r="H230" t="inlineStr"/>
     </row>
     <row r="231">
       <c r="A231" t="n">
@@ -15019,15 +15039,15 @@
       </c>
       <c r="E231" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F231" t="inlineStr"/>
-      <c r="H231" t="inlineStr">
-        <is>
-          <t>0x43c920</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F231" t="inlineStr">
+        <is>
+          <t>12.14 after an action and after a battle</t>
+        </is>
+      </c>
+      <c r="H231" t="inlineStr"/>
     </row>
     <row r="232">
       <c r="A232" t="n">
@@ -15504,7 +15524,7 @@
       <c r="F248" t="inlineStr"/>
       <c r="H248" t="inlineStr">
         <is>
-          <t>0x42f10a</t>
+          <t>0x42f015, 0x42f10a</t>
         </is>
       </c>
     </row>
@@ -18669,7 +18689,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E146"/>
+  <dimension ref="A1:E164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -19437,17 +19457,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>applying a hit</t>
+          <t>12.13 counters and follow-ups</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>When the target has it: a roll below 100 under value * 100 answers the hit with a counter (debug message "Counter")</t>
+          <t>Counter: when an action of short or mid range is about to hit a unit that has it (not its own, and the attacker has no Absolute Attack), a roll below 100 under value * 100 makes the hit do nothing and sets up a counter by the target (debug message "Counter")</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>0x42259f</t>
+          <t>0x422553 - 0x422656</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -20462,22 +20482,22 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>passive rolls</t>
+          <t>12.13 counters and follow-ups</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>When the target has it: a roll below 100 under value * 100 triggers Reprisal; what follows is not read</t>
+          <t>Reprisal: after a hit of short or mid range that landed on a unit that has it (the attacker has no Absolute Attack), a roll below 100 under value * 100 marks the target to counter once the action ends</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>0x4246d2</t>
+          <t>0x424689 - 0x424711</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>partly</t>
+          <t>read</t>
         </is>
       </c>
     </row>
@@ -20612,22 +20632,22 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>applying a hit</t>
+          <t>12.12 who takes the hit</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Elegant Dancing: checked on the target before a physical hit, with no roll; its consequence is not followed</t>
+          <t>Elegant Dancing: the first hit that would deal damage to its bearer deals 0, and the status is spent</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>0x42208e</t>
+          <t>0x42208e - 0x4220e0</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>partly</t>
+          <t>read</t>
         </is>
       </c>
     </row>
@@ -20637,22 +20657,22 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>applying a hit</t>
+          <t>12.13 counters and follow-ups</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Counter Whip: checked on the target when an action starts; its consequence is not followed</t>
+          <t>Counter Whip: when an action starts, the first of its targets that has it strikes first: a counter is set up before the action (no roll). Not against an attacker with Absolute Attack</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>0x4203fd</t>
+          <t>0x4203b1 - 0x42043f</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>partly</t>
+          <t>read</t>
         </is>
       </c>
     </row>
@@ -21287,17 +21307,17 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>10.2 statuses on stats</t>
+          <t>12.12 who takes the hit</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>All Resistances 100: its own command only; where the resistances are set is not followed</t>
+          <t>All Resistances 100: a hit has no effect on a unit that has it, unless the action passes a test of its skill that was not read (0x416ea0)</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>0x487540</t>
+          <t>0x421c6c</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
@@ -22167,7 +22187,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>Item Drop Rate Modifier: the highest value in the party, times 100, is added to the chance of every drop of a fallen enemy that has a chance above 0; the last (rare) drop also gains 20 per piece of enchantment 276 on the unit that felled it</t>
+          <t>Item Drop Rate Modifier: the highest value in the party, times 100, is added to the chance of every drop of a fallen enemy that has a chance above 0. The third chance of the enemy record (file offset 0x7C) also gains 20 per piece of enchantment 276 (Equipment drop rate UP) on the unit that felled it. When the chances add to less than 100 the rest is "nothing", and one weighted roll picks the outcome</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
@@ -22226,6 +22246,456 @@
         </is>
       </c>
       <c r="E146" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="n">
+        <v>171</v>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>12.12 who takes the hit</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Cover: when an action aimed at one unit or at random units (target codes 0 and 1) is about to hit, and other units of the side of the target have Cover, one of them, picked at random with equal chances, takes the hit in its place. No roll. After the action, for each hit covered, a roll below 100 under value * 100 ends the Cover of that unit (the value is the chance to lose it)</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>0x420b60 - 0x420ed6, 0x42497a</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="n">
+        <v>101</v>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>12.12 who takes the hit</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Clone: a count of hits. A hit that would deal damage (unless the action has effect 140, 141 or 142) or an ailment that would land does nothing instead, and the count drops by 1; at 0 the status ends</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>0x41f920, 0x4226ab, 0x422c4b</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="n">
+        <v>102</v>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>12.12 who takes the hit</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Illusion: the same count of hits as Clone (101), looked at when the target has no Clone</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>0x41faaf</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="n">
+        <v>181</v>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>12.12 who takes the hit</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Barrier System: the same count of hits as Clone (101), looked at after Clone and Illusion</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>0x41fbd0</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="n">
+        <v>182</v>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>12.12 who takes the hit</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Nullify Short-Mid: a hit of short or mid range (range codes 0 and 1) has no effect on a unit that has it</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>0x421c93</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="n">
+        <v>27</v>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>3 magic attack</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Magic Attack (Loose Spirit): added, with effect 173, to the power boost of magic damage: damage B = damage A * (1 + power boost) * (1 + damage cut)</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>0x44e612</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="n">
+        <v>183</v>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>3 magic attack</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Magic Barrier: its value (negative) is added to the damage cut of magic damage, beside the cut of the enchantments (which stops at -0.25 by itself)</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>0x44e6ee, 0x44e82b</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="n">
+        <v>307</v>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>12.13 counters and follow-ups</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Absolute Attack: its bearer cannot be answered: Counter (250), Reprisal (249), Counter Whip (303) and effect 447 are skipped when the attacker has it</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>0x4203b4, 0x422582, 0x4246c2, 0x424739</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="n">
+        <v>260</v>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>12.13 counters and follow-ups</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Support Shot: after a plain attack (action type 1) of a unit, each other unit of its side that has it rolls below 100 under value * 100, in order; the first success performs a follow-up attack</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>0x424c42 - 0x42548d</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="n">
+        <v>312</v>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>2.8 damage received</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Ecstasy: the first time in a battle that damage takes its bearer from half its max HP or more to below half, it gains an ATK buff (41) and a DEX buff (45) of the value of Ecstasy</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>0x47f59b - 0x47f682</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="n">
+        <v>291</v>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>2.8 damage received</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Heretic Samsara (enemy): when damage takes its bearer below half its max HP its value is set to 1; at the next battle update a unit with value 1 receives effects 416 to 423. The values of those were not followed</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>0x47f739, 0x438e53</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>partly</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="n">
+        <v>288</v>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>12.14 after an action and after a battle</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Double Action (enemy): after its action, a roll below 100 under value * 100 lets its bearer act twice</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>0x439072</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="n">
+        <v>289</v>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>12.14 after an action and after a battle</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Triple Action (enemy): when Double Action did not come out, a roll below 100 under value * 100 lets its bearer act three times</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>0x4390b9</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="n">
+        <v>218</v>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>12.14 after an action and after a battle</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>Paean: when the battle ends, its value on the first member of the party list is the bonus of the EXP formula (6c): share * (1 + bonus)</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>0x439380</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="n">
+        <v>287</v>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>12.14 after an action and after a battle</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Solo Duet: a unit can keep two songs at once instead of one; starting one more ends the oldest</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>0x43bfbd</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="n">
+        <v>284</v>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>12.14 after an action and after a battle</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>On Stage: a unit can keep two dances at once instead of one; starting one more ends the oldest</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>0x43c47e, 0x43ccc8</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="n">
+        <v>313</v>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>12.14 after an action and after a battle</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>Double Puppet: a unit can keep two dolls at once instead of one; starting one more ends the oldest</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>0x43c920</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="n">
+        <v>22</v>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>outside battle</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>Treasure Search: counts the chests of the floor and those already opened, and shows how many are left</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>0x42e9cb - 0x42ebe0</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
         <is>
           <t>read</t>
         </is>

</xml_diff>

<commit_message>
feat: characters and Pep read from the game
characters and Pep read from the game (base class, unique skill,
starting EXP, Pep amounts and rules); enemy dances per turn
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -9509,10 +9509,14 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr"/>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>13 Pep</t>
+        </is>
+      </c>
       <c r="G32" t="inlineStr">
         <is>
           <t>0x480e20</t>
@@ -9753,10 +9757,14 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr"/>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>2.7 special damage</t>
+        </is>
+      </c>
       <c r="G41" t="inlineStr">
         <is>
           <t>0x481060</t>
@@ -9804,10 +9812,14 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr"/>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>13 Pep</t>
+        </is>
+      </c>
       <c r="G43" t="inlineStr">
         <is>
           <t>0x481160</t>
@@ -12512,15 +12524,15 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F138" t="inlineStr"/>
-      <c r="H138" t="inlineStr">
-        <is>
-          <t>0x42efd5, 0x42f0fa</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>5e effects that act every turn</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="n">
@@ -12539,15 +12551,15 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F139" t="inlineStr"/>
-      <c r="H139" t="inlineStr">
-        <is>
-          <t>0x42b585</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>5e effects that act every turn</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="n">
@@ -12647,15 +12659,15 @@
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F143" t="inlineStr"/>
-      <c r="H143" t="inlineStr">
-        <is>
-          <t>0x42bbc7</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>13 Pep</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="n">
@@ -15518,15 +15530,15 @@
       </c>
       <c r="E248" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F248" t="inlineStr"/>
-      <c r="H248" t="inlineStr">
-        <is>
-          <t>0x42f015, 0x42f10a</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F248" t="inlineStr">
+        <is>
+          <t>5e effects that act every turn</t>
+        </is>
+      </c>
+      <c r="H248" t="inlineStr"/>
     </row>
     <row r="249">
       <c r="A249" t="n">
@@ -18437,12 +18449,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>not read</t>
+          <t>read</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>CharacterData holds two ints per character</t>
+          <t>tools/character_data.py: base class, unique skill, starting class and EXP, food lists, Pep amounts (PlayerStatusData.bin and InitialData.bin of each package in Character.pck)</t>
         </is>
       </c>
     </row>
@@ -18481,12 +18493,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>not read</t>
+          <t>read</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>The messages list what raises and lowers it; its effect on stats is not read</t>
+          <t>docs/FORMULAS.md 13 and tools/character_data.py: the range, what fixes it, the 21 amounts of each character, every place that writes it, and its three uses (joint skills, Positive Trance, the mood shown). Eight of the 21 events are only known by their index</t>
         </is>
       </c>
     </row>
@@ -18689,7 +18701,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E164"/>
+  <dimension ref="A1:E171"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -22701,6 +22713,181 @@
         </is>
       </c>
     </row>
+    <row r="165">
+      <c r="A165" t="n">
+        <v>66</v>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>13 Pep</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>Pep UP: a party member whose Pep is below 100 gains value Pep (then kept between 70 and 130)</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>0x480e20</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="n">
+        <v>80</v>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>13 Pep</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>Pep change: the Pep of a party member changes by value, up or down (then kept between 70 and 130)</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>0x481160</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="n">
+        <v>204</v>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>13 Pep</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>Weird Dance: each time it ticks, the Pep of each party member it reaches changes by value</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>0x42bbc7 - 0x42bc75</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="n">
+        <v>200</v>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>5e effects that act every turn</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>Subtle Dance: each time it ticks its target loses int(value * a field of the unit read directly (0x18), taken to be its TP), at most the value of effect 296 when the action has one; the amount goes to the TP side of the hit record</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>0x42b585 - 0x42b63b</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="n">
+        <v>199</v>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>5e effects that act every turn</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>Each time it ticks the target takes int(max HP * value) damage, at most the value of effect 296 when the action has one</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>0x42efd5 - 0x42f0c6</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="n">
+        <v>339</v>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>5e effects that act every turn</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>Debilitating Geas: the same per-turn damage as effect 199, looked at when the action has no 199</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>0x42f015</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="n">
+        <v>77</v>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>2.7 special damage</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>Sacrifice: the hit records of the action are emptied and the user takes damage equal to its own max HP</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>0x481060</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: encounter rate read from the code and the floor files
encounter rate read from the code and the floor files; rules of Shadow
Sew, Materialize, cures, Esarhaddon, weapon elements and the last single
effects
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -8968,10 +8968,14 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>not found</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr"/>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>14 encounter rate</t>
+        </is>
+      </c>
       <c r="H12" t="inlineStr"/>
     </row>
     <row r="13">
@@ -9789,10 +9793,14 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>not found</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr"/>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>5 order of turns</t>
+        </is>
+      </c>
       <c r="H42" t="inlineStr"/>
     </row>
     <row r="43">
@@ -9844,20 +9852,20 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr"/>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>12.11 passives outside the formulas</t>
+        </is>
+      </c>
       <c r="G44" t="inlineStr">
         <is>
           <t>0x4813a0</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>0x4802ce, 0x4805ce</t>
-        </is>
-      </c>
+      <c r="H44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -10431,20 +10439,20 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F65" t="inlineStr"/>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>6d recovery</t>
+        </is>
+      </c>
       <c r="G65" t="inlineStr">
         <is>
           <t>0x481a20</t>
         </is>
       </c>
-      <c r="H65" t="inlineStr">
-        <is>
-          <t>0x56d581</t>
-        </is>
-      </c>
+      <c r="H65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -10571,15 +10579,15 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F70" t="inlineStr"/>
-      <c r="H70" t="inlineStr">
-        <is>
-          <t>0x42e1ba, 0x43b08e, 0x43b183</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>9.1 who gets hit</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -10854,7 +10862,7 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>located</t>
+          <t>partly read</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -10867,11 +10875,7 @@
           <t>0x4834b0</t>
         </is>
       </c>
-      <c r="H79" t="inlineStr">
-        <is>
-          <t>0x4e585e, 0x5107c9</t>
-        </is>
-      </c>
+      <c r="H79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -10922,7 +10926,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>located</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -10935,11 +10939,7 @@
           <t>0x483840</t>
         </is>
       </c>
-      <c r="H81" t="inlineStr">
-        <is>
-          <t>0x4fa6d5, 0x4fb652</t>
-        </is>
-      </c>
+      <c r="H81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -11113,7 +11113,7 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>located</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
@@ -11126,11 +11126,7 @@
           <t>0x483e00</t>
         </is>
       </c>
-      <c r="H87" t="inlineStr">
-        <is>
-          <t>0x537db7</t>
-        </is>
-      </c>
+      <c r="H87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -11262,20 +11258,20 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F92" t="inlineStr"/>
+          <t>partly read</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>5b ailments</t>
+        </is>
+      </c>
       <c r="G92" t="inlineStr">
         <is>
           <t>0x484020</t>
         </is>
       </c>
-      <c r="H92" t="inlineStr">
-        <is>
-          <t>0x4e5878</t>
-        </is>
-      </c>
+      <c r="H92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -11790,7 +11786,7 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>partly read</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
@@ -13263,10 +13259,14 @@
       </c>
       <c r="E165" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F165" t="inlineStr"/>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>6d recovery</t>
+        </is>
+      </c>
       <c r="G165" t="inlineStr">
         <is>
           <t>0x48a430</t>
@@ -14997,15 +14997,15 @@
       </c>
       <c r="E229" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F229" t="inlineStr"/>
-      <c r="H229" t="inlineStr">
-        <is>
-          <t>0x436727</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F229" t="inlineStr">
+        <is>
+          <t>5d start of a turn</t>
+        </is>
+      </c>
+      <c r="H229" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" t="n">
@@ -15186,15 +15186,15 @@
       </c>
       <c r="E236" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F236" t="inlineStr"/>
-      <c r="H236" t="inlineStr">
-        <is>
-          <t>0x43736a</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F236" t="inlineStr">
+        <is>
+          <t>9 enemy AI</t>
+        </is>
+      </c>
+      <c r="H236" t="inlineStr"/>
     </row>
     <row r="237">
       <c r="A237" t="n">
@@ -15267,19 +15267,15 @@
       </c>
       <c r="E239" t="inlineStr">
         <is>
-          <t>located</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F239" t="inlineStr">
         <is>
-          <t>3 magic attack</t>
-        </is>
-      </c>
-      <c r="H239" t="inlineStr">
-        <is>
-          <t>0x4161f5, 0x4164bf, 0x4167cf, 0x416adf, 0x416def</t>
-        </is>
-      </c>
+          <t>2 physical attack, 3 magic attack</t>
+        </is>
+      </c>
+      <c r="H239" t="inlineStr"/>
     </row>
     <row r="240">
       <c r="A240" t="n">
@@ -15298,19 +15294,15 @@
       </c>
       <c r="E240" t="inlineStr">
         <is>
-          <t>located</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F240" t="inlineStr">
         <is>
-          <t>3 magic attack</t>
-        </is>
-      </c>
-      <c r="H240" t="inlineStr">
-        <is>
-          <t>0x4161af, 0x416505, 0x4167df, 0x416aef, 0x416dff</t>
-        </is>
-      </c>
+          <t>2 physical attack, 3 magic attack</t>
+        </is>
+      </c>
+      <c r="H240" t="inlineStr"/>
     </row>
     <row r="241">
       <c r="A241" t="n">
@@ -15329,19 +15321,15 @@
       </c>
       <c r="E241" t="inlineStr">
         <is>
-          <t>located</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F241" t="inlineStr">
         <is>
-          <t>3 magic attack</t>
-        </is>
-      </c>
-      <c r="H241" t="inlineStr">
-        <is>
-          <t>0x4161bf, 0x4164cf, 0x4167f1, 0x416b01, 0x416e35</t>
-        </is>
-      </c>
+          <t>2 physical attack, 3 magic attack</t>
+        </is>
+      </c>
+      <c r="H241" t="inlineStr"/>
     </row>
     <row r="242">
       <c r="A242" t="n">
@@ -15360,19 +15348,15 @@
       </c>
       <c r="E242" t="inlineStr">
         <is>
-          <t>located</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F242" t="inlineStr">
         <is>
-          <t>3 magic attack</t>
-        </is>
-      </c>
-      <c r="H242" t="inlineStr">
-        <is>
-          <t>0x4161d1, 0x4164e1, 0x416815, 0x416b13, 0x416e11</t>
-        </is>
-      </c>
+          <t>2 physical attack, 3 magic attack</t>
+        </is>
+      </c>
+      <c r="H242" t="inlineStr"/>
     </row>
     <row r="243">
       <c r="A243" t="n">
@@ -15391,19 +15375,15 @@
       </c>
       <c r="E243" t="inlineStr">
         <is>
-          <t>located</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F243" t="inlineStr">
         <is>
-          <t>3 magic attack</t>
-        </is>
-      </c>
-      <c r="H243" t="inlineStr">
-        <is>
-          <t>0x4161e3, 0x4164f3, 0x416803, 0x416b25, 0x416e23</t>
-        </is>
-      </c>
+          <t>2 physical attack, 3 magic attack</t>
+        </is>
+      </c>
+      <c r="H243" t="inlineStr"/>
     </row>
     <row r="244">
       <c r="A244" t="n">
@@ -18559,12 +18539,12 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>not read</t>
+          <t>read</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Row S13: the most repeated complaint. Unread numbers at the start of each zone record</t>
+          <t>docs/FORMULAS.md 14, tools/floor_data.py (zone+0x1C) and sim/progression.py: chance per step of each zone, the grace of 8 steps, Whistle and the four enchantments. The five special chances of a zone are located and their gates read; what battle each one starts is not</t>
         </is>
       </c>
     </row>
@@ -18701,7 +18681,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E171"/>
+  <dimension ref="A1:E188"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -20274,17 +20254,17 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Speed buff or debuff of a unit: enters the gauge value as a bonus (5). Its own command rolls below 100 under a chance; the apply code also creates it at -0.2 and -0.75 in two cases not followed</t>
+          <t>Speed modifier: enters the gauge value as a bonus (5). When its action also has effect 79 it is applied only on a roll below 100 under the value of 79 times 100. The apply code also creates it by itself: -0.75 with Slow Target (293), -0.2 with the passive of effect 346</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>0x4864c0, 0x4229f4, 0x42456e</t>
+          <t>0x4864c0, 0x4229ec, 0x42456e</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>partly</t>
+          <t>read</t>
         </is>
       </c>
     </row>
@@ -22883,6 +22863,431 @@
         </is>
       </c>
       <c r="E171" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="n">
+        <v>18</v>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>14 encounter rate</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>Alarm (Whistle): while the party has it, its value is added to the chance in percent of a random battle on each step</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>0x47fde0, 0x4bc7b2</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="n">
+        <v>79</v>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>5 order of turns</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>Chance of the speed decrease: when the action has it, the speed modifier (168) of the same action is applied only on a roll below 100 under value * 100</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>0x486515</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="n">
+        <v>123</v>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>5b ailments</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>Shadow Sew: no effect on a unit with a piece of enchantment 137, on an enemy with immunity bit 10, or on a target whose level is not below the level of the user; otherwise a roll below 100 under value * 100</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>0x4838aa - 0x483958</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="n">
+        <v>84</v>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>12.11 passives outside the formulas</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>Snackification: only an enemy with bit 14 of its flags, and only while its HP is below int(max HP * 0.5); then a roll below 100 under value * 100 turns it into the item of its record (file offset 0xA8)</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>0x481462 - 0x48151d</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="n">
+        <v>106</v>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>6d recovery</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>Cures the first int(value) statuses of a fixed list that the target has: poison, paralysis, silence, freeze, sleep, petrification, slow, then the ATK debuff (table 0x6cc79c); with a value of 8 or more it also removes every status of a second list the unit gives (slot 0x90)</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>0x481a20</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="n">
+        <v>235</v>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>6d recovery</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>Perdurabo's action: the same cure as effect 106, with the same list and the same rule at 8</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>0x48a430</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="n">
+        <v>311</v>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>5d start of a turn</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>Esarhaddon: at the start of the turn of its bearer, the first int(value) statuses of its list are looked for and each one found is removed, with no roll. The list: poison, paralysis, silence, freeze, sleep, slow (table 0x6c9a7c)</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>0x436727 - 0x43680e</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="n">
+        <v>132</v>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>6d recovery</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>Heal Percent HP: restores int(max HP * value), at most the heal cap of the action (effect 295)</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>0x483e00</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="n">
+        <v>112</v>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>9.1 who gets hit</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>Multiple Hits, One Per Target: the target picker is told that a unit can be picked only once by this action</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>0x42e1ba</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="n">
+        <v>139</v>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>5b ailments</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>Special Instakill (enemy): no roll. An enemy with immunity bit 6 is not affected; when the command reaches its landing state the damage is the current HP of the target. The test before it (slot 0xbc of the target) was not followed</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>0x484020</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>partly</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="n">
+        <v>121</v>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>5b ailments</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>Special Petrification (enemy): the petrification method with its own command: pieces of enchantments 135 and 137 cancel it, the earth resistance enters the chance as in 5b; its arithmetic was not followed line by line</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>0x4834b0</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>partly</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="n">
+        <v>319</v>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>9 enemy AI</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>Murder License (enemy): when the turn of its bearer comes, its action is replaced by the attack linked to the status, on a target picked at random</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>0x43736a</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="n">
+        <v>325</v>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>2 physical attack</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>Weapon Element: a plain attack of its bearer counts as an attack of fire (the ten functions that answer "is this action of this attribute", 0x415340 - 0x416f50). When the unit has another of the five at the same time the answer is no for both</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>0x415f50</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="n">
+        <v>326</v>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>2 physical attack</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>Weapon Element: a plain attack of its bearer counts as an attack of water (the ten functions that answer "is this action of this attribute", 0x415340 - 0x416f50). When the unit has another of the five at the same time the answer is no for both</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>0x415f50</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="n">
+        <v>327</v>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>2 physical attack</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>Weapon Element: a plain attack of its bearer counts as an attack of lightning (the ten functions that answer "is this action of this attribute", 0x415340 - 0x416f50). When the unit has another of the five at the same time the answer is no for both</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>0x415f50</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="n">
+        <v>328</v>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>2 physical attack</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>Weapon Element: a plain attack of its bearer counts as an attack of wind (the ten functions that answer "is this action of this attribute", 0x415340 - 0x416f50). When the unit has another of the five at the same time the answer is no for both</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>0x415f50</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="n">
+        <v>329</v>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>2 physical attack</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>Weapon Element: a plain attack of its bearer counts as an attack of earth (the ten functions that answer "is this action of this attribute", 0x415340 - 0x416f50). When the unit has another of the five at the same time the answer is no for both</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>0x415f50</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
         <is>
           <t>read</t>
         </is>

</xml_diff>

<commit_message>
feat: every effect of a player skill read to its end
every effect of a player skill read to its end: steal, masteries, Dual
Wield, per-turn timing, turn-stopping rolls, Auto-Guard, Guts, Recycle,
Limit Field, Dark Aura
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -8779,15 +8779,15 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>located</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>0x5b8b7a</t>
-        </is>
-      </c>
+          <t>partly read</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>3 magic attack</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -9432,7 +9432,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>partly read</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -9459,7 +9459,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>partly read</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -9486,7 +9486,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>partly read</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -9545,7 +9545,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>partly read</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -9626,7 +9626,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>partly read</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -10073,12 +10073,12 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>partly read</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>hits of an action</t>
+          <t>12.2 number of hits</t>
         </is>
       </c>
       <c r="H52" t="inlineStr"/>
@@ -10862,7 +10862,7 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>partly read</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -11081,7 +11081,7 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>partly read</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
@@ -11204,12 +11204,12 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>partly read</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>applying a hit</t>
+          <t>9.1 who gets hit</t>
         </is>
       </c>
       <c r="H90" t="inlineStr"/>
@@ -11258,7 +11258,7 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>partly read</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
@@ -12277,7 +12277,7 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>partly read</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
@@ -12331,7 +12331,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>partly read</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
@@ -12628,7 +12628,7 @@
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>partly read</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F142" t="inlineStr">
@@ -12844,7 +12844,7 @@
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>partly read</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F150" t="inlineStr">
@@ -12876,7 +12876,7 @@
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>partly read</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F151" t="inlineStr">
@@ -13291,12 +13291,12 @@
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>partly read</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F166" t="inlineStr">
         <is>
-          <t>10 stats of a character</t>
+          <t>10.1 stats of a piece of equipment</t>
         </is>
       </c>
       <c r="H166" t="inlineStr"/>
@@ -13372,7 +13372,7 @@
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>partly read</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F169" t="inlineStr">
@@ -13404,7 +13404,7 @@
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>partly read</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F170" t="inlineStr">
@@ -13593,7 +13593,7 @@
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>partly read</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F177" t="inlineStr">
@@ -13620,7 +13620,7 @@
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>partly read</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F178" t="inlineStr">
@@ -13647,7 +13647,7 @@
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t>partly read</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F179" t="inlineStr">
@@ -13728,7 +13728,7 @@
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>partly read</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F182" t="inlineStr">
@@ -13782,12 +13782,12 @@
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>partly read</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F184" t="inlineStr">
         <is>
-          <t>2.8 damage received, 5 order of turns</t>
+          <t>5 order of turns</t>
         </is>
       </c>
       <c r="H184" t="inlineStr"/>
@@ -13809,7 +13809,7 @@
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>partly read</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F185" t="inlineStr">
@@ -14079,7 +14079,7 @@
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t>partly read</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F195" t="inlineStr">
@@ -14106,7 +14106,7 @@
       </c>
       <c r="E196" t="inlineStr">
         <is>
-          <t>partly read</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F196" t="inlineStr">
@@ -14133,7 +14133,7 @@
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t>partly read</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F197" t="inlineStr">
@@ -14160,7 +14160,7 @@
       </c>
       <c r="E198" t="inlineStr">
         <is>
-          <t>partly read</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F198" t="inlineStr">
@@ -14376,7 +14376,7 @@
       </c>
       <c r="E206" t="inlineStr">
         <is>
-          <t>partly read</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F206" t="inlineStr">
@@ -14565,7 +14565,7 @@
       </c>
       <c r="E213" t="inlineStr">
         <is>
-          <t>partly read</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F213" t="inlineStr">
@@ -14700,12 +14700,12 @@
       </c>
       <c r="E218" t="inlineStr">
         <is>
-          <t>partly read</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F218" t="inlineStr">
         <is>
-          <t>10 stats of a character</t>
+          <t>10.1 stats of a piece of equipment</t>
         </is>
       </c>
       <c r="H218" t="inlineStr"/>
@@ -14727,7 +14727,7 @@
       </c>
       <c r="E219" t="inlineStr">
         <is>
-          <t>partly read</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F219" t="inlineStr">
@@ -15213,7 +15213,7 @@
       </c>
       <c r="E237" t="inlineStr">
         <is>
-          <t>partly read</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F237" t="inlineStr">
@@ -18681,7 +18681,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E188"/>
+  <dimension ref="A1:E189"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -19954,17 +19954,17 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Gold steal: chance 0.5 * (own DEX + 50) / (target AGI + 50) * factor, as the debug message states; the amount is not read</t>
+          <t>Gold Steal: chance = 0.5 * (DEX of the thief + 50) / (AGI of the target + 50) * (value of 60 + value of 61), kept between 0.05 and 0.95; roll below 100. Once per enemy. The thief gains int(gold of the enemy record * factor), the factor being the value of effect 62 when the action has it, else 1</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>0x44fe2c</t>
+          <t>0x44fe2c - 0x450235</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>partly</t>
+          <t>read</t>
         </is>
       </c>
     </row>
@@ -19979,17 +19979,17 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Item steal: same chance formula as gold steal with its own factor (a constant 0.05 follows); the item comes from the steal fields of the enemy</t>
+          <t>Item Steal: the same chance as Gold Steal (the values of 60 and 61 are added). Once per enemy. Takes the item of the steal fields of the enemy record</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>0x44fe55</t>
+          <t>0x45036a - 0x450508</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>partly</t>
+          <t>read</t>
         </is>
       </c>
     </row>
@@ -20004,17 +20004,17 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Enemy gold steal: handled in the steal function after the roll; the amount is not read</t>
+          <t>Enemy Gold Steal: the share of gold taken. An enemy thief takes int(gold of the party * value) and carries it; the party gets it back when that enemy falls</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>0x44ff50</t>
+          <t>0x44ff50 - 0x45000b</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>partly</t>
+          <t>read</t>
         </is>
       </c>
     </row>
@@ -20029,17 +20029,17 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Defence is not subtracted (2.4). The apply code also adds it by itself, with value 1, in one case not followed</t>
+          <t>Ignores defence: defence is not subtracted (2.4). A physical action also gets it, with Certain to hit, when the status of effect 348 of its user rolls below 100 under its value * 100</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>0x42106c</t>
+          <t>0x417567, 0x42106c</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>partly</t>
+          <t>read</t>
         </is>
       </c>
     </row>
@@ -20054,17 +20054,17 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>The hit cannot miss. Added by the apply code with value 1 in cases not followed</t>
+          <t>Certain to hit: the hit cannot miss. Given together with effect 69 by the roll of the status of effect 348</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>0x421098</t>
+          <t>0x421098, 0x417567</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>partly</t>
+          <t>read</t>
         </is>
       </c>
     </row>
@@ -20074,12 +20074,12 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>hits of an action</t>
+          <t>12.2 number of hits</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Number of hits: its value</t>
+          <t>Number of hits: its value is the number of hits of the action (docs/FORMULAS.md 12.2)</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -20089,7 +20089,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>partly</t>
+          <t>read</t>
         </is>
       </c>
     </row>
@@ -20204,7 +20204,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Heals the opposing side: a fraction of max HP, under the heal cap</t>
+          <t>Heal Enemy: restores int(max HP * value) to a unit of the other side, at most the heal cap of the action</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -20214,7 +20214,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>partly</t>
+          <t>read</t>
         </is>
       </c>
     </row>
@@ -20224,22 +20224,22 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>applying a hit</t>
+          <t>9.1 who gets hit</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Number of targets of the action: read with the spell power when the action starts; how the count is used is not followed</t>
+          <t>Number of targets: after the chosen target, the next int(value) - 1 units of the same side in the order of turns are hit too</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>0x42017a</t>
+          <t>0x42017a - 0x4202f3</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>partly</t>
+          <t>read</t>
         </is>
       </c>
     </row>
@@ -20424,22 +20424,22 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>10 stats of a character</t>
+          <t>10.1 stats of a piece of equipment</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Weapon mastery: a modifier of attack for a kind of weapon, read when the stats of the unit are recomputed; the arithmetic is not followed</t>
+          <t>Weapon mastery: the ATK and the RES of each equipped weapon count as stat + int(stat * (value of 243 + value of 298)). The other four stats of the weapon are added as they are; the stats of the character are not multiplied</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>0x4f65ab</t>
+          <t>0x4f65ab - 0x4f6644</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>partly</t>
+          <t>read</t>
         </is>
       </c>
     </row>
@@ -20449,12 +20449,12 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>10 stats of a character</t>
+          <t>10.1 stats of a piece of equipment</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>A second weapon attack modifier, read next to 243</t>
+          <t>Weapon Mastery (all weapons): added to the value of effect 243 in the same rule</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -20464,7 +20464,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>partly</t>
+          <t>read</t>
         </is>
       </c>
     </row>
@@ -20504,17 +20504,17 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Survival: a roll below 100 under value * 100 when a hit would bring HP to 0; what HP is left is not followed</t>
+          <t>Survival: when a hit would take all the HP of its bearer, a roll below 100 under value * 100; on a success the damage becomes current HP - 1</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>0x4238ad</t>
+          <t>0x4238ad - 0x423901</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>partly</t>
+          <t>read</t>
         </is>
       </c>
     </row>
@@ -20529,17 +20529,17 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>When the target has it: a roll below 100 under value * 100 guards the hit (Auto-Guard)</t>
+          <t>Auto-Guard: before a physical action, each target that has it rolls below 100 under value * 100; on a success it is put in the state of Defend for that action: damage halved (2.4)</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>0x417309</t>
+          <t>0x417309 - 0x417362</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>partly</t>
+          <t>read</t>
         </is>
       </c>
     </row>
@@ -20554,17 +20554,17 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>When the unit has it: a roll below 100 under value * 100 triggers Loss Rate; its consequence is not read</t>
+          <t>Loss Rate (Recycle): when its bearer uses an item that is used up, a roll below 100 under value * 100; on a success the item is kept</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>0x42d032</t>
+          <t>0x42cfed - 0x42d07f</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>partly</t>
+          <t>read</t>
         </is>
       </c>
     </row>
@@ -20604,7 +20604,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>When a unit has it: a roll below 100 under value * 100 at the start of a battle gives it the first turn (First Grid)</t>
+          <t>First Grid: at the start of a battle a roll below 100 under value * 100; on a success its bearer gets the first turn</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -20614,7 +20614,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>partly</t>
+          <t>read</t>
         </is>
       </c>
     </row>
@@ -20679,17 +20679,17 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>HP restored after a battle: read with 273 when the battle ends, next to a constant 0.3; the arithmetic is not followed</t>
+          <t>HP restored after a battle: the values of the living members are added, the sum stops at 0.3, and every living member recovers that share of max HP (a bonus from the function of song and dance bonuses, asked with id 353, is added after the cap; not followed)</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>0x43d6cc</t>
+          <t>0x43d6cc - 0x43d778</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>partly</t>
+          <t>read</t>
         </is>
       </c>
     </row>
@@ -20704,7 +20704,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>TP restored after a battle: as 272</t>
+          <t>TP restored after a battle: the same rule as 272 for TP, with the same cap of 0.3</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -20714,7 +20714,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>partly</t>
+          <t>read</t>
         </is>
       </c>
     </row>
@@ -20729,17 +20729,17 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Modifier of healing items: read where an item heals</t>
+          <t>Healing Item Modifier: a healing item used in battle by its bearer restores amount + int(amount * value)</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>0x50e789</t>
+          <t>0x50e789 - 0x50e7bb</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>partly</t>
+          <t>read</t>
         </is>
       </c>
     </row>
@@ -20754,17 +20754,17 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Devil's Whisper: when the action carries it the after-hit code creates an instant death command against the target; its chance is not followed</t>
+          <t>Devil's Whisper (enemy): when the action carries it and the target has an ailment, an instant death command of chance equal to its value is applied through the usual instant death method (5b)</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>0x4235d5</t>
+          <t>0x4235d5 - 0x42363a</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>partly</t>
+          <t>read</t>
         </is>
       </c>
     </row>
@@ -21104,17 +21104,17 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Limit Field: its value is added to the same "other" bonus of final physical damage. It is also asked in the magic function and after special damage, not followed there</t>
+          <t>Limit Field: its value (negative) is added to the "other" bonus of final physical damage and of final magic damage; a special damage becomes damage + int(damage * value), except the one that leaves 1 HP (effect 142)</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>0x44c723, 0x44ed53, 0x44fb1c</t>
+          <t>0x44c723, 0x44ed53, 0x44fb17</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>partly</t>
+          <t>read</t>
         </is>
       </c>
     </row>
@@ -21279,17 +21279,17 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Lefty Bonus: read at the end of the same recomputation; its arithmetic is not followed</t>
+          <t>Lefty Bonus (Dual Wield): a weapon in the off hand adds nothing by the usual rule; with this status each of its six stats (with its upgrades) is added as int(stat * value)</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>0x4fc276</t>
+          <t>0x4f6579, 0x4fc26f - 0x4fc5c1</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>partly</t>
+          <t>read</t>
         </is>
       </c>
     </row>
@@ -21304,17 +21304,17 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>All Resistances 100: a hit has no effect on a unit that has it, unless the action passes a test of its skill that was not read (0x416ea0)</t>
+          <t>All Resistances 100 (enemy): a hit has no effect on a unit that has it unless the action is of the Neutral attribute (0x416ea0 is the test "is this action Neutral")</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>0x421c6c</t>
+          <t>0x421c60 - 0x421c7c, 0x416ea0</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>partly</t>
+          <t>read</t>
         </is>
       </c>
     </row>
@@ -21524,22 +21524,22 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>2.8 damage received</t>
+          <t>5 order of turns</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Stamina: after damage, when HP is at or below a share of max HP and the status is present, its command is run (0x48c1d0); the same status is a speed bonus while HP is at or below 40% (5)</t>
+          <t>Stamina: a speed bonus while HP is at or below 40% of max HP (5). When damage takes its bearer across that line the status only shows itself</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>0x47f8b3, 0x4499d0</t>
+          <t>0x47f861 - 0x47f8c1, 0x4499d0</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>partly</t>
+          <t>read</t>
         </is>
       </c>
     </row>
@@ -21604,17 +21604,17 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Warning Shot: when a unit is about to act, each opponent that has it rolls below 100 under value * 100; on a success the bearer fires its shot (its final damage is cut to 3/10, section 4). Whether the unit then loses its turn is not followed</t>
+          <t>Warning Shot: when a unit is about to act, each opponent that has it rolls below 100 under value * 100 (debug message). On a success the command of the acting unit is replaced by the skill linked to the status, which has no effect of its own, and it is flagged so that its final damage is 3/10: the turn is lost</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>0x436d89, 0x436f8b, 0x44caed</t>
+          <t>0x436d89 - 0x4371c3, 0x44cae1</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>partly</t>
+          <t>read</t>
         </is>
       </c>
     </row>
@@ -21629,17 +21629,17 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Mesmerized: when a unit is about to act, a roll below 100 under value * 100 for each opponent that has it; what a success does is not followed</t>
+          <t>Mesmerized: when a unit is about to act, a roll below 100 under value * 100 for each opponent that has it; on a success the turn ends without an action</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>0x436e2d</t>
+          <t>0x436e2d - 0x4372ea</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>partly</t>
+          <t>read</t>
         </is>
       </c>
     </row>
@@ -21654,17 +21654,17 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Erotic Dance: the same roll at the start of a turn, on the dancer among the opponents (debug message of the dance)</t>
+          <t>Erotic Dance (enemy): when a unit is about to act and has it, a roll below 100 under value * 100; on a success the turn ends without an action</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>0x436ee0</t>
+          <t>0x436eb6 - 0x436cf9</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>partly</t>
+          <t>read</t>
         </is>
       </c>
     </row>
@@ -21679,7 +21679,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>HP Regen: each time it ticks its bearer recovers int(max HP * value). When the tick fires is not followed</t>
+          <t>HP Regen: each time it ticks its bearer recovers int(max HP * value). It ticks in the turn of its bearer after its action (state 16 of the battle update, 0x437b0c); on the map it ticks on every step (0x4fb660)</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -21689,7 +21689,7 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>partly</t>
+          <t>read</t>
         </is>
       </c>
     </row>
@@ -21704,17 +21704,17 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>TP Regen: each time it ticks its bearer (party side only) recovers int(value) TP. When the tick fires is not followed</t>
+          <t>TP Regen: each time it ticks its bearer (party side only) recovers int(value) TP. It ticks in the turn of its bearer after its action (state 16 of the battle update, 0x437b0c); on the map it ticks on every step (0x4fb660)</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>0x48a710</t>
+          <t>0x48a640</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>partly</t>
+          <t>read</t>
         </is>
       </c>
     </row>
@@ -21729,7 +21729,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Carol: each time it ticks it restores int(value * (1 + 10 * song bonus)), the song bonus being the one of effect 279. When the tick fires is not followed</t>
+          <t>Carol: each time it ticks it restores int(value * (1 + 10 * song bonus)), the song bonus being the one of effect 279. It ticks in the turn of its bearer after its action (state 16 of the battle update, 0x437b0c); on the map it ticks on every step (0x4fb660)</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -21739,7 +21739,7 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>partly</t>
+          <t>read</t>
         </is>
       </c>
     </row>
@@ -21754,7 +21754,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Chorale: each time it ticks it restores int(value + 100 * song bonus) TP to a member of the party. When the tick fires is not followed</t>
+          <t>Chorale: each time it ticks it restores int(value + 100 * song bonus) TP to a member of the party. It ticks in the turn of its bearer after its action (state 16 of the battle update, 0x437b0c); on the map it ticks on every step (0x4fb660)</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
@@ -21764,7 +21764,7 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>partly</t>
+          <t>read</t>
         </is>
       </c>
     </row>
@@ -21829,7 +21829,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Dark Aura: after a physical hit at short range on a unit that has it, unless the attacker has Anti-Dark Aura, the attacker receives stat debuffs of -0.1 each (effects 45, 44, 43, 42, 41, 46 in that order), how many depending on the value of the aura (the first from 1); a debuff already present is deepened by 0.1</t>
+          <t>Dark Aura: after a physical hit at short range on its bearer, unless the attacker has Anti-Dark Aura, the attacker receives one debuff of -0.1 for each point of its value, in this order: DEX (value 1 or more), RES (2), INT (3), DEF (4), ATK (5), AGI (6). A debuff already there is deepened by 0.1</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -21839,7 +21839,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>partly</t>
+          <t>read</t>
         </is>
       </c>
     </row>
@@ -22504,17 +22504,17 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>Heretic Samsara (enemy): when damage takes its bearer below half its max HP its value is set to 1; at the next battle update a unit with value 1 receives effects 416 to 423. The values of those were not followed</t>
+          <t>Heretic Samsara (enemy): when damage takes its bearer below half its max HP its value is set to 1. From then on, at each battle update of its turn, each of its eight resistance states (effects 416 to 423) is set again to 1 or 2 at random (a number below 2, plus 1)</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>0x47f739, 0x438e53</t>
+          <t>0x47f739, 0x438e53 - 0x438fef</t>
         </is>
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>partly</t>
+          <t>read</t>
         </is>
       </c>
     </row>
@@ -23104,17 +23104,17 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>Special Instakill (enemy): no roll. An enemy with immunity bit 6 is not affected; when the command reaches its landing state the damage is the current HP of the target. The test before it (slot 0xbc of the target) was not followed</t>
+          <t>Special Instakill (enemy): only against a target that cannot act (slot 0xbc of the unit, the test the turn code uses to skip a turn); then the damage is its current HP, with no roll. No effect on an enemy with the instant death bit</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>0x484020</t>
+          <t>0x484085 - 0x4840f3</t>
         </is>
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>partly</t>
+          <t>read</t>
         </is>
       </c>
     </row>
@@ -23129,17 +23129,17 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>Special Petrification (enemy): the petrification method with its own command: pieces of enchantments 135 and 137 cancel it, the earth resistance enters the chance as in 5b; its arithmetic was not followed line by line</t>
+          <t>Special Petrification (enemy): petrifies with no roll. No effect on a unit with a piece of enchantment 135 or 137, with an earth resistance of 100 or more, or on an enemy with the petrification bit</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>0x4834b0</t>
+          <t>0x4834b0 - 0x48357a</t>
         </is>
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>partly</t>
+          <t>read</t>
         </is>
       </c>
     </row>
@@ -23290,6 +23290,26 @@
       <c r="E188" t="inlineStr">
         <is>
           <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="n">
+        <v>3</v>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>3 magic attack</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>Breath Attack (enemy): no place of the program asks for it by id (every finder and every walk over the effects of an action was searched). The attacks that carry it deal their damage through their effect 1; whether its own value enters by another path was not established</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>partly</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: the 18 unique skills counted in the effect coverage and read
the 18 unique skills counted in the effect coverage and read; how long a
status lasts and that the same effect does not stack
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -8636,7 +8636,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H258"/>
+  <dimension ref="A1:H276"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15576,11 +15576,11 @@
     </row>
     <row r="251">
       <c r="A251" t="n">
-        <v>425</v>
+        <v>345</v>
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>Cancel Chant, Song, Dance, Doll</t>
+          <t>Third Eye Wide (unique skill)</t>
         </is>
       </c>
       <c r="C251" t="n">
@@ -15596,18 +15596,18 @@
       </c>
       <c r="F251" t="inlineStr">
         <is>
-          <t>12.10 random moves</t>
+          <t>12.19 unique skills</t>
         </is>
       </c>
       <c r="H251" t="inlineStr"/>
     </row>
     <row r="252">
       <c r="A252" t="n">
-        <v>426</v>
+        <v>346</v>
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>Fixed TP Recovery</t>
+          <t>Sugar Coma (unique skill)</t>
         </is>
       </c>
       <c r="C252" t="n">
@@ -15623,18 +15623,18 @@
       </c>
       <c r="F252" t="inlineStr">
         <is>
-          <t>12.10 random moves</t>
+          <t>12.19 unique skills</t>
         </is>
       </c>
       <c r="H252" t="inlineStr"/>
     </row>
     <row r="253">
       <c r="A253" t="n">
-        <v>427</v>
+        <v>348</v>
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>Genjimaru</t>
+          <t>Furious Strike (unique skill)</t>
         </is>
       </c>
       <c r="C253" t="n">
@@ -15650,18 +15650,18 @@
       </c>
       <c r="F253" t="inlineStr">
         <is>
-          <t>12.10 random moves</t>
+          <t>12.19 unique skills</t>
         </is>
       </c>
       <c r="H253" t="inlineStr"/>
     </row>
     <row r="254">
       <c r="A254" t="n">
-        <v>428</v>
+        <v>349</v>
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>Quadruple Money</t>
+          <t>Alter Fate (unique skill)</t>
         </is>
       </c>
       <c r="C254" t="n">
@@ -15677,18 +15677,18 @@
       </c>
       <c r="F254" t="inlineStr">
         <is>
-          <t>6c EXP</t>
+          <t>12.19 unique skills</t>
         </is>
       </c>
       <c r="H254" t="inlineStr"/>
     </row>
     <row r="255">
       <c r="A255" t="n">
-        <v>432</v>
+        <v>350</v>
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>Enemies Flee</t>
+          <t>Usurper of Souls (unique skill)</t>
         </is>
       </c>
       <c r="C255" t="n">
@@ -15704,18 +15704,18 @@
       </c>
       <c r="F255" t="inlineStr">
         <is>
-          <t>12.10 random moves</t>
+          <t>12.19 unique skills</t>
         </is>
       </c>
       <c r="H255" t="inlineStr"/>
     </row>
     <row r="256">
       <c r="A256" t="n">
-        <v>433</v>
+        <v>352</v>
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>Money Loss</t>
+          <t>Wreathed in Glory (unique skill)</t>
         </is>
       </c>
       <c r="C256" t="n">
@@ -15731,23 +15731,18 @@
       </c>
       <c r="F256" t="inlineStr">
         <is>
-          <t>12.10 random moves</t>
-        </is>
-      </c>
-      <c r="G256" t="inlineStr">
-        <is>
-          <t>0x48b490</t>
+          <t>12.19 unique skills</t>
         </is>
       </c>
       <c r="H256" t="inlineStr"/>
     </row>
     <row r="257">
       <c r="A257" t="n">
-        <v>434</v>
+        <v>353</v>
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>User's HP-1 Damage</t>
+          <t>Maximum Maid (unique skill)</t>
         </is>
       </c>
       <c r="C257" t="n">
@@ -15763,18 +15758,18 @@
       </c>
       <c r="F257" t="inlineStr">
         <is>
-          <t>2.7 special damage</t>
+          <t>3 magic attack</t>
         </is>
       </c>
       <c r="H257" t="inlineStr"/>
     </row>
     <row r="258">
       <c r="A258" t="n">
-        <v>435</v>
+        <v>354</v>
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>Fixed Damage Based on User's Level</t>
+          <t>Did You Call for Me? (unique skill)</t>
         </is>
       </c>
       <c r="C258" t="n">
@@ -15790,10 +15785,501 @@
       </c>
       <c r="F258" t="inlineStr">
         <is>
+          <t>12.19 unique skills</t>
+        </is>
+      </c>
+      <c r="H258" t="inlineStr"/>
+    </row>
+    <row r="259">
+      <c r="A259" t="n">
+        <v>355</v>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>Undaunted Spirit (unique skill)</t>
+        </is>
+      </c>
+      <c r="C259" t="n">
+        <v>1</v>
+      </c>
+      <c r="D259" t="n">
+        <v>0</v>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F259" t="inlineStr">
+        <is>
+          <t>12.19 unique skills</t>
+        </is>
+      </c>
+      <c r="H259" t="inlineStr"/>
+    </row>
+    <row r="260">
+      <c r="A260" t="n">
+        <v>356</v>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>Demon Wall (unique skill)</t>
+        </is>
+      </c>
+      <c r="C260" t="n">
+        <v>1</v>
+      </c>
+      <c r="D260" t="n">
+        <v>0</v>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>2 physical attack, 3 magic attack</t>
+        </is>
+      </c>
+      <c r="H260" t="inlineStr"/>
+    </row>
+    <row r="261">
+      <c r="A261" t="n">
+        <v>357</v>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>Tranquil Song (unique skill)</t>
+        </is>
+      </c>
+      <c r="C261" t="n">
+        <v>1</v>
+      </c>
+      <c r="D261" t="n">
+        <v>0</v>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F261" t="inlineStr">
+        <is>
+          <t>12.19 unique skills</t>
+        </is>
+      </c>
+      <c r="H261" t="inlineStr"/>
+    </row>
+    <row r="262">
+      <c r="A262" t="n">
+        <v>358</v>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>Forerunner (unique skill)</t>
+        </is>
+      </c>
+      <c r="C262" t="n">
+        <v>1</v>
+      </c>
+      <c r="D262" t="n">
+        <v>0</v>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F262" t="inlineStr">
+        <is>
+          <t>12.19 unique skills</t>
+        </is>
+      </c>
+      <c r="H262" t="inlineStr"/>
+    </row>
+    <row r="263">
+      <c r="A263" t="n">
+        <v>425</v>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>Cancel Chant, Song, Dance, Doll</t>
+        </is>
+      </c>
+      <c r="C263" t="n">
+        <v>1</v>
+      </c>
+      <c r="D263" t="n">
+        <v>0</v>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F263" t="inlineStr">
+        <is>
+          <t>12.10 random moves</t>
+        </is>
+      </c>
+      <c r="H263" t="inlineStr"/>
+    </row>
+    <row r="264">
+      <c r="A264" t="n">
+        <v>426</v>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>Fixed TP Recovery</t>
+        </is>
+      </c>
+      <c r="C264" t="n">
+        <v>1</v>
+      </c>
+      <c r="D264" t="n">
+        <v>0</v>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F264" t="inlineStr">
+        <is>
+          <t>12.10 random moves</t>
+        </is>
+      </c>
+      <c r="H264" t="inlineStr"/>
+    </row>
+    <row r="265">
+      <c r="A265" t="n">
+        <v>427</v>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>Genjimaru</t>
+        </is>
+      </c>
+      <c r="C265" t="n">
+        <v>1</v>
+      </c>
+      <c r="D265" t="n">
+        <v>0</v>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F265" t="inlineStr">
+        <is>
+          <t>12.10 random moves</t>
+        </is>
+      </c>
+      <c r="H265" t="inlineStr"/>
+    </row>
+    <row r="266">
+      <c r="A266" t="n">
+        <v>428</v>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>Quadruple Money</t>
+        </is>
+      </c>
+      <c r="C266" t="n">
+        <v>1</v>
+      </c>
+      <c r="D266" t="n">
+        <v>0</v>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F266" t="inlineStr">
+        <is>
+          <t>6c EXP</t>
+        </is>
+      </c>
+      <c r="H266" t="inlineStr"/>
+    </row>
+    <row r="267">
+      <c r="A267" t="n">
+        <v>432</v>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>Enemies Flee</t>
+        </is>
+      </c>
+      <c r="C267" t="n">
+        <v>1</v>
+      </c>
+      <c r="D267" t="n">
+        <v>0</v>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>12.10 random moves</t>
+        </is>
+      </c>
+      <c r="H267" t="inlineStr"/>
+    </row>
+    <row r="268">
+      <c r="A268" t="n">
+        <v>433</v>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>Money Loss</t>
+        </is>
+      </c>
+      <c r="C268" t="n">
+        <v>1</v>
+      </c>
+      <c r="D268" t="n">
+        <v>0</v>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F268" t="inlineStr">
+        <is>
+          <t>12.10 random moves</t>
+        </is>
+      </c>
+      <c r="G268" t="inlineStr">
+        <is>
+          <t>0x48b490</t>
+        </is>
+      </c>
+      <c r="H268" t="inlineStr"/>
+    </row>
+    <row r="269">
+      <c r="A269" t="n">
+        <v>434</v>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>User's HP-1 Damage</t>
+        </is>
+      </c>
+      <c r="C269" t="n">
+        <v>1</v>
+      </c>
+      <c r="D269" t="n">
+        <v>0</v>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F269" t="inlineStr">
+        <is>
           <t>2.7 special damage</t>
         </is>
       </c>
-      <c r="H258" t="inlineStr"/>
+      <c r="H269" t="inlineStr"/>
+    </row>
+    <row r="270">
+      <c r="A270" t="n">
+        <v>435</v>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>Fixed Damage Based on User's Level</t>
+        </is>
+      </c>
+      <c r="C270" t="n">
+        <v>1</v>
+      </c>
+      <c r="D270" t="n">
+        <v>0</v>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F270" t="inlineStr">
+        <is>
+          <t>2.7 special damage</t>
+        </is>
+      </c>
+      <c r="H270" t="inlineStr"/>
+    </row>
+    <row r="271">
+      <c r="A271" t="n">
+        <v>440</v>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>Positive Trance (unique skill)</t>
+        </is>
+      </c>
+      <c r="C271" t="n">
+        <v>1</v>
+      </c>
+      <c r="D271" t="n">
+        <v>0</v>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F271" t="inlineStr">
+        <is>
+          <t>2 physical attack</t>
+        </is>
+      </c>
+      <c r="H271" t="inlineStr"/>
+    </row>
+    <row r="272">
+      <c r="A272" t="n">
+        <v>443</v>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>Elbow Grease (unique skill)</t>
+        </is>
+      </c>
+      <c r="C272" t="n">
+        <v>1</v>
+      </c>
+      <c r="D272" t="n">
+        <v>0</v>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F272" t="inlineStr">
+        <is>
+          <t>2 physical attack</t>
+        </is>
+      </c>
+      <c r="H272" t="inlineStr"/>
+    </row>
+    <row r="273">
+      <c r="A273" t="n">
+        <v>446</v>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>Overstock Clearance (unique skill)</t>
+        </is>
+      </c>
+      <c r="C273" t="n">
+        <v>1</v>
+      </c>
+      <c r="D273" t="n">
+        <v>0</v>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F273" t="inlineStr">
+        <is>
+          <t>12.19 unique skills</t>
+        </is>
+      </c>
+      <c r="H273" t="inlineStr"/>
+    </row>
+    <row r="274">
+      <c r="A274" t="n">
+        <v>447</v>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>Arcane Shield (unique skill)</t>
+        </is>
+      </c>
+      <c r="C274" t="n">
+        <v>1</v>
+      </c>
+      <c r="D274" t="n">
+        <v>0</v>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F274" t="inlineStr">
+        <is>
+          <t>12.19 unique skills</t>
+        </is>
+      </c>
+      <c r="H274" t="inlineStr"/>
+    </row>
+    <row r="275">
+      <c r="A275" t="n">
+        <v>448</v>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>Shadow Heart (unique skill)</t>
+        </is>
+      </c>
+      <c r="C275" t="n">
+        <v>1</v>
+      </c>
+      <c r="D275" t="n">
+        <v>0</v>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F275" t="inlineStr">
+        <is>
+          <t>12.19 unique skills</t>
+        </is>
+      </c>
+      <c r="H275" t="inlineStr"/>
+    </row>
+    <row r="276">
+      <c r="A276" t="n">
+        <v>449</v>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>Yearning (unique skill)</t>
+        </is>
+      </c>
+      <c r="C276" t="n">
+        <v>1</v>
+      </c>
+      <c r="D276" t="n">
+        <v>0</v>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F276" t="inlineStr">
+        <is>
+          <t>12.19 unique skills</t>
+        </is>
+      </c>
+      <c r="H276" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -18275,12 +18761,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>in progress</t>
+          <t>read</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Measured by tools/exe_effects.py: docs/generated/EFFECT_COVERAGE.md and the sheet EffectCoverage. Closed when no effect a skill uses is "located" or "not found"</t>
+          <t>Measured by tools/exe_effects.py: docs/generated/EFFECT_COVERAGE.md. Every effect a skill of the player uses is "read"; one effect that only enemy attacks carry (3, Breath Attack) has no reader and is stated as such</t>
         </is>
       </c>
     </row>
@@ -18297,12 +18783,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>partly</t>
+          <t>read</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>docs/FORMULAS.md 12: passive rolls on the target, barrier, dispel, absorption, the ailments of plain attacks and special damage are read; the order of the whole and several branches are not</t>
+          <t>docs/FORMULAS.md 12.9 and 12.12 to 12.15: who takes the hit, what turns it away, the counters, what follows a hit and the order of the states of a turn</t>
         </is>
       </c>
     </row>
@@ -18319,12 +18805,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>partly</t>
+          <t>read</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>docs/FORMULAS.md 12.2: every multi-hit table, Double and Triple Attack read; the number of targets (effect 137) not followed</t>
+          <t>docs/FORMULAS.md 12.2 and sheet EffectRules: every multi-hit table, Double and Triple Attack, the number of targets (137) and the one-per-target rule (112)</t>
         </is>
       </c>
     </row>
@@ -18341,12 +18827,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>partly</t>
+          <t>read</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>docs/FORMULAS.md 12.4 to 12.6: what stops a unit from acting, natural recovery, poison, statuses on stats; when the per-turn method runs is not followed</t>
+          <t>docs/FORMULAS.md 12.4 to 12.6, 12.15 and 12.18: what stops a unit, natural recovery, poison, statuses on stats, when the per-turn method runs, how turns are counted</t>
         </is>
       </c>
     </row>
@@ -18363,12 +18849,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>partly</t>
+          <t>read</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Rolls of Counter, Pretend, Knock Down, Auto-Guard, Reprisal, Survival, First Grid, Warning Shot, Mesmerized located and their chance read (sheet EffectRules); their consequences and the unique skills of the girls are not</t>
+          <t>Every effect of a passive or unique skill is "read" in docs/generated/EFFECT_COVERAGE.md (the 18 unique skills are counted since their effect field was found); docs/FORMULAS.md 12.19</t>
         </is>
       </c>
     </row>
@@ -18385,12 +18871,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>partly</t>
+          <t>read</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>How an effect is built and applied is read (docs/FORMULAS.md 12.1); how long one lasts and whether two stack are not</t>
+          <t>docs/FORMULAS.md 12.18: turns are counted after the action of the bearer (five steps on the map), 0 turns means until removed, a status of the same effect replaces the old one, dispel in 12</t>
         </is>
       </c>
     </row>
@@ -18681,7 +19167,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E189"/>
+  <dimension ref="A1:E203"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -23313,6 +23799,356 @@
         </is>
       </c>
     </row>
+    <row r="190">
+      <c r="A190" t="n">
+        <v>345</v>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>12.19 unique skills</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>Third Eye Wide: at the start of the turn of each opponent (state 2), each bearer rolls below 100 under value * 100; on a success it applies to that unit one of seven effects picked with equal chances: poison, paralysis, sleep, freeze, silence, stun or dispel (table 0x6c9af8), created with a value of 0.75</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>0x43697b, 0x439643</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="n">
+        <v>346</v>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>12.19 unique skills</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>Sugar Coma: when a short-range action is about to hit its bearer, a roll below 100 under value * 100; on a success the attacker receives Slow (value 1) and a speed modifier of -0.2</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>0x422824 - 0x422a3d</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="n">
+        <v>348</v>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>12.19 unique skills</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>Furious Strike: when its bearer starts a physical action, a roll below 100 under value * 100; on a success every hit of the action ignores defence (69) and cannot miss (72)</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>0x417567, 0x42106c</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="n">
+        <v>349</v>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>12.19 unique skills</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>Alter Fate: when a hit is about to land on its bearer, a roll below 100 under value * 100; on a success the hit deals no damage</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>0x421ca9 - 0x421d1d</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="n">
+        <v>350</v>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>12.19 unique skills</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>Usurper of Souls: before the action of its bearer (state 14), a roll below 100 under value * 100; on a success the summoned units of the other side (dolls and the like) are removed from the battle</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>0x4376e9</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="n">
+        <v>352</v>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>12.19 unique skills</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>Wreathed in Glory: its value is added to the speed of the skill or spell its bearer uses, the term the order of turns reads (5)</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>0x4f72a7</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="n">
+        <v>354</v>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>12.19 unique skills</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>Did You Call for Me?: after the action of its bearer, a roll below 100 under value * 100; on a success it acts twice (asked after Double and Triple Action)</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>0x439103</t>
+        </is>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="n">
+        <v>355</v>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>12.19 unique skills</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>Undaunted Spirit: at the end of a turn (state 22), each fallen unit that has it rolls below 100 under value * 100; on a success it rises. The record of the revival carries the value 1 twice, taken to be 1 HP</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>0x43852d - 0x4386b1</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="n">
+        <v>357</v>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>12.19 unique skills</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>Tranquil Song: before the action of its bearer (state 13), a roll below 100 under value * 100; on a success every unit of the other side receives an ATK debuff and an INT debuff of -0.1 (effects 41 and 43), asked for 4 turns</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>0x43749f - 0x437650</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="n">
+        <v>358</v>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>12.19 unique skills</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>Forerunner: when its bearer chooses a spell that needs a chant, a roll below 100 under value * 100; on a success the spell is cast at once (the kind of the command changes from 3 to 2)</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>0x4176c3 - 0x41772d</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="n">
+        <v>446</v>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>12.19 unique skills</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>Overstock Clearance: before the action of its bearer (state 3), a roll below 100 under value * 100; on a success it first uses an item of its own stock</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>0x436aa2</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="n">
+        <v>447</v>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>12.19 unique skills</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>Arcane Shield: after a hit that dealt damage to its bearer (the attacker has no Absolute Attack), a number below 100 under 15, a figure written in the program; on a success the attacker takes int(that damage * value) as fixed damage once the action ends</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>0x424749 - 0x42476e, 0x425157 - 0x425203</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="n">
+        <v>448</v>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>12.19 unique skills</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>Shadow Heart: before the action of its bearer (state 15), a roll below 100 under value * 100; on a success, unless its shadow is already in the battle, a unit of its own is created to attack</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>0x4378e2</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="n">
+        <v>449</v>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>12.19 unique skills</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>Yearning: value * 0.01 is added to each class modifier of its bearer (0x4f7f73; 0.02 more with a piece of enchantment 264)</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>0x4f7f78, 0x4f7fe3</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: which class learns which skill
which class learns which skill, read from the class mask of the skill
files; range and pattern of a skill
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -8706,7 +8706,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -8733,7 +8732,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -8760,7 +8758,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -8787,7 +8784,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -8814,7 +8810,6 @@
           <t>2.7 special damage</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -8841,7 +8836,6 @@
           <t>6b healing</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -8868,7 +8862,6 @@
           <t>actions</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -8895,7 +8888,6 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -8922,7 +8914,6 @@
           <t>2.7 special damage, 3 magic attack</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -8949,7 +8940,6 @@
           <t>outside battle</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -8976,7 +8966,6 @@
           <t>14 encounter rate</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -9008,7 +8997,6 @@
           <t>0x47ffc0</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -9035,7 +9023,6 @@
           <t>outside battle</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -9062,7 +9049,6 @@
           <t>applying a hit</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -9089,7 +9075,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -9116,7 +9101,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -9143,7 +9127,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -9170,7 +9153,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -9197,7 +9179,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -9224,7 +9205,6 @@
           <t>4 critical hits</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -9251,7 +9231,6 @@
           <t>4 critical hits</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -9278,7 +9257,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -9305,7 +9283,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -9332,7 +9309,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -9359,7 +9335,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -9386,7 +9361,6 @@
           <t>5c turn delay</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -9413,7 +9387,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -9440,7 +9413,6 @@
           <t>steal</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -9467,7 +9439,6 @@
           <t>steal</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -9494,7 +9465,6 @@
           <t>steal</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -9526,7 +9496,6 @@
           <t>0x480e20</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -9553,7 +9522,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -9580,7 +9548,6 @@
           <t>4 critical hits</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -9607,7 +9574,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -9634,7 +9600,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -9661,7 +9626,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -9688,7 +9652,6 @@
           <t>applying a hit</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -9715,7 +9678,6 @@
           <t>applying a hit</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -9742,7 +9704,6 @@
           <t>applying a hit</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -9774,7 +9735,6 @@
           <t>0x481060</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -9801,7 +9761,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -9833,7 +9792,6 @@
           <t>0x481160</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -9865,7 +9823,6 @@
           <t>0x4813a0</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -9892,7 +9849,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -9919,7 +9875,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -9946,7 +9901,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -9973,7 +9927,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -10000,7 +9953,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -10027,7 +9979,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -10054,7 +10005,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -10081,7 +10031,6 @@
           <t>12.2 number of hits</t>
         </is>
       </c>
-      <c r="H52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -10108,7 +10057,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -10135,7 +10083,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -10162,7 +10109,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -10189,7 +10135,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -10216,7 +10161,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -10243,7 +10187,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -10270,7 +10213,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -10297,7 +10239,6 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
-      <c r="H60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -10324,7 +10265,6 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
-      <c r="H61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -10356,7 +10296,6 @@
           <t>0x4817c0</t>
         </is>
       </c>
-      <c r="H62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -10388,7 +10327,6 @@
           <t>0x481890</t>
         </is>
       </c>
-      <c r="H63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -10420,7 +10358,6 @@
           <t>0x481950</t>
         </is>
       </c>
-      <c r="H64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -10452,7 +10389,6 @@
           <t>0x481a20</t>
         </is>
       </c>
-      <c r="H65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -10479,7 +10415,6 @@
           <t>outside battle</t>
         </is>
       </c>
-      <c r="H66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -10506,7 +10441,6 @@
           <t>outside battle</t>
         </is>
       </c>
-      <c r="H67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -10533,7 +10467,6 @@
           <t>4 critical hits</t>
         </is>
       </c>
-      <c r="H68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -10560,7 +10493,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -10587,7 +10519,6 @@
           <t>9.1 who gets hit</t>
         </is>
       </c>
-      <c r="H70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -10619,7 +10550,6 @@
           <t>0x481ea0</t>
         </is>
       </c>
-      <c r="H71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -10651,7 +10581,6 @@
           <t>0x4822c0</t>
         </is>
       </c>
-      <c r="H72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -10683,7 +10612,6 @@
           <t>0x482530</t>
         </is>
       </c>
-      <c r="H73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -10715,7 +10643,6 @@
           <t>0x4827a0</t>
         </is>
       </c>
-      <c r="H74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -10747,7 +10674,6 @@
           <t>0x482a10</t>
         </is>
       </c>
-      <c r="H75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -10779,7 +10705,6 @@
           <t>0x482c80</t>
         </is>
       </c>
-      <c r="H76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -10811,7 +10736,6 @@
           <t>0x482e40</t>
         </is>
       </c>
-      <c r="H77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -10843,7 +10767,6 @@
           <t>0x4831f0</t>
         </is>
       </c>
-      <c r="H78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -10875,7 +10798,6 @@
           <t>0x4834b0</t>
         </is>
       </c>
-      <c r="H79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -10907,7 +10829,6 @@
           <t>0x4835d0</t>
         </is>
       </c>
-      <c r="H80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -10939,7 +10860,6 @@
           <t>0x483840</t>
         </is>
       </c>
-      <c r="H81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -10966,7 +10886,6 @@
           <t>4 critical hits</t>
         </is>
       </c>
-      <c r="H82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -10998,7 +10917,6 @@
           <t>0x483a60</t>
         </is>
       </c>
-      <c r="H83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -11030,7 +10948,6 @@
           <t>0x483b30</t>
         </is>
       </c>
-      <c r="H84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -11062,7 +10979,6 @@
           <t>0x483c20</t>
         </is>
       </c>
-      <c r="H85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -11094,7 +11010,6 @@
           <t>0x483d20</t>
         </is>
       </c>
-      <c r="H86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -11126,7 +11041,6 @@
           <t>0x483e00</t>
         </is>
       </c>
-      <c r="H87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -11158,7 +11072,6 @@
           <t>0x483ee0</t>
         </is>
       </c>
-      <c r="H88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -11185,7 +11098,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -11212,7 +11124,6 @@
           <t>9.1 who gets hit</t>
         </is>
       </c>
-      <c r="H90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -11239,7 +11150,6 @@
           <t>2.7 special damage</t>
         </is>
       </c>
-      <c r="H91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -11271,7 +11181,6 @@
           <t>0x484020</t>
         </is>
       </c>
-      <c r="H92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -11298,7 +11207,6 @@
           <t>2.7 special damage</t>
         </is>
       </c>
-      <c r="H93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -11325,7 +11233,6 @@
           <t>2.7 special damage</t>
         </is>
       </c>
-      <c r="H94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -11357,7 +11264,6 @@
           <t>0x484150</t>
         </is>
       </c>
-      <c r="H95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -11389,7 +11295,6 @@
           <t>0x484330</t>
         </is>
       </c>
-      <c r="H96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -11416,7 +11321,6 @@
           <t>11.1 dolls</t>
         </is>
       </c>
-      <c r="H97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -11443,7 +11347,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -11470,7 +11373,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -11497,7 +11399,6 @@
           <t>12.10 random moves</t>
         </is>
       </c>
-      <c r="H100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -11524,7 +11425,6 @@
           <t>12.10 random moves</t>
         </is>
       </c>
-      <c r="H101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -11551,7 +11451,6 @@
           <t>12.10 random moves</t>
         </is>
       </c>
-      <c r="H102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -11578,7 +11477,6 @@
           <t>12.10 random moves</t>
         </is>
       </c>
-      <c r="H103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -11605,7 +11503,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -11632,7 +11529,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -11659,7 +11555,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -11686,7 +11581,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -11713,7 +11607,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="n">
@@ -11740,7 +11633,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="n">
@@ -11767,7 +11659,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -11799,7 +11690,6 @@
           <t>0x4864c0</t>
         </is>
       </c>
-      <c r="H111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="n">
@@ -11826,7 +11716,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="n">
@@ -11853,7 +11742,6 @@
           <t>9.1 targets</t>
         </is>
       </c>
-      <c r="H113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -11880,7 +11768,6 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
-      <c r="H114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="n">
@@ -11907,7 +11794,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="n">
@@ -11934,7 +11820,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="n">
@@ -11961,7 +11846,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="n">
@@ -11988,7 +11872,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="n">
@@ -12015,7 +11898,6 @@
           <t>applying a hit</t>
         </is>
       </c>
-      <c r="H119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="n">
@@ -12042,7 +11924,6 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
-      <c r="H120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="n">
@@ -12069,7 +11950,6 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
-      <c r="H121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="n">
@@ -12096,7 +11976,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="n">
@@ -12123,7 +12002,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="n">
@@ -12150,7 +12028,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="n">
@@ -12177,7 +12054,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="n">
@@ -12204,7 +12080,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="n">
@@ -12231,7 +12106,6 @@
           <t>2.8 damage received</t>
         </is>
       </c>
-      <c r="H127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="n">
@@ -12258,7 +12132,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="n">
@@ -12285,7 +12158,6 @@
           <t>2 physical attack, 2.4 other bonuses of final damage, 3 magic attack</t>
         </is>
       </c>
-      <c r="H129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="n">
@@ -12312,7 +12184,6 @@
           <t>2 physical attack, 2.4 other bonuses of final damage</t>
         </is>
       </c>
-      <c r="H130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="n">
@@ -12339,7 +12210,6 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
-      <c r="H131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="n">
@@ -12366,7 +12236,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="n">
@@ -12393,7 +12262,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -12420,7 +12288,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="n">
@@ -12447,7 +12314,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="n">
@@ -12474,7 +12340,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="n">
@@ -12501,7 +12366,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="n">
@@ -12528,7 +12392,6 @@
           <t>5e effects that act every turn</t>
         </is>
       </c>
-      <c r="H138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="n">
@@ -12555,7 +12418,6 @@
           <t>5e effects that act every turn</t>
         </is>
       </c>
-      <c r="H139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="n">
@@ -12582,7 +12444,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="n">
@@ -12609,7 +12470,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="n">
@@ -12636,7 +12496,6 @@
           <t>5d start of a turn</t>
         </is>
       </c>
-      <c r="H142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="n">
@@ -12663,7 +12522,6 @@
           <t>13 Pep</t>
         </is>
       </c>
-      <c r="H143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="n">
@@ -12690,7 +12548,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="n">
@@ -12717,7 +12574,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="n">
@@ -12744,7 +12600,6 @@
           <t>4 critical hits</t>
         </is>
       </c>
-      <c r="H146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="n">
@@ -12771,7 +12626,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="n">
@@ -12798,7 +12652,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="n">
@@ -12825,7 +12678,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="n">
@@ -12857,7 +12709,6 @@
           <t>0x4894a0</t>
         </is>
       </c>
-      <c r="H150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="n">
@@ -12889,7 +12740,6 @@
           <t>0x4895e0</t>
         </is>
       </c>
-      <c r="H151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="n">
@@ -12916,7 +12766,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="n">
@@ -12943,7 +12792,6 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
-      <c r="H153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="n">
@@ -12970,7 +12818,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="n">
@@ -12997,7 +12844,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="n">
@@ -13024,7 +12870,6 @@
           <t>2 physical attack, 5 order of turns</t>
         </is>
       </c>
-      <c r="H156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="n">
@@ -13051,7 +12896,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" t="n">
@@ -13078,7 +12922,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="n">
@@ -13105,7 +12948,6 @@
           <t>11.1 dolls</t>
         </is>
       </c>
-      <c r="H159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="n">
@@ -13132,7 +12974,6 @@
           <t>11.1 dolls</t>
         </is>
       </c>
-      <c r="H160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" t="n">
@@ -13159,7 +13000,6 @@
           <t>11.1 dolls</t>
         </is>
       </c>
-      <c r="H161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" t="n">
@@ -13186,7 +13026,6 @@
           <t>11.1 dolls</t>
         </is>
       </c>
-      <c r="H162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" t="n">
@@ -13213,7 +13052,6 @@
           <t>11.1 dolls</t>
         </is>
       </c>
-      <c r="H163" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" t="n">
@@ -13240,7 +13078,6 @@
           <t>11.1 dolls</t>
         </is>
       </c>
-      <c r="H164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="n">
@@ -13272,7 +13109,6 @@
           <t>0x48a430</t>
         </is>
       </c>
-      <c r="H165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="n">
@@ -13299,7 +13135,6 @@
           <t>10.1 stats of a piece of equipment</t>
         </is>
       </c>
-      <c r="H166" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" t="n">
@@ -13326,7 +13161,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H167" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" t="n">
@@ -13353,7 +13187,6 @@
           <t>6b healing</t>
         </is>
       </c>
-      <c r="H168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="n">
@@ -13385,7 +13218,6 @@
           <t>0x48a640</t>
         </is>
       </c>
-      <c r="H169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" t="n">
@@ -13412,7 +13244,6 @@
           <t>5e effects that act every turn</t>
         </is>
       </c>
-      <c r="H170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="n">
@@ -13439,7 +13270,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="n">
@@ -13466,7 +13296,6 @@
           <t>12.13 counters and follow-ups</t>
         </is>
       </c>
-      <c r="H172" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" t="n">
@@ -13493,7 +13322,6 @@
           <t>12.13 counters and follow-ups</t>
         </is>
       </c>
-      <c r="H173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="n">
@@ -13520,7 +13348,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H174" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" t="n">
@@ -13547,7 +13374,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" t="n">
@@ -13574,7 +13400,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H176" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" t="n">
@@ -13601,7 +13426,6 @@
           <t>passive rolls</t>
         </is>
       </c>
-      <c r="H177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="n">
@@ -13628,7 +13452,6 @@
           <t>passive rolls</t>
         </is>
       </c>
-      <c r="H178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" t="n">
@@ -13655,7 +13478,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H179" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" t="n">
@@ -13682,7 +13504,6 @@
           <t>2.8 damage received</t>
         </is>
       </c>
-      <c r="H180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" t="n">
@@ -13709,7 +13530,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H181" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" t="n">
@@ -13736,7 +13556,6 @@
           <t>5d start of a turn</t>
         </is>
       </c>
-      <c r="H182" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" t="n">
@@ -13763,7 +13582,6 @@
           <t>12.13 counters and follow-ups</t>
         </is>
       </c>
-      <c r="H183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="n">
@@ -13790,7 +13608,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="n">
@@ -13817,7 +13634,6 @@
           <t>12.9 after a hit</t>
         </is>
       </c>
-      <c r="H185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="n">
@@ -13844,7 +13660,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H186" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" t="n">
@@ -13871,7 +13686,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="n">
@@ -13898,7 +13712,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H188" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" t="n">
@@ -13925,7 +13738,6 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
-      <c r="H189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" t="n">
@@ -13952,7 +13764,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H190" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" t="n">
@@ -13979,7 +13790,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" t="n">
@@ -14006,7 +13816,6 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
-      <c r="H192" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" t="n">
@@ -14033,7 +13842,6 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
-      <c r="H193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" t="n">
@@ -14060,7 +13868,6 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
-      <c r="H194" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" t="n">
@@ -14087,7 +13894,6 @@
           <t>after a battle</t>
         </is>
       </c>
-      <c r="H195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" t="n">
@@ -14114,7 +13920,6 @@
           <t>after a battle</t>
         </is>
       </c>
-      <c r="H196" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" t="n">
@@ -14141,7 +13946,6 @@
           <t>passive rolls</t>
         </is>
       </c>
-      <c r="H197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" t="n">
@@ -14168,7 +13972,6 @@
           <t>items</t>
         </is>
       </c>
-      <c r="H198" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" t="n">
@@ -14195,7 +13998,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H199" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" t="n">
@@ -14222,7 +14024,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H200" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" t="n">
@@ -14249,7 +14050,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H201" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" t="n">
@@ -14276,7 +14076,6 @@
           <t>11.2 songs and dances</t>
         </is>
       </c>
-      <c r="H202" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" t="n">
@@ -14303,7 +14102,6 @@
           <t>11.2 songs and dances</t>
         </is>
       </c>
-      <c r="H203" t="inlineStr"/>
     </row>
     <row r="204">
       <c r="A204" t="n">
@@ -14330,7 +14128,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H204" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" t="n">
@@ -14357,7 +14154,6 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
-      <c r="H205" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" t="n">
@@ -14384,7 +14180,6 @@
           <t>5d start of a turn</t>
         </is>
       </c>
-      <c r="H206" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" t="n">
@@ -14411,7 +14206,6 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
-      <c r="H207" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" t="n">
@@ -14438,7 +14232,6 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
-      <c r="H208" t="inlineStr"/>
     </row>
     <row r="209">
       <c r="A209" t="n">
@@ -14465,7 +14258,6 @@
           <t>11.1 dolls, 2 physical attack, 3 magic attack, 6b healing</t>
         </is>
       </c>
-      <c r="H209" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" t="n">
@@ -14492,7 +14284,6 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
-      <c r="H210" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" t="n">
@@ -14519,7 +14310,6 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
-      <c r="H211" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" t="n">
@@ -14546,7 +14336,6 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
-      <c r="H212" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" t="n">
@@ -14573,7 +14362,6 @@
           <t>2.8 damage received</t>
         </is>
       </c>
-      <c r="H213" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" t="n">
@@ -14600,7 +14388,6 @@
           <t>12.9 after a hit</t>
         </is>
       </c>
-      <c r="H214" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" t="n">
@@ -14627,7 +14414,6 @@
           <t>6b heal cap, 6b healing</t>
         </is>
       </c>
-      <c r="H215" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" t="n">
@@ -14654,7 +14440,6 @@
           <t>3 magic attack, 6b heal cap</t>
         </is>
       </c>
-      <c r="H216" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" t="n">
@@ -14681,7 +14466,6 @@
           <t>11.1 dolls</t>
         </is>
       </c>
-      <c r="H217" t="inlineStr"/>
     </row>
     <row r="218">
       <c r="A218" t="n">
@@ -14708,7 +14492,6 @@
           <t>10.1 stats of a piece of equipment</t>
         </is>
       </c>
-      <c r="H218" t="inlineStr"/>
     </row>
     <row r="219">
       <c r="A219" t="n">
@@ -14735,7 +14518,6 @@
           <t>passive rolls</t>
         </is>
       </c>
-      <c r="H219" t="inlineStr"/>
     </row>
     <row r="220">
       <c r="A220" t="n">
@@ -14762,7 +14544,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H220" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" t="n">
@@ -14789,7 +14570,6 @@
           <t>12.13 counters and follow-ups</t>
         </is>
       </c>
-      <c r="H221" t="inlineStr"/>
     </row>
     <row r="222">
       <c r="A222" t="n">
@@ -14816,7 +14596,6 @@
           <t>12.9 after a hit</t>
         </is>
       </c>
-      <c r="H222" t="inlineStr"/>
     </row>
     <row r="223">
       <c r="A223" t="n">
@@ -14843,7 +14622,6 @@
           <t>applying a hit</t>
         </is>
       </c>
-      <c r="H223" t="inlineStr"/>
     </row>
     <row r="224">
       <c r="A224" t="n">
@@ -14870,7 +14648,6 @@
           <t>outside battle</t>
         </is>
       </c>
-      <c r="H224" t="inlineStr"/>
     </row>
     <row r="225">
       <c r="A225" t="n">
@@ -14897,7 +14674,6 @@
           <t>12.13 counters and follow-ups</t>
         </is>
       </c>
-      <c r="H225" t="inlineStr"/>
     </row>
     <row r="226">
       <c r="A226" t="n">
@@ -14924,7 +14700,6 @@
           <t>2 physical attack, 2.4 other bonuses of final damage</t>
         </is>
       </c>
-      <c r="H226" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" t="n">
@@ -14951,7 +14726,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H227" t="inlineStr"/>
     </row>
     <row r="228">
       <c r="A228" t="n">
@@ -14978,7 +14752,6 @@
           <t>applying a hit</t>
         </is>
       </c>
-      <c r="H228" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" t="n">
@@ -15005,7 +14778,6 @@
           <t>5d start of a turn</t>
         </is>
       </c>
-      <c r="H229" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" t="n">
@@ -15032,7 +14804,6 @@
           <t>2.8 damage received</t>
         </is>
       </c>
-      <c r="H230" t="inlineStr"/>
     </row>
     <row r="231">
       <c r="A231" t="n">
@@ -15059,7 +14830,6 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
-      <c r="H231" t="inlineStr"/>
     </row>
     <row r="232">
       <c r="A232" t="n">
@@ -15086,7 +14856,6 @@
           <t>11.1 dolls</t>
         </is>
       </c>
-      <c r="H232" t="inlineStr"/>
     </row>
     <row r="233">
       <c r="A233" t="n">
@@ -15113,7 +14882,6 @@
           <t>12.10 random moves</t>
         </is>
       </c>
-      <c r="H233" t="inlineStr"/>
     </row>
     <row r="234">
       <c r="A234" t="n">
@@ -15140,7 +14908,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H234" t="inlineStr"/>
     </row>
     <row r="235">
       <c r="A235" t="n">
@@ -15167,7 +14934,6 @@
           <t>6b heal cap</t>
         </is>
       </c>
-      <c r="H235" t="inlineStr"/>
     </row>
     <row r="236">
       <c r="A236" t="n">
@@ -15194,7 +14960,6 @@
           <t>9 enemy AI</t>
         </is>
       </c>
-      <c r="H236" t="inlineStr"/>
     </row>
     <row r="237">
       <c r="A237" t="n">
@@ -15221,7 +14986,6 @@
           <t>12.9 after a hit</t>
         </is>
       </c>
-      <c r="H237" t="inlineStr"/>
     </row>
     <row r="238">
       <c r="A238" t="n">
@@ -15248,7 +15012,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H238" t="inlineStr"/>
     </row>
     <row r="239">
       <c r="A239" t="n">
@@ -15275,7 +15038,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H239" t="inlineStr"/>
     </row>
     <row r="240">
       <c r="A240" t="n">
@@ -15302,7 +15064,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H240" t="inlineStr"/>
     </row>
     <row r="241">
       <c r="A241" t="n">
@@ -15329,7 +15090,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H241" t="inlineStr"/>
     </row>
     <row r="242">
       <c r="A242" t="n">
@@ -15356,7 +15116,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H242" t="inlineStr"/>
     </row>
     <row r="243">
       <c r="A243" t="n">
@@ -15383,7 +15142,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H243" t="inlineStr"/>
     </row>
     <row r="244">
       <c r="A244" t="n">
@@ -15410,7 +15168,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H244" t="inlineStr"/>
     </row>
     <row r="245">
       <c r="A245" t="n">
@@ -15437,7 +15194,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H245" t="inlineStr"/>
     </row>
     <row r="246">
       <c r="A246" t="n">
@@ -15464,7 +15220,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H246" t="inlineStr"/>
     </row>
     <row r="247">
       <c r="A247" t="n">
@@ -15491,7 +15246,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H247" t="inlineStr"/>
     </row>
     <row r="248">
       <c r="A248" t="n">
@@ -15518,7 +15272,6 @@
           <t>5e effects that act every turn</t>
         </is>
       </c>
-      <c r="H248" t="inlineStr"/>
     </row>
     <row r="249">
       <c r="A249" t="n">
@@ -15545,7 +15298,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H249" t="inlineStr"/>
     </row>
     <row r="250">
       <c r="A250" t="n">
@@ -15572,7 +15324,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H250" t="inlineStr"/>
     </row>
     <row r="251">
       <c r="A251" t="n">
@@ -15599,7 +15350,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H251" t="inlineStr"/>
     </row>
     <row r="252">
       <c r="A252" t="n">
@@ -15626,7 +15376,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H252" t="inlineStr"/>
     </row>
     <row r="253">
       <c r="A253" t="n">
@@ -15653,7 +15402,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H253" t="inlineStr"/>
     </row>
     <row r="254">
       <c r="A254" t="n">
@@ -15680,7 +15428,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H254" t="inlineStr"/>
     </row>
     <row r="255">
       <c r="A255" t="n">
@@ -15707,7 +15454,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H255" t="inlineStr"/>
     </row>
     <row r="256">
       <c r="A256" t="n">
@@ -15734,7 +15480,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H256" t="inlineStr"/>
     </row>
     <row r="257">
       <c r="A257" t="n">
@@ -15761,7 +15506,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H257" t="inlineStr"/>
     </row>
     <row r="258">
       <c r="A258" t="n">
@@ -15788,7 +15532,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H258" t="inlineStr"/>
     </row>
     <row r="259">
       <c r="A259" t="n">
@@ -15815,7 +15558,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H259" t="inlineStr"/>
     </row>
     <row r="260">
       <c r="A260" t="n">
@@ -15842,7 +15584,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H260" t="inlineStr"/>
     </row>
     <row r="261">
       <c r="A261" t="n">
@@ -15869,7 +15610,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H261" t="inlineStr"/>
     </row>
     <row r="262">
       <c r="A262" t="n">
@@ -15896,7 +15636,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H262" t="inlineStr"/>
     </row>
     <row r="263">
       <c r="A263" t="n">
@@ -15923,7 +15662,6 @@
           <t>12.10 random moves</t>
         </is>
       </c>
-      <c r="H263" t="inlineStr"/>
     </row>
     <row r="264">
       <c r="A264" t="n">
@@ -15950,7 +15688,6 @@
           <t>12.10 random moves</t>
         </is>
       </c>
-      <c r="H264" t="inlineStr"/>
     </row>
     <row r="265">
       <c r="A265" t="n">
@@ -15977,7 +15714,6 @@
           <t>12.10 random moves</t>
         </is>
       </c>
-      <c r="H265" t="inlineStr"/>
     </row>
     <row r="266">
       <c r="A266" t="n">
@@ -16004,7 +15740,6 @@
           <t>6c EXP</t>
         </is>
       </c>
-      <c r="H266" t="inlineStr"/>
     </row>
     <row r="267">
       <c r="A267" t="n">
@@ -16031,7 +15766,6 @@
           <t>12.10 random moves</t>
         </is>
       </c>
-      <c r="H267" t="inlineStr"/>
     </row>
     <row r="268">
       <c r="A268" t="n">
@@ -16063,7 +15797,6 @@
           <t>0x48b490</t>
         </is>
       </c>
-      <c r="H268" t="inlineStr"/>
     </row>
     <row r="269">
       <c r="A269" t="n">
@@ -16090,7 +15823,6 @@
           <t>2.7 special damage</t>
         </is>
       </c>
-      <c r="H269" t="inlineStr"/>
     </row>
     <row r="270">
       <c r="A270" t="n">
@@ -16117,7 +15849,6 @@
           <t>2.7 special damage</t>
         </is>
       </c>
-      <c r="H270" t="inlineStr"/>
     </row>
     <row r="271">
       <c r="A271" t="n">
@@ -16144,7 +15875,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H271" t="inlineStr"/>
     </row>
     <row r="272">
       <c r="A272" t="n">
@@ -16171,7 +15901,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H272" t="inlineStr"/>
     </row>
     <row r="273">
       <c r="A273" t="n">
@@ -16198,7 +15927,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H273" t="inlineStr"/>
     </row>
     <row r="274">
       <c r="A274" t="n">
@@ -16225,7 +15953,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H274" t="inlineStr"/>
     </row>
     <row r="275">
       <c r="A275" t="n">
@@ -16252,7 +15979,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H275" t="inlineStr"/>
     </row>
     <row r="276">
       <c r="A276" t="n">
@@ -16279,7 +16005,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H276" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -18893,12 +18618,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>not read</t>
+          <t>read</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>ClassData is ten unnamed ints; the skill files hold a group field not decoded</t>
+          <t>tools/skill_tree_data.py and docs/generated/BALANCE_BASELINE.md: the class mask of every skill file (confirmed at 0x56dc10), SP cost per level, pattern of the action, range of a technique. At what level a skill opens was not looked for: SP is the only cost the files carry</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: class modifiers read from the tables of the executable
class modifiers read from the tables of the executable (38 tables, the
rule of the gain, Yearning)
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -18442,7 +18442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -18878,6 +18878,28 @@
       <c r="D20" t="inlineStr">
         <is>
           <t>tools/ and docs/generated/</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Class modifiers</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>What a class gains from the weapon or piece it specialises in</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>tools/class_modifier_data.py, docs/FORMULAS.md 10.4: 38 tables of the executable, the rule of the gain, Yearning. Which piece slots 2 to 4 are on screen was not checked</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: guest allies read from NPC.pck
guest allies read from NPC.pck; passive skills of enemies read from
their status record
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -18652,7 +18652,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Mercenaries</t>
+          <t>Guest allies (the program calls them NPC)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -18662,12 +18662,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>not read</t>
+          <t>read</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Their table (program global 0x738a04) is not located in the data files yet</t>
+          <t>tools/npc_data.py and docs/generated/BALANCE_BASELINE.md: NPC.pck, 107 records of 31 allies: level, six stats, HP, attacks, passive, script. Three ints of the record are not identified</t>
         </is>
       </c>
     </row>
@@ -18772,12 +18772,12 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>not read</t>
+          <t>read</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Row S03. Where they are stored is not known</t>
+          <t>tools/enemy_data.py: up to five ids at 0xF4 of the status record, entries of EnemyAttackData; listed with their effects in docs/generated/BALANCE_BASELINE.md, and their effects are in the effect coverage</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: item effect types, enemy attack fields named, joint skill power
item effect types, enemy attack fields named, joint skill power; the
extraction checklist has no open row
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -8706,6 +8706,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -8732,6 +8733,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -8758,6 +8760,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -8784,6 +8787,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -8810,6 +8814,7 @@
           <t>2.7 special damage</t>
         </is>
       </c>
+      <c r="H6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -8836,6 +8841,7 @@
           <t>6b healing</t>
         </is>
       </c>
+      <c r="H7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -8862,6 +8868,7 @@
           <t>actions</t>
         </is>
       </c>
+      <c r="H8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -8888,6 +8895,7 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
+      <c r="H9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -8914,6 +8922,7 @@
           <t>2.7 special damage, 3 magic attack</t>
         </is>
       </c>
+      <c r="H10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -8940,6 +8949,7 @@
           <t>outside battle</t>
         </is>
       </c>
+      <c r="H11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -8966,6 +8976,7 @@
           <t>14 encounter rate</t>
         </is>
       </c>
+      <c r="H12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -8997,6 +9008,7 @@
           <t>0x47ffc0</t>
         </is>
       </c>
+      <c r="H13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -9023,6 +9035,7 @@
           <t>outside battle</t>
         </is>
       </c>
+      <c r="H14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -9049,6 +9062,7 @@
           <t>applying a hit</t>
         </is>
       </c>
+      <c r="H15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -9075,6 +9089,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -9101,6 +9116,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -9127,6 +9143,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -9153,6 +9170,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -9179,6 +9197,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -9205,6 +9224,7 @@
           <t>4 critical hits</t>
         </is>
       </c>
+      <c r="H21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -9231,6 +9251,7 @@
           <t>4 critical hits</t>
         </is>
       </c>
+      <c r="H22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -9257,6 +9278,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -9283,6 +9305,7 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
+      <c r="H24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -9309,6 +9332,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -9335,6 +9359,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -9361,6 +9386,7 @@
           <t>5c turn delay</t>
         </is>
       </c>
+      <c r="H27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -9387,6 +9413,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -9413,6 +9440,7 @@
           <t>steal</t>
         </is>
       </c>
+      <c r="H29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -9439,6 +9467,7 @@
           <t>steal</t>
         </is>
       </c>
+      <c r="H30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -9465,6 +9494,7 @@
           <t>steal</t>
         </is>
       </c>
+      <c r="H31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -9496,6 +9526,7 @@
           <t>0x480e20</t>
         </is>
       </c>
+      <c r="H32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -9522,6 +9553,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -9548,6 +9580,7 @@
           <t>4 critical hits</t>
         </is>
       </c>
+      <c r="H34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -9574,6 +9607,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -9600,6 +9634,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -9626,6 +9661,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -9652,6 +9688,7 @@
           <t>applying a hit</t>
         </is>
       </c>
+      <c r="H38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -9678,6 +9715,7 @@
           <t>applying a hit</t>
         </is>
       </c>
+      <c r="H39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -9704,6 +9742,7 @@
           <t>applying a hit</t>
         </is>
       </c>
+      <c r="H40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -9735,6 +9774,7 @@
           <t>0x481060</t>
         </is>
       </c>
+      <c r="H41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -9761,6 +9801,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -9792,6 +9833,7 @@
           <t>0x481160</t>
         </is>
       </c>
+      <c r="H43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -9823,6 +9865,7 @@
           <t>0x4813a0</t>
         </is>
       </c>
+      <c r="H44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -9849,6 +9892,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -9875,6 +9919,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -9901,6 +9946,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -9927,6 +9973,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -9953,6 +10000,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -9979,6 +10027,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -10005,6 +10054,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -10031,6 +10081,7 @@
           <t>12.2 number of hits</t>
         </is>
       </c>
+      <c r="H52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -10057,6 +10108,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -10083,6 +10135,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -10109,6 +10162,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -10135,6 +10189,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -10161,6 +10216,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -10187,6 +10243,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -10213,6 +10270,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -10239,6 +10297,7 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
+      <c r="H60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -10265,6 +10324,7 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
+      <c r="H61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -10296,6 +10356,7 @@
           <t>0x4817c0</t>
         </is>
       </c>
+      <c r="H62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -10327,6 +10388,7 @@
           <t>0x481890</t>
         </is>
       </c>
+      <c r="H63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -10358,6 +10420,7 @@
           <t>0x481950</t>
         </is>
       </c>
+      <c r="H64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -10389,6 +10452,7 @@
           <t>0x481a20</t>
         </is>
       </c>
+      <c r="H65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -10415,6 +10479,7 @@
           <t>outside battle</t>
         </is>
       </c>
+      <c r="H66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -10441,6 +10506,7 @@
           <t>outside battle</t>
         </is>
       </c>
+      <c r="H67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -10467,6 +10533,7 @@
           <t>4 critical hits</t>
         </is>
       </c>
+      <c r="H68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -10493,6 +10560,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -10519,6 +10587,7 @@
           <t>9.1 who gets hit</t>
         </is>
       </c>
+      <c r="H70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -10550,6 +10619,7 @@
           <t>0x481ea0</t>
         </is>
       </c>
+      <c r="H71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -10581,6 +10651,7 @@
           <t>0x4822c0</t>
         </is>
       </c>
+      <c r="H72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -10612,6 +10683,7 @@
           <t>0x482530</t>
         </is>
       </c>
+      <c r="H73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -10643,6 +10715,7 @@
           <t>0x4827a0</t>
         </is>
       </c>
+      <c r="H74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -10674,6 +10747,7 @@
           <t>0x482a10</t>
         </is>
       </c>
+      <c r="H75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -10705,6 +10779,7 @@
           <t>0x482c80</t>
         </is>
       </c>
+      <c r="H76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -10736,6 +10811,7 @@
           <t>0x482e40</t>
         </is>
       </c>
+      <c r="H77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -10767,6 +10843,7 @@
           <t>0x4831f0</t>
         </is>
       </c>
+      <c r="H78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -10798,6 +10875,7 @@
           <t>0x4834b0</t>
         </is>
       </c>
+      <c r="H79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -10829,6 +10907,7 @@
           <t>0x4835d0</t>
         </is>
       </c>
+      <c r="H80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -10860,6 +10939,7 @@
           <t>0x483840</t>
         </is>
       </c>
+      <c r="H81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -10886,6 +10966,7 @@
           <t>4 critical hits</t>
         </is>
       </c>
+      <c r="H82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -10917,6 +10998,7 @@
           <t>0x483a60</t>
         </is>
       </c>
+      <c r="H83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -10948,6 +11030,7 @@
           <t>0x483b30</t>
         </is>
       </c>
+      <c r="H84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -10979,6 +11062,7 @@
           <t>0x483c20</t>
         </is>
       </c>
+      <c r="H85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -11010,6 +11094,7 @@
           <t>0x483d20</t>
         </is>
       </c>
+      <c r="H86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -11041,6 +11126,7 @@
           <t>0x483e00</t>
         </is>
       </c>
+      <c r="H87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -11072,6 +11158,7 @@
           <t>0x483ee0</t>
         </is>
       </c>
+      <c r="H88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -11098,6 +11185,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -11124,6 +11212,7 @@
           <t>9.1 who gets hit</t>
         </is>
       </c>
+      <c r="H90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -11150,6 +11239,7 @@
           <t>2.7 special damage</t>
         </is>
       </c>
+      <c r="H91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -11181,6 +11271,7 @@
           <t>0x484020</t>
         </is>
       </c>
+      <c r="H92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -11207,6 +11298,7 @@
           <t>2.7 special damage</t>
         </is>
       </c>
+      <c r="H93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -11233,6 +11325,7 @@
           <t>2.7 special damage</t>
         </is>
       </c>
+      <c r="H94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -11264,6 +11357,7 @@
           <t>0x484150</t>
         </is>
       </c>
+      <c r="H95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -11295,6 +11389,7 @@
           <t>0x484330</t>
         </is>
       </c>
+      <c r="H96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -11321,6 +11416,7 @@
           <t>11.1 dolls</t>
         </is>
       </c>
+      <c r="H97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -11347,6 +11443,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -11373,6 +11470,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -11399,6 +11497,7 @@
           <t>12.10 random moves</t>
         </is>
       </c>
+      <c r="H100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -11425,6 +11524,7 @@
           <t>12.10 random moves</t>
         </is>
       </c>
+      <c r="H101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -11451,6 +11551,7 @@
           <t>12.10 random moves</t>
         </is>
       </c>
+      <c r="H102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -11477,6 +11578,7 @@
           <t>12.10 random moves</t>
         </is>
       </c>
+      <c r="H103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -11503,6 +11605,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -11529,6 +11632,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -11555,6 +11659,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -11581,6 +11686,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -11607,6 +11713,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="n">
@@ -11633,6 +11740,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="n">
@@ -11659,6 +11767,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -11690,6 +11799,7 @@
           <t>0x4864c0</t>
         </is>
       </c>
+      <c r="H111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="n">
@@ -11716,6 +11826,7 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
+      <c r="H112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="n">
@@ -11742,6 +11853,7 @@
           <t>9.1 targets</t>
         </is>
       </c>
+      <c r="H113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -11768,6 +11880,7 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
+      <c r="H114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="n">
@@ -11794,6 +11907,7 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
+      <c r="H115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="n">
@@ -11820,6 +11934,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="n">
@@ -11846,6 +11961,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="n">
@@ -11872,6 +11988,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="n">
@@ -11898,6 +12015,7 @@
           <t>applying a hit</t>
         </is>
       </c>
+      <c r="H119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="n">
@@ -11924,6 +12042,7 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
+      <c r="H120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="n">
@@ -11950,6 +12069,7 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
+      <c r="H121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="n">
@@ -11976,6 +12096,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="n">
@@ -12002,6 +12123,7 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
+      <c r="H123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="n">
@@ -12028,6 +12150,7 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
+      <c r="H124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="n">
@@ -12054,6 +12177,7 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
+      <c r="H125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="n">
@@ -12080,6 +12204,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="n">
@@ -12106,6 +12231,7 @@
           <t>2.8 damage received</t>
         </is>
       </c>
+      <c r="H127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="n">
@@ -12132,6 +12258,7 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
+      <c r="H128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="n">
@@ -12158,6 +12285,7 @@
           <t>2 physical attack, 2.4 other bonuses of final damage, 3 magic attack</t>
         </is>
       </c>
+      <c r="H129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="n">
@@ -12184,6 +12312,7 @@
           <t>2 physical attack, 2.4 other bonuses of final damage</t>
         </is>
       </c>
+      <c r="H130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="n">
@@ -12210,6 +12339,7 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
+      <c r="H131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="n">
@@ -12236,6 +12366,7 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
+      <c r="H132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="n">
@@ -12262,6 +12393,7 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
+      <c r="H133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -12288,6 +12420,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="n">
@@ -12314,6 +12447,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="n">
@@ -12340,6 +12474,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="n">
@@ -12366,6 +12501,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="n">
@@ -12392,6 +12528,7 @@
           <t>5e effects that act every turn</t>
         </is>
       </c>
+      <c r="H138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="n">
@@ -12418,6 +12555,7 @@
           <t>5e effects that act every turn</t>
         </is>
       </c>
+      <c r="H139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="n">
@@ -12444,6 +12582,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="n">
@@ -12470,6 +12609,7 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
+      <c r="H141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="n">
@@ -12496,6 +12636,7 @@
           <t>5d start of a turn</t>
         </is>
       </c>
+      <c r="H142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="n">
@@ -12522,6 +12663,7 @@
           <t>13 Pep</t>
         </is>
       </c>
+      <c r="H143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="n">
@@ -12548,6 +12690,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="n">
@@ -12574,6 +12717,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="n">
@@ -12600,6 +12744,7 @@
           <t>4 critical hits</t>
         </is>
       </c>
+      <c r="H146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="n">
@@ -12626,6 +12771,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="n">
@@ -12652,6 +12798,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="n">
@@ -12678,6 +12825,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="n">
@@ -12709,6 +12857,7 @@
           <t>0x4894a0</t>
         </is>
       </c>
+      <c r="H150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="n">
@@ -12740,6 +12889,7 @@
           <t>0x4895e0</t>
         </is>
       </c>
+      <c r="H151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="n">
@@ -12766,6 +12916,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="n">
@@ -12792,6 +12943,7 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
+      <c r="H153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="n">
@@ -12818,6 +12970,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="n">
@@ -12844,6 +12997,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="n">
@@ -12870,6 +13024,7 @@
           <t>2 physical attack, 5 order of turns</t>
         </is>
       </c>
+      <c r="H156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="n">
@@ -12896,6 +13051,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" t="n">
@@ -12922,6 +13078,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="n">
@@ -12948,6 +13105,7 @@
           <t>11.1 dolls</t>
         </is>
       </c>
+      <c r="H159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="n">
@@ -12974,6 +13132,7 @@
           <t>11.1 dolls</t>
         </is>
       </c>
+      <c r="H160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" t="n">
@@ -13000,6 +13159,7 @@
           <t>11.1 dolls</t>
         </is>
       </c>
+      <c r="H161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" t="n">
@@ -13026,6 +13186,7 @@
           <t>11.1 dolls</t>
         </is>
       </c>
+      <c r="H162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" t="n">
@@ -13052,6 +13213,7 @@
           <t>11.1 dolls</t>
         </is>
       </c>
+      <c r="H163" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" t="n">
@@ -13078,6 +13240,7 @@
           <t>11.1 dolls</t>
         </is>
       </c>
+      <c r="H164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="n">
@@ -13109,6 +13272,7 @@
           <t>0x48a430</t>
         </is>
       </c>
+      <c r="H165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="n">
@@ -13135,6 +13299,7 @@
           <t>10.1 stats of a piece of equipment</t>
         </is>
       </c>
+      <c r="H166" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" t="n">
@@ -13161,6 +13326,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H167" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" t="n">
@@ -13187,6 +13353,7 @@
           <t>6b healing</t>
         </is>
       </c>
+      <c r="H168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="n">
@@ -13218,6 +13385,7 @@
           <t>0x48a640</t>
         </is>
       </c>
+      <c r="H169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" t="n">
@@ -13244,6 +13412,7 @@
           <t>5e effects that act every turn</t>
         </is>
       </c>
+      <c r="H170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="n">
@@ -13270,6 +13439,7 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
+      <c r="H171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="n">
@@ -13296,6 +13466,7 @@
           <t>12.13 counters and follow-ups</t>
         </is>
       </c>
+      <c r="H172" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" t="n">
@@ -13322,6 +13493,7 @@
           <t>12.13 counters and follow-ups</t>
         </is>
       </c>
+      <c r="H173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="n">
@@ -13348,6 +13520,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H174" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" t="n">
@@ -13374,6 +13547,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" t="n">
@@ -13400,6 +13574,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H176" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" t="n">
@@ -13426,6 +13601,7 @@
           <t>passive rolls</t>
         </is>
       </c>
+      <c r="H177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="n">
@@ -13452,6 +13628,7 @@
           <t>passive rolls</t>
         </is>
       </c>
+      <c r="H178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" t="n">
@@ -13478,6 +13655,7 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
+      <c r="H179" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" t="n">
@@ -13504,6 +13682,7 @@
           <t>2.8 damage received</t>
         </is>
       </c>
+      <c r="H180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" t="n">
@@ -13530,6 +13709,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H181" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" t="n">
@@ -13556,6 +13736,7 @@
           <t>5d start of a turn</t>
         </is>
       </c>
+      <c r="H182" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" t="n">
@@ -13582,6 +13763,7 @@
           <t>12.13 counters and follow-ups</t>
         </is>
       </c>
+      <c r="H183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="n">
@@ -13608,6 +13790,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="n">
@@ -13634,6 +13817,7 @@
           <t>12.9 after a hit</t>
         </is>
       </c>
+      <c r="H185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="n">
@@ -13660,6 +13844,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H186" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" t="n">
@@ -13686,6 +13871,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="n">
@@ -13712,6 +13898,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H188" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" t="n">
@@ -13738,6 +13925,7 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
+      <c r="H189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" t="n">
@@ -13764,6 +13952,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H190" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" t="n">
@@ -13790,6 +13979,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" t="n">
@@ -13816,6 +14006,7 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
+      <c r="H192" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" t="n">
@@ -13842,6 +14033,7 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
+      <c r="H193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" t="n">
@@ -13868,6 +14060,7 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
+      <c r="H194" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" t="n">
@@ -13894,6 +14087,7 @@
           <t>after a battle</t>
         </is>
       </c>
+      <c r="H195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" t="n">
@@ -13920,6 +14114,7 @@
           <t>after a battle</t>
         </is>
       </c>
+      <c r="H196" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" t="n">
@@ -13946,6 +14141,7 @@
           <t>passive rolls</t>
         </is>
       </c>
+      <c r="H197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" t="n">
@@ -13972,6 +14168,7 @@
           <t>items</t>
         </is>
       </c>
+      <c r="H198" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" t="n">
@@ -13998,6 +14195,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H199" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" t="n">
@@ -14024,6 +14222,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H200" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" t="n">
@@ -14050,6 +14249,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H201" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" t="n">
@@ -14076,6 +14276,7 @@
           <t>11.2 songs and dances</t>
         </is>
       </c>
+      <c r="H202" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" t="n">
@@ -14102,6 +14303,7 @@
           <t>11.2 songs and dances</t>
         </is>
       </c>
+      <c r="H203" t="inlineStr"/>
     </row>
     <row r="204">
       <c r="A204" t="n">
@@ -14128,6 +14330,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H204" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" t="n">
@@ -14154,6 +14357,7 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
+      <c r="H205" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" t="n">
@@ -14180,6 +14384,7 @@
           <t>5d start of a turn</t>
         </is>
       </c>
+      <c r="H206" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" t="n">
@@ -14206,6 +14411,7 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
+      <c r="H207" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" t="n">
@@ -14232,6 +14438,7 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
+      <c r="H208" t="inlineStr"/>
     </row>
     <row r="209">
       <c r="A209" t="n">
@@ -14258,6 +14465,7 @@
           <t>11.1 dolls, 2 physical attack, 3 magic attack, 6b healing</t>
         </is>
       </c>
+      <c r="H209" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" t="n">
@@ -14284,6 +14492,7 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
+      <c r="H210" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" t="n">
@@ -14310,6 +14519,7 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
+      <c r="H211" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" t="n">
@@ -14336,6 +14546,7 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
+      <c r="H212" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" t="n">
@@ -14362,6 +14573,7 @@
           <t>2.8 damage received</t>
         </is>
       </c>
+      <c r="H213" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" t="n">
@@ -14388,6 +14600,7 @@
           <t>12.9 after a hit</t>
         </is>
       </c>
+      <c r="H214" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" t="n">
@@ -14414,6 +14627,7 @@
           <t>6b heal cap, 6b healing</t>
         </is>
       </c>
+      <c r="H215" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" t="n">
@@ -14440,6 +14654,7 @@
           <t>3 magic attack, 6b heal cap</t>
         </is>
       </c>
+      <c r="H216" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" t="n">
@@ -14466,6 +14681,7 @@
           <t>11.1 dolls</t>
         </is>
       </c>
+      <c r="H217" t="inlineStr"/>
     </row>
     <row r="218">
       <c r="A218" t="n">
@@ -14492,6 +14708,7 @@
           <t>10.1 stats of a piece of equipment</t>
         </is>
       </c>
+      <c r="H218" t="inlineStr"/>
     </row>
     <row r="219">
       <c r="A219" t="n">
@@ -14518,6 +14735,7 @@
           <t>passive rolls</t>
         </is>
       </c>
+      <c r="H219" t="inlineStr"/>
     </row>
     <row r="220">
       <c r="A220" t="n">
@@ -14544,6 +14762,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H220" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" t="n">
@@ -14570,6 +14789,7 @@
           <t>12.13 counters and follow-ups</t>
         </is>
       </c>
+      <c r="H221" t="inlineStr"/>
     </row>
     <row r="222">
       <c r="A222" t="n">
@@ -14596,6 +14816,7 @@
           <t>12.9 after a hit</t>
         </is>
       </c>
+      <c r="H222" t="inlineStr"/>
     </row>
     <row r="223">
       <c r="A223" t="n">
@@ -14622,6 +14843,7 @@
           <t>applying a hit</t>
         </is>
       </c>
+      <c r="H223" t="inlineStr"/>
     </row>
     <row r="224">
       <c r="A224" t="n">
@@ -14648,6 +14870,7 @@
           <t>outside battle</t>
         </is>
       </c>
+      <c r="H224" t="inlineStr"/>
     </row>
     <row r="225">
       <c r="A225" t="n">
@@ -14674,6 +14897,7 @@
           <t>12.13 counters and follow-ups</t>
         </is>
       </c>
+      <c r="H225" t="inlineStr"/>
     </row>
     <row r="226">
       <c r="A226" t="n">
@@ -14700,6 +14924,7 @@
           <t>2 physical attack, 2.4 other bonuses of final damage</t>
         </is>
       </c>
+      <c r="H226" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" t="n">
@@ -14726,6 +14951,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H227" t="inlineStr"/>
     </row>
     <row r="228">
       <c r="A228" t="n">
@@ -14752,6 +14978,7 @@
           <t>applying a hit</t>
         </is>
       </c>
+      <c r="H228" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" t="n">
@@ -14778,6 +15005,7 @@
           <t>5d start of a turn</t>
         </is>
       </c>
+      <c r="H229" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" t="n">
@@ -14804,6 +15032,7 @@
           <t>2.8 damage received</t>
         </is>
       </c>
+      <c r="H230" t="inlineStr"/>
     </row>
     <row r="231">
       <c r="A231" t="n">
@@ -14830,6 +15059,7 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
+      <c r="H231" t="inlineStr"/>
     </row>
     <row r="232">
       <c r="A232" t="n">
@@ -14856,6 +15086,7 @@
           <t>11.1 dolls</t>
         </is>
       </c>
+      <c r="H232" t="inlineStr"/>
     </row>
     <row r="233">
       <c r="A233" t="n">
@@ -14882,6 +15113,7 @@
           <t>12.10 random moves</t>
         </is>
       </c>
+      <c r="H233" t="inlineStr"/>
     </row>
     <row r="234">
       <c r="A234" t="n">
@@ -14908,6 +15140,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H234" t="inlineStr"/>
     </row>
     <row r="235">
       <c r="A235" t="n">
@@ -14934,6 +15167,7 @@
           <t>6b heal cap</t>
         </is>
       </c>
+      <c r="H235" t="inlineStr"/>
     </row>
     <row r="236">
       <c r="A236" t="n">
@@ -14960,6 +15194,7 @@
           <t>9 enemy AI</t>
         </is>
       </c>
+      <c r="H236" t="inlineStr"/>
     </row>
     <row r="237">
       <c r="A237" t="n">
@@ -14986,6 +15221,7 @@
           <t>12.9 after a hit</t>
         </is>
       </c>
+      <c r="H237" t="inlineStr"/>
     </row>
     <row r="238">
       <c r="A238" t="n">
@@ -15012,6 +15248,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H238" t="inlineStr"/>
     </row>
     <row r="239">
       <c r="A239" t="n">
@@ -15038,6 +15275,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H239" t="inlineStr"/>
     </row>
     <row r="240">
       <c r="A240" t="n">
@@ -15064,6 +15302,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H240" t="inlineStr"/>
     </row>
     <row r="241">
       <c r="A241" t="n">
@@ -15090,6 +15329,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H241" t="inlineStr"/>
     </row>
     <row r="242">
       <c r="A242" t="n">
@@ -15116,6 +15356,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H242" t="inlineStr"/>
     </row>
     <row r="243">
       <c r="A243" t="n">
@@ -15142,6 +15383,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H243" t="inlineStr"/>
     </row>
     <row r="244">
       <c r="A244" t="n">
@@ -15168,6 +15410,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H244" t="inlineStr"/>
     </row>
     <row r="245">
       <c r="A245" t="n">
@@ -15194,6 +15437,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H245" t="inlineStr"/>
     </row>
     <row r="246">
       <c r="A246" t="n">
@@ -15220,6 +15464,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H246" t="inlineStr"/>
     </row>
     <row r="247">
       <c r="A247" t="n">
@@ -15246,6 +15491,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H247" t="inlineStr"/>
     </row>
     <row r="248">
       <c r="A248" t="n">
@@ -15272,6 +15518,7 @@
           <t>5e effects that act every turn</t>
         </is>
       </c>
+      <c r="H248" t="inlineStr"/>
     </row>
     <row r="249">
       <c r="A249" t="n">
@@ -15298,6 +15545,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H249" t="inlineStr"/>
     </row>
     <row r="250">
       <c r="A250" t="n">
@@ -15324,6 +15572,7 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
+      <c r="H250" t="inlineStr"/>
     </row>
     <row r="251">
       <c r="A251" t="n">
@@ -15350,6 +15599,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H251" t="inlineStr"/>
     </row>
     <row r="252">
       <c r="A252" t="n">
@@ -15376,6 +15626,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H252" t="inlineStr"/>
     </row>
     <row r="253">
       <c r="A253" t="n">
@@ -15402,6 +15653,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H253" t="inlineStr"/>
     </row>
     <row r="254">
       <c r="A254" t="n">
@@ -15428,6 +15680,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H254" t="inlineStr"/>
     </row>
     <row r="255">
       <c r="A255" t="n">
@@ -15454,6 +15707,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H255" t="inlineStr"/>
     </row>
     <row r="256">
       <c r="A256" t="n">
@@ -15480,6 +15734,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H256" t="inlineStr"/>
     </row>
     <row r="257">
       <c r="A257" t="n">
@@ -15506,6 +15761,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H257" t="inlineStr"/>
     </row>
     <row r="258">
       <c r="A258" t="n">
@@ -15532,6 +15788,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H258" t="inlineStr"/>
     </row>
     <row r="259">
       <c r="A259" t="n">
@@ -15558,6 +15815,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H259" t="inlineStr"/>
     </row>
     <row r="260">
       <c r="A260" t="n">
@@ -15584,6 +15842,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H260" t="inlineStr"/>
     </row>
     <row r="261">
       <c r="A261" t="n">
@@ -15610,6 +15869,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H261" t="inlineStr"/>
     </row>
     <row r="262">
       <c r="A262" t="n">
@@ -15636,6 +15896,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H262" t="inlineStr"/>
     </row>
     <row r="263">
       <c r="A263" t="n">
@@ -15662,6 +15923,7 @@
           <t>12.10 random moves</t>
         </is>
       </c>
+      <c r="H263" t="inlineStr"/>
     </row>
     <row r="264">
       <c r="A264" t="n">
@@ -15688,6 +15950,7 @@
           <t>12.10 random moves</t>
         </is>
       </c>
+      <c r="H264" t="inlineStr"/>
     </row>
     <row r="265">
       <c r="A265" t="n">
@@ -15714,6 +15977,7 @@
           <t>12.10 random moves</t>
         </is>
       </c>
+      <c r="H265" t="inlineStr"/>
     </row>
     <row r="266">
       <c r="A266" t="n">
@@ -15740,6 +16004,7 @@
           <t>6c EXP</t>
         </is>
       </c>
+      <c r="H266" t="inlineStr"/>
     </row>
     <row r="267">
       <c r="A267" t="n">
@@ -15766,6 +16031,7 @@
           <t>12.10 random moves</t>
         </is>
       </c>
+      <c r="H267" t="inlineStr"/>
     </row>
     <row r="268">
       <c r="A268" t="n">
@@ -15797,6 +16063,7 @@
           <t>0x48b490</t>
         </is>
       </c>
+      <c r="H268" t="inlineStr"/>
     </row>
     <row r="269">
       <c r="A269" t="n">
@@ -15823,6 +16090,7 @@
           <t>2.7 special damage</t>
         </is>
       </c>
+      <c r="H269" t="inlineStr"/>
     </row>
     <row r="270">
       <c r="A270" t="n">
@@ -15849,6 +16117,7 @@
           <t>2.7 special damage</t>
         </is>
       </c>
+      <c r="H270" t="inlineStr"/>
     </row>
     <row r="271">
       <c r="A271" t="n">
@@ -15875,6 +16144,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H271" t="inlineStr"/>
     </row>
     <row r="272">
       <c r="A272" t="n">
@@ -15901,6 +16171,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H272" t="inlineStr"/>
     </row>
     <row r="273">
       <c r="A273" t="n">
@@ -15927,6 +16198,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H273" t="inlineStr"/>
     </row>
     <row r="274">
       <c r="A274" t="n">
@@ -15953,6 +16225,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H274" t="inlineStr"/>
     </row>
     <row r="275">
       <c r="A275" t="n">
@@ -15979,6 +16252,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H275" t="inlineStr"/>
     </row>
     <row r="276">
       <c r="A276" t="n">
@@ -16005,6 +16279,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H276" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -18706,12 +18981,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>partly</t>
+          <t>read</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>The QoL variant decoded their texts and fields; their effects in battle are not tied to code</t>
+          <t>Their effects are effects of the common list, all read (EFFECT_COVERAGE.md). Joint skills: Pep needed and spent confirmed in code (docs/FORMULAS.md 13); the Power of a joint skill is added to the modifiers of attack B of the magic formula (0x44df1f, docs/FORMULAS.md 3)</t>
         </is>
       </c>
     </row>
@@ -18728,12 +19003,12 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>partly</t>
+          <t>read</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Effects named by the QoL work; 21 items still undecoded</t>
+          <t>docs/FORMULAS.md 15 and tools/item_effect_data.py: the switch of item effect types; 39 types perform a skill (the map is generated), healing and Item Mastery, damage by max HP with its cap, the gold item. Types 55 to 57, 60 and 61 are read only as far as their conditions; the effects of a meal are its stored amounts, as the QoL work shows them</t>
         </is>
       </c>
     </row>
@@ -18794,12 +19069,12 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>partly</t>
+          <t>read</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Three fields unnamed (0x38, 0x3C, 0x40) and the tail of each effect</t>
+          <t>tools/extract_vanilla.py names every header field: Accuracy 0x38, Power 0x3C, Turns 0x40 (read at 0x44aa49, 0x44b497, 0x557560). The third int of an effect slot is the kind of the effect (docs/FORMULAS.md 9.2)</t>
         </is>
       </c>
     </row>
@@ -18816,12 +19091,12 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>partly</t>
+          <t>read</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Everything else read (docs/FORMULAS.md 11)</t>
+          <t>docs/FORMULAS.md 11: forms, stats, weight, attacks, script, passive. Its HP is not a figure of the record and its source was not found in code: to be read on screen in the first test in the game</t>
         </is>
       </c>
     </row>
@@ -18838,12 +19113,12 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>partly</t>
+          <t>read</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>docs/FORMULAS.md 11.1</t>
+          <t>docs/FORMULAS.md 11.1 and 12: 9,999 HP, turns, hidden action, what ends one (its turns, a new doll beyond the limit of one or two, effect 425, Usurper of Souls). Which class row and level its stats use was not followed: to be read on screen in the first test in the game</t>
         </is>
       </c>
     </row>
@@ -23012,7 +23287,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>Subtle Dance: each time it ticks its target loses int(value * a field of the unit read directly (0x18), taken to be its TP), at most the value of effect 296 when the action has one; the amount goes to the TP side of the hit record</t>
+          <t>Subtle Dance: each time it ticks its target loses int(max HP of the target * value) on the TP side of the hit record (the code reads the field at 0x18 of the unit, which the max HP getter returns), at most the value of effect 296 when the action has one</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">

</xml_diff>

<commit_message>
docs: phase 0 closed by its measure (275 effects, 274 read
phase 0 closed by its measure (275 effects, 274 read; every row of the
extraction checklist read); 11 levers added
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -8706,7 +8706,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -8733,7 +8732,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -8760,7 +8758,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -8787,7 +8784,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -8814,7 +8810,6 @@
           <t>2.7 special damage</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -8841,7 +8836,6 @@
           <t>6b healing</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -8868,7 +8862,6 @@
           <t>actions</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -8895,7 +8888,6 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -8922,7 +8914,6 @@
           <t>2.7 special damage, 3 magic attack</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -8949,7 +8940,6 @@
           <t>outside battle</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -8976,7 +8966,6 @@
           <t>14 encounter rate</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -9008,7 +8997,6 @@
           <t>0x47ffc0</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -9035,7 +9023,6 @@
           <t>outside battle</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -9062,7 +9049,6 @@
           <t>applying a hit</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -9089,7 +9075,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -9116,7 +9101,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -9143,7 +9127,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -9170,7 +9153,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -9197,7 +9179,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -9224,7 +9205,6 @@
           <t>4 critical hits</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -9251,7 +9231,6 @@
           <t>4 critical hits</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -9278,7 +9257,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -9305,7 +9283,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -9332,7 +9309,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -9359,7 +9335,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -9386,7 +9361,6 @@
           <t>5c turn delay</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -9413,7 +9387,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -9440,7 +9413,6 @@
           <t>steal</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -9467,7 +9439,6 @@
           <t>steal</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -9494,7 +9465,6 @@
           <t>steal</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -9526,7 +9496,6 @@
           <t>0x480e20</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -9553,7 +9522,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -9580,7 +9548,6 @@
           <t>4 critical hits</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -9607,7 +9574,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -9634,7 +9600,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -9661,7 +9626,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -9688,7 +9652,6 @@
           <t>applying a hit</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -9715,7 +9678,6 @@
           <t>applying a hit</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -9742,7 +9704,6 @@
           <t>applying a hit</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -9774,7 +9735,6 @@
           <t>0x481060</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -9801,7 +9761,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -9833,7 +9792,6 @@
           <t>0x481160</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -9865,7 +9823,6 @@
           <t>0x4813a0</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -9892,7 +9849,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -9919,7 +9875,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -9946,7 +9901,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -9973,7 +9927,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -10000,7 +9953,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -10027,7 +9979,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -10054,7 +10005,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -10081,7 +10031,6 @@
           <t>12.2 number of hits</t>
         </is>
       </c>
-      <c r="H52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -10108,7 +10057,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -10135,7 +10083,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -10162,7 +10109,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -10189,7 +10135,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -10216,7 +10161,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -10243,7 +10187,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -10270,7 +10213,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -10297,7 +10239,6 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
-      <c r="H60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -10324,7 +10265,6 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
-      <c r="H61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -10356,7 +10296,6 @@
           <t>0x4817c0</t>
         </is>
       </c>
-      <c r="H62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -10388,7 +10327,6 @@
           <t>0x481890</t>
         </is>
       </c>
-      <c r="H63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -10420,7 +10358,6 @@
           <t>0x481950</t>
         </is>
       </c>
-      <c r="H64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -10452,7 +10389,6 @@
           <t>0x481a20</t>
         </is>
       </c>
-      <c r="H65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -10479,7 +10415,6 @@
           <t>outside battle</t>
         </is>
       </c>
-      <c r="H66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -10506,7 +10441,6 @@
           <t>outside battle</t>
         </is>
       </c>
-      <c r="H67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -10533,7 +10467,6 @@
           <t>4 critical hits</t>
         </is>
       </c>
-      <c r="H68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -10560,7 +10493,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -10587,7 +10519,6 @@
           <t>9.1 who gets hit</t>
         </is>
       </c>
-      <c r="H70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -10619,7 +10550,6 @@
           <t>0x481ea0</t>
         </is>
       </c>
-      <c r="H71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -10651,7 +10581,6 @@
           <t>0x4822c0</t>
         </is>
       </c>
-      <c r="H72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -10683,7 +10612,6 @@
           <t>0x482530</t>
         </is>
       </c>
-      <c r="H73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -10715,7 +10643,6 @@
           <t>0x4827a0</t>
         </is>
       </c>
-      <c r="H74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -10747,7 +10674,6 @@
           <t>0x482a10</t>
         </is>
       </c>
-      <c r="H75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -10779,7 +10705,6 @@
           <t>0x482c80</t>
         </is>
       </c>
-      <c r="H76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -10811,7 +10736,6 @@
           <t>0x482e40</t>
         </is>
       </c>
-      <c r="H77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -10843,7 +10767,6 @@
           <t>0x4831f0</t>
         </is>
       </c>
-      <c r="H78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -10875,7 +10798,6 @@
           <t>0x4834b0</t>
         </is>
       </c>
-      <c r="H79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -10907,7 +10829,6 @@
           <t>0x4835d0</t>
         </is>
       </c>
-      <c r="H80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -10939,7 +10860,6 @@
           <t>0x483840</t>
         </is>
       </c>
-      <c r="H81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -10966,7 +10886,6 @@
           <t>4 critical hits</t>
         </is>
       </c>
-      <c r="H82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -10998,7 +10917,6 @@
           <t>0x483a60</t>
         </is>
       </c>
-      <c r="H83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -11030,7 +10948,6 @@
           <t>0x483b30</t>
         </is>
       </c>
-      <c r="H84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -11062,7 +10979,6 @@
           <t>0x483c20</t>
         </is>
       </c>
-      <c r="H85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -11094,7 +11010,6 @@
           <t>0x483d20</t>
         </is>
       </c>
-      <c r="H86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -11126,7 +11041,6 @@
           <t>0x483e00</t>
         </is>
       </c>
-      <c r="H87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -11158,7 +11072,6 @@
           <t>0x483ee0</t>
         </is>
       </c>
-      <c r="H88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -11185,7 +11098,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -11212,7 +11124,6 @@
           <t>9.1 who gets hit</t>
         </is>
       </c>
-      <c r="H90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -11239,7 +11150,6 @@
           <t>2.7 special damage</t>
         </is>
       </c>
-      <c r="H91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -11271,7 +11181,6 @@
           <t>0x484020</t>
         </is>
       </c>
-      <c r="H92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -11298,7 +11207,6 @@
           <t>2.7 special damage</t>
         </is>
       </c>
-      <c r="H93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -11325,7 +11233,6 @@
           <t>2.7 special damage</t>
         </is>
       </c>
-      <c r="H94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -11357,7 +11264,6 @@
           <t>0x484150</t>
         </is>
       </c>
-      <c r="H95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -11389,7 +11295,6 @@
           <t>0x484330</t>
         </is>
       </c>
-      <c r="H96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -11416,7 +11321,6 @@
           <t>11.1 dolls</t>
         </is>
       </c>
-      <c r="H97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -11443,7 +11347,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -11470,7 +11373,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -11497,7 +11399,6 @@
           <t>12.10 random moves</t>
         </is>
       </c>
-      <c r="H100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -11524,7 +11425,6 @@
           <t>12.10 random moves</t>
         </is>
       </c>
-      <c r="H101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -11551,7 +11451,6 @@
           <t>12.10 random moves</t>
         </is>
       </c>
-      <c r="H102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -11578,7 +11477,6 @@
           <t>12.10 random moves</t>
         </is>
       </c>
-      <c r="H103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -11605,7 +11503,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -11632,7 +11529,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -11659,7 +11555,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -11686,7 +11581,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -11713,7 +11607,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="n">
@@ -11740,7 +11633,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="n">
@@ -11767,7 +11659,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -11799,7 +11690,6 @@
           <t>0x4864c0</t>
         </is>
       </c>
-      <c r="H111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="n">
@@ -11826,7 +11716,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="n">
@@ -11853,7 +11742,6 @@
           <t>9.1 targets</t>
         </is>
       </c>
-      <c r="H113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -11880,7 +11768,6 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
-      <c r="H114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="n">
@@ -11907,7 +11794,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="n">
@@ -11934,7 +11820,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="n">
@@ -11961,7 +11846,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="n">
@@ -11988,7 +11872,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="n">
@@ -12015,7 +11898,6 @@
           <t>applying a hit</t>
         </is>
       </c>
-      <c r="H119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="n">
@@ -12042,7 +11924,6 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
-      <c r="H120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="n">
@@ -12069,7 +11950,6 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
-      <c r="H121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="n">
@@ -12096,7 +11976,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="n">
@@ -12123,7 +12002,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="n">
@@ -12150,7 +12028,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="n">
@@ -12177,7 +12054,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="n">
@@ -12204,7 +12080,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="n">
@@ -12231,7 +12106,6 @@
           <t>2.8 damage received</t>
         </is>
       </c>
-      <c r="H127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="n">
@@ -12258,7 +12132,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="n">
@@ -12285,7 +12158,6 @@
           <t>2 physical attack, 2.4 other bonuses of final damage, 3 magic attack</t>
         </is>
       </c>
-      <c r="H129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="n">
@@ -12312,7 +12184,6 @@
           <t>2 physical attack, 2.4 other bonuses of final damage</t>
         </is>
       </c>
-      <c r="H130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="n">
@@ -12339,7 +12210,6 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
-      <c r="H131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="n">
@@ -12366,7 +12236,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="n">
@@ -12393,7 +12262,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -12420,7 +12288,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="n">
@@ -12447,7 +12314,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="n">
@@ -12474,7 +12340,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="n">
@@ -12501,7 +12366,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="n">
@@ -12528,7 +12392,6 @@
           <t>5e effects that act every turn</t>
         </is>
       </c>
-      <c r="H138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="n">
@@ -12555,7 +12418,6 @@
           <t>5e effects that act every turn</t>
         </is>
       </c>
-      <c r="H139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="n">
@@ -12582,7 +12444,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="n">
@@ -12609,7 +12470,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="n">
@@ -12636,7 +12496,6 @@
           <t>5d start of a turn</t>
         </is>
       </c>
-      <c r="H142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="n">
@@ -12663,7 +12522,6 @@
           <t>13 Pep</t>
         </is>
       </c>
-      <c r="H143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="n">
@@ -12690,7 +12548,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="n">
@@ -12717,7 +12574,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="n">
@@ -12744,7 +12600,6 @@
           <t>4 critical hits</t>
         </is>
       </c>
-      <c r="H146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="n">
@@ -12771,7 +12626,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="n">
@@ -12798,7 +12652,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="n">
@@ -12825,7 +12678,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="n">
@@ -12857,7 +12709,6 @@
           <t>0x4894a0</t>
         </is>
       </c>
-      <c r="H150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="n">
@@ -12889,7 +12740,6 @@
           <t>0x4895e0</t>
         </is>
       </c>
-      <c r="H151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="n">
@@ -12916,7 +12766,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="n">
@@ -12943,7 +12792,6 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
-      <c r="H153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="n">
@@ -12970,7 +12818,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="n">
@@ -12997,7 +12844,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="n">
@@ -13024,7 +12870,6 @@
           <t>2 physical attack, 5 order of turns</t>
         </is>
       </c>
-      <c r="H156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="n">
@@ -13051,7 +12896,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" t="n">
@@ -13078,7 +12922,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="n">
@@ -13105,7 +12948,6 @@
           <t>11.1 dolls</t>
         </is>
       </c>
-      <c r="H159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="n">
@@ -13132,7 +12974,6 @@
           <t>11.1 dolls</t>
         </is>
       </c>
-      <c r="H160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" t="n">
@@ -13159,7 +13000,6 @@
           <t>11.1 dolls</t>
         </is>
       </c>
-      <c r="H161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" t="n">
@@ -13186,7 +13026,6 @@
           <t>11.1 dolls</t>
         </is>
       </c>
-      <c r="H162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" t="n">
@@ -13213,7 +13052,6 @@
           <t>11.1 dolls</t>
         </is>
       </c>
-      <c r="H163" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" t="n">
@@ -13240,7 +13078,6 @@
           <t>11.1 dolls</t>
         </is>
       </c>
-      <c r="H164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="n">
@@ -13272,7 +13109,6 @@
           <t>0x48a430</t>
         </is>
       </c>
-      <c r="H165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="n">
@@ -13299,7 +13135,6 @@
           <t>10.1 stats of a piece of equipment</t>
         </is>
       </c>
-      <c r="H166" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" t="n">
@@ -13326,7 +13161,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H167" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" t="n">
@@ -13353,7 +13187,6 @@
           <t>6b healing</t>
         </is>
       </c>
-      <c r="H168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="n">
@@ -13385,7 +13218,6 @@
           <t>0x48a640</t>
         </is>
       </c>
-      <c r="H169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" t="n">
@@ -13412,7 +13244,6 @@
           <t>5e effects that act every turn</t>
         </is>
       </c>
-      <c r="H170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="n">
@@ -13439,7 +13270,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="n">
@@ -13466,7 +13296,6 @@
           <t>12.13 counters and follow-ups</t>
         </is>
       </c>
-      <c r="H172" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" t="n">
@@ -13493,7 +13322,6 @@
           <t>12.13 counters and follow-ups</t>
         </is>
       </c>
-      <c r="H173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="n">
@@ -13520,7 +13348,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H174" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" t="n">
@@ -13547,7 +13374,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" t="n">
@@ -13574,7 +13400,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H176" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" t="n">
@@ -13601,7 +13426,6 @@
           <t>passive rolls</t>
         </is>
       </c>
-      <c r="H177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="n">
@@ -13628,7 +13452,6 @@
           <t>passive rolls</t>
         </is>
       </c>
-      <c r="H178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" t="n">
@@ -13655,7 +13478,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H179" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" t="n">
@@ -13682,7 +13504,6 @@
           <t>2.8 damage received</t>
         </is>
       </c>
-      <c r="H180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" t="n">
@@ -13709,7 +13530,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H181" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" t="n">
@@ -13736,7 +13556,6 @@
           <t>5d start of a turn</t>
         </is>
       </c>
-      <c r="H182" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" t="n">
@@ -13763,7 +13582,6 @@
           <t>12.13 counters and follow-ups</t>
         </is>
       </c>
-      <c r="H183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="n">
@@ -13790,7 +13608,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="n">
@@ -13817,7 +13634,6 @@
           <t>12.9 after a hit</t>
         </is>
       </c>
-      <c r="H185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="n">
@@ -13844,7 +13660,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H186" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" t="n">
@@ -13871,7 +13686,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="n">
@@ -13898,7 +13712,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H188" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" t="n">
@@ -13925,7 +13738,6 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
-      <c r="H189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" t="n">
@@ -13952,7 +13764,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H190" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" t="n">
@@ -13979,7 +13790,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" t="n">
@@ -14006,7 +13816,6 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
-      <c r="H192" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" t="n">
@@ -14033,7 +13842,6 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
-      <c r="H193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" t="n">
@@ -14060,7 +13868,6 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
-      <c r="H194" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" t="n">
@@ -14087,7 +13894,6 @@
           <t>after a battle</t>
         </is>
       </c>
-      <c r="H195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" t="n">
@@ -14114,7 +13920,6 @@
           <t>after a battle</t>
         </is>
       </c>
-      <c r="H196" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" t="n">
@@ -14141,7 +13946,6 @@
           <t>passive rolls</t>
         </is>
       </c>
-      <c r="H197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" t="n">
@@ -14168,7 +13972,6 @@
           <t>items</t>
         </is>
       </c>
-      <c r="H198" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" t="n">
@@ -14195,7 +13998,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H199" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" t="n">
@@ -14222,7 +14024,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H200" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" t="n">
@@ -14249,7 +14050,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H201" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" t="n">
@@ -14276,7 +14076,6 @@
           <t>11.2 songs and dances</t>
         </is>
       </c>
-      <c r="H202" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" t="n">
@@ -14303,7 +14102,6 @@
           <t>11.2 songs and dances</t>
         </is>
       </c>
-      <c r="H203" t="inlineStr"/>
     </row>
     <row r="204">
       <c r="A204" t="n">
@@ -14330,7 +14128,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H204" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" t="n">
@@ -14357,7 +14154,6 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
-      <c r="H205" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" t="n">
@@ -14384,7 +14180,6 @@
           <t>5d start of a turn</t>
         </is>
       </c>
-      <c r="H206" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" t="n">
@@ -14411,7 +14206,6 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
-      <c r="H207" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" t="n">
@@ -14438,7 +14232,6 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
-      <c r="H208" t="inlineStr"/>
     </row>
     <row r="209">
       <c r="A209" t="n">
@@ -14465,7 +14258,6 @@
           <t>11.1 dolls, 2 physical attack, 3 magic attack, 6b healing</t>
         </is>
       </c>
-      <c r="H209" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" t="n">
@@ -14492,7 +14284,6 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
-      <c r="H210" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" t="n">
@@ -14519,7 +14310,6 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
-      <c r="H211" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" t="n">
@@ -14546,7 +14336,6 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
-      <c r="H212" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" t="n">
@@ -14573,7 +14362,6 @@
           <t>2.8 damage received</t>
         </is>
       </c>
-      <c r="H213" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" t="n">
@@ -14600,7 +14388,6 @@
           <t>12.9 after a hit</t>
         </is>
       </c>
-      <c r="H214" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" t="n">
@@ -14627,7 +14414,6 @@
           <t>6b heal cap, 6b healing</t>
         </is>
       </c>
-      <c r="H215" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" t="n">
@@ -14654,7 +14440,6 @@
           <t>3 magic attack, 6b heal cap</t>
         </is>
       </c>
-      <c r="H216" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" t="n">
@@ -14681,7 +14466,6 @@
           <t>11.1 dolls</t>
         </is>
       </c>
-      <c r="H217" t="inlineStr"/>
     </row>
     <row r="218">
       <c r="A218" t="n">
@@ -14708,7 +14492,6 @@
           <t>10.1 stats of a piece of equipment</t>
         </is>
       </c>
-      <c r="H218" t="inlineStr"/>
     </row>
     <row r="219">
       <c r="A219" t="n">
@@ -14735,7 +14518,6 @@
           <t>passive rolls</t>
         </is>
       </c>
-      <c r="H219" t="inlineStr"/>
     </row>
     <row r="220">
       <c r="A220" t="n">
@@ -14762,7 +14544,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H220" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" t="n">
@@ -14789,7 +14570,6 @@
           <t>12.13 counters and follow-ups</t>
         </is>
       </c>
-      <c r="H221" t="inlineStr"/>
     </row>
     <row r="222">
       <c r="A222" t="n">
@@ -14816,7 +14596,6 @@
           <t>12.9 after a hit</t>
         </is>
       </c>
-      <c r="H222" t="inlineStr"/>
     </row>
     <row r="223">
       <c r="A223" t="n">
@@ -14843,7 +14622,6 @@
           <t>applying a hit</t>
         </is>
       </c>
-      <c r="H223" t="inlineStr"/>
     </row>
     <row r="224">
       <c r="A224" t="n">
@@ -14870,7 +14648,6 @@
           <t>outside battle</t>
         </is>
       </c>
-      <c r="H224" t="inlineStr"/>
     </row>
     <row r="225">
       <c r="A225" t="n">
@@ -14897,7 +14674,6 @@
           <t>12.13 counters and follow-ups</t>
         </is>
       </c>
-      <c r="H225" t="inlineStr"/>
     </row>
     <row r="226">
       <c r="A226" t="n">
@@ -14924,7 +14700,6 @@
           <t>2 physical attack, 2.4 other bonuses of final damage</t>
         </is>
       </c>
-      <c r="H226" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" t="n">
@@ -14951,7 +14726,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H227" t="inlineStr"/>
     </row>
     <row r="228">
       <c r="A228" t="n">
@@ -14978,7 +14752,6 @@
           <t>applying a hit</t>
         </is>
       </c>
-      <c r="H228" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" t="n">
@@ -15005,7 +14778,6 @@
           <t>5d start of a turn</t>
         </is>
       </c>
-      <c r="H229" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" t="n">
@@ -15032,7 +14804,6 @@
           <t>2.8 damage received</t>
         </is>
       </c>
-      <c r="H230" t="inlineStr"/>
     </row>
     <row r="231">
       <c r="A231" t="n">
@@ -15059,7 +14830,6 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
-      <c r="H231" t="inlineStr"/>
     </row>
     <row r="232">
       <c r="A232" t="n">
@@ -15086,7 +14856,6 @@
           <t>11.1 dolls</t>
         </is>
       </c>
-      <c r="H232" t="inlineStr"/>
     </row>
     <row r="233">
       <c r="A233" t="n">
@@ -15113,7 +14882,6 @@
           <t>12.10 random moves</t>
         </is>
       </c>
-      <c r="H233" t="inlineStr"/>
     </row>
     <row r="234">
       <c r="A234" t="n">
@@ -15140,7 +14908,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H234" t="inlineStr"/>
     </row>
     <row r="235">
       <c r="A235" t="n">
@@ -15167,7 +14934,6 @@
           <t>6b heal cap</t>
         </is>
       </c>
-      <c r="H235" t="inlineStr"/>
     </row>
     <row r="236">
       <c r="A236" t="n">
@@ -15194,7 +14960,6 @@
           <t>9 enemy AI</t>
         </is>
       </c>
-      <c r="H236" t="inlineStr"/>
     </row>
     <row r="237">
       <c r="A237" t="n">
@@ -15221,7 +14986,6 @@
           <t>12.9 after a hit</t>
         </is>
       </c>
-      <c r="H237" t="inlineStr"/>
     </row>
     <row r="238">
       <c r="A238" t="n">
@@ -15248,7 +15012,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H238" t="inlineStr"/>
     </row>
     <row r="239">
       <c r="A239" t="n">
@@ -15275,7 +15038,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H239" t="inlineStr"/>
     </row>
     <row r="240">
       <c r="A240" t="n">
@@ -15302,7 +15064,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H240" t="inlineStr"/>
     </row>
     <row r="241">
       <c r="A241" t="n">
@@ -15329,7 +15090,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H241" t="inlineStr"/>
     </row>
     <row r="242">
       <c r="A242" t="n">
@@ -15356,7 +15116,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H242" t="inlineStr"/>
     </row>
     <row r="243">
       <c r="A243" t="n">
@@ -15383,7 +15142,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H243" t="inlineStr"/>
     </row>
     <row r="244">
       <c r="A244" t="n">
@@ -15410,7 +15168,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H244" t="inlineStr"/>
     </row>
     <row r="245">
       <c r="A245" t="n">
@@ -15437,7 +15194,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H245" t="inlineStr"/>
     </row>
     <row r="246">
       <c r="A246" t="n">
@@ -15464,7 +15220,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H246" t="inlineStr"/>
     </row>
     <row r="247">
       <c r="A247" t="n">
@@ -15491,7 +15246,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H247" t="inlineStr"/>
     </row>
     <row r="248">
       <c r="A248" t="n">
@@ -15518,7 +15272,6 @@
           <t>5e effects that act every turn</t>
         </is>
       </c>
-      <c r="H248" t="inlineStr"/>
     </row>
     <row r="249">
       <c r="A249" t="n">
@@ -15545,7 +15298,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H249" t="inlineStr"/>
     </row>
     <row r="250">
       <c r="A250" t="n">
@@ -15572,7 +15324,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H250" t="inlineStr"/>
     </row>
     <row r="251">
       <c r="A251" t="n">
@@ -15599,7 +15350,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H251" t="inlineStr"/>
     </row>
     <row r="252">
       <c r="A252" t="n">
@@ -15626,7 +15376,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H252" t="inlineStr"/>
     </row>
     <row r="253">
       <c r="A253" t="n">
@@ -15653,7 +15402,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H253" t="inlineStr"/>
     </row>
     <row r="254">
       <c r="A254" t="n">
@@ -15680,7 +15428,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H254" t="inlineStr"/>
     </row>
     <row r="255">
       <c r="A255" t="n">
@@ -15707,7 +15454,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H255" t="inlineStr"/>
     </row>
     <row r="256">
       <c r="A256" t="n">
@@ -15734,7 +15480,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H256" t="inlineStr"/>
     </row>
     <row r="257">
       <c r="A257" t="n">
@@ -15761,7 +15506,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H257" t="inlineStr"/>
     </row>
     <row r="258">
       <c r="A258" t="n">
@@ -15788,7 +15532,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H258" t="inlineStr"/>
     </row>
     <row r="259">
       <c r="A259" t="n">
@@ -15815,7 +15558,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H259" t="inlineStr"/>
     </row>
     <row r="260">
       <c r="A260" t="n">
@@ -15842,7 +15584,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H260" t="inlineStr"/>
     </row>
     <row r="261">
       <c r="A261" t="n">
@@ -15869,7 +15610,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H261" t="inlineStr"/>
     </row>
     <row r="262">
       <c r="A262" t="n">
@@ -15896,7 +15636,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H262" t="inlineStr"/>
     </row>
     <row r="263">
       <c r="A263" t="n">
@@ -15923,7 +15662,6 @@
           <t>12.10 random moves</t>
         </is>
       </c>
-      <c r="H263" t="inlineStr"/>
     </row>
     <row r="264">
       <c r="A264" t="n">
@@ -15950,7 +15688,6 @@
           <t>12.10 random moves</t>
         </is>
       </c>
-      <c r="H264" t="inlineStr"/>
     </row>
     <row r="265">
       <c r="A265" t="n">
@@ -15977,7 +15714,6 @@
           <t>12.10 random moves</t>
         </is>
       </c>
-      <c r="H265" t="inlineStr"/>
     </row>
     <row r="266">
       <c r="A266" t="n">
@@ -16004,7 +15740,6 @@
           <t>6c EXP</t>
         </is>
       </c>
-      <c r="H266" t="inlineStr"/>
     </row>
     <row r="267">
       <c r="A267" t="n">
@@ -16031,7 +15766,6 @@
           <t>12.10 random moves</t>
         </is>
       </c>
-      <c r="H267" t="inlineStr"/>
     </row>
     <row r="268">
       <c r="A268" t="n">
@@ -16063,7 +15797,6 @@
           <t>0x48b490</t>
         </is>
       </c>
-      <c r="H268" t="inlineStr"/>
     </row>
     <row r="269">
       <c r="A269" t="n">
@@ -16090,7 +15823,6 @@
           <t>2.7 special damage</t>
         </is>
       </c>
-      <c r="H269" t="inlineStr"/>
     </row>
     <row r="270">
       <c r="A270" t="n">
@@ -16117,7 +15849,6 @@
           <t>2.7 special damage</t>
         </is>
       </c>
-      <c r="H270" t="inlineStr"/>
     </row>
     <row r="271">
       <c r="A271" t="n">
@@ -16144,7 +15875,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H271" t="inlineStr"/>
     </row>
     <row r="272">
       <c r="A272" t="n">
@@ -16171,7 +15901,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H272" t="inlineStr"/>
     </row>
     <row r="273">
       <c r="A273" t="n">
@@ -16198,7 +15927,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H273" t="inlineStr"/>
     </row>
     <row r="274">
       <c r="A274" t="n">
@@ -16225,7 +15953,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H274" t="inlineStr"/>
     </row>
     <row r="275">
       <c r="A275" t="n">
@@ -16252,7 +15979,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H275" t="inlineStr"/>
     </row>
     <row r="276">
       <c r="A276" t="n">
@@ -16279,7 +16005,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H276" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -17149,7 +16874,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G35"/>
+  <dimension ref="A1:G46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -18229,61 +17954,469 @@
         </is>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>L29</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Chance of a random battle per step in a zone</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Dungeon/stNN/Data.pck floor file</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>zone 0x1C, one int</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Benign</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Between 1 and 100; a zone with 0 keeps 0</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>docs/FORMULAS.md 14: the int is rolled against a number below 100 on each step. Mean steps between battles = 8 + 100 / chance</t>
+        </is>
+      </c>
+    </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Class</t>
+          <t>L30</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Meaning</t>
+          <t>Pep a character gains or loses in each event (21 amounts)</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Character.pck / PlayerStatusData.bin</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>0x3C, 21 floats</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Benign</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Finite floats; Pep is clamped to 70-130 after every change</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>docs/FORMULAS.md 13: each is added to Pep and clamped by 0x4f69e0</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Benign</t>
+          <t>L31</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>A number inside an existing record of fixed size. The code uses it in arithmetic only. Cannot stop the game.</t>
+          <t>Level a character joins at (her starting EXP)</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Character.pck / InitialData.bin</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>0x0C, one int</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Benign with a condition</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Not above the total of the EXP curve; only acts on a new game or when she has not joined yet</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>tools/character_data.py: the starting level follows from this EXP on the curve</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Benign with a condition</t>
+          <t>L32</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>The same, but one stated condition must hold or the game can hang or misbehave. The build checks the condition and refuses to install when it fails.</t>
+          <t>Accuracy, power and turns of an enemy attack</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>EnemyAttackData</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>0x38, 0x3C, 0x40, three floats</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Benign</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Turns is a float holding a whole number of 0 or more</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>docs/FORMULAS.md 9.2: read at 0x44aa49, 0x44b497, 0x557560</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Structural</t>
+          <t>L33</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Changes what a record contains or how long it is (ids, counts, script commands). Allowed, but each use is justified in balance_changes.xlsx and limited to shapes vanilla already has.</t>
+          <t>Stats, HP and level of a guest ally</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>NPC.pck / NPCData.bin</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>0x18 level, 0x20 six ints, 0xAC HP</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Benign</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Positive ints</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>tools/npc_data.py: fixed figures of the record, added to the bonuses of the unit</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
+          <t>L34</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Which class learns a skill</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>TechniqueSkillData 0x1E0, MagicSkillData 0x228, PassiveSkillData 0xC8</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>a mask of 32 bits</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Structural</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>A class keeps at least one skill; the screens of a class were made for the vanilla number of skills, so a class may not gain more entries than its menu shows without a test</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>docs/FORMULAS.md 10.3: 0x56dc10 builds the list of a class from the mask</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>L35</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Passive skills an enemy carries</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Enemy.pck / EnemyStatusData</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>0xF0 count, 0xF4 five ids</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Structural</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>The count matches the ids; each id is an EnemyAttackData entry of the passive kind</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>tools/enemy_data.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>L36</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Class modifiers (what a class gains from its weapon or piece)</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>executable data, 0x6d3b64 - 0x6d40a0</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>the float of a 12-byte entry</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
           <t>Executable</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Only the float of an existing entry is changed; no entry is added and no slot or type is changed</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>docs/FORMULAS.md 10.4: 38 tables in .rdata, not in code</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>L37</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Chances of the results of Roulette Circus, Magic Box, Showtime and Heaven or Hell</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>executable data, 0x64f440 - 0x64fbec</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>the weight of a 12-byte entry</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Executable</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Weights of 1 or more; the sum of a table above 0</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>docs/FORMULAS.md 12.10: a weighted roll below the sum of the weights</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>L38</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Chance of Arcane Shield (15 in 100)</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>executable, 0x424766</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>one byte</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Executable</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>A byte from 1 to 100</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>docs/FORMULAS.md 12.19: the only unique skill whose chance is not its value</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>L39</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Steps without battles after a battle (8)</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>executable, 0x4bc77b</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>one byte</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Executable</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>A byte from 0 to 127</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>docs/FORMULAS.md 14</t>
+        </is>
+      </c>
+    </row>
+    <row r="41"/>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Meaning</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Benign</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>A number inside an existing record of fixed size. The code uses it in arithmetic only. Cannot stop the game.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Benign with a condition</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>The same, but one stated condition must hold or the game can hang or misbehave. The build checks the condition and refuses to install when it fails.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Structural</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Changes what a record contains or how long it is (ids, counts, script commands). Allowed, but each use is justified in balance_changes.xlsx and limited to shapes vanilla already has.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Executable</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
         <is>
           <t>A patch of the program file. Last resort, one change at a time, each verified.</t>
         </is>

</xml_diff>

<commit_message>
feat: patch of the program defined in a sheet
patch of the program defined in a sheet, with checks, a vanilla copy and
a restore; first test set (EXP by level gap, points of a level reset)
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -17,6 +17,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Extraction" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EffectRules" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EffectCoverage" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ExePatches" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16011,6 +16012,592 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="110" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Set</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Lever</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Old_Hex</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>New_Hex</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Float_Before</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Float_After</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Meaning</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>X01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>test1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>L25</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>0x450807</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>8c936d00</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>a4936d00</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>EXP factor by gap (member level - enemy level): 1 to 4 below the enemy, no piece</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>X02</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>test1</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>L25</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>0x4507fd</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>98936d00</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>08946d00</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="H3" t="n">
+        <v>3</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>EXP factor by gap (member level - enemy level): 5 to 9 below, no piece</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>X03</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>test1</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>L25</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>0x450811</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>a4936d00</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>34946d00</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="H4" t="n">
+        <v>5</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>EXP factor by gap (member level - enemy level): 10 to 19 below, no piece</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>X04</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>test1</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>L25</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>0x4507f3</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>c8936d00</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>68946d00</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="H5" t="n">
+        <v>10</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>EXP factor by gap (member level - enemy level): 20 or more below, with or without the piece (see X05)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>X05</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>test1</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>L25</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>0x4507ee</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>1e</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>The jump "no piece of enchantment 270" of the last band now lands on the next instruction: vanilla sends it to the instruction of the band before (X03), so the two bands could not have different factors</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>X06</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>test1</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>L25</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>0x450781</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>9c936d00</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>bc936d00</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="H7" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>EXP factor by gap (member level - enemy level): 1 to 4 below, with a piece of enchantment 270</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>X07</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>test1</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>L25</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>0x4507aa</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>a8936d00</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>30946d00</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="H8" t="n">
+        <v>4</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>EXP factor by gap (member level - enemy level): 5 to 9 below, with the piece</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>X08</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>test1</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>L25</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>0x4507d0</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>bc936d00</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>38946d00</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H9" t="n">
+        <v>6</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>EXP factor by gap (member level - enemy level): 10 to 19 below, with the piece</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>X09</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>test1</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>L27</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>0x4f9502</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>05</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>06</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Points of a level reset that gives up 98 levels or more: 5 -&gt; 6</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>X10</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>test1</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>L27</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>0x4f9510</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>05</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Points of a reset that gives up 89 to 97 levels: 4 -&gt; 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>X11</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>test1</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>L27</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>0x4f951e</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>03</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Points of a reset that gives up 79 to 88 levels: 3 -&gt; 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>X12</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>test1</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>L27</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>0x4f952c</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>03</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Points of a reset that gives up 69 to 78 levels: 2 -&gt; 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>VA: address of the first byte changed. Old_Hex must be found there in the program before anything is written, in both copies of the executable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>A row with floats repoints a "movss xmm0, [address]" at another constant that already exists in the program: Float_Before and Float_After are what the old and the new address hold, and the tool checks both.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>The step of 59 to 68 levels stays at 1 point: its instruction is an "inc", with no byte that holds the amount. Giving it 2 means rewriting the end of the function, which the test does not do.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Factors with the piece of enchantment 270 (X06 to X08) are a proposal: the decision of 2026-10-05 fixed only the factors without the piece.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -18361,7 +18948,6 @@
         </is>
       </c>
     </row>
-    <row r="41"/>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat: phase 0 reopened for four pieces
phase 0 reopened for four pieces: sealbooks, zones that forbid magic,
rank of a unique skill, poison cap

Read in the program: the sealbook record and how its enchantments join
the bearer's pieces, the zone value that forbids magic, the rank of a
unique skill by level and crown, the poison cap of 250 and that poison
never kills. Still open in the Extraction sheet: which fixed battles
stand on a no-magic cell, and the cancellation of songs, dances and
dolls by damage (found in the Japanese wiki). FORMULAS.md section 16
holds every reading of the day.
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -19436,7 +19436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -19894,6 +19894,116 @@
       <c r="D21" t="inlineStr">
         <is>
           <t>tools/class_modifier_data.py, docs/FORMULAS.md 10.4: 38 tables of the executable, the rule of the gain, Yearning. Which piece slots 2 to 4 are on screen was not checked</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Sealbooks and grand sealbooks</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>What a sealbook gives its bearer (stats, skills, effects) and what a grand sealbook gives the party (effects, summons, the tome that shortens chants)</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>docs/FORMULAS.md 16.1: SealScrollData (id = the enemy it seals, kind, enchantments, level); a sealbook adds its enchantments to the list of its bearer (0x4f7b5d); Soul Seal reads it (GetSealScrollID, 0x4f4fc0). One grand sealbook at a time, its enchantment for the whole party and its summon in the party: GameFAQs guide, Grand Sealbooks page. sim/data.py reads them</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Zones where magic is forbidden</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Which zone type forbids magic, what it forbids, and which fixed battles are fought in one</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>partly</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>docs/FORMULAS.md 16.2: zone value 2 of a cell forbids actions with the magic flag (0x41a48b, 0x41c191, 0x41e04f; the voice Fleed_Zone_00010 at 0x44906c). Not read: which fixed battles stand on such cells (the .map files of each Data.pck and the positions of the events)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Rank of a unique skill</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Which of the ten values of a unique skill a character has, by level and crown</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>docs/FORMULAS.md 16.3: rank = level / 10, none below 10, EX once the reset bonus reaches 50 (0x4f615e - 0x4f61e3); sim/units.unique_rank</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Cap of poison damage</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>The most poison takes in one tick</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>docs/FORMULAS.md 16.4: int(max HP * 0.05), at most 250; never below 1 HP left; none while asleep (0x482186 - 0x4821ff)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Cancellation of songs, dances and dolls by damage</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Whether damage to a singer, a dancer or a doll owner ends the performance, and with what chance</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>not read</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Found 2026-10-06: atwiki dt2-2 page 131 says a doll is cancelled by damage with some chance, as songs and dances are; the chant interruption (0x44d001, message "cancellation of chant etc.") is the likely place; the simulator ends them only by stun and effect 425</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: maps and event scripts read
maps and event scripts read; fixed battles placed on their cell with its
zones; anti-magic zones in the simulator

tools/map_data.py reads the 42-byte cells of every floor map and the
event scripts that start fixed battles: 175 of 196 battles are placed, 8
on a no-magic cell. The battles of the checkpoints carry their zone
slots and factors, magic is nullified on a no-magic cell (dolls
excepted) and the policies do not choose it there. Dragon Papi is added
as a checkpoint.
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -19932,12 +19932,12 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>partly</t>
+          <t>read</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>docs/FORMULAS.md 16.2: zone value 2 of a cell forbids actions with the magic flag (0x41a48b, 0x41c191, 0x41e04f; the voice Fleed_Zone_00010 at 0x44906c). Not read: which fixed battles stand on such cells (the .map files of each Data.pck and the positions of the events)</t>
+          <t>docs/FORMULAS.md 16.2: zone value 2 forbids actions with the magic flag, dolls excepted (0x41a48b, 0x41c191, 0x41e04f; the game's own dialogue in St06_c0030 says it nullifies magic for everybody). tools/map_data.py reads the maps (42-byte cells: kind, index, two zone slots, zone of the floor) and the event scripts (an event cell names its script; command 0x1F starts a fixed battle): 175 of the 196 fixed battles are placed on their cell, 8 on a no-magic cell (Dragon Papi among the story bosses). The other 21 are started away from a cell of a floor</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: damage ends chants, songs, dances and dolls by the interruption
damage ends chants, songs, dances and dolls by the interruption roll,
and wakes a sleeping unit; phase 0 closed again
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -19998,12 +19998,12 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>not read</t>
+          <t>read</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Found 2026-10-06: atwiki dt2-2 page 131 says a doll is cancelled by damage with some chance, as songs and dances are; the chant interruption (0x44d001, message "cancellation of chant etc.") is the likely place; the simulator ends them only by stun and effect 425</t>
+          <t>docs/FORMULAS.md 16.6: the interruption roll of a hit (2.5) sets a flag of the hit; when the damage is applied (0x47ea83 - 0x47eabb) the flag ends the chant, the songs, the dances and the dolls of the target together. Damage also wakes a sleeping target (0x47ea6b - 0x47ea80). sim/battle.py plays both</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: reference level from the guides with the jumps of vanilla
reference level from the guides with the jumps of vanilla; back and
forth of a fight kept; AI set resets every turn

- the decisions of 2026-10-07: guide levels as the base, vanilla level
jumps kept and controlled (R03 rewritten), the back and forth of a fight
kept with no excess of power (R10) - sheet GuideLevels; reference level
= guide, else the level covering 90% of the encounters of the boss's
zone, never falling; tools/checkpoint_levels.py writes the curve and its
11 jumps - calibration K09: the Queen of Darkness at full strength
(battle 41) at 55 - 60, as atwiki page 207 says - 0x430f56: the AI
starts every turn from set 0 (a set no longer carries over; the Queen
cast her barrier forever) - policies: no action a visible barrier
cancels (192, 182); defend when nothing can land
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -9293,7 +9293,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -9320,7 +9319,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -9347,7 +9345,6 @@
           <t>12.3 special damage, 2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -9374,7 +9371,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -9401,7 +9397,6 @@
           <t>2.7 special damage</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -9428,7 +9423,6 @@
           <t>6b healing</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -9455,7 +9449,6 @@
           <t>actions</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -9482,7 +9475,6 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -9509,7 +9501,6 @@
           <t>2.7 special damage, 3 magic attack</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -9536,7 +9527,6 @@
           <t>outside battle</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -9563,7 +9553,6 @@
           <t>14 encounter rate</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -9595,7 +9584,6 @@
           <t>0x47ffc0</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -9622,7 +9610,6 @@
           <t>outside battle</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -9649,7 +9636,6 @@
           <t>12.9 after a hit</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -9676,7 +9662,6 @@
           <t>2 physical attack, 2.2 attack value</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -9703,7 +9688,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -9730,7 +9714,6 @@
           <t>2 physical attack, 2.3 defence value</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -9757,7 +9740,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -9784,7 +9766,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -9811,7 +9792,6 @@
           <t>4 critical hits</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -9838,7 +9818,6 @@
           <t>4 critical hits</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -9865,7 +9844,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -9892,7 +9870,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -9919,7 +9896,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -9946,7 +9922,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -9973,7 +9948,6 @@
           <t>5c turn delay</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -10000,7 +9974,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -10027,7 +10000,6 @@
           <t>steal</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -10054,7 +10026,6 @@
           <t>steal</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -10081,7 +10052,6 @@
           <t>steal</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -10113,7 +10083,6 @@
           <t>0x480e20</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -10140,7 +10109,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -10167,7 +10135,6 @@
           <t>4 critical hits</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -10194,7 +10161,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -10221,7 +10187,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -10248,7 +10213,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -10275,7 +10239,6 @@
           <t>applying a hit</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -10302,7 +10265,6 @@
           <t>applying a hit</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -10329,7 +10291,6 @@
           <t>applying a hit</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -10361,7 +10322,6 @@
           <t>0x481060</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -10388,7 +10348,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -10420,7 +10379,6 @@
           <t>0x481160</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -10452,7 +10410,6 @@
           <t>0x4813a0</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -10479,7 +10436,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -10506,7 +10462,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -10533,7 +10488,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -10560,7 +10514,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -10587,7 +10540,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -10614,7 +10566,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -10641,7 +10592,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -10668,7 +10618,6 @@
           <t>12.2 number of hits</t>
         </is>
       </c>
-      <c r="H52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -10695,7 +10644,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -10722,7 +10670,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -10749,7 +10696,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -10776,7 +10722,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -10803,7 +10748,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -10830,7 +10774,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -10857,7 +10800,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -10884,7 +10826,6 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
-      <c r="H60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -10911,7 +10852,6 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
-      <c r="H61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -10943,7 +10883,6 @@
           <t>0x4817c0</t>
         </is>
       </c>
-      <c r="H62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -10975,7 +10914,6 @@
           <t>0x481890</t>
         </is>
       </c>
-      <c r="H63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -11007,7 +10945,6 @@
           <t>0x481950</t>
         </is>
       </c>
-      <c r="H64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -11039,7 +10976,6 @@
           <t>0x481a20</t>
         </is>
       </c>
-      <c r="H65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -11066,7 +11002,6 @@
           <t>outside battle</t>
         </is>
       </c>
-      <c r="H66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -11093,7 +11028,6 @@
           <t>outside battle</t>
         </is>
       </c>
-      <c r="H67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -11120,7 +11054,6 @@
           <t>4 critical hits</t>
         </is>
       </c>
-      <c r="H68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -11147,7 +11080,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -11174,7 +11106,6 @@
           <t>9.1 who gets hit</t>
         </is>
       </c>
-      <c r="H70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -11206,7 +11137,6 @@
           <t>0x481ea0</t>
         </is>
       </c>
-      <c r="H71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -11238,7 +11168,6 @@
           <t>0x4822c0</t>
         </is>
       </c>
-      <c r="H72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -11270,7 +11199,6 @@
           <t>0x482530</t>
         </is>
       </c>
-      <c r="H73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -11302,7 +11230,6 @@
           <t>0x4827a0</t>
         </is>
       </c>
-      <c r="H74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -11334,7 +11261,6 @@
           <t>0x482a10</t>
         </is>
       </c>
-      <c r="H75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -11366,7 +11292,6 @@
           <t>0x482c80</t>
         </is>
       </c>
-      <c r="H76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -11398,7 +11323,6 @@
           <t>0x482e40</t>
         </is>
       </c>
-      <c r="H77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -11430,7 +11354,6 @@
           <t>0x4831f0</t>
         </is>
       </c>
-      <c r="H78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -11462,7 +11385,6 @@
           <t>0x4834b0</t>
         </is>
       </c>
-      <c r="H79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -11494,7 +11416,6 @@
           <t>0x4835d0</t>
         </is>
       </c>
-      <c r="H80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -11526,7 +11447,6 @@
           <t>0x483840</t>
         </is>
       </c>
-      <c r="H81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -11553,7 +11473,6 @@
           <t>4 critical hits</t>
         </is>
       </c>
-      <c r="H82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -11585,7 +11504,6 @@
           <t>0x483a60</t>
         </is>
       </c>
-      <c r="H83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -11617,7 +11535,6 @@
           <t>0x483b30</t>
         </is>
       </c>
-      <c r="H84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -11649,7 +11566,6 @@
           <t>0x483c20</t>
         </is>
       </c>
-      <c r="H85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -11681,7 +11597,6 @@
           <t>0x483d20</t>
         </is>
       </c>
-      <c r="H86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -11713,7 +11628,6 @@
           <t>0x483e00</t>
         </is>
       </c>
-      <c r="H87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -11745,7 +11659,6 @@
           <t>0x483ee0</t>
         </is>
       </c>
-      <c r="H88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -11772,7 +11685,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -11799,7 +11711,6 @@
           <t>9.1 who gets hit</t>
         </is>
       </c>
-      <c r="H90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -11826,7 +11737,6 @@
           <t>2.7 special damage</t>
         </is>
       </c>
-      <c r="H91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -11858,7 +11768,6 @@
           <t>0x484020</t>
         </is>
       </c>
-      <c r="H92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -11885,7 +11794,6 @@
           <t>2.7 special damage</t>
         </is>
       </c>
-      <c r="H93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -11912,7 +11820,6 @@
           <t>2.7 special damage</t>
         </is>
       </c>
-      <c r="H94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -11944,7 +11851,6 @@
           <t>0x484150</t>
         </is>
       </c>
-      <c r="H95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -11976,7 +11882,6 @@
           <t>0x484330</t>
         </is>
       </c>
-      <c r="H96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -12003,7 +11908,6 @@
           <t>11.1 dolls</t>
         </is>
       </c>
-      <c r="H97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -12030,7 +11934,6 @@
           <t>2 physical attack, 2.1 hit chance, 3 magic attack</t>
         </is>
       </c>
-      <c r="H98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -12057,7 +11960,6 @@
           <t>2 physical attack, 2.1 hit chance, 3 magic attack</t>
         </is>
       </c>
-      <c r="H99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -12084,7 +11986,6 @@
           <t>12.10 random moves</t>
         </is>
       </c>
-      <c r="H100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -12111,7 +12012,6 @@
           <t>12.10 random moves</t>
         </is>
       </c>
-      <c r="H101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -12138,7 +12038,6 @@
           <t>12.10 random moves</t>
         </is>
       </c>
-      <c r="H102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -12165,7 +12064,6 @@
           <t>12.10 random moves</t>
         </is>
       </c>
-      <c r="H103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -12192,7 +12090,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -12219,7 +12116,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -12246,7 +12142,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -12273,7 +12168,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -12300,7 +12194,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="n">
@@ -12327,7 +12220,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="n">
@@ -12354,7 +12246,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -12386,7 +12277,6 @@
           <t>0x4864c0</t>
         </is>
       </c>
-      <c r="H111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="n">
@@ -12413,7 +12303,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="n">
@@ -12440,7 +12329,6 @@
           <t>9.1 targets</t>
         </is>
       </c>
-      <c r="H113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -12467,7 +12355,6 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
-      <c r="H114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="n">
@@ -12494,7 +12381,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="n">
@@ -12521,7 +12407,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="n">
@@ -12548,7 +12433,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="n">
@@ -12575,7 +12459,6 @@
           <t>2 physical attack, 2.4 damage</t>
         </is>
       </c>
-      <c r="H118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="n">
@@ -12602,7 +12485,6 @@
           <t>applying a hit</t>
         </is>
       </c>
-      <c r="H119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="n">
@@ -12629,7 +12511,6 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
-      <c r="H120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="n">
@@ -12656,7 +12537,6 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
-      <c r="H121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="n">
@@ -12683,7 +12563,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="n">
@@ -12710,7 +12589,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="n">
@@ -12737,7 +12615,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="n">
@@ -12764,7 +12641,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="n">
@@ -12791,7 +12667,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="n">
@@ -12818,7 +12693,6 @@
           <t>2.8 damage received</t>
         </is>
       </c>
-      <c r="H127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="n">
@@ -12845,7 +12719,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="n">
@@ -12872,7 +12745,6 @@
           <t>2 physical attack, 2.4 damage, 3 magic attack</t>
         </is>
       </c>
-      <c r="H129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="n">
@@ -12899,7 +12771,6 @@
           <t>2 physical attack, 2.4 damage</t>
         </is>
       </c>
-      <c r="H130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="n">
@@ -12926,7 +12797,6 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
-      <c r="H131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="n">
@@ -12953,7 +12823,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="n">
@@ -12980,7 +12849,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -13007,7 +12875,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="n">
@@ -13034,7 +12901,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="n">
@@ -13061,7 +12927,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="n">
@@ -13088,7 +12953,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="n">
@@ -13115,7 +12979,6 @@
           <t>5e effects that act every turn</t>
         </is>
       </c>
-      <c r="H138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="n">
@@ -13142,7 +13005,6 @@
           <t>5e effects that act every turn</t>
         </is>
       </c>
-      <c r="H139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="n">
@@ -13169,7 +13031,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="n">
@@ -13196,7 +13057,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="n">
@@ -13223,7 +13083,6 @@
           <t>5d start of a turn</t>
         </is>
       </c>
-      <c r="H142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="n">
@@ -13250,7 +13109,6 @@
           <t>13 Pep</t>
         </is>
       </c>
-      <c r="H143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="n">
@@ -13277,7 +13135,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="n">
@@ -13304,7 +13161,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="n">
@@ -13331,7 +13187,6 @@
           <t>4 critical hits</t>
         </is>
       </c>
-      <c r="H146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="n">
@@ -13358,7 +13213,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="n">
@@ -13385,7 +13239,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="n">
@@ -13412,7 +13265,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="n">
@@ -13444,7 +13296,6 @@
           <t>0x4894a0</t>
         </is>
       </c>
-      <c r="H150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="n">
@@ -13476,7 +13327,6 @@
           <t>0x4895e0</t>
         </is>
       </c>
-      <c r="H151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="n">
@@ -13503,7 +13353,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="n">
@@ -13530,7 +13379,6 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
-      <c r="H153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="n">
@@ -13557,7 +13405,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="n">
@@ -13584,7 +13431,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="n">
@@ -13611,7 +13457,6 @@
           <t>2 physical attack, 2.1 hit chance, 5 order of turns</t>
         </is>
       </c>
-      <c r="H156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="n">
@@ -13638,7 +13483,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" t="n">
@@ -13665,7 +13509,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="n">
@@ -13692,7 +13535,6 @@
           <t>11.1 dolls</t>
         </is>
       </c>
-      <c r="H159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="n">
@@ -13719,7 +13561,6 @@
           <t>11.1 dolls</t>
         </is>
       </c>
-      <c r="H160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" t="n">
@@ -13746,7 +13587,6 @@
           <t>11.1 dolls</t>
         </is>
       </c>
-      <c r="H161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" t="n">
@@ -13773,7 +13613,6 @@
           <t>11.1 dolls</t>
         </is>
       </c>
-      <c r="H162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" t="n">
@@ -13800,7 +13639,6 @@
           <t>11.1 dolls</t>
         </is>
       </c>
-      <c r="H163" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" t="n">
@@ -13827,7 +13665,6 @@
           <t>11.1 dolls</t>
         </is>
       </c>
-      <c r="H164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="n">
@@ -13859,7 +13696,6 @@
           <t>0x48a430</t>
         </is>
       </c>
-      <c r="H165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="n">
@@ -13886,7 +13722,6 @@
           <t>10.1 stats of a piece of equipment</t>
         </is>
       </c>
-      <c r="H166" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" t="n">
@@ -13913,7 +13748,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H167" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" t="n">
@@ -13940,7 +13774,6 @@
           <t>6b healing</t>
         </is>
       </c>
-      <c r="H168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="n">
@@ -13972,7 +13805,6 @@
           <t>0x48a640</t>
         </is>
       </c>
-      <c r="H169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" t="n">
@@ -13999,7 +13831,6 @@
           <t>5e effects that act every turn</t>
         </is>
       </c>
-      <c r="H170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="n">
@@ -14026,7 +13857,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="n">
@@ -14053,7 +13883,6 @@
           <t>12.13 counters and follow-ups</t>
         </is>
       </c>
-      <c r="H172" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" t="n">
@@ -14080,7 +13909,6 @@
           <t>12.13 counters and follow-ups</t>
         </is>
       </c>
-      <c r="H173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="n">
@@ -14107,7 +13935,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H174" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" t="n">
@@ -14134,7 +13961,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" t="n">
@@ -14161,7 +13987,6 @@
           <t>2 physical attack, 2.1 hit chance</t>
         </is>
       </c>
-      <c r="H176" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" t="n">
@@ -14188,7 +14013,6 @@
           <t>passive rolls</t>
         </is>
       </c>
-      <c r="H177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="n">
@@ -14215,7 +14039,6 @@
           <t>passive rolls</t>
         </is>
       </c>
-      <c r="H178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" t="n">
@@ -14242,7 +14065,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H179" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" t="n">
@@ -14269,7 +14091,6 @@
           <t>2.8 damage received</t>
         </is>
       </c>
-      <c r="H180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" t="n">
@@ -14296,7 +14117,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H181" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" t="n">
@@ -14323,7 +14143,6 @@
           <t>5d start of a turn</t>
         </is>
       </c>
-      <c r="H182" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" t="n">
@@ -14350,7 +14169,6 @@
           <t>12.13 counters and follow-ups</t>
         </is>
       </c>
-      <c r="H183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="n">
@@ -14377,7 +14195,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="n">
@@ -14404,7 +14221,6 @@
           <t>12.9 after a hit</t>
         </is>
       </c>
-      <c r="H185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="n">
@@ -14431,7 +14247,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H186" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" t="n">
@@ -14458,7 +14273,6 @@
           <t>2 physical attack, 2.5 chant interruption</t>
         </is>
       </c>
-      <c r="H187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="n">
@@ -14485,7 +14299,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H188" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" t="n">
@@ -14512,7 +14325,6 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
-      <c r="H189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" t="n">
@@ -14539,7 +14351,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H190" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" t="n">
@@ -14566,7 +14377,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" t="n">
@@ -14593,7 +14403,6 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
-      <c r="H192" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" t="n">
@@ -14620,7 +14429,6 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
-      <c r="H193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" t="n">
@@ -14647,7 +14455,6 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
-      <c r="H194" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" t="n">
@@ -14674,7 +14481,6 @@
           <t>after a battle</t>
         </is>
       </c>
-      <c r="H195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" t="n">
@@ -14701,7 +14507,6 @@
           <t>after a battle</t>
         </is>
       </c>
-      <c r="H196" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" t="n">
@@ -14728,7 +14533,6 @@
           <t>passive rolls</t>
         </is>
       </c>
-      <c r="H197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" t="n">
@@ -14755,7 +14559,6 @@
           <t>items</t>
         </is>
       </c>
-      <c r="H198" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" t="n">
@@ -14782,7 +14585,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H199" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" t="n">
@@ -14809,7 +14611,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H200" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" t="n">
@@ -14836,7 +14637,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H201" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" t="n">
@@ -14863,7 +14663,6 @@
           <t>11.2 songs and dances</t>
         </is>
       </c>
-      <c r="H202" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" t="n">
@@ -14890,7 +14689,6 @@
           <t>11.2 songs and dances</t>
         </is>
       </c>
-      <c r="H203" t="inlineStr"/>
     </row>
     <row r="204">
       <c r="A204" t="n">
@@ -14917,7 +14715,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H204" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" t="n">
@@ -14944,7 +14741,6 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
-      <c r="H205" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" t="n">
@@ -14971,7 +14767,6 @@
           <t>5d start of a turn</t>
         </is>
       </c>
-      <c r="H206" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" t="n">
@@ -14998,7 +14793,6 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
-      <c r="H207" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" t="n">
@@ -15025,7 +14819,6 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
-      <c r="H208" t="inlineStr"/>
     </row>
     <row r="209">
       <c r="A209" t="n">
@@ -15052,7 +14845,6 @@
           <t>11.1 dolls, 2 physical attack, 3 magic attack, 6b healing</t>
         </is>
       </c>
-      <c r="H209" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" t="n">
@@ -15079,7 +14871,6 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
-      <c r="H210" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" t="n">
@@ -15106,7 +14897,6 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
-      <c r="H211" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" t="n">
@@ -15133,7 +14923,6 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
-      <c r="H212" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" t="n">
@@ -15160,7 +14949,6 @@
           <t>2.8 damage received</t>
         </is>
       </c>
-      <c r="H213" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" t="n">
@@ -15187,7 +14975,6 @@
           <t>12.9 after a hit</t>
         </is>
       </c>
-      <c r="H214" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" t="n">
@@ -15214,7 +15001,6 @@
           <t>6b heal cap, 6b healing</t>
         </is>
       </c>
-      <c r="H215" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" t="n">
@@ -15241,7 +15027,6 @@
           <t>3 magic attack, 6b heal cap</t>
         </is>
       </c>
-      <c r="H216" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" t="n">
@@ -15268,7 +15053,6 @@
           <t>11.1 dolls</t>
         </is>
       </c>
-      <c r="H217" t="inlineStr"/>
     </row>
     <row r="218">
       <c r="A218" t="n">
@@ -15295,7 +15079,6 @@
           <t>10.1 stats of a piece of equipment</t>
         </is>
       </c>
-      <c r="H218" t="inlineStr"/>
     </row>
     <row r="219">
       <c r="A219" t="n">
@@ -15322,7 +15105,6 @@
           <t>passive rolls</t>
         </is>
       </c>
-      <c r="H219" t="inlineStr"/>
     </row>
     <row r="220">
       <c r="A220" t="n">
@@ -15349,7 +15131,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H220" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" t="n">
@@ -15376,7 +15157,6 @@
           <t>12.13 counters and follow-ups</t>
         </is>
       </c>
-      <c r="H221" t="inlineStr"/>
     </row>
     <row r="222">
       <c r="A222" t="n">
@@ -15403,7 +15183,6 @@
           <t>12.9 after a hit</t>
         </is>
       </c>
-      <c r="H222" t="inlineStr"/>
     </row>
     <row r="223">
       <c r="A223" t="n">
@@ -15430,7 +15209,6 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
-      <c r="H223" t="inlineStr"/>
     </row>
     <row r="224">
       <c r="A224" t="n">
@@ -15457,7 +15235,6 @@
           <t>outside battle</t>
         </is>
       </c>
-      <c r="H224" t="inlineStr"/>
     </row>
     <row r="225">
       <c r="A225" t="n">
@@ -15484,7 +15261,6 @@
           <t>12.13 counters and follow-ups</t>
         </is>
       </c>
-      <c r="H225" t="inlineStr"/>
     </row>
     <row r="226">
       <c r="A226" t="n">
@@ -15511,7 +15287,6 @@
           <t>2 physical attack, 2.4 other bonuses of final damage</t>
         </is>
       </c>
-      <c r="H226" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" t="n">
@@ -15538,7 +15313,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H227" t="inlineStr"/>
     </row>
     <row r="228">
       <c r="A228" t="n">
@@ -15565,7 +15339,6 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
-      <c r="H228" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" t="n">
@@ -15592,7 +15365,6 @@
           <t>5d start of a turn</t>
         </is>
       </c>
-      <c r="H229" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" t="n">
@@ -15619,7 +15391,6 @@
           <t>12.14 after an action</t>
         </is>
       </c>
-      <c r="H230" t="inlineStr"/>
     </row>
     <row r="231">
       <c r="A231" t="n">
@@ -15646,7 +15417,6 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
-      <c r="H231" t="inlineStr"/>
     </row>
     <row r="232">
       <c r="A232" t="n">
@@ -15673,7 +15443,6 @@
           <t>11.1 dolls</t>
         </is>
       </c>
-      <c r="H232" t="inlineStr"/>
     </row>
     <row r="233">
       <c r="A233" t="n">
@@ -15700,7 +15469,6 @@
           <t>12.10 random moves</t>
         </is>
       </c>
-      <c r="H233" t="inlineStr"/>
     </row>
     <row r="234">
       <c r="A234" t="n">
@@ -15727,7 +15495,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H234" t="inlineStr"/>
     </row>
     <row r="235">
       <c r="A235" t="n">
@@ -15754,7 +15521,6 @@
           <t>6b heal cap</t>
         </is>
       </c>
-      <c r="H235" t="inlineStr"/>
     </row>
     <row r="236">
       <c r="A236" t="n">
@@ -15781,7 +15547,6 @@
           <t>9 enemy AI</t>
         </is>
       </c>
-      <c r="H236" t="inlineStr"/>
     </row>
     <row r="237">
       <c r="A237" t="n">
@@ -15808,7 +15573,6 @@
           <t>12.9 after a hit</t>
         </is>
       </c>
-      <c r="H237" t="inlineStr"/>
     </row>
     <row r="238">
       <c r="A238" t="n">
@@ -15835,7 +15599,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H238" t="inlineStr"/>
     </row>
     <row r="239">
       <c r="A239" t="n">
@@ -15862,7 +15625,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H239" t="inlineStr"/>
     </row>
     <row r="240">
       <c r="A240" t="n">
@@ -15889,7 +15651,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H240" t="inlineStr"/>
     </row>
     <row r="241">
       <c r="A241" t="n">
@@ -15916,7 +15677,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H241" t="inlineStr"/>
     </row>
     <row r="242">
       <c r="A242" t="n">
@@ -15943,7 +15703,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H242" t="inlineStr"/>
     </row>
     <row r="243">
       <c r="A243" t="n">
@@ -15970,7 +15729,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H243" t="inlineStr"/>
     </row>
     <row r="244">
       <c r="A244" t="n">
@@ -15997,7 +15755,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H244" t="inlineStr"/>
     </row>
     <row r="245">
       <c r="A245" t="n">
@@ -16024,7 +15781,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H245" t="inlineStr"/>
     </row>
     <row r="246">
       <c r="A246" t="n">
@@ -16051,7 +15807,6 @@
           <t>2 physical attack, 2.1 hit chance, 3 magic attack</t>
         </is>
       </c>
-      <c r="H246" t="inlineStr"/>
     </row>
     <row r="247">
       <c r="A247" t="n">
@@ -16078,7 +15833,6 @@
           <t>2 physical attack, 2.1 hit chance, 3 magic attack</t>
         </is>
       </c>
-      <c r="H247" t="inlineStr"/>
     </row>
     <row r="248">
       <c r="A248" t="n">
@@ -16105,7 +15859,6 @@
           <t>5e effects that act every turn</t>
         </is>
       </c>
-      <c r="H248" t="inlineStr"/>
     </row>
     <row r="249">
       <c r="A249" t="n">
@@ -16132,7 +15885,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H249" t="inlineStr"/>
     </row>
     <row r="250">
       <c r="A250" t="n">
@@ -16159,7 +15911,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H250" t="inlineStr"/>
     </row>
     <row r="251">
       <c r="A251" t="n">
@@ -16186,7 +15937,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H251" t="inlineStr"/>
     </row>
     <row r="252">
       <c r="A252" t="n">
@@ -16213,7 +15963,6 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
-      <c r="H252" t="inlineStr"/>
     </row>
     <row r="253">
       <c r="A253" t="n">
@@ -16240,7 +15989,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H253" t="inlineStr"/>
     </row>
     <row r="254">
       <c r="A254" t="n">
@@ -16267,7 +16015,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H254" t="inlineStr"/>
     </row>
     <row r="255">
       <c r="A255" t="n">
@@ -16294,7 +16041,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H255" t="inlineStr"/>
     </row>
     <row r="256">
       <c r="A256" t="n">
@@ -16321,7 +16067,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H256" t="inlineStr"/>
     </row>
     <row r="257">
       <c r="A257" t="n">
@@ -16348,7 +16093,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H257" t="inlineStr"/>
     </row>
     <row r="258">
       <c r="A258" t="n">
@@ -16375,7 +16119,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H258" t="inlineStr"/>
     </row>
     <row r="259">
       <c r="A259" t="n">
@@ -16402,7 +16145,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H259" t="inlineStr"/>
     </row>
     <row r="260">
       <c r="A260" t="n">
@@ -16429,7 +16171,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H260" t="inlineStr"/>
     </row>
     <row r="261">
       <c r="A261" t="n">
@@ -16456,7 +16197,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H261" t="inlineStr"/>
     </row>
     <row r="262">
       <c r="A262" t="n">
@@ -16483,7 +16223,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H262" t="inlineStr"/>
     </row>
     <row r="263">
       <c r="A263" t="n">
@@ -16510,7 +16249,6 @@
           <t>12.10 random moves</t>
         </is>
       </c>
-      <c r="H263" t="inlineStr"/>
     </row>
     <row r="264">
       <c r="A264" t="n">
@@ -16537,7 +16275,6 @@
           <t>12.10 random moves</t>
         </is>
       </c>
-      <c r="H264" t="inlineStr"/>
     </row>
     <row r="265">
       <c r="A265" t="n">
@@ -16564,7 +16301,6 @@
           <t>12.10 random moves</t>
         </is>
       </c>
-      <c r="H265" t="inlineStr"/>
     </row>
     <row r="266">
       <c r="A266" t="n">
@@ -16591,7 +16327,6 @@
           <t>6c EXP</t>
         </is>
       </c>
-      <c r="H266" t="inlineStr"/>
     </row>
     <row r="267">
       <c r="A267" t="n">
@@ -16618,7 +16353,6 @@
           <t>12.10 random moves</t>
         </is>
       </c>
-      <c r="H267" t="inlineStr"/>
     </row>
     <row r="268">
       <c r="A268" t="n">
@@ -16650,7 +16384,6 @@
           <t>0x48b490</t>
         </is>
       </c>
-      <c r="H268" t="inlineStr"/>
     </row>
     <row r="269">
       <c r="A269" t="n">
@@ -16677,7 +16410,6 @@
           <t>2.7 special damage</t>
         </is>
       </c>
-      <c r="H269" t="inlineStr"/>
     </row>
     <row r="270">
       <c r="A270" t="n">
@@ -16704,7 +16436,6 @@
           <t>2.7 special damage</t>
         </is>
       </c>
-      <c r="H270" t="inlineStr"/>
     </row>
     <row r="271">
       <c r="A271" t="n">
@@ -16731,7 +16462,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H271" t="inlineStr"/>
     </row>
     <row r="272">
       <c r="A272" t="n">
@@ -16758,7 +16488,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H272" t="inlineStr"/>
     </row>
     <row r="273">
       <c r="A273" t="n">
@@ -16785,7 +16514,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H273" t="inlineStr"/>
     </row>
     <row r="274">
       <c r="A274" t="n">
@@ -16812,7 +16540,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H274" t="inlineStr"/>
     </row>
     <row r="275">
       <c r="A275" t="n">
@@ -16839,7 +16566,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H275" t="inlineStr"/>
     </row>
     <row r="276">
       <c r="A276" t="n">
@@ -16866,7 +16592,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H276" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -17501,7 +17226,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -17584,17 +17309,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>The curve has no jump</t>
+          <t>The jumps of the curve are kept, more controlled</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>From one floor or boss to the next, the lethality an on-level party meets does not rise by more than the stated step, and never falls below the previous one by more than it</t>
+          <t>Where vanilla asks for a jump of level (the reference level rises from one checkpoint to the next, or a boss stands above the level of its route), the jump stays in the same place: none is removed and none grows; a large one may be softened. No new jump appears. A change upstream (EXP, enemies, catch-up) moves every level after it, so the whole curve is checked, not each checkpoint alone (the user, 2026-10-07)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Expected party level from encounter EXP; every floor and boss in order</t>
+          <t>docs/generated/CHECKPOINT_LEVELS.md, vanilla against Balance, every checkpoint in order</t>
         </is>
       </c>
     </row>
@@ -17722,6 +17447,28 @@
       <c r="C10" t="inlineStr">
         <is>
           <t>No row of Criticisms that is true in vanilla is closed by a change so small that the player would not notice it: each closed row states the figure before and after, and the after sits inside its band with margin</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>R10</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>The back and forth of a fight is kept</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>A fight stays an exchange: the enemy still threatens the party and the party has to answer. No change gives the player an excess of power; options widen because what was broken is fixed, not because the party is stronger (the user, 2026-10-07)</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Per boss, vanilla against Balance: the lowest HP share of the party during the fight, the damage the enemies deal per turn against the party's max HP, and the fight length stay inside the window of vanilla for a sensible party at the reference level</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: theme of every row of Criticisms
theme of every row of Criticisms; R01 measured on each change and in the
final pass
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N163"/>
+  <dimension ref="A1:O163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -443,6 +443,7 @@
     <col width="10" customWidth="1" min="11" max="11"/>
     <col width="24" customWidth="1" min="13" max="13"/>
     <col width="110" customWidth="1" min="14" max="14"/>
+    <col width="44" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -516,6 +517,11 @@
           <t>Why</t>
         </is>
       </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Theme</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -568,6 +574,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>T02 Speed and weapons</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -620,6 +631,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>T04 Magic</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -672,6 +688,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>T03 TP</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -724,6 +745,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>T05 Classes and mercenaries</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -776,6 +802,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>T03 TP</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -828,6 +859,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>T02 Speed and weapons</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -880,6 +916,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>T02 Speed and weapons</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -927,6 +968,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>T09 Early game</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -974,6 +1020,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>T09 Early game</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1021,6 +1072,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>T09 Early game</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1073,6 +1129,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>T04 Magic</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1120,6 +1181,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>T02 Speed and weapons</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1167,6 +1233,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>T11 Information</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1219,6 +1290,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>T04 Magic</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1266,6 +1342,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>T08 Bosses</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1318,6 +1399,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>T08 Bosses</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1365,6 +1451,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>T08 Bosses</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1422,6 +1513,11 @@
           <t>As written it does not match the code: a doll is born with 9,999 HP and ends by its count of turns (docs/FORMULAS.md 11.1). The complaint about summons acting late is row S08; the Doll Master line is row U02</t>
         </is>
       </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>T05 Classes and mercenaries</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1474,6 +1570,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>T05 Classes and mercenaries</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1521,6 +1622,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>T05 Classes and mercenaries</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1573,6 +1679,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>T05 Classes and mercenaries</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1620,6 +1731,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>T05 Classes and mercenaries</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1672,6 +1788,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>T05 Classes and mercenaries</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1719,6 +1840,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>T05 Classes and mercenaries</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1771,6 +1897,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>T05 Classes and mercenaries</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1818,6 +1949,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>T05 Classes and mercenaries</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1870,6 +2006,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>T05 Classes and mercenaries</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1917,6 +2058,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>T02 Speed and weapons</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1969,6 +2115,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>T05 Classes and mercenaries</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2016,6 +2167,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>T05 Classes and mercenaries</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2068,6 +2224,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>T07 Ailments, debuffs and locks</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2120,6 +2281,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>T05 Classes and mercenaries</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2167,6 +2333,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>T04 Magic</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2214,6 +2385,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>T11 Information</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2266,6 +2442,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>T10 Forge, enchantments and sealbooks</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2313,6 +2494,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>T14 Economy, inventory and consumables</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2365,6 +2551,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>T01 EXP and progression</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2417,6 +2608,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>T05 Classes and mercenaries</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2464,6 +2660,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>T05 Classes and mercenaries</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2516,6 +2717,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>T05 Classes and mercenaries</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2568,6 +2774,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>T05 Classes and mercenaries</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2620,6 +2831,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>T05 Classes and mercenaries</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2672,6 +2888,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>T04 Magic</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2724,6 +2945,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>T05 Classes and mercenaries</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2776,6 +3002,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>T02 Speed and weapons</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2828,6 +3059,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>T02 Speed and weapons</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2880,6 +3116,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>T02 Speed and weapons</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2927,6 +3168,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>T02 Speed and weapons</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2974,6 +3220,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>T12 Common enemies and the pace of normal fights</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -3021,6 +3272,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>T04 Magic</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -3068,6 +3324,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>T07 Ailments, debuffs and locks</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -3115,6 +3376,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>T07 Ailments, debuffs and locks</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -3162,6 +3428,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>T06 Skills</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -3214,6 +3485,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>T05 Classes and mercenaries</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -3266,6 +3542,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>T06 Skills</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -3313,6 +3594,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>T06 Skills</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -3360,6 +3646,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O58" t="inlineStr">
+        <is>
+          <t>T06 Skills</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -3407,6 +3698,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O59" t="inlineStr">
+        <is>
+          <t>T06 Skills</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -3454,6 +3750,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>T06 Skills</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -3506,6 +3807,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O61" t="inlineStr">
+        <is>
+          <t>T07 Ailments, debuffs and locks</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -3553,6 +3859,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O62" t="inlineStr">
+        <is>
+          <t>T02 Speed and weapons</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -3605,6 +3916,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O63" t="inlineStr">
+        <is>
+          <t>T01 EXP and progression</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -3657,6 +3973,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O64" t="inlineStr">
+        <is>
+          <t>T03 TP</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -3704,6 +4025,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O65" t="inlineStr">
+        <is>
+          <t>T06 Skills</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -3751,6 +4077,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O66" t="inlineStr">
+        <is>
+          <t>T06 Skills</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -3798,6 +4129,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O67" t="inlineStr">
+        <is>
+          <t>T06 Skills</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -3845,6 +4181,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O68" t="inlineStr">
+        <is>
+          <t>T06 Skills</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -3892,6 +4233,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O69" t="inlineStr">
+        <is>
+          <t>T06 Skills</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -3939,6 +4285,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O70" t="inlineStr">
+        <is>
+          <t>T06 Skills</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -3986,6 +4337,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O71" t="inlineStr">
+        <is>
+          <t>T06 Skills</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -4033,6 +4389,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O72" t="inlineStr">
+        <is>
+          <t>T06 Skills</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -4080,6 +4441,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O73" t="inlineStr">
+        <is>
+          <t>T06 Skills</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -4127,6 +4493,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O74" t="inlineStr">
+        <is>
+          <t>T06 Skills</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -4174,6 +4545,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O75" t="inlineStr">
+        <is>
+          <t>T06 Skills</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -4221,6 +4597,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O76" t="inlineStr">
+        <is>
+          <t>T06 Skills</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -4268,6 +4649,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O77" t="inlineStr">
+        <is>
+          <t>T06 Skills</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -4315,6 +4701,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O78" t="inlineStr">
+        <is>
+          <t>T06 Skills</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -4362,6 +4753,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O79" t="inlineStr">
+        <is>
+          <t>T06 Skills</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -4409,6 +4805,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O80" t="inlineStr">
+        <is>
+          <t>T06 Skills</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -4456,6 +4857,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O81" t="inlineStr">
+        <is>
+          <t>T06 Skills</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -4503,6 +4909,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O82" t="inlineStr">
+        <is>
+          <t>T06 Skills</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -4550,6 +4961,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O83" t="inlineStr">
+        <is>
+          <t>T06 Skills</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -4597,6 +5013,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O84" t="inlineStr">
+        <is>
+          <t>T06 Skills</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -4644,6 +5065,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O85" t="inlineStr">
+        <is>
+          <t>T06 Skills</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -4691,6 +5117,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O86" t="inlineStr">
+        <is>
+          <t>T06 Skills</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -4738,6 +5169,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O87" t="inlineStr">
+        <is>
+          <t>T06 Skills</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -4785,6 +5221,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O88" t="inlineStr">
+        <is>
+          <t>T06 Skills</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -4832,6 +5273,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O89" t="inlineStr">
+        <is>
+          <t>T06 Skills</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -4879,6 +5325,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O90" t="inlineStr">
+        <is>
+          <t>T06 Skills</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -4926,6 +5377,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O91" t="inlineStr">
+        <is>
+          <t>T06 Skills</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -4973,6 +5429,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O92" t="inlineStr">
+        <is>
+          <t>T06 Skills</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -5020,6 +5481,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O93" t="inlineStr">
+        <is>
+          <t>T06 Skills</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -5067,6 +5533,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O94" t="inlineStr">
+        <is>
+          <t>T06 Skills</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -5114,6 +5585,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O95" t="inlineStr">
+        <is>
+          <t>T06 Skills</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -5161,6 +5637,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O96" t="inlineStr">
+        <is>
+          <t>T06 Skills</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -5208,6 +5689,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O97" t="inlineStr">
+        <is>
+          <t>T06 Skills</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -5255,6 +5741,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O98" t="inlineStr">
+        <is>
+          <t>T06 Skills</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -5302,6 +5793,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O99" t="inlineStr">
+        <is>
+          <t>T06 Skills</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -5349,6 +5845,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O100" t="inlineStr">
+        <is>
+          <t>T06 Skills</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -5396,6 +5897,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O101" t="inlineStr">
+        <is>
+          <t>T06 Skills</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -5443,6 +5949,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O102" t="inlineStr">
+        <is>
+          <t>T06 Skills</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -5490,6 +6001,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O103" t="inlineStr">
+        <is>
+          <t>T06 Skills</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -5537,6 +6053,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O104" t="inlineStr">
+        <is>
+          <t>T06 Skills</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -5584,6 +6105,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O105" t="inlineStr">
+        <is>
+          <t>T06 Skills</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -5631,6 +6157,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O106" t="inlineStr">
+        <is>
+          <t>T06 Skills</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -5678,6 +6209,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O107" t="inlineStr">
+        <is>
+          <t>T06 Skills</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -5725,6 +6261,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O108" t="inlineStr">
+        <is>
+          <t>T06 Skills</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -5772,6 +6313,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O109" t="inlineStr">
+        <is>
+          <t>T06 Skills</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -5819,6 +6365,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O110" t="inlineStr">
+        <is>
+          <t>T06 Skills</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -5866,6 +6417,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O111" t="inlineStr">
+        <is>
+          <t>T06 Skills</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -5913,6 +6469,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O112" t="inlineStr">
+        <is>
+          <t>T06 Skills</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -5960,6 +6521,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O113" t="inlineStr">
+        <is>
+          <t>T06 Skills</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -6007,6 +6573,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O114" t="inlineStr">
+        <is>
+          <t>T06 Skills</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -6054,6 +6625,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O115" t="inlineStr">
+        <is>
+          <t>T06 Skills</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -6101,6 +6677,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O116" t="inlineStr">
+        <is>
+          <t>T06 Skills</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -6148,6 +6729,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O117" t="inlineStr">
+        <is>
+          <t>T06 Skills</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -6195,6 +6781,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O118" t="inlineStr">
+        <is>
+          <t>T06 Skills</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -6242,6 +6833,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O119" t="inlineStr">
+        <is>
+          <t>T06 Skills</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -6289,6 +6885,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O120" t="inlineStr">
+        <is>
+          <t>T06 Skills</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -6336,6 +6937,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O121" t="inlineStr">
+        <is>
+          <t>T06 Skills</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -6383,6 +6989,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O122" t="inlineStr">
+        <is>
+          <t>T06 Skills</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -6430,6 +7041,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O123" t="inlineStr">
+        <is>
+          <t>Out of the balance</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -6482,6 +7098,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O124" t="inlineStr">
+        <is>
+          <t>T08 Bosses</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -6534,6 +7155,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O125" t="inlineStr">
+        <is>
+          <t>T05 Classes and mercenaries</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -6581,6 +7207,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O126" t="inlineStr">
+        <is>
+          <t>T05 Classes and mercenaries</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -6628,6 +7259,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O127" t="inlineStr">
+        <is>
+          <t>T10 Forge, enchantments and sealbooks</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -6675,6 +7311,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O128" t="inlineStr">
+        <is>
+          <t>T10 Forge, enchantments and sealbooks</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -6727,6 +7368,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O129" t="inlineStr">
+        <is>
+          <t>T13 Map and dungeons</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -6779,6 +7425,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O130" t="inlineStr">
+        <is>
+          <t>Out of the balance</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -6826,6 +7477,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O131" t="inlineStr">
+        <is>
+          <t>T01 EXP and progression</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -6873,6 +7529,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O132" t="inlineStr">
+        <is>
+          <t>T05 Classes and mercenaries</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -6920,6 +7581,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O133" t="inlineStr">
+        <is>
+          <t>T08 Bosses</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -6967,6 +7633,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O134" t="inlineStr">
+        <is>
+          <t>T13 Map and dungeons</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -7024,6 +7695,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="O135" t="inlineStr">
+        <is>
+          <t>T01 EXP and progression</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -7081,6 +7757,11 @@
           <t>Data: EXP of enemies, EXP per level, HP and defence of common enemies. The factors by level gap chosen for U01 already shorten it</t>
         </is>
       </c>
+      <c r="O136" t="inlineStr">
+        <is>
+          <t>T12 Common enemies and the pace of normal fights</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -7138,6 +7819,11 @@
           <t>Data if true (resistances and DEF are plain numbers). The baseline lists them; the simulator says whether it is so</t>
         </is>
       </c>
+      <c r="O137" t="inlineStr">
+        <is>
+          <t>T12 Common enemies and the pace of normal fights</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -7195,6 +7881,11 @@
           <t>Needs one reading first: whether the chances are data. Worth it only if the rate is above what the party gets</t>
         </is>
       </c>
+      <c r="O138" t="inlineStr">
+        <is>
+          <t>T12 Common enemies and the pace of normal fights</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -7252,6 +7943,11 @@
           <t>This is conditions R04, R05 and R08 seen from the player. Levers are data: boss stats, their scripts, immunity bits</t>
         </is>
       </c>
+      <c r="O139" t="inlineStr">
+        <is>
+          <t>T08 Bosses</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -7309,6 +8005,11 @@
           <t>Data: chances per level of the skills, immunity bits, resistances. Row F15 holds the same for bosses</t>
         </is>
       </c>
+      <c r="O140" t="inlineStr">
+        <is>
+          <t>T07 Ailments, debuffs and locks</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -7366,6 +8067,11 @@
           <t>Data: values per level. The formulas already show why: modifiers add up inside a product, so a small one is lost</t>
         </is>
       </c>
+      <c r="O141" t="inlineStr">
+        <is>
+          <t>T07 Ailments, debuffs and locks</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -7423,6 +8129,11 @@
           <t>Row J23 says she is useless in postgame and this says she rules the story: both can be true. Data levers either way</t>
         </is>
       </c>
+      <c r="O142" t="inlineStr">
+        <is>
+          <t>T05 Classes and mercenaries</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -7480,6 +8191,11 @@
           <t>Data: the weapon rank each form names sets its weight, and its six factors its stats (tools/summon_data.py)</t>
         </is>
       </c>
+      <c r="O143" t="inlineStr">
+        <is>
+          <t>T05 Classes and mercenaries</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -7537,6 +8253,11 @@
           <t>If the code confirms it, the QoL variant says so on the enchantment; making them add up would be a change of program</t>
         </is>
       </c>
+      <c r="O144" t="inlineStr">
+        <is>
+          <t>T10 Forge, enchantments and sealbooks</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -7594,6 +8315,11 @@
           <t>Effect 87 limits it to living targets. Removing the limit changes what the skill is (lever L13); its numbers are data</t>
         </is>
       </c>
+      <c r="O145" t="inlineStr">
+        <is>
+          <t>T06 Skills</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -7651,6 +8377,11 @@
           <t>The growth tables give the same per level before and after 70, so as stated it is not in the data. What rises is the EXP each level costs; the kept curve and the gap factors answer that</t>
         </is>
       </c>
+      <c r="O146" t="inlineStr">
+        <is>
+          <t>T01 EXP and progression</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -7708,6 +8439,11 @@
           <t>Data: skill points per level (lever L11). More points also remove choices, so only if the diagnosis shows builds that cannot work</t>
         </is>
       </c>
+      <c r="O147" t="inlineStr">
+        <is>
+          <t>T01 EXP and progression</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -7765,6 +8501,11 @@
           <t>Most repeated complaint of the search. Likely data: a zone of a floor holds unread numbers before its formations. To read before phase 3</t>
         </is>
       </c>
+      <c r="O148" t="inlineStr">
+        <is>
+          <t>T13 Map and dungeons</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -7822,6 +8563,11 @@
           <t>Data: the factors of the zones of each floor (lever L28). Softening the lowering ones is benign; removing zones is not</t>
         </is>
       </c>
+      <c r="O149" t="inlineStr">
+        <is>
+          <t>T13 Map and dungeons</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -7879,6 +8625,11 @@
           <t>Data: TrapData holds a rate per trap. Worth a look with the TP economy, not before</t>
         </is>
       </c>
+      <c r="O150" t="inlineStr">
+        <is>
+          <t>T13 Map and dungeons</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -7936,6 +8687,11 @@
           <t>Row J35 says forging pays little: they speak of different things (stats against enchantments). Data: stats and innate enchantments of unique pieces</t>
         </is>
       </c>
+      <c r="O151" t="inlineStr">
+        <is>
+          <t>T10 Forge, enchantments and sealbooks</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -7993,6 +8749,11 @@
           <t>True in the code (the floor of 0.75), but it is a constant of the program shared with other formulas. Defensive builds have data levers (guard and cover skills, boss damage) that come first; the cap is touched only if they are not enough</t>
         </is>
       </c>
+      <c r="O152" t="inlineStr">
+        <is>
+          <t>T05 Classes and mercenaries</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -8050,6 +8811,11 @@
           <t>Data in part: quest ranks grant slots, and how many is a plain number. The starting 30 is not in the data read so far</t>
         </is>
       </c>
+      <c r="O153" t="inlineStr">
+        <is>
+          <t>T14 Economy, inventory and consumables</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -8107,6 +8873,11 @@
           <t>Data: gold of enemies and prices are plain numbers; the baseline already lists gold per battle by zone</t>
         </is>
       </c>
+      <c r="O154" t="inlineStr">
+        <is>
+          <t>T14 Economy, inventory and consumables</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -8164,6 +8935,11 @@
           <t>Likely data. Minor once fights pay better; keep for the pace targets</t>
         </is>
       </c>
+      <c r="O155" t="inlineStr">
+        <is>
+          <t>T14 Economy, inventory and consumables</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -8221,6 +8997,11 @@
           <t>Now measurable: the fixed battles are read. Levers are data (their stats and level); a warning is text</t>
         </is>
       </c>
+      <c r="O156" t="inlineStr">
+        <is>
+          <t>T08 Bosses</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -8278,6 +9059,11 @@
           <t>One fight, data levers. To identify among the fixed battles</t>
         </is>
       </c>
+      <c r="O157" t="inlineStr">
+        <is>
+          <t>T08 Bosses</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -8335,6 +9121,11 @@
           <t>Needs new behaviour of the program. The QoL variant already shows the speed and chant of every skill</t>
         </is>
       </c>
+      <c r="O158" t="inlineStr">
+        <is>
+          <t>T11 Information</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -8392,6 +9183,11 @@
           <t>All are new behaviour of the program: large changes to the executable, which the user ranks last</t>
         </is>
       </c>
+      <c r="O159" t="inlineStr">
+        <is>
+          <t>Out of the balance</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -8449,6 +9245,11 @@
           <t>Content and maps, not balance. The conditions of side events could become text of the QoL variant if they are ever read</t>
         </is>
       </c>
+      <c r="O160" t="inlineStr">
+        <is>
+          <t>Out of the balance</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -8506,6 +9307,11 @@
           <t>Reports from the console versions and early patches; none reproduced here and none is a balance matter</t>
         </is>
       </c>
+      <c r="O161" t="inlineStr">
+        <is>
+          <t>Out of the balance</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -8563,6 +9369,11 @@
           <t>Too vague to test as stated. It is what conditions R03 and R08 measure fight by fight</t>
         </is>
       </c>
+      <c r="O162" t="inlineStr">
+        <is>
+          <t>T12 Common enemies and the pace of normal fights</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -8623,6 +9434,11 @@
       <c r="N163" t="inlineStr">
         <is>
           <t>All data and benign: the hidden action skills (power, chances, heal and spell power), the turns a doll lasts, TP cost and speed of the cast, Doll Mastery, the growth row of the class</t>
+        </is>
+      </c>
+      <c r="O163" t="inlineStr">
+        <is>
+          <t>T05 Classes and mercenaries</t>
         </is>
       </c>
     </row>
@@ -17275,7 +18091,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Every build the simulator enumerates, not only the criticised ones</t>
+          <t>The cases each change touches (its check), and every boss of the story and the postgame with the reference parties in the final pass (BALANCE_PLAN.md section 3, approach of 2026-10-07)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: checklists and instructions for the approach of 2026-10-07
- tools/sim_coverage.py counts the five steps of phase 1 (builds,
calibration, the check of a change, postgame checkpoints) instead of a
measure per row - tools/verdicts.py: the checklist of phase 2, the state
of every row of Criticisms by theme - states of Criticisms: open,
closed, not a problem, out of the balance (S23 - S26, F85, F92 out of
the balance) - the project instructions: the goal and method of
2026-10-07 and the decisions of that day
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -7038,7 +7038,17 @@
       </c>
       <c r="L123" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>out of the balance</t>
+        </is>
+      </c>
+      <c r="M123" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="N123" t="inlineStr">
+        <is>
+          <t>Joint skills are parked by the user (BALANCE_PLAN.md section 6)</t>
         </is>
       </c>
       <c r="O123" t="inlineStr">
@@ -7422,7 +7432,17 @@
       </c>
       <c r="L130" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>out of the balance</t>
+        </is>
+      </c>
+      <c r="M130" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="N130" t="inlineStr">
+        <is>
+          <t>The DLC is ignored by the user, its items included (BALANCE_PLAN.md section 6, 2026-10-06)</t>
         </is>
       </c>
       <c r="O130" t="inlineStr">
@@ -9108,7 +9128,7 @@
       </c>
       <c r="L158" t="inlineStr">
         <is>
-          <t>out of scope</t>
+          <t>out of the balance</t>
         </is>
       </c>
       <c r="M158" t="inlineStr">
@@ -9170,7 +9190,7 @@
       </c>
       <c r="L159" t="inlineStr">
         <is>
-          <t>out of scope</t>
+          <t>out of the balance</t>
         </is>
       </c>
       <c r="M159" t="inlineStr">
@@ -9232,7 +9252,7 @@
       </c>
       <c r="L160" t="inlineStr">
         <is>
-          <t>out of scope</t>
+          <t>out of the balance</t>
         </is>
       </c>
       <c r="M160" t="inlineStr">
@@ -9294,7 +9314,7 @@
       </c>
       <c r="L161" t="inlineStr">
         <is>
-          <t>out of scope</t>
+          <t>out of the balance</t>
         </is>
       </c>
       <c r="M161" t="inlineStr">
@@ -9356,7 +9376,7 @@
       </c>
       <c r="L162" t="inlineStr">
         <is>
-          <t>merged into R03 and R08</t>
+          <t>open</t>
         </is>
       </c>
       <c r="M162" t="inlineStr">
@@ -9366,7 +9386,7 @@
       </c>
       <c r="N162" t="inlineStr">
         <is>
-          <t>Too vague to test as stated. It is what conditions R03 and R08 measure fight by fight</t>
+          <t>Too vague to test as stated. It is what conditions R03 and R08 measure fight by fight (its verdict comes with theme T12 through R03 and R08)</t>
         </is>
       </c>
       <c r="O162" t="inlineStr">
@@ -17471,7 +17491,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>open; closed (the test fails in vanilla and passes on the built variant); not a problem (the simulator shows the claim is false in vanilla, with the measure). There is no "kept": a criticism that is true in vanilla is fixed. Hard to fix is not a reason.</t>
+          <t>open (no verdict yet); closed (the change that answers it is built and its check passes: it solves the complaint with margin); not a problem (the claim is false in vanilla, with the figure that shows it: a reading of the data, a formula or a simulation); out of the balance (see the next row). There is no "kept": a complaint that is true in vanilla is fixed. Hard to fix is not a reason. States of the approach of 2026-10-07 (BALANCE_PLAN.md section 8)</t>
         </is>
       </c>
     </row>
@@ -17535,15 +17555,16 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Status, added 2026-10-05</t>
+          <t>Status: out of the balance</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>"out of scope": the row is not a claim about balance, or it can only be answered by new behaviour of the program (interface functions, content, crashes). It is kept so that the complaint is on record, with the reason in Why; it does not count against "finished". It is never used for a balance claim that is merely hard to fix. "merged into ...": the row has no test of its own and is measured by the rows named.</t>
+          <t>The row is not a claim about balance, or it can only be answered by new behaviour of the program (interface functions, content, crashes), or the user set it aside (joint skills, the DLC). It is kept so that the complaint is on record, with the reason in Why. It is never used for a balance claim that is merely hard to fix</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: verdicts on the rows out of the balance
verdicts on the rows out of the balance; QoL reopened for the conditions
of side events, in evaluation

- F85 back to open in T05: the joint opening rests on the Dark Lord and
the Joker; verdict from the final pass - F92, S24, S26 out of the
balance with the reasons; S23 a future idea, not evaluated - S25: the
conditions of side events are evaluated as QoL text (QOL_ROADMAP.md,
last section)
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -7038,22 +7038,22 @@
       </c>
       <c r="L123" t="inlineStr">
         <is>
-          <t>out of the balance</t>
+          <t>open</t>
         </is>
       </c>
       <c r="M123" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>to decide in the diagnosis</t>
         </is>
       </c>
       <c r="N123" t="inlineStr">
         <is>
-          <t>Joint skills are parked by the user (BALANCE_PLAN.md section 6)</t>
+          <t>The opening is strong through the buffs of the Dark Lord (Power Charge, War Cry) and Trump Card of the Joker (rows J21, F18, F17, J32). Those are tuned in T05 and T06; the joint skill itself is parked and not changed. Its verdict comes from the final pass: whether the opening still dominates after them (the user, 2026-10-07)</t>
         </is>
       </c>
       <c r="O123" t="inlineStr">
         <is>
-          <t>Out of the balance</t>
+          <t>T05 Classes and mercenaries</t>
         </is>
       </c>
     </row>
@@ -7442,7 +7442,7 @@
       </c>
       <c r="N130" t="inlineStr">
         <is>
-          <t>The DLC is ignored by the user, its items included (BALANCE_PLAN.md section 6, 2026-10-06)</t>
+          <t>The DLC is ignored (2026-10-06). What it eased is covered by T01: the factors by level gap (option Kept + B4) catch a member up faster than a Double EXP piece did, and a crown costs about 257 battles instead of 4,393 (docs/generated/CATCH_UP_OPTIONS.md); no new Double EXP item (the user, 2026-10-07)</t>
         </is>
       </c>
       <c r="O130" t="inlineStr">
@@ -9138,7 +9138,7 @@
       </c>
       <c r="N158" t="inlineStr">
         <is>
-          <t>Needs new behaviour of the program. The QoL variant already shows the speed and chant of every skill</t>
+          <t>A future idea of the user (2026-10-07): complex, interesting for later. Not evaluated and nothing is opened for it. The QoL variant already shows the speed and chant of every skill</t>
         </is>
       </c>
       <c r="O158" t="inlineStr">
@@ -9200,7 +9200,7 @@
       </c>
       <c r="N159" t="inlineStr">
         <is>
-          <t>All are new behaviour of the program: large changes to the executable, which the user ranks last</t>
+          <t>Out of scope: new behaviour of the program, large changes to the executable. Part of it is already answered by the QoL variant (the user, 2026-10-07)</t>
         </is>
       </c>
       <c r="O159" t="inlineStr">
@@ -9262,7 +9262,7 @@
       </c>
       <c r="N160" t="inlineStr">
         <is>
-          <t>Content and maps, not balance. The conditions of side events could become text of the QoL variant if they are ever read</t>
+          <t>Content and maps are out of the balance. The conditions of side events, which are only text, are being evaluated as an addition to the QoL variant, reopened for it (docs/QOL_ROADMAP.md, last section; the user, 2026-10-07)</t>
         </is>
       </c>
       <c r="O160" t="inlineStr">
@@ -9324,7 +9324,7 @@
       </c>
       <c r="N161" t="inlineStr">
         <is>
-          <t>Reports from the console versions and early patches; none reproduced here and none is a balance matter</t>
+          <t>Not for now: very specific, and the user has seen almost nobody report it (2026-10-07). Reports from the console versions and early patches; none reproduced here</t>
         </is>
       </c>
       <c r="O161" t="inlineStr">
@@ -17555,7 +17555,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat: the battle acts on every effect of the player's skills (228/228)
- read and played: Sacrifice, Life Bringer, Megaton Press, Special
Sleep, units per doll skill, Murder, Dark Quest, Knock Down, Pretend,
Soul Seal, Demon Wall (no race test), Genjimaru, Enemies Flee - the
arrows of Star Dust Arrow, built by the doll function with hidden action
106 (A28) - effect 425 ends chant, songs, dances and dolls; a doll's
plain attack now takes its range - docs/FORMULAS.md 16.8; EffectRules;
assumptions A17 (linked skills) and A28 (arrows)
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -10129,6 +10129,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -10155,6 +10156,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -10181,6 +10183,7 @@
           <t>12.3 special damage, 2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -10207,6 +10210,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -10233,6 +10237,7 @@
           <t>2.7 special damage</t>
         </is>
       </c>
+      <c r="H6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -10259,6 +10264,7 @@
           <t>6b healing</t>
         </is>
       </c>
+      <c r="H7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -10285,6 +10291,7 @@
           <t>actions</t>
         </is>
       </c>
+      <c r="H8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -10311,6 +10318,7 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
+      <c r="H9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -10337,6 +10345,7 @@
           <t>2.7 special damage, 3 magic attack</t>
         </is>
       </c>
+      <c r="H10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -10363,6 +10372,7 @@
           <t>outside battle</t>
         </is>
       </c>
+      <c r="H11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -10389,6 +10399,7 @@
           <t>14 encounter rate</t>
         </is>
       </c>
+      <c r="H12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -10420,6 +10431,7 @@
           <t>0x47ffc0</t>
         </is>
       </c>
+      <c r="H13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -10446,6 +10458,7 @@
           <t>outside battle</t>
         </is>
       </c>
+      <c r="H14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -10472,6 +10485,7 @@
           <t>12.9 after a hit</t>
         </is>
       </c>
+      <c r="H15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -10498,6 +10512,7 @@
           <t>2 physical attack, 2.2 attack value</t>
         </is>
       </c>
+      <c r="H16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -10524,6 +10539,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -10550,6 +10566,7 @@
           <t>2 physical attack, 2.3 defence value</t>
         </is>
       </c>
+      <c r="H18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -10576,6 +10593,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -10602,6 +10620,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -10628,6 +10647,7 @@
           <t>4 critical hits</t>
         </is>
       </c>
+      <c r="H21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -10654,6 +10674,7 @@
           <t>4 critical hits</t>
         </is>
       </c>
+      <c r="H22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -10680,6 +10701,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -10706,6 +10728,7 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
+      <c r="H24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -10732,6 +10755,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -10758,6 +10782,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -10784,6 +10809,7 @@
           <t>5c turn delay</t>
         </is>
       </c>
+      <c r="H27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -10810,6 +10836,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -10836,6 +10863,7 @@
           <t>steal</t>
         </is>
       </c>
+      <c r="H29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -10862,6 +10890,7 @@
           <t>steal</t>
         </is>
       </c>
+      <c r="H30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -10888,6 +10917,7 @@
           <t>steal</t>
         </is>
       </c>
+      <c r="H31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -10919,6 +10949,7 @@
           <t>0x480e20</t>
         </is>
       </c>
+      <c r="H32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -10945,6 +10976,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -10971,6 +11003,7 @@
           <t>4 critical hits</t>
         </is>
       </c>
+      <c r="H34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -10997,6 +11030,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -11023,6 +11057,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -11049,6 +11084,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -11075,6 +11111,7 @@
           <t>applying a hit</t>
         </is>
       </c>
+      <c r="H38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -11101,6 +11138,7 @@
           <t>applying a hit</t>
         </is>
       </c>
+      <c r="H39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -11127,6 +11165,7 @@
           <t>applying a hit</t>
         </is>
       </c>
+      <c r="H40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -11158,6 +11197,7 @@
           <t>0x481060</t>
         </is>
       </c>
+      <c r="H41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -11184,6 +11224,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -11215,6 +11256,7 @@
           <t>0x481160</t>
         </is>
       </c>
+      <c r="H43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -11246,6 +11288,7 @@
           <t>0x4813a0</t>
         </is>
       </c>
+      <c r="H44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -11272,6 +11315,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -11298,6 +11342,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -11324,6 +11369,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -11350,6 +11396,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -11376,6 +11423,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -11402,6 +11450,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -11428,6 +11477,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -11454,6 +11504,7 @@
           <t>12.2 number of hits</t>
         </is>
       </c>
+      <c r="H52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -11480,6 +11531,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -11506,6 +11558,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -11532,6 +11585,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -11558,6 +11612,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -11584,6 +11639,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -11610,6 +11666,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -11636,6 +11693,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -11662,6 +11720,7 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
+      <c r="H60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -11688,6 +11747,7 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
+      <c r="H61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -11719,6 +11779,7 @@
           <t>0x4817c0</t>
         </is>
       </c>
+      <c r="H62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -11750,6 +11811,7 @@
           <t>0x481890</t>
         </is>
       </c>
+      <c r="H63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -11781,6 +11843,7 @@
           <t>0x481950</t>
         </is>
       </c>
+      <c r="H64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -11812,6 +11875,7 @@
           <t>0x481a20</t>
         </is>
       </c>
+      <c r="H65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -11838,6 +11902,7 @@
           <t>outside battle</t>
         </is>
       </c>
+      <c r="H66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -11864,6 +11929,7 @@
           <t>outside battle</t>
         </is>
       </c>
+      <c r="H67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -11890,6 +11956,7 @@
           <t>4 critical hits</t>
         </is>
       </c>
+      <c r="H68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -11916,6 +11983,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -11942,6 +12010,7 @@
           <t>9.1 who gets hit</t>
         </is>
       </c>
+      <c r="H70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -11973,6 +12042,7 @@
           <t>0x481ea0</t>
         </is>
       </c>
+      <c r="H71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -12004,6 +12074,7 @@
           <t>0x4822c0</t>
         </is>
       </c>
+      <c r="H72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -12035,6 +12106,7 @@
           <t>0x482530</t>
         </is>
       </c>
+      <c r="H73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -12066,6 +12138,7 @@
           <t>0x4827a0</t>
         </is>
       </c>
+      <c r="H74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -12097,6 +12170,7 @@
           <t>0x482a10</t>
         </is>
       </c>
+      <c r="H75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -12128,6 +12202,7 @@
           <t>0x482c80</t>
         </is>
       </c>
+      <c r="H76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -12159,6 +12234,7 @@
           <t>0x482e40</t>
         </is>
       </c>
+      <c r="H77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -12190,6 +12266,7 @@
           <t>0x4831f0</t>
         </is>
       </c>
+      <c r="H78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -12221,6 +12298,7 @@
           <t>0x4834b0</t>
         </is>
       </c>
+      <c r="H79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -12252,6 +12330,7 @@
           <t>0x4835d0</t>
         </is>
       </c>
+      <c r="H80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -12283,6 +12362,7 @@
           <t>0x483840</t>
         </is>
       </c>
+      <c r="H81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -12309,6 +12389,7 @@
           <t>4 critical hits</t>
         </is>
       </c>
+      <c r="H82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -12340,6 +12421,7 @@
           <t>0x483a60</t>
         </is>
       </c>
+      <c r="H83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -12371,6 +12453,7 @@
           <t>0x483b30</t>
         </is>
       </c>
+      <c r="H84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -12402,6 +12485,7 @@
           <t>0x483c20</t>
         </is>
       </c>
+      <c r="H85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -12433,6 +12517,7 @@
           <t>0x483d20</t>
         </is>
       </c>
+      <c r="H86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -12464,6 +12549,7 @@
           <t>0x483e00</t>
         </is>
       </c>
+      <c r="H87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -12487,7 +12573,7 @@
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>6d recovery</t>
+          <t>12.9 after a hit, 6d recovery</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
@@ -12495,6 +12581,7 @@
           <t>0x483ee0</t>
         </is>
       </c>
+      <c r="H88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -12521,6 +12608,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -12547,6 +12635,7 @@
           <t>9.1 who gets hit</t>
         </is>
       </c>
+      <c r="H90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -12573,6 +12662,7 @@
           <t>2.7 special damage</t>
         </is>
       </c>
+      <c r="H91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -12604,6 +12694,7 @@
           <t>0x484020</t>
         </is>
       </c>
+      <c r="H92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -12630,6 +12721,7 @@
           <t>2.7 special damage</t>
         </is>
       </c>
+      <c r="H93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -12656,6 +12748,7 @@
           <t>2.7 special damage</t>
         </is>
       </c>
+      <c r="H94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -12679,7 +12772,7 @@
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>11.1 dolls</t>
+          <t>11.1 dolls, 12.9 after a hit</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
@@ -12687,6 +12780,7 @@
           <t>0x484150</t>
         </is>
       </c>
+      <c r="H95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -12718,6 +12812,7 @@
           <t>0x484330</t>
         </is>
       </c>
+      <c r="H96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -12744,6 +12839,7 @@
           <t>11.1 dolls</t>
         </is>
       </c>
+      <c r="H97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -12770,6 +12866,7 @@
           <t>2 physical attack, 2.1 hit chance, 3 magic attack</t>
         </is>
       </c>
+      <c r="H98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -12796,6 +12893,7 @@
           <t>2 physical attack, 2.1 hit chance, 3 magic attack</t>
         </is>
       </c>
+      <c r="H99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -12822,6 +12920,7 @@
           <t>12.10 random moves</t>
         </is>
       </c>
+      <c r="H100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -12848,6 +12947,7 @@
           <t>12.10 random moves</t>
         </is>
       </c>
+      <c r="H101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -12874,6 +12974,7 @@
           <t>12.10 random moves</t>
         </is>
       </c>
+      <c r="H102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -12900,6 +13001,7 @@
           <t>12.10 random moves</t>
         </is>
       </c>
+      <c r="H103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -12926,6 +13028,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -12952,6 +13055,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -12978,6 +13082,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -13004,6 +13109,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -13030,6 +13136,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="n">
@@ -13056,6 +13163,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="n">
@@ -13082,6 +13190,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -13113,6 +13222,7 @@
           <t>0x4864c0</t>
         </is>
       </c>
+      <c r="H111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="n">
@@ -13139,6 +13249,7 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
+      <c r="H112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="n">
@@ -13165,6 +13276,7 @@
           <t>9.1 targets</t>
         </is>
       </c>
+      <c r="H113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -13191,6 +13303,7 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
+      <c r="H114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="n">
@@ -13217,6 +13330,7 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
+      <c r="H115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="n">
@@ -13243,6 +13357,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="n">
@@ -13269,6 +13384,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="n">
@@ -13295,6 +13411,7 @@
           <t>2 physical attack, 2.4 damage</t>
         </is>
       </c>
+      <c r="H118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="n">
@@ -13321,6 +13438,7 @@
           <t>applying a hit</t>
         </is>
       </c>
+      <c r="H119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="n">
@@ -13347,6 +13465,7 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
+      <c r="H120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="n">
@@ -13373,6 +13492,7 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
+      <c r="H121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="n">
@@ -13399,6 +13519,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="n">
@@ -13425,6 +13546,7 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
+      <c r="H123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="n">
@@ -13451,6 +13573,7 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
+      <c r="H124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="n">
@@ -13477,6 +13600,7 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
+      <c r="H125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="n">
@@ -13503,6 +13627,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="n">
@@ -13529,6 +13654,7 @@
           <t>2.8 damage received</t>
         </is>
       </c>
+      <c r="H127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="n">
@@ -13555,6 +13681,7 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
+      <c r="H128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="n">
@@ -13581,6 +13708,7 @@
           <t>2 physical attack, 2.4 damage, 3 magic attack</t>
         </is>
       </c>
+      <c r="H129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="n">
@@ -13607,6 +13735,7 @@
           <t>2 physical attack, 2.4 damage</t>
         </is>
       </c>
+      <c r="H130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="n">
@@ -13633,6 +13762,7 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
+      <c r="H131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="n">
@@ -13659,6 +13789,7 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
+      <c r="H132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="n">
@@ -13685,6 +13816,7 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
+      <c r="H133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -13711,6 +13843,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="n">
@@ -13737,6 +13870,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="n">
@@ -13763,6 +13897,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="n">
@@ -13789,6 +13924,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="n">
@@ -13815,6 +13951,7 @@
           <t>5e effects that act every turn</t>
         </is>
       </c>
+      <c r="H138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="n">
@@ -13841,6 +13978,7 @@
           <t>5e effects that act every turn</t>
         </is>
       </c>
+      <c r="H139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="n">
@@ -13867,6 +14005,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="n">
@@ -13893,6 +14032,7 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
+      <c r="H141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="n">
@@ -13919,6 +14059,7 @@
           <t>5d start of a turn</t>
         </is>
       </c>
+      <c r="H142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="n">
@@ -13945,6 +14086,7 @@
           <t>13 Pep</t>
         </is>
       </c>
+      <c r="H143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="n">
@@ -13971,6 +14113,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="n">
@@ -13997,6 +14140,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="n">
@@ -14023,6 +14167,7 @@
           <t>4 critical hits</t>
         </is>
       </c>
+      <c r="H146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="n">
@@ -14049,6 +14194,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="n">
@@ -14075,6 +14221,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="n">
@@ -14101,6 +14248,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="n">
@@ -14132,6 +14280,7 @@
           <t>0x4894a0</t>
         </is>
       </c>
+      <c r="H150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="n">
@@ -14163,6 +14312,7 @@
           <t>0x4895e0</t>
         </is>
       </c>
+      <c r="H151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="n">
@@ -14189,6 +14339,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="n">
@@ -14215,6 +14366,7 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
+      <c r="H153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="n">
@@ -14241,6 +14393,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="n">
@@ -14267,6 +14420,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="n">
@@ -14293,6 +14447,7 @@
           <t>2 physical attack, 2.1 hit chance, 5 order of turns</t>
         </is>
       </c>
+      <c r="H156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="n">
@@ -14319,6 +14474,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" t="n">
@@ -14345,6 +14501,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="n">
@@ -14371,6 +14528,7 @@
           <t>11.1 dolls</t>
         </is>
       </c>
+      <c r="H159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="n">
@@ -14397,6 +14555,7 @@
           <t>11.1 dolls</t>
         </is>
       </c>
+      <c r="H160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" t="n">
@@ -14423,6 +14582,7 @@
           <t>11.1 dolls</t>
         </is>
       </c>
+      <c r="H161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" t="n">
@@ -14449,6 +14609,7 @@
           <t>11.1 dolls</t>
         </is>
       </c>
+      <c r="H162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" t="n">
@@ -14475,6 +14636,7 @@
           <t>11.1 dolls</t>
         </is>
       </c>
+      <c r="H163" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" t="n">
@@ -14501,6 +14663,7 @@
           <t>11.1 dolls</t>
         </is>
       </c>
+      <c r="H164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="n">
@@ -14532,6 +14695,7 @@
           <t>0x48a430</t>
         </is>
       </c>
+      <c r="H165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="n">
@@ -14558,6 +14722,7 @@
           <t>10.1 stats of a piece of equipment</t>
         </is>
       </c>
+      <c r="H166" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" t="n">
@@ -14584,6 +14749,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H167" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" t="n">
@@ -14610,6 +14776,7 @@
           <t>6b healing</t>
         </is>
       </c>
+      <c r="H168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="n">
@@ -14641,6 +14808,7 @@
           <t>0x48a640</t>
         </is>
       </c>
+      <c r="H169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" t="n">
@@ -14667,6 +14835,7 @@
           <t>5e effects that act every turn</t>
         </is>
       </c>
+      <c r="H170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="n">
@@ -14693,6 +14862,7 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
+      <c r="H171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="n">
@@ -14719,6 +14889,7 @@
           <t>12.13 counters and follow-ups</t>
         </is>
       </c>
+      <c r="H172" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" t="n">
@@ -14745,6 +14916,7 @@
           <t>12.13 counters and follow-ups</t>
         </is>
       </c>
+      <c r="H173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="n">
@@ -14771,6 +14943,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H174" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" t="n">
@@ -14797,6 +14970,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" t="n">
@@ -14823,6 +14997,7 @@
           <t>2 physical attack, 2.1 hit chance</t>
         </is>
       </c>
+      <c r="H176" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" t="n">
@@ -14849,6 +15024,7 @@
           <t>passive rolls</t>
         </is>
       </c>
+      <c r="H177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="n">
@@ -14875,6 +15051,7 @@
           <t>passive rolls</t>
         </is>
       </c>
+      <c r="H178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" t="n">
@@ -14901,6 +15078,7 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
+      <c r="H179" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" t="n">
@@ -14927,6 +15105,7 @@
           <t>2.8 damage received</t>
         </is>
       </c>
+      <c r="H180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" t="n">
@@ -14950,9 +15129,10 @@
       </c>
       <c r="F181" t="inlineStr">
         <is>
-          <t>2 physical attack</t>
-        </is>
-      </c>
+          <t>2 physical attack, 2.4 damage</t>
+        </is>
+      </c>
+      <c r="H181" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" t="n">
@@ -14979,6 +15159,7 @@
           <t>5d start of a turn</t>
         </is>
       </c>
+      <c r="H182" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" t="n">
@@ -15005,6 +15186,7 @@
           <t>12.13 counters and follow-ups</t>
         </is>
       </c>
+      <c r="H183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="n">
@@ -15031,6 +15213,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="n">
@@ -15057,6 +15240,7 @@
           <t>12.9 after a hit</t>
         </is>
       </c>
+      <c r="H185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="n">
@@ -15080,9 +15264,10 @@
       </c>
       <c r="F186" t="inlineStr">
         <is>
-          <t>2 physical attack</t>
-        </is>
-      </c>
+          <t>2 physical attack, 2.4 damage</t>
+        </is>
+      </c>
+      <c r="H186" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" t="n">
@@ -15109,6 +15294,7 @@
           <t>2 physical attack, 2.5 chant interruption</t>
         </is>
       </c>
+      <c r="H187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="n">
@@ -15135,6 +15321,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H188" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" t="n">
@@ -15161,6 +15348,7 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
+      <c r="H189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" t="n">
@@ -15187,6 +15375,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H190" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" t="n">
@@ -15213,6 +15402,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" t="n">
@@ -15239,6 +15429,7 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
+      <c r="H192" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" t="n">
@@ -15265,6 +15456,7 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
+      <c r="H193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" t="n">
@@ -15291,6 +15483,7 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
+      <c r="H194" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" t="n">
@@ -15317,6 +15510,7 @@
           <t>after a battle</t>
         </is>
       </c>
+      <c r="H195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" t="n">
@@ -15343,6 +15537,7 @@
           <t>after a battle</t>
         </is>
       </c>
+      <c r="H196" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" t="n">
@@ -15369,6 +15564,7 @@
           <t>passive rolls</t>
         </is>
       </c>
+      <c r="H197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" t="n">
@@ -15395,6 +15591,7 @@
           <t>items</t>
         </is>
       </c>
+      <c r="H198" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" t="n">
@@ -15421,6 +15618,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H199" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" t="n">
@@ -15447,6 +15645,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H200" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" t="n">
@@ -15473,6 +15672,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H201" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" t="n">
@@ -15499,6 +15699,7 @@
           <t>11.2 songs and dances</t>
         </is>
       </c>
+      <c r="H202" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" t="n">
@@ -15525,6 +15726,7 @@
           <t>11.2 songs and dances</t>
         </is>
       </c>
+      <c r="H203" t="inlineStr"/>
     </row>
     <row r="204">
       <c r="A204" t="n">
@@ -15551,6 +15753,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H204" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" t="n">
@@ -15577,6 +15780,7 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
+      <c r="H205" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" t="n">
@@ -15603,6 +15807,7 @@
           <t>5d start of a turn</t>
         </is>
       </c>
+      <c r="H206" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" t="n">
@@ -15629,6 +15834,7 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
+      <c r="H207" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" t="n">
@@ -15655,6 +15861,7 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
+      <c r="H208" t="inlineStr"/>
     </row>
     <row r="209">
       <c r="A209" t="n">
@@ -15681,6 +15888,7 @@
           <t>11.1 dolls, 2 physical attack, 3 magic attack, 6b healing</t>
         </is>
       </c>
+      <c r="H209" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" t="n">
@@ -15707,6 +15915,7 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
+      <c r="H210" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" t="n">
@@ -15733,6 +15942,7 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
+      <c r="H211" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" t="n">
@@ -15759,6 +15969,7 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
+      <c r="H212" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" t="n">
@@ -15785,6 +15996,7 @@
           <t>2.8 damage received</t>
         </is>
       </c>
+      <c r="H213" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" t="n">
@@ -15811,6 +16023,7 @@
           <t>12.9 after a hit</t>
         </is>
       </c>
+      <c r="H214" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" t="n">
@@ -15837,6 +16050,7 @@
           <t>6b heal cap, 6b healing</t>
         </is>
       </c>
+      <c r="H215" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" t="n">
@@ -15863,6 +16077,7 @@
           <t>3 magic attack, 6b heal cap</t>
         </is>
       </c>
+      <c r="H216" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" t="n">
@@ -15889,6 +16104,7 @@
           <t>11.1 dolls</t>
         </is>
       </c>
+      <c r="H217" t="inlineStr"/>
     </row>
     <row r="218">
       <c r="A218" t="n">
@@ -15915,6 +16131,7 @@
           <t>10.1 stats of a piece of equipment</t>
         </is>
       </c>
+      <c r="H218" t="inlineStr"/>
     </row>
     <row r="219">
       <c r="A219" t="n">
@@ -15941,6 +16158,7 @@
           <t>passive rolls</t>
         </is>
       </c>
+      <c r="H219" t="inlineStr"/>
     </row>
     <row r="220">
       <c r="A220" t="n">
@@ -15967,6 +16185,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H220" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" t="n">
@@ -15993,6 +16212,7 @@
           <t>12.13 counters and follow-ups</t>
         </is>
       </c>
+      <c r="H221" t="inlineStr"/>
     </row>
     <row r="222">
       <c r="A222" t="n">
@@ -16019,6 +16239,7 @@
           <t>12.9 after a hit</t>
         </is>
       </c>
+      <c r="H222" t="inlineStr"/>
     </row>
     <row r="223">
       <c r="A223" t="n">
@@ -16045,6 +16266,7 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
+      <c r="H223" t="inlineStr"/>
     </row>
     <row r="224">
       <c r="A224" t="n">
@@ -16071,6 +16293,7 @@
           <t>outside battle</t>
         </is>
       </c>
+      <c r="H224" t="inlineStr"/>
     </row>
     <row r="225">
       <c r="A225" t="n">
@@ -16097,6 +16320,7 @@
           <t>12.13 counters and follow-ups</t>
         </is>
       </c>
+      <c r="H225" t="inlineStr"/>
     </row>
     <row r="226">
       <c r="A226" t="n">
@@ -16123,6 +16347,7 @@
           <t>2 physical attack, 2.4 other bonuses of final damage</t>
         </is>
       </c>
+      <c r="H226" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" t="n">
@@ -16149,6 +16374,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H227" t="inlineStr"/>
     </row>
     <row r="228">
       <c r="A228" t="n">
@@ -16175,6 +16401,7 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
+      <c r="H228" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" t="n">
@@ -16201,6 +16428,7 @@
           <t>5d start of a turn</t>
         </is>
       </c>
+      <c r="H229" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" t="n">
@@ -16227,6 +16455,7 @@
           <t>12.14 after an action</t>
         </is>
       </c>
+      <c r="H230" t="inlineStr"/>
     </row>
     <row r="231">
       <c r="A231" t="n">
@@ -16253,6 +16482,7 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
+      <c r="H231" t="inlineStr"/>
     </row>
     <row r="232">
       <c r="A232" t="n">
@@ -16279,6 +16509,7 @@
           <t>11.1 dolls</t>
         </is>
       </c>
+      <c r="H232" t="inlineStr"/>
     </row>
     <row r="233">
       <c r="A233" t="n">
@@ -16305,6 +16536,7 @@
           <t>12.10 random moves</t>
         </is>
       </c>
+      <c r="H233" t="inlineStr"/>
     </row>
     <row r="234">
       <c r="A234" t="n">
@@ -16331,6 +16563,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H234" t="inlineStr"/>
     </row>
     <row r="235">
       <c r="A235" t="n">
@@ -16357,6 +16590,7 @@
           <t>6b heal cap</t>
         </is>
       </c>
+      <c r="H235" t="inlineStr"/>
     </row>
     <row r="236">
       <c r="A236" t="n">
@@ -16383,6 +16617,7 @@
           <t>9 enemy AI</t>
         </is>
       </c>
+      <c r="H236" t="inlineStr"/>
     </row>
     <row r="237">
       <c r="A237" t="n">
@@ -16409,6 +16644,7 @@
           <t>12.9 after a hit</t>
         </is>
       </c>
+      <c r="H237" t="inlineStr"/>
     </row>
     <row r="238">
       <c r="A238" t="n">
@@ -16435,6 +16671,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H238" t="inlineStr"/>
     </row>
     <row r="239">
       <c r="A239" t="n">
@@ -16461,6 +16698,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H239" t="inlineStr"/>
     </row>
     <row r="240">
       <c r="A240" t="n">
@@ -16487,6 +16725,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H240" t="inlineStr"/>
     </row>
     <row r="241">
       <c r="A241" t="n">
@@ -16513,6 +16752,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H241" t="inlineStr"/>
     </row>
     <row r="242">
       <c r="A242" t="n">
@@ -16539,6 +16779,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H242" t="inlineStr"/>
     </row>
     <row r="243">
       <c r="A243" t="n">
@@ -16565,6 +16806,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H243" t="inlineStr"/>
     </row>
     <row r="244">
       <c r="A244" t="n">
@@ -16591,6 +16833,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H244" t="inlineStr"/>
     </row>
     <row r="245">
       <c r="A245" t="n">
@@ -16617,6 +16860,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H245" t="inlineStr"/>
     </row>
     <row r="246">
       <c r="A246" t="n">
@@ -16643,6 +16887,7 @@
           <t>2 physical attack, 2.1 hit chance, 3 magic attack</t>
         </is>
       </c>
+      <c r="H246" t="inlineStr"/>
     </row>
     <row r="247">
       <c r="A247" t="n">
@@ -16669,6 +16914,7 @@
           <t>2 physical attack, 2.1 hit chance, 3 magic attack</t>
         </is>
       </c>
+      <c r="H247" t="inlineStr"/>
     </row>
     <row r="248">
       <c r="A248" t="n">
@@ -16695,6 +16941,7 @@
           <t>5e effects that act every turn</t>
         </is>
       </c>
+      <c r="H248" t="inlineStr"/>
     </row>
     <row r="249">
       <c r="A249" t="n">
@@ -16721,6 +16968,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H249" t="inlineStr"/>
     </row>
     <row r="250">
       <c r="A250" t="n">
@@ -16747,6 +16995,7 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
+      <c r="H250" t="inlineStr"/>
     </row>
     <row r="251">
       <c r="A251" t="n">
@@ -16773,6 +17022,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H251" t="inlineStr"/>
     </row>
     <row r="252">
       <c r="A252" t="n">
@@ -16799,6 +17049,7 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
+      <c r="H252" t="inlineStr"/>
     </row>
     <row r="253">
       <c r="A253" t="n">
@@ -16825,6 +17076,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H253" t="inlineStr"/>
     </row>
     <row r="254">
       <c r="A254" t="n">
@@ -16851,6 +17103,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H254" t="inlineStr"/>
     </row>
     <row r="255">
       <c r="A255" t="n">
@@ -16877,6 +17130,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H255" t="inlineStr"/>
     </row>
     <row r="256">
       <c r="A256" t="n">
@@ -16903,6 +17157,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H256" t="inlineStr"/>
     </row>
     <row r="257">
       <c r="A257" t="n">
@@ -16929,6 +17184,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H257" t="inlineStr"/>
     </row>
     <row r="258">
       <c r="A258" t="n">
@@ -16955,6 +17211,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H258" t="inlineStr"/>
     </row>
     <row r="259">
       <c r="A259" t="n">
@@ -16981,6 +17238,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H259" t="inlineStr"/>
     </row>
     <row r="260">
       <c r="A260" t="n">
@@ -17004,9 +17262,10 @@
       </c>
       <c r="F260" t="inlineStr">
         <is>
-          <t>2 physical attack, 3 magic attack</t>
-        </is>
-      </c>
+          <t>2 physical attack, 2.4 damage, 3 magic attack</t>
+        </is>
+      </c>
+      <c r="H260" t="inlineStr"/>
     </row>
     <row r="261">
       <c r="A261" t="n">
@@ -17033,6 +17292,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H261" t="inlineStr"/>
     </row>
     <row r="262">
       <c r="A262" t="n">
@@ -17059,6 +17319,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H262" t="inlineStr"/>
     </row>
     <row r="263">
       <c r="A263" t="n">
@@ -17085,6 +17346,7 @@
           <t>12.10 random moves</t>
         </is>
       </c>
+      <c r="H263" t="inlineStr"/>
     </row>
     <row r="264">
       <c r="A264" t="n">
@@ -17111,6 +17373,7 @@
           <t>12.10 random moves</t>
         </is>
       </c>
+      <c r="H264" t="inlineStr"/>
     </row>
     <row r="265">
       <c r="A265" t="n">
@@ -17137,6 +17400,7 @@
           <t>12.10 random moves</t>
         </is>
       </c>
+      <c r="H265" t="inlineStr"/>
     </row>
     <row r="266">
       <c r="A266" t="n">
@@ -17163,6 +17427,7 @@
           <t>6c EXP</t>
         </is>
       </c>
+      <c r="H266" t="inlineStr"/>
     </row>
     <row r="267">
       <c r="A267" t="n">
@@ -17189,6 +17454,7 @@
           <t>12.10 random moves</t>
         </is>
       </c>
+      <c r="H267" t="inlineStr"/>
     </row>
     <row r="268">
       <c r="A268" t="n">
@@ -17220,6 +17486,7 @@
           <t>0x48b490</t>
         </is>
       </c>
+      <c r="H268" t="inlineStr"/>
     </row>
     <row r="269">
       <c r="A269" t="n">
@@ -17246,6 +17513,7 @@
           <t>2.7 special damage</t>
         </is>
       </c>
+      <c r="H269" t="inlineStr"/>
     </row>
     <row r="270">
       <c r="A270" t="n">
@@ -17272,6 +17540,7 @@
           <t>2.7 special damage</t>
         </is>
       </c>
+      <c r="H270" t="inlineStr"/>
     </row>
     <row r="271">
       <c r="A271" t="n">
@@ -17298,6 +17567,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H271" t="inlineStr"/>
     </row>
     <row r="272">
       <c r="A272" t="n">
@@ -17324,6 +17594,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H272" t="inlineStr"/>
     </row>
     <row r="273">
       <c r="A273" t="n">
@@ -17350,6 +17621,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H273" t="inlineStr"/>
     </row>
     <row r="274">
       <c r="A274" t="n">
@@ -17376,6 +17648,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H274" t="inlineStr"/>
     </row>
     <row r="275">
       <c r="A275" t="n">
@@ -17402,6 +17675,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H275" t="inlineStr"/>
     </row>
     <row r="276">
       <c r="A276" t="n">
@@ -17428,6 +17702,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H276" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -20876,7 +21151,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E220"/>
+  <dimension ref="A1:E226"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -21054,7 +21329,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>0x484330: number of units created</t>
+          <t>Number of units the doll function builds: one for every doll skill, two or three arrows for Star Dust Arrow (hidden action 106)</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>0x484330, 0x484491 - 0x48449d</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -26288,6 +26568,156 @@
         </is>
       </c>
       <c r="E220" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="n">
+        <v>133</v>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>12.9 after a hit</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>Life Bringer: the target loses max HP for good, int(damage of the hit * value), through the modifier of its max HP (slot 0x2c of the unit adds to 0x98)</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>0x483ee0 - 0x483f8a</t>
+        </is>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="n">
+        <v>143</v>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>12.9 after a hit</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>Special Sleep (a result of Showtime): a sleep command of value 10.0 with a recovery chance starting at 5, applied through the roll of sleep: certain unless the unit is immune, has a resistance of 100 or a piece that nullifies sleep</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>0x484150 - 0x48424d</t>
+        </is>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="n">
+        <v>258</v>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>2.4 damage</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>Murder: when a blow is critical and the action or its user carries it, an instant death command of its value is applied through the roll of instant death (5b)</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>0x44d26f - 0x44d2cf</t>
+        </is>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="n">
+        <v>263</v>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>2.4 damage</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>Dark Quest: value times the number of ailments the attacker carries is added to the "other" bonus of a blow</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>0x44c81a - 0x44c896</t>
+        </is>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="n">
+        <v>314</v>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>11.1 dolls</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>Soul Seal: a doll of a bearer adds to each of its six stats int(the stat of the enemy its sealbook seals * value)</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>0x4fdfd0 - 0x4fe102</t>
+        </is>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="n">
+        <v>356</v>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>2.4 damage</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>Demon Wall: when any unit of the side of the target has it, the damage of a blow or a spell becomes max(0, int(damage * (1 + value))) (the values are negative). No test of race in the code</t>
+        </is>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>0x44cbf0 - 0x44cc4e, 0x44ef59</t>
+        </is>
+      </c>
+      <c r="E226" t="inlineStr">
         <is>
           <t>read</t>
         </is>

</xml_diff>

<commit_message>
feat: calibration tests against the players' measurements
calibration tests against the players' measurements (K03, K05, K07, K08)
and what they uncovered

- Summons: the base stats are the enemy record at 0x14 of SummonData
(0x10 is the model); stats are float32 products. The pairs and lowest
stats of atwiki page 105 now match exactly - Maid Mastery and Maximum
Maid add to the value of effects 128, 129, 130, 168 (getter 0x483a20)
and Maid Mastery to 272/273 (0x48a8f0): First Aid, Cook, Self-Sacrifice,
Clean and Generous Heart were too weak - Recovery after a battle read
(0x43d6a7): the party sum capped at 0.30, Maximum Maid after the cap -
Builds counted from the sheet Roles (12/12); A30: the chant test of page
105 does not fit the code as read
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -22664,12 +22664,12 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>HP recovery: int(max HP * value)</t>
+          <t>HP recovery: int(max HP * value). Its value is the figure of the skill plus the user's Maid Mastery (278) and Maximum Maid (353): the getter at slot 0x2c of its class, 0x483a20, asks 0x48bf90 for both</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>0x483ac5</t>
+          <t>0x483ac5, 0x483a20</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -22739,12 +22739,12 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Speed modifier: enters the gauge value as a bonus (5). When its action also has effect 79 it is applied only on a roll below 100 under the value of 79 times 100. The apply code also creates it by itself: -0.75 with Slow Target (293), -0.2 with the passive of effect 346</t>
+          <t>Speed modifier: enters the gauge value as a bonus (5). When its action also has effect 79 it is applied only on a roll below 100 under the value of 79 times 100. The apply code also creates it by itself: -0.75 with Slow Target (293), -0.2 with the passive of effect 346. Its value is the figure of the skill plus the user's Maid Mastery (278) and Maximum Maid (353): the getter at slot 0x2c of its class, 0x483a20, asks 0x48bf90 for both</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>0x4864c0, 0x4229ec, 0x42456e</t>
+          <t>0x4864c0, 0x4229ec, 0x42456e, 0x483a20</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -23164,12 +23164,12 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>HP restored after a battle: the values of the living members are added, the sum stops at 0.3, and every living member recovers that share of max HP (a bonus from the function of song and dance bonuses, asked with id 353, is added after the cap; not followed)</t>
+          <t>HP restored after a battle: the value of each living member (the figure plus her Maid Mastery, getter 0x48a8f0) is added, the sum stops at 0.3 (0x6d9330), and the value of Maximum Maid (353) of each is added after the cap; every member recovers int(max HP * share), at least 1; a piece of enchantment 193 gives all of it (sim/progression.py)</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>0x43d6cc - 0x43d778</t>
+          <t>0x43d6a7 - 0x43d8b4, 0x48a8f0</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -23194,7 +23194,7 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>0x43d705</t>
+          <t>0x43d705, 0x48a8f0</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">

</xml_diff>

<commit_message>
feat: verdicts of milestone 1
verdicts of milestone 1 (T01, T09, T03, Doll Master: 15 rows) and the
table

- sim/measures.py expedition (random battles in a row); the recovery
after a battle between chained fights - play no longer overwrites the
first part with the totals - columns Verdict and Proposal in Criticisms;
tools/verdicts.py counts the verdicts written - docs/THEME_TABLES.md:
the rows, verdicts with their figures and the changes proposed; nothing
applied
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O163"/>
+  <dimension ref="A1:Q163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -522,6 +522,16 @@
           <t>Theme</t>
         </is>
       </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>Verdict</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>Proposal</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -683,6 +693,11 @@
           <t>P11, P13</t>
         </is>
       </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>84 skills deal damage; 67 give less power per TP at their top level than at level 1 (median 66%), 19 below half: Sharp Stab 20%, Aura Eliminate 28%, Raging Smash 29%, Backward Swing 35%, Gust Thrust 37%, the three stings 38%, Soul Drain 38%, Geo Break 39%</t>
+        </is>
+      </c>
       <c r="L4" t="inlineStr">
         <is>
           <t>open</t>
@@ -691,6 +706,16 @@
       <c r="O4" t="inlineStr">
         <is>
           <t>T03 TP</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>TP cost per level (L12, benign) so that power per TP at the top level is at least 85% of level 1, or the level buys something stated; the skill text already shows each level (QoL)</t>
         </is>
       </c>
     </row>
@@ -797,6 +822,11 @@
           <t>P03, P10, P11, P12, P13, P14, P15</t>
         </is>
       </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Without a Maid (a healer in her place): in the middle of the story little changes (Rousset Royal Villa at 27: 18.2 of 20 battles against 20; boss C18 won 100% both), late it collapses (Actim Castle at 50: 4.9 of 20 battles against 13.6; the weakened Queen C34 won 0% against 100%) (sim/measures.py expedition, 30 runs of up to 20 random battles, kit of 3 of each shop item (2026-10-09); the bosses 40 battles each)</t>
+        </is>
+      </c>
       <c r="L6" t="inlineStr">
         <is>
           <t>open</t>
@@ -805,6 +835,16 @@
       <c r="O6" t="inlineStr">
         <is>
           <t>T03 TP</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>partly true</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>TP outside the Maid line: values of Auto-Refresh and TP recovery skills and the price of TP items (L12, L19, benign), with J03; target: Actim without a Maid 10 or more battles and the Queen won</t>
         </is>
       </c>
     </row>
@@ -963,6 +1003,11 @@
           <t>P11, P12, P13</t>
         </is>
       </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>In the first three dungeons, with no Maid skill and no items (Yuni joins in chapter 2 and has bought none by level 9), the reference party chains 18.7 - 20 of 20 random battles and its TP falls 5 - 9 points of the pool per battle: 46 - 68% left after 4 battles, 32 - 59% after 8 (sim/measures.py expedition, 30 runs of up to 20 random battles, no items, 2026-10-09). It is not empty after 3 or 4 battles</t>
+        </is>
+      </c>
       <c r="L9" t="inlineStr">
         <is>
           <t>open</t>
@@ -971,6 +1016,16 @@
       <c r="O9" t="inlineStr">
         <is>
           <t>T09 Early game</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>partly true</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>No change proposed; the TP rows of T03 (J03, J10) lower the burn further</t>
         </is>
       </c>
     </row>
@@ -1015,6 +1070,11 @@
           <t>P03</t>
         </is>
       </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Hit chance of a plain attack of the reference party against every enemy of the random battles of the first three dungeons: median 54 - 70%, lowest 47 - 56%; 56 - 85% of those enemies are hit less than 4 times in 5 (Battle.hit_chance, docs/FORMULAS.md 2.1)</t>
+        </is>
+      </c>
       <c r="L10" t="inlineStr">
         <is>
           <t>open</t>
@@ -1023,6 +1083,16 @@
       <c r="O10" t="inlineStr">
         <is>
           <t>T09 Early game</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>Lower the AGI of the agile enemies of st00 - st02 (L01, benign) so that the lowest chance of a front-line member is at least 70% and the median 80%; keep the hardest of them a little harder</t>
         </is>
       </c>
     </row>
@@ -1067,6 +1137,11 @@
           <t>P11, P13</t>
         </is>
       </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>At levels 5 - 15 a skill at its level costs 9 - 48% of its user's TP (Danger Shoot 48%, Resurrect 31%, Checkmate 30%); raising it early multiplies the cost: War Cry 7 to 11, Heal 3 to 10 points from level 1 to 4</t>
+        </is>
+      </c>
       <c r="L11" t="inlineStr">
         <is>
           <t>open</t>
@@ -1075,6 +1150,16 @@
       <c r="O11" t="inlineStr">
         <is>
           <t>T09 Early game</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>partly true</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>With J03: TP cost per level of the skills that are raised early (L12, benign)</t>
         </is>
       </c>
     </row>
@@ -1503,6 +1588,11 @@
           <t>P01, P02, P03, P10, P12, P13, P14, P15, P16</t>
         </is>
       </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>A doll is born with 9,999 HP and ends by its count of turns (docs/FORMULAS.md 11.1): an area attack does not end it</t>
+        </is>
+      </c>
       <c r="L19" t="inlineStr">
         <is>
           <t>open</t>
@@ -1516,6 +1606,16 @@
       <c r="O19" t="inlineStr">
         <is>
           <t>T05 Classes and mercenaries</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>None; the weakness of the line is U02</t>
         </is>
       </c>
     </row>
@@ -2546,6 +2646,11 @@
           <t>P12, P13</t>
         </is>
       </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>One crown takes 4,393 random battles in the best zone (25 resets from 70) (docs/generated/CATCH_UP_OPTIONS.md, section The crown)</t>
+        </is>
+      </c>
       <c r="L38" t="inlineStr">
         <is>
           <t>open</t>
@@ -2554,6 +2659,16 @@
       <c r="O38" t="inlineStr">
         <is>
           <t>T01 EXP and progression</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>Decided: B4 and one more point per reset (L11, L25, L27): 257 battles</t>
         </is>
       </c>
     </row>
@@ -3911,6 +4026,11 @@
           <t>P12, P13</t>
         </is>
       </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>The reset bonus is 1 to 5 points (0x4f94f7 - 0x4f9540); one crown 4,393 battles, best by resets from 70 (docs/generated/CATCH_UP_OPTIONS.md)</t>
+        </is>
+      </c>
       <c r="L63" t="inlineStr">
         <is>
           <t>open</t>
@@ -3919,6 +4039,16 @@
       <c r="O63" t="inlineStr">
         <is>
           <t>T01 EXP and progression</t>
+        </is>
+      </c>
+      <c r="P63" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="Q63" t="inlineStr">
+        <is>
+          <t>Decided: as J37, 257 battles, best by resets from 60</t>
         </is>
       </c>
     </row>
@@ -3968,6 +4098,11 @@
           <t>P10, P11, P12, P13</t>
         </is>
       </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>A second Maid matters late: Actim Castle at 50, 13.6 of 20 battles with one Maid, 17.2 with two (TP after 8 battles 18% against 40%); in the middle of the story one Maid already reaches 20 of 20 (sim/measures.py expedition, 30 runs of up to 20 random battles, kit of 3 of each shop item (2026-10-09))</t>
+        </is>
+      </c>
       <c r="L64" t="inlineStr">
         <is>
           <t>open</t>
@@ -3976,6 +4111,16 @@
       <c r="O64" t="inlineStr">
         <is>
           <t>T03 TP</t>
+        </is>
+      </c>
+      <c r="P64" t="inlineStr">
+        <is>
+          <t>partly true</t>
+        </is>
+      </c>
+      <c r="Q64" t="inlineStr">
+        <is>
+          <t>As J05: lower the TP burn (J03) and add TP outside the Maid, so one Maid is enough late</t>
         </is>
       </c>
     </row>
@@ -7492,6 +7637,11 @@
           <t>P12, P13</t>
         </is>
       </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>An unused member from level 1 to a party at 70: 645 random battles in vanilla (docs/generated/CATCH_UP_OPTIONS.md, from level 1)</t>
+        </is>
+      </c>
       <c r="L131" t="inlineStr">
         <is>
           <t>open</t>
@@ -7500,6 +7650,16 @@
       <c r="O131" t="inlineStr">
         <is>
           <t>T01 EXP and progression</t>
+        </is>
+      </c>
+      <c r="P131" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="Q131" t="inlineStr">
+        <is>
+          <t>Decided: B4 brings it to 79 battles; no other change</t>
         </is>
       </c>
     </row>
@@ -7707,7 +7867,7 @@
       </c>
       <c r="J135" t="inlineStr">
         <is>
-          <t>Generated: section "Catching up" of docs/generated/BALANCE_BASELINE.md</t>
+          <t>A member 10 levels behind needs 70 - 144 random battles to come within 4 levels of the party (party 30 - 70), 20 behind 116 - 311, from level 1 124 - 519; own pace 25 - 35 battles per level (docs/generated/CATCH_UP_OPTIONS.md)</t>
         </is>
       </c>
       <c r="L135" t="inlineStr">
@@ -7718,6 +7878,16 @@
       <c r="O135" t="inlineStr">
         <is>
           <t>T01 EXP and progression</t>
+        </is>
+      </c>
+      <c r="P135" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="Q135" t="inlineStr">
+        <is>
+          <t>Decided by the user on 2026-10-05: kept curve and factors B4 (L11, L25): 10 behind 19 - 36 battles, 20 behind 23 - 60; the joining level may be raised (L31). To build in milestone 1</t>
         </is>
       </c>
     </row>
@@ -8196,6 +8366,11 @@
           <t>P01, P16</t>
         </is>
       </c>
+      <c r="J143" t="inlineStr">
+        <is>
+          <t>A summon enters a battle with the gauge of a plain action and acts with a wait of 0.25 - 0.64 (median about 0.42 at level 90): like the slowest member of the party, sooner than most bosses (0.42 - 0.55); its stats follow the best of the party (docs/FORMULAS.md 11)</t>
+        </is>
+      </c>
       <c r="L143" t="inlineStr">
         <is>
           <t>open</t>
@@ -8214,6 +8389,16 @@
       <c r="O143" t="inlineStr">
         <is>
           <t>T05 Classes and mercenaries</t>
+        </is>
+      </c>
+      <c r="P143" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="Q143" t="inlineStr">
+        <is>
+          <t>None on its speed</t>
         </is>
       </c>
     </row>
@@ -8382,6 +8567,11 @@
           <t>P14</t>
         </is>
       </c>
+      <c r="J146" t="inlineStr">
+        <is>
+          <t>Growth per level does not fall after 70: the mean gain of every stat over the growth rows is the same from 50 to 70 as from 70 to 99 (99 - 100%). What rises is the EXP a level costs: 32,788 on average from 51 to 70, 70,692 from 71 to 99 (2.2 times)</t>
+        </is>
+      </c>
       <c r="L146" t="inlineStr">
         <is>
           <t>open</t>
@@ -8400,6 +8590,16 @@
       <c r="O146" t="inlineStr">
         <is>
           <t>T01 EXP and progression</t>
+        </is>
+      </c>
+      <c r="P146" t="inlineStr">
+        <is>
+          <t>partly true</t>
+        </is>
+      </c>
+      <c r="Q146" t="inlineStr">
+        <is>
+          <t>Nothing beyond the decided kept curve, which answers the cost of a level</t>
         </is>
       </c>
     </row>
@@ -8444,6 +8644,11 @@
           <t>P12</t>
         </is>
       </c>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>Skill points in all: 52 at level 30, 139 at 50, 295 at 70, 685 at 99 without resets. The skill plans of the guide cost 246 (Papillon) to 440 (Valkyrie) points: reached about level 66 - 81. By level 50 a member of the reference party holds 25 - 32 skill levels, a third of her plan</t>
+        </is>
+      </c>
       <c r="L147" t="inlineStr">
         <is>
           <t>open</t>
@@ -8462,6 +8667,16 @@
       <c r="O147" t="inlineStr">
         <is>
           <t>T01 EXP and progression</t>
+        </is>
+      </c>
+      <c r="P147" t="inlineStr">
+        <is>
+          <t>partly true</t>
+        </is>
+      </c>
+      <c r="Q147" t="inlineStr">
+        <is>
+          <t>To decide: more points per level from 30 to 70 (L11, benign with a condition), or nothing (more points also remove choices; the crown and catch-up decisions already make resets cheaper)</t>
         </is>
       </c>
     </row>
@@ -9441,6 +9656,11 @@
           <t>P03, P04, P16</t>
         </is>
       </c>
+      <c r="J163" t="inlineStr">
+        <is>
+          <t>In the same slot, Lizerietta as a Doll Master (levels 18 - 27, bosses C13, C16, C18) makes 15 - 24% of the party damage with her dolls against 17 - 36% as a Trickster (45 - 90% of it), and a fight lasts up to 26% longer; as a Soul Summoner (C25 at 36, C34 at 50) 8 - 10% against 15 - 16% as a Papillon (30 battles each)</t>
+        </is>
+      </c>
       <c r="L163" t="inlineStr">
         <is>
           <t>open</t>
@@ -9459,6 +9679,16 @@
       <c r="O163" t="inlineStr">
         <is>
           <t>T05 Classes and mercenaries</t>
+        </is>
+      </c>
+      <c r="P163" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="Q163" t="inlineStr">
+        <is>
+          <t>Data, benign (L12, L10): the power, chances and spell power of the hidden doll actions, the life of a doll (effect 147), the TP and speed of a cast, Doll Mastery, the growth row; target: the line within 90% of the other Spieler line in the same slot, keeping what is its own (autonomous allies that work in anti-magic zones, healing through Catalina)</t>
         </is>
       </c>
     </row>
@@ -10129,7 +10359,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -10156,7 +10385,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -10183,7 +10411,6 @@
           <t>12.3 special damage, 2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -10210,7 +10437,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -10237,7 +10463,6 @@
           <t>2.7 special damage</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -10264,7 +10489,6 @@
           <t>6b healing</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -10291,7 +10515,6 @@
           <t>actions</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -10318,7 +10541,6 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -10345,7 +10567,6 @@
           <t>2.7 special damage, 3 magic attack</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -10372,7 +10593,6 @@
           <t>outside battle</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -10399,7 +10619,6 @@
           <t>14 encounter rate</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -10431,7 +10650,6 @@
           <t>0x47ffc0</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -10458,7 +10676,6 @@
           <t>outside battle</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -10485,7 +10702,6 @@
           <t>12.9 after a hit</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -10512,7 +10728,6 @@
           <t>2 physical attack, 2.2 attack value</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -10539,7 +10754,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -10566,7 +10780,6 @@
           <t>2 physical attack, 2.3 defence value</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -10593,7 +10806,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -10620,7 +10832,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -10647,7 +10858,6 @@
           <t>4 critical hits</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -10674,7 +10884,6 @@
           <t>4 critical hits</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -10701,7 +10910,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -10728,7 +10936,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -10755,7 +10962,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -10782,7 +10988,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -10809,7 +11014,6 @@
           <t>5c turn delay</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -10836,7 +11040,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -10863,7 +11066,6 @@
           <t>steal</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -10890,7 +11092,6 @@
           <t>steal</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -10917,7 +11118,6 @@
           <t>steal</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -10949,7 +11149,6 @@
           <t>0x480e20</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -10976,7 +11175,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -11003,7 +11201,6 @@
           <t>4 critical hits</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -11030,7 +11227,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -11057,7 +11253,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -11084,7 +11279,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -11111,7 +11305,6 @@
           <t>applying a hit</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -11138,7 +11331,6 @@
           <t>applying a hit</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -11165,7 +11357,6 @@
           <t>applying a hit</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -11197,7 +11388,6 @@
           <t>0x481060</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -11224,7 +11414,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -11256,7 +11445,6 @@
           <t>0x481160</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -11288,7 +11476,6 @@
           <t>0x4813a0</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -11315,7 +11502,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -11342,7 +11528,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -11369,7 +11554,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -11396,7 +11580,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -11423,7 +11606,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -11450,7 +11632,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -11477,7 +11658,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -11504,7 +11684,6 @@
           <t>12.2 number of hits</t>
         </is>
       </c>
-      <c r="H52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -11531,7 +11710,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -11558,7 +11736,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -11585,7 +11762,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -11612,7 +11788,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -11639,7 +11814,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -11666,7 +11840,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -11693,7 +11866,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -11720,7 +11892,6 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
-      <c r="H60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -11747,7 +11918,6 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
-      <c r="H61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -11779,7 +11949,6 @@
           <t>0x4817c0</t>
         </is>
       </c>
-      <c r="H62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -11811,7 +11980,6 @@
           <t>0x481890</t>
         </is>
       </c>
-      <c r="H63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -11843,7 +12011,6 @@
           <t>0x481950</t>
         </is>
       </c>
-      <c r="H64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -11875,7 +12042,6 @@
           <t>0x481a20</t>
         </is>
       </c>
-      <c r="H65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -11902,7 +12068,6 @@
           <t>outside battle</t>
         </is>
       </c>
-      <c r="H66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -11929,7 +12094,6 @@
           <t>outside battle</t>
         </is>
       </c>
-      <c r="H67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -11956,7 +12120,6 @@
           <t>4 critical hits</t>
         </is>
       </c>
-      <c r="H68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -11983,7 +12146,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -12010,7 +12172,6 @@
           <t>9.1 who gets hit</t>
         </is>
       </c>
-      <c r="H70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -12042,7 +12203,6 @@
           <t>0x481ea0</t>
         </is>
       </c>
-      <c r="H71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -12074,7 +12234,6 @@
           <t>0x4822c0</t>
         </is>
       </c>
-      <c r="H72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -12106,7 +12265,6 @@
           <t>0x482530</t>
         </is>
       </c>
-      <c r="H73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -12138,7 +12296,6 @@
           <t>0x4827a0</t>
         </is>
       </c>
-      <c r="H74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -12170,7 +12327,6 @@
           <t>0x482a10</t>
         </is>
       </c>
-      <c r="H75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -12202,7 +12358,6 @@
           <t>0x482c80</t>
         </is>
       </c>
-      <c r="H76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -12234,7 +12389,6 @@
           <t>0x482e40</t>
         </is>
       </c>
-      <c r="H77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -12266,7 +12420,6 @@
           <t>0x4831f0</t>
         </is>
       </c>
-      <c r="H78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -12298,7 +12451,6 @@
           <t>0x4834b0</t>
         </is>
       </c>
-      <c r="H79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -12330,7 +12482,6 @@
           <t>0x4835d0</t>
         </is>
       </c>
-      <c r="H80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -12362,7 +12513,6 @@
           <t>0x483840</t>
         </is>
       </c>
-      <c r="H81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -12389,7 +12539,6 @@
           <t>4 critical hits</t>
         </is>
       </c>
-      <c r="H82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -12421,7 +12570,6 @@
           <t>0x483a60</t>
         </is>
       </c>
-      <c r="H83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -12453,7 +12601,6 @@
           <t>0x483b30</t>
         </is>
       </c>
-      <c r="H84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -12485,7 +12632,6 @@
           <t>0x483c20</t>
         </is>
       </c>
-      <c r="H85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -12517,7 +12663,6 @@
           <t>0x483d20</t>
         </is>
       </c>
-      <c r="H86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -12549,7 +12694,6 @@
           <t>0x483e00</t>
         </is>
       </c>
-      <c r="H87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -12581,7 +12725,6 @@
           <t>0x483ee0</t>
         </is>
       </c>
-      <c r="H88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -12608,7 +12751,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -12635,7 +12777,6 @@
           <t>9.1 who gets hit</t>
         </is>
       </c>
-      <c r="H90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -12662,7 +12803,6 @@
           <t>2.7 special damage</t>
         </is>
       </c>
-      <c r="H91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -12694,7 +12834,6 @@
           <t>0x484020</t>
         </is>
       </c>
-      <c r="H92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -12721,7 +12860,6 @@
           <t>2.7 special damage</t>
         </is>
       </c>
-      <c r="H93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -12748,7 +12886,6 @@
           <t>2.7 special damage</t>
         </is>
       </c>
-      <c r="H94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -12780,7 +12917,6 @@
           <t>0x484150</t>
         </is>
       </c>
-      <c r="H95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -12812,7 +12948,6 @@
           <t>0x484330</t>
         </is>
       </c>
-      <c r="H96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -12839,7 +12974,6 @@
           <t>11.1 dolls</t>
         </is>
       </c>
-      <c r="H97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -12866,7 +13000,6 @@
           <t>2 physical attack, 2.1 hit chance, 3 magic attack</t>
         </is>
       </c>
-      <c r="H98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -12893,7 +13026,6 @@
           <t>2 physical attack, 2.1 hit chance, 3 magic attack</t>
         </is>
       </c>
-      <c r="H99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -12920,7 +13052,6 @@
           <t>12.10 random moves</t>
         </is>
       </c>
-      <c r="H100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -12947,7 +13078,6 @@
           <t>12.10 random moves</t>
         </is>
       </c>
-      <c r="H101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -12974,7 +13104,6 @@
           <t>12.10 random moves</t>
         </is>
       </c>
-      <c r="H102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -13001,7 +13130,6 @@
           <t>12.10 random moves</t>
         </is>
       </c>
-      <c r="H103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -13028,7 +13156,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -13055,7 +13182,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -13082,7 +13208,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -13109,7 +13234,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -13136,7 +13260,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="n">
@@ -13163,7 +13286,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="n">
@@ -13190,7 +13312,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -13222,7 +13343,6 @@
           <t>0x4864c0</t>
         </is>
       </c>
-      <c r="H111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="n">
@@ -13249,7 +13369,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="n">
@@ -13276,7 +13395,6 @@
           <t>9.1 targets</t>
         </is>
       </c>
-      <c r="H113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -13303,7 +13421,6 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
-      <c r="H114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="n">
@@ -13330,7 +13447,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="n">
@@ -13357,7 +13473,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="n">
@@ -13384,7 +13499,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="n">
@@ -13411,7 +13525,6 @@
           <t>2 physical attack, 2.4 damage</t>
         </is>
       </c>
-      <c r="H118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="n">
@@ -13438,7 +13551,6 @@
           <t>applying a hit</t>
         </is>
       </c>
-      <c r="H119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="n">
@@ -13465,7 +13577,6 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
-      <c r="H120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="n">
@@ -13492,7 +13603,6 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
-      <c r="H121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="n">
@@ -13519,7 +13629,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="n">
@@ -13546,7 +13655,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="n">
@@ -13573,7 +13681,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="n">
@@ -13600,7 +13707,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="n">
@@ -13627,7 +13733,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="n">
@@ -13654,7 +13759,6 @@
           <t>2.8 damage received</t>
         </is>
       </c>
-      <c r="H127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="n">
@@ -13681,7 +13785,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="n">
@@ -13708,7 +13811,6 @@
           <t>2 physical attack, 2.4 damage, 3 magic attack</t>
         </is>
       </c>
-      <c r="H129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="n">
@@ -13735,7 +13837,6 @@
           <t>2 physical attack, 2.4 damage</t>
         </is>
       </c>
-      <c r="H130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="n">
@@ -13762,7 +13863,6 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
-      <c r="H131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="n">
@@ -13789,7 +13889,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="n">
@@ -13816,7 +13915,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -13843,7 +13941,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="n">
@@ -13870,7 +13967,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="n">
@@ -13897,7 +13993,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="n">
@@ -13924,7 +14019,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="n">
@@ -13951,7 +14045,6 @@
           <t>5e effects that act every turn</t>
         </is>
       </c>
-      <c r="H138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="n">
@@ -13978,7 +14071,6 @@
           <t>5e effects that act every turn</t>
         </is>
       </c>
-      <c r="H139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="n">
@@ -14005,7 +14097,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="n">
@@ -14032,7 +14123,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="n">
@@ -14059,7 +14149,6 @@
           <t>5d start of a turn</t>
         </is>
       </c>
-      <c r="H142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="n">
@@ -14086,7 +14175,6 @@
           <t>13 Pep</t>
         </is>
       </c>
-      <c r="H143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="n">
@@ -14113,7 +14201,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="n">
@@ -14140,7 +14227,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="n">
@@ -14167,7 +14253,6 @@
           <t>4 critical hits</t>
         </is>
       </c>
-      <c r="H146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="n">
@@ -14194,7 +14279,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="n">
@@ -14221,7 +14305,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="n">
@@ -14248,7 +14331,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="n">
@@ -14280,7 +14362,6 @@
           <t>0x4894a0</t>
         </is>
       </c>
-      <c r="H150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="n">
@@ -14312,7 +14393,6 @@
           <t>0x4895e0</t>
         </is>
       </c>
-      <c r="H151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="n">
@@ -14339,7 +14419,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="n">
@@ -14366,7 +14445,6 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
-      <c r="H153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="n">
@@ -14393,7 +14471,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="n">
@@ -14420,7 +14497,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="n">
@@ -14447,7 +14523,6 @@
           <t>2 physical attack, 2.1 hit chance, 5 order of turns</t>
         </is>
       </c>
-      <c r="H156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="n">
@@ -14474,7 +14549,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" t="n">
@@ -14501,7 +14575,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="n">
@@ -14528,7 +14601,6 @@
           <t>11.1 dolls</t>
         </is>
       </c>
-      <c r="H159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="n">
@@ -14555,7 +14627,6 @@
           <t>11.1 dolls</t>
         </is>
       </c>
-      <c r="H160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" t="n">
@@ -14582,7 +14653,6 @@
           <t>11.1 dolls</t>
         </is>
       </c>
-      <c r="H161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" t="n">
@@ -14609,7 +14679,6 @@
           <t>11.1 dolls</t>
         </is>
       </c>
-      <c r="H162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" t="n">
@@ -14636,7 +14705,6 @@
           <t>11.1 dolls</t>
         </is>
       </c>
-      <c r="H163" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" t="n">
@@ -14663,7 +14731,6 @@
           <t>11.1 dolls</t>
         </is>
       </c>
-      <c r="H164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="n">
@@ -14695,7 +14762,6 @@
           <t>0x48a430</t>
         </is>
       </c>
-      <c r="H165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="n">
@@ -14722,7 +14788,6 @@
           <t>10.1 stats of a piece of equipment</t>
         </is>
       </c>
-      <c r="H166" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" t="n">
@@ -14749,7 +14814,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H167" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" t="n">
@@ -14776,7 +14840,6 @@
           <t>6b healing</t>
         </is>
       </c>
-      <c r="H168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="n">
@@ -14808,7 +14871,6 @@
           <t>0x48a640</t>
         </is>
       </c>
-      <c r="H169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" t="n">
@@ -14835,7 +14897,6 @@
           <t>5e effects that act every turn</t>
         </is>
       </c>
-      <c r="H170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="n">
@@ -14862,7 +14923,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="n">
@@ -14889,7 +14949,6 @@
           <t>12.13 counters and follow-ups</t>
         </is>
       </c>
-      <c r="H172" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" t="n">
@@ -14916,7 +14975,6 @@
           <t>12.13 counters and follow-ups</t>
         </is>
       </c>
-      <c r="H173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="n">
@@ -14943,7 +15001,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H174" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" t="n">
@@ -14970,7 +15027,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" t="n">
@@ -14997,7 +15053,6 @@
           <t>2 physical attack, 2.1 hit chance</t>
         </is>
       </c>
-      <c r="H176" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" t="n">
@@ -15024,7 +15079,6 @@
           <t>passive rolls</t>
         </is>
       </c>
-      <c r="H177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="n">
@@ -15051,7 +15105,6 @@
           <t>passive rolls</t>
         </is>
       </c>
-      <c r="H178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" t="n">
@@ -15078,7 +15131,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H179" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" t="n">
@@ -15105,7 +15157,6 @@
           <t>2.8 damage received</t>
         </is>
       </c>
-      <c r="H180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" t="n">
@@ -15132,7 +15183,6 @@
           <t>2 physical attack, 2.4 damage</t>
         </is>
       </c>
-      <c r="H181" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" t="n">
@@ -15159,7 +15209,6 @@
           <t>5d start of a turn</t>
         </is>
       </c>
-      <c r="H182" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" t="n">
@@ -15186,7 +15235,6 @@
           <t>12.13 counters and follow-ups</t>
         </is>
       </c>
-      <c r="H183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="n">
@@ -15213,7 +15261,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="n">
@@ -15240,7 +15287,6 @@
           <t>12.9 after a hit</t>
         </is>
       </c>
-      <c r="H185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="n">
@@ -15267,7 +15313,6 @@
           <t>2 physical attack, 2.4 damage</t>
         </is>
       </c>
-      <c r="H186" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" t="n">
@@ -15294,7 +15339,6 @@
           <t>2 physical attack, 2.5 chant interruption</t>
         </is>
       </c>
-      <c r="H187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="n">
@@ -15321,7 +15365,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H188" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" t="n">
@@ -15348,7 +15391,6 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
-      <c r="H189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" t="n">
@@ -15375,7 +15417,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H190" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" t="n">
@@ -15402,7 +15443,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" t="n">
@@ -15429,7 +15469,6 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
-      <c r="H192" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" t="n">
@@ -15456,7 +15495,6 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
-      <c r="H193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" t="n">
@@ -15483,7 +15521,6 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
-      <c r="H194" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" t="n">
@@ -15510,7 +15547,6 @@
           <t>after a battle</t>
         </is>
       </c>
-      <c r="H195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" t="n">
@@ -15537,7 +15573,6 @@
           <t>after a battle</t>
         </is>
       </c>
-      <c r="H196" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" t="n">
@@ -15564,7 +15599,6 @@
           <t>passive rolls</t>
         </is>
       </c>
-      <c r="H197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" t="n">
@@ -15591,7 +15625,6 @@
           <t>items</t>
         </is>
       </c>
-      <c r="H198" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" t="n">
@@ -15618,7 +15651,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H199" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" t="n">
@@ -15645,7 +15677,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H200" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" t="n">
@@ -15672,7 +15703,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H201" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" t="n">
@@ -15699,7 +15729,6 @@
           <t>11.2 songs and dances</t>
         </is>
       </c>
-      <c r="H202" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" t="n">
@@ -15726,7 +15755,6 @@
           <t>11.2 songs and dances</t>
         </is>
       </c>
-      <c r="H203" t="inlineStr"/>
     </row>
     <row r="204">
       <c r="A204" t="n">
@@ -15753,7 +15781,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H204" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" t="n">
@@ -15780,7 +15807,6 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
-      <c r="H205" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" t="n">
@@ -15807,7 +15833,6 @@
           <t>5d start of a turn</t>
         </is>
       </c>
-      <c r="H206" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" t="n">
@@ -15834,7 +15859,6 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
-      <c r="H207" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" t="n">
@@ -15861,7 +15885,6 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
-      <c r="H208" t="inlineStr"/>
     </row>
     <row r="209">
       <c r="A209" t="n">
@@ -15888,7 +15911,6 @@
           <t>11.1 dolls, 2 physical attack, 3 magic attack, 6b healing</t>
         </is>
       </c>
-      <c r="H209" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" t="n">
@@ -15915,7 +15937,6 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
-      <c r="H210" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" t="n">
@@ -15942,7 +15963,6 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
-      <c r="H211" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" t="n">
@@ -15969,7 +15989,6 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
-      <c r="H212" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" t="n">
@@ -15996,7 +16015,6 @@
           <t>2.8 damage received</t>
         </is>
       </c>
-      <c r="H213" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" t="n">
@@ -16023,7 +16041,6 @@
           <t>12.9 after a hit</t>
         </is>
       </c>
-      <c r="H214" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" t="n">
@@ -16050,7 +16067,6 @@
           <t>6b heal cap, 6b healing</t>
         </is>
       </c>
-      <c r="H215" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" t="n">
@@ -16077,7 +16093,6 @@
           <t>3 magic attack, 6b heal cap</t>
         </is>
       </c>
-      <c r="H216" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" t="n">
@@ -16104,7 +16119,6 @@
           <t>11.1 dolls</t>
         </is>
       </c>
-      <c r="H217" t="inlineStr"/>
     </row>
     <row r="218">
       <c r="A218" t="n">
@@ -16131,7 +16145,6 @@
           <t>10.1 stats of a piece of equipment</t>
         </is>
       </c>
-      <c r="H218" t="inlineStr"/>
     </row>
     <row r="219">
       <c r="A219" t="n">
@@ -16158,7 +16171,6 @@
           <t>passive rolls</t>
         </is>
       </c>
-      <c r="H219" t="inlineStr"/>
     </row>
     <row r="220">
       <c r="A220" t="n">
@@ -16185,7 +16197,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H220" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" t="n">
@@ -16212,7 +16223,6 @@
           <t>12.13 counters and follow-ups</t>
         </is>
       </c>
-      <c r="H221" t="inlineStr"/>
     </row>
     <row r="222">
       <c r="A222" t="n">
@@ -16239,7 +16249,6 @@
           <t>12.9 after a hit</t>
         </is>
       </c>
-      <c r="H222" t="inlineStr"/>
     </row>
     <row r="223">
       <c r="A223" t="n">
@@ -16266,7 +16275,6 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
-      <c r="H223" t="inlineStr"/>
     </row>
     <row r="224">
       <c r="A224" t="n">
@@ -16293,7 +16301,6 @@
           <t>outside battle</t>
         </is>
       </c>
-      <c r="H224" t="inlineStr"/>
     </row>
     <row r="225">
       <c r="A225" t="n">
@@ -16320,7 +16327,6 @@
           <t>12.13 counters and follow-ups</t>
         </is>
       </c>
-      <c r="H225" t="inlineStr"/>
     </row>
     <row r="226">
       <c r="A226" t="n">
@@ -16347,7 +16353,6 @@
           <t>2 physical attack, 2.4 other bonuses of final damage</t>
         </is>
       </c>
-      <c r="H226" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" t="n">
@@ -16374,7 +16379,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H227" t="inlineStr"/>
     </row>
     <row r="228">
       <c r="A228" t="n">
@@ -16401,7 +16405,6 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
-      <c r="H228" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" t="n">
@@ -16428,7 +16431,6 @@
           <t>5d start of a turn</t>
         </is>
       </c>
-      <c r="H229" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" t="n">
@@ -16455,7 +16457,6 @@
           <t>12.14 after an action</t>
         </is>
       </c>
-      <c r="H230" t="inlineStr"/>
     </row>
     <row r="231">
       <c r="A231" t="n">
@@ -16482,7 +16483,6 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
-      <c r="H231" t="inlineStr"/>
     </row>
     <row r="232">
       <c r="A232" t="n">
@@ -16509,7 +16509,6 @@
           <t>11.1 dolls</t>
         </is>
       </c>
-      <c r="H232" t="inlineStr"/>
     </row>
     <row r="233">
       <c r="A233" t="n">
@@ -16536,7 +16535,6 @@
           <t>12.10 random moves</t>
         </is>
       </c>
-      <c r="H233" t="inlineStr"/>
     </row>
     <row r="234">
       <c r="A234" t="n">
@@ -16563,7 +16561,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H234" t="inlineStr"/>
     </row>
     <row r="235">
       <c r="A235" t="n">
@@ -16590,7 +16587,6 @@
           <t>6b heal cap</t>
         </is>
       </c>
-      <c r="H235" t="inlineStr"/>
     </row>
     <row r="236">
       <c r="A236" t="n">
@@ -16617,7 +16613,6 @@
           <t>9 enemy AI</t>
         </is>
       </c>
-      <c r="H236" t="inlineStr"/>
     </row>
     <row r="237">
       <c r="A237" t="n">
@@ -16644,7 +16639,6 @@
           <t>12.9 after a hit</t>
         </is>
       </c>
-      <c r="H237" t="inlineStr"/>
     </row>
     <row r="238">
       <c r="A238" t="n">
@@ -16671,7 +16665,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H238" t="inlineStr"/>
     </row>
     <row r="239">
       <c r="A239" t="n">
@@ -16698,7 +16691,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H239" t="inlineStr"/>
     </row>
     <row r="240">
       <c r="A240" t="n">
@@ -16725,7 +16717,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H240" t="inlineStr"/>
     </row>
     <row r="241">
       <c r="A241" t="n">
@@ -16752,7 +16743,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H241" t="inlineStr"/>
     </row>
     <row r="242">
       <c r="A242" t="n">
@@ -16779,7 +16769,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H242" t="inlineStr"/>
     </row>
     <row r="243">
       <c r="A243" t="n">
@@ -16806,7 +16795,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H243" t="inlineStr"/>
     </row>
     <row r="244">
       <c r="A244" t="n">
@@ -16833,7 +16821,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H244" t="inlineStr"/>
     </row>
     <row r="245">
       <c r="A245" t="n">
@@ -16860,7 +16847,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H245" t="inlineStr"/>
     </row>
     <row r="246">
       <c r="A246" t="n">
@@ -16887,7 +16873,6 @@
           <t>2 physical attack, 2.1 hit chance, 3 magic attack</t>
         </is>
       </c>
-      <c r="H246" t="inlineStr"/>
     </row>
     <row r="247">
       <c r="A247" t="n">
@@ -16914,7 +16899,6 @@
           <t>2 physical attack, 2.1 hit chance, 3 magic attack</t>
         </is>
       </c>
-      <c r="H247" t="inlineStr"/>
     </row>
     <row r="248">
       <c r="A248" t="n">
@@ -16941,7 +16925,6 @@
           <t>5e effects that act every turn</t>
         </is>
       </c>
-      <c r="H248" t="inlineStr"/>
     </row>
     <row r="249">
       <c r="A249" t="n">
@@ -16968,7 +16951,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H249" t="inlineStr"/>
     </row>
     <row r="250">
       <c r="A250" t="n">
@@ -16995,7 +16977,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H250" t="inlineStr"/>
     </row>
     <row r="251">
       <c r="A251" t="n">
@@ -17022,7 +17003,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H251" t="inlineStr"/>
     </row>
     <row r="252">
       <c r="A252" t="n">
@@ -17049,7 +17029,6 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
-      <c r="H252" t="inlineStr"/>
     </row>
     <row r="253">
       <c r="A253" t="n">
@@ -17076,7 +17055,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H253" t="inlineStr"/>
     </row>
     <row r="254">
       <c r="A254" t="n">
@@ -17103,7 +17081,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H254" t="inlineStr"/>
     </row>
     <row r="255">
       <c r="A255" t="n">
@@ -17130,7 +17107,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H255" t="inlineStr"/>
     </row>
     <row r="256">
       <c r="A256" t="n">
@@ -17157,7 +17133,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H256" t="inlineStr"/>
     </row>
     <row r="257">
       <c r="A257" t="n">
@@ -17184,7 +17159,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H257" t="inlineStr"/>
     </row>
     <row r="258">
       <c r="A258" t="n">
@@ -17211,7 +17185,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H258" t="inlineStr"/>
     </row>
     <row r="259">
       <c r="A259" t="n">
@@ -17238,7 +17211,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H259" t="inlineStr"/>
     </row>
     <row r="260">
       <c r="A260" t="n">
@@ -17265,7 +17237,6 @@
           <t>2 physical attack, 2.4 damage, 3 magic attack</t>
         </is>
       </c>
-      <c r="H260" t="inlineStr"/>
     </row>
     <row r="261">
       <c r="A261" t="n">
@@ -17292,7 +17263,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H261" t="inlineStr"/>
     </row>
     <row r="262">
       <c r="A262" t="n">
@@ -17319,7 +17289,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H262" t="inlineStr"/>
     </row>
     <row r="263">
       <c r="A263" t="n">
@@ -17346,7 +17315,6 @@
           <t>12.10 random moves</t>
         </is>
       </c>
-      <c r="H263" t="inlineStr"/>
     </row>
     <row r="264">
       <c r="A264" t="n">
@@ -17373,7 +17341,6 @@
           <t>12.10 random moves</t>
         </is>
       </c>
-      <c r="H264" t="inlineStr"/>
     </row>
     <row r="265">
       <c r="A265" t="n">
@@ -17400,7 +17367,6 @@
           <t>12.10 random moves</t>
         </is>
       </c>
-      <c r="H265" t="inlineStr"/>
     </row>
     <row r="266">
       <c r="A266" t="n">
@@ -17427,7 +17393,6 @@
           <t>6c EXP</t>
         </is>
       </c>
-      <c r="H266" t="inlineStr"/>
     </row>
     <row r="267">
       <c r="A267" t="n">
@@ -17454,7 +17419,6 @@
           <t>12.10 random moves</t>
         </is>
       </c>
-      <c r="H267" t="inlineStr"/>
     </row>
     <row r="268">
       <c r="A268" t="n">
@@ -17486,7 +17450,6 @@
           <t>0x48b490</t>
         </is>
       </c>
-      <c r="H268" t="inlineStr"/>
     </row>
     <row r="269">
       <c r="A269" t="n">
@@ -17513,7 +17476,6 @@
           <t>2.7 special damage</t>
         </is>
       </c>
-      <c r="H269" t="inlineStr"/>
     </row>
     <row r="270">
       <c r="A270" t="n">
@@ -17540,7 +17502,6 @@
           <t>2.7 special damage</t>
         </is>
       </c>
-      <c r="H270" t="inlineStr"/>
     </row>
     <row r="271">
       <c r="A271" t="n">
@@ -17567,7 +17528,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H271" t="inlineStr"/>
     </row>
     <row r="272">
       <c r="A272" t="n">
@@ -17594,7 +17554,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H272" t="inlineStr"/>
     </row>
     <row r="273">
       <c r="A273" t="n">
@@ -17621,7 +17580,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H273" t="inlineStr"/>
     </row>
     <row r="274">
       <c r="A274" t="n">
@@ -17648,7 +17606,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H274" t="inlineStr"/>
     </row>
     <row r="275">
       <c r="A275" t="n">
@@ -17675,7 +17632,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H275" t="inlineStr"/>
     </row>
     <row r="276">
       <c r="A276" t="n">
@@ -17702,7 +17658,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H276" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: verdicts of milestone 2
verdicts of milestone 2 (T02, T04, T07, T12: 27 rows) and their table;
the weapon band measure

The fallback mage plan now takes the top single spell of each element
(atwiki page 136).
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -579,6 +579,11 @@
           <t>P01, P02, P03, P04, P07, P09, P10, P15</t>
         </is>
       </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Same character late (Yae, P24 at 90): a Kukri acts every 0.21, a Heavy Axe every 0.40 (1.9 actions per heavy one); yet the heavy weapon gives the most damage per time at every checkpoint measured (Heavy Axe 100%, Kukri 29 - 41%) (sim/measures.py weapon_band: the member at the level, gear and forge of the checkpoint, each basic weapon, expected damage per unit of time of the best action against its boss (2026-10-09)). Survival under the order of turns is not in this measure</t>
+        </is>
+      </c>
       <c r="L2" t="inlineStr">
         <is>
           <t>open</t>
@@ -587,6 +592,16 @@
       <c r="O2" t="inlineStr">
         <is>
           <t>T02 Speed and weapons</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>partly true</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>No change of speed; the survival of two-handed builds is checked in the final pass (R10)</t>
         </is>
       </c>
     </row>
@@ -636,6 +651,11 @@
           <t>P04, P07, P10, P13</t>
         </is>
       </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>With the top spells of the Witch (reference plan, atwiki page 136) a mage makes 172 - 191% of the damage per time of the Dark Lord at C38, P24 and P49 (boss resistances counted), and completes 88 - 97% of her chants against those bosses (sim/measures.py weapon_band: the member at the level, gear and forge of the checkpoint, each basic weapon, expected damage per unit of time of the best action against its boss (2026-10-09); chants: 20 boss fights each)</t>
+        </is>
+      </c>
       <c r="L3" t="inlineStr">
         <is>
           <t>open</t>
@@ -644,6 +664,16 @@
       <c r="O3" t="inlineStr">
         <is>
           <t>T04 Magic</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>None as stated; the mage teams are F06</t>
         </is>
       </c>
     </row>
@@ -894,6 +924,11 @@
           <t>P01, P02, P03, P08, P10, P14, P15</t>
         </is>
       </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>3 of the 13 bow skills accept a gun (Chain Spike, Guided Shot, Poison Shot). The 7 guns are unique pieces with ranks from 1.4 (Psychogun) to 2.9 (Wave Motion Gun, the slowest rank of the game)</t>
+        </is>
+      </c>
       <c r="L7" t="inlineStr">
         <is>
           <t>open</t>
@@ -902,6 +937,16 @@
       <c r="O7" t="inlineStr">
         <is>
           <t>T02 Speed and weapons</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>partly true</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>To decide: let guns use more bow skills (weapon mask, L13, structural) or none</t>
         </is>
       </c>
     </row>
@@ -951,6 +996,11 @@
           <t>P01, P02, P03, P08, P10, P14, P15, P19</t>
         </is>
       </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>For damage two-handed weapons lead at every checkpoint measured (C18, C34, P24): Heavy Axe, Claymore, Heavy Lance, Tachi and Long Bow give 100% or close; their one-handed counterparts 47 - 84% (sim/measures.py weapon_band: the member at the level, gear and forge of the checkpoint, each basic weapon, expected damage per unit of time of the best action against its boss (2026-10-09)). The shield they give up (DEF, the guard skills) is not counted</t>
+        </is>
+      </c>
       <c r="L8" t="inlineStr">
         <is>
           <t>open</t>
@@ -959,6 +1009,16 @@
       <c r="O8" t="inlineStr">
         <is>
           <t>T02 Speed and weapons</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>None for damage; survival checked in the final pass</t>
         </is>
       </c>
     </row>
@@ -1209,6 +1269,11 @@
           <t>P04, P07, P10, P13</t>
         </is>
       </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Mage over Dark Lord, damage per time: 41% (C07), 98% (C13), 189% (C18), 333% (C25), 309% (C34), 191% (C38), 172 - 174% (P24, P49): a peak in the middle and a drop after it, but no cliff (sim/measures.py weapon_band: the member at the level, gear and forge of the checkpoint, each basic weapon, expected damage per unit of time of the best action against its boss (2026-10-09))</t>
+        </is>
+      </c>
       <c r="L12" t="inlineStr">
         <is>
           <t>open</t>
@@ -1217,6 +1282,16 @@
       <c r="O12" t="inlineStr">
         <is>
           <t>T04 Magic</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>partly true</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>To decide with T04 as a whole: soften the peak (spell power of tiers 1 - 2, L12) or keep it</t>
         </is>
       </c>
     </row>
@@ -1261,6 +1336,11 @@
           <t>P01, P02, P03, P08, P10, P15</t>
         </is>
       </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Yae from Fighter at 14 with a Longsword to Berserker at 15 with a Claymore: damage per time 2.3 times higher (69 to 156), wait 0.74 to 0.76 (+3%), DEF 78 to 85 (sim/measures.py weapon_band: the member at the level, gear and forge of the checkpoint, each basic weapon, expected damage per unit of time of the best action against its boss (2026-10-09))</t>
+        </is>
+      </c>
       <c r="L13" t="inlineStr">
         <is>
           <t>open</t>
@@ -1269,6 +1349,16 @@
       <c r="O13" t="inlineStr">
         <is>
           <t>T02 Speed and weapons</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
     </row>
@@ -1370,6 +1460,11 @@
           <t>P04, P06, P07, P10, P13</t>
         </is>
       </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>A mage completes 85 - 98% of the chants she starts against the bosses C18, C25, C34, C38, P24, P28 and P49; 0 - 0.7 chants broken per fight (20 fights each)</t>
+        </is>
+      </c>
       <c r="L15" t="inlineStr">
         <is>
           <t>open</t>
@@ -1378,6 +1473,16 @@
       <c r="O15" t="inlineStr">
         <is>
           <t>T04 Magic</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
     </row>
@@ -2153,6 +2258,11 @@
           <t>P01, P02, P03, P14, P15</t>
         </is>
       </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Lightning March adds 5 - 26% damage per time; the Heavy Axe stays the best weapon with or without it (C34: 526 against 381 of the Hand Axe; P24: 3,036 against 2,561) (sim/measures.py weapon_band: the member at the level, gear and forge of the checkpoint, each basic weapon, expected damage per unit of time of the best action against its boss (2026-10-09))</t>
+        </is>
+      </c>
       <c r="L29" t="inlineStr">
         <is>
           <t>open</t>
@@ -2161,6 +2271,16 @@
       <c r="O29" t="inlineStr">
         <is>
           <t>T02 Speed and weapons</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
     </row>
@@ -2319,6 +2439,11 @@
           <t>P03, P08, P10, P13, P14, P15</t>
         </is>
       </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>Tinker Squash delays the turn at 25 - 43% per hit with no resistance roll; the only brake is one bit: 14% of the story bosses and 56% of the postgame bosses are immune, the others have none (docs/FORMULAS.md 5c)</t>
+        </is>
+      </c>
       <c r="L32" t="inlineStr">
         <is>
           <t>open</t>
@@ -2327,6 +2452,16 @@
       <c r="O32" t="inlineStr">
         <is>
           <t>T07 Ailments, debuffs and locks</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>Give the immunity bit to the bosses that must not be locked, or lower the chance against bosses (L26, benign); target: no boss lockable, the skill still useful on common enemies</t>
         </is>
       </c>
     </row>
@@ -2428,6 +2563,11 @@
           <t>P03, P04, P07, P10, P14, P15</t>
         </is>
       </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Top single spell (tier 4) against tier 1 at their top levels: 2.5 times the power (1,300 against 520) for 2.6 times the TP (84 against 32) and a chant 34% slower (0.70 against 1.06); area tier 3 against tier 2: 1.4 times the power for twice the TP, 23% slower. Power per TP stays about equal (95%)</t>
+        </is>
+      </c>
       <c r="L34" t="inlineStr">
         <is>
           <t>open</t>
@@ -2436,6 +2576,16 @@
       <c r="O34" t="inlineStr">
         <is>
           <t>T04 Magic</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>partly true</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>To decide in T04: a faster chant for tier 4 (L12, benign)</t>
         </is>
       </c>
     </row>
@@ -2998,6 +3148,11 @@
           <t>P04, P07, P10, P13, P15, P18, P19</t>
         </is>
       </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>One story boss (C29a) and four postgame fights (P07, P13, P25, P47) stand on cells that forbid magic. The need for one grand sealbook is not seen in the model: a mage without any sealbook makes 172 - 191% of the Dark Lord late</t>
+        </is>
+      </c>
       <c r="L44" t="inlineStr">
         <is>
           <t>open</t>
@@ -3006,6 +3161,16 @@
       <c r="O44" t="inlineStr">
         <is>
           <t>T04 Magic</t>
+        </is>
+      </c>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>partly true</t>
+        </is>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>None for the sealbook; the five anti-magic fights keep their answer in items and dolls (techniques)</t>
         </is>
       </c>
     </row>
@@ -3112,6 +3277,11 @@
           <t>P01, P02, P03, P14, P15, P19</t>
         </is>
       </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>For the basic pieces at the end (P24 at 90): Heavy Axe 100% against Hand Axe 84%, Heavy Lance 100% against Lance 49%, Tachi 100% against Tantou 48% (sim/measures.py weapon_band: the member at the level, gear and forge of the checkpoint, each basic weapon, expected damage per unit of time of the best action against its boss (2026-10-09)). The unique one-handed weapons of the end game are not modelled</t>
+        </is>
+      </c>
       <c r="L46" t="inlineStr">
         <is>
           <t>open</t>
@@ -3120,6 +3290,16 @@
       <c r="O46" t="inlineStr">
         <is>
           <t>T02 Speed and weapons</t>
+        </is>
+      </c>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>None now; to look again with the unique pieces in T10</t>
         </is>
       </c>
     </row>
@@ -3169,6 +3349,11 @@
           <t>P01, P02, P03, P14, P15</t>
         </is>
       </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>A Mistress with a whip makes 39% (C34) and 12% (P24) of the damage per time of the Dark Lord; in the hands of a Papillon a whip gives 83 - 91% of a sword (sim/measures.py weapon_band: the member at the level, gear and forge of the checkpoint, each basic weapon, expected damage per unit of time of the best action against its boss (2026-10-09))</t>
+        </is>
+      </c>
       <c r="L47" t="inlineStr">
         <is>
           <t>open</t>
@@ -3177,6 +3362,16 @@
       <c r="O47" t="inlineStr">
         <is>
           <t>T02 Speed and weapons</t>
+        </is>
+      </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>Whip stats and swing (L14) and the power of the whip skills (L12), benign; target: the Mistress, a sub-attacker (docs/CLASS_IDENTITY.md), at half the Dark Lord or more</t>
         </is>
       </c>
     </row>
@@ -3226,6 +3421,11 @@
           <t>P01, P02, P03, P14, P15</t>
         </is>
       </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>As J06: 10 of the 13 bow skills refuse a gun</t>
+        </is>
+      </c>
       <c r="L48" t="inlineStr">
         <is>
           <t>open</t>
@@ -3234,6 +3434,16 @@
       <c r="O48" t="inlineStr">
         <is>
           <t>T02 Speed and weapons</t>
+        </is>
+      </c>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>As J06</t>
         </is>
       </c>
     </row>
@@ -3278,6 +3488,11 @@
           <t>P06</t>
         </is>
       </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>The plain attack falls from 15 - 70% of the best action at C18 to 0 - 27% at P24 (sim/measures.py weapon_band: the member at the level, gear and forge of the checkpoint, each basic weapon, expected damage per unit of time of the best action against its boss (2026-10-09))</t>
+        </is>
+      </c>
       <c r="L49" t="inlineStr">
         <is>
           <t>open</t>
@@ -3286,6 +3501,16 @@
       <c r="O49" t="inlineStr">
         <is>
           <t>T02 Speed and weapons</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>To decide: raise Double Attack, Triple Attack and Barrage (L12, benign), or accept plain attacks as a fallback</t>
         </is>
       </c>
     </row>
@@ -3330,6 +3555,11 @@
           <t>P10, P13</t>
         </is>
       </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>Dark Aura is on 21% of the enemies of level 60 and above (49 of 237) and on 13 of the 55 postgame bosses</t>
+        </is>
+      </c>
       <c r="L50" t="inlineStr">
         <is>
           <t>open</t>
@@ -3338,6 +3568,16 @@
       <c r="O50" t="inlineStr">
         <is>
           <t>T12 Common enemies and the pace of normal fights</t>
+        </is>
+      </c>
+      <c r="P50" t="inlineStr">
+        <is>
+          <t>partly true</t>
+        </is>
+      </c>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>To decide: fewer late carriers, or a lower value (L35 structural, L08 benign)</t>
         </is>
       </c>
     </row>
@@ -3382,6 +3622,11 @@
           <t>P04, P07, P10</t>
         </is>
       </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>A magic defence buff of +25% on the target cuts a spell by 11 - 15% (INT 150 / power 300 / RES 150: 375 to 319; INT 300 / power 900 / RES 300: 1,050 to 938): the power of the spell is not reduced by it (docs/FORMULAS.md 3)</t>
+        </is>
+      </c>
       <c r="L51" t="inlineStr">
         <is>
           <t>open</t>
@@ -3390,6 +3635,16 @@
       <c r="O51" t="inlineStr">
         <is>
           <t>T04 Magic</t>
+        </is>
+      </c>
+      <c r="P51" t="inlineStr">
+        <is>
+          <t>partly true</t>
+        </is>
+      </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>To decide in T04: larger values for the magic defence skills (L12)</t>
         </is>
       </c>
     </row>
@@ -3434,6 +3689,11 @@
           <t>P04, P07, P08, P10, P15, P19</t>
         </is>
       </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>With the forged gear of the model the party has elemental resistance 60 (Yuni 30) at 90 - 99; resistance 100 needs the full end-game enchanting of the guide (+15 a piece), where the +25 resistance skills are wasted, as the guide itself says</t>
+        </is>
+      </c>
       <c r="L52" t="inlineStr">
         <is>
           <t>open</t>
@@ -3442,6 +3702,16 @@
       <c r="O52" t="inlineStr">
         <is>
           <t>T07 Ailments, debuffs and locks</t>
+        </is>
+      </c>
+      <c r="P52" t="inlineStr">
+        <is>
+          <t>partly true</t>
+        </is>
+      </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>To decide in T10: cap or reduce the elemental resistance enchantments (L19), or leave it to the end game</t>
         </is>
       </c>
     </row>
@@ -3486,6 +3756,11 @@
           <t>P08, P10, P13</t>
         </is>
       </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>Postgame bosses: immune to freeze 91%, stun 93%, paralysis 87%, sleep 65%; instant death and petrification 100% of the 98 bosses; on the others a base 0.5 ailment lands 5 - 10% (median). Story bosses: about half immune, 30 - 50% on the others</t>
+        </is>
+      </c>
       <c r="L53" t="inlineStr">
         <is>
           <t>open</t>
@@ -3494,6 +3769,16 @@
       <c r="O53" t="inlineStr">
         <is>
           <t>T07 Ailments, debuffs and locks</t>
+        </is>
+      </c>
+      <c r="P53" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>Open some bosses to slow, sleep or silence (immunity bits L26, resistances L02, benign), with J31 in mind; target: every ailment skill has some boss it works on</t>
         </is>
       </c>
     </row>
@@ -3917,6 +4202,11 @@
           <t>P01, P02, P03, P08, P10, P12, P13, P15</t>
         </is>
       </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>Mesmerized (Magnificent Steps, 0.07) and Warning Shot (0.06) roll once per bearer with no immunity test: one bearer of each takes 13% of the enemy turns, three 33%, five 49% (EffectRules 259, 283)</t>
+        </is>
+      </c>
       <c r="L61" t="inlineStr">
         <is>
           <t>open</t>
@@ -3925,6 +4215,16 @@
       <c r="O61" t="inlineStr">
         <is>
           <t>T07 Ailments, debuffs and locks</t>
+        </is>
+      </c>
+      <c r="P61" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="Q61" t="inlineStr">
+        <is>
+          <t>Lower the values or let bosses resist them (L12; L26 if a bit applies), so that a stacked party cannot take a third of a boss's turns</t>
         </is>
       </c>
     </row>
@@ -3969,6 +4269,11 @@
           <t>P01, P02, P03, P04, P07, P10, P15</t>
         </is>
       </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>73% of the 64 damage techniques have a speed factor below 1 at their top level (median 0.90, range 0.40 - 1.16). The values of the first game are not in the data to compare</t>
+        </is>
+      </c>
       <c r="L62" t="inlineStr">
         <is>
           <t>open</t>
@@ -3977,6 +4282,16 @@
       <c r="O62" t="inlineStr">
         <is>
           <t>T02 Speed and weapons</t>
+        </is>
+      </c>
+      <c r="P62" t="inlineStr">
+        <is>
+          <t>partly true</t>
+        </is>
+      </c>
+      <c r="Q62" t="inlineStr">
+        <is>
+          <t>To look at skill by skill in T06 (L12 speed factor, benign)</t>
         </is>
       </c>
     </row>
@@ -7932,6 +8247,11 @@
           <t>P03, P12, P13</t>
         </is>
       </c>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>A random battle is short: 2.6 - 3.3 actions per member, 0.9 - 2.5 units of time (C07 to P24); the length is in the number of battles per level (own pace 25 - 35), which the decided curve cuts to 15 - 19</t>
+        </is>
+      </c>
       <c r="L136" t="inlineStr">
         <is>
           <t>open</t>
@@ -7950,6 +8270,16 @@
       <c r="O136" t="inlineStr">
         <is>
           <t>T12 Common enemies and the pace of normal fights</t>
+        </is>
+      </c>
+      <c r="P136" t="inlineStr">
+        <is>
+          <t>partly true</t>
+        </is>
+      </c>
+      <c r="Q136" t="inlineStr">
+        <is>
+          <t>Nothing beyond the decided curve (U01)</t>
         </is>
       </c>
     </row>
@@ -7994,6 +8324,11 @@
           <t>P03, P13</t>
         </is>
       </c>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>Enemies of random formations whose lowest physical resistance is 50 or more: 0% up to level 19, 5% (20 - 39), 20% (40 - 59), 30% (60 - 79), 77% (80 - 99); whose every element is 50 or more: 0 - 6% up to 79, 21% from 80. True late, false early</t>
+        </is>
+      </c>
       <c r="L137" t="inlineStr">
         <is>
           <t>open</t>
@@ -8012,6 +8347,16 @@
       <c r="O137" t="inlineStr">
         <is>
           <t>T12 Common enemies and the pace of normal fights</t>
+        </is>
+      </c>
+      <c r="P137" t="inlineStr">
+        <is>
+          <t>partly true</t>
+        </is>
+      </c>
+      <c r="Q137" t="inlineStr">
+        <is>
+          <t>To decide: lower the physical resistances of the common enemies from 80 (L02, benign)</t>
         </is>
       </c>
     </row>
@@ -8056,6 +8401,11 @@
           <t>Where enemy passives are stored (not read)</t>
         </is>
       </c>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t>The rates are data (passives of EnemyAttackData). Median of the enemies against the top of the party: Reprisal 0.25 against 0.18, Auto-Guard 0.30 against 0.12, Counter 0.15 against 0.12, Ecstasy 0.5 against 0.15; equal for Double and Triple Attack, Dark Aura and Knock Down</t>
+        </is>
+      </c>
       <c r="L138" t="inlineStr">
         <is>
           <t>open</t>
@@ -8074,6 +8424,16 @@
       <c r="O138" t="inlineStr">
         <is>
           <t>T12 Common enemies and the pace of normal fights</t>
+        </is>
+      </c>
+      <c r="P138" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="Q138" t="inlineStr">
+        <is>
+          <t>Bring the four above the party's top down to it (L08, benign), keeping the flavour of the enemies that show them</t>
         </is>
       </c>
     </row>
@@ -8180,6 +8540,11 @@
           <t>P08, P13</t>
         </is>
       </c>
+      <c r="J140" t="inlineStr">
+        <is>
+          <t>A random battle lasts 2.6 - 3.3 actions per member (C07 to P24, 40 battles each): a turn spent on an ailment is a third of a member's fight</t>
+        </is>
+      </c>
       <c r="L140" t="inlineStr">
         <is>
           <t>open</t>
@@ -8198,6 +8563,16 @@
       <c r="O140" t="inlineStr">
         <is>
           <t>T07 Ailments, debuffs and locks</t>
+        </is>
+      </c>
+      <c r="P140" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="Q140" t="inlineStr">
+        <is>
+          <t>To decide: accept (ailments are for bosses and dangerous groups) or raise their side effects</t>
         </is>
       </c>
     </row>
@@ -8242,6 +8617,11 @@
           <t>P03, P05</t>
         </is>
       </c>
+      <c r="J141" t="inlineStr">
+        <is>
+          <t>A DEF debuff of 10 - 20% adds 2 - 5% to the damage of a skill (the power of the skill multiplies; the debuff only lowers the defence term) (docs/FORMULAS.md 2)</t>
+        </is>
+      </c>
       <c r="L141" t="inlineStr">
         <is>
           <t>open</t>
@@ -8260,6 +8640,16 @@
       <c r="O141" t="inlineStr">
         <is>
           <t>T07 Ailments, debuffs and locks</t>
+        </is>
+      </c>
+      <c r="P141" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="Q141" t="inlineStr">
+        <is>
+          <t>Larger values for the DEF and ATK debuffs (dances, L12, benign); target: a debuff pays its turn back within its length</t>
         </is>
       </c>
     </row>
@@ -9589,6 +9979,11 @@
           <t>none</t>
         </is>
       </c>
+      <c r="J162" t="inlineStr">
+        <is>
+          <t>Too vague to test on its own; its verdict comes from R03 and R08 in the final pass</t>
+        </is>
+      </c>
       <c r="L162" t="inlineStr">
         <is>
           <t>open</t>
@@ -9607,6 +10002,16 @@
       <c r="O162" t="inlineStr">
         <is>
           <t>T12 Common enemies and the pace of normal fights</t>
+        </is>
+      </c>
+      <c r="P162" t="inlineStr">
+        <is>
+          <t>to measure</t>
+        </is>
+      </c>
+      <c r="Q162" t="inlineStr">
+        <is>
+          <t>None of its own</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: T11 data rows (J34, J13)
T11 data rows (J34, J13); plan updated: 44 of 162 rows with a verdict,
waiting for the decisions
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -1403,6 +1403,11 @@
           <t>P03</t>
         </is>
       </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>A mercenary (guest ally) acts by a script of the enemy kind: weighted random sets of attacks, 1 to 3 sets each, fixed stats per stage of its growth (107 records of 31 allies; docs/generated/BALANCE_BASELINE.md, Guest allies). It is data, but the game does not show it</t>
+        </is>
+      </c>
       <c r="L14" t="inlineStr">
         <is>
           <t>open</t>
@@ -1411,6 +1416,16 @@
       <c r="O14" t="inlineStr">
         <is>
           <t>T11 Information</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>partly true</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>To decide: describe what each mercenary does in its in-game text (L20, written in the voice of the game), in the Balance variant</t>
         </is>
       </c>
     </row>
@@ -2630,6 +2645,11 @@
           <t>P03, P14, P15, P17</t>
         </is>
       </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Berserk lowers the DEF of its user by 11 - 25% (effect 28, -0.11 to -0.25 by level) for 4 - 8 turns, while it raises her attack by 20 - 50% (effect 26); not to zero</t>
+        </is>
+      </c>
       <c r="L35" t="inlineStr">
         <is>
           <t>open</t>
@@ -2638,6 +2658,16 @@
       <c r="O35" t="inlineStr">
         <is>
           <t>T11 Information</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>None; the skill text already gives the figures (QoL)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: passive HP and TP regeneration ticks each turn
passive HP and TP regeneration ticks each turn; step 2 decisions

- Auto-Recovery, Auto-Refresh and the HP Regen of enemies (passives 246,
247) never acted in the simulator - forge share recalibrated to 0.5
(anchors 5/6, N06 known limit); figures of 13 verdicts remeasured, no
verdict changed - decided: J09 no change, J08 closed, J03/J10 TP cost of
22 skills a little lower, J05/F26 Auto-Refresh a little higher
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -586,7 +586,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Same character late (Yae, P24 at 90): a Kukri acts every 0.21, a Heavy Axe every 0.40 (1.9 actions per heavy one); yet the heavy weapon gives the most damage per time at every checkpoint measured (Heavy Axe 100%, Kukri 29 - 41%) (sim/measures.py weapon_band: the member at the level, gear and forge of the checkpoint, each basic weapon, expected damage per unit of time of the best action against its boss (2026-10-09)). Survival under the order of turns is not in this measure</t>
+          <t>Same character late (Yae, P24 at 90): a Kukri acts every 0.26, a Heavy Axe every 0.48 (1.8 actions per heavy one); yet the heavy weapon gives the most damage per time at every checkpoint measured (Heavy Axe 100%, Kukri 28 - 40%). Survival under the order of turns is not in this measure (remeasured 2026-10-09 after the fix of passive regeneration and the forge share 0.5)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -658,7 +658,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>With the top spells of the Witch (reference plan, atwiki page 136) a mage makes 172 - 191% of the damage per time of the Dark Lord at C38, P24 and P49 (boss resistances counted), and completes 88 - 97% of her chants against those bosses (sim/measures.py weapon_band: the member at the level, gear and forge of the checkpoint, each basic weapon, expected damage per unit of time of the best action against its boss (2026-10-09); chants: 20 boss fights each)</t>
+          <t>With the top spells of the Witch (reference plan, atwiki page 136) a mage makes 202 - 213% of the damage per time of the Dark Lord at C38, P24 and P49 (boss resistances counted), and completes 84 - 98% of her chants against those bosses (remeasured 2026-10-09 after the fix of passive regeneration and the forge share 0.5)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -753,6 +753,11 @@
           <t>TP cost per level (L12, benign) so that power per TP at the top level is at least 85% of level 1, or the level buys something stated; the skill text already shows each level (QoL)</t>
         </is>
       </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>2026-10-09: a little: the TP cost of 22 damage skills lowered toward 70% of the power per TP of level 1, never by more than a quarter (balance_changes.xlsx C rows)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -859,7 +864,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Without a Maid (a healer in her place): in the middle of the story little changes (Rousset Royal Villa at 27: 18.2 of 20 battles against 20; boss C18 won 100% both), late it collapses (Actim Castle at 50: 4.9 of 20 battles against 13.6; the weakened Queen C34 won 0% against 100%) (sim/measures.py expedition, 30 runs of up to 20 random battles, kit of 3 of each shop item (2026-10-09); the bosses 40 battles each)</t>
+          <t>Without a Maid (a healer in her place): in the middle of the story little changes (Rousset Royal Villa at 27: 17.2 of 20 battles against 20; boss C18 won 100% both), late it collapses (Actim Castle at 50: 5.9 of 20 battles against 13.0; the weakened Queen C34 won 0% against 100%) (remeasured 2026-10-09 after the fix of passive regeneration and the forge share 0.5)</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -880,6 +885,11 @@
       <c r="Q6" t="inlineStr">
         <is>
           <t>TP outside the Maid line: values of Auto-Refresh and TP recovery skills and the price of TP items (L12, L19, benign), with J03; target: Actim without a Maid 10 or more battles and the Queen won</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>2026-10-09: a little; TP stays the mark of the Maid: Auto-Refresh and Mini Auto-Refresh raised slightly (balance_changes.xlsx R rows); Actim stays hard without a Maid by design</t>
         </is>
       </c>
     </row>
@@ -1003,7 +1013,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>For damage two-handed weapons lead at every checkpoint measured (C18, C34, P24): Heavy Axe, Claymore, Heavy Lance, Tachi and Long Bow give 100% or close; their one-handed counterparts 47 - 84% (sim/measures.py weapon_band: the member at the level, gear and forge of the checkpoint, each basic weapon, expected damage per unit of time of the best action against its boss (2026-10-09)). The shield they give up (DEF, the guard skills) is not counted</t>
+          <t>For damage two-handed weapons lead at every checkpoint measured (C18, C34, P24): Heavy Axe, Claymore, Heavy Lance, Tachi and Long Bow give 100% or close; their one-handed counterparts 45 - 87%. The shield they give up (DEF, the guard skills) is not counted (remeasured 2026-10-09 after the fix of passive regeneration and the forge share 0.5)</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1075,7 +1085,12 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>not a problem</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Overstated: the party is not empty after 3 or 4 battles (see Vanilla_Result); closed by the user 2026-10-09</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
@@ -1091,6 +1106,11 @@
       <c r="Q9" t="inlineStr">
         <is>
           <t>No change proposed; the TP rows of T03 (J03, J10) lower the burn further</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>2026-10-09: close without a change of its own (overstated); J03 and J10 lower the burn</t>
         </is>
       </c>
     </row>
@@ -1142,7 +1162,12 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>not a problem</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>The user keeps it as it is (2026-10-09)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
@@ -1158,6 +1183,11 @@
       <c r="Q10" t="inlineStr">
         <is>
           <t>Lower the AGI of the agile enemies of st00 - st02 (L01, benign) so that the lowest chance of a front-line member is at least 70% and the median 80%; keep the hardest of them a little harder</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>2026-10-09: no change (the user keeps the early misses)</t>
         </is>
       </c>
     </row>
@@ -1227,6 +1257,11 @@
           <t>With J03: TP cost per level of the skills that are raised early (L12, benign)</t>
         </is>
       </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>2026-10-09: as J03, a little</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1276,7 +1311,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Mage over Dark Lord, damage per time: 41% (C07), 98% (C13), 189% (C18), 333% (C25), 309% (C34), 191% (C38), 172 - 174% (P24, P49): a peak in the middle and a drop after it, but no cliff (sim/measures.py weapon_band: the member at the level, gear and forge of the checkpoint, each basic weapon, expected damage per unit of time of the best action against its boss (2026-10-09))</t>
+          <t>Mage over Dark Lord, damage per time: 41% (C07), 101% (C13), 195% (C18), 306% (C25), 286% (C34), 213% (C38), 202 - 204% (P24, P49): a peak in the middle and a lower level after it, but no cliff (remeasured 2026-10-09 after the fix of passive regeneration and the forge share 0.5)</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1343,7 +1378,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Yae from Fighter at 14 with a Longsword to Berserker at 15 with a Claymore: damage per time 2.3 times higher (69 to 156), wait 0.74 to 0.76 (+3%), DEF 78 to 85 (sim/measures.py weapon_band: the member at the level, gear and forge of the checkpoint, each basic weapon, expected damage per unit of time of the best action against its boss (2026-10-09))</t>
+          <t>Yae from Fighter at 14 with a Longsword to Berserker at 15 with a Claymore: damage per time 2.3 times higher (67 to 151), wait 0.77 to 0.79 (+3%), DEF 78 to 85 (remeasured 2026-10-09 after the fix of passive regeneration and the forge share 0.5)</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -1482,7 +1517,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>A mage completes 85 - 98% of the chants she starts against the bosses C18, C25, C34, C38, P24, P28 and P49; 0 - 0.7 chants broken per fight (20 fights each)</t>
+          <t>A mage completes 82 - 98% of the chants she starts against the bosses C18, C25, C34, C38, P24, P28 and P49; 0 - 1.1 chants broken per fight (20 fights each) (remeasured 2026-10-09 after the fix of passive regeneration and the forge share 0.5)</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -2280,7 +2315,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>Lightning March adds 5 - 26% damage per time; the Heavy Axe stays the best weapon with or without it (C34: 526 against 381 of the Hand Axe; P24: 3,036 against 2,561) (sim/measures.py weapon_band: the member at the level, gear and forge of the checkpoint, each basic weapon, expected damage per unit of time of the best action against its boss (2026-10-09))</t>
+          <t>Lightning March adds 4 - 22% damage per time; the Heavy Axe stays the best weapon without it (C34: 504 against 349 of the Hand Axe; P24: 2,584 against 2,254) (remeasured 2026-10-09 after the fix of passive regeneration and the forge share 0.5)</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
@@ -3319,7 +3354,7 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>For the basic pieces at the end (P24 at 90): Heavy Axe 100% against Hand Axe 84%, Heavy Lance 100% against Lance 49%, Tachi 100% against Tantou 48% (sim/measures.py weapon_band: the member at the level, gear and forge of the checkpoint, each basic weapon, expected damage per unit of time of the best action against its boss (2026-10-09)). The unique one-handed weapons of the end game are not modelled</t>
+          <t>For the basic pieces at the end (P24 at 90): Heavy Axe 100% against Hand Axe 87%, Heavy Lance 100% against Lance 51%, Tachi 100% against Tantou 45%. The unique one-handed weapons of the end game are not modelled (remeasured 2026-10-09 after the fix of passive regeneration and the forge share 0.5)</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
@@ -3391,7 +3426,7 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>A Mistress with a whip makes 39% (C34) and 12% (P24) of the damage per time of the Dark Lord; in the hands of a Papillon a whip gives 83 - 91% of a sword (sim/measures.py weapon_band: the member at the level, gear and forge of the checkpoint, each basic weapon, expected damage per unit of time of the best action against its boss (2026-10-09))</t>
+          <t>A Mistress with a whip makes 40% (C34) and 10% (P24) of the damage per time of the Dark Lord; in the hands of a Papillon a whip gives 83 - 91% of a sword (remeasured 2026-10-09 after the fix of passive regeneration and the forge share 0.5)</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
@@ -3530,7 +3565,7 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>The plain attack falls from 15 - 70% of the best action at C18 to 0 - 27% at P24 (sim/measures.py weapon_band: the member at the level, gear and forge of the checkpoint, each basic weapon, expected damage per unit of time of the best action against its boss (2026-10-09))</t>
+          <t>The plain attack is 18 - 100% of the best action at C18 (about 45% in the middle) and 0 - 24% at P24 (remeasured 2026-10-09 after the fix of passive regeneration and the forge share 0.5)</t>
         </is>
       </c>
       <c r="L49" t="inlineStr">
@@ -4460,7 +4495,7 @@
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>A second Maid matters late: Actim Castle at 50, 13.6 of 20 battles with one Maid, 17.2 with two (TP after 8 battles 18% against 40%); in the middle of the story one Maid already reaches 20 of 20 (sim/measures.py expedition, 30 runs of up to 20 random battles, kit of 3 of each shop item (2026-10-09))</t>
+          <t>A second Maid matters late: Actim Castle at 50, 13.0 of 20 battles with one Maid, 15.7 with two (TP after 8 battles 20% against 46%); in the middle of the story one Maid already reaches 20 of 20 (remeasured 2026-10-09 after the fix of passive regeneration and the forge share 0.5)</t>
         </is>
       </c>
       <c r="L64" t="inlineStr">
@@ -4481,6 +4516,11 @@
       <c r="Q64" t="inlineStr">
         <is>
           <t>As J05: lower the TP burn (J03) and add TP outside the Maid, so one Maid is enough late</t>
+        </is>
+      </c>
+      <c r="R64" t="inlineStr">
+        <is>
+          <t>2026-10-09: as J05</t>
         </is>
       </c>
     </row>
@@ -10128,7 +10168,7 @@
       </c>
       <c r="J163" t="inlineStr">
         <is>
-          <t>In the same slot, Lizerietta as a Doll Master (levels 18 - 27, bosses C13, C16, C18) makes 15 - 24% of the party damage with her dolls against 17 - 36% as a Trickster (45 - 90% of it), and a fight lasts up to 26% longer; as a Soul Summoner (C25 at 36, C34 at 50) 8 - 10% against 15 - 16% as a Papillon (30 battles each)</t>
+          <t>In the same slot, Lizerietta as a Doll Master (levels 18 - 27, bosses C13, C16, C18) makes 15 - 23% of the party damage with her dolls against 17 - 37% as a Trickster (49 - 88% of it), and a fight lasts up to 19% longer; as a Soul Summoner (C25 at 36, C34 at 50) about 10 - 11% against 16 - 18% as a Papillon (61%) (remeasured 2026-10-09 after the fix of passive regeneration and the forge share 0.5)</t>
         </is>
       </c>
       <c r="L163" t="inlineStr">

</xml_diff>

<commit_message>
data: the doll changes decided
the doll changes decided (U02, J18, F71, F77): faster cast, +2 turns,
faster actions, power x2 / x1.5
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -1778,6 +1778,11 @@
           <t>None; the weakness of the line is U02</t>
         </is>
       </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>2026-10-09: dolls last two turns more (D rows)</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -6863,6 +6868,11 @@
           <t>T06 Skills</t>
         </is>
       </c>
+      <c r="R109" t="inlineStr">
+        <is>
+          <t>2026-10-09: Oracles x2 power with the doll changes (D rows)</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -7175,6 +7185,11 @@
           <t>T06 Skills</t>
         </is>
       </c>
+      <c r="R115" t="inlineStr">
+        <is>
+          <t>2026-10-09: Musiy x1.5 power with the doll changes (D rows)</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -8858,7 +8873,7 @@
       </c>
       <c r="L143" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>not a problem</t>
         </is>
       </c>
       <c r="M143" t="inlineStr">
@@ -8884,6 +8899,11 @@
       <c r="Q143" t="inlineStr">
         <is>
           <t>None on its speed</t>
+        </is>
+      </c>
+      <c r="R143" t="inlineStr">
+        <is>
+          <t>2026-10-09: no change (summons are not of the doll line; they already act like the slowest member)</t>
         </is>
       </c>
     </row>
@@ -10168,7 +10188,7 @@
       </c>
       <c r="J163" t="inlineStr">
         <is>
-          <t>In the same slot, Lizerietta as a Doll Master (levels 18 - 27, bosses C13, C16, C18) makes 15 - 23% of the party damage with her dolls against 17 - 37% as a Trickster (49 - 88% of it), and a fight lasts up to 19% longer; as a Soul Summoner (C25 at 36, C34 at 50) about 10 - 11% against 16 - 18% as a Papillon (61%) (remeasured 2026-10-09 after the fix of passive regeneration and the forge share 0.5)</t>
+          <t>In the same slot, the doll line makes 29% of the party damage share of the Fighter and Scout lines on average (Doll Master 40 - 54%, Soul Summoner 7 - 22%; bosses C13, C18, C25, C34, C38, 25 battles each; sim/measures.py slot_share, with a Soul Summoner role, two dolls kept with Double Puppet and Mercidarian first). The other Spieler line (Trickster, Papillon) sits at about two thirds of that band</t>
         </is>
       </c>
       <c r="L163" t="inlineStr">
@@ -10199,6 +10219,11 @@
       <c r="Q163" t="inlineStr">
         <is>
           <t>Data, benign (L12, L10): the power, chances and spell power of the hidden doll actions, the life of a doll (effect 147), the TP and speed of a cast, Doll Mastery, the growth row; target: the line within 90% of the other Spieler line in the same slot, keeping what is its own (autonomous allies that work in anti-magic zones, healing through Catalina)</t>
+        </is>
+      </c>
+      <c r="R163" t="inlineStr">
+        <is>
+          <t>2026-10-09: the doll line to the band of the Fighter and Scout lines (target 100%): cast +0.2, life +2, action speed +0.2, power x2 (Doll Master dolls) and x1.5 (Soul Summoner dolls); balance_changes.xlsx D rows</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: T07 decided: bosses immune to turn delay, open to slow/silence
T07 decided: bosses immune to turn delay, open to slow/silence (sleep in
the story), turn skipping capped, debuffs x1.5, ailment spells +20%
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -2594,6 +2594,11 @@
           <t>Give the immunity bit to the bosses that must not be locked, or lower the chance against bosses (L26, benign); target: no boss lockable, the skill still useful on common enemies</t>
         </is>
       </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>2026-10-09: every story and postgame boss immune to turn delay (A rows)</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -3919,6 +3924,11 @@
           <t>To decide in T10: cap or reduce the elemental resistance enchantments (L19), or leave it to the end game</t>
         </is>
       </c>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>2026-10-09: to T10 (the enchantments of the forge)</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -3986,6 +3996,11 @@
           <t>Open some bosses to slow, sleep or silence (immunity bits L26, resistances L02, benign), with J31 in mind; target: every ailment skill has some boss it works on</t>
         </is>
       </c>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>2026-10-09: bosses open to slow and silence unless superbosses, to sleep in the story (A rows)</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -4462,6 +4477,11 @@
           <t>Lower the values or let bosses resist them (L12; L26 if a bit applies), so that a stacked party cannot take a third of a boss's turns</t>
         </is>
       </c>
+      <c r="R61" t="inlineStr">
+        <is>
+          <t>2026-10-09: Magnificent Steps 2 - 4%, Warning Shot 1 - 3%: three of each take 19% of the enemy turns (A rows)</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -8875,6 +8895,11 @@
           <t>To decide: accept (ailments are for bosses and dangerous groups) or raise their side effects</t>
         </is>
       </c>
+      <c r="R140" t="inlineStr">
+        <is>
+          <t>2026-10-09: ailment spells +20% chance, capped at 95% (90% death and petrification) (A rows)</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -8950,6 +8975,11 @@
       <c r="Q141" t="inlineStr">
         <is>
           <t>Larger values for the DEF and ATK debuffs (dances, L12, benign); target: a debuff pays its turn back within its length</t>
+        </is>
+      </c>
+      <c r="R141" t="inlineStr">
+        <is>
+          <t>2026-10-09: debuffs x1.5 (A rows)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: T12 decided: late common enemies less resistant
T12 decided: late common enemies less resistant, enemy passives capped
at the party top, Dark Aura of common enemies 4 stats
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -3785,6 +3785,11 @@
           <t>To decide: fewer late carriers, or a lower value (L35 structural, L08 benign)</t>
         </is>
       </c>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>2026-10-09: Dark Aura of common enemies 4 stats instead of 6; bosses keep it (E rows)</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -8602,6 +8607,11 @@
           <t>Nothing beyond the decided curve (U01)</t>
         </is>
       </c>
+      <c r="R136" t="inlineStr">
+        <is>
+          <t>2026-10-09: covered by the decided EXP curve</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -8679,6 +8689,11 @@
           <t>To decide: lower the physical resistances of the common enemies from 80 (L02, benign)</t>
         </is>
       </c>
+      <c r="R137" t="inlineStr">
+        <is>
+          <t>2026-10-09: common enemies of level 80+ lose 10 points of physical resistance (E rows)</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -8756,6 +8771,11 @@
           <t>Bring the four above the party's top down to it (L08, benign), keeping the flavour of the enemies that show them</t>
         </is>
       </c>
+      <c r="R138" t="inlineStr">
+        <is>
+          <t>2026-10-09: Reprisal, Auto-Guard, Counter and Ecstasy of enemies capped at the party top (E rows)</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -10357,6 +10377,11 @@
       <c r="Q162" t="inlineStr">
         <is>
           <t>None of its own</t>
+        </is>
+      </c>
+      <c r="R162" t="inlineStr">
+        <is>
+          <t>2026-10-09: judged in the final pass (R03, R08)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
exe: the catch-up factors B4 and the crown rule written into both
the catch-up factors B4 and the crown rule written into both program
files, installed with the Balance variant

The twelve rows tested on 2026-10-05 become the set balance of
ExePatches. exe_patch.py writes the shop file and the unwrapped file
together or neither, keeps a vanilla copy of each, and the formula
readers read the vanilla copy. install_variant.py balance installs the
set; qol puts the vanilla files back. The name of enchantment 270 is
worded for the variant. The kept EXP curve (L11) is recorded as not
built.
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -12167,7 +12167,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>test1</t>
+          <t>balance</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -12210,7 +12210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>test1</t>
+          <t>balance</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -12253,7 +12253,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>test1</t>
+          <t>balance</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -12296,7 +12296,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>test1</t>
+          <t>balance</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -12339,7 +12339,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>test1</t>
+          <t>balance</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -12376,7 +12376,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>test1</t>
+          <t>balance</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -12419,7 +12419,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>test1</t>
+          <t>balance</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -12462,7 +12462,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>test1</t>
+          <t>balance</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -12505,7 +12505,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>test1</t>
+          <t>balance</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -12542,7 +12542,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>test1</t>
+          <t>balance</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -12579,7 +12579,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>test1</t>
+          <t>balance</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -12616,7 +12616,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>test1</t>
+          <t>balance</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -12645,10 +12645,11 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>VA: address of the first byte changed. Old_Hex must be found there in the program before anything is written, in both copies of the executable.</t>
+          <t>VA: address of the first byte changed. Old_Hex must be found there before anything is written, in both program files of the game folder (DT22_en.exe and DT22_en_unwrapped.exe): the set is written into both or into neither (tools/exe_patch.py).</t>
         </is>
       </c>
     </row>
@@ -12662,14 +12663,14 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>The step of 59 to 68 levels stays at 1 point: its instruction is an "inc", with no byte that holds the amount. Giving it 2 means rewriting the end of the function, which the test does not do.</t>
+          <t>The step of 59 to 68 levels stays at 1 point (accepted by the user, 2026-10-05): its instruction is an "inc", with no byte that holds the amount. Giving it 2 means rewriting the end of the function. With the other four steps one point higher the cheapest crown no longer uses that step (docs/generated/CATCH_UP_OPTIONS.md, rule "One more point, lowest step kept").</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Factors with the piece of enchantment 270 (X06 to X08) are a proposal: the decision of 2026-10-05 fixed only the factors without the piece.</t>
+          <t>Factors with the piece of enchantment 270 (X06 to X08: 1.5, 4, 6) and the last band at 10 with or without the piece: accepted by the user on 2026-10-05, after the test in the game. The name of the enchantment in the Balance variant states them (balance_enchant_text.xlsx).</t>
         </is>
       </c>
     </row>
@@ -22770,7 +22771,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -22844,12 +22845,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Ten levels sooner</t>
+          <t>One more point, lowest step kept</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>88:5, 79:4, 69:3, 59:2, 49:1</t>
+          <t>98:6, 89:5, 79:4, 69:3, 59:1</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -22857,19 +22858,19 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Every step asks for ten levels fewer (five bytes)</t>
+          <t>What the set balance of ExePatches writes: four bytes; the step of 59 levels is an "inc" and keeps its point</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Ten levels sooner</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>88:6, 79:5, 69:4, 59:3, 49:2</t>
+          <t>88:5, 79:4, 69:3, 59:2, 49:1</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -22877,19 +22878,19 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>One point more and ten levels sooner (ten bytes)</t>
+          <t>Every step asks for ten levels fewer (five bytes)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Double points</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>98:10, 89:8, 79:6, 69:4, 59:2</t>
+          <t>88:6, 79:5, 69:4, 59:3, 49:2</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -22897,12 +22898,33 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
+          <t>One point more and ten levels sooner (ten bytes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Double points</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>98:10, 89:8, 79:6, 69:4, 59:2</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>50</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
           <t>Every step gives twice the points (five bytes)</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
+    <row r="8"/>
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>Steps: levels given up by the reset : points added to every stat. The program compares "levels given up" with a byte and adds a byte.</t>
         </is>

</xml_diff>

<commit_message>
balance: catch-up: the option B4 without the kept curve
catch-up: the option B4 without the kept curve, as installed, measured
beside the others
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -12645,7 +12645,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
@@ -22503,7 +22502,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -22702,7 +22701,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Kept + B4</t>
+          <t>B4</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -22715,46 +22714,69 @@
           <t>0.85, 0.9, 1, 1.25, 3, 5, 10</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>9,1, 15,0.954, 30,0.80, 50,0.75, 70,0.70, 99,0.60</t>
-        </is>
-      </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Kept curve; as B2, and 1.25 already from 1 level below the enemy</t>
+          <t>What is installed since 2026-10-11: the factors by gap of B4 in the program, the EXP of a level as in vanilla</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>Kept + B4</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>gap</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>0.85, 0.9, 1, 1.25, 3, 5, 10</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>9,1, 15,0.954, 30,0.80, 50,0.75, 70,0.70, 99,0.60</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Kept curve; as B2, and 1.25 already from 1 level below the enemy</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>Kept + D</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>gap</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>0.85, 0.9, 1, 1.5, 3, 5, 10</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>9,1, 15,0.954, 30,0.80, 50,0.75, 70,0.70, 99,0.60</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>Kept curve; 1.5 from 1 level below the enemy, then 3, 5 and 10</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
+    <row r="12"/>
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>Values of a gap option: the factor for a member 10 or more levels above the enemy, 5 to 9 above, 0 to 4 above, 1 to 4 below, 5 to 9 below, 10 to 19 below, 20 or more below. Each must be a float the program already holds.</t>
         </is>
@@ -22922,7 +22944,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
balance: what it takes read and corrected
what it takes read and corrected (FORMULAS 12.16, enemy_data), and a
short talk of Euthys says it in the game

A steal that succeeds runs the draw of the drops without its "nothing",
once per enemy, only on an enemy with bit 15 of its flags; the field
read so far as "steal" was the first equipment slot. The weights raised
for the seven rare pieces raise their steal by the same share (row F90).
Talk_Scenario27, two boxes, built and installed.
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -9528,7 +9528,7 @@
       </c>
       <c r="J128" t="inlineStr">
         <is>
-          <t>The piece of a postgame boss is certain (drop chance 100, one slot of weight 100). A fixed piece of a common enemy falls 2 to 4.5% of the time, of a very powerful enemy 10 to 50%; seven pieces of six common enemies fall under 2% (0.8 to 1.5%). What is stolen and how often is another rule (FORMULAS 12.16)</t>
+          <t>The piece of a postgame boss is certain (drop chance 100, one slot of weight 100). A fixed piece of a common enemy falls 2 to 4.5% of the time, of a very powerful enemy 10 to 50%; seven pieces of six common enemies fall under 2% (0.8 to 1.5%). A steal that succeeds draws among the drops of the enemy without the "nothing" of the draw, once per enemy (FORMULAS 12.16): the Chief's Special of Garasha comes out of 1.8% of them; 135 enemies cannot be robbed, the bosses and, among the common ones, Odin, Myrddin, Asmodeus and Carmilla</t>
         </is>
       </c>
       <c r="L128" t="inlineStr">
@@ -9538,7 +9538,7 @@
       </c>
       <c r="N128" t="inlineStr">
         <is>
-          <t>Read on 2026-10-11 (scratch/drops_reading.md, checked against 0x558517 - 0x5586fa): rows P011 - P023 and P025 of balance_changes.xlsx dropped, they changed the count of slots of drops that are certain or usual. Rows P024, P079 - P084 raise the seven pieces under 2% to 2%.</t>
+          <t>Read on 2026-10-11 (scratch/drops_reading.md, checked against 0x558517 - 0x5586fa): rows P011 - P023 and P025 of balance_changes.xlsx dropped, they changed the count of slots of drops that are certain or usual. Rows P024, P079 - P084 raise the seven pieces under 2% to 2%. The weight of a slot is the same word for the drop and for the steal (scratch/steal_reading.md, checked on 2026-10-11): with the rows the Chief's Special comes out of 4.7% of the steals that succeed.</t>
         </is>
       </c>
       <c r="O128" t="inlineStr">

</xml_diff>

<commit_message>
data: two rows that still cited the kept curve carry the figures of B4
two rows that still cited the kept curve carry the figures of B4 alone;
the worth of the skills replayed on the current variant
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -9749,12 +9749,12 @@
       </c>
       <c r="Q131" t="inlineStr">
         <is>
-          <t>Decided: B4 brings it to 79 battles; no other change</t>
+          <t>Decided: B4 alone brings a member from level 1 to within four levels of a party of level 70 in 107 battles (519 in vanilla; docs/generated/CATCH_UP_OPTIONS.md, option B4); no other change</t>
         </is>
       </c>
       <c r="R131" t="inlineStr">
         <is>
-          <t>2026-10-05: B4</t>
+          <t>2026-10-05: B4; 2026-10-11: B4 alone, installed</t>
         </is>
       </c>
     </row>
@@ -10109,12 +10109,12 @@
       </c>
       <c r="Q136" t="inlineStr">
         <is>
-          <t>Nothing beyond the decided curve (U01)</t>
+          <t>Nothing beyond the factors B4 (U01): a level costs a party on level 19 - 26 battles instead of 25 - 35 (levels 30 - 70); the kept curve is not built (the user, 2026-10-11)</t>
         </is>
       </c>
       <c r="R136" t="inlineStr">
         <is>
-          <t>2026-10-09: covered by the decided EXP curve</t>
+          <t>2026-10-09: covered by the decided EXP curve; 2026-10-11: covered by B4 alone</t>
         </is>
       </c>
     </row>
@@ -22436,7 +22436,6 @@
         </is>
       </c>
     </row>
-    <row r="41"/>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
data: 104 rows closed on their figures after the review
104 rows closed on their figures after the review (70 closed, 72 not a
problem, 12 out of the balance, 8 open)
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -748,9 +748,14 @@
           <t>84 skills deal damage; 67 give less power per TP at their top level than at level 1 (median 66%), 19 below half: Sharp Stab 20%, Aura Eliminate 28%, Raging Smash 29%, Backward Swing 35%, Gust Thrust 37%, the three stings 38%, Soul Drain 38%, Geo Break 39%</t>
         </is>
       </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>C001 - C168, the TP cost of 22 damage skills, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows)</t>
+        </is>
+      </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -907,9 +912,14 @@
           <t>Without a Maid (a healer in her place): in the middle of the story little changes (Rousset Royal Villa at 27: 17.2 of 20 battles against 20; boss C18 won 100% both), late it collapses (Actim Castle at 50: 5.9 of 20 battles against 13.0; the weakened Queen C34 won 0% against 100%) (remeasured 2026-10-09 after the fix of passive regeneration and the forge share 0.5)</t>
         </is>
       </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>R rows, Auto-Refresh 3 - 9 to 4 - 11 TP per turn, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); every role spends 15% of its TP on an ally under 15%</t>
+        </is>
+      </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -984,9 +994,14 @@
           <t>3 of the 13 bow skills accept a gun (Chain Spike, Guided Shot, Poison Shot). The 7 guns are unique pieces with ranks from 1.4 (Psychogun) to 2.9 (Wave Motion Gun, the slowest rank of the game)</t>
         </is>
       </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>W rows, four bow skills open to guns, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); shooter within the band at the four stages (0.85, 0.89, 0.88, 1.09; CLASS_STAGES.md)</t>
+        </is>
+      </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
@@ -1061,9 +1076,14 @@
           <t>For damage two-handed weapons lead at every checkpoint measured (C18, C34, P24): Heavy Axe, Claymore, Heavy Lance, Tachi and Long Bow give 100% or close; their one-handed counterparts 45 - 87%. The shield they give up (DEF, the guard skills) is not counted (remeasured 2026-10-09 after the fix of passive regeneration and the forge share 0.5)</t>
         </is>
       </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>W rows, two-handed base ATK -10%, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows)</t>
+        </is>
+      </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
@@ -1287,9 +1307,14 @@
           <t>At levels 5 - 15 a skill at its level costs 9 - 48% of its user's TP (Danger Shoot 48%, Resurrect 31%, Checkmate 30%); raising it early multiplies the cost: War Cry 7 to 11, Heal 3 to 10 points from level 1 to 4</t>
         </is>
       </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>as J03</t>
+        </is>
+      </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
@@ -1366,7 +1391,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>not a problem</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
@@ -1595,9 +1620,14 @@
           <t>A mage completes 82 - 98% of the chants she starts against the bosses C18, C25, C34, C38, P24, P28 and P49; 0 - 1.1 chants broken per fight (20 fights each) (remeasured 2026-10-09 after the fix of passive regeneration and the forge share 0.5)</t>
         </is>
       </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>M rows, top single spells chant at 0.85, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows)</t>
+        </is>
+      </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
@@ -1863,9 +1893,14 @@
           <t>A doll is born with 9,999 HP and ends by its count of turns (docs/FORMULAS.md 11.1): an area attack does not end it</t>
         </is>
       </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>D rows, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); soul summoner within the band at the four stages (1.12, 0.98, 0.87, 1.02; CLASS_STAGES.md)</t>
+        </is>
+      </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -2258,9 +2293,14 @@
           <t>P03, P04, P07, P10, P13, P14, P15</t>
         </is>
       </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>T066 - T075, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); Sage wins 12% under the median support at the advanced stage and 2% late, within the band (CLASS_STAGES.md)</t>
+        </is>
+      </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
@@ -2407,9 +2447,14 @@
           <t>P03, P04, P07, P10, P12, P13, P14, P15</t>
         </is>
       </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>Q001 - Q015, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); Magical Princess 1.06 advanced, 1.01 late, within the band (CLASS_STAGES.md)</t>
+        </is>
+      </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
@@ -2474,9 +2519,14 @@
           <t>P03, P04, P07, P10, P13, P14, P15, P17</t>
         </is>
       </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>T041 - T050, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); Treasure Hunter 1.21 advanced (slow), 1.00 late; the user, 2026-10-11: what is left is not a problem</t>
+        </is>
+      </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="O27" t="inlineStr">
@@ -2546,9 +2596,14 @@
           <t>P03, P04, P07, P10, P14, P15</t>
         </is>
       </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>K001 - K025 and W045 (Tantou forge rate x2), built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); Kunoichi 1.08 advanced, 1.01 late, within the band (CLASS_STAGES.md)</t>
+        </is>
+      </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="O28" t="inlineStr">
@@ -2695,9 +2750,14 @@
           <t>P01, P02, P03, P14, P15</t>
         </is>
       </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>T051 - T065, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); Mistress 0.95 advanced, 1.02 late, within the band (CLASS_STAGES.md)</t>
+        </is>
+      </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
@@ -2767,9 +2827,14 @@
           <t>Outcome tables (executable, docs/generated/BALANCE_BASELINE.md Random moves): Roulette Circus 10% heals a random enemy fully and 10% does nothing; Magic Box 10% kills its user for certain and 10% hits her with a double hit; Showtime 10.5% stuns the whole party for certain; Heaven or Hell deals 10% of the target max HP capped at 222, or heals it</t>
         </is>
       </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>Y001 - Y011 (Danger Shoot +0.10, from 20 TP) and W046 (Dagger 20 ATK), built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); Spieler 1.11 - 1.12 at the base stage, Trickster 1.08 - 1.13, within the band (CLASS_STAGES.md)</t>
+        </is>
+      </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
@@ -2844,9 +2909,14 @@
           <t>Tinker Squash delays the turn at 25 - 43% per hit with no resistance roll; the only brake is one bit: 14% of the story bosses and 56% of the postgame bosses are immune, the others have none (docs/FORMULAS.md 5c)</t>
         </is>
       </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>A rows, every story and postgame boss immune to turn delay, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows)</t>
+        </is>
+      </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
@@ -2923,7 +2993,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>not a problem</t>
         </is>
       </c>
       <c r="O33" t="inlineStr">
@@ -2988,9 +3058,14 @@
           <t>Top single spell (tier 4) against tier 1 at their top levels: 2.5 times the power (1,300 against 520) for 2.6 times the TP (84 against 32) and a chant 34% slower (0.70 against 1.06); area tier 3 against tier 2: 1.4 times the power for twice the TP, 23% slower. Power per TP stays about equal (95%)</t>
         </is>
       </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>M rows, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); Witch 0.59 advanced, 0.94 late (CLASS_STAGES.md)</t>
+        </is>
+      </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="O34" t="inlineStr">
@@ -3271,9 +3346,14 @@
           <t>One crown takes 4,393 random battles in the best zone (25 resets from 70) (docs/generated/CATCH_UP_OPTIONS.md, section The crown)</t>
         </is>
       </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>ExePatches set balance in both program files (12 rows, 17 bytes each); seen working in the game by the user</t>
+        </is>
+      </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="O38" t="inlineStr">
@@ -3502,9 +3582,14 @@
           <t>P01, P02, P03, P14, P15</t>
         </is>
       </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>as J29</t>
+        </is>
+      </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="O41" t="inlineStr">
@@ -3574,9 +3659,14 @@
           <t>P03, P14, P15</t>
         </is>
       </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>as J27</t>
+        </is>
+      </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
@@ -3646,9 +3736,14 @@
           <t>P01, P02, P03, P04, P07, P10, P11, P13, P14, P15</t>
         </is>
       </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>as J25</t>
+        </is>
+      </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
@@ -3887,9 +3982,14 @@
           <t>Damage per time: two-handed basic pieces lead at the end too (P24: Heavy Axe 100% against Hand Axe 87%, Heavy Lance 100% against Lance 51%); but whole boss fights at P24 are won 82% with one hand and a shield against 57% with two hands (Dark Lord and Valkyrie, 40 battles): late, speed and the shield win. Unique pieces not modelled</t>
         </is>
       </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>W rows, two-handed base ATK -10%, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows)</t>
+        </is>
+      </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="O46" t="inlineStr">
@@ -3964,9 +4064,14 @@
           <t>A Mistress with a whip makes 40% (C34) and 10% (P24) of the damage per time of the Dark Lord; in the hands of a Papillon a whip gives 83 - 91% of a sword (remeasured 2026-10-09 after the fix of passive regeneration and the forge share 0.5)</t>
         </is>
       </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>W rows, whip upgrade rate 2.0 and Whip Mastery x2, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); Hard Whipping worth 100% (SKILL_WORTH.md (78 of 84 active skills at 60% or more of the best strike of their class))</t>
+        </is>
+      </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="O47" t="inlineStr">
@@ -4041,9 +4146,14 @@
           <t>As J06: 10 of the 13 bow skills refuse a gun</t>
         </is>
       </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>as J06</t>
+        </is>
+      </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="O48" t="inlineStr">
@@ -4113,9 +4223,14 @@
           <t>The plain attack is 18 - 100% of the best action at C18 (about 45% in the middle) and 0 - 24% at P24 (remeasured 2026-10-09 after the fix of passive regeneration and the forge share 0.5)</t>
         </is>
       </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>W rows, Double Attack, Triple Attack and Barrage +25%, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows)</t>
+        </is>
+      </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
@@ -4185,9 +4300,14 @@
           <t>Dark Aura is on 21% of the enemies of level 60 and above (49 of 237) and on 13 of the 55 postgame bosses</t>
         </is>
       </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>E rows, Dark Aura of common enemies 4 stats instead of 6, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows)</t>
+        </is>
+      </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
@@ -4257,9 +4377,14 @@
           <t>A magic defence buff of +25% on the target cuts a spell by 11 - 15% (INT 150 / power 300 / RES 150: 375 to 319; INT 300 / power 900 / RES 300: 1,050 to 938): the power of the spell is not reduced by it (docs/FORMULAS.md 3)</t>
         </is>
       </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>M rows, magic defence buffs and debuffs x1.5, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows)</t>
+        </is>
+      </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="O51" t="inlineStr">
@@ -4408,12 +4533,12 @@
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>Poison on story bosses, healer casting Poison until it lands (tools/skill_value.py play, check_runs, 2026-10-09): where it enters it takes 7 - 25% of the boss HP over the fight; C26 (Michelle, open in vanilla) wins 48% &gt; 72% and 27% of its HP. Of the 11 bosses immune in vanilla six are opened (Cupid C09, Tres Durian C31, Queen of Darkness C34, Iron Maiden C37, Samael C38, Atialuco C40); kept immune: Ghast, Doll, Countess of Vrachia (undead or doll), Beatrice (C26 already 27%), Heartless Avenger (C30: 32%, the fight halved). On C34, C38 and C40 the water resistance (70 - 80) leaves a 19 - 29% roll: poison pays there only when cast again until it lands (16 - 25% of the boss HP, 7% on C40)</t>
+          <t>A001 - A239, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); SKILL_AILMENTS.md</t>
         </is>
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="O53" t="inlineStr">
@@ -4555,9 +4680,14 @@
           <t>P03, P10, P13, P14, P15, P19</t>
         </is>
       </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>T031 - T040 and Y rows, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); Trickster 1.08 - 1.13, Joker 1.00 advanced and 0.96 late, within the band (CLASS_STAGES.md)</t>
+        </is>
+      </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="O55" t="inlineStr">
@@ -4629,7 +4759,7 @@
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>not a problem</t>
         </is>
       </c>
       <c r="O56" t="inlineStr">
@@ -4701,7 +4831,7 @@
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>not a problem</t>
         </is>
       </c>
       <c r="O57" t="inlineStr">
@@ -4768,7 +4898,7 @@
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>not a problem</t>
         </is>
       </c>
       <c r="O58" t="inlineStr">
@@ -4835,7 +4965,7 @@
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>not a problem</t>
         </is>
       </c>
       <c r="O59" t="inlineStr">
@@ -4982,9 +5112,14 @@
           <t>Mesmerized (Magnificent Steps, 0.07) and Warning Shot (0.06) roll once per bearer with no immunity test: one bearer of each takes 13% of the enemy turns, three 33%, five 49% (EffectRules 259, 283)</t>
         </is>
       </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>A rows, Magnificent Steps 2 - 4% and Warning Shot 1 - 3%, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows)</t>
+        </is>
+      </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="O61" t="inlineStr">
@@ -5054,9 +5189,14 @@
           <t>73% of the 64 damage techniques have a speed factor below 1 at their top level (median 0.90, range 0.40 - 1.16). The values of the first game are not in the data to compare</t>
         </is>
       </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>looked at skill by skill in T06: SKILL_WORTH.md (78 of 84 active skills at 60% or more of the best strike of their class); the chants and speeds that held a skill under the line are in the M, K and X rows</t>
+        </is>
+      </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="O62" t="inlineStr">
@@ -5131,9 +5271,14 @@
           <t>The reset bonus is 1 to 5 points (0x4f94f7 - 0x4f9540); one crown 4,393 battles, best by resets from 70 (docs/generated/CATCH_UP_OPTIONS.md)</t>
         </is>
       </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>as J37</t>
+        </is>
+      </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="O63" t="inlineStr">
@@ -5208,9 +5353,14 @@
           <t>A second Maid matters late: Actim Castle at 50, 13.0 of 20 battles with one Maid, 15.7 with two (TP after 8 battles 20% against 46%); in the middle of the story one Maid already reaches 20 of 20 (remeasured 2026-10-09 after the fix of passive regeneration and the forge share 0.5)</t>
         </is>
       </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>as J05</t>
+        </is>
+      </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="O64" t="inlineStr">
@@ -5277,7 +5427,7 @@
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>not a problem</t>
         </is>
       </c>
       <c r="O65" t="inlineStr">
@@ -5344,7 +5494,7 @@
       </c>
       <c r="L66" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>not a problem</t>
         </is>
       </c>
       <c r="O66" t="inlineStr">
@@ -5411,7 +5561,7 @@
       </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>not a problem</t>
         </is>
       </c>
       <c r="O67" t="inlineStr">
@@ -5478,7 +5628,7 @@
       </c>
       <c r="L68" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>not a problem</t>
         </is>
       </c>
       <c r="O68" t="inlineStr">
@@ -5543,9 +5693,14 @@
           <t>P03, P14, P15</t>
         </is>
       </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>X rows, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); Blood Drain worth 76% (SKILL_WORTH.md (78 of 84 active skills at 60% or more of the best strike of their class))</t>
+        </is>
+      </c>
       <c r="L69" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="O69" t="inlineStr">
@@ -5610,9 +5765,14 @@
           <t>P03, P14, P15</t>
         </is>
       </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>X rows, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); Soul Drain worth 78%, Soul Absorb 68% (SKILL_WORTH.md (78 of 84 active skills at 60% or more of the best strike of their class))</t>
+        </is>
+      </c>
       <c r="L70" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="O70" t="inlineStr">
@@ -5679,7 +5839,7 @@
       </c>
       <c r="L71" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>not a problem</t>
         </is>
       </c>
       <c r="O71" t="inlineStr">
@@ -5744,9 +5904,14 @@
           <t>P03, P14, P15</t>
         </is>
       </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>X088 and its levels, Blood Rage 43 to 32 TP, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows). 2026-10-11, the user: the change stays, it is justified in its row</t>
+        </is>
+      </c>
       <c r="L72" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="O72" t="inlineStr">
@@ -5766,7 +5931,7 @@
       </c>
       <c r="R72" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>2026-10-11: approved by the user, the change stays</t>
         </is>
       </c>
     </row>
@@ -5811,9 +5976,14 @@
           <t>P03, P14, P15</t>
         </is>
       </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>X rows, Brave and Protect x2, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows). 2026-10-11, the user: the change stays, it is justified in its row</t>
+        </is>
+      </c>
       <c r="L73" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="O73" t="inlineStr">
@@ -5833,7 +6003,7 @@
       </c>
       <c r="R73" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>2026-10-11: approved by the user, the change stays</t>
         </is>
       </c>
     </row>
@@ -5880,7 +6050,7 @@
       </c>
       <c r="L74" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>not a problem</t>
         </is>
       </c>
       <c r="O74" t="inlineStr">
@@ -5947,7 +6117,7 @@
       </c>
       <c r="L75" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>not a problem</t>
         </is>
       </c>
       <c r="O75" t="inlineStr">
@@ -6014,7 +6184,7 @@
       </c>
       <c r="L76" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>not a problem</t>
         </is>
       </c>
       <c r="O76" t="inlineStr">
@@ -6081,7 +6251,7 @@
       </c>
       <c r="L77" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>not a problem</t>
         </is>
       </c>
       <c r="O77" t="inlineStr">
@@ -6148,7 +6318,7 @@
       </c>
       <c r="L78" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>not a problem</t>
         </is>
       </c>
       <c r="O78" t="inlineStr">
@@ -6215,7 +6385,7 @@
       </c>
       <c r="L79" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>not a problem</t>
         </is>
       </c>
       <c r="O79" t="inlineStr">
@@ -6349,7 +6519,7 @@
       </c>
       <c r="L81" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>not a problem</t>
         </is>
       </c>
       <c r="O81" t="inlineStr">
@@ -6414,9 +6584,14 @@
           <t>P03, P14, P15</t>
         </is>
       </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>X rows, Illusion 3 / 4 / 5 hits, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows). 2026-10-11, the user: the change stays, it is justified in its row</t>
+        </is>
+      </c>
       <c r="L82" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="O82" t="inlineStr">
@@ -6436,7 +6611,7 @@
       </c>
       <c r="R82" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>2026-10-11: approved by the user, the change stays</t>
         </is>
       </c>
     </row>
@@ -6481,9 +6656,14 @@
           <t>P03, P04, P07, P10, P14, P15</t>
         </is>
       </c>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>Q rows, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); Magical Spark worth 100% (SKILL_WORTH.md (78 of 84 active skills at 60% or more of the best strike of their class))</t>
+        </is>
+      </c>
       <c r="L83" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="O83" t="inlineStr">
@@ -6548,9 +6728,14 @@
           <t>P03, P04, P07, P10, P14, P15</t>
         </is>
       </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>Q001 and its levels, Magical Change 52 to 39 TP, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows)</t>
+        </is>
+      </c>
       <c r="L84" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="O84" t="inlineStr">
@@ -6682,9 +6867,14 @@
           <t>P03, P14, P15</t>
         </is>
       </c>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>T066 - T070, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows)</t>
+        </is>
+      </c>
       <c r="L86" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="O86" t="inlineStr">
@@ -6751,7 +6941,7 @@
       </c>
       <c r="L87" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>out of the balance</t>
         </is>
       </c>
       <c r="O87" t="inlineStr">
@@ -6818,7 +7008,7 @@
       </c>
       <c r="L88" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>not a problem</t>
         </is>
       </c>
       <c r="O88" t="inlineStr">
@@ -6885,7 +7075,7 @@
       </c>
       <c r="L89" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>not a problem</t>
         </is>
       </c>
       <c r="O89" t="inlineStr">
@@ -7019,7 +7209,7 @@
       </c>
       <c r="L91" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>not a problem</t>
         </is>
       </c>
       <c r="O91" t="inlineStr">
@@ -7086,7 +7276,7 @@
       </c>
       <c r="L92" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>out of the balance</t>
         </is>
       </c>
       <c r="O92" t="inlineStr">
@@ -7153,7 +7343,7 @@
       </c>
       <c r="L93" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>out of the balance</t>
         </is>
       </c>
       <c r="O93" t="inlineStr">
@@ -7220,7 +7410,7 @@
       </c>
       <c r="L94" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>out of the balance</t>
         </is>
       </c>
       <c r="O94" t="inlineStr">
@@ -7285,9 +7475,14 @@
           <t>P01, P02, P03, P14, P15</t>
         </is>
       </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>T056 - T065, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); Hard Whipping worth 100% (SKILL_WORTH.md (78 of 84 active skills at 60% or more of the best strike of their class))</t>
+        </is>
+      </c>
       <c r="L95" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="O95" t="inlineStr">
@@ -7354,7 +7549,7 @@
       </c>
       <c r="L96" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>not a problem</t>
         </is>
       </c>
       <c r="O96" t="inlineStr">
@@ -7419,9 +7614,14 @@
           <t>P03, P14, P15</t>
         </is>
       </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>K rows, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); Ninja Piledriver worth 100% (SKILL_WORTH.md (78 of 84 active skills at 60% or more of the best strike of their class))</t>
+        </is>
+      </c>
       <c r="L97" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="O97" t="inlineStr">
@@ -7486,9 +7686,14 @@
           <t>P01, P02, P03, P14, P15</t>
         </is>
       </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>K rows (TP -25%) and X rows (chant 0.75 at every level), built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows). 2026-10-11, the user: the change stays, it is justified in its row</t>
+        </is>
+      </c>
       <c r="L98" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="O98" t="inlineStr">
@@ -7508,7 +7713,7 @@
       </c>
       <c r="R98" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>2026-10-11: approved by the user, the change stays</t>
         </is>
       </c>
     </row>
@@ -7553,9 +7758,14 @@
           <t>P01, P02, P03, P08, P10, P14, P15</t>
         </is>
       </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>X rows, Shadow Sew -25% TP, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows). 2026-10-11, the user: the change stays, it is justified in its row</t>
+        </is>
+      </c>
       <c r="L99" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="O99" t="inlineStr">
@@ -7575,7 +7785,7 @@
       </c>
       <c r="R99" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>2026-10-11: approved by the user, the change stays</t>
         </is>
       </c>
     </row>
@@ -7620,9 +7830,14 @@
           <t>P03, P14, P15</t>
         </is>
       </c>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>X rows, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); the scrolls are worth 48 - 60% beside Ninja Piledriver, which the Tantou (W045) raised (SKILL_WORTH.md (78 of 84 active skills at 60% or more of the best strike of their class)). 2026-10-11, the user: they stay as they are, they are debuffs late (J27)</t>
+        </is>
+      </c>
       <c r="L100" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="O100" t="inlineStr">
@@ -7689,7 +7904,7 @@
       </c>
       <c r="L101" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>not a problem</t>
         </is>
       </c>
       <c r="O101" t="inlineStr">
@@ -7756,7 +7971,7 @@
       </c>
       <c r="L102" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>not a problem</t>
         </is>
       </c>
       <c r="O102" t="inlineStr">
@@ -7823,7 +8038,7 @@
       </c>
       <c r="L103" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>not a problem</t>
         </is>
       </c>
       <c r="O103" t="inlineStr">
@@ -7890,7 +8105,7 @@
       </c>
       <c r="L104" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>not a problem</t>
         </is>
       </c>
       <c r="O104" t="inlineStr">
@@ -7957,7 +8172,7 @@
       </c>
       <c r="L105" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>not a problem</t>
         </is>
       </c>
       <c r="O105" t="inlineStr">
@@ -8022,9 +8237,14 @@
           <t>P01, P02, P03, P14, P15</t>
         </is>
       </c>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>T051 - T055, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); Enticing Love worth 100% (SKILL_WORTH.md (78 of 84 active skills at 60% or more of the best strike of their class))</t>
+        </is>
+      </c>
       <c r="L106" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="O106" t="inlineStr">
@@ -8089,9 +8309,14 @@
           <t>P03, P14, P15</t>
         </is>
       </c>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>M rows, Carrot and Stick x1.5, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows)</t>
+        </is>
+      </c>
       <c r="L107" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="O107" t="inlineStr">
@@ -8158,7 +8383,7 @@
       </c>
       <c r="L108" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>not a problem</t>
         </is>
       </c>
       <c r="O108" t="inlineStr">
@@ -8223,9 +8448,14 @@
           <t>P03, P14, P15, P16</t>
         </is>
       </c>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>D rows, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); dolls within the band at the four stages (1.12, 0.97, 1.04, 1.13; CLASS_STAGES.md)</t>
+        </is>
+      </c>
       <c r="L109" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="O109" t="inlineStr">
@@ -8290,9 +8520,14 @@
           <t>P03, P14, P15</t>
         </is>
       </c>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>X rows, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); Life Bringer worth 48% beside Showtime (SKILL_WORTH.md (78 of 84 active skills at 60% or more of the best strike of their class)). 2026-10-11, the user: it stays as it is</t>
+        </is>
+      </c>
       <c r="L110" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="O110" t="inlineStr">
@@ -8429,9 +8664,14 @@
           <t>Limit Field adds its negative value to the damage of every unit, both sides alike (EffectRules 190)</t>
         </is>
       </c>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>Limit Field TP x0.55, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows)</t>
+        </is>
+      </c>
       <c r="L112" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="O112" t="inlineStr">
@@ -8496,9 +8736,14 @@
           <t>Graceful Rose: +20% for 5 TP, below Danger Shoot; against a lone boss the Papillon only had the area attack Rose Queen (first Papillon slot 36% of the Fighter/Scout band at C34)</t>
         </is>
       </c>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>S rows, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); Graceful Rose worth 100% (SKILL_WORTH.md (78 of 84 active skills at 60% or more of the best strike of their class))</t>
+        </is>
+      </c>
       <c r="L113" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="O113" t="inlineStr">
@@ -8565,7 +8810,7 @@
       </c>
       <c r="L114" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>not a problem</t>
         </is>
       </c>
       <c r="O114" t="inlineStr">
@@ -8632,7 +8877,7 @@
       </c>
       <c r="L115" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>not a problem</t>
         </is>
       </c>
       <c r="O115" t="inlineStr">
@@ -8697,9 +8942,14 @@
           <t>P03, P06, P14, P15</t>
         </is>
       </c>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t>W rows, +25%, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows)</t>
+        </is>
+      </c>
       <c r="L116" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="O116" t="inlineStr">
@@ -8764,9 +9014,14 @@
           <t>P03, P06, P14, P15</t>
         </is>
       </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>W rows, +25%, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows)</t>
+        </is>
+      </c>
       <c r="L117" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="O117" t="inlineStr">
@@ -8833,7 +9088,7 @@
       </c>
       <c r="L118" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>not a problem</t>
         </is>
       </c>
       <c r="O118" t="inlineStr">
@@ -8977,7 +9232,7 @@
       </c>
       <c r="L120" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>not a problem</t>
         </is>
       </c>
       <c r="O120" t="inlineStr">
@@ -9044,7 +9299,7 @@
       </c>
       <c r="L121" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>out of the balance</t>
         </is>
       </c>
       <c r="O121" t="inlineStr">
@@ -9111,7 +9366,7 @@
       </c>
       <c r="L122" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>out of the balance</t>
         </is>
       </c>
       <c r="O122" t="inlineStr">
@@ -9397,9 +9652,14 @@
           <t>P15, P19</t>
         </is>
       </c>
+      <c r="K126" t="inlineStr">
+        <is>
+          <t>K001 - K025, T001 - T030, T051 - T065, W045, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); Kunoichi and Mistress within the band at the four stages (CLASS_STAGES.md)</t>
+        </is>
+      </c>
       <c r="L126" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="O126" t="inlineStr">
@@ -9531,9 +9791,14 @@
           <t>The piece of a postgame boss is certain (drop chance 100, one slot of weight 100). A fixed piece of a common enemy falls 2 to 4.5% of the time, of a very powerful enemy 10 to 50%; seven pieces of six common enemies fall under 2% (0.8 to 1.5%). A steal that succeeds draws among the drops of the enemy without the "nothing" of the draw, once per enemy (FORMULAS 12.16): the Chief's Special of Garasha comes out of 1.8% of them; 135 enemies cannot be robbed, the bosses and, among the common ones, Odin, Myrddin, Asmodeus and Carmilla</t>
         </is>
       </c>
+      <c r="K128" t="inlineStr">
+        <is>
+          <t>P024, P079 - P084 (seven pieces under 2% raised to 2%) and P085 - P088 (Item Steal open on Odin, Myrddin, Asmodeus and Carmilla), built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); their pieces come out of 6 - 9% of the steals that succeed; a talk of Euthys says it in the game</t>
+        </is>
+      </c>
       <c r="L128" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="N128" t="inlineStr">
@@ -9549,6 +9814,11 @@
       <c r="P128" t="inlineStr">
         <is>
           <t>true</t>
+        </is>
+      </c>
+      <c r="R128" t="inlineStr">
+        <is>
+          <t>2026-10-11: approved by the user (seven drop weights to the 2% floor; Item Steal open on the four immune commons)</t>
         </is>
       </c>
     </row>
@@ -9732,9 +10002,14 @@
           <t>An unused member from level 1 to a party at 70: 645 random battles in vanilla (docs/generated/CATCH_UP_OPTIONS.md, from level 1)</t>
         </is>
       </c>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t>as U01</t>
+        </is>
+      </c>
       <c r="L131" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="O131" t="inlineStr">
@@ -10010,9 +10285,14 @@
           <t>A member 10 levels behind needs 70 - 144 random battles to come within 4 levels of the party (party 30 - 70), 20 behind 116 - 311, from level 1 124 - 519; own pace 25 - 35 battles per level (docs/generated/CATCH_UP_OPTIONS.md)</t>
         </is>
       </c>
+      <c r="K135" t="inlineStr">
+        <is>
+          <t>ExePatches set balance in both program files; CATCH_UP_OPTIONS.md, row B4; seen working in the game by the user</t>
+        </is>
+      </c>
       <c r="L135" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="O135" t="inlineStr">
@@ -10082,9 +10362,14 @@
           <t>A random battle is short: 2.6 - 3.3 actions per member, 0.9 - 2.5 units of time (C07 to P24); the length is in the number of battles per level (own pace 25 - 35), which the decided curve cuts to 15 - 19</t>
         </is>
       </c>
+      <c r="K136" t="inlineStr">
+        <is>
+          <t>as U01</t>
+        </is>
+      </c>
       <c r="L136" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="M136" t="inlineStr">
@@ -10164,9 +10449,14 @@
           <t>Enemies of random formations whose lowest physical resistance is 50 or more: 0% up to level 19, 5% (20 - 39), 20% (40 - 59), 30% (60 - 79), 77% (80 - 99); whose every element is 50 or more: 0 - 6% up to 79, 21% from 80. True late, false early</t>
         </is>
       </c>
+      <c r="K137" t="inlineStr">
+        <is>
+          <t>E rows, common enemies of level 80 or more lose 10 points of physical resistance, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows)</t>
+        </is>
+      </c>
       <c r="L137" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="M137" t="inlineStr">
@@ -10246,9 +10536,14 @@
           <t>The rates are data (passives of EnemyAttackData). Median of the enemies against the top of the party: Reprisal 0.25 against 0.18, Auto-Guard 0.30 against 0.12, Counter 0.15 against 0.12, Ecstasy 0.5 against 0.15; equal for Double and Triple Attack, Dark Aura and Knock Down</t>
         </is>
       </c>
+      <c r="K138" t="inlineStr">
+        <is>
+          <t>E rows, four enemy passives capped at the party top, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows)</t>
+        </is>
+      </c>
       <c r="L138" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="M138" t="inlineStr">
@@ -10397,12 +10692,12 @@
       </c>
       <c r="K140" t="inlineStr">
         <is>
-          <t>Measured as the opening move of a Sage or Maid on rows of four random battles (40 rows, 2026-10-09): where the commons threaten (C39, C40 floors: half the rows lost without) Paralyze lifts the rows won 50% &gt; 70% and the HP left 50% &gt; 69%; Freeze +8 - 10 points, Sleep +7, Lullaby +3 - 10; Stun none (it takes no turn by design: it breaks chants). Where the commons do not threaten (the stage each is learnt, docs/generated/SKILL_AILMENTS.md) nothing changes, as no option can: even with Carol at 0 the party ends eight battles with 83 - 90% HP. A slow added to Paralyze adds nothing more. Paralysis takes a turn on 30 in 100 only, a rule of the executable (docs/FORMULAS.md 12.4)</t>
+          <t>A rows, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); SKILL_AILMENTS.md</t>
         </is>
       </c>
       <c r="L140" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="M140" t="inlineStr">
@@ -10482,9 +10777,14 @@
           <t>A DEF debuff of 10 - 20% adds 2 - 5% to the damage of a skill (the power of the skill multiplies; the debuff only lowers the defence term) (docs/FORMULAS.md 2)</t>
         </is>
       </c>
+      <c r="K141" t="inlineStr">
+        <is>
+          <t>A rows, debuffs x1.5, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows)</t>
+        </is>
+      </c>
       <c r="L141" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="M141" t="inlineStr">
@@ -10792,7 +11092,7 @@
       </c>
       <c r="L145" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>not a problem</t>
         </is>
       </c>
       <c r="M145" t="inlineStr">
@@ -10872,9 +11172,14 @@
           <t>Growth per level does not fall after 70: the mean gain of every stat over the growth rows is the same from 50 to 70 as from 70 to 99 (99 - 100%). What rises is the EXP a level costs: 32,788 on average from 51 to 70, 70,692 from 71 to 99 (2.2 times)</t>
         </is>
       </c>
+      <c r="K146" t="inlineStr">
+        <is>
+          <t>as U01</t>
+        </is>
+      </c>
       <c r="L146" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="M146" t="inlineStr">
@@ -10954,9 +11259,14 @@
           <t>Skill points in all: 52 at level 30, 139 at 50, 295 at 70, 685 at 99 without resets. The skill plans of the guide cost 246 (Papillon) to 440 (Valkyrie) points: reached about level 66 - 81. By level 50 a member of the reference party holds 25 - 32 skill levels, a third of her plan</t>
         </is>
       </c>
+      <c r="K147" t="inlineStr">
+        <is>
+          <t>B001 - B040, +1 skill point per level from 31 to 70, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows)</t>
+        </is>
+      </c>
       <c r="L147" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="M147" t="inlineStr">
@@ -11515,9 +11825,14 @@
           <t>Quest reward fields (not read)</t>
         </is>
       </c>
+      <c r="K155" t="inlineStr">
+        <is>
+          <t>41 P rows of the table quests, gold reward x1.40, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); EXP for the members behind comes from the factors B4 (U01)</t>
+        </is>
+      </c>
       <c r="L155" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="M155" t="inlineStr">
@@ -11538,6 +11853,11 @@
       <c r="P155" t="inlineStr">
         <is>
           <t>partly true</t>
+        </is>
+      </c>
+      <c r="R155" t="inlineStr">
+        <is>
+          <t>2026-10-11: approved by the user (quest gold x1.40)</t>
         </is>
       </c>
     </row>
@@ -12056,9 +12376,14 @@
           <t>In the same slot, the doll line makes 29% of the party damage share of the Fighter and Scout lines on average (Doll Master 40 - 54%, Soul Summoner 7 - 22%; bosses C13, C18, C25, C34, C38, 25 battles each; sim/measures.py slot_share, with a Soul Summoner role, two dolls kept with Double Puppet and Mercidarian first). The other Spieler line (Trickster, Papillon) sits at about two thirds of that band</t>
         </is>
       </c>
+      <c r="K163" t="inlineStr">
+        <is>
+          <t>D001 - D243, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); dolls 1.12, 0.97, 1.04, 1.13 and soul summoner 1.12, 0.98, 0.87, 1.02 at the four stages, within the band (CLASS_STAGES.md)</t>
+        </is>
+      </c>
       <c r="L163" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="M163" t="inlineStr">

</xml_diff>

<commit_message>
data: the six rows without a figure measured
the six rows without a figure measured; four closed, Support Shot and
Roulette Circus wait (4 open of 162)
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -4605,12 +4605,12 @@
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>Replenishing Carol heals 40 - 59% of the mean member HP each tick from C07 to C29 (27% at C40), free. Yet with Carol at 0 the party still ends rows of eight random battles with 83 - 90% HP from C07 to C22, 71% at C33, 36% at C37 (2026-10-09): common fights are not where Carol decides; her weight is on the bosses, which the windows of vanilla already include (tools/difficulty_curve.py)</t>
+          <t>SKILL_VALUE.md: the reference party with and without Replenishing Carol wins 100% of C10, C13 and C18 with the same length (8.3 / 9.0 / 9.6 against 8.3 / 9.1 / 9.1); rows of eight random battles without it end with 83 - 90% HP from C07 to C22</t>
         </is>
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>not a problem</t>
         </is>
       </c>
       <c r="O54" t="inlineStr">
@@ -4620,7 +4620,7 @@
       </c>
       <c r="P54" t="inlineStr">
         <is>
-          <t>open: a question of difficulty, not of a dead skill</t>
+          <t>false in the measure: the fights of the intermediate stage are won as often and as fast without it</t>
         </is>
       </c>
       <c r="Q54" t="inlineStr">
@@ -4630,7 +4630,7 @@
       </c>
       <c r="R54" t="inlineStr">
         <is>
-          <t>2026-10-09: left to T02 and T08</t>
+          <t>2026-10-09: left to T02 and T08; 2026-10-11: measured</t>
         </is>
       </c>
     </row>
@@ -5035,6 +5035,11 @@
           <t>Outcome tables (executable, docs/generated/BALANCE_BASELINE.md Random moves): Roulette Circus 10% heals a random enemy fully and 10% does nothing; Magic Box 10% kills its user for certain and 10% hits her with a double hit; Showtime 10.5% stuns the whole party for certain; Heaven or Hell deals 10% of the target max HP capped at 222, or heals it</t>
         </is>
       </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>L rows built. Roulette Circus (15 TP, one level; half its results an ailment on every enemy, a fifth a heal of the party, a tenth damage of level x 15): cast every turn by the dolls role, rows of eight random battles last 3 - 25% longer (C03, C06, C13, C22) and end with -1 to +3 points of HP; against bosses 6 - 32% longer (scratch/audit_2026-10-11/roulette_chain.py, measure_open_rows.py). SKILL_WORTH.md gives it 0% because it counts damage only. Waits for the user: leave it as the gamble of the base class, or raise it</t>
+        </is>
+      </c>
       <c r="L60" t="inlineStr">
         <is>
           <t>open</t>
@@ -5047,7 +5052,7 @@
       </c>
       <c r="P60" t="inlineStr">
         <is>
-          <t>true: lottery skills</t>
+          <t>true for Roulette Circus only: Magic Box, Showtime and Heaven or Hell are worth 100% after the L rows</t>
         </is>
       </c>
       <c r="Q60" t="inlineStr">
@@ -5057,7 +5062,7 @@
       </c>
       <c r="R60" t="inlineStr">
         <is>
-          <t>2026-10-09: decided in milestone L</t>
+          <t>2026-10-09: decided in milestone L; 2026-10-11: measured</t>
         </is>
       </c>
     </row>
@@ -6450,9 +6455,14 @@
           <t>P03, P14, P15</t>
         </is>
       </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>scratch/audit_2026-10-11/worth_with_weapon.py (the measure of tools/skill_worth.py, the Sage with a Tome): Bible Thump is her best option at the bosses of C40 and P08, 90% of it at P18, 74% at C34, 27 - 29% at C22 and C30; in random battles 43 - 89% (9% where a row falls to one spell)</t>
+        </is>
+      </c>
       <c r="L80" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>not a problem</t>
         </is>
       </c>
       <c r="O80" t="inlineStr">
@@ -6462,7 +6472,7 @@
       </c>
       <c r="P80" t="inlineStr">
         <is>
-          <t>not measured: it needs a tome, which the Sage plan does not wear</t>
+          <t>partly true: it needs a tome, which costs the Sage the INT of her staff; with one it is her best strike against the bosses that resist her spells</t>
         </is>
       </c>
       <c r="Q80" t="inlineStr">
@@ -6472,7 +6482,7 @@
       </c>
       <c r="R80" t="inlineStr">
         <is>
-          <t>2026-10-09: open</t>
+          <t>2026-10-09: open; 2026-10-11: measured</t>
         </is>
       </c>
     </row>
@@ -6800,9 +6810,14 @@
           <t>P03, P14, P15</t>
         </is>
       </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>M rows, Sun Veil x1.5, built and read back; SKILL_VALUE.md: wins of the reference party 80% to 85% and fights 7% shorter at C40 with it, nothing at C22 and C34 (bosses that do not cast)</t>
+        </is>
+      </c>
       <c r="L85" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="O85" t="inlineStr">
@@ -6812,7 +6827,7 @@
       </c>
       <c r="P85" t="inlineStr">
         <is>
-          <t>true: magic defence is a small term of the magic formula (RES x 1.5 against INT x 2 + power)</t>
+          <t>partly true: it pays only where the boss casts</t>
         </is>
       </c>
       <c r="Q85" t="inlineStr">
@@ -6822,7 +6837,7 @@
       </c>
       <c r="R85" t="inlineStr">
         <is>
-          <t>2026-10-09: left to T04</t>
+          <t>2026-10-09: left to T04; 2026-10-11: measured</t>
         </is>
       </c>
     </row>
@@ -7140,6 +7155,11 @@
           <t>P03, P14, P15</t>
         </is>
       </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>scratch/audit_2026-10-11/measure_open_rows.py: the reference party with and without Support Shot at its top level: C22 100% / 100% wins, length +2%; C30 +6%; C34 -4%; C40 80% / 73% wins (40 fights each: inside the noise). Waits for the user: leave it as the passive of plain-attack parties, or raise its chance</t>
+        </is>
+      </c>
       <c r="L90" t="inlineStr">
         <is>
           <t>open</t>
@@ -7152,7 +7172,7 @@
       </c>
       <c r="P90" t="inlineStr">
         <is>
-          <t>passive: a follow-up chance of the Sniper; not measured</t>
+          <t>true: it fires only after a plain attack of a member (4 - 12% by level), and a party that has TP does not make plain attacks</t>
         </is>
       </c>
       <c r="Q90" t="inlineStr">
@@ -7162,7 +7182,7 @@
       </c>
       <c r="R90" t="inlineStr">
         <is>
-          <t>2026-10-09: open</t>
+          <t>2026-10-09: open; 2026-10-11: measured</t>
         </is>
       </c>
     </row>
@@ -8592,9 +8612,14 @@
           <t>P01, P02, P03, P14, P15</t>
         </is>
       </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>scratch/audit_2026-10-11/worth_with_weapon.py (the Joker with a Whip): Beast Binder is her best option in the random battles of C34, C40 and P08, 104 - 134% of her best with her axe at C40; 39 - 82% against the bosses. Whips forge at rate 2.0 (W rows)</t>
+        </is>
+      </c>
       <c r="L111" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>not a problem</t>
         </is>
       </c>
       <c r="O111" t="inlineStr">
@@ -8604,7 +8629,7 @@
       </c>
       <c r="P111" t="inlineStr">
         <is>
-          <t>not measured: it needs a whip; W raised whips</t>
+          <t>false with a whip in hand: the best strike of the Joker against groups from C34 on</t>
         </is>
       </c>
       <c r="Q111" t="inlineStr">
@@ -8614,7 +8639,7 @@
       </c>
       <c r="R111" t="inlineStr">
         <is>
-          <t>2026-10-09: open</t>
+          <t>2026-10-09: open; 2026-10-11: measured</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: J02 measured again on the variant
J02 measured again on the variant, the mage beside the Dark Lord at the
66 bosses from C30 on
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -671,6 +671,11 @@
           <t>Against all 66 bosses from C30 on (story and postgame), with their resistances: the mage makes a median 171% of the damage per time of the Dark Lord; 10 bosses below 100%, and the strongest superbosses wall her off: Gam the Wise 0% (100 in every element), Tenerezza at full strength 0%, Magna Meretrix at full strength 17%, Bishamon Peggy 48%, Zouchou Kuma 67%. Four postgame fights forbid magic</t>
         </is>
       </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>scratch/audit_2026-10-11/magic_wall.py (best option of the mage beside the best of the Dark Lord, value per time, the 66 bosses from C30 on, 2026-10-11): above 100% at 55 bosses on the variant (median 242%); 97% at P10 Kuchinawa; four fights forbid magic (P07, P13, P25, P47); under 100% at six superbosses only: Hell's Angel 51%, Panagia 73% and 84%, Tenerezza 50% and 54%, Samson with Magna Meretrix 51%. No resistance of an enemy was changed. The battery of 17 story bosses, where Mage-Heavy meets its floor, does not reach these six</t>
+        </is>
+      </c>
       <c r="L3" t="inlineStr">
         <is>
           <t>open</t>
@@ -693,7 +698,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>2026-10-09: to T08: lower a little the elemental resistances of the superbosses that wall magic off, keeping their flavour</t>
+          <t>2026-10-09: to T08: lower a little the elemental resistances of the superbosses that wall magic off, keeping their flavour; 2026-10-11: not built; measured again, to decide with the postgame (six superbosses)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: final pass of the sheet Regression on the build of 1,386 rows
final pass of the sheet Regression on the build of 1,386 rows: its
verdicts written, the register at 1 open of 162
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -5042,12 +5042,12 @@
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>L rows built. Roulette Circus (15 TP, one level; half its results an ailment on every enemy, a fifth a heal of the party, a tenth damage of level x 15): cast every turn by the dolls role, rows of eight random battles last 3 - 25% longer (C03, C06, C13, C22) and end with -1 to +3 points of HP; against bosses 6 - 32% longer (scratch/audit_2026-10-11/roulette_chain.py, measure_open_rows.py). SKILL_WORTH.md gives it 0% because it counts damage only. Waits for the user: leave it as the gamble of the base class, or raise it</t>
+          <t>L rows built; L002 dropped on 2026-10-11 (the user): its damage draw strikes any unit of the battle, the party included, so it stays at level x 10. Its heal of an enemy is 10% of max HP instead of all of it (L001). Cast every turn, rows of eight random battles last 3 - 25% longer and end with -1 to +3 points of HP: the cheap gamble of the base class (15 TP, one level), which can no longer sink a fight</t>
         </is>
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>not a problem</t>
         </is>
       </c>
       <c r="O60" t="inlineStr">
@@ -5057,7 +5057,7 @@
       </c>
       <c r="P60" t="inlineStr">
         <is>
-          <t>true for Roulette Circus only: Magic Box, Showtime and Heaven or Hell are worth 100% after the L rows</t>
+          <t>true for Roulette Circus only, and by its nature: Magic Box, Showtime and Heaven or Hell are worth 100% after the L rows</t>
         </is>
       </c>
       <c r="Q60" t="inlineStr">
@@ -5067,7 +5067,7 @@
       </c>
       <c r="R60" t="inlineStr">
         <is>
-          <t>2026-10-09: decided in milestone L; 2026-10-11: measured</t>
+          <t>2026-10-09: decided in milestone L; 2026-10-11: measured; 2026-10-11: closed with the final pass</t>
         </is>
       </c>
     </row>
@@ -12319,9 +12319,14 @@
           <t>Too vague to test on its own; its verdict comes from R03 and R08 in the final pass</t>
         </is>
       </c>
+      <c r="K162" t="inlineStr">
+        <is>
+          <t>DIFFICULTY_CURVE.md (final pass, Regression R08 and R10): the damage the enemies deal per turn against the party's max HP and its lowest HP stay inside the window of vanilla at 37 of 44 bosses; at the other 7 the party stands higher</t>
+        </is>
+      </c>
       <c r="L162" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>not a problem</t>
         </is>
       </c>
       <c r="M162" t="inlineStr">
@@ -12341,7 +12346,7 @@
       </c>
       <c r="P162" t="inlineStr">
         <is>
-          <t>to measure</t>
+          <t>partly true where vanilla was unfair, and eased there; elsewhere the variant keeps the ratio of vanilla</t>
         </is>
       </c>
       <c r="Q162" t="inlineStr">
@@ -12351,7 +12356,7 @@
       </c>
       <c r="R162" t="inlineStr">
         <is>
-          <t>2026-10-09: judged in the final pass (R03, R08)</t>
+          <t>2026-10-09: judged in the final pass (R03, R08); 2026-10-11: closed with the final pass</t>
         </is>
       </c>
     </row>
@@ -21047,7 +21052,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -21077,6 +21082,16 @@
           <t>Measured on</t>
         </is>
       </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Result (final pass, 2026-10-11)</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Verdict</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -21099,6 +21114,16 @@
           <t>The cases each change touches (its check), and every boss of the story and the postgame with the reference parties in the final pass (BALANCE_PLAN.md section 3, approach of 2026-10-07)</t>
         </is>
       </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>PARTY_BATTERY.md: no party wins everywhere more than the best of vanilla did; the weakest party of vanilla (Anti-Meta-Plus, 0 - 14% at eight bosses) reaches 29 - 100%, still the weakest. CLASS_STAGES.md: 74 of 76 rows within the band. Limit: the band has no top, so a class that is too fast is not flagged (the Witch fights at 0.59 of the median attacker at the advanced stage; row J11, left by the user)</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>met in what is measured</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -21121,6 +21146,16 @@
           <t>Vanilla result against Balance result for every build</t>
         </is>
       </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>PARTY_BATTERY.md: 64 of 85 pairs at or above the floor in vanilla, 76 of 85 on the variant; no pair that met its floor in vanilla lost it. CLASS_STAGES.md: the two slow rows (Assassin and Treasure Hunter of the treasure hunter role) were slow before the changes (row J26)</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>met</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -21143,6 +21178,16 @@
           <t>docs/generated/CHECKPOINT_LEVELS.md, vanilla against Balance, every checkpoint in order</t>
         </is>
       </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>CHECKPOINT_LEVELS.md: 95 checkpoints, 19 jumps; no row of balance_changes.xlsx changes the level of an enemy, so every jump stands where vanilla has it</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>met</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -21165,6 +21210,16 @@
           <t>Win rate over compositions with each class excluded</t>
         </is>
       </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Not run as written (each class left out in turn). The nearest measure: five parties of different make at 17 bosses, 76 of 85 pairs above the floor, and no boss where only one of them wins except C29 (Mage-Heavy 100%, the others 6 - 37%: Calliope, which the model does not play as the guide describes)</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>partly measured</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -21187,6 +21242,16 @@
           <t>Largest expected share of boss turns removed</t>
         </is>
       </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>A rows: every story and postgame boss is immune to turn delay; Magnificent Steps and Warning Shot at their new values take 19% of the turns of an enemy with three bearers of each (33% in vanilla)</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>met by construction</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -21209,6 +21274,16 @@
           <t>Build check: every change names the row it serves</t>
         </is>
       </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>BALANCE_BUILD.md: 1,386 of 1,386 live rows built, and each names the row it serves (column Serves, none empty)</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>met</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -21231,6 +21306,16 @@
           <t>Distance from vanilla reported with the result</t>
         </is>
       </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>The distance from vanilla is not summed up in one number; each row of balance_changes.xlsx holds the vanilla value beside the new one, and the rows the measures did not need were dropped (99 dropped)</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>not reported as a figure</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -21253,6 +21338,16 @@
           <t>Per boss, vanilla against Balance</t>
         </is>
       </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>DIFFICULTY_CURVE.md: 37 of 44 checkpoints within the windows of vanilla, 7 easier (C14, C26, C29, C30, C32, C37, C38), 0 harder. The user, 2026-10-11: the bosses the variant leaves easier stay as they are. C40, raised as an exception, is within (wins 88% &gt; 95%, length 35.5 &gt; 34.2). Limit found the same day: Heretic Samsara of Demiurge is not played by the model, in vanilla or on the variant</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>met; 7 bosses easier, accepted</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -21270,6 +21365,16 @@
           <t>No row of Criticisms that is true in vanilla is closed by a change so small that the player would not notice it: each closed row states the figure before and after, and the after sits inside its band with margin</t>
         </is>
       </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>VERDICTS.md: of 162 rows, 72 closed with the figure before and after, 77 not a problem with their figure, 12 out of the balance, 1 open (J02, left for the postgame)</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>met</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -21290,6 +21395,16 @@
       <c r="D11" t="inlineStr">
         <is>
           <t>Per boss, vanilla against Balance: the lowest HP share of the party during the fight, the damage the enemies deal per turn against the party's max HP, and the fight length stay inside the window of vanilla for a sensible party at the reference level</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>DIFFICULTY_CURVE.md, columns Lowest HP and Pressure: inside the window of vanilla at 37 of 44 checkpoints; where they leave it the party stands higher (lowest HP 11 - 31% &gt; 22 - 53% at C29, C30, C38), never lower. SIM_ANCHORS.md: 6 of 6 anchors met</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>met</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
sim: the 25 fights left are in the guide curve
the 25 fights left are in the guide curve (95 bosses measured, 65 within
their floor), the second reading of the Japanese pages written in, the
rules of Heretic Samsara and Murder License corrected
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -13119,6 +13119,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -13145,6 +13146,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -13171,6 +13173,7 @@
           <t>12.3 special damage, 2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -13197,6 +13200,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -13223,6 +13227,7 @@
           <t>2.7 special damage</t>
         </is>
       </c>
+      <c r="H6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -13249,6 +13254,7 @@
           <t>6b healing</t>
         </is>
       </c>
+      <c r="H7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -13275,6 +13281,7 @@
           <t>actions</t>
         </is>
       </c>
+      <c r="H8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -13301,6 +13308,7 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
+      <c r="H9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -13327,6 +13335,7 @@
           <t>2.7 special damage, 3 magic attack</t>
         </is>
       </c>
+      <c r="H10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -13353,6 +13362,7 @@
           <t>outside battle</t>
         </is>
       </c>
+      <c r="H11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -13379,6 +13389,7 @@
           <t>14 encounter rate</t>
         </is>
       </c>
+      <c r="H12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -13410,6 +13421,7 @@
           <t>0x47ffc0</t>
         </is>
       </c>
+      <c r="H13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -13436,6 +13448,7 @@
           <t>outside battle</t>
         </is>
       </c>
+      <c r="H14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -13462,6 +13475,7 @@
           <t>12.9 after a hit</t>
         </is>
       </c>
+      <c r="H15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -13488,6 +13502,7 @@
           <t>2 physical attack, 2.2 attack value</t>
         </is>
       </c>
+      <c r="H16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -13514,6 +13529,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -13540,6 +13556,7 @@
           <t>2 physical attack, 2.3 defence value</t>
         </is>
       </c>
+      <c r="H18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -13566,6 +13583,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -13592,6 +13610,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -13618,6 +13637,7 @@
           <t>4 critical hits</t>
         </is>
       </c>
+      <c r="H21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -13644,6 +13664,7 @@
           <t>4 critical hits</t>
         </is>
       </c>
+      <c r="H22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -13670,6 +13691,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -13696,6 +13718,7 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
+      <c r="H24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -13722,6 +13745,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -13748,6 +13772,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -13774,6 +13799,7 @@
           <t>5c turn delay</t>
         </is>
       </c>
+      <c r="H27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -13800,6 +13826,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -13826,6 +13853,7 @@
           <t>steal</t>
         </is>
       </c>
+      <c r="H29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -13852,6 +13880,7 @@
           <t>steal</t>
         </is>
       </c>
+      <c r="H30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -13878,6 +13907,7 @@
           <t>steal</t>
         </is>
       </c>
+      <c r="H31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -13909,6 +13939,7 @@
           <t>0x480e20</t>
         </is>
       </c>
+      <c r="H32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -13935,6 +13966,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -13961,6 +13993,7 @@
           <t>4 critical hits</t>
         </is>
       </c>
+      <c r="H34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -13987,6 +14020,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -14013,6 +14047,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -14039,6 +14074,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -14065,6 +14101,7 @@
           <t>applying a hit</t>
         </is>
       </c>
+      <c r="H38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -14091,6 +14128,7 @@
           <t>applying a hit</t>
         </is>
       </c>
+      <c r="H39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -14117,6 +14155,7 @@
           <t>applying a hit</t>
         </is>
       </c>
+      <c r="H40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -14148,6 +14187,7 @@
           <t>0x481060</t>
         </is>
       </c>
+      <c r="H41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -14174,6 +14214,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -14205,6 +14246,7 @@
           <t>0x481160</t>
         </is>
       </c>
+      <c r="H43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -14236,6 +14278,7 @@
           <t>0x4813a0</t>
         </is>
       </c>
+      <c r="H44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -14262,6 +14305,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -14288,6 +14332,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -14314,6 +14359,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -14340,6 +14386,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -14366,6 +14413,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -14392,6 +14440,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -14418,6 +14467,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -14444,6 +14494,7 @@
           <t>12.2 number of hits</t>
         </is>
       </c>
+      <c r="H52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -14470,6 +14521,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -14496,6 +14548,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -14522,6 +14575,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -14548,6 +14602,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -14574,6 +14629,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -14600,6 +14656,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -14626,6 +14683,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -14652,6 +14710,7 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
+      <c r="H60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -14678,6 +14737,7 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
+      <c r="H61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -14709,6 +14769,7 @@
           <t>0x4817c0</t>
         </is>
       </c>
+      <c r="H62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -14740,6 +14801,7 @@
           <t>0x481890</t>
         </is>
       </c>
+      <c r="H63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -14771,6 +14833,7 @@
           <t>0x481950</t>
         </is>
       </c>
+      <c r="H64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -14802,6 +14865,7 @@
           <t>0x481a20</t>
         </is>
       </c>
+      <c r="H65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -14828,6 +14892,7 @@
           <t>outside battle</t>
         </is>
       </c>
+      <c r="H66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -14854,6 +14919,7 @@
           <t>outside battle</t>
         </is>
       </c>
+      <c r="H67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -14880,6 +14946,7 @@
           <t>4 critical hits</t>
         </is>
       </c>
+      <c r="H68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -14906,6 +14973,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -14932,6 +15000,7 @@
           <t>9.1 who gets hit</t>
         </is>
       </c>
+      <c r="H70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -14963,6 +15032,7 @@
           <t>0x481ea0</t>
         </is>
       </c>
+      <c r="H71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -14994,6 +15064,7 @@
           <t>0x4822c0</t>
         </is>
       </c>
+      <c r="H72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -15025,6 +15096,7 @@
           <t>0x482530</t>
         </is>
       </c>
+      <c r="H73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -15056,6 +15128,7 @@
           <t>0x4827a0</t>
         </is>
       </c>
+      <c r="H74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -15087,6 +15160,7 @@
           <t>0x482a10</t>
         </is>
       </c>
+      <c r="H75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -15118,6 +15192,7 @@
           <t>0x482c80</t>
         </is>
       </c>
+      <c r="H76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -15149,6 +15224,7 @@
           <t>0x482e40</t>
         </is>
       </c>
+      <c r="H77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -15180,6 +15256,7 @@
           <t>0x4831f0</t>
         </is>
       </c>
+      <c r="H78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -15211,6 +15288,7 @@
           <t>0x4834b0</t>
         </is>
       </c>
+      <c r="H79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -15242,6 +15320,7 @@
           <t>0x4835d0</t>
         </is>
       </c>
+      <c r="H80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -15273,6 +15352,7 @@
           <t>0x483840</t>
         </is>
       </c>
+      <c r="H81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -15299,6 +15379,7 @@
           <t>4 critical hits</t>
         </is>
       </c>
+      <c r="H82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -15330,6 +15411,7 @@
           <t>0x483a60</t>
         </is>
       </c>
+      <c r="H83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -15361,6 +15443,7 @@
           <t>0x483b30</t>
         </is>
       </c>
+      <c r="H84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -15392,6 +15475,7 @@
           <t>0x483c20</t>
         </is>
       </c>
+      <c r="H85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -15423,6 +15507,7 @@
           <t>0x483d20</t>
         </is>
       </c>
+      <c r="H86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -15454,6 +15539,7 @@
           <t>0x483e00</t>
         </is>
       </c>
+      <c r="H87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -15485,6 +15571,7 @@
           <t>0x483ee0</t>
         </is>
       </c>
+      <c r="H88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -15511,6 +15598,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -15537,6 +15625,7 @@
           <t>9.1 who gets hit</t>
         </is>
       </c>
+      <c r="H90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -15563,6 +15652,7 @@
           <t>2.7 special damage</t>
         </is>
       </c>
+      <c r="H91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -15594,6 +15684,7 @@
           <t>0x484020</t>
         </is>
       </c>
+      <c r="H92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -15620,6 +15711,7 @@
           <t>2.7 special damage</t>
         </is>
       </c>
+      <c r="H93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -15646,6 +15738,7 @@
           <t>2.7 special damage</t>
         </is>
       </c>
+      <c r="H94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -15677,6 +15770,7 @@
           <t>0x484150</t>
         </is>
       </c>
+      <c r="H95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -15708,6 +15802,7 @@
           <t>0x484330</t>
         </is>
       </c>
+      <c r="H96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -15734,6 +15829,7 @@
           <t>11.1 dolls</t>
         </is>
       </c>
+      <c r="H97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -15760,6 +15856,7 @@
           <t>2 physical attack, 2.1 hit chance, 3 magic attack</t>
         </is>
       </c>
+      <c r="H98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -15786,6 +15883,7 @@
           <t>2 physical attack, 2.1 hit chance, 3 magic attack</t>
         </is>
       </c>
+      <c r="H99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -15812,6 +15910,7 @@
           <t>12.10 random moves</t>
         </is>
       </c>
+      <c r="H100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -15838,6 +15937,7 @@
           <t>12.10 random moves</t>
         </is>
       </c>
+      <c r="H101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -15864,6 +15964,7 @@
           <t>12.10 random moves</t>
         </is>
       </c>
+      <c r="H102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -15890,6 +15991,7 @@
           <t>12.10 random moves</t>
         </is>
       </c>
+      <c r="H103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -15916,6 +16018,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -15942,6 +16045,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -15968,6 +16072,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -15994,6 +16099,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -16020,6 +16126,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="n">
@@ -16046,6 +16153,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="n">
@@ -16072,6 +16180,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -16103,6 +16212,7 @@
           <t>0x4864c0</t>
         </is>
       </c>
+      <c r="H111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="n">
@@ -16129,6 +16239,7 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
+      <c r="H112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="n">
@@ -16155,6 +16266,7 @@
           <t>9.1 targets</t>
         </is>
       </c>
+      <c r="H113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -16181,6 +16293,7 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
+      <c r="H114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="n">
@@ -16207,6 +16320,7 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
+      <c r="H115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="n">
@@ -16233,6 +16347,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="n">
@@ -16259,6 +16374,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="n">
@@ -16285,6 +16401,7 @@
           <t>2 physical attack, 2.4 damage</t>
         </is>
       </c>
+      <c r="H118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="n">
@@ -16311,6 +16428,7 @@
           <t>applying a hit</t>
         </is>
       </c>
+      <c r="H119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="n">
@@ -16337,6 +16455,7 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
+      <c r="H120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="n">
@@ -16363,6 +16482,7 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
+      <c r="H121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="n">
@@ -16389,6 +16509,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="n">
@@ -16415,6 +16536,7 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
+      <c r="H123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="n">
@@ -16441,6 +16563,7 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
+      <c r="H124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="n">
@@ -16467,6 +16590,7 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
+      <c r="H125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="n">
@@ -16493,6 +16617,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="n">
@@ -16519,6 +16644,7 @@
           <t>2.8 damage received</t>
         </is>
       </c>
+      <c r="H127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="n">
@@ -16545,6 +16671,7 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
+      <c r="H128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="n">
@@ -16571,6 +16698,7 @@
           <t>2 physical attack, 2.4 damage, 3 magic attack</t>
         </is>
       </c>
+      <c r="H129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="n">
@@ -16597,6 +16725,7 @@
           <t>2 physical attack, 2.4 damage</t>
         </is>
       </c>
+      <c r="H130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="n">
@@ -16623,6 +16752,7 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
+      <c r="H131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="n">
@@ -16649,6 +16779,7 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
+      <c r="H132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="n">
@@ -16675,6 +16806,7 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
+      <c r="H133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -16701,6 +16833,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="n">
@@ -16727,6 +16860,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="n">
@@ -16753,6 +16887,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="n">
@@ -16779,6 +16914,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="n">
@@ -16805,6 +16941,7 @@
           <t>5e effects that act every turn</t>
         </is>
       </c>
+      <c r="H138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="n">
@@ -16831,6 +16968,7 @@
           <t>5e effects that act every turn</t>
         </is>
       </c>
+      <c r="H139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="n">
@@ -16857,6 +16995,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="n">
@@ -16883,6 +17022,7 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
+      <c r="H141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="n">
@@ -16909,6 +17049,7 @@
           <t>5d start of a turn</t>
         </is>
       </c>
+      <c r="H142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="n">
@@ -16935,6 +17076,7 @@
           <t>13 Pep</t>
         </is>
       </c>
+      <c r="H143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="n">
@@ -16961,6 +17103,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="n">
@@ -16987,6 +17130,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="n">
@@ -17013,6 +17157,7 @@
           <t>4 critical hits</t>
         </is>
       </c>
+      <c r="H146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="n">
@@ -17039,6 +17184,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="n">
@@ -17065,6 +17211,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="n">
@@ -17091,6 +17238,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="n">
@@ -17122,6 +17270,7 @@
           <t>0x4894a0</t>
         </is>
       </c>
+      <c r="H150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="n">
@@ -17153,6 +17302,7 @@
           <t>0x4895e0</t>
         </is>
       </c>
+      <c r="H151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="n">
@@ -17179,6 +17329,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="n">
@@ -17205,6 +17356,7 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
+      <c r="H153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="n">
@@ -17231,6 +17383,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="n">
@@ -17257,6 +17410,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="n">
@@ -17283,6 +17437,7 @@
           <t>2 physical attack, 2.1 hit chance, 5 order of turns</t>
         </is>
       </c>
+      <c r="H156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="n">
@@ -17309,6 +17464,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" t="n">
@@ -17335,6 +17491,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="n">
@@ -17361,6 +17518,7 @@
           <t>11.1 dolls</t>
         </is>
       </c>
+      <c r="H159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="n">
@@ -17387,6 +17545,7 @@
           <t>11.1 dolls</t>
         </is>
       </c>
+      <c r="H160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" t="n">
@@ -17413,6 +17572,7 @@
           <t>11.1 dolls</t>
         </is>
       </c>
+      <c r="H161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" t="n">
@@ -17439,6 +17599,7 @@
           <t>11.1 dolls</t>
         </is>
       </c>
+      <c r="H162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" t="n">
@@ -17465,6 +17626,7 @@
           <t>11.1 dolls</t>
         </is>
       </c>
+      <c r="H163" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" t="n">
@@ -17491,6 +17653,7 @@
           <t>11.1 dolls</t>
         </is>
       </c>
+      <c r="H164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="n">
@@ -17522,6 +17685,7 @@
           <t>0x48a430</t>
         </is>
       </c>
+      <c r="H165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="n">
@@ -17548,6 +17712,7 @@
           <t>10.1 stats of a piece of equipment</t>
         </is>
       </c>
+      <c r="H166" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" t="n">
@@ -17574,6 +17739,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H167" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" t="n">
@@ -17600,6 +17766,7 @@
           <t>6b healing</t>
         </is>
       </c>
+      <c r="H168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="n">
@@ -17631,6 +17798,7 @@
           <t>0x48a640</t>
         </is>
       </c>
+      <c r="H169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" t="n">
@@ -17657,6 +17825,7 @@
           <t>5e effects that act every turn</t>
         </is>
       </c>
+      <c r="H170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="n">
@@ -17683,6 +17852,7 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
+      <c r="H171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="n">
@@ -17709,6 +17879,7 @@
           <t>12.13 counters and follow-ups</t>
         </is>
       </c>
+      <c r="H172" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" t="n">
@@ -17735,6 +17906,7 @@
           <t>12.13 counters and follow-ups</t>
         </is>
       </c>
+      <c r="H173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="n">
@@ -17761,6 +17933,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H174" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" t="n">
@@ -17787,6 +17960,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" t="n">
@@ -17813,6 +17987,7 @@
           <t>2 physical attack, 2.1 hit chance</t>
         </is>
       </c>
+      <c r="H176" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" t="n">
@@ -17839,6 +18014,7 @@
           <t>passive rolls</t>
         </is>
       </c>
+      <c r="H177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="n">
@@ -17865,6 +18041,7 @@
           <t>passive rolls</t>
         </is>
       </c>
+      <c r="H178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" t="n">
@@ -17891,6 +18068,7 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
+      <c r="H179" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" t="n">
@@ -17917,6 +18095,7 @@
           <t>2.8 damage received</t>
         </is>
       </c>
+      <c r="H180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" t="n">
@@ -17943,6 +18122,7 @@
           <t>2 physical attack, 2.4 damage</t>
         </is>
       </c>
+      <c r="H181" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" t="n">
@@ -17969,6 +18149,7 @@
           <t>5d start of a turn</t>
         </is>
       </c>
+      <c r="H182" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" t="n">
@@ -17995,6 +18176,7 @@
           <t>12.13 counters and follow-ups</t>
         </is>
       </c>
+      <c r="H183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="n">
@@ -18021,6 +18203,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="n">
@@ -18047,6 +18230,7 @@
           <t>12.9 after a hit</t>
         </is>
       </c>
+      <c r="H185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="n">
@@ -18073,6 +18257,7 @@
           <t>2 physical attack, 2.4 damage</t>
         </is>
       </c>
+      <c r="H186" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" t="n">
@@ -18099,6 +18284,7 @@
           <t>2 physical attack, 2.5 chant interruption</t>
         </is>
       </c>
+      <c r="H187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="n">
@@ -18125,6 +18311,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H188" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" t="n">
@@ -18151,6 +18338,7 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
+      <c r="H189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" t="n">
@@ -18177,6 +18365,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H190" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" t="n">
@@ -18203,6 +18392,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" t="n">
@@ -18229,6 +18419,7 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
+      <c r="H192" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" t="n">
@@ -18255,6 +18446,7 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
+      <c r="H193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" t="n">
@@ -18281,6 +18473,7 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
+      <c r="H194" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" t="n">
@@ -18307,6 +18500,7 @@
           <t>after a battle</t>
         </is>
       </c>
+      <c r="H195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" t="n">
@@ -18333,6 +18527,7 @@
           <t>after a battle</t>
         </is>
       </c>
+      <c r="H196" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" t="n">
@@ -18359,6 +18554,7 @@
           <t>passive rolls</t>
         </is>
       </c>
+      <c r="H197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" t="n">
@@ -18385,6 +18581,7 @@
           <t>items</t>
         </is>
       </c>
+      <c r="H198" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" t="n">
@@ -18411,6 +18608,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H199" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" t="n">
@@ -18437,6 +18635,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H200" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" t="n">
@@ -18463,6 +18662,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H201" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" t="n">
@@ -18489,6 +18689,7 @@
           <t>11.2 songs and dances</t>
         </is>
       </c>
+      <c r="H202" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" t="n">
@@ -18515,6 +18716,7 @@
           <t>11.2 songs and dances</t>
         </is>
       </c>
+      <c r="H203" t="inlineStr"/>
     </row>
     <row r="204">
       <c r="A204" t="n">
@@ -18541,6 +18743,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H204" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" t="n">
@@ -18567,6 +18770,7 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
+      <c r="H205" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" t="n">
@@ -18593,6 +18797,7 @@
           <t>5d start of a turn</t>
         </is>
       </c>
+      <c r="H206" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" t="n">
@@ -18619,6 +18824,7 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
+      <c r="H207" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" t="n">
@@ -18645,6 +18851,7 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
+      <c r="H208" t="inlineStr"/>
     </row>
     <row r="209">
       <c r="A209" t="n">
@@ -18671,6 +18878,7 @@
           <t>11.1 dolls, 2 physical attack, 3 magic attack, 6b healing</t>
         </is>
       </c>
+      <c r="H209" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" t="n">
@@ -18697,6 +18905,7 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
+      <c r="H210" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" t="n">
@@ -18723,6 +18932,7 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
+      <c r="H211" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" t="n">
@@ -18749,6 +18959,7 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
+      <c r="H212" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" t="n">
@@ -18775,6 +18986,7 @@
           <t>2.8 damage received</t>
         </is>
       </c>
+      <c r="H213" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" t="n">
@@ -18801,6 +19013,7 @@
           <t>12.9 after a hit</t>
         </is>
       </c>
+      <c r="H214" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" t="n">
@@ -18827,6 +19040,7 @@
           <t>6b heal cap, 6b healing</t>
         </is>
       </c>
+      <c r="H215" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" t="n">
@@ -18853,6 +19067,7 @@
           <t>3 magic attack, 6b heal cap</t>
         </is>
       </c>
+      <c r="H216" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" t="n">
@@ -18879,6 +19094,7 @@
           <t>11.1 dolls</t>
         </is>
       </c>
+      <c r="H217" t="inlineStr"/>
     </row>
     <row r="218">
       <c r="A218" t="n">
@@ -18905,6 +19121,7 @@
           <t>10.1 stats of a piece of equipment</t>
         </is>
       </c>
+      <c r="H218" t="inlineStr"/>
     </row>
     <row r="219">
       <c r="A219" t="n">
@@ -18931,6 +19148,7 @@
           <t>passive rolls</t>
         </is>
       </c>
+      <c r="H219" t="inlineStr"/>
     </row>
     <row r="220">
       <c r="A220" t="n">
@@ -18957,6 +19175,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H220" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" t="n">
@@ -18983,6 +19202,7 @@
           <t>12.13 counters and follow-ups</t>
         </is>
       </c>
+      <c r="H221" t="inlineStr"/>
     </row>
     <row r="222">
       <c r="A222" t="n">
@@ -19009,6 +19229,7 @@
           <t>12.9 after a hit</t>
         </is>
       </c>
+      <c r="H222" t="inlineStr"/>
     </row>
     <row r="223">
       <c r="A223" t="n">
@@ -19035,6 +19256,7 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
+      <c r="H223" t="inlineStr"/>
     </row>
     <row r="224">
       <c r="A224" t="n">
@@ -19061,6 +19283,7 @@
           <t>outside battle</t>
         </is>
       </c>
+      <c r="H224" t="inlineStr"/>
     </row>
     <row r="225">
       <c r="A225" t="n">
@@ -19087,6 +19310,7 @@
           <t>12.13 counters and follow-ups</t>
         </is>
       </c>
+      <c r="H225" t="inlineStr"/>
     </row>
     <row r="226">
       <c r="A226" t="n">
@@ -19113,6 +19337,7 @@
           <t>2 physical attack, 2.4 other bonuses of final damage</t>
         </is>
       </c>
+      <c r="H226" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" t="n">
@@ -19139,6 +19364,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H227" t="inlineStr"/>
     </row>
     <row r="228">
       <c r="A228" t="n">
@@ -19165,6 +19391,7 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
+      <c r="H228" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" t="n">
@@ -19191,6 +19418,7 @@
           <t>5d start of a turn</t>
         </is>
       </c>
+      <c r="H229" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" t="n">
@@ -19217,6 +19445,7 @@
           <t>12.14 after an action</t>
         </is>
       </c>
+      <c r="H230" t="inlineStr"/>
     </row>
     <row r="231">
       <c r="A231" t="n">
@@ -19243,6 +19472,7 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
+      <c r="H231" t="inlineStr"/>
     </row>
     <row r="232">
       <c r="A232" t="n">
@@ -19269,6 +19499,7 @@
           <t>11.1 dolls</t>
         </is>
       </c>
+      <c r="H232" t="inlineStr"/>
     </row>
     <row r="233">
       <c r="A233" t="n">
@@ -19295,6 +19526,7 @@
           <t>12.10 random moves</t>
         </is>
       </c>
+      <c r="H233" t="inlineStr"/>
     </row>
     <row r="234">
       <c r="A234" t="n">
@@ -19321,6 +19553,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H234" t="inlineStr"/>
     </row>
     <row r="235">
       <c r="A235" t="n">
@@ -19347,6 +19580,7 @@
           <t>6b heal cap</t>
         </is>
       </c>
+      <c r="H235" t="inlineStr"/>
     </row>
     <row r="236">
       <c r="A236" t="n">
@@ -19373,6 +19607,7 @@
           <t>9 enemy AI</t>
         </is>
       </c>
+      <c r="H236" t="inlineStr"/>
     </row>
     <row r="237">
       <c r="A237" t="n">
@@ -19399,6 +19634,7 @@
           <t>12.9 after a hit</t>
         </is>
       </c>
+      <c r="H237" t="inlineStr"/>
     </row>
     <row r="238">
       <c r="A238" t="n">
@@ -19425,6 +19661,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H238" t="inlineStr"/>
     </row>
     <row r="239">
       <c r="A239" t="n">
@@ -19451,6 +19688,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H239" t="inlineStr"/>
     </row>
     <row r="240">
       <c r="A240" t="n">
@@ -19477,6 +19715,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H240" t="inlineStr"/>
     </row>
     <row r="241">
       <c r="A241" t="n">
@@ -19503,6 +19742,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H241" t="inlineStr"/>
     </row>
     <row r="242">
       <c r="A242" t="n">
@@ -19529,6 +19769,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H242" t="inlineStr"/>
     </row>
     <row r="243">
       <c r="A243" t="n">
@@ -19555,6 +19796,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H243" t="inlineStr"/>
     </row>
     <row r="244">
       <c r="A244" t="n">
@@ -19581,6 +19823,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H244" t="inlineStr"/>
     </row>
     <row r="245">
       <c r="A245" t="n">
@@ -19607,6 +19850,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H245" t="inlineStr"/>
     </row>
     <row r="246">
       <c r="A246" t="n">
@@ -19633,6 +19877,7 @@
           <t>2 physical attack, 2.1 hit chance, 3 magic attack</t>
         </is>
       </c>
+      <c r="H246" t="inlineStr"/>
     </row>
     <row r="247">
       <c r="A247" t="n">
@@ -19659,6 +19904,7 @@
           <t>2 physical attack, 2.1 hit chance, 3 magic attack</t>
         </is>
       </c>
+      <c r="H247" t="inlineStr"/>
     </row>
     <row r="248">
       <c r="A248" t="n">
@@ -19685,6 +19931,7 @@
           <t>5e effects that act every turn</t>
         </is>
       </c>
+      <c r="H248" t="inlineStr"/>
     </row>
     <row r="249">
       <c r="A249" t="n">
@@ -19711,6 +19958,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H249" t="inlineStr"/>
     </row>
     <row r="250">
       <c r="A250" t="n">
@@ -19737,6 +19985,7 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
+      <c r="H250" t="inlineStr"/>
     </row>
     <row r="251">
       <c r="A251" t="n">
@@ -19763,6 +20012,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H251" t="inlineStr"/>
     </row>
     <row r="252">
       <c r="A252" t="n">
@@ -19789,6 +20039,7 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
+      <c r="H252" t="inlineStr"/>
     </row>
     <row r="253">
       <c r="A253" t="n">
@@ -19815,6 +20066,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H253" t="inlineStr"/>
     </row>
     <row r="254">
       <c r="A254" t="n">
@@ -19841,6 +20093,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H254" t="inlineStr"/>
     </row>
     <row r="255">
       <c r="A255" t="n">
@@ -19867,6 +20120,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H255" t="inlineStr"/>
     </row>
     <row r="256">
       <c r="A256" t="n">
@@ -19893,6 +20147,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H256" t="inlineStr"/>
     </row>
     <row r="257">
       <c r="A257" t="n">
@@ -19919,6 +20174,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H257" t="inlineStr"/>
     </row>
     <row r="258">
       <c r="A258" t="n">
@@ -19945,6 +20201,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H258" t="inlineStr"/>
     </row>
     <row r="259">
       <c r="A259" t="n">
@@ -19971,6 +20228,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H259" t="inlineStr"/>
     </row>
     <row r="260">
       <c r="A260" t="n">
@@ -19997,6 +20255,7 @@
           <t>2 physical attack, 2.4 damage, 3 magic attack</t>
         </is>
       </c>
+      <c r="H260" t="inlineStr"/>
     </row>
     <row r="261">
       <c r="A261" t="n">
@@ -20023,6 +20282,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H261" t="inlineStr"/>
     </row>
     <row r="262">
       <c r="A262" t="n">
@@ -20049,6 +20309,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H262" t="inlineStr"/>
     </row>
     <row r="263">
       <c r="A263" t="n">
@@ -20075,6 +20336,7 @@
           <t>12.10 random moves</t>
         </is>
       </c>
+      <c r="H263" t="inlineStr"/>
     </row>
     <row r="264">
       <c r="A264" t="n">
@@ -20101,6 +20363,7 @@
           <t>12.10 random moves</t>
         </is>
       </c>
+      <c r="H264" t="inlineStr"/>
     </row>
     <row r="265">
       <c r="A265" t="n">
@@ -20127,6 +20390,7 @@
           <t>12.10 random moves</t>
         </is>
       </c>
+      <c r="H265" t="inlineStr"/>
     </row>
     <row r="266">
       <c r="A266" t="n">
@@ -20153,6 +20417,7 @@
           <t>6c EXP</t>
         </is>
       </c>
+      <c r="H266" t="inlineStr"/>
     </row>
     <row r="267">
       <c r="A267" t="n">
@@ -20179,6 +20444,7 @@
           <t>12.10 random moves</t>
         </is>
       </c>
+      <c r="H267" t="inlineStr"/>
     </row>
     <row r="268">
       <c r="A268" t="n">
@@ -20210,6 +20476,7 @@
           <t>0x48b490</t>
         </is>
       </c>
+      <c r="H268" t="inlineStr"/>
     </row>
     <row r="269">
       <c r="A269" t="n">
@@ -20236,6 +20503,7 @@
           <t>2.7 special damage</t>
         </is>
       </c>
+      <c r="H269" t="inlineStr"/>
     </row>
     <row r="270">
       <c r="A270" t="n">
@@ -20262,6 +20530,7 @@
           <t>2.7 special damage</t>
         </is>
       </c>
+      <c r="H270" t="inlineStr"/>
     </row>
     <row r="271">
       <c r="A271" t="n">
@@ -20288,6 +20557,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H271" t="inlineStr"/>
     </row>
     <row r="272">
       <c r="A272" t="n">
@@ -20314,6 +20584,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H272" t="inlineStr"/>
     </row>
     <row r="273">
       <c r="A273" t="n">
@@ -20340,6 +20611,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H273" t="inlineStr"/>
     </row>
     <row r="274">
       <c r="A274" t="n">
@@ -20366,6 +20638,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H274" t="inlineStr"/>
     </row>
     <row r="275">
       <c r="A275" t="n">
@@ -20392,6 +20665,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H275" t="inlineStr"/>
     </row>
     <row r="276">
       <c r="A276" t="n">
@@ -20418,6 +20692,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H276" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -27893,7 +28168,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>Heretic Samsara (enemy): when damage takes its bearer below half its max HP its value is set to 1. From then on, at each battle update of its turn, each of its eight resistance states (effects 416 to 423) is set again to 1 or 2 at random (a number below 2, plus 1)</t>
+          <t>Heretic Samsara (enemy): when damage takes its bearer below half its max HP its value is set to 1. From then on, at each battle update of its turn, each of its eight resistance states (effects 416 to 423) is put again with value (rand(2) + 1) * 50: 50 or 100 (0x438f15 - 0x438f1e). When the stats of the unit are recomputed the state of a type replaces that resistance, after its clamp (0x4fc76f - 0x4fc880). The Japanese page 317 adds that putting the bearer to sleep ends it (not read in the code, not played)</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
@@ -28543,7 +28818,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>Murder License (enemy): when the turn of its bearer comes, its action is replaced by the attack linked to the status, on a target picked at random</t>
+          <t>Murder License (enemy): at step 12 of the turn of its bearer an action is built from the skill linked to the status, on one target drawn at random (0x43736a - 0x43743a). Whether the own command of the bearer still follows, which skill is linked and its chance are not read yet; the Japanese pages 207 and 334 say that before each action of the bearer one member may die at once unless immune to instant death or of high earth resistance. An earlier wording here, that the action of the bearer is replaced, did not fit them</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">

</xml_diff>

<commit_message>
sim: R04 measured (no new mandatory class
R04 measured (no new mandatory class; the Diva is needed at the last
boss, as in vanilla)
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -21212,12 +21212,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Not run as written (each class left out in turn). The nearest measure: five parties of different make at 17 bosses, 76 of 85 pairs above the floor, and no boss where only one of them wins except C29 (Mage-Heavy 100%, the others 6 - 37%: Calliope, which the model does not play as the guide describes)</t>
+          <t>scratch/audit_2026-10-11/REGRESSION_R04.md (2026-10-12): at the 17 bosses of the battery, 27 pairs of boss and class on the variant (34 in vanilla) where every winning party of the battery holds the class. With the role of that class changed for a neighbour of the same job (60 battles), a party without it reaches the floor at 20 of the 27 (27 of 34 in vanilla): without a Diva or a Bard at 14 bosses (67 - 100%), without a Valkyrie at C29, C32, C36 and C40 (53 - 92%), without a Bishop at C29. Not reached: the Diva at C40 (the best party without her wins 22%, 13% in vanilla: needed there in vanilla too, and less so on the variant); the Sage and the Witch at C29, where only the mage party wins on either side (Calliope, which the model does not play as the guide describes); and the four base classes at C06, where five characters have joined and no other party can be made</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>partly measured</t>
+          <t>met: no new mandatory class; the Diva is needed at the last boss, as in vanilla</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: F01 reopened with its figure
F01 reopened with its figure (no party without the Maid line wins from
C30 on, in vanilla and on the variant)
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -3433,9 +3433,14 @@
           <t>A dedicated healer and buff management remain standard in hardcore DRPGs, but TP flattening (J03) and Auto-Refresh (J05) reduce Maid lock during exploration, while items and debuffers allow alternative party comps</t>
         </is>
       </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>scratch/audit_2026-10-11/no_maid_line.py (2026-10-12, 40 battles): the Meta party with a Bishop or a Sage in the place of its Diva, so that nobody of the Maid line stands in it, vanilla &gt; variant. Up to C28 it wins as the party with the Diva or little less (C17 45% &gt; 82% and 95% &gt; 98%, C26 42% &gt; 88% and 52% &gt; 98%, C28 68% &gt; 90% and 62% &gt; 95%). From C30 on it does not: C30 0% &gt; 2% and 0% &gt; 0%, C34 10% &gt; 2% and 0% &gt; 0%, C36 0% &gt; 10% and 2% &gt; 5%, C40 0% &gt; 0% both; only C38 with the Bishop moves (8% &gt; 62%). The same party with the Diva wins 88 - 100% there. With an Etoile or a Mistress, who are of the Maid line, see Regression R04</t>
+        </is>
+      </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>not a problem</t>
+          <t>open</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
@@ -3450,7 +3455,7 @@
       </c>
       <c r="P39" t="inlineStr">
         <is>
-          <t>partly true</t>
+          <t>true from C30 on, in vanilla and on the variant: no party without a member of the Maid line wins the last third of the story</t>
         </is>
       </c>
       <c r="Q39" t="inlineStr">
@@ -3460,7 +3465,7 @@
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>2026-10-10: no further change; party flexibility improved by T03 and class balance</t>
+          <t>2026-10-10: no further change; party flexibility improved by T03 and class balance; 2026-10-12: reopened, the closing held no figure; waits for the user</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: measures after the TP fruit
measures after the TP fruit: curve 37 of 44, battery 75 of 85, classes
74 of 76; F01 closed on its figures (register 0 open of 162)
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -3435,12 +3435,12 @@
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>scratch/audit_2026-10-11/no_maid_line.py (2026-10-12, 40 battles): the Meta party with a Bishop or a Sage in the place of its Diva, so that nobody of the Maid line stands in it, vanilla &gt; variant. Up to C28 it wins as the party with the Diva or little less (C17 45% &gt; 82% and 95% &gt; 98%, C26 42% &gt; 88% and 52% &gt; 98%, C28 68% &gt; 90% and 62% &gt; 95%). From C30 on it does not: C30 0% &gt; 2% and 0% &gt; 0%, C34 10% &gt; 2% and 0% &gt; 0%, C36 0% &gt; 10% and 2% &gt; 5%, C40 0% &gt; 0% both; only C38 with the Bishop moves (8% &gt; 62%). The same party with the Diva wins 88 - 100% there. With an Etoile or a Mistress, who are of the Maid line, see Regression R04</t>
+          <t>Y012 - Y014 (Magical Fruit 25 to 30 TP, Fairy Apple 50 to 60, Golden Apple 100 to 120), built and read back (1,401 of 1,401 rows). The Meta party with a Bishop in the place of its Diva, nobody of the Maid line in it (scratch/audit_2026-10-11/tp_items_trial.py, 60 battles): with the 8 fruit of the sheets 3% / 3% / 18% / 68% at C30 / C34 / C36 / C38; with 24 fruit in the bag 67% / 82% / 45% / 98% (47% / 52% / 38% / 97% before the raise). What stops such a party at C30 and C34 is TP (100% with TP at will); C36 does not turn on it, and the last boss is not won without the Maid line (0%; 45% with 99 fruit). Up to C28 the party wins 78 - 100% without her. Nothing else moved: curve 37 of 44, battery 75 of 85, classes 74 of 76, anchors 6 of 6</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
@@ -3455,17 +3455,17 @@
       </c>
       <c r="P39" t="inlineStr">
         <is>
-          <t>true from C30 on, in vanilla and on the variant: no party without a member of the Maid line wins the last third of the story</t>
+          <t>true from C30 on in vanilla; on the variant a party without the Maid line wins C30 to C38 with a bag of fruit, and needs her at the last boss</t>
         </is>
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>Solved by systemic changes in T03 and T05</t>
+          <t>Y012 - Y014: the three TP fruits of the shop x1.2</t>
         </is>
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>2026-10-10: no further change; party flexibility improved by T03 and class balance; 2026-10-12: reopened, the closing held no figure; waits for the user</t>
+          <t>2026-10-10: no further change; party flexibility improved by T03 and class balance; 2026-10-12: reopened, the closing held no figure; waits for the user; the user, 2026-10-12: a fifth more TP from the fruit and no new cut of TP costs; the Maid keeps her part and a party without her gets through with effort</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: the eighteen unique skills as rows I01 - I18
the eighteen unique skills as rows I01 - I18 (what the Japanese pages
and the English guide say, the values of the game, and the measure of
each with and without)
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R163"/>
+  <dimension ref="A1:R181"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -12454,6 +12454,1122 @@
       <c r="R163" t="inlineStr">
         <is>
           <t>2026-10-09: the doll line to the band of the Fighter and Scout lines (target 100%): cast +0.2, life +2, action speed +0.2, power x2 (Doll Master dolls) and x1.5 (Soul Summoner dolls); balance_changes.xlsx D rows</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>I01</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>JP community; GameFAQs DT2-2</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>Forerunner (Irena)</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>atwiki dt2-2 page 44: called a strong unique outright, above all with attack magic of long chant; with the crown said to fire one time in two | GameFAQs faqs/80834, Girl Unique Skills: the most powerful passive; the chance felt very high, close to 40 - 50% with the crown</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>Dominant</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>The reference party with the girl, with and without her unique skill: it adds wins, speed or HP left, and not more than the strongest of the others</t>
+        </is>
+      </c>
+      <c r="J164" t="inlineStr">
+        <is>
+          <t>Effect 358, values by rank 0.07, 0.08, 0.09, 0.1, 0.11, 0.12, 0.13, 0.14, 0.15; crown 0.2 (UniqueSkillData; rule in docs/FORMULAS.md 12.19; rank = level / 10, the crown value once the reset bonus reaches 50)</t>
+        </is>
+      </c>
+      <c r="K164" t="inlineStr">
+        <is>
+          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Irena as mage, without the skill &gt; with it): C36 84% &gt; 85%, C38 98% &gt; 95%, C40 76% &gt; 77%, P24 88% &gt; 87%, P27 crowned 49% &gt; 48%. In the mean -1 points of wins, fights +7% shorter, +1 points of HP left (a cell moves by about 5 points by chance). Read again on 2026-10-12: one roll below 100 under value * 100 for each chanted command (0x4176a0, called at 0x41d69c for a spell and at 0x419c55 for the other chanted kind, each behind a flag that keeps it to one roll): 7 - 15% by rank, 20% crowned. Both guides felt 40 - 50% with the crown</t>
+        </is>
+      </c>
+      <c r="L164" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="O164" t="inlineStr">
+        <is>
+          <t>T15 Unique skills</t>
+        </is>
+      </c>
+      <c r="P164" t="inlineStr">
+        <is>
+          <t>measured; to be read with the user</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>I02</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>JP community; GameFAQs DT2-2</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>Did You Call for Me? (Yae)</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>atwiki dt2-2 page 109: two actions are strong and easy to use in any class; with Power Charge the damage explodes; it costs more TP | GameFAQs faqs/80834, Girl Unique Skills: monstrous value as a Dark Lord when it fires during Power Charge; the extra turn does not spend buffs and cannot fire twice in a row</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>Dominant</t>
+        </is>
+      </c>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>The reference party with the girl, with and without her unique skill: it adds wins, speed or HP left, and not more than the strongest of the others</t>
+        </is>
+      </c>
+      <c r="J165" t="inlineStr">
+        <is>
+          <t>Effect 354, values by rank 0.07, 0.08, 0.09, 0.1, 0.11, 0.12, 0.13, 0.14, 0.15; crown 0.2 (UniqueSkillData; rule in docs/FORMULAS.md 12.19; rank = level / 10, the crown value once the reset bonus reaches 50)</t>
+        </is>
+      </c>
+      <c r="K165" t="inlineStr">
+        <is>
+          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Yae as dark lord, without the skill &gt; with it): C36 95% &gt; 93%, C38 91% &gt; 93%, C40 94% &gt; 94%, P24 100% &gt; 99%, P27 crowned 91% &gt; 92%. In the mean +0 points of wins, fights +3% shorter, -0 points of HP left (a cell moves by about 5 points by chance).</t>
+        </is>
+      </c>
+      <c r="L165" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="O165" t="inlineStr">
+        <is>
+          <t>T15 Unique skills</t>
+        </is>
+      </c>
+      <c r="P165" t="inlineStr">
+        <is>
+          <t>measured; to be read with the user</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>I03</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>JP community; GameFAQs DT2-2</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>Maximum Maid (Ist)</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>atwiki dt2-2 page 260: a very good unique, useful in any class; with the crown First Aid heals about half the HP at once | GameFAQs faqs/80834, Girl Unique Skills: improves every maid skill by 1 - 13%, Clean included; best as an Etoile</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>Dominant</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>The reference party with the girl, with and without her unique skill: it adds wins, speed or HP left, and not more than the strongest of the others</t>
+        </is>
+      </c>
+      <c r="J166" t="inlineStr">
+        <is>
+          <t>Effect 353, values by rank 0.01, 0.02, 0.03, 0.04, 0.05, 0.06, 0.07, 0.08, 0.1; crown 0.13 (UniqueSkillData; rule in docs/FORMULAS.md 12.19; rank = level / 10, the crown value once the reset bonus reaches 50)</t>
+        </is>
+      </c>
+      <c r="K166" t="inlineStr">
+        <is>
+          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Ist as etoile, without the skill &gt; with it): C36 74% &gt; 81%, C38 97% &gt; 97%, C40 95% &gt; 94%, P24 97% &gt; 98%, P27 crowned 68% &gt; 68%. In the mean +1 points of wins, fights +1% shorter, +0 points of HP left (a cell moves by about 5 points by chance).</t>
+        </is>
+      </c>
+      <c r="L166" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="O166" t="inlineStr">
+        <is>
+          <t>T15 Unique skills</t>
+        </is>
+      </c>
+      <c r="P166" t="inlineStr">
+        <is>
+          <t>measured; to be read with the user</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>I04</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>JP community; GameFAQs DT2-2</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>Yearning (Melvy)</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>atwiki dt2-2 page 261: brutal figures with the crown, up to +20% in all; as a Magical Princess her ATK passes 1,000 | GameFAQs faqs/80834, Girl Unique Skills: one of the few ways to make the Princess somewhat viable</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>Dominant</t>
+        </is>
+      </c>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>The reference party with the girl, with and without her unique skill: it adds wins, speed or HP left, and not more than the strongest of the others</t>
+        </is>
+      </c>
+      <c r="J167" t="inlineStr">
+        <is>
+          <t>Effect 449, values by rank 2, 3, 4, 5, 6, 7, 8, 9, 10; crown 15 (UniqueSkillData; rule in docs/FORMULAS.md 12.19; rank = level / 10, the crown value once the reset bonus reaches 50)</t>
+        </is>
+      </c>
+      <c r="K167" t="inlineStr">
+        <is>
+          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Melvy as magical princess, without the skill &gt; with it): C36 82% &gt; 83%, C38 98% &gt; 99%, C40 74% &gt; 72%, P24 82% &gt; 79%, P27 crowned 58% &gt; 57%. In the mean -1 points of wins, fights +2% shorter, -1 points of HP left (a cell moves by about 5 points by chance).</t>
+        </is>
+      </c>
+      <c r="L167" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="O167" t="inlineStr">
+        <is>
+          <t>T15 Unique skills</t>
+        </is>
+      </c>
+      <c r="P167" t="inlineStr">
+        <is>
+          <t>measured; to be read with the user</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>I05</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>JP community; GameFAQs DT2-2</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>Demon Wall (Mefmera)</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>atwiki dt2-2 page 253: depends on the enemy but a strong unique; at a high level it cuts a lot | GameFAQs faqs/80834, Girl Unique Skills: the cut is noticeable, but few endgame bosses are of those races</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>The reference party with the girl, with and without her unique skill: it adds wins, speed or HP left, and not more than the strongest of the others</t>
+        </is>
+      </c>
+      <c r="J168" t="inlineStr">
+        <is>
+          <t>Effect 356, values by rank -0.12, -0.13, -0.14, -0.15, -0.16, -0.17, -0.18, -0.19, -0.2; crown -0.25 (UniqueSkillData; rule in docs/FORMULAS.md 12.19; rank = level / 10, the crown value once the reset bonus reaches 50)</t>
+        </is>
+      </c>
+      <c r="K168" t="inlineStr">
+        <is>
+          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Mefmera as papillon, without the skill &gt; with it): C36 82% &gt; 88%, C38 98% &gt; 100%, C40 87% &gt; 95%, P24 93% &gt; 98%, P27 crowned 88% &gt; 98%. In the mean +6 points of wins, fights +3% shorter, +6 points of HP left (a cell moves by about 5 points by chance). It cuts the damage of demons, undead and apparitions: Samael (C38) and Melek Taus (P27) are demons; the race of the others was not checked against its list</t>
+        </is>
+      </c>
+      <c r="L168" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="O168" t="inlineStr">
+        <is>
+          <t>T15 Unique skills</t>
+        </is>
+      </c>
+      <c r="P168" t="inlineStr">
+        <is>
+          <t>measured; to be read with the user</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>I06</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>JP community; GameFAQs DT2-2</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>Wreathed in Glory (Eltricia)</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>atwiki dt2-2 page 229: crowned and with high AGI it is always her turn; worse for casters of long chants since it no longer shortens the chant | GameFAQs faqs/80834, Girl Unique Skills: the less time spent chanting the more it gives; pairs with the best grand sealbook of casters</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>The reference party with the girl, with and without her unique skill: it adds wins, speed or HP left, and not more than the strongest of the others</t>
+        </is>
+      </c>
+      <c r="J169" t="inlineStr">
+        <is>
+          <t>Effect 352, values by rank 0.07, 0.08, 0.09, 0.1, 0.11, 0.12, 0.13, 0.14, 0.15; crown 0.2 (UniqueSkillData; rule in docs/FORMULAS.md 12.19; rank = level / 10, the crown value once the reset bonus reaches 50)</t>
+        </is>
+      </c>
+      <c r="K169" t="inlineStr">
+        <is>
+          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Eltricia as magical princess, without the skill &gt; with it): C36 82% &gt; 88%, C38 98% &gt; 97%, C40 74% &gt; 76%, P24 82% &gt; 75%, P27 crowned 58% &gt; 64%. In the mean +1 points of wins, fights +1% shorter, +1 points of HP left (a cell moves by about 5 points by chance).</t>
+        </is>
+      </c>
+      <c r="L169" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="O169" t="inlineStr">
+        <is>
+          <t>T15 Unique skills</t>
+        </is>
+      </c>
+      <c r="P169" t="inlineStr">
+        <is>
+          <t>measured; to be read with the user</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>I07</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>JP community; GameFAQs DT2-2</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>Positive Trance (Alisia)</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>atwiki dt2-2 page 230: always on, so her damage is stable; weak against bosses that take Pep, and escaping lowers it | GameFAQs faqs/80834, Girl Unique Skills: about +15% damage at level 90 from the default Pep to the maximum; on par with Yae and Luco in mean power</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>The reference party with the girl, with and without her unique skill: it adds wins, speed or HP left, and not more than the strongest of the others</t>
+        </is>
+      </c>
+      <c r="J170" t="inlineStr">
+        <is>
+          <t>Effect 440, values by rank 10, 9, 8, 7, 6, 5, 4, 3, 2; crown 1 (UniqueSkillData; rule in docs/FORMULAS.md 12.19; rank = level / 10, the crown value once the reset bonus reaches 50)</t>
+        </is>
+      </c>
+      <c r="K170" t="inlineStr">
+        <is>
+          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Alisia as attacker, without the skill &gt; with it): C36 92% &gt; 91%, C38 82% &gt; 84%, C40 40% &gt; 49%, P24 98% &gt; 98%, P27 crowned 65% &gt; 65%. In the mean +2 points of wins, fights +2% shorter, +2 points of HP left (a cell moves by about 5 points by chance). The simulator holds Pep at 100; she was played at Pep 130, the most it can be, so this is the most the skill gives: +6% damage at rank 5 - 6, +15% at rank 9, +30% crowned (the guide measured about +15% at level 90)</t>
+        </is>
+      </c>
+      <c r="L170" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="O170" t="inlineStr">
+        <is>
+          <t>T15 Unique skills</t>
+        </is>
+      </c>
+      <c r="P170" t="inlineStr">
+        <is>
+          <t>measured; to be read with the user</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>I08</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>JP community; GameFAQs DT2-2</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>Shadow Heart (Luco)</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>atwiki dt2-2 page 43: the shadow strikes with about twice her attack for three actions; low chance (about 5% at rank 1); a fault: if the shadow drains HP or TP its attack falls back to hers | GameFAQs faqs/80834, Girl Unique Skills: very powerful for a long while, falls off a little in the very late game; chance about 5% +1% a rank</t>
+        </is>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="H171" t="inlineStr">
+        <is>
+          <t>The reference party with the girl, with and without her unique skill: it adds wins, speed or HP left, and not more than the strongest of the others</t>
+        </is>
+      </c>
+      <c r="J171" t="inlineStr">
+        <is>
+          <t>Effect 448, values by rank 0.04, 0.05, 0.06, 0.07, 0.08, 0.09, 0.1, 0.11, 0.12; crown 0.2 (UniqueSkillData; rule in docs/FORMULAS.md 12.19; rank = level / 10, the crown value once the reset bonus reaches 50)</t>
+        </is>
+      </c>
+      <c r="K171" t="inlineStr">
+        <is>
+          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Luco as dark lord, without the skill &gt; with it): C36 82% &gt; 79%, C38 98% &gt; 99%, C40 83% &gt; 74%, P24 95% &gt; 93%, P27 crowned 82% &gt; 80%. In the mean -3 points of wins, fights +1% shorter, -3 points of HP left (a cell moves by about 5 points by chance). The fault the Japanese page tells (the attack of the shadow falling back when it drains HP or TP) is neither read in the program nor played</t>
+        </is>
+      </c>
+      <c r="L171" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="O171" t="inlineStr">
+        <is>
+          <t>T15 Unique skills</t>
+        </is>
+      </c>
+      <c r="P171" t="inlineStr">
+        <is>
+          <t>measured; to be read with the user</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>I09</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>JP community; GameFAQs DT2-2</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>Furious Strike (Grishna)</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>atwiki dt2-2 page 257: useful for any attacker; best with strikes of many hits (Samurai, attacking Valkyrie) | GameFAQs faqs/80834, Girl Unique Skills: a slight buff from the first game that hardly matters; best with Daedalus Attack</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>The reference party with the girl, with and without her unique skill: it adds wins, speed or HP left, and not more than the strongest of the others</t>
+        </is>
+      </c>
+      <c r="J172" t="inlineStr">
+        <is>
+          <t>Effect 348, values by rank 0.12, 0.13, 0.14, 0.15, 0.16, 0.17, 0.18, 0.19, 0.2; crown 0.3 (UniqueSkillData; rule in docs/FORMULAS.md 12.19; rank = level / 10, the crown value once the reset bonus reaches 50)</t>
+        </is>
+      </c>
+      <c r="K172" t="inlineStr">
+        <is>
+          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Grishna as attacker, without the skill &gt; with it): C36 91% &gt; 87%, C38 92% &gt; 94%, C40 76% &gt; 67%, P24 86% &gt; 89%, P27 crowned 63% &gt; 71%. In the mean -0 points of wins, fights +2% shorter, -2 points of HP left (a cell moves by about 5 points by chance).</t>
+        </is>
+      </c>
+      <c r="L172" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="O172" t="inlineStr">
+        <is>
+          <t>T15 Unique skills</t>
+        </is>
+      </c>
+      <c r="P172" t="inlineStr">
+        <is>
+          <t>measured; to be read with the user</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>I10</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>JP community; GameFAQs DT2-2</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>Elbow Grease (Monica)</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>atwiki dt2-2 page 254: the highest weapon damage of the Scout line; wasted as a Kunoichi, who turns to ninjutsu | GameFAQs faqs/80834, Girl Unique Skills: felt like a chance of +20 - 25% damage with no pattern he could find; pure damage scouts are weak anyway</t>
+        </is>
+      </c>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="H173" t="inlineStr">
+        <is>
+          <t>The reference party with the girl, with and without her unique skill: it adds wins, speed or HP left, and not more than the strongest of the others</t>
+        </is>
+      </c>
+      <c r="J173" t="inlineStr">
+        <is>
+          <t>Effect 443, values by rank 0.1, 0.11, 0.12, 0.13, 0.14, 0.15, 0.16, 0.17, 0.18; crown 0.25 (UniqueSkillData; rule in docs/FORMULAS.md 12.19; rank = level / 10, the crown value once the reset bonus reaches 50)</t>
+        </is>
+      </c>
+      <c r="K173" t="inlineStr">
+        <is>
+          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Monica as shooter, without the skill &gt; with it): C36 81% &gt; 83%, C38 96% &gt; 95%, C40 63% &gt; 66%, P24 89% &gt; 90%, P27 crowned 44% &gt; 46%. In the mean +1 points of wins, fights +6% shorter, +0 points of HP left (a cell moves by about 5 points by chance).</t>
+        </is>
+      </c>
+      <c r="L173" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="O173" t="inlineStr">
+        <is>
+          <t>T15 Unique skills</t>
+        </is>
+      </c>
+      <c r="P173" t="inlineStr">
+        <is>
+          <t>measured; to be read with the user</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>I11</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>JP community; GameFAQs DT2-2</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>Usurper of Souls (Lizerietta)</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>atwiki dt2-2 page 107: a good skill of narrow use: it takes turns from bosses that summon | GameFAQs faqs/80834, Girl Unique Skills: nice against bosses with familiars or dolls, useless outside of them; the chance is pretty high</t>
+        </is>
+      </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="H174" t="inlineStr">
+        <is>
+          <t>The reference party with the girl, with and without her unique skill: it adds wins, speed or HP left, and not more than the strongest of the others</t>
+        </is>
+      </c>
+      <c r="J174" t="inlineStr">
+        <is>
+          <t>Effect 350, values by rank 0.25, 0.29, 0.33, 0.37, 0.41, 0.45, 0.49, 0.53, 0.57; crown 0.75 (UniqueSkillData; rule in docs/FORMULAS.md 12.19; rank = level / 10, the crown value once the reset bonus reaches 50)</t>
+        </is>
+      </c>
+      <c r="K174" t="inlineStr">
+        <is>
+          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Lizerietta as papillon, without the skill &gt; with it): C36 99% &gt; 92%, C38 96% &gt; 94%, C40 89% &gt; 93%, P24 100% &gt; 100%, P27 crowned 86% &gt; 86%. In the mean -1 points of wins, fights -1% shorter, -1 points of HP left (a cell moves by about 5 points by chance). It only acts on what an enemy summons; which of these five fights hold a summoner was not looked at</t>
+        </is>
+      </c>
+      <c r="L174" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="O174" t="inlineStr">
+        <is>
+          <t>T15 Unique skills</t>
+        </is>
+      </c>
+      <c r="P174" t="inlineStr">
+        <is>
+          <t>measured; to be read with the user</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>I12</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>JP community; GameFAQs DT2-2</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>Overstock Clearance (Souffle)</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>atwiki dt2-2 page 255: only a Treasure Hunter gets the most of it | GameFAQs faqs/80834, Girl Unique Skills: its line damage item is massive when she joins and next to nothing late; her worth is her party skills</t>
+        </is>
+      </c>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="H175" t="inlineStr">
+        <is>
+          <t>The reference party with the girl, with and without her unique skill: it adds wins, speed or HP left, and not more than the strongest of the others</t>
+        </is>
+      </c>
+      <c r="J175" t="inlineStr">
+        <is>
+          <t>Effect 446, values by rank 0.1, 0.11, 0.12, 0.13, 0.14, 0.15, 0.16, 0.17, 0.18; crown 0.25 (UniqueSkillData; rule in docs/FORMULAS.md 12.19; rank = level / 10, the crown value once the reset bonus reaches 50)</t>
+        </is>
+      </c>
+      <c r="K175" t="inlineStr">
+        <is>
+          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Souffle as treasure hunter, without the skill &gt; with it): C36 85% &gt; 92%, C38 86% &gt; 94%, C40 95% &gt; 92%, P24 100% &gt; 99%, P27 crowned 86% &gt; 83%. In the mean +2 points of wins, fights +2% shorter, +1 points of HP left (a cell moves by about 5 points by chance).</t>
+        </is>
+      </c>
+      <c r="L175" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="O175" t="inlineStr">
+        <is>
+          <t>T15 Unique skills</t>
+        </is>
+      </c>
+      <c r="P175" t="inlineStr">
+        <is>
+          <t>measured; to be read with the user</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>I13</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>JP community; GameFAQs DT2-2</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>Sugar Coma (Conette)</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>atwiki dt2-2 page 111: a little stronger than in the first game (the speed cut lands often); only in the front row | GameFAQs faqs/80834, Girl Unique Skills: a great effect even when the slow is blocked; needs her in front taking hits</t>
+        </is>
+      </c>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="H176" t="inlineStr">
+        <is>
+          <t>The reference party with the girl, with and without her unique skill: it adds wins, speed or HP left, and not more than the strongest of the others</t>
+        </is>
+      </c>
+      <c r="J176" t="inlineStr">
+        <is>
+          <t>Effect 346, values by rank 0.16, 0.18, 0.2, 0.22, 0.24, 0.27, 0.3, 0.34, 0.38; crown 0.5 (UniqueSkillData; rule in docs/FORMULAS.md 12.19; rank = level / 10, the crown value once the reset bonus reaches 50)</t>
+        </is>
+      </c>
+      <c r="K176" t="inlineStr">
+        <is>
+          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Conette as mistress, without the skill &gt; with it): C36 75% &gt; 83%, C38 98% &gt; 97%, C40 93% &gt; 97%, P24 97% &gt; 97%, P27 crowned 63% &gt; 84%. In the mean +6 points of wins, fights +2% shorter, +8 points of HP left (a cell moves by about 5 points by chance).</t>
+        </is>
+      </c>
+      <c r="L176" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="O176" t="inlineStr">
+        <is>
+          <t>T15 Unique skills</t>
+        </is>
+      </c>
+      <c r="P176" t="inlineStr">
+        <is>
+          <t>measured; to be read with the user</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>I14</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>JP community; GameFAQs DT2-2</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>Alter Fate (Fiora)</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>atwiki dt2-2 page 259: an insurance | GameFAQs faqs/80834, Girl Unique Skills: the common 5 - 20% chance; nothing more said</t>
+        </is>
+      </c>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="H177" t="inlineStr">
+        <is>
+          <t>The reference party with the girl, with and without her unique skill: it adds wins, speed or HP left, and not more than the strongest of the others</t>
+        </is>
+      </c>
+      <c r="J177" t="inlineStr">
+        <is>
+          <t>Effect 349, values by rank 0.07, 0.08, 0.09, 0.1, 0.11, 0.12, 0.13, 0.14, 0.15; crown 0.2 (UniqueSkillData; rule in docs/FORMULAS.md 12.19; rank = level / 10, the crown value once the reset bonus reaches 50)</t>
+        </is>
+      </c>
+      <c r="K177" t="inlineStr">
+        <is>
+          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Fiora as healer, without the skill &gt; with it): C36 90% &gt; 86%, C38 94% &gt; 97%, C40 95% &gt; 97%, P24 98% &gt; 99%, P27 crowned 73% &gt; 81%. In the mean +2 points of wins, fights +1% shorter, +3 points of HP left (a cell moves by about 5 points by chance).</t>
+        </is>
+      </c>
+      <c r="L177" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="O177" t="inlineStr">
+        <is>
+          <t>T15 Unique skills</t>
+        </is>
+      </c>
+      <c r="P177" t="inlineStr">
+        <is>
+          <t>measured; to be read with the user</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>I15</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>JP community; GameFAQs DT2-2</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>Tranquil Song (Yuni)</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>atwiki dt2-2 page 97: the debuff now ends after a few turns: a fix or a plain nerf; fine for a Maid line girl | GameFAQs faqs/80834, Girl Unique Skills: a slight indirect nerf since debuffs no longer last for ever; it also overwrites the ATK and INT buffs of the enemy</t>
+        </is>
+      </c>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>Dead</t>
+        </is>
+      </c>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t>The reference party with the girl, with and without her unique skill: it adds wins, speed or HP left, and not more than the strongest of the others</t>
+        </is>
+      </c>
+      <c r="J178" t="inlineStr">
+        <is>
+          <t>Effect 357, values by rank 0.07, 0.07, 0.08, 0.08, 0.09, 0.1, 0.11, 0.12, 0.13; crown 0.2 (UniqueSkillData; rule in docs/FORMULAS.md 12.19; rank = level / 10, the crown value once the reset bonus reaches 50)</t>
+        </is>
+      </c>
+      <c r="K178" t="inlineStr">
+        <is>
+          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Yuni as diva, without the skill &gt; with it): C36 98% &gt; 93%, C38 89% &gt; 94%, C40 90% &gt; 91%, P24 94% &gt; 99%, P27 crowned 85% &gt; 93%. In the mean +3 points of wins, fights +2% shorter, +3 points of HP left (a cell moves by about 5 points by chance).</t>
+        </is>
+      </c>
+      <c r="L178" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="O178" t="inlineStr">
+        <is>
+          <t>T15 Unique skills</t>
+        </is>
+      </c>
+      <c r="P178" t="inlineStr">
+        <is>
+          <t>measured; to be read with the user</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>I16</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>JP community; GameFAQs DT2-2</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>Third Eye Wide (Lilian)</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>atwiki dt2-2 page 258: the ailment may be blocked by resistances, and the dispel does not fire as of version 1.05 (a bug) | GameFAQs faqs/80834, Girl Unique Skills: the dispel is useful at the right moment but that is very rare; less useful late since most enemies are immune</t>
+        </is>
+      </c>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>Dead</t>
+        </is>
+      </c>
+      <c r="H179" t="inlineStr">
+        <is>
+          <t>The reference party with the girl, with and without her unique skill: it adds wins, speed or HP left, and not more than the strongest of the others</t>
+        </is>
+      </c>
+      <c r="J179" t="inlineStr">
+        <is>
+          <t>Effect 345, values by rank 0.07, 0.08, 0.09, 0.1, 0.11, 0.12, 0.13, 0.14, 0.15; crown 0.25 (UniqueSkillData; rule in docs/FORMULAS.md 12.19; rank = level / 10, the crown value once the reset bonus reaches 50)</t>
+        </is>
+      </c>
+      <c r="K179" t="inlineStr">
+        <is>
+          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Lilian as soul summoner, without the skill &gt; with it): C36 83% &gt; 83%, C38 87% &gt; 96%, C40 64% &gt; 74%, P24 80% &gt; 83%, P27 crowned 53% &gt; 55%. In the mean +5 points of wins, fights +1% shorter, +6 points of HP left (a cell moves by about 5 points by chance). The program draws one of seven results, the dispel among them (0x43697b); the Japanese page says the dispel never fires in version 1.05 and the English guide says it does: not settled</t>
+        </is>
+      </c>
+      <c r="L179" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="O179" t="inlineStr">
+        <is>
+          <t>T15 Unique skills</t>
+        </is>
+      </c>
+      <c r="P179" t="inlineStr">
+        <is>
+          <t>measured; to be read with the user</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>I17</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>JP community; GameFAQs DT2-2</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>Undaunted Spirit (Tsurara)</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>atwiki dt2-2 page 41: she rises with 1 HP at a time nobody can tell, so it is lost unless healed at once, and it gets in the way of Resurrect | GameFAQs faqs/80834, Girl Unique Skills: kind of pointless: a revive item costs almost no time and is more reliable</t>
+        </is>
+      </c>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>Dead</t>
+        </is>
+      </c>
+      <c r="H180" t="inlineStr">
+        <is>
+          <t>The reference party with the girl, with and without her unique skill: it adds wins, speed or HP left, and not more than the strongest of the others</t>
+        </is>
+      </c>
+      <c r="J180" t="inlineStr">
+        <is>
+          <t>Effect 355, values by rank 0.08, 0.1, 0.12, 0.14, 0.16, 0.18, 0.2, 0.22, 0.24; crown 0.3 (UniqueSkillData; rule in docs/FORMULAS.md 12.19; rank = level / 10, the crown value once the reset bonus reaches 50)</t>
+        </is>
+      </c>
+      <c r="K180" t="inlineStr">
+        <is>
+          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Tsurara as treasure hunter, without the skill &gt; with it): C36 85% &gt; 94%, C38 86% &gt; 90%, C40 95% &gt; 92%, P24 100% &gt; 100%, P27 crowned 86% &gt; 97%. In the mean +4 points of wins, fights -1% shorter, +2 points of HP left (a cell moves by about 5 points by chance).</t>
+        </is>
+      </c>
+      <c r="L180" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="O180" t="inlineStr">
+        <is>
+          <t>T15 Unique skills</t>
+        </is>
+      </c>
+      <c r="P180" t="inlineStr">
+        <is>
+          <t>measured; to be read with the user</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>I18</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>JP community; GameFAQs DT2-2</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>Arcane Shield (Siena)</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>atwiki dt2-2 page 42: never useless in a class, never of real use either; a comment asks why such a pointless unique was left | GameFAQs faqs/80834, Girl Unique Skills: chance always about 15%, the share reflected from 50% to 200%; true damage; best in the front row</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>Dead</t>
+        </is>
+      </c>
+      <c r="H181" t="inlineStr">
+        <is>
+          <t>The reference party with the girl, with and without her unique skill: it adds wins, speed or HP left, and not more than the strongest of the others</t>
+        </is>
+      </c>
+      <c r="J181" t="inlineStr">
+        <is>
+          <t>Effect 447, values by rank 0.5, 0.55, 0.6, 0.65, 0.7, 0.75, 0.8, 0.9, 1; crown 2 (UniqueSkillData; rule in docs/FORMULAS.md 12.19; rank = level / 10, the crown value once the reset bonus reaches 50)</t>
+        </is>
+      </c>
+      <c r="K181" t="inlineStr">
+        <is>
+          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Siena as magical princess, without the skill &gt; with it): C36 82% &gt; 82%, C38 98% &gt; 97%, C40 74% &gt; 81%, P24 82% &gt; 83%, P27 crowned 58% &gt; 67%. In the mean +3 points of wins, fights -1% shorter, +2 points of HP left (a cell moves by about 5 points by chance).</t>
+        </is>
+      </c>
+      <c r="L181" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="O181" t="inlineStr">
+        <is>
+          <t>T15 Unique skills</t>
+        </is>
+      </c>
+      <c r="P181" t="inlineStr">
+        <is>
+          <t>measured; to be read with the user</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
sim: the shadow of Shadow Heart
the shadow of Shadow Heart, the second action of Did You Call for Me?
and the dispel of Third Eye Wide played as read; the catalogue of
fields: item pairs, meals and spell accuracy verified; the unique skills
measured again
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -12500,7 +12500,7 @@
       </c>
       <c r="K164" t="inlineStr">
         <is>
-          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Irena as mage, without the skill &gt; with it): C36 84% &gt; 85%, C38 98% &gt; 95%, C40 76% &gt; 77%, P24 88% &gt; 87%, P27 crowned 49% &gt; 48%. In the mean -1 points of wins, fights +7% shorter, +1 points of HP left (a cell moves by about 5 points by chance). Read again on 2026-10-12: one roll below 100 under value * 100 for each chanted command (0x4176a0, called at 0x41d69c for a spell and at 0x419c55 for the other chanted kind, each behind a flag that keeps it to one roll): 7 - 15% by rank, 20% crowned. Both guides felt 40 - 50% with the crown</t>
+          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Irena as mage, without the skill &gt; with it): C36 87% &gt; 88%, C38 98% &gt; 95%, C40 78% &gt; 75%, P24 88% &gt; 86%, P27 crowned 51% &gt; 52%. In the mean -1 points of wins, fights +4% shorter, -1 points of HP left (a cell moves by about 5 points by chance). Read again on 2026-10-12: one roll below 100 under value * 100 for each chanted command (0x4176a0, called at 0x41d69c for a spell and at 0x419c55 for the other chanted kind, each behind a flag that keeps it to one roll): 7 - 15% by rank, 20% crowned. Both guides felt 40 - 50% with the crown</t>
         </is>
       </c>
       <c r="L164" t="inlineStr">
@@ -12562,7 +12562,7 @@
       </c>
       <c r="K165" t="inlineStr">
         <is>
-          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Yae as dark lord, without the skill &gt; with it): C36 95% &gt; 93%, C38 91% &gt; 93%, C40 94% &gt; 94%, P24 100% &gt; 99%, P27 crowned 91% &gt; 92%. In the mean +0 points of wins, fights +3% shorter, -0 points of HP left (a cell moves by about 5 points by chance).</t>
+          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Yae as dark lord, without the skill &gt; with it): C36 95% &gt; 93%, C38 91% &gt; 95%, C40 94% &gt; 96%, P24 100% &gt; 99%, P27 crowned 91% &gt; 92%. In the mean +1 points of wins, fights +7% shorter, -0 points of HP left (a cell moves by about 5 points by chance). Played since 2026-10-12 as read: the second action belongs to the same turn, so her statuses do not lose a turn between the two (Power Charge serves both blows)</t>
         </is>
       </c>
       <c r="L165" t="inlineStr">
@@ -12624,7 +12624,7 @@
       </c>
       <c r="K166" t="inlineStr">
         <is>
-          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Ist as etoile, without the skill &gt; with it): C36 74% &gt; 81%, C38 97% &gt; 97%, C40 95% &gt; 94%, P24 97% &gt; 98%, P27 crowned 68% &gt; 68%. In the mean +1 points of wins, fights +1% shorter, +0 points of HP left (a cell moves by about 5 points by chance).</t>
+          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Ist as etoile, without the skill &gt; with it): C36 76% &gt; 83%, C38 96% &gt; 98%, C40 96% &gt; 97%, P24 98% &gt; 99%, P27 crowned 71% &gt; 72%. In the mean +2 points of wins, fights +0% shorter, +2 points of HP left (a cell moves by about 5 points by chance).</t>
         </is>
       </c>
       <c r="L166" t="inlineStr">
@@ -12686,7 +12686,7 @@
       </c>
       <c r="K167" t="inlineStr">
         <is>
-          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Melvy as magical princess, without the skill &gt; with it): C36 82% &gt; 83%, C38 98% &gt; 99%, C40 74% &gt; 72%, P24 82% &gt; 79%, P27 crowned 58% &gt; 57%. In the mean -1 points of wins, fights +2% shorter, -1 points of HP left (a cell moves by about 5 points by chance).</t>
+          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Melvy as magical princess, without the skill &gt; with it): C36 79% &gt; 82%, C38 99% &gt; 100%, C40 76% &gt; 73%, P24 85% &gt; 79%, P27 crowned 64% &gt; 63%. In the mean -1 points of wins, fights +2% shorter, -2 points of HP left (a cell moves by about 5 points by chance).</t>
         </is>
       </c>
       <c r="L167" t="inlineStr">
@@ -12748,7 +12748,7 @@
       </c>
       <c r="K168" t="inlineStr">
         <is>
-          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Mefmera as papillon, without the skill &gt; with it): C36 82% &gt; 88%, C38 98% &gt; 100%, C40 87% &gt; 95%, P24 93% &gt; 98%, P27 crowned 88% &gt; 98%. In the mean +6 points of wins, fights +3% shorter, +6 points of HP left (a cell moves by about 5 points by chance). It cuts the damage of demons, undead and apparitions: Samael (C38) and Melek Taus (P27) are demons; the race of the others was not checked against its list</t>
+          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Mefmera as papillon, without the skill &gt; with it): C36 81% &gt; 84%, C38 97% &gt; 100%, C40 86% &gt; 95%, P24 94% &gt; 98%, P27 crowned 89% &gt; 98%. In the mean +6 points of wins, fights +4% shorter, +5 points of HP left (a cell moves by about 5 points by chance). It cuts the damage of demons, undead and apparitions: Samael (C38) and Melek Taus (P27) are demons; the race of the others was not checked against its list</t>
         </is>
       </c>
       <c r="L168" t="inlineStr">
@@ -12810,7 +12810,7 @@
       </c>
       <c r="K169" t="inlineStr">
         <is>
-          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Eltricia as magical princess, without the skill &gt; with it): C36 82% &gt; 88%, C38 98% &gt; 97%, C40 74% &gt; 76%, P24 82% &gt; 75%, P27 crowned 58% &gt; 64%. In the mean +1 points of wins, fights +1% shorter, +1 points of HP left (a cell moves by about 5 points by chance).</t>
+          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Eltricia as magical princess, without the skill &gt; with it): C36 79% &gt; 89%, C38 99% &gt; 97%, C40 76% &gt; 75%, P24 85% &gt; 78%, P27 crowned 64% &gt; 68%. In the mean +1 points of wins, fights +1% shorter, -0 points of HP left (a cell moves by about 5 points by chance).</t>
         </is>
       </c>
       <c r="L169" t="inlineStr">
@@ -12872,7 +12872,7 @@
       </c>
       <c r="K170" t="inlineStr">
         <is>
-          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Alisia as attacker, without the skill &gt; with it): C36 92% &gt; 91%, C38 82% &gt; 84%, C40 40% &gt; 49%, P24 98% &gt; 98%, P27 crowned 65% &gt; 65%. In the mean +2 points of wins, fights +2% shorter, +2 points of HP left (a cell moves by about 5 points by chance). The simulator holds Pep at 100; she was played at Pep 130, the most it can be, so this is the most the skill gives: +6% damage at rank 5 - 6, +15% at rank 9, +30% crowned (the guide measured about +15% at level 90)</t>
+          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Alisia as attacker, without the skill &gt; with it): C36 93% &gt; 91%, C38 80% &gt; 82%, C40 45% &gt; 49%, P24 99% &gt; 98%, P27 crowned 69% &gt; 68%. In the mean +0 points of wins, fights +2% shorter, -0 points of HP left (a cell moves by about 5 points by chance). The simulator holds Pep at 100; she was played at Pep 130, the most it can be, so this is the most the skill gives: +6% damage at rank 5 - 6, +15% at rank 9, +30% crowned (the guide measured about +15% at level 90)</t>
         </is>
       </c>
       <c r="L170" t="inlineStr">
@@ -12934,7 +12934,7 @@
       </c>
       <c r="K171" t="inlineStr">
         <is>
-          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Luco as dark lord, without the skill &gt; with it): C36 82% &gt; 79%, C38 98% &gt; 99%, C40 83% &gt; 74%, P24 95% &gt; 93%, P27 crowned 82% &gt; 80%. In the mean -3 points of wins, fights +1% shorter, -3 points of HP left (a cell moves by about 5 points by chance). The fault the Japanese page tells (the attack of the shadow falling back when it drains HP or TP) is neither read in the program nor played Read on 2026-10-12 (0x4fe2e0): the shadow is built by the doll constructor and then walks a list of statuses of its own, keeping some and dropping others, so it does carry statuses of its owner, as both guides say (the buffs she holds when it appears, Double and Triple Attack). The simulator gives it the base stats of its owner and no status at all: this measure is a floor, not the worth of the skill. Which statuses stay, and whether its attack is twice hers, are not read</t>
+          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Luco as dark lord, without the skill &gt; with it): C36 82% &gt; 88%, C38 98% &gt; 100%, C40 88% &gt; 86%, P24 95% &gt; 90%, P27 crowned 83% &gt; 77%. In the mean -1 points of wins, fights +8% shorter, -1 points of HP left (a cell moves by about 5 points by chance). Played since 2026-10-12 as read (scratch/qol_fields_reading.md 5, checked): the shadow has the stats of its owner at that moment with twice the ATK, her passives, none of the statuses techniques put, a life of 3. The fault the Japanese page tells (its attack falling back after a drain) is not in the program by that reading</t>
         </is>
       </c>
       <c r="L171" t="inlineStr">
@@ -12996,7 +12996,7 @@
       </c>
       <c r="K172" t="inlineStr">
         <is>
-          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Grishna as attacker, without the skill &gt; with it): C36 91% &gt; 87%, C38 92% &gt; 94%, C40 76% &gt; 67%, P24 86% &gt; 89%, P27 crowned 63% &gt; 71%. In the mean -0 points of wins, fights +2% shorter, -2 points of HP left (a cell moves by about 5 points by chance).</t>
+          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Grishna as attacker, without the skill &gt; with it): C36 90% &gt; 88%, C38 98% &gt; 97%, C40 71% &gt; 72%, P24 87% &gt; 89%, P27 crowned 67% &gt; 75%. In the mean +2 points of wins, fights +4% shorter, +0 points of HP left (a cell moves by about 5 points by chance).</t>
         </is>
       </c>
       <c r="L172" t="inlineStr">
@@ -13058,7 +13058,7 @@
       </c>
       <c r="K173" t="inlineStr">
         <is>
-          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Monica as shooter, without the skill &gt; with it): C36 81% &gt; 83%, C38 96% &gt; 95%, C40 63% &gt; 66%, P24 89% &gt; 90%, P27 crowned 44% &gt; 46%. In the mean +1 points of wins, fights +6% shorter, +0 points of HP left (a cell moves by about 5 points by chance).</t>
+          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Monica as shooter, without the skill &gt; with it): C36 81% &gt; 89%, C38 97% &gt; 98%, C40 76% &gt; 72%, P24 86% &gt; 88%, P27 crowned 50% &gt; 53%. In the mean +2 points of wins, fights +6% shorter, +2 points of HP left (a cell moves by about 5 points by chance).</t>
         </is>
       </c>
       <c r="L173" t="inlineStr">
@@ -13120,7 +13120,7 @@
       </c>
       <c r="K174" t="inlineStr">
         <is>
-          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Lizerietta as papillon, without the skill &gt; with it): C36 99% &gt; 92%, C38 96% &gt; 94%, C40 89% &gt; 93%, P24 100% &gt; 100%, P27 crowned 86% &gt; 86%. In the mean -1 points of wins, fights -1% shorter, -1 points of HP left (a cell moves by about 5 points by chance). It only acts on what an enemy summons; which of these five fights hold a summoner was not looked at</t>
+          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Lizerietta as papillon, without the skill &gt; with it): C36 95% &gt; 92%, C38 96% &gt; 97%, C40 96% &gt; 96%, P24 100% &gt; 100%, P27 crowned 85% &gt; 86%. In the mean -0 points of wins, fights -2% shorter, -1 points of HP left (a cell moves by about 5 points by chance). It only acts on what an enemy summons; which of these five fights hold a summoner was not looked at</t>
         </is>
       </c>
       <c r="L174" t="inlineStr">
@@ -13182,7 +13182,7 @@
       </c>
       <c r="K175" t="inlineStr">
         <is>
-          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Souffle as treasure hunter, without the skill &gt; with it): C36 85% &gt; 92%, C38 86% &gt; 94%, C40 95% &gt; 92%, P24 100% &gt; 99%, P27 crowned 86% &gt; 83%. In the mean +2 points of wins, fights +2% shorter, +1 points of HP left (a cell moves by about 5 points by chance).</t>
+          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Souffle as treasure hunter, without the skill &gt; with it): C36 87% &gt; 94%, C38 91% &gt; 96%, C40 91% &gt; 94%, P24 100% &gt; 99%, P27 crowned 86% &gt; 85%. In the mean +3 points of wins, fights +4% shorter, +4 points of HP left (a cell moves by about 5 points by chance).</t>
         </is>
       </c>
       <c r="L175" t="inlineStr">
@@ -13244,7 +13244,7 @@
       </c>
       <c r="K176" t="inlineStr">
         <is>
-          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Conette as mistress, without the skill &gt; with it): C36 75% &gt; 83%, C38 98% &gt; 97%, C40 93% &gt; 97%, P24 97% &gt; 97%, P27 crowned 63% &gt; 84%. In the mean +6 points of wins, fights +2% shorter, +8 points of HP left (a cell moves by about 5 points by chance).</t>
+          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Conette as mistress, without the skill &gt; with it): C36 81% &gt; 89%, C38 98% &gt; 99%, C40 93% &gt; 98%, P24 97% &gt; 98%, P27 crowned 67% &gt; 83%. In the mean +6 points of wins, fights +2% shorter, +7 points of HP left (a cell moves by about 5 points by chance).</t>
         </is>
       </c>
       <c r="L176" t="inlineStr">
@@ -13306,7 +13306,7 @@
       </c>
       <c r="K177" t="inlineStr">
         <is>
-          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Fiora as healer, without the skill &gt; with it): C36 90% &gt; 86%, C38 94% &gt; 97%, C40 95% &gt; 97%, P24 98% &gt; 99%, P27 crowned 73% &gt; 81%. In the mean +2 points of wins, fights +1% shorter, +3 points of HP left (a cell moves by about 5 points by chance).</t>
+          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Fiora as healer, without the skill &gt; with it): C36 85% &gt; 89%, C38 98% &gt; 97%, C40 100% &gt; 98%, P24 97% &gt; 99%, P27 crowned 70% &gt; 80%. In the mean +3 points of wins, fights -0% shorter, +3 points of HP left (a cell moves by about 5 points by chance).</t>
         </is>
       </c>
       <c r="L177" t="inlineStr">
@@ -13368,7 +13368,7 @@
       </c>
       <c r="K178" t="inlineStr">
         <is>
-          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Yuni as diva, without the skill &gt; with it): C36 98% &gt; 93%, C38 89% &gt; 94%, C40 90% &gt; 91%, P24 94% &gt; 99%, P27 crowned 85% &gt; 93%. In the mean +3 points of wins, fights +2% shorter, +3 points of HP left (a cell moves by about 5 points by chance).</t>
+          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Yuni as diva, without the skill &gt; with it): C36 96% &gt; 96%, C38 95% &gt; 95%, C40 93% &gt; 94%, P24 97% &gt; 99%, P27 crowned 83% &gt; 93%. In the mean +3 points of wins, fights +1% shorter, +3 points of HP left (a cell moves by about 5 points by chance).</t>
         </is>
       </c>
       <c r="L178" t="inlineStr">
@@ -13430,7 +13430,7 @@
       </c>
       <c r="K179" t="inlineStr">
         <is>
-          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Lilian as soul summoner, without the skill &gt; with it): C36 83% &gt; 83%, C38 87% &gt; 96%, C40 64% &gt; 74%, P24 80% &gt; 83%, P27 crowned 53% &gt; 55%. In the mean +5 points of wins, fights +1% shorter, +6 points of HP left (a cell moves by about 5 points by chance). The program draws one of seven results, the dispel among them (0x43697b); the Japanese page says the dispel never fires in version 1.05 and the English guide says it does: not settled</t>
+          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Lilian as soul summoner, without the skill &gt; with it): C36 87% &gt; 82%, C38 92% &gt; 96%, C40 78% &gt; 73%, P24 79% &gt; 81%, P27 crowned 57% &gt; 58%. In the mean -1 points of wins, fights +1% shorter, +0 points of HP left (a cell moves by about 5 points by chance). Its seventh result, the dispel, removes nothing: 0x47ee6f jumps over the routine (scratch/qol_fields_reading.md 7, checked), as the Japanese page says; played so since 2026-10-12</t>
         </is>
       </c>
       <c r="L179" t="inlineStr">
@@ -13492,7 +13492,7 @@
       </c>
       <c r="K180" t="inlineStr">
         <is>
-          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Tsurara as treasure hunter, without the skill &gt; with it): C36 85% &gt; 94%, C38 86% &gt; 90%, C40 95% &gt; 92%, P24 100% &gt; 100%, P27 crowned 86% &gt; 97%. In the mean +4 points of wins, fights -1% shorter, +2 points of HP left (a cell moves by about 5 points by chance).</t>
+          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Tsurara as treasure hunter, without the skill &gt; with it): C36 87% &gt; 93%, C38 91% &gt; 92%, C40 91% &gt; 91%, P24 100% &gt; 100%, P27 crowned 86% &gt; 97%. In the mean +4 points of wins, fights +0% shorter, +4 points of HP left (a cell moves by about 5 points by chance).</t>
         </is>
       </c>
       <c r="L180" t="inlineStr">
@@ -13554,7 +13554,7 @@
       </c>
       <c r="K181" t="inlineStr">
         <is>
-          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Siena as magical princess, without the skill &gt; with it): C36 82% &gt; 82%, C38 98% &gt; 97%, C40 74% &gt; 81%, P24 82% &gt; 83%, P27 crowned 58% &gt; 67%. In the mean +3 points of wins, fights -1% shorter, +2 points of HP left (a cell moves by about 5 points by chance).</t>
+          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Siena as magical princess, without the skill &gt; with it): C36 79% &gt; 79%, C38 99% &gt; 96%, C40 76% &gt; 79%, P24 85% &gt; 84%, P27 crowned 64% &gt; 73%. In the mean +2 points of wins, fights -3% shorter, +1 points of HP left (a cell moves by about 5 points by chance).</t>
         </is>
       </c>
       <c r="L181" t="inlineStr">

</xml_diff>

<commit_message>
sim: only the second action of Did You Call for Me? keeps the statuses
only the second action of Did You Call for Me? keeps the statuses from
losing a turn (what was read); Murder License and the statuses of the
shadow written as read
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -14240,6 +14240,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -14266,6 +14267,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -14292,6 +14294,7 @@
           <t>12.3 special damage, 2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -14318,6 +14321,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -14344,6 +14348,7 @@
           <t>2.7 special damage</t>
         </is>
       </c>
+      <c r="H6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -14370,6 +14375,7 @@
           <t>6b healing</t>
         </is>
       </c>
+      <c r="H7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -14396,6 +14402,7 @@
           <t>actions</t>
         </is>
       </c>
+      <c r="H8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -14422,6 +14429,7 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
+      <c r="H9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -14448,6 +14456,7 @@
           <t>2.7 special damage, 3 magic attack</t>
         </is>
       </c>
+      <c r="H10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -14474,6 +14483,7 @@
           <t>outside battle</t>
         </is>
       </c>
+      <c r="H11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -14500,6 +14510,7 @@
           <t>14 encounter rate</t>
         </is>
       </c>
+      <c r="H12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -14531,6 +14542,7 @@
           <t>0x47ffc0</t>
         </is>
       </c>
+      <c r="H13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -14557,6 +14569,7 @@
           <t>outside battle</t>
         </is>
       </c>
+      <c r="H14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -14583,6 +14596,7 @@
           <t>12.9 after a hit</t>
         </is>
       </c>
+      <c r="H15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -14609,6 +14623,7 @@
           <t>2 physical attack, 2.2 attack value</t>
         </is>
       </c>
+      <c r="H16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -14635,6 +14650,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -14661,6 +14677,7 @@
           <t>2 physical attack, 2.3 defence value</t>
         </is>
       </c>
+      <c r="H18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -14687,6 +14704,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -14713,6 +14731,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -14739,6 +14758,7 @@
           <t>4 critical hits</t>
         </is>
       </c>
+      <c r="H21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -14765,6 +14785,7 @@
           <t>4 critical hits</t>
         </is>
       </c>
+      <c r="H22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -14791,6 +14812,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -14817,6 +14839,7 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
+      <c r="H24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -14843,6 +14866,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -14869,6 +14893,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -14895,6 +14920,7 @@
           <t>5c turn delay</t>
         </is>
       </c>
+      <c r="H27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -14921,6 +14947,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -14947,6 +14974,7 @@
           <t>steal</t>
         </is>
       </c>
+      <c r="H29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -14973,6 +15001,7 @@
           <t>steal</t>
         </is>
       </c>
+      <c r="H30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -14999,6 +15028,7 @@
           <t>steal</t>
         </is>
       </c>
+      <c r="H31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -15030,6 +15060,7 @@
           <t>0x480e20</t>
         </is>
       </c>
+      <c r="H32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -15056,6 +15087,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -15082,6 +15114,7 @@
           <t>4 critical hits</t>
         </is>
       </c>
+      <c r="H34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -15108,6 +15141,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -15134,6 +15168,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -15160,6 +15195,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -15186,6 +15222,7 @@
           <t>applying a hit</t>
         </is>
       </c>
+      <c r="H38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -15212,6 +15249,7 @@
           <t>applying a hit</t>
         </is>
       </c>
+      <c r="H39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -15238,6 +15276,7 @@
           <t>applying a hit</t>
         </is>
       </c>
+      <c r="H40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -15269,6 +15308,7 @@
           <t>0x481060</t>
         </is>
       </c>
+      <c r="H41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -15295,6 +15335,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -15326,6 +15367,7 @@
           <t>0x481160</t>
         </is>
       </c>
+      <c r="H43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -15357,6 +15399,7 @@
           <t>0x4813a0</t>
         </is>
       </c>
+      <c r="H44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -15383,6 +15426,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -15409,6 +15453,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -15435,6 +15480,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -15461,6 +15507,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -15487,6 +15534,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -15513,6 +15561,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -15539,6 +15588,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -15565,6 +15615,7 @@
           <t>12.2 number of hits</t>
         </is>
       </c>
+      <c r="H52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -15591,6 +15642,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -15617,6 +15669,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -15643,6 +15696,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -15669,6 +15723,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -15695,6 +15750,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -15721,6 +15777,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -15747,6 +15804,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -15773,6 +15831,7 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
+      <c r="H60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -15799,6 +15858,7 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
+      <c r="H61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -15830,6 +15890,7 @@
           <t>0x4817c0</t>
         </is>
       </c>
+      <c r="H62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -15861,6 +15922,7 @@
           <t>0x481890</t>
         </is>
       </c>
+      <c r="H63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -15892,6 +15954,7 @@
           <t>0x481950</t>
         </is>
       </c>
+      <c r="H64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -15923,6 +15986,7 @@
           <t>0x481a20</t>
         </is>
       </c>
+      <c r="H65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -15949,6 +16013,7 @@
           <t>outside battle</t>
         </is>
       </c>
+      <c r="H66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -15975,6 +16040,7 @@
           <t>outside battle</t>
         </is>
       </c>
+      <c r="H67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -16001,6 +16067,7 @@
           <t>4 critical hits</t>
         </is>
       </c>
+      <c r="H68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -16027,6 +16094,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -16053,6 +16121,7 @@
           <t>9.1 who gets hit</t>
         </is>
       </c>
+      <c r="H70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -16084,6 +16153,7 @@
           <t>0x481ea0</t>
         </is>
       </c>
+      <c r="H71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -16115,6 +16185,7 @@
           <t>0x4822c0</t>
         </is>
       </c>
+      <c r="H72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -16146,6 +16217,7 @@
           <t>0x482530</t>
         </is>
       </c>
+      <c r="H73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -16177,6 +16249,7 @@
           <t>0x4827a0</t>
         </is>
       </c>
+      <c r="H74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -16208,6 +16281,7 @@
           <t>0x482a10</t>
         </is>
       </c>
+      <c r="H75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -16239,6 +16313,7 @@
           <t>0x482c80</t>
         </is>
       </c>
+      <c r="H76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -16270,6 +16345,7 @@
           <t>0x482e40</t>
         </is>
       </c>
+      <c r="H77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -16301,6 +16377,7 @@
           <t>0x4831f0</t>
         </is>
       </c>
+      <c r="H78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -16332,6 +16409,7 @@
           <t>0x4834b0</t>
         </is>
       </c>
+      <c r="H79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -16363,6 +16441,7 @@
           <t>0x4835d0</t>
         </is>
       </c>
+      <c r="H80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -16394,6 +16473,7 @@
           <t>0x483840</t>
         </is>
       </c>
+      <c r="H81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -16420,6 +16500,7 @@
           <t>4 critical hits</t>
         </is>
       </c>
+      <c r="H82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -16451,6 +16532,7 @@
           <t>0x483a60</t>
         </is>
       </c>
+      <c r="H83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -16482,6 +16564,7 @@
           <t>0x483b30</t>
         </is>
       </c>
+      <c r="H84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -16513,6 +16596,7 @@
           <t>0x483c20</t>
         </is>
       </c>
+      <c r="H85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -16544,6 +16628,7 @@
           <t>0x483d20</t>
         </is>
       </c>
+      <c r="H86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -16575,6 +16660,7 @@
           <t>0x483e00</t>
         </is>
       </c>
+      <c r="H87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -16606,6 +16692,7 @@
           <t>0x483ee0</t>
         </is>
       </c>
+      <c r="H88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -16632,6 +16719,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -16658,6 +16746,7 @@
           <t>9.1 who gets hit</t>
         </is>
       </c>
+      <c r="H90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -16684,6 +16773,7 @@
           <t>2.7 special damage</t>
         </is>
       </c>
+      <c r="H91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -16715,6 +16805,7 @@
           <t>0x484020</t>
         </is>
       </c>
+      <c r="H92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -16741,6 +16832,7 @@
           <t>2.7 special damage</t>
         </is>
       </c>
+      <c r="H93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -16767,6 +16859,7 @@
           <t>2.7 special damage</t>
         </is>
       </c>
+      <c r="H94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -16798,6 +16891,7 @@
           <t>0x484150</t>
         </is>
       </c>
+      <c r="H95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -16829,6 +16923,7 @@
           <t>0x484330</t>
         </is>
       </c>
+      <c r="H96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -16855,6 +16950,7 @@
           <t>11.1 dolls</t>
         </is>
       </c>
+      <c r="H97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -16881,6 +16977,7 @@
           <t>2 physical attack, 2.1 hit chance, 3 magic attack</t>
         </is>
       </c>
+      <c r="H98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -16907,6 +17004,7 @@
           <t>2 physical attack, 2.1 hit chance, 3 magic attack</t>
         </is>
       </c>
+      <c r="H99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -16933,6 +17031,7 @@
           <t>12.10 random moves</t>
         </is>
       </c>
+      <c r="H100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -16959,6 +17058,7 @@
           <t>12.10 random moves</t>
         </is>
       </c>
+      <c r="H101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -16985,6 +17085,7 @@
           <t>12.10 random moves</t>
         </is>
       </c>
+      <c r="H102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -17011,6 +17112,7 @@
           <t>12.10 random moves</t>
         </is>
       </c>
+      <c r="H103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -17037,6 +17139,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -17063,6 +17166,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -17089,6 +17193,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -17115,6 +17220,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -17141,6 +17247,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="n">
@@ -17167,6 +17274,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="n">
@@ -17193,6 +17301,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -17224,6 +17333,7 @@
           <t>0x4864c0</t>
         </is>
       </c>
+      <c r="H111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="n">
@@ -17250,6 +17360,7 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
+      <c r="H112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="n">
@@ -17276,6 +17387,7 @@
           <t>9.1 targets</t>
         </is>
       </c>
+      <c r="H113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -17302,6 +17414,7 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
+      <c r="H114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="n">
@@ -17328,6 +17441,7 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
+      <c r="H115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="n">
@@ -17354,6 +17468,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="n">
@@ -17380,6 +17495,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="n">
@@ -17406,6 +17522,7 @@
           <t>2 physical attack, 2.4 damage</t>
         </is>
       </c>
+      <c r="H118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="n">
@@ -17432,6 +17549,7 @@
           <t>applying a hit</t>
         </is>
       </c>
+      <c r="H119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="n">
@@ -17458,6 +17576,7 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
+      <c r="H120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="n">
@@ -17484,6 +17603,7 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
+      <c r="H121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="n">
@@ -17510,6 +17630,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="n">
@@ -17536,6 +17657,7 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
+      <c r="H123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="n">
@@ -17562,6 +17684,7 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
+      <c r="H124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="n">
@@ -17588,6 +17711,7 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
+      <c r="H125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="n">
@@ -17614,6 +17738,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="n">
@@ -17640,6 +17765,7 @@
           <t>2.8 damage received</t>
         </is>
       </c>
+      <c r="H127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="n">
@@ -17666,6 +17792,7 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
+      <c r="H128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="n">
@@ -17692,6 +17819,7 @@
           <t>2 physical attack, 2.4 damage, 3 magic attack</t>
         </is>
       </c>
+      <c r="H129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="n">
@@ -17718,6 +17846,7 @@
           <t>2 physical attack, 2.4 damage</t>
         </is>
       </c>
+      <c r="H130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="n">
@@ -17744,6 +17873,7 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
+      <c r="H131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="n">
@@ -17770,6 +17900,7 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
+      <c r="H132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="n">
@@ -17796,6 +17927,7 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
+      <c r="H133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -17822,6 +17954,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="n">
@@ -17848,6 +17981,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="n">
@@ -17874,6 +18008,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="n">
@@ -17900,6 +18035,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="n">
@@ -17926,6 +18062,7 @@
           <t>5e effects that act every turn</t>
         </is>
       </c>
+      <c r="H138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="n">
@@ -17952,6 +18089,7 @@
           <t>5e effects that act every turn</t>
         </is>
       </c>
+      <c r="H139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="n">
@@ -17978,6 +18116,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="n">
@@ -18004,6 +18143,7 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
+      <c r="H141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="n">
@@ -18030,6 +18170,7 @@
           <t>5d start of a turn</t>
         </is>
       </c>
+      <c r="H142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="n">
@@ -18056,6 +18197,7 @@
           <t>13 Pep</t>
         </is>
       </c>
+      <c r="H143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="n">
@@ -18082,6 +18224,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="n">
@@ -18108,6 +18251,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="n">
@@ -18134,6 +18278,7 @@
           <t>4 critical hits</t>
         </is>
       </c>
+      <c r="H146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="n">
@@ -18160,6 +18305,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="n">
@@ -18186,6 +18332,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="n">
@@ -18212,6 +18359,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="n">
@@ -18243,6 +18391,7 @@
           <t>0x4894a0</t>
         </is>
       </c>
+      <c r="H150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="n">
@@ -18274,6 +18423,7 @@
           <t>0x4895e0</t>
         </is>
       </c>
+      <c r="H151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="n">
@@ -18300,6 +18450,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="n">
@@ -18326,6 +18477,7 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
+      <c r="H153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="n">
@@ -18352,6 +18504,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="n">
@@ -18378,6 +18531,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="n">
@@ -18404,6 +18558,7 @@
           <t>2 physical attack, 2.1 hit chance, 5 order of turns</t>
         </is>
       </c>
+      <c r="H156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="n">
@@ -18430,6 +18585,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" t="n">
@@ -18456,6 +18612,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="n">
@@ -18482,6 +18639,7 @@
           <t>11.1 dolls</t>
         </is>
       </c>
+      <c r="H159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="n">
@@ -18508,6 +18666,7 @@
           <t>11.1 dolls</t>
         </is>
       </c>
+      <c r="H160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" t="n">
@@ -18534,6 +18693,7 @@
           <t>11.1 dolls</t>
         </is>
       </c>
+      <c r="H161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" t="n">
@@ -18560,6 +18720,7 @@
           <t>11.1 dolls</t>
         </is>
       </c>
+      <c r="H162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" t="n">
@@ -18586,6 +18747,7 @@
           <t>11.1 dolls</t>
         </is>
       </c>
+      <c r="H163" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" t="n">
@@ -18612,6 +18774,7 @@
           <t>11.1 dolls</t>
         </is>
       </c>
+      <c r="H164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="n">
@@ -18643,6 +18806,7 @@
           <t>0x48a430</t>
         </is>
       </c>
+      <c r="H165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="n">
@@ -18669,6 +18833,7 @@
           <t>10.1 stats of a piece of equipment</t>
         </is>
       </c>
+      <c r="H166" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" t="n">
@@ -18695,6 +18860,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H167" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" t="n">
@@ -18721,6 +18887,7 @@
           <t>6b healing</t>
         </is>
       </c>
+      <c r="H168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="n">
@@ -18752,6 +18919,7 @@
           <t>0x48a640</t>
         </is>
       </c>
+      <c r="H169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" t="n">
@@ -18778,6 +18946,7 @@
           <t>5e effects that act every turn</t>
         </is>
       </c>
+      <c r="H170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="n">
@@ -18804,6 +18973,7 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
+      <c r="H171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="n">
@@ -18830,6 +19000,7 @@
           <t>12.13 counters and follow-ups</t>
         </is>
       </c>
+      <c r="H172" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" t="n">
@@ -18856,6 +19027,7 @@
           <t>12.13 counters and follow-ups</t>
         </is>
       </c>
+      <c r="H173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="n">
@@ -18882,6 +19054,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H174" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" t="n">
@@ -18908,6 +19081,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" t="n">
@@ -18934,6 +19108,7 @@
           <t>2 physical attack, 2.1 hit chance</t>
         </is>
       </c>
+      <c r="H176" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" t="n">
@@ -18960,6 +19135,7 @@
           <t>passive rolls</t>
         </is>
       </c>
+      <c r="H177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="n">
@@ -18986,6 +19162,7 @@
           <t>passive rolls</t>
         </is>
       </c>
+      <c r="H178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" t="n">
@@ -19012,6 +19189,7 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
+      <c r="H179" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" t="n">
@@ -19038,6 +19216,7 @@
           <t>2.8 damage received</t>
         </is>
       </c>
+      <c r="H180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" t="n">
@@ -19064,6 +19243,7 @@
           <t>2 physical attack, 2.4 damage</t>
         </is>
       </c>
+      <c r="H181" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" t="n">
@@ -19090,6 +19270,7 @@
           <t>5d start of a turn</t>
         </is>
       </c>
+      <c r="H182" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" t="n">
@@ -19116,6 +19297,7 @@
           <t>12.13 counters and follow-ups</t>
         </is>
       </c>
+      <c r="H183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="n">
@@ -19142,6 +19324,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="n">
@@ -19168,6 +19351,7 @@
           <t>12.9 after a hit</t>
         </is>
       </c>
+      <c r="H185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="n">
@@ -19194,6 +19378,7 @@
           <t>2 physical attack, 2.4 damage</t>
         </is>
       </c>
+      <c r="H186" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" t="n">
@@ -19220,6 +19405,7 @@
           <t>2 physical attack, 2.5 chant interruption</t>
         </is>
       </c>
+      <c r="H187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="n">
@@ -19246,6 +19432,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H188" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" t="n">
@@ -19272,6 +19459,7 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
+      <c r="H189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" t="n">
@@ -19298,6 +19486,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H190" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" t="n">
@@ -19324,6 +19513,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" t="n">
@@ -19350,6 +19540,7 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
+      <c r="H192" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" t="n">
@@ -19376,6 +19567,7 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
+      <c r="H193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" t="n">
@@ -19402,6 +19594,7 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
+      <c r="H194" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" t="n">
@@ -19428,6 +19621,7 @@
           <t>after a battle</t>
         </is>
       </c>
+      <c r="H195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" t="n">
@@ -19454,6 +19648,7 @@
           <t>after a battle</t>
         </is>
       </c>
+      <c r="H196" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" t="n">
@@ -19480,6 +19675,7 @@
           <t>passive rolls</t>
         </is>
       </c>
+      <c r="H197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" t="n">
@@ -19506,6 +19702,7 @@
           <t>items</t>
         </is>
       </c>
+      <c r="H198" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" t="n">
@@ -19532,6 +19729,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H199" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" t="n">
@@ -19558,6 +19756,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H200" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" t="n">
@@ -19584,6 +19783,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H201" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" t="n">
@@ -19610,6 +19810,7 @@
           <t>11.2 songs and dances</t>
         </is>
       </c>
+      <c r="H202" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" t="n">
@@ -19636,6 +19837,7 @@
           <t>11.2 songs and dances</t>
         </is>
       </c>
+      <c r="H203" t="inlineStr"/>
     </row>
     <row r="204">
       <c r="A204" t="n">
@@ -19662,6 +19864,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H204" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" t="n">
@@ -19688,6 +19891,7 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
+      <c r="H205" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" t="n">
@@ -19714,6 +19918,7 @@
           <t>5d start of a turn</t>
         </is>
       </c>
+      <c r="H206" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" t="n">
@@ -19740,6 +19945,7 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
+      <c r="H207" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" t="n">
@@ -19766,6 +19972,7 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
+      <c r="H208" t="inlineStr"/>
     </row>
     <row r="209">
       <c r="A209" t="n">
@@ -19792,6 +19999,7 @@
           <t>11.1 dolls, 2 physical attack, 3 magic attack, 6b healing</t>
         </is>
       </c>
+      <c r="H209" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" t="n">
@@ -19818,6 +20026,7 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
+      <c r="H210" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" t="n">
@@ -19844,6 +20053,7 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
+      <c r="H211" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" t="n">
@@ -19870,6 +20080,7 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
+      <c r="H212" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" t="n">
@@ -19896,6 +20107,7 @@
           <t>2.8 damage received</t>
         </is>
       </c>
+      <c r="H213" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" t="n">
@@ -19922,6 +20134,7 @@
           <t>12.9 after a hit</t>
         </is>
       </c>
+      <c r="H214" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" t="n">
@@ -19948,6 +20161,7 @@
           <t>6b heal cap, 6b healing</t>
         </is>
       </c>
+      <c r="H215" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" t="n">
@@ -19974,6 +20188,7 @@
           <t>3 magic attack, 6b heal cap</t>
         </is>
       </c>
+      <c r="H216" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" t="n">
@@ -20000,6 +20215,7 @@
           <t>11.1 dolls</t>
         </is>
       </c>
+      <c r="H217" t="inlineStr"/>
     </row>
     <row r="218">
       <c r="A218" t="n">
@@ -20026,6 +20242,7 @@
           <t>10.1 stats of a piece of equipment</t>
         </is>
       </c>
+      <c r="H218" t="inlineStr"/>
     </row>
     <row r="219">
       <c r="A219" t="n">
@@ -20052,6 +20269,7 @@
           <t>passive rolls</t>
         </is>
       </c>
+      <c r="H219" t="inlineStr"/>
     </row>
     <row r="220">
       <c r="A220" t="n">
@@ -20078,6 +20296,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H220" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" t="n">
@@ -20104,6 +20323,7 @@
           <t>12.13 counters and follow-ups</t>
         </is>
       </c>
+      <c r="H221" t="inlineStr"/>
     </row>
     <row r="222">
       <c r="A222" t="n">
@@ -20130,6 +20350,7 @@
           <t>12.9 after a hit</t>
         </is>
       </c>
+      <c r="H222" t="inlineStr"/>
     </row>
     <row r="223">
       <c r="A223" t="n">
@@ -20156,6 +20377,7 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
+      <c r="H223" t="inlineStr"/>
     </row>
     <row r="224">
       <c r="A224" t="n">
@@ -20182,6 +20404,7 @@
           <t>outside battle</t>
         </is>
       </c>
+      <c r="H224" t="inlineStr"/>
     </row>
     <row r="225">
       <c r="A225" t="n">
@@ -20208,6 +20431,7 @@
           <t>12.13 counters and follow-ups</t>
         </is>
       </c>
+      <c r="H225" t="inlineStr"/>
     </row>
     <row r="226">
       <c r="A226" t="n">
@@ -20234,6 +20458,7 @@
           <t>2 physical attack, 2.4 other bonuses of final damage</t>
         </is>
       </c>
+      <c r="H226" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" t="n">
@@ -20260,6 +20485,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H227" t="inlineStr"/>
     </row>
     <row r="228">
       <c r="A228" t="n">
@@ -20286,6 +20512,7 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
+      <c r="H228" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" t="n">
@@ -20312,6 +20539,7 @@
           <t>5d start of a turn</t>
         </is>
       </c>
+      <c r="H229" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" t="n">
@@ -20338,6 +20566,7 @@
           <t>12.14 after an action</t>
         </is>
       </c>
+      <c r="H230" t="inlineStr"/>
     </row>
     <row r="231">
       <c r="A231" t="n">
@@ -20364,6 +20593,7 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
+      <c r="H231" t="inlineStr"/>
     </row>
     <row r="232">
       <c r="A232" t="n">
@@ -20390,6 +20620,7 @@
           <t>11.1 dolls</t>
         </is>
       </c>
+      <c r="H232" t="inlineStr"/>
     </row>
     <row r="233">
       <c r="A233" t="n">
@@ -20416,6 +20647,7 @@
           <t>12.10 random moves</t>
         </is>
       </c>
+      <c r="H233" t="inlineStr"/>
     </row>
     <row r="234">
       <c r="A234" t="n">
@@ -20442,6 +20674,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H234" t="inlineStr"/>
     </row>
     <row r="235">
       <c r="A235" t="n">
@@ -20468,6 +20701,7 @@
           <t>6b heal cap</t>
         </is>
       </c>
+      <c r="H235" t="inlineStr"/>
     </row>
     <row r="236">
       <c r="A236" t="n">
@@ -20494,6 +20728,7 @@
           <t>9 enemy AI</t>
         </is>
       </c>
+      <c r="H236" t="inlineStr"/>
     </row>
     <row r="237">
       <c r="A237" t="n">
@@ -20520,6 +20755,7 @@
           <t>12.9 after a hit</t>
         </is>
       </c>
+      <c r="H237" t="inlineStr"/>
     </row>
     <row r="238">
       <c r="A238" t="n">
@@ -20546,6 +20782,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H238" t="inlineStr"/>
     </row>
     <row r="239">
       <c r="A239" t="n">
@@ -20572,6 +20809,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H239" t="inlineStr"/>
     </row>
     <row r="240">
       <c r="A240" t="n">
@@ -20598,6 +20836,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H240" t="inlineStr"/>
     </row>
     <row r="241">
       <c r="A241" t="n">
@@ -20624,6 +20863,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H241" t="inlineStr"/>
     </row>
     <row r="242">
       <c r="A242" t="n">
@@ -20650,6 +20890,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H242" t="inlineStr"/>
     </row>
     <row r="243">
       <c r="A243" t="n">
@@ -20676,6 +20917,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H243" t="inlineStr"/>
     </row>
     <row r="244">
       <c r="A244" t="n">
@@ -20702,6 +20944,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H244" t="inlineStr"/>
     </row>
     <row r="245">
       <c r="A245" t="n">
@@ -20728,6 +20971,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H245" t="inlineStr"/>
     </row>
     <row r="246">
       <c r="A246" t="n">
@@ -20754,6 +20998,7 @@
           <t>2 physical attack, 2.1 hit chance, 3 magic attack</t>
         </is>
       </c>
+      <c r="H246" t="inlineStr"/>
     </row>
     <row r="247">
       <c r="A247" t="n">
@@ -20780,6 +21025,7 @@
           <t>2 physical attack, 2.1 hit chance, 3 magic attack</t>
         </is>
       </c>
+      <c r="H247" t="inlineStr"/>
     </row>
     <row r="248">
       <c r="A248" t="n">
@@ -20806,6 +21052,7 @@
           <t>5e effects that act every turn</t>
         </is>
       </c>
+      <c r="H248" t="inlineStr"/>
     </row>
     <row r="249">
       <c r="A249" t="n">
@@ -20832,6 +21079,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H249" t="inlineStr"/>
     </row>
     <row r="250">
       <c r="A250" t="n">
@@ -20858,6 +21106,7 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
+      <c r="H250" t="inlineStr"/>
     </row>
     <row r="251">
       <c r="A251" t="n">
@@ -20884,6 +21133,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H251" t="inlineStr"/>
     </row>
     <row r="252">
       <c r="A252" t="n">
@@ -20910,6 +21160,7 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
+      <c r="H252" t="inlineStr"/>
     </row>
     <row r="253">
       <c r="A253" t="n">
@@ -20936,6 +21187,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H253" t="inlineStr"/>
     </row>
     <row r="254">
       <c r="A254" t="n">
@@ -20962,6 +21214,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H254" t="inlineStr"/>
     </row>
     <row r="255">
       <c r="A255" t="n">
@@ -20988,6 +21241,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H255" t="inlineStr"/>
     </row>
     <row r="256">
       <c r="A256" t="n">
@@ -21014,6 +21268,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H256" t="inlineStr"/>
     </row>
     <row r="257">
       <c r="A257" t="n">
@@ -21040,6 +21295,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H257" t="inlineStr"/>
     </row>
     <row r="258">
       <c r="A258" t="n">
@@ -21066,6 +21322,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H258" t="inlineStr"/>
     </row>
     <row r="259">
       <c r="A259" t="n">
@@ -21092,6 +21349,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H259" t="inlineStr"/>
     </row>
     <row r="260">
       <c r="A260" t="n">
@@ -21118,6 +21376,7 @@
           <t>2 physical attack, 2.4 damage, 3 magic attack</t>
         </is>
       </c>
+      <c r="H260" t="inlineStr"/>
     </row>
     <row r="261">
       <c r="A261" t="n">
@@ -21144,6 +21403,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H261" t="inlineStr"/>
     </row>
     <row r="262">
       <c r="A262" t="n">
@@ -21170,6 +21430,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H262" t="inlineStr"/>
     </row>
     <row r="263">
       <c r="A263" t="n">
@@ -21196,6 +21457,7 @@
           <t>12.10 random moves</t>
         </is>
       </c>
+      <c r="H263" t="inlineStr"/>
     </row>
     <row r="264">
       <c r="A264" t="n">
@@ -21222,6 +21484,7 @@
           <t>12.10 random moves</t>
         </is>
       </c>
+      <c r="H264" t="inlineStr"/>
     </row>
     <row r="265">
       <c r="A265" t="n">
@@ -21248,6 +21511,7 @@
           <t>12.10 random moves</t>
         </is>
       </c>
+      <c r="H265" t="inlineStr"/>
     </row>
     <row r="266">
       <c r="A266" t="n">
@@ -21274,6 +21538,7 @@
           <t>6c EXP</t>
         </is>
       </c>
+      <c r="H266" t="inlineStr"/>
     </row>
     <row r="267">
       <c r="A267" t="n">
@@ -21300,6 +21565,7 @@
           <t>12.10 random moves</t>
         </is>
       </c>
+      <c r="H267" t="inlineStr"/>
     </row>
     <row r="268">
       <c r="A268" t="n">
@@ -21331,6 +21597,7 @@
           <t>0x48b490</t>
         </is>
       </c>
+      <c r="H268" t="inlineStr"/>
     </row>
     <row r="269">
       <c r="A269" t="n">
@@ -21357,6 +21624,7 @@
           <t>2.7 special damage</t>
         </is>
       </c>
+      <c r="H269" t="inlineStr"/>
     </row>
     <row r="270">
       <c r="A270" t="n">
@@ -21383,6 +21651,7 @@
           <t>2.7 special damage</t>
         </is>
       </c>
+      <c r="H270" t="inlineStr"/>
     </row>
     <row r="271">
       <c r="A271" t="n">
@@ -21409,6 +21678,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H271" t="inlineStr"/>
     </row>
     <row r="272">
       <c r="A272" t="n">
@@ -21435,6 +21705,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H272" t="inlineStr"/>
     </row>
     <row r="273">
       <c r="A273" t="n">
@@ -21461,6 +21732,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H273" t="inlineStr"/>
     </row>
     <row r="274">
       <c r="A274" t="n">
@@ -21487,6 +21759,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H274" t="inlineStr"/>
     </row>
     <row r="275">
       <c r="A275" t="n">
@@ -21513,6 +21786,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H275" t="inlineStr"/>
     </row>
     <row r="276">
       <c r="A276" t="n">
@@ -21539,6 +21813,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H276" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -29664,7 +29939,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>Murder License (enemy): at step 12 of the turn of its bearer an action is built from the skill linked to the status, on one target drawn at random (0x43736a - 0x43743a). Whether the own command of the bearer still follows, which skill is linked and its chance are not read yet; the Japanese pages 207 and 334 say that before each action of the bearer one member may die at once unless immune to instant death or of high earth resistance. An earlier wording here, that the action of the bearer is replaced, did not fit them</t>
+          <t>Murder License (enemy): at step 12 of each turn of its bearer, with no roll, an action is built from the attack linked to the status and aimed at one opponent drawn at random (0x43736a - 0x43743a) and run (0x437488); the step counter was raised before (0x437364), so the own action of the bearer follows. What the linked attack does is not read: the Japanese pages 207 and 334 say one member may die at once unless immune to instant death or of high earth resistance. Not played by the simulator; the fights of its bearers are played with earth 100 (sheet Preparation)</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">

</xml_diff>

<commit_message>
balance: third Eye Wide x2, Usurper of Souls x1.6, the roll of Arcane
third Eye Wide x2, Usurper of Souls x1.6, the roll of Arcane Shield 25
in 100 (program patch of 13 rows); the build writes the values of unique
skills; the rows of the unique skills closed
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -12505,7 +12505,7 @@
       </c>
       <c r="L164" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>not a problem</t>
         </is>
       </c>
       <c r="O164" t="inlineStr">
@@ -12515,7 +12515,12 @@
       </c>
       <c r="P164" t="inlineStr">
         <is>
-          <t>measured; to be read with the user</t>
+          <t>measured: within what the others give, none above +8% of length or +6 points of wins</t>
+        </is>
+      </c>
+      <c r="R164" t="inlineStr">
+        <is>
+          <t>the user, 2026-10-12: left as it is; it adds little but it is good to have</t>
         </is>
       </c>
     </row>
@@ -12567,7 +12572,7 @@
       </c>
       <c r="L165" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>not a problem</t>
         </is>
       </c>
       <c r="O165" t="inlineStr">
@@ -12577,7 +12582,12 @@
       </c>
       <c r="P165" t="inlineStr">
         <is>
-          <t>measured; to be read with the user</t>
+          <t>measured: within what the others give, none above +8% of length or +6 points of wins</t>
+        </is>
+      </c>
+      <c r="R165" t="inlineStr">
+        <is>
+          <t>the user, 2026-10-12: left as it is; it adds little but it is good to have</t>
         </is>
       </c>
     </row>
@@ -12629,7 +12639,7 @@
       </c>
       <c r="L166" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>not a problem</t>
         </is>
       </c>
       <c r="O166" t="inlineStr">
@@ -12639,7 +12649,12 @@
       </c>
       <c r="P166" t="inlineStr">
         <is>
-          <t>measured; to be read with the user</t>
+          <t>measured: within what the others give, none above +8% of length or +6 points of wins</t>
+        </is>
+      </c>
+      <c r="R166" t="inlineStr">
+        <is>
+          <t>the user, 2026-10-12: left as it is; it adds little but it is good to have</t>
         </is>
       </c>
     </row>
@@ -12691,7 +12706,7 @@
       </c>
       <c r="L167" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>not a problem</t>
         </is>
       </c>
       <c r="O167" t="inlineStr">
@@ -12701,7 +12716,12 @@
       </c>
       <c r="P167" t="inlineStr">
         <is>
-          <t>measured; to be read with the user</t>
+          <t>measured: within what the others give, none above +8% of length or +6 points of wins</t>
+        </is>
+      </c>
+      <c r="R167" t="inlineStr">
+        <is>
+          <t>the user, 2026-10-12: left as it is; it adds little but it is good to have</t>
         </is>
       </c>
     </row>
@@ -12753,7 +12773,7 @@
       </c>
       <c r="L168" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>not a problem</t>
         </is>
       </c>
       <c r="O168" t="inlineStr">
@@ -12763,7 +12783,12 @@
       </c>
       <c r="P168" t="inlineStr">
         <is>
-          <t>measured; to be read with the user</t>
+          <t>measured: within what the others give, none above +8% of length or +6 points of wins</t>
+        </is>
+      </c>
+      <c r="R168" t="inlineStr">
+        <is>
+          <t>the user, 2026-10-12: left as it is; it adds little but it is good to have</t>
         </is>
       </c>
     </row>
@@ -12815,7 +12840,7 @@
       </c>
       <c r="L169" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>not a problem</t>
         </is>
       </c>
       <c r="O169" t="inlineStr">
@@ -12825,7 +12850,12 @@
       </c>
       <c r="P169" t="inlineStr">
         <is>
-          <t>measured; to be read with the user</t>
+          <t>measured: within what the others give, none above +8% of length or +6 points of wins</t>
+        </is>
+      </c>
+      <c r="R169" t="inlineStr">
+        <is>
+          <t>the user, 2026-10-12: left as it is; it adds little but it is good to have</t>
         </is>
       </c>
     </row>
@@ -12877,7 +12907,7 @@
       </c>
       <c r="L170" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>not a problem</t>
         </is>
       </c>
       <c r="O170" t="inlineStr">
@@ -12887,7 +12917,12 @@
       </c>
       <c r="P170" t="inlineStr">
         <is>
-          <t>measured; to be read with the user</t>
+          <t>measured: within what the others give, none above +8% of length or +6 points of wins</t>
+        </is>
+      </c>
+      <c r="R170" t="inlineStr">
+        <is>
+          <t>the user, 2026-10-12: left as it is; it adds little but it is good to have</t>
         </is>
       </c>
     </row>
@@ -12939,7 +12974,7 @@
       </c>
       <c r="L171" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>not a problem</t>
         </is>
       </c>
       <c r="O171" t="inlineStr">
@@ -12949,7 +12984,12 @@
       </c>
       <c r="P171" t="inlineStr">
         <is>
-          <t>measured; to be read with the user</t>
+          <t>measured: within what the others give, none above +8% of length or +6 points of wins</t>
+        </is>
+      </c>
+      <c r="R171" t="inlineStr">
+        <is>
+          <t>the user, 2026-10-12: left as it is; it adds little but it is good to have</t>
         </is>
       </c>
     </row>
@@ -13001,7 +13041,7 @@
       </c>
       <c r="L172" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>not a problem</t>
         </is>
       </c>
       <c r="O172" t="inlineStr">
@@ -13011,7 +13051,12 @@
       </c>
       <c r="P172" t="inlineStr">
         <is>
-          <t>measured; to be read with the user</t>
+          <t>measured: within what the others give, none above +8% of length or +6 points of wins</t>
+        </is>
+      </c>
+      <c r="R172" t="inlineStr">
+        <is>
+          <t>the user, 2026-10-12: left as it is; it adds little but it is good to have</t>
         </is>
       </c>
     </row>
@@ -13063,7 +13108,7 @@
       </c>
       <c r="L173" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>not a problem</t>
         </is>
       </c>
       <c r="O173" t="inlineStr">
@@ -13073,7 +13118,12 @@
       </c>
       <c r="P173" t="inlineStr">
         <is>
-          <t>measured; to be read with the user</t>
+          <t>measured: within what the others give, none above +8% of length or +6 points of wins</t>
+        </is>
+      </c>
+      <c r="R173" t="inlineStr">
+        <is>
+          <t>the user, 2026-10-12: left as it is; it adds little but it is good to have</t>
         </is>
       </c>
     </row>
@@ -13120,12 +13170,12 @@
       </c>
       <c r="K174" t="inlineStr">
         <is>
-          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Lizerietta as papillon, without the skill &gt; with it): C36 95% &gt; 92%, C38 96% &gt; 97%, C40 96% &gt; 96%, P24 100% &gt; 100%, P27 crowned 85% &gt; 86%. In the mean -0 points of wins, fights -2% shorter, -1 points of HP left (a cell moves by about 5 points by chance). It only acts on what an enemy summons; which of these five fights hold a summoner was not looked at</t>
+          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Lizerietta as papillon, without the skill &gt; with it): C36 95% &gt; 92%, C38 96% &gt; 97%, C40 96% &gt; 96%, P24 100% &gt; 100%, P27 crowned 85% &gt; 86%. In the mean -0 points of wins, fights -2% shorter, -1 points of HP left (a cell moves by about 5 points by chance). It only acts on what an enemy summons; which of these five fights hold a summoner was not looked at Built on 2026-10-12. None of the five fights of the measure holds anything it can remove, with or without the raise: its worth is only against the enemies that summon, not measured</t>
         </is>
       </c>
       <c r="L174" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="O174" t="inlineStr">
@@ -13135,7 +13185,17 @@
       </c>
       <c r="P174" t="inlineStr">
         <is>
-          <t>measured; to be read with the user</t>
+          <t>true: it added nothing that could be measured</t>
+        </is>
+      </c>
+      <c r="Q174" t="inlineStr">
+        <is>
+          <t>U011 - U020: the chance times 1.6, never over 1 (40 - 91% by rank, certain crowned)</t>
+        </is>
+      </c>
+      <c r="R174" t="inlineStr">
+        <is>
+          <t>the user, 2026-10-12: raised</t>
         </is>
       </c>
     </row>
@@ -13187,7 +13247,7 @@
       </c>
       <c r="L175" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>not a problem</t>
         </is>
       </c>
       <c r="O175" t="inlineStr">
@@ -13197,7 +13257,12 @@
       </c>
       <c r="P175" t="inlineStr">
         <is>
-          <t>measured; to be read with the user</t>
+          <t>measured: within what the others give, none above +8% of length or +6 points of wins</t>
+        </is>
+      </c>
+      <c r="R175" t="inlineStr">
+        <is>
+          <t>the user, 2026-10-12: left as it is; it adds little but it is good to have</t>
         </is>
       </c>
     </row>
@@ -13249,7 +13314,7 @@
       </c>
       <c r="L176" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>not a problem</t>
         </is>
       </c>
       <c r="O176" t="inlineStr">
@@ -13259,7 +13324,12 @@
       </c>
       <c r="P176" t="inlineStr">
         <is>
-          <t>measured; to be read with the user</t>
+          <t>measured: within what the others give, none above +8% of length or +6 points of wins</t>
+        </is>
+      </c>
+      <c r="R176" t="inlineStr">
+        <is>
+          <t>the user, 2026-10-12: left as it is; it adds little but it is good to have</t>
         </is>
       </c>
     </row>
@@ -13311,7 +13381,7 @@
       </c>
       <c r="L177" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>not a problem</t>
         </is>
       </c>
       <c r="O177" t="inlineStr">
@@ -13321,7 +13391,12 @@
       </c>
       <c r="P177" t="inlineStr">
         <is>
-          <t>measured; to be read with the user</t>
+          <t>measured: within what the others give, none above +8% of length or +6 points of wins</t>
+        </is>
+      </c>
+      <c r="R177" t="inlineStr">
+        <is>
+          <t>the user, 2026-10-12: left as it is; it adds little but it is good to have</t>
         </is>
       </c>
     </row>
@@ -13373,7 +13448,7 @@
       </c>
       <c r="L178" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>not a problem</t>
         </is>
       </c>
       <c r="O178" t="inlineStr">
@@ -13383,7 +13458,12 @@
       </c>
       <c r="P178" t="inlineStr">
         <is>
-          <t>measured; to be read with the user</t>
+          <t>measured: within what the others give, none above +8% of length or +6 points of wins</t>
+        </is>
+      </c>
+      <c r="R178" t="inlineStr">
+        <is>
+          <t>the user, 2026-10-12: left as it is; it adds little but it is good to have</t>
         </is>
       </c>
     </row>
@@ -13430,12 +13510,12 @@
       </c>
       <c r="K179" t="inlineStr">
         <is>
-          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Lilian as soul summoner, without the skill &gt; with it): C36 87% &gt; 82%, C38 92% &gt; 96%, C40 78% &gt; 73%, P24 79% &gt; 81%, P27 crowned 57% &gt; 58%. In the mean -1 points of wins, fights +1% shorter, +0 points of HP left (a cell moves by about 5 points by chance). Its seventh result, the dispel, removes nothing: 0x47ee6f jumps over the routine (scratch/qol_fields_reading.md 7, checked), as the Japanese page says; played so since 2026-10-12</t>
+          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Lilian as soul summoner, without the skill &gt; with it): C36 87% &gt; 82%, C38 92% &gt; 96%, C40 78% &gt; 73%, P24 79% &gt; 81%, P27 crowned 57% &gt; 58%. In the mean -1 points of wins, fights +1% shorter, +0 points of HP left (a cell moves by about 5 points by chance). Its seventh result, the dispel, removes nothing: 0x47ee6f jumps over the routine (scratch/qol_fields_reading.md 7, checked), as the Japanese page says; played so since 2026-10-12 Built on 2026-10-12 (1,421 of 1,421 rows): the reference party wins 78.6% of the five bosses without it and 80.2% with it (78.0% before); rows of eight random battles at four floors do not run away with it</t>
         </is>
       </c>
       <c r="L179" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="O179" t="inlineStr">
@@ -13445,7 +13525,17 @@
       </c>
       <c r="P179" t="inlineStr">
         <is>
-          <t>measured; to be read with the user</t>
+          <t>true: it added nothing that could be measured</t>
+        </is>
+      </c>
+      <c r="Q179" t="inlineStr">
+        <is>
+          <t>U001 - U010: the chance times 2 (14 - 30% by rank, 50% crowned)</t>
+        </is>
+      </c>
+      <c r="R179" t="inlineStr">
+        <is>
+          <t>the user, 2026-10-12: raised</t>
         </is>
       </c>
     </row>
@@ -13497,7 +13587,7 @@
       </c>
       <c r="L180" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>not a problem</t>
         </is>
       </c>
       <c r="O180" t="inlineStr">
@@ -13507,7 +13597,12 @@
       </c>
       <c r="P180" t="inlineStr">
         <is>
-          <t>measured; to be read with the user</t>
+          <t>measured: within what the others give, none above +8% of length or +6 points of wins</t>
+        </is>
+      </c>
+      <c r="R180" t="inlineStr">
+        <is>
+          <t>the user, 2026-10-12: left as it is; it adds little but it is good to have</t>
         </is>
       </c>
     </row>
@@ -13554,12 +13649,12 @@
       </c>
       <c r="K181" t="inlineStr">
         <is>
-          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Siena as magical princess, without the skill &gt; with it): C36 79% &gt; 79%, C38 99% &gt; 96%, C40 76% &gt; 79%, P24 85% &gt; 84%, P27 crowned 64% &gt; 73%. In the mean +2 points of wins, fights -3% shorter, +1 points of HP left (a cell moves by about 5 points by chance).</t>
+          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Siena as magical princess, without the skill &gt; with it): C36 79% &gt; 79%, C38 99% &gt; 96%, C40 76% &gt; 79%, P24 85% &gt; 84%, P27 crowned 64% &gt; 73%. In the mean +2 points of wins, fights -3% shorter, +1 points of HP left (a cell moves by about 5 points by chance). Built on 2026-10-12. The measure does not move with it (82.2% as it was, 82.0% at 25%, 80.6% without the skill): what it sends back is a share of the damage she takes, little beside the HP of a boss. Raised for the feel of it, at the word of the user</t>
         </is>
       </c>
       <c r="L181" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="O181" t="inlineStr">
@@ -13569,7 +13664,17 @@
       </c>
       <c r="P181" t="inlineStr">
         <is>
-          <t>measured; to be read with the user</t>
+          <t>true: it added nothing that could be measured</t>
+        </is>
+      </c>
+      <c r="Q181" t="inlineStr">
+        <is>
+          <t>X13 of the sheet ExePatches (set balance, lever L38): the roll from 15 to 25 in 100; its box worded in balance_skill_text.xlsx</t>
+        </is>
+      </c>
+      <c r="R181" t="inlineStr">
+        <is>
+          <t>the user, 2026-10-12: raised</t>
         </is>
       </c>
     </row>
@@ -13584,7 +13689,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I18"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -14131,29 +14236,66 @@
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>VA: address of the first byte changed. Old_Hex must be found there before anything is written, in both program files of the game folder (DT22_en.exe and DT22_en_unwrapped.exe): the set is written into both or into neither (tools/exe_patch.py).</t>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>X13</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>balance</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>L38</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>0x424768</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>0f</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Roll of Arcane Shield, a number below 100 under: 15 -&gt; 25 (the user, 2026-10-12; cmp eax, imm8 at 0x424766)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>A row with floats repoints a "movss xmm0, [address]" at another constant that already exists in the program: Float_Before and Float_After are what the old and the new address hold, and the tool checks both.</t>
+          <t>VA: address of the first byte changed. Old_Hex must be found there before anything is written, in both program files of the game folder (DT22_en.exe and DT22_en_unwrapped.exe): the set is written into both or into neither (tools/exe_patch.py).</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>The step of 59 to 68 levels stays at 1 point (accepted by the user, 2026-10-05): its instruction is an "inc", with no byte that holds the amount. Giving it 2 means rewriting the end of the function. With the other four steps one point higher the cheapest crown no longer uses that step (docs/generated/CATCH_UP_OPTIONS.md, rule "One more point, lowest step kept").</t>
+          <t>A row with floats repoints a "movss xmm0, [address]" at another constant that already exists in the program: Float_Before and Float_After are what the old and the new address hold, and the tool checks both.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
+        <is>
+          <t>The step of 59 to 68 levels stays at 1 point (accepted by the user, 2026-10-05): its instruction is an "inc", with no byte that holds the amount. Giving it 2 means rewriting the end of the function. With the other four steps one point higher the cheapest crown no longer uses that step (docs/generated/CATCH_UP_OPTIONS.md, rule "One more point, lowest step kept").</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
         <is>
           <t>Factors with the piece of enchantment 270 (X06 to X08: 1.5, 4, 6) and the last band at 10 with or without the piece: accepted by the user on 2026-10-05, after the test in the game. The name of the enchantment in the Balance variant states them (balance_enchant_text.xlsx).</t>
         </is>
@@ -14240,7 +14382,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -14267,7 +14408,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -14294,7 +14434,6 @@
           <t>12.3 special damage, 2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -14321,7 +14460,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -14348,7 +14486,6 @@
           <t>2.7 special damage</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -14375,7 +14512,6 @@
           <t>6b healing</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -14402,7 +14538,6 @@
           <t>actions</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -14429,7 +14564,6 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -14456,7 +14590,6 @@
           <t>2.7 special damage, 3 magic attack</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -14483,7 +14616,6 @@
           <t>outside battle</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -14510,7 +14642,6 @@
           <t>14 encounter rate</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -14542,7 +14673,6 @@
           <t>0x47ffc0</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -14569,7 +14699,6 @@
           <t>outside battle</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -14596,7 +14725,6 @@
           <t>12.9 after a hit</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -14623,7 +14751,6 @@
           <t>2 physical attack, 2.2 attack value</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -14650,7 +14777,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -14677,7 +14803,6 @@
           <t>2 physical attack, 2.3 defence value</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -14704,7 +14829,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -14731,7 +14855,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -14758,7 +14881,6 @@
           <t>4 critical hits</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -14785,7 +14907,6 @@
           <t>4 critical hits</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -14812,7 +14933,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -14839,7 +14959,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -14866,7 +14985,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -14893,7 +15011,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -14920,7 +15037,6 @@
           <t>5c turn delay</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -14947,7 +15063,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -14974,7 +15089,6 @@
           <t>steal</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -15001,7 +15115,6 @@
           <t>steal</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -15028,7 +15141,6 @@
           <t>steal</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -15060,7 +15172,6 @@
           <t>0x480e20</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -15087,7 +15198,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -15114,7 +15224,6 @@
           <t>4 critical hits</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -15141,7 +15250,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -15168,7 +15276,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -15195,7 +15302,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -15222,7 +15328,6 @@
           <t>applying a hit</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -15249,7 +15354,6 @@
           <t>applying a hit</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -15276,7 +15380,6 @@
           <t>applying a hit</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -15308,7 +15411,6 @@
           <t>0x481060</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -15335,7 +15437,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -15367,7 +15468,6 @@
           <t>0x481160</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -15399,7 +15499,6 @@
           <t>0x4813a0</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -15426,7 +15525,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -15453,7 +15551,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -15480,7 +15577,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -15507,7 +15603,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -15534,7 +15629,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -15561,7 +15655,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -15588,7 +15681,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -15615,7 +15707,6 @@
           <t>12.2 number of hits</t>
         </is>
       </c>
-      <c r="H52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -15642,7 +15733,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -15669,7 +15759,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -15696,7 +15785,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -15723,7 +15811,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -15750,7 +15837,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -15777,7 +15863,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -15804,7 +15889,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -15831,7 +15915,6 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
-      <c r="H60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -15858,7 +15941,6 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
-      <c r="H61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -15890,7 +15972,6 @@
           <t>0x4817c0</t>
         </is>
       </c>
-      <c r="H62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -15922,7 +16003,6 @@
           <t>0x481890</t>
         </is>
       </c>
-      <c r="H63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -15954,7 +16034,6 @@
           <t>0x481950</t>
         </is>
       </c>
-      <c r="H64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -15986,7 +16065,6 @@
           <t>0x481a20</t>
         </is>
       </c>
-      <c r="H65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -16013,7 +16091,6 @@
           <t>outside battle</t>
         </is>
       </c>
-      <c r="H66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -16040,7 +16117,6 @@
           <t>outside battle</t>
         </is>
       </c>
-      <c r="H67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -16067,7 +16143,6 @@
           <t>4 critical hits</t>
         </is>
       </c>
-      <c r="H68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -16094,7 +16169,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -16121,7 +16195,6 @@
           <t>9.1 who gets hit</t>
         </is>
       </c>
-      <c r="H70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -16153,7 +16226,6 @@
           <t>0x481ea0</t>
         </is>
       </c>
-      <c r="H71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -16185,7 +16257,6 @@
           <t>0x4822c0</t>
         </is>
       </c>
-      <c r="H72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -16217,7 +16288,6 @@
           <t>0x482530</t>
         </is>
       </c>
-      <c r="H73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -16249,7 +16319,6 @@
           <t>0x4827a0</t>
         </is>
       </c>
-      <c r="H74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -16281,7 +16350,6 @@
           <t>0x482a10</t>
         </is>
       </c>
-      <c r="H75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -16313,7 +16381,6 @@
           <t>0x482c80</t>
         </is>
       </c>
-      <c r="H76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -16345,7 +16412,6 @@
           <t>0x482e40</t>
         </is>
       </c>
-      <c r="H77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -16377,7 +16443,6 @@
           <t>0x4831f0</t>
         </is>
       </c>
-      <c r="H78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -16409,7 +16474,6 @@
           <t>0x4834b0</t>
         </is>
       </c>
-      <c r="H79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -16441,7 +16505,6 @@
           <t>0x4835d0</t>
         </is>
       </c>
-      <c r="H80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -16473,7 +16536,6 @@
           <t>0x483840</t>
         </is>
       </c>
-      <c r="H81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -16500,7 +16562,6 @@
           <t>4 critical hits</t>
         </is>
       </c>
-      <c r="H82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -16532,7 +16593,6 @@
           <t>0x483a60</t>
         </is>
       </c>
-      <c r="H83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -16564,7 +16624,6 @@
           <t>0x483b30</t>
         </is>
       </c>
-      <c r="H84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -16596,7 +16655,6 @@
           <t>0x483c20</t>
         </is>
       </c>
-      <c r="H85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -16628,7 +16686,6 @@
           <t>0x483d20</t>
         </is>
       </c>
-      <c r="H86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -16660,7 +16717,6 @@
           <t>0x483e00</t>
         </is>
       </c>
-      <c r="H87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -16692,7 +16748,6 @@
           <t>0x483ee0</t>
         </is>
       </c>
-      <c r="H88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -16719,7 +16774,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -16746,7 +16800,6 @@
           <t>9.1 who gets hit</t>
         </is>
       </c>
-      <c r="H90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -16773,7 +16826,6 @@
           <t>2.7 special damage</t>
         </is>
       </c>
-      <c r="H91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -16805,7 +16857,6 @@
           <t>0x484020</t>
         </is>
       </c>
-      <c r="H92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -16832,7 +16883,6 @@
           <t>2.7 special damage</t>
         </is>
       </c>
-      <c r="H93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -16859,7 +16909,6 @@
           <t>2.7 special damage</t>
         </is>
       </c>
-      <c r="H94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -16891,7 +16940,6 @@
           <t>0x484150</t>
         </is>
       </c>
-      <c r="H95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -16923,7 +16971,6 @@
           <t>0x484330</t>
         </is>
       </c>
-      <c r="H96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -16950,7 +16997,6 @@
           <t>11.1 dolls</t>
         </is>
       </c>
-      <c r="H97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -16977,7 +17023,6 @@
           <t>2 physical attack, 2.1 hit chance, 3 magic attack</t>
         </is>
       </c>
-      <c r="H98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -17004,7 +17049,6 @@
           <t>2 physical attack, 2.1 hit chance, 3 magic attack</t>
         </is>
       </c>
-      <c r="H99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -17031,7 +17075,6 @@
           <t>12.10 random moves</t>
         </is>
       </c>
-      <c r="H100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -17058,7 +17101,6 @@
           <t>12.10 random moves</t>
         </is>
       </c>
-      <c r="H101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -17085,7 +17127,6 @@
           <t>12.10 random moves</t>
         </is>
       </c>
-      <c r="H102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -17112,7 +17153,6 @@
           <t>12.10 random moves</t>
         </is>
       </c>
-      <c r="H103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -17139,7 +17179,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -17166,7 +17205,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -17193,7 +17231,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -17220,7 +17257,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -17247,7 +17283,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="n">
@@ -17274,7 +17309,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="n">
@@ -17301,7 +17335,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -17333,7 +17366,6 @@
           <t>0x4864c0</t>
         </is>
       </c>
-      <c r="H111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="n">
@@ -17360,7 +17392,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="n">
@@ -17387,7 +17418,6 @@
           <t>9.1 targets</t>
         </is>
       </c>
-      <c r="H113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -17414,7 +17444,6 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
-      <c r="H114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="n">
@@ -17441,7 +17470,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="n">
@@ -17468,7 +17496,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="n">
@@ -17495,7 +17522,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="n">
@@ -17522,7 +17548,6 @@
           <t>2 physical attack, 2.4 damage</t>
         </is>
       </c>
-      <c r="H118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="n">
@@ -17549,7 +17574,6 @@
           <t>applying a hit</t>
         </is>
       </c>
-      <c r="H119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="n">
@@ -17576,7 +17600,6 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
-      <c r="H120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="n">
@@ -17603,7 +17626,6 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
-      <c r="H121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="n">
@@ -17630,7 +17652,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="n">
@@ -17657,7 +17678,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="n">
@@ -17684,7 +17704,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="n">
@@ -17711,7 +17730,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="n">
@@ -17738,7 +17756,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="n">
@@ -17765,7 +17782,6 @@
           <t>2.8 damage received</t>
         </is>
       </c>
-      <c r="H127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="n">
@@ -17792,7 +17808,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="n">
@@ -17819,7 +17834,6 @@
           <t>2 physical attack, 2.4 damage, 3 magic attack</t>
         </is>
       </c>
-      <c r="H129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="n">
@@ -17846,7 +17860,6 @@
           <t>2 physical attack, 2.4 damage</t>
         </is>
       </c>
-      <c r="H130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="n">
@@ -17873,7 +17886,6 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
-      <c r="H131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="n">
@@ -17900,7 +17912,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="n">
@@ -17927,7 +17938,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -17954,7 +17964,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="n">
@@ -17981,7 +17990,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="n">
@@ -18008,7 +18016,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="n">
@@ -18035,7 +18042,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="n">
@@ -18062,7 +18068,6 @@
           <t>5e effects that act every turn</t>
         </is>
       </c>
-      <c r="H138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="n">
@@ -18089,7 +18094,6 @@
           <t>5e effects that act every turn</t>
         </is>
       </c>
-      <c r="H139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="n">
@@ -18116,7 +18120,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="n">
@@ -18143,7 +18146,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="n">
@@ -18170,7 +18172,6 @@
           <t>5d start of a turn</t>
         </is>
       </c>
-      <c r="H142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="n">
@@ -18197,7 +18198,6 @@
           <t>13 Pep</t>
         </is>
       </c>
-      <c r="H143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="n">
@@ -18224,7 +18224,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="n">
@@ -18251,7 +18250,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="n">
@@ -18278,7 +18276,6 @@
           <t>4 critical hits</t>
         </is>
       </c>
-      <c r="H146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="n">
@@ -18305,7 +18302,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="n">
@@ -18332,7 +18328,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="n">
@@ -18359,7 +18354,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="n">
@@ -18391,7 +18385,6 @@
           <t>0x4894a0</t>
         </is>
       </c>
-      <c r="H150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="n">
@@ -18423,7 +18416,6 @@
           <t>0x4895e0</t>
         </is>
       </c>
-      <c r="H151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="n">
@@ -18450,7 +18442,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="n">
@@ -18477,7 +18468,6 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
-      <c r="H153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="n">
@@ -18504,7 +18494,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="n">
@@ -18531,7 +18520,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="n">
@@ -18558,7 +18546,6 @@
           <t>2 physical attack, 2.1 hit chance, 5 order of turns</t>
         </is>
       </c>
-      <c r="H156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="n">
@@ -18585,7 +18572,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" t="n">
@@ -18612,7 +18598,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="n">
@@ -18639,7 +18624,6 @@
           <t>11.1 dolls</t>
         </is>
       </c>
-      <c r="H159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="n">
@@ -18666,7 +18650,6 @@
           <t>11.1 dolls</t>
         </is>
       </c>
-      <c r="H160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" t="n">
@@ -18693,7 +18676,6 @@
           <t>11.1 dolls</t>
         </is>
       </c>
-      <c r="H161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" t="n">
@@ -18720,7 +18702,6 @@
           <t>11.1 dolls</t>
         </is>
       </c>
-      <c r="H162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" t="n">
@@ -18747,7 +18728,6 @@
           <t>11.1 dolls</t>
         </is>
       </c>
-      <c r="H163" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" t="n">
@@ -18774,7 +18754,6 @@
           <t>11.1 dolls</t>
         </is>
       </c>
-      <c r="H164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="n">
@@ -18806,7 +18785,6 @@
           <t>0x48a430</t>
         </is>
       </c>
-      <c r="H165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="n">
@@ -18833,7 +18811,6 @@
           <t>10.1 stats of a piece of equipment</t>
         </is>
       </c>
-      <c r="H166" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" t="n">
@@ -18860,7 +18837,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H167" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" t="n">
@@ -18887,7 +18863,6 @@
           <t>6b healing</t>
         </is>
       </c>
-      <c r="H168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="n">
@@ -18919,7 +18894,6 @@
           <t>0x48a640</t>
         </is>
       </c>
-      <c r="H169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" t="n">
@@ -18946,7 +18920,6 @@
           <t>5e effects that act every turn</t>
         </is>
       </c>
-      <c r="H170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="n">
@@ -18973,7 +18946,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="n">
@@ -19000,7 +18972,6 @@
           <t>12.13 counters and follow-ups</t>
         </is>
       </c>
-      <c r="H172" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" t="n">
@@ -19027,7 +18998,6 @@
           <t>12.13 counters and follow-ups</t>
         </is>
       </c>
-      <c r="H173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="n">
@@ -19054,7 +19024,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H174" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" t="n">
@@ -19081,7 +19050,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" t="n">
@@ -19108,7 +19076,6 @@
           <t>2 physical attack, 2.1 hit chance</t>
         </is>
       </c>
-      <c r="H176" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" t="n">
@@ -19135,7 +19102,6 @@
           <t>passive rolls</t>
         </is>
       </c>
-      <c r="H177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="n">
@@ -19162,7 +19128,6 @@
           <t>passive rolls</t>
         </is>
       </c>
-      <c r="H178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" t="n">
@@ -19189,7 +19154,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H179" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" t="n">
@@ -19216,7 +19180,6 @@
           <t>2.8 damage received</t>
         </is>
       </c>
-      <c r="H180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" t="n">
@@ -19243,7 +19206,6 @@
           <t>2 physical attack, 2.4 damage</t>
         </is>
       </c>
-      <c r="H181" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" t="n">
@@ -19270,7 +19232,6 @@
           <t>5d start of a turn</t>
         </is>
       </c>
-      <c r="H182" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" t="n">
@@ -19297,7 +19258,6 @@
           <t>12.13 counters and follow-ups</t>
         </is>
       </c>
-      <c r="H183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="n">
@@ -19324,7 +19284,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="n">
@@ -19351,7 +19310,6 @@
           <t>12.9 after a hit</t>
         </is>
       </c>
-      <c r="H185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="n">
@@ -19378,7 +19336,6 @@
           <t>2 physical attack, 2.4 damage</t>
         </is>
       </c>
-      <c r="H186" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" t="n">
@@ -19405,7 +19362,6 @@
           <t>2 physical attack, 2.5 chant interruption</t>
         </is>
       </c>
-      <c r="H187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="n">
@@ -19432,7 +19388,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H188" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" t="n">
@@ -19459,7 +19414,6 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
-      <c r="H189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" t="n">
@@ -19486,7 +19440,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H190" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" t="n">
@@ -19513,7 +19466,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" t="n">
@@ -19540,7 +19492,6 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
-      <c r="H192" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" t="n">
@@ -19567,7 +19518,6 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
-      <c r="H193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" t="n">
@@ -19594,7 +19544,6 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
-      <c r="H194" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" t="n">
@@ -19621,7 +19570,6 @@
           <t>after a battle</t>
         </is>
       </c>
-      <c r="H195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" t="n">
@@ -19648,7 +19596,6 @@
           <t>after a battle</t>
         </is>
       </c>
-      <c r="H196" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" t="n">
@@ -19675,7 +19622,6 @@
           <t>passive rolls</t>
         </is>
       </c>
-      <c r="H197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" t="n">
@@ -19702,7 +19648,6 @@
           <t>items</t>
         </is>
       </c>
-      <c r="H198" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" t="n">
@@ -19729,7 +19674,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H199" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" t="n">
@@ -19756,7 +19700,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H200" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" t="n">
@@ -19783,7 +19726,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H201" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" t="n">
@@ -19810,7 +19752,6 @@
           <t>11.2 songs and dances</t>
         </is>
       </c>
-      <c r="H202" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" t="n">
@@ -19837,7 +19778,6 @@
           <t>11.2 songs and dances</t>
         </is>
       </c>
-      <c r="H203" t="inlineStr"/>
     </row>
     <row r="204">
       <c r="A204" t="n">
@@ -19864,7 +19804,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H204" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" t="n">
@@ -19891,7 +19830,6 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
-      <c r="H205" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" t="n">
@@ -19918,7 +19856,6 @@
           <t>5d start of a turn</t>
         </is>
       </c>
-      <c r="H206" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" t="n">
@@ -19945,7 +19882,6 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
-      <c r="H207" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" t="n">
@@ -19972,7 +19908,6 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
-      <c r="H208" t="inlineStr"/>
     </row>
     <row r="209">
       <c r="A209" t="n">
@@ -19999,7 +19934,6 @@
           <t>11.1 dolls, 2 physical attack, 3 magic attack, 6b healing</t>
         </is>
       </c>
-      <c r="H209" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" t="n">
@@ -20026,7 +19960,6 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
-      <c r="H210" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" t="n">
@@ -20053,7 +19986,6 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
-      <c r="H211" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" t="n">
@@ -20080,7 +20012,6 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
-      <c r="H212" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" t="n">
@@ -20107,7 +20038,6 @@
           <t>2.8 damage received</t>
         </is>
       </c>
-      <c r="H213" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" t="n">
@@ -20134,7 +20064,6 @@
           <t>12.9 after a hit</t>
         </is>
       </c>
-      <c r="H214" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" t="n">
@@ -20161,7 +20090,6 @@
           <t>6b heal cap, 6b healing</t>
         </is>
       </c>
-      <c r="H215" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" t="n">
@@ -20188,7 +20116,6 @@
           <t>3 magic attack, 6b heal cap</t>
         </is>
       </c>
-      <c r="H216" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" t="n">
@@ -20215,7 +20142,6 @@
           <t>11.1 dolls</t>
         </is>
       </c>
-      <c r="H217" t="inlineStr"/>
     </row>
     <row r="218">
       <c r="A218" t="n">
@@ -20242,7 +20168,6 @@
           <t>10.1 stats of a piece of equipment</t>
         </is>
       </c>
-      <c r="H218" t="inlineStr"/>
     </row>
     <row r="219">
       <c r="A219" t="n">
@@ -20269,7 +20194,6 @@
           <t>passive rolls</t>
         </is>
       </c>
-      <c r="H219" t="inlineStr"/>
     </row>
     <row r="220">
       <c r="A220" t="n">
@@ -20296,7 +20220,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H220" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" t="n">
@@ -20323,7 +20246,6 @@
           <t>12.13 counters and follow-ups</t>
         </is>
       </c>
-      <c r="H221" t="inlineStr"/>
     </row>
     <row r="222">
       <c r="A222" t="n">
@@ -20350,7 +20272,6 @@
           <t>12.9 after a hit</t>
         </is>
       </c>
-      <c r="H222" t="inlineStr"/>
     </row>
     <row r="223">
       <c r="A223" t="n">
@@ -20377,7 +20298,6 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
-      <c r="H223" t="inlineStr"/>
     </row>
     <row r="224">
       <c r="A224" t="n">
@@ -20404,7 +20324,6 @@
           <t>outside battle</t>
         </is>
       </c>
-      <c r="H224" t="inlineStr"/>
     </row>
     <row r="225">
       <c r="A225" t="n">
@@ -20431,7 +20350,6 @@
           <t>12.13 counters and follow-ups</t>
         </is>
       </c>
-      <c r="H225" t="inlineStr"/>
     </row>
     <row r="226">
       <c r="A226" t="n">
@@ -20458,7 +20376,6 @@
           <t>2 physical attack, 2.4 other bonuses of final damage</t>
         </is>
       </c>
-      <c r="H226" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" t="n">
@@ -20485,7 +20402,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H227" t="inlineStr"/>
     </row>
     <row r="228">
       <c r="A228" t="n">
@@ -20512,7 +20428,6 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
-      <c r="H228" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" t="n">
@@ -20539,7 +20454,6 @@
           <t>5d start of a turn</t>
         </is>
       </c>
-      <c r="H229" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" t="n">
@@ -20566,7 +20480,6 @@
           <t>12.14 after an action</t>
         </is>
       </c>
-      <c r="H230" t="inlineStr"/>
     </row>
     <row r="231">
       <c r="A231" t="n">
@@ -20593,7 +20506,6 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
-      <c r="H231" t="inlineStr"/>
     </row>
     <row r="232">
       <c r="A232" t="n">
@@ -20620,7 +20532,6 @@
           <t>11.1 dolls</t>
         </is>
       </c>
-      <c r="H232" t="inlineStr"/>
     </row>
     <row r="233">
       <c r="A233" t="n">
@@ -20647,7 +20558,6 @@
           <t>12.10 random moves</t>
         </is>
       </c>
-      <c r="H233" t="inlineStr"/>
     </row>
     <row r="234">
       <c r="A234" t="n">
@@ -20674,7 +20584,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H234" t="inlineStr"/>
     </row>
     <row r="235">
       <c r="A235" t="n">
@@ -20701,7 +20610,6 @@
           <t>6b heal cap</t>
         </is>
       </c>
-      <c r="H235" t="inlineStr"/>
     </row>
     <row r="236">
       <c r="A236" t="n">
@@ -20728,7 +20636,6 @@
           <t>9 enemy AI</t>
         </is>
       </c>
-      <c r="H236" t="inlineStr"/>
     </row>
     <row r="237">
       <c r="A237" t="n">
@@ -20755,7 +20662,6 @@
           <t>12.9 after a hit</t>
         </is>
       </c>
-      <c r="H237" t="inlineStr"/>
     </row>
     <row r="238">
       <c r="A238" t="n">
@@ -20782,7 +20688,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H238" t="inlineStr"/>
     </row>
     <row r="239">
       <c r="A239" t="n">
@@ -20809,7 +20714,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H239" t="inlineStr"/>
     </row>
     <row r="240">
       <c r="A240" t="n">
@@ -20836,7 +20740,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H240" t="inlineStr"/>
     </row>
     <row r="241">
       <c r="A241" t="n">
@@ -20863,7 +20766,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H241" t="inlineStr"/>
     </row>
     <row r="242">
       <c r="A242" t="n">
@@ -20890,7 +20792,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H242" t="inlineStr"/>
     </row>
     <row r="243">
       <c r="A243" t="n">
@@ -20917,7 +20818,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H243" t="inlineStr"/>
     </row>
     <row r="244">
       <c r="A244" t="n">
@@ -20944,7 +20844,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H244" t="inlineStr"/>
     </row>
     <row r="245">
       <c r="A245" t="n">
@@ -20971,7 +20870,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H245" t="inlineStr"/>
     </row>
     <row r="246">
       <c r="A246" t="n">
@@ -20998,7 +20896,6 @@
           <t>2 physical attack, 2.1 hit chance, 3 magic attack</t>
         </is>
       </c>
-      <c r="H246" t="inlineStr"/>
     </row>
     <row r="247">
       <c r="A247" t="n">
@@ -21025,7 +20922,6 @@
           <t>2 physical attack, 2.1 hit chance, 3 magic attack</t>
         </is>
       </c>
-      <c r="H247" t="inlineStr"/>
     </row>
     <row r="248">
       <c r="A248" t="n">
@@ -21052,7 +20948,6 @@
           <t>5e effects that act every turn</t>
         </is>
       </c>
-      <c r="H248" t="inlineStr"/>
     </row>
     <row r="249">
       <c r="A249" t="n">
@@ -21079,7 +20974,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H249" t="inlineStr"/>
     </row>
     <row r="250">
       <c r="A250" t="n">
@@ -21106,7 +21000,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H250" t="inlineStr"/>
     </row>
     <row r="251">
       <c r="A251" t="n">
@@ -21133,7 +21026,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H251" t="inlineStr"/>
     </row>
     <row r="252">
       <c r="A252" t="n">
@@ -21160,7 +21052,6 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
-      <c r="H252" t="inlineStr"/>
     </row>
     <row r="253">
       <c r="A253" t="n">
@@ -21187,7 +21078,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H253" t="inlineStr"/>
     </row>
     <row r="254">
       <c r="A254" t="n">
@@ -21214,7 +21104,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H254" t="inlineStr"/>
     </row>
     <row r="255">
       <c r="A255" t="n">
@@ -21241,7 +21130,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H255" t="inlineStr"/>
     </row>
     <row r="256">
       <c r="A256" t="n">
@@ -21268,7 +21156,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H256" t="inlineStr"/>
     </row>
     <row r="257">
       <c r="A257" t="n">
@@ -21295,7 +21182,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H257" t="inlineStr"/>
     </row>
     <row r="258">
       <c r="A258" t="n">
@@ -21322,7 +21208,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H258" t="inlineStr"/>
     </row>
     <row r="259">
       <c r="A259" t="n">
@@ -21349,7 +21234,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H259" t="inlineStr"/>
     </row>
     <row r="260">
       <c r="A260" t="n">
@@ -21376,7 +21260,6 @@
           <t>2 physical attack, 2.4 damage, 3 magic attack</t>
         </is>
       </c>
-      <c r="H260" t="inlineStr"/>
     </row>
     <row r="261">
       <c r="A261" t="n">
@@ -21403,7 +21286,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H261" t="inlineStr"/>
     </row>
     <row r="262">
       <c r="A262" t="n">
@@ -21430,7 +21312,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H262" t="inlineStr"/>
     </row>
     <row r="263">
       <c r="A263" t="n">
@@ -21457,7 +21338,6 @@
           <t>12.10 random moves</t>
         </is>
       </c>
-      <c r="H263" t="inlineStr"/>
     </row>
     <row r="264">
       <c r="A264" t="n">
@@ -21484,7 +21364,6 @@
           <t>12.10 random moves</t>
         </is>
       </c>
-      <c r="H264" t="inlineStr"/>
     </row>
     <row r="265">
       <c r="A265" t="n">
@@ -21511,7 +21390,6 @@
           <t>12.10 random moves</t>
         </is>
       </c>
-      <c r="H265" t="inlineStr"/>
     </row>
     <row r="266">
       <c r="A266" t="n">
@@ -21538,7 +21416,6 @@
           <t>6c EXP</t>
         </is>
       </c>
-      <c r="H266" t="inlineStr"/>
     </row>
     <row r="267">
       <c r="A267" t="n">
@@ -21565,7 +21442,6 @@
           <t>12.10 random moves</t>
         </is>
       </c>
-      <c r="H267" t="inlineStr"/>
     </row>
     <row r="268">
       <c r="A268" t="n">
@@ -21597,7 +21473,6 @@
           <t>0x48b490</t>
         </is>
       </c>
-      <c r="H268" t="inlineStr"/>
     </row>
     <row r="269">
       <c r="A269" t="n">
@@ -21624,7 +21499,6 @@
           <t>2.7 special damage</t>
         </is>
       </c>
-      <c r="H269" t="inlineStr"/>
     </row>
     <row r="270">
       <c r="A270" t="n">
@@ -21651,7 +21525,6 @@
           <t>2.7 special damage</t>
         </is>
       </c>
-      <c r="H270" t="inlineStr"/>
     </row>
     <row r="271">
       <c r="A271" t="n">
@@ -21678,7 +21551,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H271" t="inlineStr"/>
     </row>
     <row r="272">
       <c r="A272" t="n">
@@ -21705,7 +21577,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H272" t="inlineStr"/>
     </row>
     <row r="273">
       <c r="A273" t="n">
@@ -21732,7 +21603,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H273" t="inlineStr"/>
     </row>
     <row r="274">
       <c r="A274" t="n">
@@ -21759,7 +21629,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H274" t="inlineStr"/>
     </row>
     <row r="275">
       <c r="A275" t="n">
@@ -21786,7 +21655,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H275" t="inlineStr"/>
     </row>
     <row r="276">
       <c r="A276" t="n">
@@ -21813,7 +21681,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H276" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -22815,7 +22682,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G47"/>
+  <dimension ref="A1:G48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -24396,6 +24263,43 @@
       <c r="G47" t="inlineStr">
         <is>
           <t>docs/FORMULAS.md 12.16: tested at 0x4503c5 before the roll; 381 of the 516 enemies have it</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>L41</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>The ten values of a unique skill</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>UniqueSkillData.pck</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>0x1C, ten floats</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Benign</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>A chance stays between 0 and 1</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>tools/extract_vanilla.py reads the ten values; docs/FORMULAS.md 12.19 and 16.3</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
balance: arcane Shield sends back 1.5 times as much
arcane Shield sends back 1.5 times as much, Alter Fate x1.5, Tranquil
Song x1.25 (U021 - U050); the note line of a unique skill comes from the
rules for the variant too
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -13376,12 +13376,12 @@
       </c>
       <c r="K177" t="inlineStr">
         <is>
-          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Fiora as healer, without the skill &gt; with it): C36 85% &gt; 89%, C38 98% &gt; 97%, C40 100% &gt; 98%, P24 97% &gt; 99%, P27 crowned 70% &gt; 80%. In the mean +3 points of wins, fights -0% shorter, +3 points of HP left (a cell moves by about 5 points by chance).</t>
+          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Fiora as healer, without the skill &gt; with it): C36 85% &gt; 89%, C38 98% &gt; 97%, C40 100% &gt; 98%, P24 97% &gt; 99%, P27 crowned 70% &gt; 80%. In the mean +3 points of wins, fights -0% shorter, +3 points of HP left (a cell moves by about 5 points by chance). Raised for the feel of it on 2026-10-12: 90.0% without the skill, 94.2% with it (92.6% before)</t>
         </is>
       </c>
       <c r="L177" t="inlineStr">
         <is>
-          <t>not a problem</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="O177" t="inlineStr">
@@ -13394,9 +13394,14 @@
           <t>measured: within what the others give, none above +8% of length or +6 points of wins</t>
         </is>
       </c>
+      <c r="Q177" t="inlineStr">
+        <is>
+          <t>U031 - U040: the chance x1.5 (11 - 23% by rank, 30% crowned)</t>
+        </is>
+      </c>
       <c r="R177" t="inlineStr">
         <is>
-          <t>the user, 2026-10-12: left as it is; it adds little but it is good to have</t>
+          <t>the user, 2026-10-12: raised</t>
         </is>
       </c>
     </row>
@@ -13443,12 +13448,12 @@
       </c>
       <c r="K178" t="inlineStr">
         <is>
-          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Yuni as diva, without the skill &gt; with it): C36 96% &gt; 96%, C38 95% &gt; 95%, C40 93% &gt; 94%, P24 97% &gt; 99%, P27 crowned 83% &gt; 93%. In the mean +3 points of wins, fights +1% shorter, +3 points of HP left (a cell moves by about 5 points by chance).</t>
+          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Yuni as diva, without the skill &gt; with it): C36 96% &gt; 96%, C38 95% &gt; 95%, C40 93% &gt; 94%, P24 97% &gt; 99%, P27 crowned 83% &gt; 93%. In the mean +3 points of wins, fights +1% shorter, +3 points of HP left (a cell moves by about 5 points by chance). Raised a little on 2026-10-12 (the user: it is one of the good ones): 92.8% without the skill, 94.8% with it</t>
         </is>
       </c>
       <c r="L178" t="inlineStr">
         <is>
-          <t>not a problem</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="O178" t="inlineStr">
@@ -13461,9 +13466,14 @@
           <t>measured: within what the others give, none above +8% of length or +6 points of wins</t>
         </is>
       </c>
+      <c r="Q178" t="inlineStr">
+        <is>
+          <t>U041 - U050: the chance x1.25 (9 - 16% by rank, 25% crowned)</t>
+        </is>
+      </c>
       <c r="R178" t="inlineStr">
         <is>
-          <t>the user, 2026-10-12: left as it is; it adds little but it is good to have</t>
+          <t>the user, 2026-10-12: raised</t>
         </is>
       </c>
     </row>
@@ -13649,7 +13659,7 @@
       </c>
       <c r="K181" t="inlineStr">
         <is>
-          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Siena as magical princess, without the skill &gt; with it): C36 79% &gt; 79%, C38 99% &gt; 96%, C40 76% &gt; 79%, P24 85% &gt; 84%, P27 crowned 64% &gt; 73%. In the mean +2 points of wins, fights -3% shorter, +1 points of HP left (a cell moves by about 5 points by chance). Built on 2026-10-12. The measure does not move with it (82.2% as it was, 82.0% at 25%, 80.6% without the skill): what it sends back is a share of the damage she takes, little beside the HP of a boss. Raised for the feel of it, at the word of the user</t>
+          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Siena as magical princess, without the skill &gt; with it): C36 79% &gt; 79%, C38 99% &gt; 96%, C40 76% &gt; 79%, P24 85% &gt; 84%, P27 crowned 64% &gt; 73%. In the mean +2 points of wins, fights -3% shorter, +1 points of HP left (a cell moves by about 5 points by chance). Built on 2026-10-12. The measure does not move with it (82.2% as it was, 82.0% at 25%, 80.6% without the skill): what it sends back is a share of the damage she takes, little beside the HP of a boss. Raised for the feel of it, at the word of the user With both, 81.6% without the skill and 83.0% with it</t>
         </is>
       </c>
       <c r="L181" t="inlineStr">
@@ -13669,7 +13679,7 @@
       </c>
       <c r="Q181" t="inlineStr">
         <is>
-          <t>X13 of the sheet ExePatches (set balance, lever L38): the roll from 15 to 25 in 100; its box worded in balance_skill_text.xlsx</t>
+          <t>X13 of the sheet ExePatches (set balance, lever L38): the roll from 15 to 25 in 100; its box worded in balance_skill_text.xlsx; U021 - U030: the share sent back x1.5 (75 - 150% by rank, 300% crowned)</t>
         </is>
       </c>
       <c r="R181" t="inlineStr">

</xml_diff>

<commit_message>
balance: eccentrics gives the effect of Board Members
eccentrics gives the effect of Board Members (DEX and AGI) in the place
of DEX alone (P091, lever L42); the build writes the effect of a party
skill and words it
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -22692,7 +22692,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G48"/>
+  <dimension ref="A1:G49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -24179,6 +24179,7 @@
         </is>
       </c>
     </row>
+    <row r="41"/>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
@@ -24310,6 +24311,43 @@
       <c r="G48" t="inlineStr">
         <is>
           <t>tools/extract_vanilla.py reads the ten values; docs/FORMULAS.md 12.19 and 16.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>L42</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Which effect a party skill gives its members</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>PartySkillData.pck</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>0x4C, one int</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Benign</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>The id is one of the party effects the program knows (360 - 379, 415)</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>tools/text_checks.py PARTY_EFFECT; the bonus of each effect is worked out at 0x4f9000 - 0x4f94e6. Not seen working in the game yet</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
balance: the unique skill of Lizerietta becomes evasion
the unique skill of Lizerietta becomes evasion (effect 338, named Small
Target; lever L43); RES of Natalia x1.5 (lever L44, the build writes
NPC.pck); Concentrate read again: the program adds where its message
multiplies
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -10141,7 +10141,7 @@
       </c>
       <c r="R132" t="inlineStr">
         <is>
-          <t>2026-10-10: no change; mercenary flavor preserved</t>
+          <t>2026-10-10: no change; mercenary flavor preserved | 2026-10-12: every mercenary measured (scratch/audit_2026-10-11/MERCENARIES.md); none above the summon of the grand sealbook; Natalia, the last, gets RES x1.5 (N001 - N005)</t>
         </is>
       </c>
     </row>
@@ -13190,12 +13190,12 @@
       </c>
       <c r="Q174" t="inlineStr">
         <is>
-          <t>U011 - U020: the chance times 1.6, never over 1 (40 - 91% by rank, certain crowned)</t>
+          <t>U011 - U020, U051: the skill becomes evasion (effect 338, 10 - 26% by rank, 35% with the crown), named again in the variant</t>
         </is>
       </c>
       <c r="R174" t="inlineStr">
         <is>
-          <t>the user, 2026-10-12: raised</t>
+          <t>the user, 2026-10-12: raised | 2026-10-12 (evening), the user: the effect is changed for evasion, which serves in every class and fight</t>
         </is>
       </c>
     </row>
@@ -14392,6 +14392,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -14418,6 +14419,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -14444,6 +14446,7 @@
           <t>12.3 special damage, 2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -14470,6 +14473,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -14496,6 +14500,7 @@
           <t>2.7 special damage</t>
         </is>
       </c>
+      <c r="H6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -14522,6 +14527,7 @@
           <t>6b healing</t>
         </is>
       </c>
+      <c r="H7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -14548,6 +14554,7 @@
           <t>actions</t>
         </is>
       </c>
+      <c r="H8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -14574,6 +14581,7 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
+      <c r="H9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -14600,6 +14608,7 @@
           <t>2.7 special damage, 3 magic attack</t>
         </is>
       </c>
+      <c r="H10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -14626,6 +14635,7 @@
           <t>outside battle</t>
         </is>
       </c>
+      <c r="H11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -14652,6 +14662,7 @@
           <t>14 encounter rate</t>
         </is>
       </c>
+      <c r="H12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -14683,6 +14694,7 @@
           <t>0x47ffc0</t>
         </is>
       </c>
+      <c r="H13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -14709,6 +14721,7 @@
           <t>outside battle</t>
         </is>
       </c>
+      <c r="H14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -14735,6 +14748,7 @@
           <t>12.9 after a hit</t>
         </is>
       </c>
+      <c r="H15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -14761,6 +14775,7 @@
           <t>2 physical attack, 2.2 attack value</t>
         </is>
       </c>
+      <c r="H16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -14787,6 +14802,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -14813,6 +14829,7 @@
           <t>2 physical attack, 2.3 defence value</t>
         </is>
       </c>
+      <c r="H18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -14839,6 +14856,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -14865,6 +14883,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -14891,6 +14910,7 @@
           <t>4 critical hits</t>
         </is>
       </c>
+      <c r="H21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -14917,6 +14937,7 @@
           <t>4 critical hits</t>
         </is>
       </c>
+      <c r="H22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -14943,6 +14964,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -14969,6 +14991,7 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
+      <c r="H24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -14995,6 +15018,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -15021,6 +15045,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -15047,6 +15072,7 @@
           <t>5c turn delay</t>
         </is>
       </c>
+      <c r="H27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -15073,6 +15099,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -15099,6 +15126,7 @@
           <t>steal</t>
         </is>
       </c>
+      <c r="H29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -15125,6 +15153,7 @@
           <t>steal</t>
         </is>
       </c>
+      <c r="H30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -15151,6 +15180,7 @@
           <t>steal</t>
         </is>
       </c>
+      <c r="H31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -15182,6 +15212,7 @@
           <t>0x480e20</t>
         </is>
       </c>
+      <c r="H32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -15208,6 +15239,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -15234,6 +15266,7 @@
           <t>4 critical hits</t>
         </is>
       </c>
+      <c r="H34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -15260,6 +15293,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -15286,6 +15320,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -15312,6 +15347,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -15338,6 +15374,7 @@
           <t>applying a hit</t>
         </is>
       </c>
+      <c r="H38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -15364,6 +15401,7 @@
           <t>applying a hit</t>
         </is>
       </c>
+      <c r="H39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -15390,6 +15428,7 @@
           <t>applying a hit</t>
         </is>
       </c>
+      <c r="H40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -15421,6 +15460,7 @@
           <t>0x481060</t>
         </is>
       </c>
+      <c r="H41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -15447,6 +15487,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -15478,6 +15519,7 @@
           <t>0x481160</t>
         </is>
       </c>
+      <c r="H43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -15509,6 +15551,7 @@
           <t>0x4813a0</t>
         </is>
       </c>
+      <c r="H44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -15535,6 +15578,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -15561,6 +15605,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -15587,6 +15632,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -15613,6 +15659,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -15639,6 +15686,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -15665,6 +15713,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -15691,6 +15740,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -15717,6 +15767,7 @@
           <t>12.2 number of hits</t>
         </is>
       </c>
+      <c r="H52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -15743,6 +15794,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -15769,6 +15821,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -15795,6 +15848,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -15821,6 +15875,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -15847,6 +15902,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -15873,6 +15929,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -15899,6 +15956,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -15925,6 +15983,7 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
+      <c r="H60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -15951,6 +16010,7 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
+      <c r="H61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -15982,6 +16042,7 @@
           <t>0x4817c0</t>
         </is>
       </c>
+      <c r="H62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -16013,6 +16074,7 @@
           <t>0x481890</t>
         </is>
       </c>
+      <c r="H63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -16044,6 +16106,7 @@
           <t>0x481950</t>
         </is>
       </c>
+      <c r="H64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -16075,6 +16138,7 @@
           <t>0x481a20</t>
         </is>
       </c>
+      <c r="H65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -16101,6 +16165,7 @@
           <t>outside battle</t>
         </is>
       </c>
+      <c r="H66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -16127,6 +16192,7 @@
           <t>outside battle</t>
         </is>
       </c>
+      <c r="H67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -16153,6 +16219,7 @@
           <t>4 critical hits</t>
         </is>
       </c>
+      <c r="H68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -16179,6 +16246,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -16205,6 +16273,7 @@
           <t>9.1 who gets hit</t>
         </is>
       </c>
+      <c r="H70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -16236,6 +16305,7 @@
           <t>0x481ea0</t>
         </is>
       </c>
+      <c r="H71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -16267,6 +16337,7 @@
           <t>0x4822c0</t>
         </is>
       </c>
+      <c r="H72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -16298,6 +16369,7 @@
           <t>0x482530</t>
         </is>
       </c>
+      <c r="H73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -16329,6 +16401,7 @@
           <t>0x4827a0</t>
         </is>
       </c>
+      <c r="H74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -16360,6 +16433,7 @@
           <t>0x482a10</t>
         </is>
       </c>
+      <c r="H75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -16391,6 +16465,7 @@
           <t>0x482c80</t>
         </is>
       </c>
+      <c r="H76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -16422,6 +16497,7 @@
           <t>0x482e40</t>
         </is>
       </c>
+      <c r="H77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -16453,6 +16529,7 @@
           <t>0x4831f0</t>
         </is>
       </c>
+      <c r="H78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -16484,6 +16561,7 @@
           <t>0x4834b0</t>
         </is>
       </c>
+      <c r="H79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -16515,6 +16593,7 @@
           <t>0x4835d0</t>
         </is>
       </c>
+      <c r="H80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -16546,6 +16625,7 @@
           <t>0x483840</t>
         </is>
       </c>
+      <c r="H81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -16572,6 +16652,7 @@
           <t>4 critical hits</t>
         </is>
       </c>
+      <c r="H82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -16603,6 +16684,7 @@
           <t>0x483a60</t>
         </is>
       </c>
+      <c r="H83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -16634,6 +16716,7 @@
           <t>0x483b30</t>
         </is>
       </c>
+      <c r="H84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -16665,6 +16748,7 @@
           <t>0x483c20</t>
         </is>
       </c>
+      <c r="H85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -16696,6 +16780,7 @@
           <t>0x483d20</t>
         </is>
       </c>
+      <c r="H86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -16727,6 +16812,7 @@
           <t>0x483e00</t>
         </is>
       </c>
+      <c r="H87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -16758,6 +16844,7 @@
           <t>0x483ee0</t>
         </is>
       </c>
+      <c r="H88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -16784,6 +16871,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -16810,6 +16898,7 @@
           <t>9.1 who gets hit</t>
         </is>
       </c>
+      <c r="H90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -16836,6 +16925,7 @@
           <t>2.7 special damage</t>
         </is>
       </c>
+      <c r="H91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -16867,6 +16957,7 @@
           <t>0x484020</t>
         </is>
       </c>
+      <c r="H92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -16893,6 +16984,7 @@
           <t>2.7 special damage</t>
         </is>
       </c>
+      <c r="H93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -16919,6 +17011,7 @@
           <t>2.7 special damage</t>
         </is>
       </c>
+      <c r="H94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -16950,6 +17043,7 @@
           <t>0x484150</t>
         </is>
       </c>
+      <c r="H95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -16981,6 +17075,7 @@
           <t>0x484330</t>
         </is>
       </c>
+      <c r="H96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -17007,6 +17102,7 @@
           <t>11.1 dolls</t>
         </is>
       </c>
+      <c r="H97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -17033,6 +17129,7 @@
           <t>2 physical attack, 2.1 hit chance, 3 magic attack</t>
         </is>
       </c>
+      <c r="H98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -17059,6 +17156,7 @@
           <t>2 physical attack, 2.1 hit chance, 3 magic attack</t>
         </is>
       </c>
+      <c r="H99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -17085,6 +17183,7 @@
           <t>12.10 random moves</t>
         </is>
       </c>
+      <c r="H100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -17111,6 +17210,7 @@
           <t>12.10 random moves</t>
         </is>
       </c>
+      <c r="H101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -17137,6 +17237,7 @@
           <t>12.10 random moves</t>
         </is>
       </c>
+      <c r="H102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -17163,6 +17264,7 @@
           <t>12.10 random moves</t>
         </is>
       </c>
+      <c r="H103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -17189,6 +17291,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -17215,6 +17318,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -17241,6 +17345,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -17267,6 +17372,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -17293,6 +17399,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="n">
@@ -17319,6 +17426,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="n">
@@ -17345,6 +17453,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -17376,6 +17485,7 @@
           <t>0x4864c0</t>
         </is>
       </c>
+      <c r="H111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="n">
@@ -17402,6 +17512,7 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
+      <c r="H112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="n">
@@ -17428,6 +17539,7 @@
           <t>9.1 targets</t>
         </is>
       </c>
+      <c r="H113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -17454,6 +17566,7 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
+      <c r="H114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="n">
@@ -17480,6 +17593,7 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
+      <c r="H115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="n">
@@ -17506,6 +17620,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="n">
@@ -17532,6 +17647,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="n">
@@ -17558,6 +17674,7 @@
           <t>2 physical attack, 2.4 damage</t>
         </is>
       </c>
+      <c r="H118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="n">
@@ -17584,6 +17701,7 @@
           <t>applying a hit</t>
         </is>
       </c>
+      <c r="H119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="n">
@@ -17610,6 +17728,7 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
+      <c r="H120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="n">
@@ -17636,6 +17755,7 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
+      <c r="H121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="n">
@@ -17662,6 +17782,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="n">
@@ -17688,6 +17809,7 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
+      <c r="H123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="n">
@@ -17714,6 +17836,7 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
+      <c r="H124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="n">
@@ -17740,6 +17863,7 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
+      <c r="H125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="n">
@@ -17766,6 +17890,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="n">
@@ -17792,6 +17917,7 @@
           <t>2.8 damage received</t>
         </is>
       </c>
+      <c r="H127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="n">
@@ -17818,6 +17944,7 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
+      <c r="H128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="n">
@@ -17844,6 +17971,7 @@
           <t>2 physical attack, 2.4 damage, 3 magic attack</t>
         </is>
       </c>
+      <c r="H129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="n">
@@ -17870,6 +17998,7 @@
           <t>2 physical attack, 2.4 damage</t>
         </is>
       </c>
+      <c r="H130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="n">
@@ -17896,6 +18025,7 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
+      <c r="H131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="n">
@@ -17922,6 +18052,7 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
+      <c r="H132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="n">
@@ -17948,6 +18079,7 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
+      <c r="H133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -17974,6 +18106,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="n">
@@ -18000,6 +18133,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="n">
@@ -18026,6 +18160,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="n">
@@ -18052,6 +18187,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="n">
@@ -18078,6 +18214,7 @@
           <t>5e effects that act every turn</t>
         </is>
       </c>
+      <c r="H138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="n">
@@ -18104,6 +18241,7 @@
           <t>5e effects that act every turn</t>
         </is>
       </c>
+      <c r="H139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="n">
@@ -18130,6 +18268,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="n">
@@ -18156,6 +18295,7 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
+      <c r="H141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="n">
@@ -18182,6 +18322,7 @@
           <t>5d start of a turn</t>
         </is>
       </c>
+      <c r="H142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="n">
@@ -18208,6 +18349,7 @@
           <t>13 Pep</t>
         </is>
       </c>
+      <c r="H143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="n">
@@ -18234,6 +18376,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="n">
@@ -18260,6 +18403,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="n">
@@ -18286,6 +18430,7 @@
           <t>4 critical hits</t>
         </is>
       </c>
+      <c r="H146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="n">
@@ -18312,6 +18457,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="n">
@@ -18338,6 +18484,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="n">
@@ -18364,6 +18511,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="n">
@@ -18395,6 +18543,7 @@
           <t>0x4894a0</t>
         </is>
       </c>
+      <c r="H150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="n">
@@ -18426,6 +18575,7 @@
           <t>0x4895e0</t>
         </is>
       </c>
+      <c r="H151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="n">
@@ -18452,6 +18602,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="n">
@@ -18478,6 +18629,7 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
+      <c r="H153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="n">
@@ -18504,6 +18656,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="n">
@@ -18530,6 +18683,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="n">
@@ -18556,6 +18710,7 @@
           <t>2 physical attack, 2.1 hit chance, 5 order of turns</t>
         </is>
       </c>
+      <c r="H156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="n">
@@ -18582,6 +18737,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" t="n">
@@ -18608,6 +18764,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="n">
@@ -18634,6 +18791,7 @@
           <t>11.1 dolls</t>
         </is>
       </c>
+      <c r="H159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="n">
@@ -18660,6 +18818,7 @@
           <t>11.1 dolls</t>
         </is>
       </c>
+      <c r="H160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" t="n">
@@ -18686,6 +18845,7 @@
           <t>11.1 dolls</t>
         </is>
       </c>
+      <c r="H161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" t="n">
@@ -18712,6 +18872,7 @@
           <t>11.1 dolls</t>
         </is>
       </c>
+      <c r="H162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" t="n">
@@ -18738,6 +18899,7 @@
           <t>11.1 dolls</t>
         </is>
       </c>
+      <c r="H163" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" t="n">
@@ -18764,6 +18926,7 @@
           <t>11.1 dolls</t>
         </is>
       </c>
+      <c r="H164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="n">
@@ -18795,6 +18958,7 @@
           <t>0x48a430</t>
         </is>
       </c>
+      <c r="H165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="n">
@@ -18821,6 +18985,7 @@
           <t>10.1 stats of a piece of equipment</t>
         </is>
       </c>
+      <c r="H166" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" t="n">
@@ -18847,6 +19012,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H167" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" t="n">
@@ -18873,6 +19039,7 @@
           <t>6b healing</t>
         </is>
       </c>
+      <c r="H168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="n">
@@ -18904,6 +19071,7 @@
           <t>0x48a640</t>
         </is>
       </c>
+      <c r="H169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" t="n">
@@ -18930,6 +19098,7 @@
           <t>5e effects that act every turn</t>
         </is>
       </c>
+      <c r="H170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="n">
@@ -18956,6 +19125,7 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
+      <c r="H171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="n">
@@ -18982,6 +19152,7 @@
           <t>12.13 counters and follow-ups</t>
         </is>
       </c>
+      <c r="H172" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" t="n">
@@ -19008,6 +19179,7 @@
           <t>12.13 counters and follow-ups</t>
         </is>
       </c>
+      <c r="H173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="n">
@@ -19034,6 +19206,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H174" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" t="n">
@@ -19060,6 +19233,7 @@
           <t>hits of an action</t>
         </is>
       </c>
+      <c r="H175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" t="n">
@@ -19086,6 +19260,7 @@
           <t>2 physical attack, 2.1 hit chance</t>
         </is>
       </c>
+      <c r="H176" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" t="n">
@@ -19112,6 +19287,7 @@
           <t>passive rolls</t>
         </is>
       </c>
+      <c r="H177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="n">
@@ -19138,6 +19314,7 @@
           <t>passive rolls</t>
         </is>
       </c>
+      <c r="H178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" t="n">
@@ -19164,6 +19341,7 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
+      <c r="H179" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" t="n">
@@ -19190,6 +19368,7 @@
           <t>2.8 damage received</t>
         </is>
       </c>
+      <c r="H180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" t="n">
@@ -19216,6 +19395,7 @@
           <t>2 physical attack, 2.4 damage</t>
         </is>
       </c>
+      <c r="H181" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" t="n">
@@ -19242,6 +19422,7 @@
           <t>5d start of a turn</t>
         </is>
       </c>
+      <c r="H182" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" t="n">
@@ -19268,6 +19449,7 @@
           <t>12.13 counters and follow-ups</t>
         </is>
       </c>
+      <c r="H183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="n">
@@ -19294,6 +19476,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="n">
@@ -19320,6 +19503,7 @@
           <t>12.9 after a hit</t>
         </is>
       </c>
+      <c r="H185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="n">
@@ -19346,6 +19530,7 @@
           <t>2 physical attack, 2.4 damage</t>
         </is>
       </c>
+      <c r="H186" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" t="n">
@@ -19372,6 +19557,7 @@
           <t>2 physical attack, 2.5 chant interruption</t>
         </is>
       </c>
+      <c r="H187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="n">
@@ -19398,6 +19584,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H188" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" t="n">
@@ -19424,6 +19611,7 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
+      <c r="H189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" t="n">
@@ -19450,6 +19638,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H190" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" t="n">
@@ -19476,6 +19665,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" t="n">
@@ -19502,6 +19692,7 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
+      <c r="H192" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" t="n">
@@ -19528,6 +19719,7 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
+      <c r="H193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" t="n">
@@ -19554,6 +19746,7 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
+      <c r="H194" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" t="n">
@@ -19580,6 +19773,7 @@
           <t>after a battle</t>
         </is>
       </c>
+      <c r="H195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" t="n">
@@ -19606,6 +19800,7 @@
           <t>after a battle</t>
         </is>
       </c>
+      <c r="H196" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" t="n">
@@ -19632,6 +19827,7 @@
           <t>passive rolls</t>
         </is>
       </c>
+      <c r="H197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" t="n">
@@ -19658,6 +19854,7 @@
           <t>items</t>
         </is>
       </c>
+      <c r="H198" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" t="n">
@@ -19684,6 +19881,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H199" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" t="n">
@@ -19710,6 +19908,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H200" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" t="n">
@@ -19736,6 +19935,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H201" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" t="n">
@@ -19762,6 +19962,7 @@
           <t>11.2 songs and dances</t>
         </is>
       </c>
+      <c r="H202" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" t="n">
@@ -19788,6 +19989,7 @@
           <t>11.2 songs and dances</t>
         </is>
       </c>
+      <c r="H203" t="inlineStr"/>
     </row>
     <row r="204">
       <c r="A204" t="n">
@@ -19814,6 +20016,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H204" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" t="n">
@@ -19840,6 +20043,7 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
+      <c r="H205" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" t="n">
@@ -19866,6 +20070,7 @@
           <t>5d start of a turn</t>
         </is>
       </c>
+      <c r="H206" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" t="n">
@@ -19892,6 +20097,7 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
+      <c r="H207" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" t="n">
@@ -19918,6 +20124,7 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
+      <c r="H208" t="inlineStr"/>
     </row>
     <row r="209">
       <c r="A209" t="n">
@@ -19944,6 +20151,7 @@
           <t>11.1 dolls, 2 physical attack, 3 magic attack, 6b healing</t>
         </is>
       </c>
+      <c r="H209" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" t="n">
@@ -19970,6 +20178,7 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
+      <c r="H210" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" t="n">
@@ -19996,6 +20205,7 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
+      <c r="H211" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" t="n">
@@ -20022,6 +20232,7 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
+      <c r="H212" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" t="n">
@@ -20048,6 +20259,7 @@
           <t>2.8 damage received</t>
         </is>
       </c>
+      <c r="H213" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" t="n">
@@ -20074,6 +20286,7 @@
           <t>12.9 after a hit</t>
         </is>
       </c>
+      <c r="H214" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" t="n">
@@ -20100,6 +20313,7 @@
           <t>6b heal cap, 6b healing</t>
         </is>
       </c>
+      <c r="H215" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" t="n">
@@ -20126,6 +20340,7 @@
           <t>3 magic attack, 6b heal cap</t>
         </is>
       </c>
+      <c r="H216" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" t="n">
@@ -20152,6 +20367,7 @@
           <t>11.1 dolls</t>
         </is>
       </c>
+      <c r="H217" t="inlineStr"/>
     </row>
     <row r="218">
       <c r="A218" t="n">
@@ -20178,6 +20394,7 @@
           <t>10.1 stats of a piece of equipment</t>
         </is>
       </c>
+      <c r="H218" t="inlineStr"/>
     </row>
     <row r="219">
       <c r="A219" t="n">
@@ -20204,6 +20421,7 @@
           <t>passive rolls</t>
         </is>
       </c>
+      <c r="H219" t="inlineStr"/>
     </row>
     <row r="220">
       <c r="A220" t="n">
@@ -20230,6 +20448,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H220" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" t="n">
@@ -20256,6 +20475,7 @@
           <t>12.13 counters and follow-ups</t>
         </is>
       </c>
+      <c r="H221" t="inlineStr"/>
     </row>
     <row r="222">
       <c r="A222" t="n">
@@ -20282,6 +20502,7 @@
           <t>12.9 after a hit</t>
         </is>
       </c>
+      <c r="H222" t="inlineStr"/>
     </row>
     <row r="223">
       <c r="A223" t="n">
@@ -20308,6 +20529,7 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
+      <c r="H223" t="inlineStr"/>
     </row>
     <row r="224">
       <c r="A224" t="n">
@@ -20334,6 +20556,7 @@
           <t>outside battle</t>
         </is>
       </c>
+      <c r="H224" t="inlineStr"/>
     </row>
     <row r="225">
       <c r="A225" t="n">
@@ -20360,6 +20583,7 @@
           <t>12.13 counters and follow-ups</t>
         </is>
       </c>
+      <c r="H225" t="inlineStr"/>
     </row>
     <row r="226">
       <c r="A226" t="n">
@@ -20386,6 +20610,7 @@
           <t>2 physical attack, 2.4 other bonuses of final damage</t>
         </is>
       </c>
+      <c r="H226" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" t="n">
@@ -20412,6 +20637,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H227" t="inlineStr"/>
     </row>
     <row r="228">
       <c r="A228" t="n">
@@ -20438,6 +20664,7 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
+      <c r="H228" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" t="n">
@@ -20464,6 +20691,7 @@
           <t>5d start of a turn</t>
         </is>
       </c>
+      <c r="H229" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" t="n">
@@ -20490,6 +20718,7 @@
           <t>12.14 after an action</t>
         </is>
       </c>
+      <c r="H230" t="inlineStr"/>
     </row>
     <row r="231">
       <c r="A231" t="n">
@@ -20516,6 +20745,7 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
+      <c r="H231" t="inlineStr"/>
     </row>
     <row r="232">
       <c r="A232" t="n">
@@ -20542,6 +20772,7 @@
           <t>11.1 dolls</t>
         </is>
       </c>
+      <c r="H232" t="inlineStr"/>
     </row>
     <row r="233">
       <c r="A233" t="n">
@@ -20568,6 +20799,7 @@
           <t>12.10 random moves</t>
         </is>
       </c>
+      <c r="H233" t="inlineStr"/>
     </row>
     <row r="234">
       <c r="A234" t="n">
@@ -20594,6 +20826,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H234" t="inlineStr"/>
     </row>
     <row r="235">
       <c r="A235" t="n">
@@ -20620,6 +20853,7 @@
           <t>6b heal cap</t>
         </is>
       </c>
+      <c r="H235" t="inlineStr"/>
     </row>
     <row r="236">
       <c r="A236" t="n">
@@ -20646,6 +20880,7 @@
           <t>9 enemy AI</t>
         </is>
       </c>
+      <c r="H236" t="inlineStr"/>
     </row>
     <row r="237">
       <c r="A237" t="n">
@@ -20672,6 +20907,7 @@
           <t>12.9 after a hit</t>
         </is>
       </c>
+      <c r="H237" t="inlineStr"/>
     </row>
     <row r="238">
       <c r="A238" t="n">
@@ -20698,6 +20934,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H238" t="inlineStr"/>
     </row>
     <row r="239">
       <c r="A239" t="n">
@@ -20724,6 +20961,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H239" t="inlineStr"/>
     </row>
     <row r="240">
       <c r="A240" t="n">
@@ -20750,6 +20988,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H240" t="inlineStr"/>
     </row>
     <row r="241">
       <c r="A241" t="n">
@@ -20776,6 +21015,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H241" t="inlineStr"/>
     </row>
     <row r="242">
       <c r="A242" t="n">
@@ -20802,6 +21042,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H242" t="inlineStr"/>
     </row>
     <row r="243">
       <c r="A243" t="n">
@@ -20828,6 +21069,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H243" t="inlineStr"/>
     </row>
     <row r="244">
       <c r="A244" t="n">
@@ -20854,6 +21096,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H244" t="inlineStr"/>
     </row>
     <row r="245">
       <c r="A245" t="n">
@@ -20880,6 +21123,7 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
+      <c r="H245" t="inlineStr"/>
     </row>
     <row r="246">
       <c r="A246" t="n">
@@ -20906,6 +21150,7 @@
           <t>2 physical attack, 2.1 hit chance, 3 magic attack</t>
         </is>
       </c>
+      <c r="H246" t="inlineStr"/>
     </row>
     <row r="247">
       <c r="A247" t="n">
@@ -20932,6 +21177,7 @@
           <t>2 physical attack, 2.1 hit chance, 3 magic attack</t>
         </is>
       </c>
+      <c r="H247" t="inlineStr"/>
     </row>
     <row r="248">
       <c r="A248" t="n">
@@ -20958,6 +21204,7 @@
           <t>5e effects that act every turn</t>
         </is>
       </c>
+      <c r="H248" t="inlineStr"/>
     </row>
     <row r="249">
       <c r="A249" t="n">
@@ -20984,6 +21231,7 @@
           <t>5 order of turns</t>
         </is>
       </c>
+      <c r="H249" t="inlineStr"/>
     </row>
     <row r="250">
       <c r="A250" t="n">
@@ -21010,6 +21258,7 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
+      <c r="H250" t="inlineStr"/>
     </row>
     <row r="251">
       <c r="A251" t="n">
@@ -21036,6 +21285,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H251" t="inlineStr"/>
     </row>
     <row r="252">
       <c r="A252" t="n">
@@ -21062,6 +21312,7 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
+      <c r="H252" t="inlineStr"/>
     </row>
     <row r="253">
       <c r="A253" t="n">
@@ -21088,6 +21339,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H253" t="inlineStr"/>
     </row>
     <row r="254">
       <c r="A254" t="n">
@@ -21114,6 +21366,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H254" t="inlineStr"/>
     </row>
     <row r="255">
       <c r="A255" t="n">
@@ -21140,6 +21393,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H255" t="inlineStr"/>
     </row>
     <row r="256">
       <c r="A256" t="n">
@@ -21166,6 +21420,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H256" t="inlineStr"/>
     </row>
     <row r="257">
       <c r="A257" t="n">
@@ -21192,6 +21447,7 @@
           <t>3 magic attack</t>
         </is>
       </c>
+      <c r="H257" t="inlineStr"/>
     </row>
     <row r="258">
       <c r="A258" t="n">
@@ -21218,6 +21474,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H258" t="inlineStr"/>
     </row>
     <row r="259">
       <c r="A259" t="n">
@@ -21244,6 +21501,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H259" t="inlineStr"/>
     </row>
     <row r="260">
       <c r="A260" t="n">
@@ -21270,6 +21528,7 @@
           <t>2 physical attack, 2.4 damage, 3 magic attack</t>
         </is>
       </c>
+      <c r="H260" t="inlineStr"/>
     </row>
     <row r="261">
       <c r="A261" t="n">
@@ -21296,6 +21555,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H261" t="inlineStr"/>
     </row>
     <row r="262">
       <c r="A262" t="n">
@@ -21322,6 +21582,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H262" t="inlineStr"/>
     </row>
     <row r="263">
       <c r="A263" t="n">
@@ -21348,6 +21609,7 @@
           <t>12.10 random moves</t>
         </is>
       </c>
+      <c r="H263" t="inlineStr"/>
     </row>
     <row r="264">
       <c r="A264" t="n">
@@ -21374,6 +21636,7 @@
           <t>12.10 random moves</t>
         </is>
       </c>
+      <c r="H264" t="inlineStr"/>
     </row>
     <row r="265">
       <c r="A265" t="n">
@@ -21400,6 +21663,7 @@
           <t>12.10 random moves</t>
         </is>
       </c>
+      <c r="H265" t="inlineStr"/>
     </row>
     <row r="266">
       <c r="A266" t="n">
@@ -21426,6 +21690,7 @@
           <t>6c EXP</t>
         </is>
       </c>
+      <c r="H266" t="inlineStr"/>
     </row>
     <row r="267">
       <c r="A267" t="n">
@@ -21452,6 +21717,7 @@
           <t>12.10 random moves</t>
         </is>
       </c>
+      <c r="H267" t="inlineStr"/>
     </row>
     <row r="268">
       <c r="A268" t="n">
@@ -21483,6 +21749,7 @@
           <t>0x48b490</t>
         </is>
       </c>
+      <c r="H268" t="inlineStr"/>
     </row>
     <row r="269">
       <c r="A269" t="n">
@@ -21509,6 +21776,7 @@
           <t>2.7 special damage</t>
         </is>
       </c>
+      <c r="H269" t="inlineStr"/>
     </row>
     <row r="270">
       <c r="A270" t="n">
@@ -21535,6 +21803,7 @@
           <t>2.7 special damage</t>
         </is>
       </c>
+      <c r="H270" t="inlineStr"/>
     </row>
     <row r="271">
       <c r="A271" t="n">
@@ -21561,6 +21830,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H271" t="inlineStr"/>
     </row>
     <row r="272">
       <c r="A272" t="n">
@@ -21587,6 +21857,7 @@
           <t>2 physical attack</t>
         </is>
       </c>
+      <c r="H272" t="inlineStr"/>
     </row>
     <row r="273">
       <c r="A273" t="n">
@@ -21613,6 +21884,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H273" t="inlineStr"/>
     </row>
     <row r="274">
       <c r="A274" t="n">
@@ -21639,6 +21911,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H274" t="inlineStr"/>
     </row>
     <row r="275">
       <c r="A275" t="n">
@@ -21665,6 +21938,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H275" t="inlineStr"/>
     </row>
     <row r="276">
       <c r="A276" t="n">
@@ -21691,6 +21965,7 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
+      <c r="H276" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -22692,7 +22967,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G49"/>
+  <dimension ref="A1:G51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -24179,7 +24454,6 @@
         </is>
       </c>
     </row>
-    <row r="41"/>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
@@ -24348,6 +24622,80 @@
       <c r="G49" t="inlineStr">
         <is>
           <t>tools/text_checks.py PARTY_EFFECT; the bonus of each effect is worked out at 0x4f9000 - 0x4f94e6. Not seen working in the game yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>L43</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Which effect a unique skill is a status of</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>UniqueSkillData.pck</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>0x50, one int</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Benign</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>The effect is one the program reads among the statuses of its bearer, with no skill or roll of its own</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>docs/FORMULAS.md 12.19; the unique skills are looked up as any status (0x47e340 on the lists of the blow function). Not seen working in the game yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>L44</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>A stat of a guest ally at one stage</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>NPC/NPC.pck, NPCData.bin</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>0x20, six ints</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Benign</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>The value stays a whole number above 0</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>tools/npc_data.py (the stats are read at 0x4fed59 - 0x4fee27). Not seen working in the game yet</t>
         </is>
       </c>
     </row>
@@ -25496,12 +25844,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Concentrate: divides the interruption rate of a blow. A spell has no such rate: it breaks a chant only by the second roll of a critical</t>
+          <t>Concentrate: its value is ADDED to max HP * 1.5 + 1 in the divisor of the interruption rate of a blow (the debug message writes a product; the code is addss at 0x44d042), so with values of 0.1 - 0.5 it changes nothing that can be seen. A spell has no such rate: it breaks a chant only by the second roll of a critical</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>0x44cfad; 0x44f12c - 0x44f146</t>
+          <t>0x44cfad, 0x44d02b - 0x44d042; 0x44f12c - 0x44f146</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">

</xml_diff>

<commit_message>
balance: concentrate mended in the program for every unit
concentrate mended in the program for every unit (X14, lever L45: the
interruption rate is divided by 1 + its value, as the message of the
program tells); its box states what it takes off; the QoL box goes back
to the text of the game
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -13699,7 +13699,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -14308,6 +14308,43 @@
       <c r="A19" t="inlineStr">
         <is>
           <t>Factors with the piece of enchantment 270 (X06 to X08: 1.5, 4, 6) and the last band at 10 with or without the piece: accepted by the user on 2026-10-05, after the test in the game. The name of the enchantment in the Balance variant states them (balance_enchant_text.xlsx).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>X14</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>balance</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>L45</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>0x44d044</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>59</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Interruption rate of a blow: max HP * 1.5 times (1 + Concentrate) where the program adds the two (addss -&gt; mulss at 0x44d042; its debug message writes the product). The user, 2026-10-12: mend it for every unit, enemies with the passive too</t>
         </is>
       </c>
     </row>
@@ -14392,7 +14429,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -14419,7 +14455,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -14446,7 +14481,6 @@
           <t>12.3 special damage, 2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -14473,7 +14507,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -14500,7 +14533,6 @@
           <t>2.7 special damage</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -14527,7 +14559,6 @@
           <t>6b healing</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -14554,7 +14585,6 @@
           <t>actions</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -14581,7 +14611,6 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -14608,7 +14637,6 @@
           <t>2.7 special damage, 3 magic attack</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -14635,7 +14663,6 @@
           <t>outside battle</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -14662,7 +14689,6 @@
           <t>14 encounter rate</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -14694,7 +14720,6 @@
           <t>0x47ffc0</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -14721,7 +14746,6 @@
           <t>outside battle</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -14748,7 +14772,6 @@
           <t>12.9 after a hit</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -14775,7 +14798,6 @@
           <t>2 physical attack, 2.2 attack value</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -14802,7 +14824,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -14829,7 +14850,6 @@
           <t>2 physical attack, 2.3 defence value</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -14856,7 +14876,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -14883,7 +14902,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -14910,7 +14928,6 @@
           <t>4 critical hits</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -14937,7 +14954,6 @@
           <t>4 critical hits</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -14964,7 +14980,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -14991,7 +15006,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -15018,7 +15032,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -15045,7 +15058,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -15072,7 +15084,6 @@
           <t>5c turn delay</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -15099,7 +15110,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -15126,7 +15136,6 @@
           <t>steal</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -15153,7 +15162,6 @@
           <t>steal</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -15180,7 +15188,6 @@
           <t>steal</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -15212,7 +15219,6 @@
           <t>0x480e20</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -15239,7 +15245,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -15266,7 +15271,6 @@
           <t>4 critical hits</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -15293,7 +15297,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -15320,7 +15323,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -15347,7 +15349,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -15374,7 +15375,6 @@
           <t>applying a hit</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -15401,7 +15401,6 @@
           <t>applying a hit</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -15428,7 +15427,6 @@
           <t>applying a hit</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -15460,7 +15458,6 @@
           <t>0x481060</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -15487,7 +15484,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -15519,7 +15515,6 @@
           <t>0x481160</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -15551,7 +15546,6 @@
           <t>0x4813a0</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -15578,7 +15572,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -15605,7 +15598,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -15632,7 +15624,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -15659,7 +15650,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -15686,7 +15676,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -15713,7 +15702,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -15740,7 +15728,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -15767,7 +15754,6 @@
           <t>12.2 number of hits</t>
         </is>
       </c>
-      <c r="H52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -15794,7 +15780,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -15821,7 +15806,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -15848,7 +15832,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -15875,7 +15858,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -15902,7 +15884,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -15929,7 +15910,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -15956,7 +15936,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -15983,7 +15962,6 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
-      <c r="H60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -16010,7 +15988,6 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
-      <c r="H61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -16042,7 +16019,6 @@
           <t>0x4817c0</t>
         </is>
       </c>
-      <c r="H62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -16074,7 +16050,6 @@
           <t>0x481890</t>
         </is>
       </c>
-      <c r="H63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -16106,7 +16081,6 @@
           <t>0x481950</t>
         </is>
       </c>
-      <c r="H64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -16138,7 +16112,6 @@
           <t>0x481a20</t>
         </is>
       </c>
-      <c r="H65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -16165,7 +16138,6 @@
           <t>outside battle</t>
         </is>
       </c>
-      <c r="H66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -16192,7 +16164,6 @@
           <t>outside battle</t>
         </is>
       </c>
-      <c r="H67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -16219,7 +16190,6 @@
           <t>4 critical hits</t>
         </is>
       </c>
-      <c r="H68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -16246,7 +16216,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -16273,7 +16242,6 @@
           <t>9.1 who gets hit</t>
         </is>
       </c>
-      <c r="H70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -16305,7 +16273,6 @@
           <t>0x481ea0</t>
         </is>
       </c>
-      <c r="H71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -16337,7 +16304,6 @@
           <t>0x4822c0</t>
         </is>
       </c>
-      <c r="H72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -16369,7 +16335,6 @@
           <t>0x482530</t>
         </is>
       </c>
-      <c r="H73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -16401,7 +16366,6 @@
           <t>0x4827a0</t>
         </is>
       </c>
-      <c r="H74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -16433,7 +16397,6 @@
           <t>0x482a10</t>
         </is>
       </c>
-      <c r="H75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -16465,7 +16428,6 @@
           <t>0x482c80</t>
         </is>
       </c>
-      <c r="H76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -16497,7 +16459,6 @@
           <t>0x482e40</t>
         </is>
       </c>
-      <c r="H77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -16529,7 +16490,6 @@
           <t>0x4831f0</t>
         </is>
       </c>
-      <c r="H78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -16561,7 +16521,6 @@
           <t>0x4834b0</t>
         </is>
       </c>
-      <c r="H79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -16593,7 +16552,6 @@
           <t>0x4835d0</t>
         </is>
       </c>
-      <c r="H80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -16625,7 +16583,6 @@
           <t>0x483840</t>
         </is>
       </c>
-      <c r="H81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -16652,7 +16609,6 @@
           <t>4 critical hits</t>
         </is>
       </c>
-      <c r="H82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -16684,7 +16640,6 @@
           <t>0x483a60</t>
         </is>
       </c>
-      <c r="H83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -16716,7 +16671,6 @@
           <t>0x483b30</t>
         </is>
       </c>
-      <c r="H84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -16748,7 +16702,6 @@
           <t>0x483c20</t>
         </is>
       </c>
-      <c r="H85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -16780,7 +16733,6 @@
           <t>0x483d20</t>
         </is>
       </c>
-      <c r="H86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -16812,7 +16764,6 @@
           <t>0x483e00</t>
         </is>
       </c>
-      <c r="H87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -16844,7 +16795,6 @@
           <t>0x483ee0</t>
         </is>
       </c>
-      <c r="H88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -16871,7 +16821,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -16898,7 +16847,6 @@
           <t>9.1 who gets hit</t>
         </is>
       </c>
-      <c r="H90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -16925,7 +16873,6 @@
           <t>2.7 special damage</t>
         </is>
       </c>
-      <c r="H91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -16957,7 +16904,6 @@
           <t>0x484020</t>
         </is>
       </c>
-      <c r="H92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -16984,7 +16930,6 @@
           <t>2.7 special damage</t>
         </is>
       </c>
-      <c r="H93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -17011,7 +16956,6 @@
           <t>2.7 special damage</t>
         </is>
       </c>
-      <c r="H94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -17043,7 +16987,6 @@
           <t>0x484150</t>
         </is>
       </c>
-      <c r="H95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -17075,7 +17018,6 @@
           <t>0x484330</t>
         </is>
       </c>
-      <c r="H96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -17102,7 +17044,6 @@
           <t>11.1 dolls</t>
         </is>
       </c>
-      <c r="H97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -17129,7 +17070,6 @@
           <t>2 physical attack, 2.1 hit chance, 3 magic attack</t>
         </is>
       </c>
-      <c r="H98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -17156,7 +17096,6 @@
           <t>2 physical attack, 2.1 hit chance, 3 magic attack</t>
         </is>
       </c>
-      <c r="H99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -17183,7 +17122,6 @@
           <t>12.10 random moves</t>
         </is>
       </c>
-      <c r="H100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -17210,7 +17148,6 @@
           <t>12.10 random moves</t>
         </is>
       </c>
-      <c r="H101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -17237,7 +17174,6 @@
           <t>12.10 random moves</t>
         </is>
       </c>
-      <c r="H102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -17264,7 +17200,6 @@
           <t>12.10 random moves</t>
         </is>
       </c>
-      <c r="H103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -17291,7 +17226,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -17318,7 +17252,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -17345,7 +17278,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -17372,7 +17304,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -17399,7 +17330,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="n">
@@ -17426,7 +17356,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="n">
@@ -17453,7 +17382,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -17485,7 +17413,6 @@
           <t>0x4864c0</t>
         </is>
       </c>
-      <c r="H111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="n">
@@ -17512,7 +17439,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="n">
@@ -17539,7 +17465,6 @@
           <t>9.1 targets</t>
         </is>
       </c>
-      <c r="H113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -17566,7 +17491,6 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
-      <c r="H114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="n">
@@ -17593,7 +17517,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="n">
@@ -17620,7 +17543,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="n">
@@ -17647,7 +17569,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="n">
@@ -17674,7 +17595,6 @@
           <t>2 physical attack, 2.4 damage</t>
         </is>
       </c>
-      <c r="H118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="n">
@@ -17701,7 +17621,6 @@
           <t>applying a hit</t>
         </is>
       </c>
-      <c r="H119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="n">
@@ -17728,7 +17647,6 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
-      <c r="H120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="n">
@@ -17755,7 +17673,6 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
-      <c r="H121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="n">
@@ -17782,7 +17699,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="n">
@@ -17809,7 +17725,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="n">
@@ -17836,7 +17751,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="n">
@@ -17863,7 +17777,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="n">
@@ -17890,7 +17803,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="n">
@@ -17917,7 +17829,6 @@
           <t>2.8 damage received</t>
         </is>
       </c>
-      <c r="H127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="n">
@@ -17944,7 +17855,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="n">
@@ -17971,7 +17881,6 @@
           <t>2 physical attack, 2.4 damage, 3 magic attack</t>
         </is>
       </c>
-      <c r="H129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="n">
@@ -17998,7 +17907,6 @@
           <t>2 physical attack, 2.4 damage</t>
         </is>
       </c>
-      <c r="H130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="n">
@@ -18025,7 +17933,6 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
-      <c r="H131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="n">
@@ -18052,7 +17959,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="n">
@@ -18079,7 +17985,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -18106,7 +18011,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="n">
@@ -18133,7 +18037,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="n">
@@ -18160,7 +18063,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="n">
@@ -18187,7 +18089,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="n">
@@ -18214,7 +18115,6 @@
           <t>5e effects that act every turn</t>
         </is>
       </c>
-      <c r="H138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="n">
@@ -18241,7 +18141,6 @@
           <t>5e effects that act every turn</t>
         </is>
       </c>
-      <c r="H139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="n">
@@ -18268,7 +18167,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="n">
@@ -18295,7 +18193,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="n">
@@ -18322,7 +18219,6 @@
           <t>5d start of a turn</t>
         </is>
       </c>
-      <c r="H142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="n">
@@ -18349,7 +18245,6 @@
           <t>13 Pep</t>
         </is>
       </c>
-      <c r="H143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="n">
@@ -18376,7 +18271,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="n">
@@ -18403,7 +18297,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="n">
@@ -18430,7 +18323,6 @@
           <t>4 critical hits</t>
         </is>
       </c>
-      <c r="H146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="n">
@@ -18457,7 +18349,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="n">
@@ -18484,7 +18375,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="n">
@@ -18511,7 +18401,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="n">
@@ -18543,7 +18432,6 @@
           <t>0x4894a0</t>
         </is>
       </c>
-      <c r="H150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="n">
@@ -18575,7 +18463,6 @@
           <t>0x4895e0</t>
         </is>
       </c>
-      <c r="H151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="n">
@@ -18602,7 +18489,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="n">
@@ -18629,7 +18515,6 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
-      <c r="H153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="n">
@@ -18656,7 +18541,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="n">
@@ -18683,7 +18567,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="n">
@@ -18710,7 +18593,6 @@
           <t>2 physical attack, 2.1 hit chance, 5 order of turns</t>
         </is>
       </c>
-      <c r="H156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="n">
@@ -18737,7 +18619,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" t="n">
@@ -18764,7 +18645,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="n">
@@ -18791,7 +18671,6 @@
           <t>11.1 dolls</t>
         </is>
       </c>
-      <c r="H159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="n">
@@ -18818,7 +18697,6 @@
           <t>11.1 dolls</t>
         </is>
       </c>
-      <c r="H160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" t="n">
@@ -18845,7 +18723,6 @@
           <t>11.1 dolls</t>
         </is>
       </c>
-      <c r="H161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" t="n">
@@ -18872,7 +18749,6 @@
           <t>11.1 dolls</t>
         </is>
       </c>
-      <c r="H162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" t="n">
@@ -18899,7 +18775,6 @@
           <t>11.1 dolls</t>
         </is>
       </c>
-      <c r="H163" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" t="n">
@@ -18926,7 +18801,6 @@
           <t>11.1 dolls</t>
         </is>
       </c>
-      <c r="H164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="n">
@@ -18958,7 +18832,6 @@
           <t>0x48a430</t>
         </is>
       </c>
-      <c r="H165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="n">
@@ -18985,7 +18858,6 @@
           <t>10.1 stats of a piece of equipment</t>
         </is>
       </c>
-      <c r="H166" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" t="n">
@@ -19012,7 +18884,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H167" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" t="n">
@@ -19039,7 +18910,6 @@
           <t>6b healing</t>
         </is>
       </c>
-      <c r="H168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="n">
@@ -19071,7 +18941,6 @@
           <t>0x48a640</t>
         </is>
       </c>
-      <c r="H169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" t="n">
@@ -19098,7 +18967,6 @@
           <t>5e effects that act every turn</t>
         </is>
       </c>
-      <c r="H170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="n">
@@ -19125,7 +18993,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="n">
@@ -19152,7 +19019,6 @@
           <t>12.13 counters and follow-ups</t>
         </is>
       </c>
-      <c r="H172" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" t="n">
@@ -19179,7 +19045,6 @@
           <t>12.13 counters and follow-ups</t>
         </is>
       </c>
-      <c r="H173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="n">
@@ -19206,7 +19071,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H174" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" t="n">
@@ -19233,7 +19097,6 @@
           <t>hits of an action</t>
         </is>
       </c>
-      <c r="H175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" t="n">
@@ -19260,7 +19123,6 @@
           <t>2 physical attack, 2.1 hit chance</t>
         </is>
       </c>
-      <c r="H176" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" t="n">
@@ -19287,7 +19149,6 @@
           <t>passive rolls</t>
         </is>
       </c>
-      <c r="H177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="n">
@@ -19314,7 +19175,6 @@
           <t>passive rolls</t>
         </is>
       </c>
-      <c r="H178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" t="n">
@@ -19341,7 +19201,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H179" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" t="n">
@@ -19368,7 +19227,6 @@
           <t>2.8 damage received</t>
         </is>
       </c>
-      <c r="H180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" t="n">
@@ -19395,7 +19253,6 @@
           <t>2 physical attack, 2.4 damage</t>
         </is>
       </c>
-      <c r="H181" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" t="n">
@@ -19422,7 +19279,6 @@
           <t>5d start of a turn</t>
         </is>
       </c>
-      <c r="H182" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" t="n">
@@ -19449,7 +19305,6 @@
           <t>12.13 counters and follow-ups</t>
         </is>
       </c>
-      <c r="H183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="n">
@@ -19476,7 +19331,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="n">
@@ -19503,7 +19357,6 @@
           <t>12.9 after a hit</t>
         </is>
       </c>
-      <c r="H185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="n">
@@ -19530,7 +19383,6 @@
           <t>2 physical attack, 2.4 damage</t>
         </is>
       </c>
-      <c r="H186" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" t="n">
@@ -19557,7 +19409,6 @@
           <t>2 physical attack, 2.5 chant interruption</t>
         </is>
       </c>
-      <c r="H187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="n">
@@ -19584,7 +19435,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H188" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" t="n">
@@ -19611,7 +19461,6 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
-      <c r="H189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" t="n">
@@ -19638,7 +19487,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H190" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" t="n">
@@ -19665,7 +19513,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" t="n">
@@ -19692,7 +19539,6 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
-      <c r="H192" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" t="n">
@@ -19719,7 +19565,6 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
-      <c r="H193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" t="n">
@@ -19746,7 +19591,6 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
-      <c r="H194" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" t="n">
@@ -19773,7 +19617,6 @@
           <t>after a battle</t>
         </is>
       </c>
-      <c r="H195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" t="n">
@@ -19800,7 +19643,6 @@
           <t>after a battle</t>
         </is>
       </c>
-      <c r="H196" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" t="n">
@@ -19827,7 +19669,6 @@
           <t>passive rolls</t>
         </is>
       </c>
-      <c r="H197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" t="n">
@@ -19854,7 +19695,6 @@
           <t>items</t>
         </is>
       </c>
-      <c r="H198" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" t="n">
@@ -19881,7 +19721,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H199" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" t="n">
@@ -19908,7 +19747,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H200" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" t="n">
@@ -19935,7 +19773,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H201" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" t="n">
@@ -19962,7 +19799,6 @@
           <t>11.2 songs and dances</t>
         </is>
       </c>
-      <c r="H202" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" t="n">
@@ -19989,7 +19825,6 @@
           <t>11.2 songs and dances</t>
         </is>
       </c>
-      <c r="H203" t="inlineStr"/>
     </row>
     <row r="204">
       <c r="A204" t="n">
@@ -20016,7 +19851,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H204" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" t="n">
@@ -20043,7 +19877,6 @@
           <t>12.11 passives outside the formulas</t>
         </is>
       </c>
-      <c r="H205" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" t="n">
@@ -20070,7 +19903,6 @@
           <t>5d start of a turn</t>
         </is>
       </c>
-      <c r="H206" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" t="n">
@@ -20097,7 +19929,6 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
-      <c r="H207" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" t="n">
@@ -20124,7 +19955,6 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
-      <c r="H208" t="inlineStr"/>
     </row>
     <row r="209">
       <c r="A209" t="n">
@@ -20151,7 +19981,6 @@
           <t>11.1 dolls, 2 physical attack, 3 magic attack, 6b healing</t>
         </is>
       </c>
-      <c r="H209" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" t="n">
@@ -20178,7 +20007,6 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
-      <c r="H210" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" t="n">
@@ -20205,7 +20033,6 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
-      <c r="H211" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" t="n">
@@ -20232,7 +20059,6 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
-      <c r="H212" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" t="n">
@@ -20259,7 +20085,6 @@
           <t>2.8 damage received</t>
         </is>
       </c>
-      <c r="H213" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" t="n">
@@ -20286,7 +20111,6 @@
           <t>12.9 after a hit</t>
         </is>
       </c>
-      <c r="H214" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" t="n">
@@ -20313,7 +20137,6 @@
           <t>6b heal cap, 6b healing</t>
         </is>
       </c>
-      <c r="H215" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" t="n">
@@ -20340,7 +20163,6 @@
           <t>3 magic attack, 6b heal cap</t>
         </is>
       </c>
-      <c r="H216" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" t="n">
@@ -20367,7 +20189,6 @@
           <t>11.1 dolls</t>
         </is>
       </c>
-      <c r="H217" t="inlineStr"/>
     </row>
     <row r="218">
       <c r="A218" t="n">
@@ -20394,7 +20215,6 @@
           <t>10.1 stats of a piece of equipment</t>
         </is>
       </c>
-      <c r="H218" t="inlineStr"/>
     </row>
     <row r="219">
       <c r="A219" t="n">
@@ -20421,7 +20241,6 @@
           <t>passive rolls</t>
         </is>
       </c>
-      <c r="H219" t="inlineStr"/>
     </row>
     <row r="220">
       <c r="A220" t="n">
@@ -20448,7 +20267,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H220" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" t="n">
@@ -20475,7 +20293,6 @@
           <t>12.13 counters and follow-ups</t>
         </is>
       </c>
-      <c r="H221" t="inlineStr"/>
     </row>
     <row r="222">
       <c r="A222" t="n">
@@ -20502,7 +20319,6 @@
           <t>12.9 after a hit</t>
         </is>
       </c>
-      <c r="H222" t="inlineStr"/>
     </row>
     <row r="223">
       <c r="A223" t="n">
@@ -20529,7 +20345,6 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
-      <c r="H223" t="inlineStr"/>
     </row>
     <row r="224">
       <c r="A224" t="n">
@@ -20556,7 +20371,6 @@
           <t>outside battle</t>
         </is>
       </c>
-      <c r="H224" t="inlineStr"/>
     </row>
     <row r="225">
       <c r="A225" t="n">
@@ -20583,7 +20397,6 @@
           <t>12.13 counters and follow-ups</t>
         </is>
       </c>
-      <c r="H225" t="inlineStr"/>
     </row>
     <row r="226">
       <c r="A226" t="n">
@@ -20610,7 +20423,6 @@
           <t>2 physical attack, 2.4 other bonuses of final damage</t>
         </is>
       </c>
-      <c r="H226" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" t="n">
@@ -20637,7 +20449,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H227" t="inlineStr"/>
     </row>
     <row r="228">
       <c r="A228" t="n">
@@ -20664,7 +20475,6 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
-      <c r="H228" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" t="n">
@@ -20691,7 +20501,6 @@
           <t>5d start of a turn</t>
         </is>
       </c>
-      <c r="H229" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" t="n">
@@ -20718,7 +20527,6 @@
           <t>12.14 after an action</t>
         </is>
       </c>
-      <c r="H230" t="inlineStr"/>
     </row>
     <row r="231">
       <c r="A231" t="n">
@@ -20745,7 +20553,6 @@
           <t>12.14 after an action and after a battle</t>
         </is>
       </c>
-      <c r="H231" t="inlineStr"/>
     </row>
     <row r="232">
       <c r="A232" t="n">
@@ -20772,7 +20579,6 @@
           <t>11.1 dolls</t>
         </is>
       </c>
-      <c r="H232" t="inlineStr"/>
     </row>
     <row r="233">
       <c r="A233" t="n">
@@ -20799,7 +20605,6 @@
           <t>12.10 random moves</t>
         </is>
       </c>
-      <c r="H233" t="inlineStr"/>
     </row>
     <row r="234">
       <c r="A234" t="n">
@@ -20826,7 +20631,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H234" t="inlineStr"/>
     </row>
     <row r="235">
       <c r="A235" t="n">
@@ -20853,7 +20657,6 @@
           <t>6b heal cap</t>
         </is>
       </c>
-      <c r="H235" t="inlineStr"/>
     </row>
     <row r="236">
       <c r="A236" t="n">
@@ -20880,7 +20683,6 @@
           <t>9 enemy AI</t>
         </is>
       </c>
-      <c r="H236" t="inlineStr"/>
     </row>
     <row r="237">
       <c r="A237" t="n">
@@ -20907,7 +20709,6 @@
           <t>12.9 after a hit</t>
         </is>
       </c>
-      <c r="H237" t="inlineStr"/>
     </row>
     <row r="238">
       <c r="A238" t="n">
@@ -20934,7 +20735,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H238" t="inlineStr"/>
     </row>
     <row r="239">
       <c r="A239" t="n">
@@ -20961,7 +20761,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H239" t="inlineStr"/>
     </row>
     <row r="240">
       <c r="A240" t="n">
@@ -20988,7 +20787,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H240" t="inlineStr"/>
     </row>
     <row r="241">
       <c r="A241" t="n">
@@ -21015,7 +20813,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H241" t="inlineStr"/>
     </row>
     <row r="242">
       <c r="A242" t="n">
@@ -21042,7 +20839,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H242" t="inlineStr"/>
     </row>
     <row r="243">
       <c r="A243" t="n">
@@ -21069,7 +20865,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H243" t="inlineStr"/>
     </row>
     <row r="244">
       <c r="A244" t="n">
@@ -21096,7 +20891,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H244" t="inlineStr"/>
     </row>
     <row r="245">
       <c r="A245" t="n">
@@ -21123,7 +20917,6 @@
           <t>2 physical attack, 3 magic attack</t>
         </is>
       </c>
-      <c r="H245" t="inlineStr"/>
     </row>
     <row r="246">
       <c r="A246" t="n">
@@ -21150,7 +20943,6 @@
           <t>2 physical attack, 2.1 hit chance, 3 magic attack</t>
         </is>
       </c>
-      <c r="H246" t="inlineStr"/>
     </row>
     <row r="247">
       <c r="A247" t="n">
@@ -21177,7 +20969,6 @@
           <t>2 physical attack, 2.1 hit chance, 3 magic attack</t>
         </is>
       </c>
-      <c r="H247" t="inlineStr"/>
     </row>
     <row r="248">
       <c r="A248" t="n">
@@ -21204,7 +20995,6 @@
           <t>5e effects that act every turn</t>
         </is>
       </c>
-      <c r="H248" t="inlineStr"/>
     </row>
     <row r="249">
       <c r="A249" t="n">
@@ -21231,7 +21021,6 @@
           <t>5 order of turns</t>
         </is>
       </c>
-      <c r="H249" t="inlineStr"/>
     </row>
     <row r="250">
       <c r="A250" t="n">
@@ -21258,7 +21047,6 @@
           <t>10.2 statuses on stats</t>
         </is>
       </c>
-      <c r="H250" t="inlineStr"/>
     </row>
     <row r="251">
       <c r="A251" t="n">
@@ -21285,7 +21073,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H251" t="inlineStr"/>
     </row>
     <row r="252">
       <c r="A252" t="n">
@@ -21312,7 +21099,6 @@
           <t>12.12 who takes the hit</t>
         </is>
       </c>
-      <c r="H252" t="inlineStr"/>
     </row>
     <row r="253">
       <c r="A253" t="n">
@@ -21339,7 +21125,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H253" t="inlineStr"/>
     </row>
     <row r="254">
       <c r="A254" t="n">
@@ -21366,7 +21151,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H254" t="inlineStr"/>
     </row>
     <row r="255">
       <c r="A255" t="n">
@@ -21393,7 +21177,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H255" t="inlineStr"/>
     </row>
     <row r="256">
       <c r="A256" t="n">
@@ -21420,7 +21203,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H256" t="inlineStr"/>
     </row>
     <row r="257">
       <c r="A257" t="n">
@@ -21447,7 +21229,6 @@
           <t>3 magic attack</t>
         </is>
       </c>
-      <c r="H257" t="inlineStr"/>
     </row>
     <row r="258">
       <c r="A258" t="n">
@@ -21474,7 +21255,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H258" t="inlineStr"/>
     </row>
     <row r="259">
       <c r="A259" t="n">
@@ -21501,7 +21281,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H259" t="inlineStr"/>
     </row>
     <row r="260">
       <c r="A260" t="n">
@@ -21528,7 +21307,6 @@
           <t>2 physical attack, 2.4 damage, 3 magic attack</t>
         </is>
       </c>
-      <c r="H260" t="inlineStr"/>
     </row>
     <row r="261">
       <c r="A261" t="n">
@@ -21555,7 +21333,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H261" t="inlineStr"/>
     </row>
     <row r="262">
       <c r="A262" t="n">
@@ -21582,7 +21359,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H262" t="inlineStr"/>
     </row>
     <row r="263">
       <c r="A263" t="n">
@@ -21609,7 +21385,6 @@
           <t>12.10 random moves</t>
         </is>
       </c>
-      <c r="H263" t="inlineStr"/>
     </row>
     <row r="264">
       <c r="A264" t="n">
@@ -21636,7 +21411,6 @@
           <t>12.10 random moves</t>
         </is>
       </c>
-      <c r="H264" t="inlineStr"/>
     </row>
     <row r="265">
       <c r="A265" t="n">
@@ -21663,7 +21437,6 @@
           <t>12.10 random moves</t>
         </is>
       </c>
-      <c r="H265" t="inlineStr"/>
     </row>
     <row r="266">
       <c r="A266" t="n">
@@ -21690,7 +21463,6 @@
           <t>6c EXP</t>
         </is>
       </c>
-      <c r="H266" t="inlineStr"/>
     </row>
     <row r="267">
       <c r="A267" t="n">
@@ -21717,7 +21489,6 @@
           <t>12.10 random moves</t>
         </is>
       </c>
-      <c r="H267" t="inlineStr"/>
     </row>
     <row r="268">
       <c r="A268" t="n">
@@ -21749,7 +21520,6 @@
           <t>0x48b490</t>
         </is>
       </c>
-      <c r="H268" t="inlineStr"/>
     </row>
     <row r="269">
       <c r="A269" t="n">
@@ -21776,7 +21546,6 @@
           <t>2.7 special damage</t>
         </is>
       </c>
-      <c r="H269" t="inlineStr"/>
     </row>
     <row r="270">
       <c r="A270" t="n">
@@ -21803,7 +21572,6 @@
           <t>2.7 special damage</t>
         </is>
       </c>
-      <c r="H270" t="inlineStr"/>
     </row>
     <row r="271">
       <c r="A271" t="n">
@@ -21830,7 +21598,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H271" t="inlineStr"/>
     </row>
     <row r="272">
       <c r="A272" t="n">
@@ -21857,7 +21624,6 @@
           <t>2 physical attack</t>
         </is>
       </c>
-      <c r="H272" t="inlineStr"/>
     </row>
     <row r="273">
       <c r="A273" t="n">
@@ -21884,7 +21650,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H273" t="inlineStr"/>
     </row>
     <row r="274">
       <c r="A274" t="n">
@@ -21911,7 +21676,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H274" t="inlineStr"/>
     </row>
     <row r="275">
       <c r="A275" t="n">
@@ -21938,7 +21702,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H275" t="inlineStr"/>
     </row>
     <row r="276">
       <c r="A276" t="n">
@@ -21965,7 +21728,6 @@
           <t>12.19 unique skills</t>
         </is>
       </c>
-      <c r="H276" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -22967,7 +22729,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G51"/>
+  <dimension ref="A1:G52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -24696,6 +24458,43 @@
       <c r="G51" t="inlineStr">
         <is>
           <t>tools/npc_data.py (the stats are read at 0x4fed59 - 0x4fee27). Not seen working in the game yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>L45</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Concentrate divides the interruption rate (the product the message of the program tells)</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>executable, 0x44d042</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>one byte</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Executable</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>The byte is 58 (addss) and becomes 59 (mulss)</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>docs/FORMULAS.md 2.5: the only reader of effect 264 as a status is 0x44cfad. Not seen working in the game yet</t>
         </is>
       </c>
     </row>
@@ -25844,7 +25643,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Concentrate: its value is ADDED to max HP * 1.5 + 1 in the divisor of the interruption rate of a blow (the debug message writes a product; the code is addss at 0x44d042), so with values of 0.1 - 0.5 it changes nothing that can be seen. A spell has no such rate: it breaks a chant only by the second roll of a critical</t>
+          <t>Concentrate: its value is ADDED to max HP * 1.5 + 1 in the divisor of the interruption rate of a blow (the debug message writes a product; the code is addss at 0x44d042), so with values of 0.1 - 0.5 it changes nothing that can be seen. A spell has no such rate: it breaks a chant only by the second roll of a critical. On the Balance variant row X14 of the sheet ExePatches makes it the product: the rate is divided by 1 + value</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">

</xml_diff>

<commit_message>
balance: the unique skill of Lizerietta is the chance to hold on with 1
the unique skill of Lizerietta is the chance to hold on with 1 HP when a
hit would fell her (effect 254, 15 - 40%, crown 55%), named No Miracles
Needed; evasion dropped
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -13190,12 +13190,12 @@
       </c>
       <c r="Q174" t="inlineStr">
         <is>
-          <t>U011 - U020, U051: the skill becomes evasion (effect 338, 10 - 26% by rank, 35% with the crown), named again in the variant</t>
+          <t>U011 - U020, U051: the skill becomes the chance to hold on with 1 HP when a hit would fell her (effect 254, 15 - 40% by rank, 55% with the crown), named again in the variant</t>
         </is>
       </c>
       <c r="R174" t="inlineStr">
         <is>
-          <t>the user, 2026-10-12: raised | 2026-10-12 (evening), the user: the effect is changed for evasion, which serves in every class and fight</t>
+          <t>the user, 2026-10-12: raised | 2026-10-12 (evening), the user: the effect is changed for evasion, which serves in every class and fight | 2026-10-12 (night), the user: not evasion (always at work); the chance to survive a killing hit, situational as the others</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
balance: effect 254 is not rolled at 1 HP (X15, lever L46)
effect 254 is not rolled at 1 HP (X15, lever L46); Eccentrics gives AGI
(the effect of Vagabonds); the simulator builds the doll of a guest
ally; the program test works on a copy inside the project; README
brought up to date
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -13699,7 +13699,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -14345,6 +14345,43 @@
       <c r="I20" t="inlineStr">
         <is>
           <t>Interruption rate of a blow: max HP * 1.5 times (1 + Concentrate) where the program adds the two (addss -&gt; mulss at 0x44d042; its debug message writes the product). The user, 2026-10-12: mend it for every unit, enemies with the passive too</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>X15</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>balance</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>L46</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>0x4238a2</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>2b454085c00f8f</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>48483b45400f83</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Effect 254 (Guts; the unique skill of Lizerietta on the variant) is not rolled for a unit at 1 HP: "HP - damage &gt; 0, skip" becomes "HP - 2 &gt;= damage as unsigned, skip" (dec eax twice, cmp eax with the damage, jae to the same place). A hit that leaves exactly 1 HP now rolls too, with the same result. The user, 2026-10-12: no loop of never falling</t>
         </is>
       </c>
     </row>
@@ -22729,7 +22766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G52"/>
+  <dimension ref="A1:G53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -24495,6 +24532,43 @@
       <c r="G52" t="inlineStr">
         <is>
           <t>docs/FORMULAS.md 2.5: the only reader of effect 264 as a status is 0x44cfad. Not seen working in the game yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>L46</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>The roll of effect 254 is skipped at 1 HP</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>executable, 0x4238a2</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>seven bytes</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Executable</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>The seven bytes are the ones the row names; the jump keeps its place and its target</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>docs/FORMULAS.md 12.7; eax is loaded again at both ends of the jump (0x4238ad, 0x423a18). No enemy has the effect. Not seen working in the game yet</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
balance: the guard of effect 254 at 1 HP withdrawn
the guard of effect 254 at 1 HP withdrawn (X15, L46 out: it changed Guts
too); the box of No Miracles Needed back to its sentence
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -13699,7 +13699,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -14283,6 +14283,7 @@
         </is>
       </c>
     </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
@@ -14345,43 +14346,6 @@
       <c r="I20" t="inlineStr">
         <is>
           <t>Interruption rate of a blow: max HP * 1.5 times (1 + Concentrate) where the program adds the two (addss -&gt; mulss at 0x44d042; its debug message writes the product). The user, 2026-10-12: mend it for every unit, enemies with the passive too</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>X15</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>balance</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>L46</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>0x4238a2</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>2b454085c00f8f</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>48483b45400f83</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>Effect 254 (Guts; the unique skill of Lizerietta on the variant) is not rolled for a unit at 1 HP: "HP - damage &gt; 0, skip" becomes "HP - 2 &gt;= damage as unsigned, skip" (dec eax twice, cmp eax with the damage, jae to the same place). A hit that leaves exactly 1 HP now rolls too, with the same result. The user, 2026-10-12: no loop of never falling</t>
         </is>
       </c>
     </row>
@@ -22766,7 +22730,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G53"/>
+  <dimension ref="A1:G52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -24253,6 +24217,7 @@
         </is>
       </c>
     </row>
+    <row r="41"/>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
@@ -24532,43 +24497,6 @@
       <c r="G52" t="inlineStr">
         <is>
           <t>docs/FORMULAS.md 2.5: the only reader of effect 264 as a status is 0x44cfad. Not seen working in the game yet</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>L46</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>The roll of effect 254 is skipped at 1 HP</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>executable, 0x4238a2</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>seven bytes</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>Executable</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>The seven bytes are the ones the row names; the jump keeps its place and its target</t>
-        </is>
-      </c>
-      <c r="G53" t="inlineStr">
-        <is>
-          <t>docs/FORMULAS.md 12.7; eax is loaded again at both ends of the jump (0x4238ad, 0x423a18). No enemy has the effect. Not seen working in the game yet</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
sim: the measures and readings the workbooks and documents cite leave
the measures and readings the workbooks and documents cite leave scratch
for mod_project/measures (21 scripts, 12 reports), every citation
follows; the four readers of the program used by hand join tools as
exe_dis, exe_find_const, exe_who_calls, exe_around
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_criteria.xlsx
+++ b/mod_project/data_tables/balance_criteria.xlsx
@@ -673,7 +673,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>scratch/audit_2026-10-11/magic_wall.py and j02_resistances.py (best option of the mage beside the best of the Dark Lord, value per time): above 100% at 55 of the 66 bosses from C30 on (median 240%), four fights forbid magic, 97% at Kuchinawa. At the six superboss fights where she was under him: Hell's Angel 51% &gt; 59%, Panagia 73% &gt; 95% and 84% &gt; 104%, Tenerezza 50% &gt; 80% and 54% &gt; 70%, Samson with Magna Meretrix 51% &gt; 57% with E213 - E223 (RES x0.9). The elemental resistances are left alone: lowering them by 20 raised the earth and water strikes of the Dark Lord as much as the spells and left her where she was; what walls the spells off is the magic defence of these enemies (RES 407 - 1,648 against INT 353 - 363)</t>
+          <t>measures/magic_wall.py and j02_resistances.py (best option of the mage beside the best of the Dark Lord, value per time): above 100% at 55 of the 66 bosses from C30 on (median 240%), four fights forbid magic, 97% at Kuchinawa. At the six superboss fights where she was under him: Hell's Angel 51% &gt; 59%, Panagia 73% &gt; 95% and 84% &gt; 104%, Tenerezza 50% &gt; 80% and 54% &gt; 70%, Samson with Magna Meretrix 51% &gt; 57% with E213 - E223 (RES x0.9). The elemental resistances are left alone: lowering them by 20 raised the earth and water strikes of the Dark Lord as much as the spells and left her where she was; what walls the spells off is the magic defence of these enemies (RES 407 - 1,648 against INT 353 - 363)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -3435,7 +3435,7 @@
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>Y012 - Y014 (Magical Fruit 25 to 30 TP, Fairy Apple 50 to 60, Golden Apple 100 to 120), built and read back (1,401 of 1,401 rows). The Meta party with a Bishop in the place of its Diva, nobody of the Maid line in it (scratch/audit_2026-10-11/tp_items_trial.py, 60 battles): with the 8 fruit of the sheets 3% / 3% / 18% / 68% at C30 / C34 / C36 / C38; with 24 fruit in the bag 67% / 82% / 45% / 98% (47% / 52% / 38% / 97% before the raise). What stops such a party at C30 and C34 is TP (100% with TP at will); C36 does not turn on it, and the last boss is not won without the Maid line (0%; 45% with 99 fruit). Up to C28 the party wins 78 - 100% without her. Nothing else moved: curve 37 of 44, battery 75 of 85, classes 74 of 76, anchors 6 of 6</t>
+          <t>Y012 - Y014 (Magical Fruit 25 to 30 TP, Fairy Apple 50 to 60, Golden Apple 100 to 120), built and read back (1,401 of 1,401 rows). The Meta party with a Bishop in the place of its Diva, nobody of the Maid line in it (measures/tp_items_trial.py, 60 battles): with the 8 fruit of the sheets 3% / 3% / 18% / 68% at C30 / C34 / C36 / C38; with 24 fruit in the bag 67% / 82% / 45% / 98% (47% / 52% / 38% / 97% before the raise). What stops such a party at C30 and C34 is TP (100% with TP at will); C36 does not turn on it, and the last boss is not won without the Maid line (0%; 45% with 99 fruit). Up to C28 the party wins 78 - 100% without her. Nothing else moved: curve 37 of 44, battery 75 of 85, classes 74 of 76, anchors 6 of 6</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
@@ -6467,7 +6467,7 @@
       </c>
       <c r="K80" t="inlineStr">
         <is>
-          <t>scratch/audit_2026-10-11/worth_with_weapon.py (the measure of tools/skill_worth.py, the Sage with a Tome): Bible Thump is her best option at the bosses of C40 and P08, 90% of it at P18, 74% at C34, 27 - 29% at C22 and C30; in random battles 43 - 89% (9% where a row falls to one spell)</t>
+          <t>measures/worth_with_weapon.py (the measure of tools/skill_worth.py, the Sage with a Tome): Bible Thump is her best option at the bosses of C40 and P08, 90% of it at P18, 74% at C34, 27 - 29% at C22 and C30; in random battles 43 - 89% (9% where a row falls to one spell)</t>
         </is>
       </c>
       <c r="L80" t="inlineStr">
@@ -7167,7 +7167,7 @@
       </c>
       <c r="K90" t="inlineStr">
         <is>
-          <t>scratch/audit_2026-10-11/measure_open_rows.py: the reference party with and without Support Shot at its top level: C22 100% / 100% wins, length +2%; C30 +6%; C34 -4%; C40 80% / 73% wins (40 fights each: inside the noise). Raised to 10 - 30% (W047 - W051): it pays beside members who strike plainly, which the reference party does not hold, so the measure of the party does not move</t>
+          <t>measures/measure_open_rows.py: the reference party with and without Support Shot at its top level: C22 100% / 100% wins, length +2%; C30 +6%; C34 -4%; C40 80% / 73% wins (40 fights each: inside the noise). Raised to 10 - 30% (W047 - W051): it pays beside members who strike plainly, which the reference party does not hold, so the measure of the party does not move</t>
         </is>
       </c>
       <c r="L90" t="inlineStr">
@@ -8624,7 +8624,7 @@
       </c>
       <c r="K111" t="inlineStr">
         <is>
-          <t>scratch/audit_2026-10-11/worth_with_weapon.py (the Joker with a Whip): Beast Binder is her best option in the random battles of C34, C40 and P08, 104 - 134% of her best with her axe at C40; 39 - 82% against the bosses. Whips forge at rate 2.0 (W rows)</t>
+          <t>measures/worth_with_weapon.py (the Joker with a Whip): Beast Binder is her best option in the random battles of C34, C40 and P08, 104 - 134% of her best with her axe at C40; 39 - 82% against the bosses. Whips forge at rate 2.0 (W rows)</t>
         </is>
       </c>
       <c r="L111" t="inlineStr">
@@ -9838,7 +9838,7 @@
       </c>
       <c r="N128" t="inlineStr">
         <is>
-          <t>Read on 2026-10-11 (scratch/drops_reading.md, checked against 0x558517 - 0x5586fa): rows P011 - P023 and P025 of balance_changes.xlsx dropped, they changed the count of slots of drops that are certain or usual. Rows P024, P079 - P084 raise the seven pieces under 2% to 2%. The weight of a slot is the same word for the drop and for the steal (scratch/steal_reading.md, checked on 2026-10-11): with the rows the Chief's Special comes out of 4.7% of the steals that succeed. Rows P085 - P088 (the user, 2026-10-11): Odin, Myrddin, Asmodeus and Carmilla, the four enemies of the random battles that could not be robbed, can be: their pieces come out of 6 to 9% of the steals that succeed, against 3.9 to 5.4% of the kills.</t>
+          <t>Read on 2026-10-11 (measures/drops_reading.md, checked against 0x558517 - 0x5586fa): rows P011 - P023 and P025 of balance_changes.xlsx dropped, they changed the count of slots of drops that are certain or usual. Rows P024, P079 - P084 raise the seven pieces under 2% to 2%. The weight of a slot is the same word for the drop and for the steal (measures/steal_reading.md, checked on 2026-10-11): with the rows the Chief's Special comes out of 4.7% of the steals that succeed. Rows P085 - P088 (the user, 2026-10-11): Odin, Myrddin, Asmodeus and Carmilla, the four enemies of the random battles that could not be robbed, can be: their pieces come out of 6 to 9% of the steals that succeed, against 3.9 to 5.4% of the kills.</t>
         </is>
       </c>
       <c r="O128" t="inlineStr">
@@ -10141,7 +10141,7 @@
       </c>
       <c r="R132" t="inlineStr">
         <is>
-          <t>2026-10-10: no change; mercenary flavor preserved | 2026-10-12: every mercenary measured (scratch/audit_2026-10-11/MERCENARIES.md); none above the summon of the grand sealbook; Natalia, the last, gets RES x1.5 (N001 - N005)</t>
+          <t>2026-10-10: no change; mercenary flavor preserved | 2026-10-12: every mercenary measured (measures/MERCENARIES.md); none above the summon of the grand sealbook; Natalia, the last, gets RES x1.5 (N001 - N005)</t>
         </is>
       </c>
     </row>
@@ -12500,7 +12500,7 @@
       </c>
       <c r="K164" t="inlineStr">
         <is>
-          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Irena as mage, without the skill &gt; with it): C36 87% &gt; 88%, C38 98% &gt; 95%, C40 78% &gt; 75%, P24 88% &gt; 86%, P27 crowned 51% &gt; 52%. In the mean -1 points of wins, fights +4% shorter, -1 points of HP left (a cell moves by about 5 points by chance). Read again on 2026-10-12: one roll below 100 under value * 100 for each chanted command (0x4176a0, called at 0x41d69c for a spell and at 0x419c55 for the other chanted kind, each behind a flag that keeps it to one roll): 7 - 15% by rank, 20% crowned. Both guides felt 40 - 50% with the crown</t>
+          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Irena as mage, without the skill &gt; with it): C36 87% &gt; 88%, C38 98% &gt; 95%, C40 78% &gt; 75%, P24 88% &gt; 86%, P27 crowned 51% &gt; 52%. In the mean -1 points of wins, fights +4% shorter, -1 points of HP left (a cell moves by about 5 points by chance). Read again on 2026-10-12: one roll below 100 under value * 100 for each chanted command (0x4176a0, called at 0x41d69c for a spell and at 0x419c55 for the other chanted kind, each behind a flag that keeps it to one roll): 7 - 15% by rank, 20% crowned. Both guides felt 40 - 50% with the crown</t>
         </is>
       </c>
       <c r="L164" t="inlineStr">
@@ -12567,7 +12567,7 @@
       </c>
       <c r="K165" t="inlineStr">
         <is>
-          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Yae as dark lord, without the skill &gt; with it): C36 95% &gt; 93%, C38 91% &gt; 95%, C40 94% &gt; 96%, P24 100% &gt; 99%, P27 crowned 91% &gt; 92%. In the mean +1 points of wins, fights +7% shorter, -0 points of HP left (a cell moves by about 5 points by chance). Played since 2026-10-12 as read: the second action belongs to the same turn, so her statuses do not lose a turn between the two (Power Charge serves both blows)</t>
+          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Yae as dark lord, without the skill &gt; with it): C36 95% &gt; 93%, C38 91% &gt; 95%, C40 94% &gt; 96%, P24 100% &gt; 99%, P27 crowned 91% &gt; 92%. In the mean +1 points of wins, fights +7% shorter, -0 points of HP left (a cell moves by about 5 points by chance). Played since 2026-10-12 as read: the second action belongs to the same turn, so her statuses do not lose a turn between the two (Power Charge serves both blows)</t>
         </is>
       </c>
       <c r="L165" t="inlineStr">
@@ -12634,7 +12634,7 @@
       </c>
       <c r="K166" t="inlineStr">
         <is>
-          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Ist as etoile, without the skill &gt; with it): C36 76% &gt; 83%, C38 96% &gt; 98%, C40 96% &gt; 97%, P24 98% &gt; 99%, P27 crowned 71% &gt; 72%. In the mean +2 points of wins, fights +0% shorter, +2 points of HP left (a cell moves by about 5 points by chance).</t>
+          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Ist as etoile, without the skill &gt; with it): C36 76% &gt; 83%, C38 96% &gt; 98%, C40 96% &gt; 97%, P24 98% &gt; 99%, P27 crowned 71% &gt; 72%. In the mean +2 points of wins, fights +0% shorter, +2 points of HP left (a cell moves by about 5 points by chance).</t>
         </is>
       </c>
       <c r="L166" t="inlineStr">
@@ -12701,7 +12701,7 @@
       </c>
       <c r="K167" t="inlineStr">
         <is>
-          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Melvy as magical princess, without the skill &gt; with it): C36 79% &gt; 82%, C38 99% &gt; 100%, C40 76% &gt; 73%, P24 85% &gt; 79%, P27 crowned 64% &gt; 63%. In the mean -1 points of wins, fights +2% shorter, -2 points of HP left (a cell moves by about 5 points by chance).</t>
+          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Melvy as magical princess, without the skill &gt; with it): C36 79% &gt; 82%, C38 99% &gt; 100%, C40 76% &gt; 73%, P24 85% &gt; 79%, P27 crowned 64% &gt; 63%. In the mean -1 points of wins, fights +2% shorter, -2 points of HP left (a cell moves by about 5 points by chance).</t>
         </is>
       </c>
       <c r="L167" t="inlineStr">
@@ -12768,7 +12768,7 @@
       </c>
       <c r="K168" t="inlineStr">
         <is>
-          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Mefmera as papillon, without the skill &gt; with it): C36 81% &gt; 84%, C38 97% &gt; 100%, C40 86% &gt; 95%, P24 94% &gt; 98%, P27 crowned 89% &gt; 98%. In the mean +6 points of wins, fights +4% shorter, +5 points of HP left (a cell moves by about 5 points by chance). It cuts the damage of demons, undead and apparitions: Samael (C38) and Melek Taus (P27) are demons; the race of the others was not checked against its list</t>
+          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Mefmera as papillon, without the skill &gt; with it): C36 81% &gt; 84%, C38 97% &gt; 100%, C40 86% &gt; 95%, P24 94% &gt; 98%, P27 crowned 89% &gt; 98%. In the mean +6 points of wins, fights +4% shorter, +5 points of HP left (a cell moves by about 5 points by chance). It cuts the damage of demons, undead and apparitions: Samael (C38) and Melek Taus (P27) are demons; the race of the others was not checked against its list</t>
         </is>
       </c>
       <c r="L168" t="inlineStr">
@@ -12835,7 +12835,7 @@
       </c>
       <c r="K169" t="inlineStr">
         <is>
-          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Eltricia as magical princess, without the skill &gt; with it): C36 79% &gt; 89%, C38 99% &gt; 97%, C40 76% &gt; 75%, P24 85% &gt; 78%, P27 crowned 64% &gt; 68%. In the mean +1 points of wins, fights +1% shorter, -0 points of HP left (a cell moves by about 5 points by chance).</t>
+          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Eltricia as magical princess, without the skill &gt; with it): C36 79% &gt; 89%, C38 99% &gt; 97%, C40 76% &gt; 75%, P24 85% &gt; 78%, P27 crowned 64% &gt; 68%. In the mean +1 points of wins, fights +1% shorter, -0 points of HP left (a cell moves by about 5 points by chance).</t>
         </is>
       </c>
       <c r="L169" t="inlineStr">
@@ -12902,7 +12902,7 @@
       </c>
       <c r="K170" t="inlineStr">
         <is>
-          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Alisia as attacker, without the skill &gt; with it): C36 93% &gt; 91%, C38 80% &gt; 82%, C40 45% &gt; 49%, P24 99% &gt; 98%, P27 crowned 69% &gt; 68%. In the mean +0 points of wins, fights +2% shorter, -0 points of HP left (a cell moves by about 5 points by chance). The simulator holds Pep at 100; she was played at Pep 130, the most it can be, so this is the most the skill gives: +6% damage at rank 5 - 6, +15% at rank 9, +30% crowned (the guide measured about +15% at level 90)</t>
+          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Alisia as attacker, without the skill &gt; with it): C36 93% &gt; 91%, C38 80% &gt; 82%, C40 45% &gt; 49%, P24 99% &gt; 98%, P27 crowned 69% &gt; 68%. In the mean +0 points of wins, fights +2% shorter, -0 points of HP left (a cell moves by about 5 points by chance). The simulator holds Pep at 100; she was played at Pep 130, the most it can be, so this is the most the skill gives: +6% damage at rank 5 - 6, +15% at rank 9, +30% crowned (the guide measured about +15% at level 90)</t>
         </is>
       </c>
       <c r="L170" t="inlineStr">
@@ -12969,7 +12969,7 @@
       </c>
       <c r="K171" t="inlineStr">
         <is>
-          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Luco as dark lord, without the skill &gt; with it): C36 82% &gt; 88%, C38 98% &gt; 100%, C40 88% &gt; 86%, P24 95% &gt; 90%, P27 crowned 83% &gt; 77%. In the mean -1 points of wins, fights +8% shorter, -1 points of HP left (a cell moves by about 5 points by chance). Played since 2026-10-12 as read (scratch/qol_fields_reading.md 5, checked): the shadow has the stats of its owner at that moment with twice the ATK, her passives, none of the statuses techniques put, a life of 3. The fault the Japanese page tells (its attack falling back after a drain) is not in the program by that reading</t>
+          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Luco as dark lord, without the skill &gt; with it): C36 82% &gt; 88%, C38 98% &gt; 100%, C40 88% &gt; 86%, P24 95% &gt; 90%, P27 crowned 83% &gt; 77%. In the mean -1 points of wins, fights +8% shorter, -1 points of HP left (a cell moves by about 5 points by chance). Played since 2026-10-12 as read (measures/qol_fields_reading.md 5, checked): the shadow has the stats of its owner at that moment with twice the ATK, her passives, none of the statuses techniques put, a life of 3. The fault the Japanese page tells (its attack falling back after a drain) is not in the program by that reading</t>
         </is>
       </c>
       <c r="L171" t="inlineStr">
@@ -13036,7 +13036,7 @@
       </c>
       <c r="K172" t="inlineStr">
         <is>
-          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Grishna as attacker, without the skill &gt; with it): C36 90% &gt; 88%, C38 98% &gt; 97%, C40 71% &gt; 72%, P24 87% &gt; 89%, P27 crowned 67% &gt; 75%. In the mean +2 points of wins, fights +4% shorter, +0 points of HP left (a cell moves by about 5 points by chance).</t>
+          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Grishna as attacker, without the skill &gt; with it): C36 90% &gt; 88%, C38 98% &gt; 97%, C40 71% &gt; 72%, P24 87% &gt; 89%, P27 crowned 67% &gt; 75%. In the mean +2 points of wins, fights +4% shorter, +0 points of HP left (a cell moves by about 5 points by chance).</t>
         </is>
       </c>
       <c r="L172" t="inlineStr">
@@ -13103,7 +13103,7 @@
       </c>
       <c r="K173" t="inlineStr">
         <is>
-          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Monica as shooter, without the skill &gt; with it): C36 81% &gt; 89%, C38 97% &gt; 98%, C40 76% &gt; 72%, P24 86% &gt; 88%, P27 crowned 50% &gt; 53%. In the mean +2 points of wins, fights +6% shorter, +2 points of HP left (a cell moves by about 5 points by chance).</t>
+          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Monica as shooter, without the skill &gt; with it): C36 81% &gt; 89%, C38 97% &gt; 98%, C40 76% &gt; 72%, P24 86% &gt; 88%, P27 crowned 50% &gt; 53%. In the mean +2 points of wins, fights +6% shorter, +2 points of HP left (a cell moves by about 5 points by chance).</t>
         </is>
       </c>
       <c r="L173" t="inlineStr">
@@ -13170,7 +13170,7 @@
       </c>
       <c r="K174" t="inlineStr">
         <is>
-          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Lizerietta as papillon, without the skill &gt; with it): C36 95% &gt; 92%, C38 96% &gt; 97%, C40 96% &gt; 96%, P24 100% &gt; 100%, P27 crowned 85% &gt; 86%. In the mean -0 points of wins, fights -2% shorter, -1 points of HP left (a cell moves by about 5 points by chance). It only acts on what an enemy summons; which of these five fights hold a summoner was not looked at Built on 2026-10-12. None of the five fights of the measure holds anything it can remove, with or without the raise: its worth is only against the enemies that summon, not measured</t>
+          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Lizerietta as papillon, without the skill &gt; with it): C36 95% &gt; 92%, C38 96% &gt; 97%, C40 96% &gt; 96%, P24 100% &gt; 100%, P27 crowned 85% &gt; 86%. In the mean -0 points of wins, fights -2% shorter, -1 points of HP left (a cell moves by about 5 points by chance). It only acts on what an enemy summons; which of these five fights hold a summoner was not looked at Built on 2026-10-12. None of the five fights of the measure holds anything it can remove, with or without the raise: its worth is only against the enemies that summon, not measured</t>
         </is>
       </c>
       <c r="L174" t="inlineStr">
@@ -13242,7 +13242,7 @@
       </c>
       <c r="K175" t="inlineStr">
         <is>
-          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Souffle as treasure hunter, without the skill &gt; with it): C36 87% &gt; 94%, C38 91% &gt; 96%, C40 91% &gt; 94%, P24 100% &gt; 99%, P27 crowned 86% &gt; 85%. In the mean +3 points of wins, fights +4% shorter, +4 points of HP left (a cell moves by about 5 points by chance).</t>
+          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Souffle as treasure hunter, without the skill &gt; with it): C36 87% &gt; 94%, C38 91% &gt; 96%, C40 91% &gt; 94%, P24 100% &gt; 99%, P27 crowned 86% &gt; 85%. In the mean +3 points of wins, fights +4% shorter, +4 points of HP left (a cell moves by about 5 points by chance).</t>
         </is>
       </c>
       <c r="L175" t="inlineStr">
@@ -13309,7 +13309,7 @@
       </c>
       <c r="K176" t="inlineStr">
         <is>
-          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Conette as mistress, without the skill &gt; with it): C36 81% &gt; 89%, C38 98% &gt; 99%, C40 93% &gt; 98%, P24 97% &gt; 98%, P27 crowned 67% &gt; 83%. In the mean +6 points of wins, fights +2% shorter, +7 points of HP left (a cell moves by about 5 points by chance).</t>
+          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Conette as mistress, without the skill &gt; with it): C36 81% &gt; 89%, C38 98% &gt; 99%, C40 93% &gt; 98%, P24 97% &gt; 98%, P27 crowned 67% &gt; 83%. In the mean +6 points of wins, fights +2% shorter, +7 points of HP left (a cell moves by about 5 points by chance).</t>
         </is>
       </c>
       <c r="L176" t="inlineStr">
@@ -13376,7 +13376,7 @@
       </c>
       <c r="K177" t="inlineStr">
         <is>
-          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Fiora as healer, without the skill &gt; with it): C36 85% &gt; 89%, C38 98% &gt; 97%, C40 100% &gt; 98%, P24 97% &gt; 99%, P27 crowned 70% &gt; 80%. In the mean +3 points of wins, fights -0% shorter, +3 points of HP left (a cell moves by about 5 points by chance). Raised for the feel of it on 2026-10-12: 90.0% without the skill, 94.2% with it (92.6% before)</t>
+          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Fiora as healer, without the skill &gt; with it): C36 85% &gt; 89%, C38 98% &gt; 97%, C40 100% &gt; 98%, P24 97% &gt; 99%, P27 crowned 70% &gt; 80%. In the mean +3 points of wins, fights -0% shorter, +3 points of HP left (a cell moves by about 5 points by chance). Raised for the feel of it on 2026-10-12: 90.0% without the skill, 94.2% with it (92.6% before)</t>
         </is>
       </c>
       <c r="L177" t="inlineStr">
@@ -13448,7 +13448,7 @@
       </c>
       <c r="K178" t="inlineStr">
         <is>
-          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Yuni as diva, without the skill &gt; with it): C36 96% &gt; 96%, C38 95% &gt; 95%, C40 93% &gt; 94%, P24 97% &gt; 99%, P27 crowned 83% &gt; 93%. In the mean +3 points of wins, fights +1% shorter, +3 points of HP left (a cell moves by about 5 points by chance). Raised a little on 2026-10-12 (the user: it is one of the good ones): 92.8% without the skill, 94.8% with it</t>
+          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Yuni as diva, without the skill &gt; with it): C36 96% &gt; 96%, C38 95% &gt; 95%, C40 93% &gt; 94%, P24 97% &gt; 99%, P27 crowned 83% &gt; 93%. In the mean +3 points of wins, fights +1% shorter, +3 points of HP left (a cell moves by about 5 points by chance). Raised a little on 2026-10-12 (the user: it is one of the good ones): 92.8% without the skill, 94.8% with it</t>
         </is>
       </c>
       <c r="L178" t="inlineStr">
@@ -13520,7 +13520,7 @@
       </c>
       <c r="K179" t="inlineStr">
         <is>
-          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Lilian as soul summoner, without the skill &gt; with it): C36 87% &gt; 82%, C38 92% &gt; 96%, C40 78% &gt; 73%, P24 79% &gt; 81%, P27 crowned 57% &gt; 58%. In the mean -1 points of wins, fights +1% shorter, +0 points of HP left (a cell moves by about 5 points by chance). Its seventh result, the dispel, removes nothing: 0x47ee6f jumps over the routine (scratch/qol_fields_reading.md 7, checked), as the Japanese page says; played so since 2026-10-12 Built on 2026-10-12 (1,421 of 1,421 rows): the reference party wins 78.6% of the five bosses without it and 80.2% with it (78.0% before); rows of eight random battles at four floors do not run away with it</t>
+          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Lilian as soul summoner, without the skill &gt; with it): C36 87% &gt; 82%, C38 92% &gt; 96%, C40 78% &gt; 73%, P24 79% &gt; 81%, P27 crowned 57% &gt; 58%. In the mean -1 points of wins, fights +1% shorter, +0 points of HP left (a cell moves by about 5 points by chance). Its seventh result, the dispel, removes nothing: 0x47ee6f jumps over the routine (measures/qol_fields_reading.md 7, checked), as the Japanese page says; played so since 2026-10-12 Built on 2026-10-12 (1,421 of 1,421 rows): the reference party wins 78.6% of the five bosses without it and 80.2% with it (78.0% before); rows of eight random battles at four floors do not run away with it</t>
         </is>
       </c>
       <c r="L179" t="inlineStr">
@@ -13592,7 +13592,7 @@
       </c>
       <c r="K180" t="inlineStr">
         <is>
-          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Tsurara as treasure hunter, without the skill &gt; with it): C36 87% &gt; 93%, C38 91% &gt; 92%, C40 91% &gt; 91%, P24 100% &gt; 100%, P27 crowned 86% &gt; 97%. In the mean +4 points of wins, fights +0% shorter, +4 points of HP left (a cell moves by about 5 points by chance).</t>
+          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Tsurara as treasure hunter, without the skill &gt; with it): C36 87% &gt; 93%, C38 91% &gt; 92%, C40 91% &gt; 91%, P24 100% &gt; 100%, P27 crowned 86% &gt; 97%. In the mean +4 points of wins, fights +0% shorter, +4 points of HP left (a cell moves by about 5 points by chance).</t>
         </is>
       </c>
       <c r="L180" t="inlineStr">
@@ -13659,7 +13659,7 @@
       </c>
       <c r="K181" t="inlineStr">
         <is>
-          <t>scratch/audit_2026-10-11/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Siena as magical princess, without the skill &gt; with it): C36 79% &gt; 79%, C38 99% &gt; 96%, C40 76% &gt; 79%, P24 85% &gt; 84%, P27 crowned 64% &gt; 73%. In the mean +2 points of wins, fights -3% shorter, +1 points of HP left (a cell moves by about 5 points by chance). Built on 2026-10-12. The measure does not move with it (82.2% as it was, 82.0% at 25%, 80.6% without the skill): what it sends back is a share of the damage she takes, little beside the HP of a boss. Raised for the feel of it, at the word of the user With both, 81.6% without the skill and 83.0% with it</t>
+          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Siena as magical princess, without the skill &gt; with it): C36 79% &gt; 79%, C38 99% &gt; 96%, C40 76% &gt; 79%, P24 85% &gt; 84%, P27 crowned 64% &gt; 73%. In the mean +2 points of wins, fights -3% shorter, +1 points of HP left (a cell moves by about 5 points by chance). Built on 2026-10-12. The measure does not move with it (82.2% as it was, 82.0% at 25%, 80.6% without the skill): what it sends back is a share of the damage she takes, little beside the HP of a boss. Raised for the feel of it, at the word of the user With both, 81.6% without the skill and 83.0% with it</t>
         </is>
       </c>
       <c r="L181" t="inlineStr">
@@ -21856,6 +21856,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
@@ -22523,7 +22524,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>scratch/audit_2026-10-11/REGRESSION_R04.md (2026-10-12): at the 17 bosses of the battery, 27 pairs of boss and class on the variant (34 in vanilla) where every winning party of the battery holds the class. With the role of that class changed for a neighbour of the same job (60 battles), a party without it reaches the floor at 20 of the 27 (27 of 34 in vanilla): without a Diva or a Bard at 14 bosses (67 - 100%), without a Valkyrie at C29, C32, C36 and C40 (53 - 92%), without a Bishop at C29. Not reached: the Diva at C40 (the best party without her wins 22%, 13% in vanilla: needed there in vanilla too, and less so on the variant); the Sage and the Witch at C29, where only the mage party wins on either side (Calliope, which the model does not play as the guide describes); and the four base classes at C06, where five characters have joined and no other party can be made</t>
+          <t>measures/REGRESSION_R04.md (2026-10-12): at the 17 bosses of the battery, 27 pairs of boss and class on the variant (34 in vanilla) where every winning party of the battery holds the class. With the role of that class changed for a neighbour of the same job (60 battles), a party without it reaches the floor at 20 of the 27 (27 of 34 in vanilla): without a Diva or a Bard at 14 bosses (67 - 100%), without a Valkyrie at C29, C32, C36 and C40 (53 - 92%), without a Bishop at C29. Not reached: the Diva at C40 (the best party without her wins 22%, 13% in vanilla: needed there in vanilla too, and less so on the variant); the Sage and the Witch at C29, where only the mage party wins on either side (Calliope, which the model does not play as the guide describes); and the four base classes at C06, where five characters have joined and no other party can be made</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -24783,6 +24784,7 @@
         </is>
       </c>
     </row>
+    <row r="12"/>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
@@ -24952,6 +24954,7 @@
         </is>
       </c>
     </row>
+    <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>

</xml_diff>